<commit_message>
connect / write / listen
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
   <si>
     <t>Key</t>
   </si>
@@ -57,6 +57,18 @@
   <si>
     <t>Press your ring’s button for &lt;strong&gt;10 seconds&lt;/strong&gt; until it appears in the list. Your ring will vibrate once for each second you press it and a distinctive vibration will signal that you can release.</t>
   </si>
+  <si>
+    <t>setup.connection.pending</t>
+  </si>
+  <si>
+    <t>Setting up, this might take up to one minute.</t>
+  </si>
+  <si>
+    <t>setup.connection.success</t>
+  </si>
+  <si>
+    <t>Success !</t>
+  </si>
 </sst>
 </file>
 
@@ -77,11 +89,11 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font/>
   </fonts>
   <fills count="5">
     <fill>
@@ -115,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -140,17 +152,14 @@
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -420,11 +429,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="6"/>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="5" t="s">
@@ -432,11 +441,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="6"/>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="7" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -444,7 +453,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="6"/>
@@ -456,11 +465,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="9" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="6"/>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="7" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="5" t="s">
@@ -468,16 +477,28 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6"/>
+      <c r="A7" s="9" t="s">
+        <v>15</v>
+      </c>
       <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
+      <c r="C7" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="6"/>
+      <c r="A8" s="9" t="s">
+        <v>17</v>
+      </c>
       <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
+      <c r="C8" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6"/>
@@ -6439,7 +6460,7 @@
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D6">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D8">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Login view + Logic (not plugged)
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="30">
   <si>
     <t>Key</t>
   </si>
@@ -57,6 +57,51 @@
   <si>
     <t>Press your ring’s button for &lt;strong&gt;10 seconds&lt;/strong&gt; until it appears in the list. Your ring will vibrate once for each second you press it and a distinctive vibration will signal that you can release.</t>
   </si>
+  <si>
+    <t>setup.connection.pending</t>
+  </si>
+  <si>
+    <t>Setting up, this might take up to one minute.</t>
+  </si>
+  <si>
+    <t>setup.connection.success</t>
+  </si>
+  <si>
+    <t>Success !</t>
+  </si>
+  <si>
+    <t>login.title</t>
+  </si>
+  <si>
+    <t>Sign in</t>
+  </si>
+  <si>
+    <t>login.email.title</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>login.email.placeholder</t>
+  </si>
+  <si>
+    <t>Tap to write</t>
+  </si>
+  <si>
+    <t>login.password.title</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>login.password.placeholder</t>
+  </si>
+  <si>
+    <t>login.login_button</t>
+  </si>
+  <si>
+    <t>Confirm</t>
+  </si>
 </sst>
 </file>
 
@@ -77,11 +122,11 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font/>
   </fonts>
   <fills count="5">
     <fill>
@@ -140,17 +185,17 @@
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -420,11 +465,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="6"/>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="5" t="s">
@@ -432,11 +477,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="6"/>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="7" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -444,7 +489,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="6"/>
@@ -456,11 +501,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="9" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="6"/>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="7" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="5" t="s">
@@ -468,52 +513,100 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6"/>
+      <c r="A7" s="9" t="s">
+        <v>15</v>
+      </c>
       <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
+      <c r="C7" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="6"/>
+      <c r="A8" s="9" t="s">
+        <v>17</v>
+      </c>
       <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
+      <c r="C8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="6"/>
+      <c r="A9" s="10" t="s">
+        <v>19</v>
+      </c>
       <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
+      <c r="C9" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="6"/>
+      <c r="A10" s="10" t="s">
+        <v>21</v>
+      </c>
       <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
+      <c r="C10" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="6"/>
+      <c r="A11" s="10" t="s">
+        <v>23</v>
+      </c>
       <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
+      <c r="C11" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="6"/>
+      <c r="A12" s="10" t="s">
+        <v>25</v>
+      </c>
       <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
+      <c r="C12" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="6"/>
+      <c r="A13" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
+      <c r="C13" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="6"/>
+      <c r="A14" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
+      <c r="C14" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6"/>
@@ -6437,9 +6530,33 @@
       <c r="C1001" s="6"/>
       <c r="D1001" s="6"/>
     </row>
+    <row r="1002">
+      <c r="A1002" s="6"/>
+      <c r="B1002" s="6"/>
+      <c r="C1002" s="6"/>
+      <c r="D1002" s="6"/>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="6"/>
+      <c r="B1003" s="6"/>
+      <c r="C1003" s="6"/>
+      <c r="D1003" s="6"/>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="6"/>
+      <c r="B1004" s="6"/>
+      <c r="C1004" s="6"/>
+      <c r="D1004" s="6"/>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="6"/>
+      <c r="B1005" s="6"/>
+      <c r="C1005" s="6"/>
+      <c r="D1005" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D6">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D14">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
show battery on header
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="32">
   <si>
     <t>Key</t>
   </si>
@@ -68,6 +68,45 @@
   </si>
   <si>
     <t>Success !</t>
+  </si>
+  <si>
+    <t>login.title</t>
+  </si>
+  <si>
+    <t>Sign in</t>
+  </si>
+  <si>
+    <t>login.email.title</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>login.email.placeholder</t>
+  </si>
+  <si>
+    <t>Tap to write</t>
+  </si>
+  <si>
+    <t>login.password.title</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>login.password.placeholder</t>
+  </si>
+  <si>
+    <t>login.login_button</t>
+  </si>
+  <si>
+    <t>Confirm</t>
+  </si>
+  <si>
+    <t>header.my_ring</t>
+  </si>
+  <si>
+    <t>My Ring</t>
   </si>
 </sst>
 </file>
@@ -127,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -157,6 +196,9 @@
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
@@ -481,7 +523,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="6"/>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="7" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="5" t="s">
@@ -493,7 +535,7 @@
         <v>17</v>
       </c>
       <c r="B8" s="6"/>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="7" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="5" t="s">
@@ -501,46 +543,88 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6"/>
+      <c r="A9" s="10" t="s">
+        <v>19</v>
+      </c>
       <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
+      <c r="C9" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="6"/>
+      <c r="A10" s="10" t="s">
+        <v>21</v>
+      </c>
       <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
+      <c r="C10" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="6"/>
+      <c r="A11" s="10" t="s">
+        <v>23</v>
+      </c>
       <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
+      <c r="C11" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="6"/>
+      <c r="A12" s="10" t="s">
+        <v>25</v>
+      </c>
       <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
+      <c r="C12" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="6"/>
+      <c r="A13" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
+      <c r="C13" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="6"/>
+      <c r="A14" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
+      <c r="C14" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="6"/>
+      <c r="A15" s="10" t="s">
+        <v>30</v>
+      </c>
       <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
+      <c r="C15" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6"/>
@@ -6458,9 +6542,33 @@
       <c r="C1001" s="6"/>
       <c r="D1001" s="6"/>
     </row>
+    <row r="1002">
+      <c r="A1002" s="6"/>
+      <c r="B1002" s="6"/>
+      <c r="C1002" s="6"/>
+      <c r="D1002" s="6"/>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="6"/>
+      <c r="B1003" s="6"/>
+      <c r="C1003" s="6"/>
+      <c r="D1003" s="6"/>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="6"/>
+      <c r="B1004" s="6"/>
+      <c r="C1004" s="6"/>
+      <c r="D1004" s="6"/>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="6"/>
+      <c r="B1005" s="6"/>
+      <c r="C1005" s="6"/>
+      <c r="D1005" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D8">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D15">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
New dev api url + refresh token
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
   <si>
     <t>Key</t>
   </si>
@@ -101,6 +101,31 @@
   </si>
   <si>
     <t>Confirm</t>
+  </si>
+  <si>
+    <t>login.error.invalid_credentials</t>
+  </si>
+  <si>
+    <t>The email or password is invalid</t>
+  </si>
+  <si>
+    <t>login.error.default</t>
+  </si>
+  <si>
+    <t>An error occurred.
+Please try again later</t>
+  </si>
+  <si>
+    <t>header.my_ring</t>
+  </si>
+  <si>
+    <t>My Ring</t>
+  </si>
+  <si>
+    <t>ring.battery.label</t>
+  </si>
+  <si>
+    <t>BATTERY</t>
   </si>
 </sst>
 </file>
@@ -537,11 +562,11 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B9" s="6"/>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="7" t="s">
         <v>20</v>
       </c>
       <c r="D9" s="5" t="s">
@@ -549,11 +574,11 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B10" s="6"/>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="7" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="5" t="s">
@@ -561,11 +586,11 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B11" s="6"/>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="7" t="s">
         <v>24</v>
       </c>
       <c r="D11" s="5" t="s">
@@ -573,11 +598,11 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B12" s="6"/>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="7" t="s">
         <v>26</v>
       </c>
       <c r="D12" s="5" t="s">
@@ -585,11 +610,11 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="5" t="s">
         <v>27</v>
       </c>
       <c r="B13" s="6"/>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="7" t="s">
         <v>24</v>
       </c>
       <c r="D13" s="5" t="s">
@@ -597,11 +622,11 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B14" s="6"/>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="7" t="s">
         <v>29</v>
       </c>
       <c r="D14" s="5" t="s">
@@ -609,34 +634,58 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6"/>
+      <c r="A15" s="10" t="s">
+        <v>30</v>
+      </c>
       <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
+      <c r="C15" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="6"/>
+      <c r="A16" s="10" t="s">
+        <v>32</v>
+      </c>
       <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
+      <c r="C16" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="6"/>
+      <c r="A17" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
+      <c r="C17" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="6"/>
+      <c r="A18" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
+      <c r="C18" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="6"/>
+      <c r="A19" s="5"/>
       <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="5"/>
     </row>
     <row r="20">
       <c r="A20" s="6"/>
@@ -6554,9 +6603,21 @@
       <c r="C1005" s="6"/>
       <c r="D1005" s="6"/>
     </row>
+    <row r="1006">
+      <c r="A1006" s="6"/>
+      <c r="B1006" s="6"/>
+      <c r="C1006" s="6"/>
+      <c r="D1006" s="6"/>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="6"/>
+      <c r="B1007" s="6"/>
+      <c r="C1007" s="6"/>
+      <c r="D1007" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D14">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D19">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Signin or Signup screen
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="41">
   <si>
     <t>Key</t>
   </si>
@@ -127,12 +127,21 @@
   <si>
     <t>BATTERY</t>
   </si>
+  <si>
+    <t>signin_signup.signin</t>
+  </si>
+  <si>
+    <t>signin_signup.signup</t>
+  </si>
+  <si>
+    <t>Sign up</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -151,7 +160,6 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
-    <font/>
   </fonts>
   <fills count="5">
     <fill>
@@ -185,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -215,12 +223,6 @@
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -634,11 +636,11 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B15" s="6"/>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="7" t="s">
         <v>31</v>
       </c>
       <c r="D15" s="5" t="s">
@@ -646,11 +648,11 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B16" s="6"/>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="7" t="s">
         <v>33</v>
       </c>
       <c r="D16" s="5" t="s">
@@ -682,16 +684,28 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5"/>
+      <c r="A19" s="5" t="s">
+        <v>38</v>
+      </c>
       <c r="B19" s="6"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="5"/>
+      <c r="C19" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="6"/>
+      <c r="A20" s="8" t="s">
+        <v>39</v>
+      </c>
       <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
+      <c r="C20" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6"/>
@@ -6617,7 +6631,7 @@
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D19">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D20">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Email password screen ok
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="102">
   <si>
     <t>Key</t>
   </si>
@@ -183,6 +183,141 @@
   </si>
   <si>
     <t>terms and conditions.</t>
+  </si>
+  <si>
+    <t>signup.error.empty_field</t>
+  </si>
+  <si>
+    <t>Some fields are empty</t>
+  </si>
+  <si>
+    <t>signup.error.email_format</t>
+  </si>
+  <si>
+    <t>Email is not correct</t>
+  </si>
+  <si>
+    <t>signup.error.password_format</t>
+  </si>
+  <si>
+    <t>Password must be at least 4 characters, 1 lowercase, 1 uppercase and 1 digit</t>
+  </si>
+  <si>
+    <t>signup.error.password_confirm</t>
+  </si>
+  <si>
+    <t>Password fields are not identical</t>
+  </si>
+  <si>
+    <t>forgot_password.question</t>
+  </si>
+  <si>
+    <t>Forgot password ?</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.title</t>
+  </si>
+  <si>
+    <t>Pasword Reset</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.description</t>
+  </si>
+  <si>
+    <t>What’s the &lt;strong&gt;email&lt;/strong&gt; you signed up with?</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.email.placeholder</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.email.error</t>
+  </si>
+  <si>
+    <t>The email address you entered doesn’t match an existing Circular account. Please try again.</t>
+  </si>
+  <si>
+    <t>global.back</t>
+  </si>
+  <si>
+    <t>Back</t>
+  </si>
+  <si>
+    <t>global.next</t>
+  </si>
+  <si>
+    <t>Next</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.email.title</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.code.description</t>
+  </si>
+  <si>
+    <t>Enter the 6-digit code that we sent to &lt;strong&gt;{email}&lt;/strong&gt;.</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.code.resend_button</t>
+  </si>
+  <si>
+    <t>Resend Code</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.code.error</t>
+  </si>
+  <si>
+    <t>Password incorrect, please try again.</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.code.resend_description</t>
+  </si>
+  <si>
+    <t>We have just sent you another code. Enter the &lt;strong&gt;latest&lt;/strong&gt; one that you received. It might take a couple of minutes. Don’t forget to check your spam folder.</t>
+  </si>
+  <si>
+    <t>forgot_password.new.description</t>
+  </si>
+  <si>
+    <t>Perfect! You can now set up your new password and sign back in.</t>
+  </si>
+  <si>
+    <t>forgot_password.new.password</t>
+  </si>
+  <si>
+    <t>forgot_password.new.confirm_password</t>
+  </si>
+  <si>
+    <t>Confim password</t>
+  </si>
+  <si>
+    <t>forgot_password.new.button</t>
+  </si>
+  <si>
+    <t>Save and Sign in</t>
+  </si>
+  <si>
+    <t>home.sync.syncing</t>
+  </si>
+  <si>
+    <t>Refreshing...</t>
+  </si>
+  <si>
+    <t>home.sync.error</t>
+  </si>
+  <si>
+    <t>Sync failed</t>
+  </si>
+  <si>
+    <t>home.sync.success</t>
+  </si>
+  <si>
+    <t>Sync success</t>
+  </si>
+  <si>
+    <t>home.sync.retry</t>
+  </si>
+  <si>
+    <t>Retry</t>
   </si>
 </sst>
 </file>
@@ -763,11 +898,11 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="5" t="s">
         <v>41</v>
       </c>
       <c r="B21" s="6"/>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="7" t="s">
         <v>40</v>
       </c>
       <c r="D21" s="5" t="s">
@@ -775,11 +910,11 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="5" t="s">
         <v>42</v>
       </c>
       <c r="B22" s="6"/>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D22" s="5" t="s">
@@ -787,11 +922,11 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="5" t="s">
         <v>44</v>
       </c>
       <c r="B23" s="6"/>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="7" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="5" t="s">
@@ -799,11 +934,11 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="5" t="s">
         <v>45</v>
       </c>
       <c r="B24" s="6"/>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="7" t="s">
         <v>24</v>
       </c>
       <c r="D24" s="5" t="s">
@@ -811,11 +946,11 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B25" s="6"/>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="7" t="s">
         <v>26</v>
       </c>
       <c r="D25" s="5" t="s">
@@ -823,11 +958,11 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="5" t="s">
         <v>47</v>
       </c>
       <c r="B26" s="6"/>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="7" t="s">
         <v>24</v>
       </c>
       <c r="D26" s="5" t="s">
@@ -835,11 +970,11 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="5" t="s">
         <v>48</v>
       </c>
       <c r="B27" s="6"/>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="7" t="s">
         <v>49</v>
       </c>
       <c r="D27" s="5" t="s">
@@ -847,11 +982,11 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="5" t="s">
         <v>50</v>
       </c>
       <c r="B28" s="6"/>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="7" t="s">
         <v>24</v>
       </c>
       <c r="D28" s="5" t="s">
@@ -859,11 +994,11 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="5" t="s">
         <v>51</v>
       </c>
       <c r="B29" s="6"/>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="7" t="s">
         <v>29</v>
       </c>
       <c r="D29" s="5" t="s">
@@ -871,11 +1006,11 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="5" t="s">
         <v>52</v>
       </c>
       <c r="B30" s="6"/>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="7" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="5" t="s">
@@ -883,11 +1018,11 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="s">
+      <c r="A31" s="5" t="s">
         <v>53</v>
       </c>
       <c r="B31" s="6"/>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="7" t="s">
         <v>54</v>
       </c>
       <c r="D31" s="5" t="s">
@@ -895,11 +1030,11 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="5" t="s">
         <v>55</v>
       </c>
       <c r="B32" s="6"/>
-      <c r="C32" s="11" t="s">
+      <c r="C32" s="7" t="s">
         <v>56</v>
       </c>
       <c r="D32" s="5" t="s">
@@ -907,148 +1042,292 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6"/>
+      <c r="A33" s="10" t="s">
+        <v>57</v>
+      </c>
       <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
+      <c r="C33" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="6"/>
+      <c r="A34" s="10" t="s">
+        <v>59</v>
+      </c>
       <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
+      <c r="C34" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="6"/>
+      <c r="A35" s="10" t="s">
+        <v>61</v>
+      </c>
       <c r="B35" s="6"/>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
+      <c r="C35" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="6"/>
+      <c r="A36" s="10" t="s">
+        <v>63</v>
+      </c>
       <c r="B36" s="6"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
+      <c r="C36" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="6"/>
+      <c r="A37" s="5" t="s">
+        <v>65</v>
+      </c>
       <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
+      <c r="C37" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="6"/>
+      <c r="A38" s="5" t="s">
+        <v>67</v>
+      </c>
       <c r="B38" s="6"/>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
+      <c r="C38" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="6"/>
+      <c r="A39" s="5" t="s">
+        <v>69</v>
+      </c>
       <c r="B39" s="6"/>
-      <c r="C39" s="6"/>
-      <c r="D39" s="6"/>
+      <c r="C39" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="6"/>
+      <c r="A40" s="5" t="s">
+        <v>71</v>
+      </c>
       <c r="B40" s="6"/>
-      <c r="C40" s="6"/>
-      <c r="D40" s="6"/>
+      <c r="C40" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="6"/>
+      <c r="A41" s="5" t="s">
+        <v>72</v>
+      </c>
       <c r="B41" s="6"/>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
+      <c r="C41" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="6"/>
+      <c r="A42" s="5" t="s">
+        <v>74</v>
+      </c>
       <c r="B42" s="6"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
+      <c r="C42" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="6"/>
+      <c r="A43" s="5" t="s">
+        <v>76</v>
+      </c>
       <c r="B43" s="6"/>
-      <c r="C43" s="6"/>
-      <c r="D43" s="6"/>
+      <c r="C43" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="6"/>
+      <c r="A44" s="5" t="s">
+        <v>78</v>
+      </c>
       <c r="B44" s="6"/>
-      <c r="C44" s="6"/>
-      <c r="D44" s="6"/>
+      <c r="C44" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="6"/>
+      <c r="A45" s="5" t="s">
+        <v>79</v>
+      </c>
       <c r="B45" s="6"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
+      <c r="C45" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="6"/>
+      <c r="A46" s="5" t="s">
+        <v>81</v>
+      </c>
       <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
+      <c r="C46" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="6"/>
+      <c r="A47" s="10" t="s">
+        <v>83</v>
+      </c>
       <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6"/>
+      <c r="C47" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="6"/>
+      <c r="A48" s="5" t="s">
+        <v>85</v>
+      </c>
       <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
+      <c r="C48" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="6"/>
+      <c r="A49" s="5" t="s">
+        <v>87</v>
+      </c>
       <c r="B49" s="6"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
+      <c r="C49" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="6"/>
+      <c r="A50" s="5" t="s">
+        <v>89</v>
+      </c>
       <c r="B50" s="6"/>
-      <c r="C50" s="6"/>
-      <c r="D50" s="6"/>
+      <c r="C50" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="6"/>
+      <c r="A51" s="5" t="s">
+        <v>90</v>
+      </c>
       <c r="B51" s="6"/>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
+      <c r="C51" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="6"/>
+      <c r="A52" s="5" t="s">
+        <v>92</v>
+      </c>
       <c r="B52" s="6"/>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
+      <c r="C52" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="6"/>
+      <c r="A53" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="B53" s="6"/>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6"/>
+      <c r="C53" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="6"/>
+      <c r="A54" s="10" t="s">
+        <v>96</v>
+      </c>
       <c r="B54" s="6"/>
-      <c r="C54" s="6"/>
-      <c r="D54" s="6"/>
+      <c r="C54" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="6"/>
+      <c r="A55" s="10" t="s">
+        <v>98</v>
+      </c>
       <c r="B55" s="6"/>
-      <c r="C55" s="6"/>
-      <c r="D55" s="6"/>
+      <c r="C55" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="6"/>
+      <c r="A56" s="10" t="s">
+        <v>100</v>
+      </c>
       <c r="B56" s="6"/>
-      <c r="C56" s="6"/>
-      <c r="D56" s="6"/>
+      <c r="C56" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6"/>
@@ -6756,9 +7035,33 @@
       <c r="C1007" s="6"/>
       <c r="D1007" s="6"/>
     </row>
+    <row r="1008">
+      <c r="A1008" s="6"/>
+      <c r="B1008" s="6"/>
+      <c r="C1008" s="6"/>
+      <c r="D1008" s="6"/>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="6"/>
+      <c r="B1009" s="6"/>
+      <c r="C1009" s="6"/>
+      <c r="D1009" s="6"/>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="6"/>
+      <c r="B1010" s="6"/>
+      <c r="C1010" s="6"/>
+      <c r="D1010" s="6"/>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="6"/>
+      <c r="B1011" s="6"/>
+      <c r="C1011" s="6"/>
+      <c r="D1011" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D32">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D56">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add two screen reset token and newPassword
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="105">
   <si>
     <t>Key</t>
   </si>
@@ -185,6 +185,30 @@
     <t>terms and conditions.</t>
   </si>
   <si>
+    <t>signup.error.empty_field</t>
+  </si>
+  <si>
+    <t>Some fields are empty</t>
+  </si>
+  <si>
+    <t>signup.error.email_format</t>
+  </si>
+  <si>
+    <t>Email is not correct</t>
+  </si>
+  <si>
+    <t>signup.error.password_format</t>
+  </si>
+  <si>
+    <t>Password must be at least 4 characters, 1 lowercase, 1 uppercase and 1 digit</t>
+  </si>
+  <si>
+    <t>signup.error.password_confirm</t>
+  </si>
+  <si>
+    <t>Password fields are not identical</t>
+  </si>
+  <si>
     <t>forgot_password.question</t>
   </si>
   <si>
@@ -212,6 +236,63 @@
     <t>The email address you entered doesn’t match an existing Circular account. Please try again.</t>
   </si>
   <si>
+    <t>forgot_password.reset.email.title</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.code.description</t>
+  </si>
+  <si>
+    <t>Enter the 6-digit code that we sent to &lt;strong&gt;{email}&lt;/strong&gt;.</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.code.resend_button</t>
+  </si>
+  <si>
+    <t>Resend Code</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.code.error</t>
+  </si>
+  <si>
+    <t>Password incorrect, please try again.</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.code.resend_description</t>
+  </si>
+  <si>
+    <t>We have just sent you another code. Enter the &lt;strong&gt;latest&lt;/strong&gt; one that you received. It might take a couple of minutes. Don’t forget to check your spam folder.</t>
+  </si>
+  <si>
+    <t>forgot_password.new.description</t>
+  </si>
+  <si>
+    <t>Perfect! You can now set up your new password and sign back in.</t>
+  </si>
+  <si>
+    <t>forgot_password.new.password.placeholder</t>
+  </si>
+  <si>
+    <t>forgot_password.new.password</t>
+  </si>
+  <si>
+    <t>forgot_password.new.confirm_password.placeholder</t>
+  </si>
+  <si>
+    <t>forgot_password.new.confirm_password</t>
+  </si>
+  <si>
+    <t>Confim password</t>
+  </si>
+  <si>
+    <t>forgot_password.new.button</t>
+  </si>
+  <si>
+    <t>Save and Sign in</t>
+  </si>
+  <si>
+    <t>forgot_password.new.error</t>
+  </si>
+  <si>
     <t>global.back</t>
   </si>
   <si>
@@ -224,14 +305,35 @@
     <t>Next</t>
   </si>
   <si>
-    <t>forgot_password.reset.email.title</t>
+    <t>home.sync.syncing</t>
+  </si>
+  <si>
+    <t>Refreshing...</t>
+  </si>
+  <si>
+    <t>home.sync.error</t>
+  </si>
+  <si>
+    <t>Sync failed</t>
+  </si>
+  <si>
+    <t>home.sync.success</t>
+  </si>
+  <si>
+    <t>Sync success</t>
+  </si>
+  <si>
+    <t>home.sync.retry</t>
+  </si>
+  <si>
+    <t>Retry</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -249,6 +351,11 @@
     <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font/>
+    <font>
+      <color rgb="FF000000"/>
+      <name val="&quot;Arial&quot;"/>
     </font>
   </fonts>
   <fills count="5">
@@ -283,7 +390,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="18">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -313,6 +420,30 @@
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -983,7 +1114,7 @@
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>6</v>
@@ -991,11 +1122,11 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>6</v>
@@ -1003,11 +1134,11 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>6</v>
@@ -1015,11 +1146,11 @@
     </row>
     <row r="39">
       <c r="A39" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>6</v>
@@ -1027,129 +1158,240 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6"/>
+      <c r="A41" s="5" t="s">
+        <v>72</v>
+      </c>
       <c r="B41" s="6"/>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
+      <c r="C41" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="6"/>
-      <c r="B42" s="6"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
+      <c r="A42" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B42" s="11"/>
+      <c r="C42" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="6"/>
-      <c r="B43" s="6"/>
-      <c r="C43" s="6"/>
-      <c r="D43" s="6"/>
+      <c r="A43" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B43" s="11"/>
+      <c r="C43" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="6"/>
-      <c r="B44" s="6"/>
-      <c r="C44" s="6"/>
-      <c r="D44" s="6"/>
+      <c r="A44" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B44" s="11"/>
+      <c r="C44" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="6"/>
-      <c r="B45" s="6"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
+      <c r="A45" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="B45" s="11"/>
+      <c r="C45" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="6"/>
-      <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
+      <c r="A46" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B46" s="11"/>
+      <c r="C46" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="6"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6"/>
+      <c r="A47" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B47" s="11"/>
+      <c r="C47" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="6"/>
+      <c r="A48" s="13" t="s">
+        <v>85</v>
+      </c>
       <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
+      <c r="C48" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="6"/>
-      <c r="B49" s="6"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
+      <c r="A49" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B49" s="11"/>
+      <c r="C49" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="6"/>
+      <c r="A50" s="13" t="s">
+        <v>87</v>
+      </c>
       <c r="B50" s="6"/>
-      <c r="C50" s="6"/>
-      <c r="D50" s="6"/>
+      <c r="C50" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="6"/>
-      <c r="B51" s="6"/>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
+      <c r="A51" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="11"/>
+      <c r="C51" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="6"/>
-      <c r="B52" s="6"/>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
+      <c r="A52" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="11"/>
+      <c r="C52" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="6"/>
-      <c r="B53" s="6"/>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6"/>
+      <c r="A53" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D53" s="16" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="6"/>
-      <c r="B54" s="6"/>
-      <c r="C54" s="6"/>
-      <c r="D54" s="6"/>
+      <c r="A54" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="C54" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D54" s="16" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="6"/>
-      <c r="B55" s="6"/>
-      <c r="C55" s="6"/>
-      <c r="D55" s="6"/>
+      <c r="A55" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="C55" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="D55" s="16" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="6"/>
+      <c r="A56" s="5" t="s">
+        <v>97</v>
+      </c>
       <c r="B56" s="6"/>
-      <c r="C56" s="6"/>
-      <c r="D56" s="6"/>
+      <c r="C56" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="6"/>
+      <c r="A57" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="B57" s="6"/>
-      <c r="C57" s="6"/>
-      <c r="D57" s="6"/>
+      <c r="C57" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="6"/>
+      <c r="A58" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="B58" s="6"/>
-      <c r="C58" s="6"/>
-      <c r="D58" s="6"/>
+      <c r="C58" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="6"/>
+      <c r="A59" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="B59" s="6"/>
-      <c r="C59" s="6"/>
-      <c r="D59" s="6"/>
+      <c r="C59" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="6"/>
@@ -6839,9 +7081,51 @@
       <c r="C1007" s="6"/>
       <c r="D1007" s="6"/>
     </row>
+    <row r="1008">
+      <c r="A1008" s="6"/>
+      <c r="B1008" s="6"/>
+      <c r="C1008" s="6"/>
+      <c r="D1008" s="6"/>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="6"/>
+      <c r="B1009" s="6"/>
+      <c r="C1009" s="6"/>
+      <c r="D1009" s="6"/>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="6"/>
+      <c r="B1010" s="6"/>
+      <c r="C1010" s="6"/>
+      <c r="D1010" s="6"/>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="6"/>
+      <c r="B1011" s="6"/>
+      <c r="C1011" s="6"/>
+      <c r="D1011" s="6"/>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="6"/>
+      <c r="B1012" s="6"/>
+      <c r="C1012" s="6"/>
+      <c r="D1012" s="6"/>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="6"/>
+      <c r="B1013" s="6"/>
+      <c r="C1013" s="6"/>
+      <c r="D1013" s="6"/>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="6"/>
+      <c r="B1014" s="6"/>
+      <c r="C1014" s="6"/>
+      <c r="D1014" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D40">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D59">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Full registration flow (normal case)
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="182">
   <si>
     <t>Key</t>
   </si>
@@ -236,6 +236,24 @@
     <t>Resend Code</t>
   </si>
   <si>
+    <t>signup_success.title</t>
+  </si>
+  <si>
+    <t>All Set</t>
+  </si>
+  <si>
+    <t>signup_success.description</t>
+  </si>
+  <si>
+    <t>Now let’s set up your ring. You first need to wake it up by placing it on the charger for at least 15 minutes. Then, press start.</t>
+  </si>
+  <si>
+    <t>signup_success.start</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
     <t>forgot_password.question</t>
   </si>
   <si>
@@ -366,6 +384,18 @@
   </si>
   <si>
     <t>Retry</t>
+  </si>
+  <si>
+    <t>home.circles.title</t>
+  </si>
+  <si>
+    <t>My Circles</t>
+  </si>
+  <si>
+    <t>home.circles.activity.label</t>
+  </si>
+  <si>
+    <t>Activity analysis</t>
   </si>
   <si>
     <t>score.quality.poor</t>
@@ -548,7 +578,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -567,6 +597,7 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <color rgb="FF000000"/>
       <name val="&quot;Arial&quot;"/>
@@ -604,7 +635,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -636,12 +667,18 @@
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1380,11 +1417,11 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="10" t="s">
         <v>74</v>
       </c>
       <c r="B42" s="6"/>
-      <c r="C42" s="7" t="s">
+      <c r="C42" s="11" t="s">
         <v>75</v>
       </c>
       <c r="D42" s="5" t="s">
@@ -1392,11 +1429,11 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="10" t="s">
         <v>76</v>
       </c>
       <c r="B43" s="6"/>
-      <c r="C43" s="7" t="s">
+      <c r="C43" s="11" t="s">
         <v>77</v>
       </c>
       <c r="D43" s="5" t="s">
@@ -1404,11 +1441,11 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="10" t="s">
         <v>78</v>
       </c>
       <c r="B44" s="6"/>
-      <c r="C44" s="7" t="s">
+      <c r="C44" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D44" s="5" t="s">
@@ -1421,7 +1458,7 @@
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="7" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>6</v>
@@ -1429,11 +1466,11 @@
     </row>
     <row r="46">
       <c r="A46" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>6</v>
@@ -1441,11 +1478,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>22</v>
+        <v>85</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>6</v>
@@ -1453,11 +1490,11 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
-        <v>85</v>
+        <v>24</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>6</v>
@@ -1465,11 +1502,11 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>6</v>
@@ -1477,11 +1514,11 @@
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="7" t="s">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>6</v>
@@ -1489,11 +1526,11 @@
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>6</v>
@@ -1501,23 +1538,23 @@
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="7" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="10" t="s">
+      <c r="A53" s="5" t="s">
         <v>93</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
-        <v>24</v>
+        <v>94</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>6</v>
@@ -1525,35 +1562,35 @@
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
-        <v>26</v>
+        <v>96</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="10" t="s">
-        <v>95</v>
+      <c r="A55" s="5" t="s">
+        <v>97</v>
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="7" t="s">
-        <v>24</v>
+        <v>98</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="s">
-        <v>96</v>
+      <c r="A56" s="12" t="s">
+        <v>99</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="7" t="s">
-        <v>97</v>
+        <v>24</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>6</v>
@@ -1561,82 +1598,82 @@
     </row>
     <row r="57">
       <c r="A57" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
-        <v>99</v>
+        <v>26</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="C58" s="12" t="s">
+      <c r="A58" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="D58" s="11" t="s">
+      <c r="B58" s="6"/>
+      <c r="C58" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D58" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="s">
+      <c r="A59" s="5" t="s">
         <v>102</v>
       </c>
+      <c r="B59" s="6"/>
       <c r="C59" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="D59" s="11" t="s">
+      <c r="D59" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="11" t="s">
+      <c r="A60" s="5" t="s">
         <v>104</v>
       </c>
+      <c r="B60" s="6"/>
       <c r="C60" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D60" s="11" t="s">
+      <c r="D60" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="s">
+      <c r="A61" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B61" s="6"/>
-      <c r="C61" s="7" t="s">
+      <c r="C61" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="D61" s="5" t="s">
+      <c r="D61" s="13" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="5" t="s">
+      <c r="A62" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B62" s="6"/>
       <c r="C62" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="D62" s="5" t="s">
+      <c r="D62" s="13" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="s">
+      <c r="A63" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="B63" s="6"/>
       <c r="C63" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="D63" s="5" t="s">
+      <c r="D63" s="13" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1689,7 +1726,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="s">
+      <c r="A68" s="5" t="s">
         <v>120</v>
       </c>
       <c r="B68" s="6"/>
@@ -1701,7 +1738,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="8" t="s">
+      <c r="A69" s="5" t="s">
         <v>122</v>
       </c>
       <c r="B69" s="6"/>
@@ -1749,7 +1786,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="s">
+      <c r="A73" s="8" t="s">
         <v>130</v>
       </c>
       <c r="B73" s="6"/>
@@ -1761,7 +1798,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="s">
+      <c r="A74" s="8" t="s">
         <v>132</v>
       </c>
       <c r="B74" s="6"/>
@@ -2001,34 +2038,64 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="6"/>
+      <c r="A94" s="5" t="s">
+        <v>172</v>
+      </c>
       <c r="B94" s="6"/>
-      <c r="C94" s="6"/>
-      <c r="D94" s="6"/>
+      <c r="C94" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="D94" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="6"/>
+      <c r="A95" s="5" t="s">
+        <v>174</v>
+      </c>
       <c r="B95" s="6"/>
-      <c r="C95" s="6"/>
-      <c r="D95" s="6"/>
+      <c r="C95" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="D95" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="6"/>
+      <c r="A96" s="5" t="s">
+        <v>176</v>
+      </c>
       <c r="B96" s="6"/>
-      <c r="C96" s="6"/>
-      <c r="D96" s="6"/>
+      <c r="C96" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="6"/>
+      <c r="A97" s="5" t="s">
+        <v>178</v>
+      </c>
       <c r="B97" s="6"/>
-      <c r="C97" s="6"/>
-      <c r="D97" s="6"/>
+      <c r="C97" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D97" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="6"/>
+      <c r="A98" s="5" t="s">
+        <v>180</v>
+      </c>
       <c r="B98" s="6"/>
-      <c r="C98" s="6"/>
-      <c r="D98" s="6"/>
+      <c r="C98" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="6"/>
@@ -7640,9 +7707,39 @@
       <c r="C1033" s="6"/>
       <c r="D1033" s="6"/>
     </row>
+    <row r="1034">
+      <c r="A1034" s="6"/>
+      <c r="B1034" s="6"/>
+      <c r="C1034" s="6"/>
+      <c r="D1034" s="6"/>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="6"/>
+      <c r="B1035" s="6"/>
+      <c r="C1035" s="6"/>
+      <c r="D1035" s="6"/>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="6"/>
+      <c r="B1036" s="6"/>
+      <c r="C1036" s="6"/>
+      <c r="D1036" s="6"/>
+    </row>
+    <row r="1037">
+      <c r="A1037" s="6"/>
+      <c r="B1037" s="6"/>
+      <c r="C1037" s="6"/>
+      <c r="D1037" s="6"/>
+    </row>
+    <row r="1038">
+      <c r="A1038" s="6"/>
+      <c r="B1038" s="6"/>
+      <c r="C1038" s="6"/>
+      <c r="D1038" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D93">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D98">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
WIP forgot password add error message
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="183">
   <si>
     <t>Key</t>
   </si>
@@ -103,17 +103,23 @@
     <t>Confirm</t>
   </si>
   <si>
+    <t>login.signup_button</t>
+  </si>
+  <si>
+    <t>Sign up</t>
+  </si>
+  <si>
     <t>login.error.invalid_credentials</t>
   </si>
   <si>
-    <t>The email or password is invalid</t>
+    <t>The email or password is invalid.</t>
   </si>
   <si>
     <t>login.error.default</t>
   </si>
   <si>
     <t>An error occurred.
-Please try again later</t>
+Please try again later.</t>
   </si>
   <si>
     <t>header.my_ring</t>
@@ -140,9 +146,6 @@
     <t>signin_signup.signup</t>
   </si>
   <si>
-    <t>Sign up</t>
-  </si>
-  <si>
     <t>signup.title</t>
   </si>
   <si>
@@ -194,25 +197,25 @@
     <t>signup.error.empty_field</t>
   </si>
   <si>
-    <t>Some fields are empty</t>
+    <t>Some fields are empty.</t>
   </si>
   <si>
     <t>signup.error.email_format</t>
   </si>
   <si>
-    <t>Email is not correct</t>
+    <t>Email is not correct.</t>
   </si>
   <si>
     <t>signup.error.password_format</t>
   </si>
   <si>
-    <t>Password must be at least 4 characters, 1 lowercase, 1 uppercase and 1 digit</t>
+    <t>Password must be at least 8 characters, 1 lowercase, 1 uppercase, 1 digit and 1 special character.</t>
   </si>
   <si>
     <t>signup.error.password_confirm</t>
   </si>
   <si>
-    <t>Password fields are not identical</t>
+    <t>Password fields are not identical.</t>
   </si>
   <si>
     <t>signup.error.default</t>
@@ -236,6 +239,24 @@
     <t>Resend Code</t>
   </si>
   <si>
+    <t>signup_success.title</t>
+  </si>
+  <si>
+    <t>All Set</t>
+  </si>
+  <si>
+    <t>signup_success.description</t>
+  </si>
+  <si>
+    <t>Now let’s set up your ring. You first need to wake it up by placing it on the charger for at least 15 minutes. Then, press start.</t>
+  </si>
+  <si>
+    <t>signup_success.start</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
     <t>forgot_password.question</t>
   </si>
   <si>
@@ -293,15 +314,9 @@
     <t>Perfect! You can now set up your new password and sign back in.</t>
   </si>
   <si>
-    <t>forgot_password.new.password.placeholder</t>
-  </si>
-  <si>
     <t>forgot_password.new.password</t>
   </si>
   <si>
-    <t>forgot_password.new.confirm_password.placeholder</t>
-  </si>
-  <si>
     <t>forgot_password.new.confirm_password</t>
   </si>
   <si>
@@ -314,12 +329,6 @@
     <t>Save and Sign in</t>
   </si>
   <si>
-    <t>forgot_password.new.error</t>
-  </si>
-  <si>
-    <t>Password must be at least 8 characters, 1 lowercase, 1 uppercase, 1 digit and 1 special character</t>
-  </si>
-  <si>
     <t>global.back</t>
   </si>
   <si>
@@ -366,6 +375,18 @@
   </si>
   <si>
     <t>Retry</t>
+  </si>
+  <si>
+    <t>home.circles.title</t>
+  </si>
+  <si>
+    <t>My Circles</t>
+  </si>
+  <si>
+    <t>home.circles.activity.label</t>
+  </si>
+  <si>
+    <t>Activity analysis</t>
   </si>
   <si>
     <t>score.quality.poor</t>
@@ -542,6 +563,18 @@
   </si>
   <si>
     <t>HR max (bpm)</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.token.error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verification code incorrect, please try again </t>
+  </si>
+  <si>
+    <t>forgot_password.reset.password.placeholder</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.confirm_password.placeholder</t>
   </si>
 </sst>
 </file>
@@ -567,10 +600,7 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <color rgb="FF000000"/>
-      <name val="&quot;Arial&quot;"/>
-    </font>
+    <font/>
   </fonts>
   <fills count="5">
     <fill>
@@ -635,11 +665,11 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
@@ -1121,31 +1151,31 @@
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>41</v>
+      <c r="A21" s="5" t="s">
+        <v>42</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="7" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="8" t="s">
         <v>43</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>6</v>
@@ -1157,7 +1187,7 @@
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="7" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>6</v>
@@ -1165,11 +1195,11 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="7" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>6</v>
@@ -1181,7 +1211,7 @@
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>6</v>
@@ -1193,7 +1223,7 @@
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>6</v>
@@ -1205,7 +1235,7 @@
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>6</v>
@@ -1217,7 +1247,7 @@
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>6</v>
@@ -1225,11 +1255,11 @@
     </row>
     <row r="29">
       <c r="A29" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="7" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>6</v>
@@ -1241,7 +1271,7 @@
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>6</v>
@@ -1253,7 +1283,7 @@
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>6</v>
@@ -1265,7 +1295,7 @@
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="7" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>6</v>
@@ -1273,11 +1303,11 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>6</v>
@@ -1285,11 +1315,11 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>6</v>
@@ -1297,11 +1327,11 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>6</v>
@@ -1309,11 +1339,11 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>6</v>
@@ -1321,11 +1351,11 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>6</v>
@@ -1333,11 +1363,11 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>6</v>
@@ -1349,7 +1379,7 @@
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="7" t="s">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>6</v>
@@ -1357,11 +1387,11 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>6</v>
@@ -1369,11 +1399,11 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>6</v>
@@ -1381,11 +1411,11 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>6</v>
@@ -1393,11 +1423,11 @@
     </row>
     <row r="43">
       <c r="A43" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>6</v>
@@ -1405,11 +1435,11 @@
     </row>
     <row r="44">
       <c r="A44" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>6</v>
@@ -1417,11 +1447,11 @@
     </row>
     <row r="45">
       <c r="A45" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="7" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>6</v>
@@ -1445,7 +1475,7 @@
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>22</v>
+        <v>84</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>6</v>
@@ -1453,11 +1483,11 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>6</v>
@@ -1465,11 +1495,11 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
-        <v>73</v>
+        <v>24</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>6</v>
@@ -1477,11 +1507,11 @@
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>6</v>
@@ -1489,11 +1519,11 @@
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="7" t="s">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>6</v>
@@ -1512,12 +1542,12 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="10" t="s">
+      <c r="A53" s="5" t="s">
         <v>93</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
-        <v>24</v>
+        <v>74</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>6</v>
@@ -1529,19 +1559,19 @@
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
-        <v>26</v>
+        <v>95</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="10" t="s">
-        <v>95</v>
+      <c r="A55" s="5" t="s">
+        <v>96</v>
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="7" t="s">
-        <v>24</v>
+        <v>97</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>6</v>
@@ -1549,11 +1579,11 @@
     </row>
     <row r="56">
       <c r="A56" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>6</v>
@@ -1561,68 +1591,69 @@
     </row>
     <row r="57">
       <c r="A57" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
-        <v>99</v>
+        <v>26</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="C58" s="12" t="s">
+      <c r="A58" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="D58" s="11" t="s">
+      <c r="B58" s="6"/>
+      <c r="C58" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D58" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="s">
-        <v>102</v>
-      </c>
+      <c r="A59" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="6"/>
       <c r="C59" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="D59" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="D59" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="11" t="s">
-        <v>104</v>
+      <c r="A60" s="10" t="s">
+        <v>105</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="D60" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="D60" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="B61" s="6"/>
+      <c r="A61" s="10" t="s">
+        <v>107</v>
+      </c>
       <c r="C61" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="D61" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D61" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B62" s="6"/>
       <c r="C62" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>6</v>
@@ -1630,11 +1661,11 @@
     </row>
     <row r="63">
       <c r="A63" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>6</v>
@@ -1642,11 +1673,11 @@
     </row>
     <row r="64">
       <c r="A64" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>6</v>
@@ -1654,11 +1685,11 @@
     </row>
     <row r="65">
       <c r="A65" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B65" s="6"/>
       <c r="C65" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>6</v>
@@ -1666,11 +1697,11 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B66" s="6"/>
       <c r="C66" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>6</v>
@@ -1678,35 +1709,35 @@
     </row>
     <row r="67">
       <c r="A67" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B67" s="6"/>
       <c r="C67" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="s">
-        <v>120</v>
+      <c r="A68" s="5" t="s">
+        <v>121</v>
       </c>
       <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="8" t="s">
-        <v>122</v>
+      <c r="A69" s="5" t="s">
+        <v>123</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>6</v>
@@ -1714,35 +1745,35 @@
     </row>
     <row r="70">
       <c r="A70" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B70" s="6"/>
       <c r="C70" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D70" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="s">
-        <v>126</v>
+      <c r="A71" s="8" t="s">
+        <v>127</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D71" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="5" t="s">
-        <v>128</v>
+      <c r="A72" s="8" t="s">
+        <v>129</v>
       </c>
       <c r="B72" s="6"/>
       <c r="C72" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>6</v>
@@ -1750,11 +1781,11 @@
     </row>
     <row r="73">
       <c r="A73" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B73" s="6"/>
       <c r="C73" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>6</v>
@@ -1762,11 +1793,11 @@
     </row>
     <row r="74">
       <c r="A74" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B74" s="6"/>
       <c r="C74" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D74" s="5" t="s">
         <v>6</v>
@@ -1774,11 +1805,11 @@
     </row>
     <row r="75">
       <c r="A75" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B75" s="6"/>
       <c r="C75" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D75" s="5" t="s">
         <v>6</v>
@@ -1786,11 +1817,11 @@
     </row>
     <row r="76">
       <c r="A76" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B76" s="6"/>
       <c r="C76" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D76" s="5" t="s">
         <v>6</v>
@@ -1798,11 +1829,11 @@
     </row>
     <row r="77">
       <c r="A77" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B77" s="6"/>
       <c r="C77" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D77" s="5" t="s">
         <v>6</v>
@@ -1810,11 +1841,11 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B78" s="6"/>
       <c r="C78" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D78" s="5" t="s">
         <v>6</v>
@@ -1822,11 +1853,11 @@
     </row>
     <row r="79">
       <c r="A79" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B79" s="6"/>
       <c r="C79" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D79" s="5" t="s">
         <v>6</v>
@@ -1834,11 +1865,11 @@
     </row>
     <row r="80">
       <c r="A80" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B80" s="6"/>
       <c r="C80" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D80" s="5" t="s">
         <v>6</v>
@@ -1846,11 +1877,11 @@
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B81" s="6"/>
       <c r="C81" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>6</v>
@@ -1858,11 +1889,11 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B82" s="6"/>
       <c r="C82" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>6</v>
@@ -1870,11 +1901,11 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B83" s="6"/>
       <c r="C83" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>6</v>
@@ -1882,11 +1913,11 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B84" s="6"/>
       <c r="C84" s="7" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>6</v>
@@ -1894,11 +1925,11 @@
     </row>
     <row r="85">
       <c r="A85" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B85" s="6"/>
       <c r="C85" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>6</v>
@@ -1906,11 +1937,11 @@
     </row>
     <row r="86">
       <c r="A86" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B86" s="6"/>
       <c r="C86" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>6</v>
@@ -1918,11 +1949,11 @@
     </row>
     <row r="87">
       <c r="A87" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B87" s="6"/>
       <c r="C87" s="7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D87" s="5" t="s">
         <v>6</v>
@@ -1930,11 +1961,11 @@
     </row>
     <row r="88">
       <c r="A88" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B88" s="6"/>
       <c r="C88" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>6</v>
@@ -1942,11 +1973,11 @@
     </row>
     <row r="89">
       <c r="A89" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B89" s="6"/>
       <c r="C89" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D89" s="5" t="s">
         <v>6</v>
@@ -1954,11 +1985,11 @@
     </row>
     <row r="90">
       <c r="A90" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B90" s="6"/>
       <c r="C90" s="7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D90" s="5" t="s">
         <v>6</v>
@@ -1966,11 +1997,11 @@
     </row>
     <row r="91">
       <c r="A91" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B91" s="6"/>
       <c r="C91" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D91" s="5" t="s">
         <v>6</v>
@@ -1978,11 +2009,11 @@
     </row>
     <row r="92">
       <c r="A92" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B92" s="6"/>
       <c r="C92" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D92" s="5" t="s">
         <v>6</v>
@@ -1990,51 +2021,87 @@
     </row>
     <row r="93">
       <c r="A93" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B93" s="6"/>
       <c r="C93" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="6"/>
+      <c r="A94" s="5" t="s">
+        <v>173</v>
+      </c>
       <c r="B94" s="6"/>
-      <c r="C94" s="6"/>
-      <c r="D94" s="6"/>
+      <c r="C94" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="D94" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="6"/>
+      <c r="A95" s="5" t="s">
+        <v>175</v>
+      </c>
       <c r="B95" s="6"/>
-      <c r="C95" s="6"/>
-      <c r="D95" s="6"/>
+      <c r="C95" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="D95" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="6"/>
+      <c r="A96" s="5" t="s">
+        <v>177</v>
+      </c>
       <c r="B96" s="6"/>
-      <c r="C96" s="6"/>
-      <c r="D96" s="6"/>
+      <c r="C96" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="6"/>
+      <c r="A97" s="11" t="s">
+        <v>179</v>
+      </c>
       <c r="B97" s="6"/>
-      <c r="C97" s="6"/>
-      <c r="D97" s="6"/>
+      <c r="C97" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D97" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="6"/>
+      <c r="A98" s="11" t="s">
+        <v>181</v>
+      </c>
       <c r="B98" s="6"/>
-      <c r="C98" s="6"/>
-      <c r="D98" s="6"/>
+      <c r="C98" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="6"/>
+      <c r="A99" s="11" t="s">
+        <v>182</v>
+      </c>
       <c r="B99" s="6"/>
-      <c r="C99" s="6"/>
-      <c r="D99" s="6"/>
+      <c r="C99" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D99" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="6"/>
@@ -7640,9 +7707,27 @@
       <c r="C1033" s="6"/>
       <c r="D1033" s="6"/>
     </row>
+    <row r="1034">
+      <c r="A1034" s="6"/>
+      <c r="B1034" s="6"/>
+      <c r="C1034" s="6"/>
+      <c r="D1034" s="6"/>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="6"/>
+      <c r="B1035" s="6"/>
+      <c r="C1035" s="6"/>
+      <c r="D1035" s="6"/>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="6"/>
+      <c r="B1036" s="6"/>
+      <c r="C1036" s="6"/>
+      <c r="D1036" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D93">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D99">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Modify button layout in signup confirmation code screen
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="185">
   <si>
     <t>Key</t>
   </si>
@@ -237,6 +237,12 @@
   </si>
   <si>
     <t>Resend Code</t>
+  </si>
+  <si>
+    <t>signup_code.validate_button</t>
+  </si>
+  <si>
+    <t>Validate</t>
   </si>
   <si>
     <t>signup_success.title</t>
@@ -563,13 +569,25 @@
   </si>
   <si>
     <t>HR max (bpm)</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.token.error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verification code incorrect, please try again </t>
+  </si>
+  <si>
+    <t>forgot_password.reset.password.placeholder</t>
+  </si>
+  <si>
+    <t>forgot_password.reset.confirm_password.placeholder</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -588,6 +606,7 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font/>
   </fonts>
   <fills count="5">
     <fill>
@@ -621,7 +640,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -651,6 +670,12 @@
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -1403,11 +1428,11 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="10" t="s">
         <v>75</v>
       </c>
       <c r="B43" s="6"/>
-      <c r="C43" s="7" t="s">
+      <c r="C43" s="11" t="s">
         <v>76</v>
       </c>
       <c r="D43" s="5" t="s">
@@ -1480,7 +1505,7 @@
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>6</v>
@@ -1488,11 +1513,11 @@
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="7" t="s">
-        <v>89</v>
+        <v>24</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>6</v>
@@ -1504,7 +1529,7 @@
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="7" t="s">
-        <v>22</v>
+        <v>91</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>6</v>
@@ -1512,11 +1537,11 @@
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="7" t="s">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>6</v>
@@ -1528,7 +1553,7 @@
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>6</v>
@@ -1536,11 +1561,11 @@
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>6</v>
@@ -1576,7 +1601,7 @@
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
-        <v>26</v>
+        <v>101</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>6</v>
@@ -1584,11 +1609,11 @@
     </row>
     <row r="58">
       <c r="A58" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="s">
-        <v>102</v>
+        <v>26</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -1607,36 +1632,36 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="10" t="s">
+      <c r="A60" s="5" t="s">
         <v>105</v>
       </c>
+      <c r="B60" s="6"/>
       <c r="C60" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D60" s="10" t="s">
+      <c r="D60" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="10" t="s">
+      <c r="A61" s="12" t="s">
         <v>107</v>
       </c>
       <c r="C61" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="D61" s="10" t="s">
+      <c r="D61" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="5" t="s">
+      <c r="A62" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="B62" s="6"/>
       <c r="C62" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D62" s="5" t="s">
+      <c r="D62" s="12" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1737,7 +1762,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="8" t="s">
+      <c r="A71" s="5" t="s">
         <v>127</v>
       </c>
       <c r="B71" s="6"/>
@@ -1761,7 +1786,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="s">
+      <c r="A73" s="8" t="s">
         <v>131</v>
       </c>
       <c r="B73" s="6"/>
@@ -2049,28 +2074,52 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="5"/>
+      <c r="A97" s="5" t="s">
+        <v>179</v>
+      </c>
       <c r="B97" s="6"/>
-      <c r="C97" s="7"/>
-      <c r="D97" s="5"/>
+      <c r="C97" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D97" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="6"/>
+      <c r="A98" s="5" t="s">
+        <v>181</v>
+      </c>
       <c r="B98" s="6"/>
-      <c r="C98" s="6"/>
-      <c r="D98" s="6"/>
+      <c r="C98" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="6"/>
+      <c r="A99" s="5" t="s">
+        <v>183</v>
+      </c>
       <c r="B99" s="6"/>
-      <c r="C99" s="6"/>
-      <c r="D99" s="6"/>
+      <c r="C99" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D99" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="6"/>
+      <c r="A100" s="5" t="s">
+        <v>184</v>
+      </c>
       <c r="B100" s="6"/>
-      <c r="C100" s="6"/>
-      <c r="D100" s="6"/>
+      <c r="C100" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="6"/>
@@ -7688,9 +7737,15 @@
       <c r="C1036" s="6"/>
       <c r="D1036" s="6"/>
     </row>
+    <row r="1037">
+      <c r="A1037" s="6"/>
+      <c r="B1037" s="6"/>
+      <c r="C1037" s="6"/>
+      <c r="D1037" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D97">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D100">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Drawer navigation + Profile screen base
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="215">
   <si>
     <t>Key</t>
   </si>
@@ -393,6 +393,12 @@
   </si>
   <si>
     <t>Activity analysis</t>
+  </si>
+  <si>
+    <t>home.circles.live.label</t>
+  </si>
+  <si>
+    <t>Live</t>
   </si>
   <si>
     <t>score.quality.poor</t>
@@ -581,13 +587,97 @@
   </si>
   <si>
     <t>forgot_password.reset.confirm_password.placeholder</t>
+  </si>
+  <si>
+    <t>profile.header.title</t>
+  </si>
+  <si>
+    <t>PROFILE</t>
+  </si>
+  <si>
+    <t>profile.logout</t>
+  </si>
+  <si>
+    <t>Log out</t>
+  </si>
+  <si>
+    <t>header.live</t>
+  </si>
+  <si>
+    <t>LIVE</t>
+  </si>
+  <si>
+    <t>live.heart_rate.label</t>
+  </si>
+  <si>
+    <t>Heart rate</t>
+  </si>
+  <si>
+    <t>live.accuracy.label</t>
+  </si>
+  <si>
+    <t>Data Accuracy:</t>
+  </si>
+  <si>
+    <t>live.intensity.label</t>
+  </si>
+  <si>
+    <t>Activity Intensity</t>
+  </si>
+  <si>
+    <t>live.hr_max.label</t>
+  </si>
+  <si>
+    <t>HR Max.</t>
+  </si>
+  <si>
+    <t>live.hr_max.ratio.label</t>
+  </si>
+  <si>
+    <t>% of Max HR</t>
+  </si>
+  <si>
+    <t>live.start</t>
+  </si>
+  <si>
+    <t>START</t>
+  </si>
+  <si>
+    <t>live.hrv_blood_ox.label</t>
+  </si>
+  <si>
+    <t>HRV &amp; Blood Ox.</t>
+  </si>
+  <si>
+    <t>live.hrv.label</t>
+  </si>
+  <si>
+    <t>HRV</t>
+  </si>
+  <si>
+    <t>live.blood_ox.label</t>
+  </si>
+  <si>
+    <t>Blood Ox.</t>
+  </si>
+  <si>
+    <t>drawer.profile</t>
+  </si>
+  <si>
+    <t>Profile</t>
+  </si>
+  <si>
+    <t>drawer.close</t>
+  </si>
+  <si>
+    <t>Close</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -606,6 +696,7 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font/>
   </fonts>
   <fills count="5">
     <fill>
@@ -639,7 +730,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -672,6 +763,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1767,7 +1864,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="s">
+      <c r="A72" s="5" t="s">
         <v>129</v>
       </c>
       <c r="B72" s="6"/>
@@ -1791,7 +1888,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="s">
+      <c r="A74" s="8" t="s">
         <v>133</v>
       </c>
       <c r="B74" s="6"/>
@@ -2096,7 +2193,7 @@
       </c>
       <c r="B99" s="6"/>
       <c r="C99" s="7" t="s">
-        <v>24</v>
+        <v>184</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>6</v>
@@ -2104,7 +2201,7 @@
     </row>
     <row r="100">
       <c r="A100" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7" t="s">
@@ -2115,94 +2212,184 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="6"/>
+      <c r="A101" s="5" t="s">
+        <v>186</v>
+      </c>
       <c r="B101" s="6"/>
-      <c r="C101" s="6"/>
-      <c r="D101" s="6"/>
+      <c r="C101" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D101" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="6"/>
+      <c r="A102" s="11" t="s">
+        <v>187</v>
+      </c>
       <c r="B102" s="6"/>
-      <c r="C102" s="6"/>
-      <c r="D102" s="6"/>
+      <c r="C102" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="6"/>
+      <c r="A103" s="11" t="s">
+        <v>189</v>
+      </c>
       <c r="B103" s="6"/>
-      <c r="C103" s="6"/>
-      <c r="D103" s="6"/>
+      <c r="C103" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="D103" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="6"/>
+      <c r="A104" s="5" t="s">
+        <v>191</v>
+      </c>
       <c r="B104" s="6"/>
-      <c r="C104" s="6"/>
-      <c r="D104" s="6"/>
+      <c r="C104" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="D104" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" s="6"/>
+      <c r="A105" s="5" t="s">
+        <v>193</v>
+      </c>
       <c r="B105" s="6"/>
-      <c r="C105" s="6"/>
-      <c r="D105" s="6"/>
+      <c r="C105" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="D105" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="6"/>
+      <c r="A106" s="5" t="s">
+        <v>195</v>
+      </c>
       <c r="B106" s="6"/>
-      <c r="C106" s="6"/>
-      <c r="D106" s="6"/>
+      <c r="C106" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D106" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="6"/>
+      <c r="A107" s="5" t="s">
+        <v>197</v>
+      </c>
       <c r="B107" s="6"/>
-      <c r="C107" s="6"/>
-      <c r="D107" s="6"/>
+      <c r="C107" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="D107" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="6"/>
+      <c r="A108" s="5" t="s">
+        <v>199</v>
+      </c>
       <c r="B108" s="6"/>
-      <c r="C108" s="6"/>
-      <c r="D108" s="6"/>
+      <c r="C108" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="6"/>
+      <c r="A109" s="5" t="s">
+        <v>201</v>
+      </c>
       <c r="B109" s="6"/>
-      <c r="C109" s="6"/>
-      <c r="D109" s="6"/>
+      <c r="C109" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="6"/>
+      <c r="A110" s="5" t="s">
+        <v>203</v>
+      </c>
       <c r="B110" s="6"/>
-      <c r="C110" s="6"/>
-      <c r="D110" s="6"/>
+      <c r="C110" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="6"/>
+      <c r="A111" s="5" t="s">
+        <v>205</v>
+      </c>
       <c r="B111" s="6"/>
-      <c r="C111" s="6"/>
-      <c r="D111" s="6"/>
+      <c r="C111" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="112">
-      <c r="A112" s="6"/>
+      <c r="A112" s="5" t="s">
+        <v>207</v>
+      </c>
       <c r="B112" s="6"/>
-      <c r="C112" s="6"/>
-      <c r="D112" s="6"/>
+      <c r="C112" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="D112" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="113">
-      <c r="A113" s="6"/>
+      <c r="A113" s="5" t="s">
+        <v>209</v>
+      </c>
       <c r="B113" s="6"/>
-      <c r="C113" s="6"/>
-      <c r="D113" s="6"/>
+      <c r="C113" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="D113" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="114">
-      <c r="A114" s="6"/>
+      <c r="A114" s="11" t="s">
+        <v>211</v>
+      </c>
       <c r="B114" s="6"/>
-      <c r="C114" s="6"/>
-      <c r="D114" s="6"/>
+      <c r="C114" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="115">
-      <c r="A115" s="6"/>
+      <c r="A115" s="11" t="s">
+        <v>213</v>
+      </c>
       <c r="B115" s="6"/>
-      <c r="C115" s="6"/>
-      <c r="D115" s="6"/>
+      <c r="C115" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="6"/>
@@ -7736,9 +7923,21 @@
       <c r="C1037" s="6"/>
       <c r="D1037" s="6"/>
     </row>
+    <row r="1038">
+      <c r="A1038" s="6"/>
+      <c r="B1038" s="6"/>
+      <c r="C1038" s="6"/>
+      <c r="D1038" s="6"/>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="6"/>
+      <c r="B1039" s="6"/>
+      <c r="C1039" s="6"/>
+      <c r="D1039" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D100">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D115">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Onboarding ring wearing info
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="233">
   <si>
     <t>Key</t>
   </si>
@@ -272,7 +272,7 @@
     <t>forgot_password.reset.title</t>
   </si>
   <si>
-    <t>Pasword Reset</t>
+    <t>Password Reset</t>
   </si>
   <si>
     <t>forgot_password.reset.description</t>
@@ -399,6 +399,18 @@
   </si>
   <si>
     <t>Live</t>
+  </si>
+  <si>
+    <t>home.circles.alarm.label</t>
+  </si>
+  <si>
+    <t>Alarm clock</t>
+  </si>
+  <si>
+    <t>header.alarm</t>
+  </si>
+  <si>
+    <t>ALARM CLOCK</t>
   </si>
   <si>
     <t>score.quality.poor</t>
@@ -671,13 +683,67 @@
   </si>
   <si>
     <t>Close</t>
+  </si>
+  <si>
+    <t>alarm.score.programmed</t>
+  </si>
+  <si>
+    <t>Programmed alarms</t>
+  </si>
+  <si>
+    <t>alarm.score.week</t>
+  </si>
+  <si>
+    <t>Week overview</t>
+  </si>
+  <si>
+    <t>alarm.score.add_button</t>
+  </si>
+  <si>
+    <t>Add an alarm</t>
+  </si>
+  <si>
+    <t>onboarding.wear.title</t>
+  </si>
+  <si>
+    <t>How to wear Circular</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>onboarding.wear.info</t>
+    </r>
+    <r>
+      <rPr/>
+      <t>.top</t>
+    </r>
+  </si>
+  <si>
+    <t>The best fingers to wear Circular are the &lt;colored&gt;index&lt;/colored&gt;, &lt;colored&gt;middle finger&lt;/colored&gt;, &lt;colored&gt;ring finger&lt;/colored&gt;, pinky finger and thumb.
+Try as much as possible to use the same finger and same ring positioning each time you wear your Circular.</t>
+  </si>
+  <si>
+    <t>onboarding.wear.info.bottom</t>
+  </si>
+  <si>
+    <t>The flat part of the ring should be on the &lt;colored&gt;palmar side&lt;/colored&gt; of your finger.
+The button should be &lt;colored&gt;facing your thumb&lt;/colored&gt;, for ease of use.</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.title</t>
+  </si>
+  <si>
+    <t>Tell us more about yourself</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -697,6 +763,10 @@
       <name val="Arial"/>
     </font>
     <font/>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -730,7 +800,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -761,14 +831,20 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1582,7 +1658,7 @@
         <v>85</v>
       </c>
       <c r="B48" s="6"/>
-      <c r="C48" s="7" t="s">
+      <c r="C48" s="10" t="s">
         <v>86</v>
       </c>
       <c r="D48" s="5" t="s">
@@ -1734,24 +1810,24 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="10" t="s">
+      <c r="A61" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C61" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="D61" s="10" t="s">
+      <c r="D61" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="10" t="s">
+      <c r="A62" s="11" t="s">
         <v>109</v>
       </c>
       <c r="C62" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D62" s="10" t="s">
+      <c r="D62" s="11" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1876,7 +1952,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="s">
+      <c r="A73" s="5" t="s">
         <v>131</v>
       </c>
       <c r="B73" s="6"/>
@@ -1888,7 +1964,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="s">
+      <c r="A74" s="5" t="s">
         <v>133</v>
       </c>
       <c r="B74" s="6"/>
@@ -1900,7 +1976,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="s">
+      <c r="A75" s="8" t="s">
         <v>135</v>
       </c>
       <c r="B75" s="6"/>
@@ -1912,7 +1988,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="5" t="s">
+      <c r="A76" s="8" t="s">
         <v>137</v>
       </c>
       <c r="B76" s="6"/>
@@ -2205,7 +2281,7 @@
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7" t="s">
-        <v>24</v>
+        <v>186</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>6</v>
@@ -2213,35 +2289,35 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B101" s="6"/>
       <c r="C101" s="7" t="s">
-        <v>24</v>
+        <v>188</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="11" t="s">
-        <v>187</v>
+      <c r="A102" s="5" t="s">
+        <v>189</v>
       </c>
       <c r="B102" s="6"/>
       <c r="C102" s="7" t="s">
-        <v>188</v>
+        <v>24</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="11" t="s">
-        <v>189</v>
+      <c r="A103" s="5" t="s">
+        <v>190</v>
       </c>
       <c r="B103" s="6"/>
-      <c r="C103" s="12" t="s">
-        <v>190</v>
+      <c r="C103" s="7" t="s">
+        <v>24</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>6</v>
@@ -2368,11 +2444,11 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="11" t="s">
+      <c r="A114" s="5" t="s">
         <v>211</v>
       </c>
       <c r="B114" s="6"/>
-      <c r="C114" s="12" t="s">
+      <c r="C114" s="7" t="s">
         <v>212</v>
       </c>
       <c r="D114" s="5" t="s">
@@ -2380,11 +2456,11 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="11" t="s">
+      <c r="A115" s="5" t="s">
         <v>213</v>
       </c>
       <c r="B115" s="6"/>
-      <c r="C115" s="12" t="s">
+      <c r="C115" s="7" t="s">
         <v>214</v>
       </c>
       <c r="D115" s="5" t="s">
@@ -2392,58 +2468,112 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="6"/>
+      <c r="A116" s="5" t="s">
+        <v>215</v>
+      </c>
       <c r="B116" s="6"/>
-      <c r="C116" s="6"/>
-      <c r="D116" s="6"/>
+      <c r="C116" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="D116" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="117">
-      <c r="A117" s="6"/>
+      <c r="A117" s="5" t="s">
+        <v>217</v>
+      </c>
       <c r="B117" s="6"/>
-      <c r="C117" s="6"/>
-      <c r="D117" s="6"/>
+      <c r="C117" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="D117" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" s="6"/>
+      <c r="A118" s="5" t="s">
+        <v>219</v>
+      </c>
       <c r="B118" s="6"/>
-      <c r="C118" s="6"/>
-      <c r="D118" s="6"/>
+      <c r="C118" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="119">
-      <c r="A119" s="6"/>
+      <c r="A119" s="5" t="s">
+        <v>221</v>
+      </c>
       <c r="B119" s="6"/>
-      <c r="C119" s="6"/>
-      <c r="D119" s="6"/>
+      <c r="C119" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="120">
-      <c r="A120" s="6"/>
+      <c r="A120" s="5" t="s">
+        <v>223</v>
+      </c>
       <c r="B120" s="6"/>
-      <c r="C120" s="6"/>
-      <c r="D120" s="6"/>
+      <c r="C120" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="121">
-      <c r="A121" s="6"/>
+      <c r="A121" s="12" t="s">
+        <v>225</v>
+      </c>
       <c r="B121" s="6"/>
-      <c r="C121" s="6"/>
-      <c r="D121" s="6"/>
+      <c r="C121" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="122">
-      <c r="A122" s="6"/>
-      <c r="B122" s="6"/>
-      <c r="C122" s="6"/>
-      <c r="D122" s="6"/>
+      <c r="A122" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="B122" s="14"/>
+      <c r="C122" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="123">
-      <c r="A123" s="6"/>
+      <c r="A123" s="12" t="s">
+        <v>229</v>
+      </c>
       <c r="B123" s="6"/>
-      <c r="C123" s="6"/>
-      <c r="D123" s="6"/>
+      <c r="C123" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="124">
-      <c r="A124" s="6"/>
+      <c r="A124" s="12" t="s">
+        <v>231</v>
+      </c>
       <c r="B124" s="6"/>
-      <c r="C124" s="6"/>
-      <c r="D124" s="6"/>
+      <c r="C124" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="D124" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="6"/>
@@ -7935,12 +8065,27 @@
       <c r="C1039" s="6"/>
       <c r="D1039" s="6"/>
     </row>
+    <row r="1040">
+      <c r="A1040" s="6"/>
+      <c r="B1040" s="6"/>
+      <c r="C1040" s="6"/>
+      <c r="D1040" s="6"/>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="6"/>
+      <c r="B1041" s="6"/>
+      <c r="C1041" s="6"/>
+      <c r="D1041" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D115">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D124">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="A122"/>
+  </hyperlinks>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
6 digit input updates
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="241">
   <si>
     <t>Key</t>
   </si>
@@ -272,7 +272,7 @@
     <t>forgot_password.reset.title</t>
   </si>
   <si>
-    <t>Pasword Reset</t>
+    <t>Password Reset</t>
   </si>
   <si>
     <t>forgot_password.reset.description</t>
@@ -393,6 +393,24 @@
   </si>
   <si>
     <t>Activity analysis</t>
+  </si>
+  <si>
+    <t>home.circles.live.label</t>
+  </si>
+  <si>
+    <t>Live</t>
+  </si>
+  <si>
+    <t>home.circles.alarm.label</t>
+  </si>
+  <si>
+    <t>Alarm clock</t>
+  </si>
+  <si>
+    <t>header.alarm</t>
+  </si>
+  <si>
+    <t>ALARM CLOCK</t>
   </si>
   <si>
     <t>score.quality.poor</t>
@@ -581,13 +599,175 @@
   </si>
   <si>
     <t>forgot_password.reset.confirm_password.placeholder</t>
+  </si>
+  <si>
+    <t>profile.header.title</t>
+  </si>
+  <si>
+    <t>PROFILE</t>
+  </si>
+  <si>
+    <t>profile.logout</t>
+  </si>
+  <si>
+    <t>Log out</t>
+  </si>
+  <si>
+    <t>header.live</t>
+  </si>
+  <si>
+    <t>LIVE</t>
+  </si>
+  <si>
+    <t>live.heart_rate.label</t>
+  </si>
+  <si>
+    <t>Heart rate</t>
+  </si>
+  <si>
+    <t>live.accuracy.label</t>
+  </si>
+  <si>
+    <t>Data Accuracy:</t>
+  </si>
+  <si>
+    <t>live.intensity.label</t>
+  </si>
+  <si>
+    <t>Activity Intensity</t>
+  </si>
+  <si>
+    <t>live.hr_max.label</t>
+  </si>
+  <si>
+    <t>HR Max.</t>
+  </si>
+  <si>
+    <t>live.hr_max.ratio.label</t>
+  </si>
+  <si>
+    <t>% of Max HR</t>
+  </si>
+  <si>
+    <t>live.start</t>
+  </si>
+  <si>
+    <t>START</t>
+  </si>
+  <si>
+    <t>live.hrv_blood_ox.label</t>
+  </si>
+  <si>
+    <t>HRV &amp; Blood Ox.</t>
+  </si>
+  <si>
+    <t>live.hrv.label</t>
+  </si>
+  <si>
+    <t>HRV</t>
+  </si>
+  <si>
+    <t>live.blood_ox.label</t>
+  </si>
+  <si>
+    <t>Blood Ox.</t>
+  </si>
+  <si>
+    <t>intensity.low</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>intensity.medium</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>intensity.high</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>intensity.none</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>drawer.profile</t>
+  </si>
+  <si>
+    <t>Profile</t>
+  </si>
+  <si>
+    <t>drawer.close</t>
+  </si>
+  <si>
+    <t>Close</t>
+  </si>
+  <si>
+    <t>alarm.score.programmed</t>
+  </si>
+  <si>
+    <t>Programmed alarms</t>
+  </si>
+  <si>
+    <t>alarm.score.week</t>
+  </si>
+  <si>
+    <t>Week overview</t>
+  </si>
+  <si>
+    <t>alarm.score.add_button</t>
+  </si>
+  <si>
+    <t>Add an alarm</t>
+  </si>
+  <si>
+    <t>onboarding.wear.title</t>
+  </si>
+  <si>
+    <t>How to wear Circular</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>onboarding.wear.info</t>
+    </r>
+    <r>
+      <rPr/>
+      <t>.top</t>
+    </r>
+  </si>
+  <si>
+    <t>The best fingers to wear Circular are the &lt;colored&gt;index&lt;/colored&gt;, &lt;colored&gt;middle finger&lt;/colored&gt;, &lt;colored&gt;ring finger&lt;/colored&gt;, pinky finger and thumb.
+Try as much as possible to use the same finger and same ring positioning each time you wear your Circular.</t>
+  </si>
+  <si>
+    <t>onboarding.wear.info.bottom</t>
+  </si>
+  <si>
+    <t>The flat part of the ring should be on the &lt;colored&gt;palmar side&lt;/colored&gt; of your finger.
+The button should be &lt;colored&gt;facing your thumb&lt;/colored&gt;, for ease of use.</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.title</t>
+  </si>
+  <si>
+    <t>Tell us more about yourself</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -605,6 +785,10 @@
     <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
   </fonts>
   <fills count="5">
@@ -639,7 +823,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -672,6 +856,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1767,7 +1954,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="s">
+      <c r="A72" s="5" t="s">
         <v>129</v>
       </c>
       <c r="B72" s="6"/>
@@ -1779,7 +1966,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="s">
+      <c r="A73" s="5" t="s">
         <v>131</v>
       </c>
       <c r="B73" s="6"/>
@@ -1803,7 +1990,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="s">
+      <c r="A75" s="8" t="s">
         <v>135</v>
       </c>
       <c r="B75" s="6"/>
@@ -1815,7 +2002,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="5" t="s">
+      <c r="A76" s="8" t="s">
         <v>137</v>
       </c>
       <c r="B76" s="6"/>
@@ -2096,7 +2283,7 @@
       </c>
       <c r="B99" s="6"/>
       <c r="C99" s="7" t="s">
-        <v>24</v>
+        <v>184</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>6</v>
@@ -2104,183 +2291,351 @@
     </row>
     <row r="100">
       <c r="A100" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" s="6"/>
+      <c r="C101" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D101" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="6"/>
+      <c r="C102" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D100" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="6"/>
-      <c r="B101" s="6"/>
-      <c r="C101" s="6"/>
-      <c r="D101" s="6"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="6"/>
-      <c r="B102" s="6"/>
-      <c r="C102" s="6"/>
-      <c r="D102" s="6"/>
+      <c r="D102" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="6"/>
+      <c r="A103" s="5" t="s">
+        <v>190</v>
+      </c>
       <c r="B103" s="6"/>
-      <c r="C103" s="6"/>
-      <c r="D103" s="6"/>
+      <c r="C103" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D103" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="6"/>
+      <c r="A104" s="5" t="s">
+        <v>191</v>
+      </c>
       <c r="B104" s="6"/>
-      <c r="C104" s="6"/>
-      <c r="D104" s="6"/>
+      <c r="C104" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="D104" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" s="6"/>
+      <c r="A105" s="5" t="s">
+        <v>193</v>
+      </c>
       <c r="B105" s="6"/>
-      <c r="C105" s="6"/>
-      <c r="D105" s="6"/>
+      <c r="C105" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="D105" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="6"/>
+      <c r="A106" s="5" t="s">
+        <v>195</v>
+      </c>
       <c r="B106" s="6"/>
-      <c r="C106" s="6"/>
-      <c r="D106" s="6"/>
+      <c r="C106" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D106" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="6"/>
+      <c r="A107" s="5" t="s">
+        <v>197</v>
+      </c>
       <c r="B107" s="6"/>
-      <c r="C107" s="6"/>
-      <c r="D107" s="6"/>
+      <c r="C107" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="D107" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="6"/>
+      <c r="A108" s="5" t="s">
+        <v>199</v>
+      </c>
       <c r="B108" s="6"/>
-      <c r="C108" s="6"/>
-      <c r="D108" s="6"/>
+      <c r="C108" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="6"/>
+      <c r="A109" s="5" t="s">
+        <v>201</v>
+      </c>
       <c r="B109" s="6"/>
-      <c r="C109" s="6"/>
-      <c r="D109" s="6"/>
+      <c r="C109" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="6"/>
+      <c r="A110" s="5" t="s">
+        <v>203</v>
+      </c>
       <c r="B110" s="6"/>
-      <c r="C110" s="6"/>
-      <c r="D110" s="6"/>
+      <c r="C110" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="6"/>
+      <c r="A111" s="5" t="s">
+        <v>205</v>
+      </c>
       <c r="B111" s="6"/>
-      <c r="C111" s="6"/>
-      <c r="D111" s="6"/>
+      <c r="C111" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="112">
-      <c r="A112" s="6"/>
+      <c r="A112" s="5" t="s">
+        <v>207</v>
+      </c>
       <c r="B112" s="6"/>
-      <c r="C112" s="6"/>
-      <c r="D112" s="6"/>
+      <c r="C112" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="D112" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="113">
-      <c r="A113" s="6"/>
+      <c r="A113" s="5" t="s">
+        <v>209</v>
+      </c>
       <c r="B113" s="6"/>
-      <c r="C113" s="6"/>
-      <c r="D113" s="6"/>
+      <c r="C113" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="D113" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="114">
-      <c r="A114" s="6"/>
+      <c r="A114" s="5" t="s">
+        <v>211</v>
+      </c>
       <c r="B114" s="6"/>
-      <c r="C114" s="6"/>
-      <c r="D114" s="6"/>
+      <c r="C114" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="115">
-      <c r="A115" s="6"/>
+      <c r="A115" s="5" t="s">
+        <v>213</v>
+      </c>
       <c r="B115" s="6"/>
-      <c r="C115" s="6"/>
-      <c r="D115" s="6"/>
+      <c r="C115" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="116">
-      <c r="A116" s="6"/>
+      <c r="A116" s="5" t="s">
+        <v>215</v>
+      </c>
       <c r="B116" s="6"/>
-      <c r="C116" s="6"/>
-      <c r="D116" s="6"/>
+      <c r="C116" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="D116" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="117">
-      <c r="A117" s="6"/>
+      <c r="A117" s="8" t="s">
+        <v>217</v>
+      </c>
       <c r="B117" s="6"/>
-      <c r="C117" s="6"/>
-      <c r="D117" s="6"/>
+      <c r="C117" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="D117" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" s="6"/>
+      <c r="A118" s="8" t="s">
+        <v>219</v>
+      </c>
       <c r="B118" s="6"/>
-      <c r="C118" s="6"/>
-      <c r="D118" s="6"/>
+      <c r="C118" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="119">
-      <c r="A119" s="6"/>
+      <c r="A119" s="8" t="s">
+        <v>221</v>
+      </c>
       <c r="B119" s="6"/>
-      <c r="C119" s="6"/>
-      <c r="D119" s="6"/>
+      <c r="C119" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="120">
-      <c r="A120" s="6"/>
+      <c r="A120" s="5" t="s">
+        <v>223</v>
+      </c>
       <c r="B120" s="6"/>
-      <c r="C120" s="6"/>
-      <c r="D120" s="6"/>
+      <c r="C120" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="121">
-      <c r="A121" s="6"/>
+      <c r="A121" s="5" t="s">
+        <v>225</v>
+      </c>
       <c r="B121" s="6"/>
-      <c r="C121" s="6"/>
-      <c r="D121" s="6"/>
+      <c r="C121" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="122">
-      <c r="A122" s="6"/>
+      <c r="A122" s="5" t="s">
+        <v>227</v>
+      </c>
       <c r="B122" s="6"/>
-      <c r="C122" s="6"/>
-      <c r="D122" s="6"/>
+      <c r="C122" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="123">
-      <c r="A123" s="6"/>
+      <c r="A123" s="5" t="s">
+        <v>229</v>
+      </c>
       <c r="B123" s="6"/>
-      <c r="C123" s="6"/>
-      <c r="D123" s="6"/>
+      <c r="C123" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="124">
-      <c r="A124" s="6"/>
+      <c r="A124" s="5" t="s">
+        <v>231</v>
+      </c>
       <c r="B124" s="6"/>
-      <c r="C124" s="6"/>
-      <c r="D124" s="6"/>
+      <c r="C124" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D124" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="125">
-      <c r="A125" s="6"/>
+      <c r="A125" s="5" t="s">
+        <v>233</v>
+      </c>
       <c r="B125" s="6"/>
-      <c r="C125" s="6"/>
-      <c r="D125" s="6"/>
+      <c r="C125" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="126">
-      <c r="A126" s="6"/>
+      <c r="A126" s="11" t="s">
+        <v>235</v>
+      </c>
       <c r="B126" s="6"/>
-      <c r="C126" s="6"/>
-      <c r="D126" s="6"/>
+      <c r="C126" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="127">
-      <c r="A127" s="6"/>
+      <c r="A127" s="5" t="s">
+        <v>237</v>
+      </c>
       <c r="B127" s="6"/>
-      <c r="C127" s="6"/>
-      <c r="D127" s="6"/>
+      <c r="C127" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="128">
-      <c r="A128" s="6"/>
+      <c r="A128" s="5" t="s">
+        <v>239</v>
+      </c>
       <c r="B128" s="6"/>
-      <c r="C128" s="6"/>
-      <c r="D128" s="6"/>
+      <c r="C128" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="6"/>
@@ -7736,12 +8091,63 @@
       <c r="C1037" s="6"/>
       <c r="D1037" s="6"/>
     </row>
+    <row r="1038">
+      <c r="A1038" s="6"/>
+      <c r="B1038" s="6"/>
+      <c r="C1038" s="6"/>
+      <c r="D1038" s="6"/>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="6"/>
+      <c r="B1039" s="6"/>
+      <c r="C1039" s="6"/>
+      <c r="D1039" s="6"/>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="6"/>
+      <c r="B1040" s="6"/>
+      <c r="C1040" s="6"/>
+      <c r="D1040" s="6"/>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="6"/>
+      <c r="B1041" s="6"/>
+      <c r="C1041" s="6"/>
+      <c r="D1041" s="6"/>
+    </row>
+    <row r="1042">
+      <c r="A1042" s="6"/>
+      <c r="B1042" s="6"/>
+      <c r="C1042" s="6"/>
+      <c r="D1042" s="6"/>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="6"/>
+      <c r="B1043" s="6"/>
+      <c r="C1043" s="6"/>
+      <c r="D1043" s="6"/>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="6"/>
+      <c r="B1044" s="6"/>
+      <c r="C1044" s="6"/>
+      <c r="D1044" s="6"/>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="6"/>
+      <c r="B1045" s="6"/>
+      <c r="C1045" s="6"/>
+      <c r="D1045" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D100">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D128">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="A126"/>
+  </hyperlinks>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updates wordings + Reset password screen layout adjustments
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="242">
   <si>
     <t>Key</t>
   </si>
@@ -323,10 +323,13 @@
     <t>forgot_password.new.password</t>
   </si>
   <si>
+    <t>New password</t>
+  </si>
+  <si>
     <t>forgot_password.new.confirm_password</t>
   </si>
   <si>
-    <t>Confim password</t>
+    <t>Confim new password</t>
   </si>
   <si>
     <t>forgot_password.new.button</t>
@@ -767,7 +770,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -786,6 +789,7 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -823,7 +827,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -854,10 +858,13 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1792,8 +1799,8 @@
         <v>102</v>
       </c>
       <c r="B58" s="6"/>
-      <c r="C58" s="7" t="s">
-        <v>26</v>
+      <c r="C58" s="10" t="s">
+        <v>103</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -1801,11 +1808,11 @@
     </row>
     <row r="59">
       <c r="A59" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B59" s="6"/>
-      <c r="C59" s="7" t="s">
-        <v>104</v>
+      <c r="C59" s="10" t="s">
+        <v>105</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>6</v>
@@ -1813,45 +1820,45 @@
     </row>
     <row r="60">
       <c r="A60" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="10" t="s">
-        <v>107</v>
+      <c r="A61" s="11" t="s">
+        <v>108</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="D61" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D61" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="10" t="s">
-        <v>109</v>
+      <c r="A62" s="11" t="s">
+        <v>110</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D62" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D62" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>6</v>
@@ -1859,11 +1866,11 @@
     </row>
     <row r="64">
       <c r="A64" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>6</v>
@@ -1871,11 +1878,11 @@
     </row>
     <row r="65">
       <c r="A65" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B65" s="6"/>
       <c r="C65" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>6</v>
@@ -1883,11 +1890,11 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B66" s="6"/>
       <c r="C66" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>6</v>
@@ -1895,11 +1902,11 @@
     </row>
     <row r="67">
       <c r="A67" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B67" s="6"/>
       <c r="C67" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>6</v>
@@ -1907,11 +1914,11 @@
     </row>
     <row r="68">
       <c r="A68" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>6</v>
@@ -1919,11 +1926,11 @@
     </row>
     <row r="69">
       <c r="A69" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>6</v>
@@ -1931,11 +1938,11 @@
     </row>
     <row r="70">
       <c r="A70" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B70" s="6"/>
       <c r="C70" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D70" s="5" t="s">
         <v>6</v>
@@ -1943,11 +1950,11 @@
     </row>
     <row r="71">
       <c r="A71" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D71" s="5" t="s">
         <v>6</v>
@@ -1955,11 +1962,11 @@
     </row>
     <row r="72">
       <c r="A72" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B72" s="6"/>
       <c r="C72" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>6</v>
@@ -1967,11 +1974,11 @@
     </row>
     <row r="73">
       <c r="A73" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B73" s="6"/>
       <c r="C73" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>6</v>
@@ -1979,11 +1986,11 @@
     </row>
     <row r="74">
       <c r="A74" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B74" s="6"/>
       <c r="C74" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D74" s="5" t="s">
         <v>6</v>
@@ -1991,11 +1998,11 @@
     </row>
     <row r="75">
       <c r="A75" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B75" s="6"/>
       <c r="C75" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D75" s="5" t="s">
         <v>6</v>
@@ -2003,11 +2010,11 @@
     </row>
     <row r="76">
       <c r="A76" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B76" s="6"/>
       <c r="C76" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D76" s="5" t="s">
         <v>6</v>
@@ -2015,11 +2022,11 @@
     </row>
     <row r="77">
       <c r="A77" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B77" s="6"/>
       <c r="C77" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D77" s="5" t="s">
         <v>6</v>
@@ -2027,11 +2034,11 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B78" s="6"/>
       <c r="C78" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D78" s="5" t="s">
         <v>6</v>
@@ -2039,11 +2046,11 @@
     </row>
     <row r="79">
       <c r="A79" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B79" s="6"/>
       <c r="C79" s="7" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D79" s="5" t="s">
         <v>6</v>
@@ -2051,11 +2058,11 @@
     </row>
     <row r="80">
       <c r="A80" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B80" s="6"/>
       <c r="C80" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D80" s="5" t="s">
         <v>6</v>
@@ -2063,11 +2070,11 @@
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B81" s="6"/>
       <c r="C81" s="7" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>6</v>
@@ -2075,11 +2082,11 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B82" s="6"/>
       <c r="C82" s="7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>6</v>
@@ -2087,11 +2094,11 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B83" s="6"/>
       <c r="C83" s="7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>6</v>
@@ -2099,11 +2106,11 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B84" s="6"/>
       <c r="C84" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>6</v>
@@ -2111,11 +2118,11 @@
     </row>
     <row r="85">
       <c r="A85" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B85" s="6"/>
       <c r="C85" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>6</v>
@@ -2123,11 +2130,11 @@
     </row>
     <row r="86">
       <c r="A86" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B86" s="6"/>
       <c r="C86" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>6</v>
@@ -2135,11 +2142,11 @@
     </row>
     <row r="87">
       <c r="A87" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B87" s="6"/>
       <c r="C87" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D87" s="5" t="s">
         <v>6</v>
@@ -2147,11 +2154,11 @@
     </row>
     <row r="88">
       <c r="A88" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B88" s="6"/>
       <c r="C88" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>6</v>
@@ -2159,11 +2166,11 @@
     </row>
     <row r="89">
       <c r="A89" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B89" s="6"/>
       <c r="C89" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D89" s="5" t="s">
         <v>6</v>
@@ -2171,11 +2178,11 @@
     </row>
     <row r="90">
       <c r="A90" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B90" s="6"/>
       <c r="C90" s="7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D90" s="5" t="s">
         <v>6</v>
@@ -2183,11 +2190,11 @@
     </row>
     <row r="91">
       <c r="A91" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B91" s="6"/>
       <c r="C91" s="7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D91" s="5" t="s">
         <v>6</v>
@@ -2195,11 +2202,11 @@
     </row>
     <row r="92">
       <c r="A92" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B92" s="6"/>
       <c r="C92" s="7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D92" s="5" t="s">
         <v>6</v>
@@ -2207,11 +2214,11 @@
     </row>
     <row r="93">
       <c r="A93" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B93" s="6"/>
       <c r="C93" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>6</v>
@@ -2219,11 +2226,11 @@
     </row>
     <row r="94">
       <c r="A94" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B94" s="6"/>
       <c r="C94" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D94" s="5" t="s">
         <v>6</v>
@@ -2231,11 +2238,11 @@
     </row>
     <row r="95">
       <c r="A95" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B95" s="6"/>
       <c r="C95" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D95" s="5" t="s">
         <v>6</v>
@@ -2243,11 +2250,11 @@
     </row>
     <row r="96">
       <c r="A96" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B96" s="6"/>
       <c r="C96" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D96" s="5" t="s">
         <v>6</v>
@@ -2255,11 +2262,11 @@
     </row>
     <row r="97">
       <c r="A97" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B97" s="6"/>
       <c r="C97" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D97" s="5" t="s">
         <v>6</v>
@@ -2267,11 +2274,11 @@
     </row>
     <row r="98">
       <c r="A98" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B98" s="6"/>
       <c r="C98" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D98" s="5" t="s">
         <v>6</v>
@@ -2279,11 +2286,11 @@
     </row>
     <row r="99">
       <c r="A99" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B99" s="6"/>
       <c r="C99" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>6</v>
@@ -2291,11 +2298,11 @@
     </row>
     <row r="100">
       <c r="A100" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>6</v>
@@ -2303,11 +2310,11 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B101" s="6"/>
       <c r="C101" s="7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>6</v>
@@ -2315,7 +2322,7 @@
     </row>
     <row r="102">
       <c r="A102" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B102" s="6"/>
       <c r="C102" s="7" t="s">
@@ -2327,7 +2334,7 @@
     </row>
     <row r="103">
       <c r="A103" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B103" s="6"/>
       <c r="C103" s="7" t="s">
@@ -2339,11 +2346,11 @@
     </row>
     <row r="104">
       <c r="A104" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B104" s="6"/>
       <c r="C104" s="7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>6</v>
@@ -2351,11 +2358,11 @@
     </row>
     <row r="105">
       <c r="A105" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="7" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D105" s="5" t="s">
         <v>6</v>
@@ -2363,11 +2370,11 @@
     </row>
     <row r="106">
       <c r="A106" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B106" s="6"/>
       <c r="C106" s="7" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D106" s="5" t="s">
         <v>6</v>
@@ -2375,11 +2382,11 @@
     </row>
     <row r="107">
       <c r="A107" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B107" s="6"/>
       <c r="C107" s="7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D107" s="5" t="s">
         <v>6</v>
@@ -2387,11 +2394,11 @@
     </row>
     <row r="108">
       <c r="A108" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B108" s="6"/>
       <c r="C108" s="7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D108" s="5" t="s">
         <v>6</v>
@@ -2399,11 +2406,11 @@
     </row>
     <row r="109">
       <c r="A109" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B109" s="6"/>
       <c r="C109" s="7" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>6</v>
@@ -2411,11 +2418,11 @@
     </row>
     <row r="110">
       <c r="A110" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B110" s="6"/>
       <c r="C110" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>6</v>
@@ -2423,11 +2430,11 @@
     </row>
     <row r="111">
       <c r="A111" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B111" s="6"/>
       <c r="C111" s="7" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>6</v>
@@ -2435,11 +2442,11 @@
     </row>
     <row r="112">
       <c r="A112" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B112" s="6"/>
       <c r="C112" s="7" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>6</v>
@@ -2447,11 +2454,11 @@
     </row>
     <row r="113">
       <c r="A113" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B113" s="6"/>
       <c r="C113" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>6</v>
@@ -2459,11 +2466,11 @@
     </row>
     <row r="114">
       <c r="A114" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B114" s="6"/>
       <c r="C114" s="7" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>6</v>
@@ -2471,11 +2478,11 @@
     </row>
     <row r="115">
       <c r="A115" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B115" s="6"/>
       <c r="C115" s="7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>6</v>
@@ -2483,11 +2490,11 @@
     </row>
     <row r="116">
       <c r="A116" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B116" s="6"/>
       <c r="C116" s="7" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D116" s="5" t="s">
         <v>6</v>
@@ -2495,11 +2502,11 @@
     </row>
     <row r="117">
       <c r="A117" s="8" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B117" s="6"/>
       <c r="C117" s="7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>6</v>
@@ -2507,11 +2514,11 @@
     </row>
     <row r="118">
       <c r="A118" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B118" s="6"/>
       <c r="C118" s="7" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>6</v>
@@ -2519,11 +2526,11 @@
     </row>
     <row r="119">
       <c r="A119" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B119" s="6"/>
       <c r="C119" s="7" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>6</v>
@@ -2531,11 +2538,11 @@
     </row>
     <row r="120">
       <c r="A120" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B120" s="6"/>
       <c r="C120" s="7" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>6</v>
@@ -2543,11 +2550,11 @@
     </row>
     <row r="121">
       <c r="A121" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B121" s="6"/>
       <c r="C121" s="7" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>6</v>
@@ -2555,11 +2562,11 @@
     </row>
     <row r="122">
       <c r="A122" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B122" s="6"/>
       <c r="C122" s="7" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>6</v>
@@ -2567,11 +2574,11 @@
     </row>
     <row r="123">
       <c r="A123" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B123" s="6"/>
       <c r="C123" s="7" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>6</v>
@@ -2579,11 +2586,11 @@
     </row>
     <row r="124">
       <c r="A124" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -2591,23 +2598,23 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="11" t="s">
-        <v>235</v>
+      <c r="A126" s="12" t="s">
+        <v>236</v>
       </c>
       <c r="B126" s="6"/>
       <c r="C126" s="7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D126" s="5" t="s">
         <v>6</v>
@@ -2615,11 +2622,11 @@
     </row>
     <row r="127">
       <c r="A127" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B127" s="6"/>
       <c r="C127" s="7" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D127" s="5" t="s">
         <v>6</v>
@@ -2627,11 +2634,11 @@
     </row>
     <row r="128">
       <c r="A128" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
Pairing start screen layout updates + No bluetooth screen
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="243">
   <si>
     <t>Key</t>
   </si>
@@ -34,16 +34,19 @@
     <t>A valider</t>
   </si>
   <si>
+    <t>setup.scan.disabled.title</t>
+  </si>
+  <si>
+    <t>Enable bluetooth</t>
+  </si>
+  <si>
     <t>setup.scan.disabled.message</t>
   </si>
   <si>
-    <t>To proceed, please enable the bluetooth on you phone</t>
+    <t>Make sure that your Bluetooth is enabled on your phone to begin pairing with a Circular ring and that you have your ring close to your phone.</t>
   </si>
   <si>
     <t>setup.scan.disabled.enable</t>
-  </si>
-  <si>
-    <t>Enable bluetooth</t>
   </si>
   <si>
     <t>setup.scan.enabled.title</t>
@@ -785,11 +788,11 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -827,7 +830,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -852,14 +855,17 @@
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -1135,11 +1141,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="6"/>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="9" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="5" t="s">
@@ -1147,11 +1153,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="6"/>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -1159,60 +1165,60 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="10" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="s">
-        <v>13</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="s">
         <v>14</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="s">
-        <v>15</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="s">
         <v>16</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="s">
-        <v>17</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="s">
         <v>18</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="s">
-        <v>19</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>6</v>
@@ -1220,11 +1226,11 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>6</v>
@@ -1232,11 +1238,11 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>6</v>
@@ -1244,11 +1250,11 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>6</v>
@@ -1256,11 +1262,11 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>6</v>
@@ -1272,7 +1278,7 @@
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>6</v>
@@ -1280,11 +1286,11 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>6</v>
@@ -1292,11 +1298,11 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>6</v>
@@ -1304,11 +1310,11 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>6</v>
@@ -1316,11 +1322,11 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>6</v>
@@ -1328,11 +1334,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>6</v>
@@ -1340,11 +1346,11 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>6</v>
@@ -1352,35 +1358,35 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="7" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="5" t="s">
         <v>43</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="10" t="s">
         <v>44</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>6</v>
@@ -1392,7 +1398,7 @@
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="7" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>6</v>
@@ -1400,11 +1406,11 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="7" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>6</v>
@@ -1416,7 +1422,7 @@
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>6</v>
@@ -1428,7 +1434,7 @@
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>6</v>
@@ -1440,7 +1446,7 @@
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>6</v>
@@ -1452,7 +1458,7 @@
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="7" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>6</v>
@@ -1460,11 +1466,11 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>6</v>
@@ -1476,7 +1482,7 @@
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>6</v>
@@ -1488,7 +1494,7 @@
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="7" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>6</v>
@@ -1500,7 +1506,7 @@
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>6</v>
@@ -1508,11 +1514,11 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>6</v>
@@ -1520,11 +1526,11 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>6</v>
@@ -1532,11 +1538,11 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>6</v>
@@ -1544,11 +1550,11 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>6</v>
@@ -1556,11 +1562,11 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>6</v>
@@ -1568,11 +1574,11 @@
     </row>
     <row r="39">
       <c r="A39" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="7" t="s">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>6</v>
@@ -1584,7 +1590,7 @@
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="s">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>6</v>
@@ -1592,11 +1598,11 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>6</v>
@@ -1604,11 +1610,11 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>6</v>
@@ -1616,11 +1622,11 @@
     </row>
     <row r="43">
       <c r="A43" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>6</v>
@@ -1628,11 +1634,11 @@
     </row>
     <row r="44">
       <c r="A44" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>6</v>
@@ -1640,11 +1646,11 @@
     </row>
     <row r="45">
       <c r="A45" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>6</v>
@@ -1652,11 +1658,11 @@
     </row>
     <row r="46">
       <c r="A46" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>6</v>
@@ -1664,11 +1670,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>6</v>
@@ -1676,11 +1682,11 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>6</v>
@@ -1688,11 +1694,11 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>6</v>
@@ -1700,11 +1706,11 @@
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="7" t="s">
-        <v>24</v>
+        <v>89</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>6</v>
@@ -1716,7 +1722,7 @@
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="7" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>6</v>
@@ -1724,11 +1730,11 @@
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="7" t="s">
-        <v>22</v>
+        <v>92</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>6</v>
@@ -1740,7 +1746,7 @@
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
-        <v>94</v>
+        <v>23</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>6</v>
@@ -1748,11 +1754,11 @@
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>6</v>
@@ -1764,7 +1770,7 @@
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="7" t="s">
-        <v>97</v>
+        <v>75</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>6</v>
@@ -1772,11 +1778,11 @@
     </row>
     <row r="56">
       <c r="A56" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>6</v>
@@ -1784,11 +1790,11 @@
     </row>
     <row r="57">
       <c r="A57" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>6</v>
@@ -1796,11 +1802,11 @@
     </row>
     <row r="58">
       <c r="A58" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="6"/>
+      <c r="C58" s="7" t="s">
         <v>102</v>
-      </c>
-      <c r="B58" s="6"/>
-      <c r="C58" s="10" t="s">
-        <v>103</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -1808,11 +1814,11 @@
     </row>
     <row r="59">
       <c r="A59" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B59" s="6"/>
+      <c r="C59" s="7" t="s">
         <v>104</v>
-      </c>
-      <c r="B59" s="6"/>
-      <c r="C59" s="10" t="s">
-        <v>105</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>6</v>
@@ -1820,57 +1826,57 @@
     </row>
     <row r="60">
       <c r="A60" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="D60" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="11" t="s">
+      <c r="B61" s="6"/>
+      <c r="C61" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="C61" s="7" t="s">
+      <c r="D61" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="D61" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="11" t="s">
+      <c r="C62" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C62" s="7" t="s">
+      <c r="D62" s="12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="D62" s="11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="s">
+      <c r="C63" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B63" s="6"/>
-      <c r="C63" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="D63" s="5" t="s">
+      <c r="D63" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>6</v>
@@ -1878,11 +1884,11 @@
     </row>
     <row r="65">
       <c r="A65" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B65" s="6"/>
       <c r="C65" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>6</v>
@@ -1890,11 +1896,11 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B66" s="6"/>
       <c r="C66" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>6</v>
@@ -1902,11 +1908,11 @@
     </row>
     <row r="67">
       <c r="A67" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B67" s="6"/>
       <c r="C67" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>6</v>
@@ -1914,11 +1920,11 @@
     </row>
     <row r="68">
       <c r="A68" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>6</v>
@@ -1926,11 +1932,11 @@
     </row>
     <row r="69">
       <c r="A69" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>6</v>
@@ -1938,11 +1944,11 @@
     </row>
     <row r="70">
       <c r="A70" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B70" s="6"/>
       <c r="C70" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D70" s="5" t="s">
         <v>6</v>
@@ -1950,11 +1956,11 @@
     </row>
     <row r="71">
       <c r="A71" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D71" s="5" t="s">
         <v>6</v>
@@ -1962,11 +1968,11 @@
     </row>
     <row r="72">
       <c r="A72" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B72" s="6"/>
       <c r="C72" s="7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>6</v>
@@ -1974,11 +1980,11 @@
     </row>
     <row r="73">
       <c r="A73" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B73" s="6"/>
       <c r="C73" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>6</v>
@@ -1986,47 +1992,47 @@
     </row>
     <row r="74">
       <c r="A74" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B74" s="6"/>
       <c r="C74" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="s">
         <v>135</v>
-      </c>
-      <c r="D74" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="s">
-        <v>136</v>
       </c>
       <c r="B75" s="6"/>
       <c r="C75" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="D75" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="s">
-        <v>138</v>
       </c>
       <c r="B76" s="6"/>
       <c r="C76" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="D76" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="s">
         <v>139</v>
-      </c>
-      <c r="D76" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="5" t="s">
-        <v>140</v>
       </c>
       <c r="B77" s="6"/>
       <c r="C77" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D77" s="5" t="s">
         <v>6</v>
@@ -2034,11 +2040,11 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B78" s="6"/>
       <c r="C78" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D78" s="5" t="s">
         <v>6</v>
@@ -2046,11 +2052,11 @@
     </row>
     <row r="79">
       <c r="A79" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B79" s="6"/>
       <c r="C79" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D79" s="5" t="s">
         <v>6</v>
@@ -2058,11 +2064,11 @@
     </row>
     <row r="80">
       <c r="A80" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B80" s="6"/>
       <c r="C80" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D80" s="5" t="s">
         <v>6</v>
@@ -2070,11 +2076,11 @@
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B81" s="6"/>
       <c r="C81" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>6</v>
@@ -2082,11 +2088,11 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B82" s="6"/>
       <c r="C82" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>6</v>
@@ -2094,11 +2100,11 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B83" s="6"/>
       <c r="C83" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>6</v>
@@ -2106,11 +2112,11 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B84" s="6"/>
       <c r="C84" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>6</v>
@@ -2118,11 +2124,11 @@
     </row>
     <row r="85">
       <c r="A85" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B85" s="6"/>
       <c r="C85" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>6</v>
@@ -2130,11 +2136,11 @@
     </row>
     <row r="86">
       <c r="A86" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B86" s="6"/>
       <c r="C86" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>6</v>
@@ -2142,11 +2148,11 @@
     </row>
     <row r="87">
       <c r="A87" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B87" s="6"/>
       <c r="C87" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D87" s="5" t="s">
         <v>6</v>
@@ -2154,11 +2160,11 @@
     </row>
     <row r="88">
       <c r="A88" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B88" s="6"/>
       <c r="C88" s="7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>6</v>
@@ -2166,11 +2172,11 @@
     </row>
     <row r="89">
       <c r="A89" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B89" s="6"/>
       <c r="C89" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D89" s="5" t="s">
         <v>6</v>
@@ -2178,11 +2184,11 @@
     </row>
     <row r="90">
       <c r="A90" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B90" s="6"/>
       <c r="C90" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D90" s="5" t="s">
         <v>6</v>
@@ -2190,11 +2196,11 @@
     </row>
     <row r="91">
       <c r="A91" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B91" s="6"/>
       <c r="C91" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D91" s="5" t="s">
         <v>6</v>
@@ -2202,11 +2208,11 @@
     </row>
     <row r="92">
       <c r="A92" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B92" s="6"/>
       <c r="C92" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D92" s="5" t="s">
         <v>6</v>
@@ -2214,11 +2220,11 @@
     </row>
     <row r="93">
       <c r="A93" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B93" s="6"/>
       <c r="C93" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>6</v>
@@ -2226,11 +2232,11 @@
     </row>
     <row r="94">
       <c r="A94" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B94" s="6"/>
       <c r="C94" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D94" s="5" t="s">
         <v>6</v>
@@ -2238,11 +2244,11 @@
     </row>
     <row r="95">
       <c r="A95" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B95" s="6"/>
       <c r="C95" s="7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D95" s="5" t="s">
         <v>6</v>
@@ -2250,11 +2256,11 @@
     </row>
     <row r="96">
       <c r="A96" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B96" s="6"/>
       <c r="C96" s="7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D96" s="5" t="s">
         <v>6</v>
@@ -2262,11 +2268,11 @@
     </row>
     <row r="97">
       <c r="A97" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B97" s="6"/>
       <c r="C97" s="7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D97" s="5" t="s">
         <v>6</v>
@@ -2274,11 +2280,11 @@
     </row>
     <row r="98">
       <c r="A98" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B98" s="6"/>
       <c r="C98" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D98" s="5" t="s">
         <v>6</v>
@@ -2286,11 +2292,11 @@
     </row>
     <row r="99">
       <c r="A99" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B99" s="6"/>
       <c r="C99" s="7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>6</v>
@@ -2298,11 +2304,11 @@
     </row>
     <row r="100">
       <c r="A100" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>6</v>
@@ -2310,11 +2316,11 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B101" s="6"/>
       <c r="C101" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>6</v>
@@ -2322,11 +2328,11 @@
     </row>
     <row r="102">
       <c r="A102" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B102" s="6"/>
       <c r="C102" s="7" t="s">
-        <v>24</v>
+        <v>190</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>6</v>
@@ -2338,7 +2344,7 @@
       </c>
       <c r="B103" s="6"/>
       <c r="C103" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>6</v>
@@ -2350,7 +2356,7 @@
       </c>
       <c r="B104" s="6"/>
       <c r="C104" s="7" t="s">
-        <v>193</v>
+        <v>25</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>6</v>
@@ -2358,11 +2364,11 @@
     </row>
     <row r="105">
       <c r="A105" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D105" s="5" t="s">
         <v>6</v>
@@ -2370,11 +2376,11 @@
     </row>
     <row r="106">
       <c r="A106" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B106" s="6"/>
       <c r="C106" s="7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D106" s="5" t="s">
         <v>6</v>
@@ -2382,11 +2388,11 @@
     </row>
     <row r="107">
       <c r="A107" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B107" s="6"/>
       <c r="C107" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D107" s="5" t="s">
         <v>6</v>
@@ -2394,11 +2400,11 @@
     </row>
     <row r="108">
       <c r="A108" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B108" s="6"/>
       <c r="C108" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D108" s="5" t="s">
         <v>6</v>
@@ -2406,11 +2412,11 @@
     </row>
     <row r="109">
       <c r="A109" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B109" s="6"/>
       <c r="C109" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>6</v>
@@ -2418,11 +2424,11 @@
     </row>
     <row r="110">
       <c r="A110" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B110" s="6"/>
       <c r="C110" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>6</v>
@@ -2430,11 +2436,11 @@
     </row>
     <row r="111">
       <c r="A111" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B111" s="6"/>
       <c r="C111" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>6</v>
@@ -2442,11 +2448,11 @@
     </row>
     <row r="112">
       <c r="A112" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B112" s="6"/>
       <c r="C112" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>6</v>
@@ -2454,11 +2460,11 @@
     </row>
     <row r="113">
       <c r="A113" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B113" s="6"/>
       <c r="C113" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>6</v>
@@ -2466,11 +2472,11 @@
     </row>
     <row r="114">
       <c r="A114" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B114" s="6"/>
       <c r="C114" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>6</v>
@@ -2478,11 +2484,11 @@
     </row>
     <row r="115">
       <c r="A115" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B115" s="6"/>
       <c r="C115" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>6</v>
@@ -2490,59 +2496,59 @@
     </row>
     <row r="116">
       <c r="A116" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B116" s="6"/>
       <c r="C116" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="D116" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="D116" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="8" t="s">
-        <v>218</v>
       </c>
       <c r="B117" s="6"/>
       <c r="C117" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="D117" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="s">
         <v>219</v>
-      </c>
-      <c r="D117" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="8" t="s">
-        <v>220</v>
       </c>
       <c r="B118" s="6"/>
       <c r="C118" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="s">
         <v>221</v>
-      </c>
-      <c r="D118" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="8" t="s">
-        <v>222</v>
       </c>
       <c r="B119" s="6"/>
       <c r="C119" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="D119" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="5" t="s">
-        <v>224</v>
       </c>
       <c r="B120" s="6"/>
       <c r="C120" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>6</v>
@@ -2550,11 +2556,11 @@
     </row>
     <row r="121">
       <c r="A121" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B121" s="6"/>
       <c r="C121" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>6</v>
@@ -2562,11 +2568,11 @@
     </row>
     <row r="122">
       <c r="A122" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B122" s="6"/>
       <c r="C122" s="7" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>6</v>
@@ -2574,11 +2580,11 @@
     </row>
     <row r="123">
       <c r="A123" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B123" s="6"/>
       <c r="C123" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>6</v>
@@ -2586,11 +2592,11 @@
     </row>
     <row r="124">
       <c r="A124" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -2598,35 +2604,35 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="s">
         <v>235</v>
-      </c>
-      <c r="D125" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="12" t="s">
-        <v>236</v>
       </c>
       <c r="B126" s="6"/>
       <c r="C126" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="13" t="s">
         <v>237</v>
-      </c>
-      <c r="D126" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="5" t="s">
-        <v>238</v>
       </c>
       <c r="B127" s="6"/>
       <c r="C127" s="7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D127" s="5" t="s">
         <v>6</v>
@@ -2634,21 +2640,27 @@
     </row>
     <row r="128">
       <c r="A128" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="D128" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="6"/>
       <c r="B129" s="6"/>
-      <c r="C129" s="6"/>
-      <c r="D129" s="6"/>
+      <c r="C129" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="6"/>
@@ -8146,14 +8158,20 @@
       <c r="C1045" s="6"/>
       <c r="D1045" s="6"/>
     </row>
+    <row r="1046">
+      <c r="A1046" s="6"/>
+      <c r="B1046" s="6"/>
+      <c r="C1046" s="6"/>
+      <c r="D1046" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D128">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D129">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A126"/>
+    <hyperlink r:id="rId1" ref="A127"/>
   </hyperlinks>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
global score in profile
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="253">
   <si>
     <t>Key</t>
   </si>
@@ -617,6 +617,12 @@
   </si>
   <si>
     <t>Log out</t>
+  </si>
+  <si>
+    <t>profile.global_score.label</t>
+  </si>
+  <si>
+    <t>Global score</t>
   </si>
   <si>
     <t>header.live</t>
@@ -768,12 +774,36 @@
   <si>
     <t>Tell us more about yourself</t>
   </si>
+  <si>
+    <t>onboarding.personal_info.firstname_title</t>
+  </si>
+  <si>
+    <t>What is your first name ?</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.lastname_title</t>
+  </si>
+  <si>
+    <t>What is your last name ?</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.country_title</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.placeholder.text</t>
+  </si>
+  <si>
+    <t>Type to write</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -788,7 +818,6 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -830,7 +859,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -855,22 +884,16 @@
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1141,11 +1164,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="6"/>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="5" t="s">
@@ -1157,7 +1180,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="6"/>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="7" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -1165,7 +1188,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="6"/>
@@ -1189,7 +1212,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="9" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="6"/>
@@ -1201,7 +1224,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="9" t="s">
         <v>16</v>
       </c>
       <c r="B8" s="6"/>
@@ -1213,7 +1236,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="9" t="s">
         <v>18</v>
       </c>
       <c r="B9" s="6"/>
@@ -1381,7 +1404,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="8" t="s">
         <v>44</v>
       </c>
       <c r="B23" s="6"/>
@@ -1849,24 +1872,24 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="12" t="s">
+      <c r="A62" s="10" t="s">
         <v>109</v>
       </c>
       <c r="C62" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D62" s="12" t="s">
+      <c r="D62" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="12" t="s">
+      <c r="A63" s="10" t="s">
         <v>111</v>
       </c>
       <c r="C63" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D63" s="12" t="s">
+      <c r="D63" s="10" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2015,7 +2038,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="10" t="s">
+      <c r="A76" s="8" t="s">
         <v>137</v>
       </c>
       <c r="B76" s="6"/>
@@ -2027,7 +2050,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="10" t="s">
+      <c r="A77" s="8" t="s">
         <v>139</v>
       </c>
       <c r="B77" s="6"/>
@@ -2519,7 +2542,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="10" t="s">
+      <c r="A118" s="5" t="s">
         <v>219</v>
       </c>
       <c r="B118" s="6"/>
@@ -2531,7 +2554,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="10" t="s">
+      <c r="A119" s="8" t="s">
         <v>221</v>
       </c>
       <c r="B119" s="6"/>
@@ -2543,7 +2566,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="10" t="s">
+      <c r="A120" s="8" t="s">
         <v>223</v>
       </c>
       <c r="B120" s="6"/>
@@ -2555,7 +2578,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="s">
+      <c r="A121" s="8" t="s">
         <v>225</v>
       </c>
       <c r="B121" s="6"/>
@@ -2627,7 +2650,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="13" t="s">
+      <c r="A127" s="5" t="s">
         <v>237</v>
       </c>
       <c r="B127" s="6"/>
@@ -2639,7 +2662,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="5" t="s">
+      <c r="A128" s="11" t="s">
         <v>239</v>
       </c>
       <c r="B128" s="6"/>
@@ -2663,34 +2686,64 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="6"/>
+      <c r="A130" s="5" t="s">
+        <v>243</v>
+      </c>
       <c r="B130" s="6"/>
-      <c r="C130" s="6"/>
-      <c r="D130" s="6"/>
+      <c r="C130" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" s="6"/>
+      <c r="A131" s="5" t="s">
+        <v>245</v>
+      </c>
       <c r="B131" s="6"/>
-      <c r="C131" s="6"/>
-      <c r="D131" s="6"/>
+      <c r="C131" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="6"/>
+      <c r="A132" s="5" t="s">
+        <v>247</v>
+      </c>
       <c r="B132" s="6"/>
-      <c r="C132" s="6"/>
-      <c r="D132" s="6"/>
+      <c r="C132" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D132" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="133">
-      <c r="A133" s="6"/>
+      <c r="A133" s="8" t="s">
+        <v>249</v>
+      </c>
       <c r="B133" s="6"/>
-      <c r="C133" s="6"/>
-      <c r="D133" s="6"/>
+      <c r="C133" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="D133" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="134">
-      <c r="A134" s="6"/>
+      <c r="A134" s="5" t="s">
+        <v>251</v>
+      </c>
       <c r="B134" s="6"/>
-      <c r="C134" s="6"/>
-      <c r="D134" s="6"/>
+      <c r="C134" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="6"/>
@@ -8164,14 +8217,20 @@
       <c r="C1046" s="6"/>
       <c r="D1046" s="6"/>
     </row>
+    <row r="1047">
+      <c r="A1047" s="6"/>
+      <c r="B1047" s="6"/>
+      <c r="C1047" s="6"/>
+      <c r="D1047" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D129">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D134">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A127"/>
+    <hyperlink r:id="rId1" ref="A128"/>
   </hyperlinks>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
Personal Info screen 1 (reuse existing TextField everywhere)
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="253">
   <si>
     <t>Key</t>
   </si>
@@ -773,6 +773,30 @@
   </si>
   <si>
     <t>Tell us more about yourself</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.firstname_title</t>
+  </si>
+  <si>
+    <t>What is your first name ?</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.lastname_title</t>
+  </si>
+  <si>
+    <t>What is your last name ?</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.country_title</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.placeholder.text</t>
+  </si>
+  <si>
+    <t>Type to write</t>
   </si>
 </sst>
 </file>
@@ -2681,28 +2705,52 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="6"/>
+      <c r="A131" s="11" t="s">
+        <v>245</v>
+      </c>
       <c r="B131" s="6"/>
-      <c r="C131" s="6"/>
-      <c r="D131" s="6"/>
+      <c r="C131" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="6"/>
+      <c r="A132" s="11" t="s">
+        <v>247</v>
+      </c>
       <c r="B132" s="6"/>
-      <c r="C132" s="6"/>
-      <c r="D132" s="6"/>
+      <c r="C132" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D132" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="133">
-      <c r="A133" s="6"/>
+      <c r="A133" s="8" t="s">
+        <v>249</v>
+      </c>
       <c r="B133" s="6"/>
-      <c r="C133" s="6"/>
-      <c r="D133" s="6"/>
+      <c r="C133" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="D133" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="134">
-      <c r="A134" s="6"/>
+      <c r="A134" s="11" t="s">
+        <v>251</v>
+      </c>
       <c r="B134" s="6"/>
-      <c r="C134" s="6"/>
-      <c r="D134" s="6"/>
+      <c r="C134" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="6"/>
@@ -8184,7 +8232,7 @@
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D130">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D134">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Personal info 1st page + Base of 2nd page + Country picker + Selectable buttons
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="352">
   <si>
     <t>Key</t>
   </si>
@@ -32,6 +32,24 @@
   </si>
   <si>
     <t>A valider</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>Ok</t>
+  </si>
+  <si>
+    <t>back</t>
+  </si>
+  <si>
+    <t>Back</t>
+  </si>
+  <si>
+    <t>continue</t>
+  </si>
+  <si>
+    <t>Continue</t>
   </si>
   <si>
     <t>setup.scan.disabled.title</t>
@@ -342,9 +360,6 @@
   </si>
   <si>
     <t>global.back</t>
-  </si>
-  <si>
-    <t>Back</t>
   </si>
   <si>
     <t>global.next</t>
@@ -661,6 +676,31 @@
     <t>% of Max HR</t>
   </si>
   <si>
+    <t>live.tutorial.warning</t>
+  </si>
+  <si>
+    <t>Warning: live measurements consume more battery.</t>
+  </si>
+  <si>
+    <t>live.tutorial.accuracy</t>
+  </si>
+  <si>
+    <t>In order to get the most accurate readings, avoid moving your finger. Data accuracy is shown from low to best in red, orange and green.</t>
+  </si>
+  <si>
+    <t>live.tutorial.hide</t>
+  </si>
+  <si>
+    <t>Don’t show this message again</t>
+  </si>
+  <si>
+    <t>live.tutorial.fist</t>
+  </si>
+  <si>
+    <t>First readings will appear after 10 seconds.
+If you do not get data for a little while, don’t worry! To achieve greater live accuracy, try closing your fist as shown above.</t>
+  </si>
+  <si>
     <t>live.start</t>
   </si>
   <si>
@@ -685,6 +725,12 @@
     <t>Blood Ox.</t>
   </si>
   <si>
+    <t>live.disconnected</t>
+  </si>
+  <si>
+    <t>Cannot start live measurements, no ring is currently connected.</t>
+  </si>
+  <si>
     <t>intensity.low</t>
   </si>
   <si>
@@ -737,6 +783,18 @@
   </si>
   <si>
     <t>Add an alarm</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.title</t>
+  </si>
+  <si>
+    <t>Edit Vibration</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.title</t>
+  </si>
+  <si>
+    <t>Repeat</t>
   </si>
   <si>
     <t>onboarding.wear.title</t>
@@ -793,10 +851,250 @@
     <t>Country</t>
   </si>
   <si>
+    <t>onboarding.personal_info.country_placeholder</t>
+  </si>
+  <si>
+    <t>Type to select</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.sex_title</t>
+  </si>
+  <si>
+    <t>What is your sex?</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.sex_female</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.sex_male</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
     <t>onboarding.personal_info.placeholder.text</t>
   </si>
   <si>
     <t>Type to write</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.born_title</t>
+  </si>
+  <si>
+    <t>When are you born?</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.born_placeholder</t>
+  </si>
+  <si>
+    <t>dd/mm/yyyy</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.error.firstname</t>
+  </si>
+  <si>
+    <t>FirstName is required.</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.error.lastname</t>
+  </si>
+  <si>
+    <t>LastName is required.</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.error.country</t>
+  </si>
+  <si>
+    <t>Country is required.</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.intensity</t>
+  </si>
+  <si>
+    <t>Intensity</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.title</t>
+  </si>
+  <si>
+    <t>Vibration type</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.alert</t>
+  </si>
+  <si>
+    <t>Alert (default)</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.heartbeat</t>
+  </si>
+  <si>
+    <t>Heartbeat</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.quick</t>
+  </si>
+  <si>
+    <t>Quick</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.rapid</t>
+  </si>
+  <si>
+    <t>Rapid</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.sos</t>
+  </si>
+  <si>
+    <t>SOS</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.staccato</t>
+  </si>
+  <si>
+    <t>Staccato</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.symphony</t>
+  </si>
+  <si>
+    <t>Symphony</t>
+  </si>
+  <si>
+    <t>alarm.new.save_button</t>
+  </si>
+  <si>
+    <t>Save</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.weekdays</t>
+  </si>
+  <si>
+    <t>Weekdays (default)</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.monday</t>
+  </si>
+  <si>
+    <t>Monday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.tuesday</t>
+  </si>
+  <si>
+    <t>Tuesday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.wednesday</t>
+  </si>
+  <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.thursday</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.friday</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.saturday</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.sunday</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>alarm.new.label.title</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>alarm.new.label.screen_title</t>
+  </si>
+  <si>
+    <t>Enter Label</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.title</t>
+  </si>
+  <si>
+    <t>Snooze</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.screen_title</t>
+  </si>
+  <si>
+    <t>Interval</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.minute</t>
+  </si>
+  <si>
+    <t>minute</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.minutes</t>
+  </si>
+  <si>
+    <t>minutes</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.hour</t>
+  </si>
+  <si>
+    <t>hour</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.off</t>
+  </si>
+  <si>
+    <t>OFF</t>
+  </si>
+  <si>
+    <t>alarm.new.smart_snooze.title</t>
+  </si>
+  <si>
+    <t>Smart Snooze</t>
+  </si>
+  <si>
+    <t>alarm.new.smart_alarm.title</t>
+  </si>
+  <si>
+    <t>Smart Alarm</t>
+  </si>
+  <si>
+    <t>alarm.new.warning.title</t>
+  </si>
+  <si>
+    <t>Warning</t>
+  </si>
+  <si>
+    <t>alarm.new.warning.description</t>
+  </si>
+  <si>
+    <t>You have created too many alarms. Delete an already existing one in order to continue.</t>
+  </si>
+  <si>
+    <t>alarm.new.warning.button</t>
+  </si>
+  <si>
+    <t>OK</t>
   </si>
 </sst>
 </file>
@@ -860,7 +1158,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -902,6 +1200,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1195,12 +1499,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="7" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>6</v>
@@ -1208,42 +1512,42 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="s">
-        <v>14</v>
+      <c r="A7" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="s">
-        <v>16</v>
+      <c r="A8" s="8" t="s">
+        <v>17</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="5" t="s">
         <v>18</v>
       </c>
       <c r="B9" s="6"/>
@@ -1255,7 +1559,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="6"/>
@@ -1267,7 +1571,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B11" s="6"/>
@@ -1279,7 +1583,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B12" s="6"/>
@@ -1308,7 +1612,7 @@
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="7" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>6</v>
@@ -1316,11 +1620,11 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>6</v>
@@ -1328,11 +1632,11 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>6</v>
@@ -1340,11 +1644,11 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="7" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>6</v>
@@ -1404,19 +1708,19 @@
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="s">
-        <v>44</v>
+      <c r="A23" s="5" t="s">
+        <v>45</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="7" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>6</v>
@@ -1424,11 +1728,11 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="7" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>6</v>
@@ -1436,23 +1740,23 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="7" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>48</v>
+      <c r="A26" s="8" t="s">
+        <v>50</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="7" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>6</v>
@@ -1460,11 +1764,11 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="7" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>6</v>
@@ -1472,11 +1776,11 @@
     </row>
     <row r="28">
       <c r="A28" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>6</v>
@@ -1484,11 +1788,11 @@
     </row>
     <row r="29">
       <c r="A29" s="5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="7" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>6</v>
@@ -1496,11 +1800,11 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>6</v>
@@ -1508,11 +1812,11 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>6</v>
@@ -1520,11 +1824,11 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>6</v>
@@ -1532,11 +1836,11 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7" t="s">
-        <v>21</v>
+        <v>59</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>6</v>
@@ -1544,11 +1848,11 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>6</v>
@@ -1556,11 +1860,11 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>6</v>
@@ -1568,11 +1872,11 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>62</v>
+        <v>27</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>6</v>
@@ -1620,7 +1924,7 @@
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="s">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>6</v>
@@ -1628,11 +1932,11 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>6</v>
@@ -1640,11 +1944,11 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>6</v>
@@ -1652,11 +1956,11 @@
     </row>
     <row r="43">
       <c r="A43" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>6</v>
@@ -1752,7 +2056,7 @@
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="7" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>6</v>
@@ -1760,11 +2064,11 @@
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>6</v>
@@ -1772,11 +2076,11 @@
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
-        <v>23</v>
+        <v>95</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>6</v>
@@ -1784,11 +2088,11 @@
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
-        <v>95</v>
+        <v>31</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>6</v>
@@ -1796,11 +2100,11 @@
     </row>
     <row r="55">
       <c r="A55" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="7" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>6</v>
@@ -1808,11 +2112,11 @@
     </row>
     <row r="56">
       <c r="A56" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="7" t="s">
-        <v>98</v>
+        <v>29</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>6</v>
@@ -1820,11 +2124,11 @@
     </row>
     <row r="57">
       <c r="A57" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>6</v>
@@ -1832,11 +2136,11 @@
     </row>
     <row r="58">
       <c r="A58" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -1879,24 +2183,26 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="10" t="s">
+      <c r="A62" s="5" t="s">
         <v>109</v>
       </c>
+      <c r="B62" s="6"/>
       <c r="C62" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D62" s="10" t="s">
+      <c r="D62" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="10" t="s">
+      <c r="A63" s="5" t="s">
         <v>111</v>
       </c>
+      <c r="B63" s="6"/>
       <c r="C63" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D63" s="10" t="s">
+      <c r="D63" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1913,36 +2219,34 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="s">
+      <c r="A65" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="B65" s="6"/>
       <c r="C65" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D65" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="D65" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="s">
+      <c r="C66" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="6"/>
-      <c r="C66" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="D66" s="5" t="s">
+      <c r="D66" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B67" s="6"/>
       <c r="C67" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>6</v>
@@ -1950,11 +2254,11 @@
     </row>
     <row r="68">
       <c r="A68" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>6</v>
@@ -1962,11 +2266,11 @@
     </row>
     <row r="69">
       <c r="A69" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>6</v>
@@ -1974,11 +2278,11 @@
     </row>
     <row r="70">
       <c r="A70" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B70" s="6"/>
       <c r="C70" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D70" s="5" t="s">
         <v>6</v>
@@ -1986,11 +2290,11 @@
     </row>
     <row r="71">
       <c r="A71" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D71" s="5" t="s">
         <v>6</v>
@@ -1998,11 +2302,11 @@
     </row>
     <row r="72">
       <c r="A72" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B72" s="6"/>
       <c r="C72" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>6</v>
@@ -2010,11 +2314,11 @@
     </row>
     <row r="73">
       <c r="A73" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B73" s="6"/>
       <c r="C73" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>6</v>
@@ -2022,11 +2326,11 @@
     </row>
     <row r="74">
       <c r="A74" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B74" s="6"/>
       <c r="C74" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D74" s="5" t="s">
         <v>6</v>
@@ -2034,35 +2338,35 @@
     </row>
     <row r="75">
       <c r="A75" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B75" s="6"/>
       <c r="C75" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="D75" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="s">
-        <v>137</v>
       </c>
       <c r="B76" s="6"/>
       <c r="C76" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="D76" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="s">
         <v>138</v>
-      </c>
-      <c r="D76" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="8" t="s">
-        <v>139</v>
       </c>
       <c r="B77" s="6"/>
       <c r="C77" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D77" s="5" t="s">
         <v>6</v>
@@ -2070,35 +2374,35 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B78" s="6"/>
       <c r="C78" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D78" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="s">
         <v>142</v>
-      </c>
-      <c r="D78" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="5" t="s">
-        <v>143</v>
       </c>
       <c r="B79" s="6"/>
       <c r="C79" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="s">
         <v>144</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="5" t="s">
-        <v>145</v>
       </c>
       <c r="B80" s="6"/>
       <c r="C80" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D80" s="5" t="s">
         <v>6</v>
@@ -2106,11 +2410,11 @@
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B81" s="6"/>
       <c r="C81" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>6</v>
@@ -2118,11 +2422,11 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B82" s="6"/>
       <c r="C82" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>6</v>
@@ -2130,11 +2434,11 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B83" s="6"/>
       <c r="C83" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>6</v>
@@ -2142,11 +2446,11 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B84" s="6"/>
       <c r="C84" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>6</v>
@@ -2154,11 +2458,11 @@
     </row>
     <row r="85">
       <c r="A85" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B85" s="6"/>
       <c r="C85" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>6</v>
@@ -2166,11 +2470,11 @@
     </row>
     <row r="86">
       <c r="A86" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B86" s="6"/>
       <c r="C86" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>6</v>
@@ -2178,11 +2482,11 @@
     </row>
     <row r="87">
       <c r="A87" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B87" s="6"/>
       <c r="C87" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D87" s="5" t="s">
         <v>6</v>
@@ -2190,11 +2494,11 @@
     </row>
     <row r="88">
       <c r="A88" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B88" s="6"/>
       <c r="C88" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>6</v>
@@ -2202,11 +2506,11 @@
     </row>
     <row r="89">
       <c r="A89" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B89" s="6"/>
       <c r="C89" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D89" s="5" t="s">
         <v>6</v>
@@ -2214,11 +2518,11 @@
     </row>
     <row r="90">
       <c r="A90" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B90" s="6"/>
       <c r="C90" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D90" s="5" t="s">
         <v>6</v>
@@ -2226,11 +2530,11 @@
     </row>
     <row r="91">
       <c r="A91" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B91" s="6"/>
       <c r="C91" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D91" s="5" t="s">
         <v>6</v>
@@ -2238,11 +2542,11 @@
     </row>
     <row r="92">
       <c r="A92" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B92" s="6"/>
       <c r="C92" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D92" s="5" t="s">
         <v>6</v>
@@ -2250,11 +2554,11 @@
     </row>
     <row r="93">
       <c r="A93" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B93" s="6"/>
       <c r="C93" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>6</v>
@@ -2262,11 +2566,11 @@
     </row>
     <row r="94">
       <c r="A94" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B94" s="6"/>
       <c r="C94" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D94" s="5" t="s">
         <v>6</v>
@@ -2274,11 +2578,11 @@
     </row>
     <row r="95">
       <c r="A95" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B95" s="6"/>
       <c r="C95" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D95" s="5" t="s">
         <v>6</v>
@@ -2286,11 +2590,11 @@
     </row>
     <row r="96">
       <c r="A96" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B96" s="6"/>
       <c r="C96" s="7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D96" s="5" t="s">
         <v>6</v>
@@ -2298,11 +2602,11 @@
     </row>
     <row r="97">
       <c r="A97" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B97" s="6"/>
       <c r="C97" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D97" s="5" t="s">
         <v>6</v>
@@ -2310,11 +2614,11 @@
     </row>
     <row r="98">
       <c r="A98" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B98" s="6"/>
       <c r="C98" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D98" s="5" t="s">
         <v>6</v>
@@ -2322,11 +2626,11 @@
     </row>
     <row r="99">
       <c r="A99" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B99" s="6"/>
       <c r="C99" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>6</v>
@@ -2334,11 +2638,11 @@
     </row>
     <row r="100">
       <c r="A100" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>6</v>
@@ -2346,11 +2650,11 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B101" s="6"/>
       <c r="C101" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>6</v>
@@ -2358,11 +2662,11 @@
     </row>
     <row r="102">
       <c r="A102" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B102" s="6"/>
       <c r="C102" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>6</v>
@@ -2370,11 +2674,11 @@
     </row>
     <row r="103">
       <c r="A103" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B103" s="6"/>
       <c r="C103" s="7" t="s">
-        <v>25</v>
+        <v>191</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>6</v>
@@ -2386,7 +2690,7 @@
       </c>
       <c r="B104" s="6"/>
       <c r="C104" s="7" t="s">
-        <v>25</v>
+        <v>193</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>6</v>
@@ -2394,11 +2698,11 @@
     </row>
     <row r="105">
       <c r="A105" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="7" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D105" s="5" t="s">
         <v>6</v>
@@ -2406,23 +2710,23 @@
     </row>
     <row r="106">
       <c r="A106" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B106" s="6"/>
       <c r="C106" s="7" t="s">
-        <v>196</v>
+        <v>31</v>
       </c>
       <c r="D106" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="11" t="s">
+      <c r="A107" s="5" t="s">
         <v>197</v>
       </c>
       <c r="B107" s="6"/>
-      <c r="C107" s="12" t="s">
-        <v>198</v>
+      <c r="C107" s="7" t="s">
+        <v>31</v>
       </c>
       <c r="D107" s="5" t="s">
         <v>6</v>
@@ -2430,11 +2734,11 @@
     </row>
     <row r="108">
       <c r="A108" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B108" s="6"/>
       <c r="C108" s="7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D108" s="5" t="s">
         <v>6</v>
@@ -2442,11 +2746,11 @@
     </row>
     <row r="109">
       <c r="A109" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B109" s="6"/>
       <c r="C109" s="7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>6</v>
@@ -2454,11 +2758,11 @@
     </row>
     <row r="110">
       <c r="A110" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B110" s="6"/>
       <c r="C110" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>6</v>
@@ -2466,11 +2770,11 @@
     </row>
     <row r="111">
       <c r="A111" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B111" s="6"/>
       <c r="C111" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>6</v>
@@ -2478,11 +2782,11 @@
     </row>
     <row r="112">
       <c r="A112" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B112" s="6"/>
       <c r="C112" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>6</v>
@@ -2490,11 +2794,11 @@
     </row>
     <row r="113">
       <c r="A113" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B113" s="6"/>
       <c r="C113" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>6</v>
@@ -2502,11 +2806,11 @@
     </row>
     <row r="114">
       <c r="A114" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B114" s="6"/>
       <c r="C114" s="7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>6</v>
@@ -2514,11 +2818,11 @@
     </row>
     <row r="115">
       <c r="A115" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B115" s="6"/>
       <c r="C115" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>6</v>
@@ -2526,11 +2830,11 @@
     </row>
     <row r="116">
       <c r="A116" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B116" s="6"/>
       <c r="C116" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D116" s="5" t="s">
         <v>6</v>
@@ -2538,11 +2842,11 @@
     </row>
     <row r="117">
       <c r="A117" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B117" s="6"/>
       <c r="C117" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>6</v>
@@ -2550,47 +2854,47 @@
     </row>
     <row r="118">
       <c r="A118" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B118" s="6"/>
       <c r="C118" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="s">
         <v>220</v>
-      </c>
-      <c r="D118" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="8" t="s">
-        <v>221</v>
       </c>
       <c r="B119" s="6"/>
       <c r="C119" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="s">
         <v>222</v>
-      </c>
-      <c r="D119" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="8" t="s">
-        <v>223</v>
       </c>
       <c r="B120" s="6"/>
       <c r="C120" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="s">
         <v>224</v>
-      </c>
-      <c r="D120" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="8" t="s">
-        <v>225</v>
       </c>
       <c r="B121" s="6"/>
       <c r="C121" s="7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>6</v>
@@ -2598,11 +2902,11 @@
     </row>
     <row r="122">
       <c r="A122" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B122" s="6"/>
       <c r="C122" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>6</v>
@@ -2610,11 +2914,11 @@
     </row>
     <row r="123">
       <c r="A123" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B123" s="6"/>
       <c r="C123" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>6</v>
@@ -2622,11 +2926,11 @@
     </row>
     <row r="124">
       <c r="A124" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -2634,11 +2938,11 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>6</v>
@@ -2646,47 +2950,47 @@
     </row>
     <row r="126">
       <c r="A126" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B126" s="6"/>
       <c r="C126" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="8" t="s">
         <v>236</v>
-      </c>
-      <c r="D126" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="5" t="s">
-        <v>237</v>
       </c>
       <c r="B127" s="6"/>
       <c r="C127" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="8" t="s">
         <v>238</v>
-      </c>
-      <c r="D127" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="13" t="s">
-        <v>239</v>
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="s">
         <v>240</v>
-      </c>
-      <c r="D128" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="5" t="s">
-        <v>241</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D129" s="5" t="s">
         <v>6</v>
@@ -2694,363 +2998,663 @@
     </row>
     <row r="130">
       <c r="A130" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B130" s="6"/>
       <c r="C130" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="D130" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="11" t="s">
+      <c r="B131" s="6"/>
+      <c r="C131" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="B131" s="6"/>
-      <c r="C131" s="12" t="s">
+      <c r="D131" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="D131" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="11" t="s">
+      <c r="B132" s="6"/>
+      <c r="C132" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="B132" s="6"/>
-      <c r="C132" s="12" t="s">
+      <c r="D132" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="D132" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="8" t="s">
+      <c r="B133" s="6"/>
+      <c r="C133" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="B133" s="6"/>
-      <c r="C133" s="12" t="s">
+      <c r="D133" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="D133" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="11" t="s">
+      <c r="B134" s="6"/>
+      <c r="C134" s="7" t="s">
         <v>251</v>
       </c>
-      <c r="B134" s="6"/>
-      <c r="C134" s="12" t="s">
+      <c r="D134" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="11" t="s">
         <v>252</v>
       </c>
-      <c r="D134" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="6"/>
       <c r="B135" s="6"/>
-      <c r="C135" s="6"/>
-      <c r="D135" s="6"/>
+      <c r="C135" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="136">
-      <c r="A136" s="6"/>
+      <c r="A136" s="11" t="s">
+        <v>254</v>
+      </c>
       <c r="B136" s="6"/>
-      <c r="C136" s="6"/>
-      <c r="D136" s="6"/>
+      <c r="C136" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="D136" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="137">
-      <c r="A137" s="6"/>
+      <c r="A137" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="B137" s="6"/>
-      <c r="C137" s="6"/>
-      <c r="D137" s="6"/>
+      <c r="C137" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="D137" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="138">
-      <c r="A138" s="6"/>
+      <c r="A138" s="13" t="s">
+        <v>258</v>
+      </c>
       <c r="B138" s="6"/>
-      <c r="C138" s="6"/>
-      <c r="D138" s="6"/>
+      <c r="C138" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="D138" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="139">
-      <c r="A139" s="6"/>
+      <c r="A139" s="5" t="s">
+        <v>260</v>
+      </c>
       <c r="B139" s="6"/>
-      <c r="C139" s="6"/>
-      <c r="D139" s="6"/>
+      <c r="C139" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="D139" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="140">
-      <c r="A140" s="6"/>
+      <c r="A140" s="5" t="s">
+        <v>262</v>
+      </c>
       <c r="B140" s="6"/>
-      <c r="C140" s="6"/>
-      <c r="D140" s="6"/>
+      <c r="C140" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="D140" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="141">
-      <c r="A141" s="6"/>
+      <c r="A141" s="5" t="s">
+        <v>264</v>
+      </c>
       <c r="B141" s="6"/>
-      <c r="C141" s="6"/>
-      <c r="D141" s="6"/>
+      <c r="C141" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="D141" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="142">
-      <c r="A142" s="6"/>
+      <c r="A142" s="5" t="s">
+        <v>266</v>
+      </c>
       <c r="B142" s="6"/>
-      <c r="C142" s="6"/>
-      <c r="D142" s="6"/>
+      <c r="C142" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="D142" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="143">
-      <c r="A143" s="6"/>
+      <c r="A143" s="8" t="s">
+        <v>268</v>
+      </c>
       <c r="B143" s="6"/>
-      <c r="C143" s="6"/>
-      <c r="D143" s="6"/>
+      <c r="C143" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="144">
-      <c r="A144" s="6"/>
+      <c r="A144" s="11" t="s">
+        <v>270</v>
+      </c>
       <c r="B144" s="6"/>
-      <c r="C144" s="6"/>
-      <c r="D144" s="6"/>
+      <c r="C144" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="D144" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="145">
-      <c r="A145" s="6"/>
+      <c r="A145" s="11" t="s">
+        <v>272</v>
+      </c>
       <c r="B145" s="6"/>
-      <c r="C145" s="6"/>
-      <c r="D145" s="6"/>
+      <c r="C145" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="D145" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="146">
-      <c r="A146" s="6"/>
+      <c r="A146" s="11" t="s">
+        <v>274</v>
+      </c>
       <c r="B146" s="6"/>
-      <c r="C146" s="6"/>
-      <c r="D146" s="6"/>
+      <c r="C146" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="D146" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="147">
-      <c r="A147" s="6"/>
+      <c r="A147" s="11" t="s">
+        <v>276</v>
+      </c>
       <c r="B147" s="6"/>
-      <c r="C147" s="6"/>
-      <c r="D147" s="6"/>
+      <c r="C147" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="D147" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="148">
-      <c r="A148" s="6"/>
+      <c r="A148" s="5" t="s">
+        <v>278</v>
+      </c>
       <c r="B148" s="6"/>
-      <c r="C148" s="6"/>
-      <c r="D148" s="6"/>
+      <c r="C148" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="D148" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="149">
-      <c r="A149" s="6"/>
+      <c r="A149" s="11" t="s">
+        <v>280</v>
+      </c>
       <c r="B149" s="6"/>
-      <c r="C149" s="6"/>
-      <c r="D149" s="6"/>
+      <c r="C149" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="D149" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="150">
-      <c r="A150" s="6"/>
+      <c r="A150" s="11" t="s">
+        <v>282</v>
+      </c>
       <c r="B150" s="6"/>
-      <c r="C150" s="6"/>
-      <c r="D150" s="6"/>
+      <c r="C150" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="D150" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="151">
-      <c r="A151" s="6"/>
+      <c r="A151" s="11" t="s">
+        <v>284</v>
+      </c>
       <c r="B151" s="6"/>
-      <c r="C151" s="6"/>
-      <c r="D151" s="6"/>
+      <c r="C151" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="D151" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="152">
-      <c r="A152" s="6"/>
+      <c r="A152" s="11" t="s">
+        <v>286</v>
+      </c>
       <c r="B152" s="6"/>
-      <c r="C152" s="6"/>
-      <c r="D152" s="6"/>
+      <c r="C152" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="D152" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="153">
-      <c r="A153" s="6"/>
+      <c r="A153" s="11" t="s">
+        <v>288</v>
+      </c>
       <c r="B153" s="6"/>
-      <c r="C153" s="6"/>
-      <c r="D153" s="6"/>
+      <c r="C153" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="D153" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="154">
-      <c r="A154" s="6"/>
+      <c r="A154" s="11" t="s">
+        <v>290</v>
+      </c>
       <c r="B154" s="6"/>
-      <c r="C154" s="6"/>
-      <c r="D154" s="6"/>
+      <c r="C154" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="D154" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="155">
-      <c r="A155" s="6"/>
+      <c r="A155" s="11" t="s">
+        <v>292</v>
+      </c>
       <c r="B155" s="6"/>
-      <c r="C155" s="6"/>
-      <c r="D155" s="6"/>
+      <c r="C155" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="D155" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="156">
-      <c r="A156" s="6"/>
+      <c r="A156" s="11" t="s">
+        <v>294</v>
+      </c>
       <c r="B156" s="6"/>
-      <c r="C156" s="6"/>
-      <c r="D156" s="6"/>
+      <c r="C156" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="D156" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="157">
-      <c r="A157" s="6"/>
+      <c r="A157" s="14" t="s">
+        <v>296</v>
+      </c>
       <c r="B157" s="6"/>
-      <c r="C157" s="6"/>
-      <c r="D157" s="6"/>
+      <c r="C157" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="D157" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="158">
-      <c r="A158" s="6"/>
+      <c r="A158" s="14" t="s">
+        <v>298</v>
+      </c>
       <c r="B158" s="6"/>
-      <c r="C158" s="6"/>
-      <c r="D158" s="6"/>
+      <c r="C158" s="12" t="s">
+        <v>299</v>
+      </c>
+      <c r="D158" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="159">
-      <c r="A159" s="6"/>
+      <c r="A159" s="14" t="s">
+        <v>300</v>
+      </c>
       <c r="B159" s="6"/>
-      <c r="C159" s="6"/>
-      <c r="D159" s="6"/>
+      <c r="C159" s="12" t="s">
+        <v>301</v>
+      </c>
+      <c r="D159" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="160">
-      <c r="A160" s="6"/>
-      <c r="B160" s="6"/>
-      <c r="C160" s="6"/>
-      <c r="D160" s="6"/>
+      <c r="A160" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="B160" s="15"/>
+      <c r="C160" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="D160" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="161">
-      <c r="A161" s="6"/>
+      <c r="A161" s="14" t="s">
+        <v>304</v>
+      </c>
       <c r="B161" s="6"/>
-      <c r="C161" s="6"/>
-      <c r="D161" s="6"/>
+      <c r="C161" s="12" t="s">
+        <v>305</v>
+      </c>
+      <c r="D161" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="162">
-      <c r="A162" s="6"/>
+      <c r="A162" s="14" t="s">
+        <v>306</v>
+      </c>
       <c r="B162" s="6"/>
-      <c r="C162" s="6"/>
-      <c r="D162" s="6"/>
+      <c r="C162" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="D162" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="163">
-      <c r="A163" s="6"/>
+      <c r="A163" s="11" t="s">
+        <v>308</v>
+      </c>
       <c r="B163" s="6"/>
-      <c r="C163" s="6"/>
-      <c r="D163" s="6"/>
+      <c r="C163" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="D163" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="164">
-      <c r="A164" s="6"/>
+      <c r="A164" s="11" t="s">
+        <v>310</v>
+      </c>
       <c r="B164" s="6"/>
-      <c r="C164" s="6"/>
-      <c r="D164" s="6"/>
+      <c r="C164" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="D164" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="165">
-      <c r="A165" s="6"/>
+      <c r="A165" s="11" t="s">
+        <v>312</v>
+      </c>
       <c r="B165" s="6"/>
-      <c r="C165" s="6"/>
-      <c r="D165" s="6"/>
+      <c r="C165" s="12" t="s">
+        <v>313</v>
+      </c>
+      <c r="D165" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="166">
-      <c r="A166" s="6"/>
+      <c r="A166" s="11" t="s">
+        <v>314</v>
+      </c>
       <c r="B166" s="6"/>
-      <c r="C166" s="6"/>
-      <c r="D166" s="6"/>
+      <c r="C166" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="D166" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="167">
-      <c r="A167" s="6"/>
+      <c r="A167" s="11" t="s">
+        <v>316</v>
+      </c>
       <c r="B167" s="6"/>
-      <c r="C167" s="6"/>
-      <c r="D167" s="6"/>
+      <c r="C167" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="D167" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="168">
-      <c r="A168" s="6"/>
+      <c r="A168" s="11" t="s">
+        <v>318</v>
+      </c>
       <c r="B168" s="6"/>
-      <c r="C168" s="6"/>
-      <c r="D168" s="6"/>
+      <c r="C168" s="12" t="s">
+        <v>319</v>
+      </c>
+      <c r="D168" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="169">
-      <c r="A169" s="6"/>
+      <c r="A169" s="11" t="s">
+        <v>320</v>
+      </c>
       <c r="B169" s="6"/>
-      <c r="C169" s="6"/>
-      <c r="D169" s="6"/>
+      <c r="C169" s="12" t="s">
+        <v>321</v>
+      </c>
+      <c r="D169" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="170">
-      <c r="A170" s="6"/>
+      <c r="A170" s="11" t="s">
+        <v>322</v>
+      </c>
       <c r="B170" s="6"/>
-      <c r="C170" s="6"/>
-      <c r="D170" s="6"/>
+      <c r="C170" s="12" t="s">
+        <v>323</v>
+      </c>
+      <c r="D170" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="171">
-      <c r="A171" s="6"/>
+      <c r="A171" s="11" t="s">
+        <v>324</v>
+      </c>
       <c r="B171" s="6"/>
-      <c r="C171" s="6"/>
-      <c r="D171" s="6"/>
+      <c r="C171" s="12" t="s">
+        <v>325</v>
+      </c>
+      <c r="D171" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="172">
-      <c r="A172" s="6"/>
+      <c r="A172" s="11" t="s">
+        <v>326</v>
+      </c>
       <c r="B172" s="6"/>
-      <c r="C172" s="6"/>
-      <c r="D172" s="6"/>
+      <c r="C172" s="12" t="s">
+        <v>327</v>
+      </c>
+      <c r="D172" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="173">
-      <c r="A173" s="6"/>
+      <c r="A173" s="11" t="s">
+        <v>328</v>
+      </c>
       <c r="B173" s="6"/>
-      <c r="C173" s="6"/>
-      <c r="D173" s="6"/>
+      <c r="C173" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="D173" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="174">
-      <c r="A174" s="6"/>
+      <c r="A174" s="11" t="s">
+        <v>330</v>
+      </c>
       <c r="B174" s="6"/>
-      <c r="C174" s="6"/>
-      <c r="D174" s="6"/>
+      <c r="C174" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="D174" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="175">
-      <c r="A175" s="6"/>
+      <c r="A175" s="11" t="s">
+        <v>332</v>
+      </c>
       <c r="B175" s="6"/>
-      <c r="C175" s="6"/>
-      <c r="D175" s="6"/>
+      <c r="C175" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="D175" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="176">
-      <c r="A176" s="6"/>
+      <c r="A176" s="11" t="s">
+        <v>334</v>
+      </c>
       <c r="B176" s="6"/>
-      <c r="C176" s="6"/>
-      <c r="D176" s="6"/>
+      <c r="C176" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="D176" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="177">
-      <c r="A177" s="6"/>
+      <c r="A177" s="11" t="s">
+        <v>336</v>
+      </c>
       <c r="B177" s="6"/>
-      <c r="C177" s="6"/>
-      <c r="D177" s="6"/>
+      <c r="C177" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="D177" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="178">
-      <c r="A178" s="6"/>
+      <c r="A178" s="11" t="s">
+        <v>338</v>
+      </c>
       <c r="B178" s="6"/>
-      <c r="C178" s="6"/>
-      <c r="D178" s="6"/>
+      <c r="C178" s="12" t="s">
+        <v>339</v>
+      </c>
+      <c r="D178" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="179">
-      <c r="A179" s="6"/>
+      <c r="A179" s="11" t="s">
+        <v>340</v>
+      </c>
       <c r="B179" s="6"/>
-      <c r="C179" s="6"/>
-      <c r="D179" s="6"/>
+      <c r="C179" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="D179" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="180">
-      <c r="A180" s="6"/>
+      <c r="A180" s="11" t="s">
+        <v>342</v>
+      </c>
       <c r="B180" s="6"/>
-      <c r="C180" s="6"/>
-      <c r="D180" s="6"/>
+      <c r="C180" s="12" t="s">
+        <v>343</v>
+      </c>
+      <c r="D180" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="181">
-      <c r="A181" s="6"/>
+      <c r="A181" s="11" t="s">
+        <v>344</v>
+      </c>
       <c r="B181" s="6"/>
-      <c r="C181" s="6"/>
-      <c r="D181" s="6"/>
+      <c r="C181" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="D181" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="182">
-      <c r="A182" s="6"/>
+      <c r="A182" s="11" t="s">
+        <v>346</v>
+      </c>
       <c r="B182" s="6"/>
-      <c r="C182" s="6"/>
-      <c r="D182" s="6"/>
+      <c r="C182" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="D182" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="183">
-      <c r="A183" s="6"/>
+      <c r="A183" s="11" t="s">
+        <v>348</v>
+      </c>
       <c r="B183" s="6"/>
-      <c r="C183" s="6"/>
-      <c r="D183" s="6"/>
+      <c r="C183" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="D183" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="184">
-      <c r="A184" s="6"/>
+      <c r="A184" s="11" t="s">
+        <v>350</v>
+      </c>
       <c r="B184" s="6"/>
-      <c r="C184" s="6"/>
-      <c r="D184" s="6"/>
+      <c r="C184" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="D184" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="6"/>
@@ -8230,14 +8834,128 @@
       <c r="C1047" s="6"/>
       <c r="D1047" s="6"/>
     </row>
+    <row r="1048">
+      <c r="A1048" s="6"/>
+      <c r="B1048" s="6"/>
+      <c r="C1048" s="6"/>
+      <c r="D1048" s="6"/>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="6"/>
+      <c r="B1049" s="6"/>
+      <c r="C1049" s="6"/>
+      <c r="D1049" s="6"/>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="6"/>
+      <c r="B1050" s="6"/>
+      <c r="C1050" s="6"/>
+      <c r="D1050" s="6"/>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="6"/>
+      <c r="B1051" s="6"/>
+      <c r="C1051" s="6"/>
+      <c r="D1051" s="6"/>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="6"/>
+      <c r="B1052" s="6"/>
+      <c r="C1052" s="6"/>
+      <c r="D1052" s="6"/>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="6"/>
+      <c r="B1053" s="6"/>
+      <c r="C1053" s="6"/>
+      <c r="D1053" s="6"/>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="6"/>
+      <c r="B1054" s="6"/>
+      <c r="C1054" s="6"/>
+      <c r="D1054" s="6"/>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="6"/>
+      <c r="B1055" s="6"/>
+      <c r="C1055" s="6"/>
+      <c r="D1055" s="6"/>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="6"/>
+      <c r="B1056" s="6"/>
+      <c r="C1056" s="6"/>
+      <c r="D1056" s="6"/>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="6"/>
+      <c r="B1057" s="6"/>
+      <c r="C1057" s="6"/>
+      <c r="D1057" s="6"/>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="6"/>
+      <c r="B1058" s="6"/>
+      <c r="C1058" s="6"/>
+      <c r="D1058" s="6"/>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="6"/>
+      <c r="B1059" s="6"/>
+      <c r="C1059" s="6"/>
+      <c r="D1059" s="6"/>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="6"/>
+      <c r="B1060" s="6"/>
+      <c r="C1060" s="6"/>
+      <c r="D1060" s="6"/>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="6"/>
+      <c r="B1061" s="6"/>
+      <c r="C1061" s="6"/>
+      <c r="D1061" s="6"/>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="6"/>
+      <c r="B1062" s="6"/>
+      <c r="C1062" s="6"/>
+      <c r="D1062" s="6"/>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="6"/>
+      <c r="B1063" s="6"/>
+      <c r="C1063" s="6"/>
+      <c r="D1063" s="6"/>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="6"/>
+      <c r="B1064" s="6"/>
+      <c r="C1064" s="6"/>
+      <c r="D1064" s="6"/>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="6"/>
+      <c r="B1065" s="6"/>
+      <c r="C1065" s="6"/>
+      <c r="D1065" s="6"/>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="6"/>
+      <c r="B1066" s="6"/>
+      <c r="C1066" s="6"/>
+      <c r="D1066" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D134">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D184">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A128"/>
+    <hyperlink r:id="rId1" ref="A138"/>
   </hyperlinks>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
WIP alarm and new alarm screen
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="360">
   <si>
     <t>Key</t>
   </si>
@@ -34,16 +34,37 @@
     <t>A valider</t>
   </si>
   <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>Ok</t>
+  </si>
+  <si>
+    <t>back</t>
+  </si>
+  <si>
+    <t>Back</t>
+  </si>
+  <si>
+    <t>continue</t>
+  </si>
+  <si>
+    <t>Continue</t>
+  </si>
+  <si>
+    <t>setup.scan.disabled.title</t>
+  </si>
+  <si>
+    <t>Enable bluetooth</t>
+  </si>
+  <si>
     <t>setup.scan.disabled.message</t>
   </si>
   <si>
-    <t>To proceed, please enable the bluetooth on you phone</t>
+    <t>Make sure that your Bluetooth is enabled on your phone to begin pairing with a Circular ring and that you have your ring close to your phone.</t>
   </si>
   <si>
     <t>setup.scan.disabled.enable</t>
-  </si>
-  <si>
-    <t>Enable bluetooth</t>
   </si>
   <si>
     <t>setup.scan.enabled.title</t>
@@ -272,7 +293,7 @@
     <t>forgot_password.reset.title</t>
   </si>
   <si>
-    <t>Pasword Reset</t>
+    <t>Password Reset</t>
   </si>
   <si>
     <t>forgot_password.reset.description</t>
@@ -323,10 +344,13 @@
     <t>forgot_password.new.password</t>
   </si>
   <si>
+    <t>New password</t>
+  </si>
+  <si>
     <t>forgot_password.new.confirm_password</t>
   </si>
   <si>
-    <t>Confim password</t>
+    <t>Confim new password</t>
   </si>
   <si>
     <t>forgot_password.new.button</t>
@@ -336,9 +360,6 @@
   </si>
   <si>
     <t>global.back</t>
-  </si>
-  <si>
-    <t>Back</t>
   </si>
   <si>
     <t>global.next</t>
@@ -613,6 +634,12 @@
     <t>Log out</t>
   </si>
   <si>
+    <t>profile.global_score.label</t>
+  </si>
+  <si>
+    <t>Global score</t>
+  </si>
+  <si>
     <t>header.live</t>
   </si>
   <si>
@@ -649,6 +676,31 @@
     <t>% of Max HR</t>
   </si>
   <si>
+    <t>live.tutorial.warning</t>
+  </si>
+  <si>
+    <t>Warning: live measurements consume more battery.</t>
+  </si>
+  <si>
+    <t>live.tutorial.accuracy</t>
+  </si>
+  <si>
+    <t>In order to get the most accurate readings, avoid moving your finger. Data accuracy is shown from low to best in red, orange and green.</t>
+  </si>
+  <si>
+    <t>live.tutorial.hide</t>
+  </si>
+  <si>
+    <t>Don’t show this message again</t>
+  </si>
+  <si>
+    <t>live.tutorial.fist</t>
+  </si>
+  <si>
+    <t>First readings will appear after 10 seconds.
+If you do not get data for a little while, don’t worry! To achieve greater live accuracy, try closing your fist as shown above.</t>
+  </si>
+  <si>
     <t>live.start</t>
   </si>
   <si>
@@ -673,6 +725,36 @@
     <t>Blood Ox.</t>
   </si>
   <si>
+    <t>live.disconnected</t>
+  </si>
+  <si>
+    <t>Cannot start live measurements, no ring is currently connected.</t>
+  </si>
+  <si>
+    <t>intensity.low</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>intensity.medium</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>intensity.high</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>intensity.none</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>drawer.profile</t>
   </si>
   <si>
@@ -701,13 +783,349 @@
   </si>
   <si>
     <t>Add an alarm</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.title</t>
+  </si>
+  <si>
+    <t>Edit Vibration</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.title</t>
+  </si>
+  <si>
+    <t>Repeat</t>
+  </si>
+  <si>
+    <t>onboarding.wear.title</t>
+  </si>
+  <si>
+    <t>How to wear Circular</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>onboarding.wear.info</t>
+    </r>
+    <r>
+      <rPr/>
+      <t>.top</t>
+    </r>
+  </si>
+  <si>
+    <t>The best fingers to wear Circular are the &lt;colored&gt;index&lt;/colored&gt;, &lt;colored&gt;middle finger&lt;/colored&gt;, &lt;colored&gt;ring finger&lt;/colored&gt;, pinky finger and thumb.
+Try as much as possible to use the same finger and same ring positioning each time you wear your Circular.</t>
+  </si>
+  <si>
+    <t>onboarding.wear.info.bottom</t>
+  </si>
+  <si>
+    <t>The flat part of the ring should be on the &lt;colored&gt;palmar side&lt;/colored&gt; of your finger.
+The button should be &lt;colored&gt;facing your thumb&lt;/colored&gt;, for ease of use.</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.title</t>
+  </si>
+  <si>
+    <t>Tell us more about yourself</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.firstname_title</t>
+  </si>
+  <si>
+    <t>What is your first name ?</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.lastname_title</t>
+  </si>
+  <si>
+    <t>What is your last name ?</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.country_title</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.country_placeholder</t>
+  </si>
+  <si>
+    <t>Type to select</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.sex_title</t>
+  </si>
+  <si>
+    <t>What is your sex?</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.sex_female</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.sex_male</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.placeholder.text</t>
+  </si>
+  <si>
+    <t>Type to write</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.born_title</t>
+  </si>
+  <si>
+    <t>When are you born?</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.born_placeholder</t>
+  </si>
+  <si>
+    <t>dd/mm/yyyy</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.weight_title</t>
+  </si>
+  <si>
+    <t>Select your weight</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.height_title</t>
+  </si>
+  <si>
+    <t>Select your height</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.error.firstname</t>
+  </si>
+  <si>
+    <t>FirstName is required.</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.error.lastname</t>
+  </si>
+  <si>
+    <t>LastName is required.</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.error.country</t>
+  </si>
+  <si>
+    <t>Country is required.</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.intensity</t>
+  </si>
+  <si>
+    <t>Intensity</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.title</t>
+  </si>
+  <si>
+    <t>Vibration type</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.alert_default</t>
+  </si>
+  <si>
+    <t>Alert (default)</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.heartbeat</t>
+  </si>
+  <si>
+    <t>Heartbeat</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.quick</t>
+  </si>
+  <si>
+    <t>Quick</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.rapid</t>
+  </si>
+  <si>
+    <t>Rapid</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.sos</t>
+  </si>
+  <si>
+    <t>SOS</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.staccato</t>
+  </si>
+  <si>
+    <t>Staccato</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.symphony</t>
+  </si>
+  <si>
+    <t>Symphony</t>
+  </si>
+  <si>
+    <t>alarm.new.save_button</t>
+  </si>
+  <si>
+    <t>Save</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.weekdays</t>
+  </si>
+  <si>
+    <t>Weekdays (default)</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.monday</t>
+  </si>
+  <si>
+    <t>Monday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.tuesday</t>
+  </si>
+  <si>
+    <t>Tuesday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.wednesday</t>
+  </si>
+  <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.thursday</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.friday</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.saturday</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.sunday</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>alarm.new.label.title</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>alarm.new.label.screen_title</t>
+  </si>
+  <si>
+    <t>Enter Label</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.title</t>
+  </si>
+  <si>
+    <t>Snooze</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.screen_title</t>
+  </si>
+  <si>
+    <t>Interval</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.minute</t>
+  </si>
+  <si>
+    <t>minute</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.minutes</t>
+  </si>
+  <si>
+    <t>minutes</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.hour</t>
+  </si>
+  <si>
+    <t>hour</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.off</t>
+  </si>
+  <si>
+    <t>OFF</t>
+  </si>
+  <si>
+    <t>alarm.new.smart_snooze.title</t>
+  </si>
+  <si>
+    <t>Smart Snooze</t>
+  </si>
+  <si>
+    <t>alarm.new.smart_alarm.title</t>
+  </si>
+  <si>
+    <t>Smart Alarm</t>
+  </si>
+  <si>
+    <t>alarm.new.warning.title</t>
+  </si>
+  <si>
+    <t>Warning</t>
+  </si>
+  <si>
+    <t>alarm.new.warning.description</t>
+  </si>
+  <si>
+    <t>You have created too many alarms. Delete an already existing one in order to continue.</t>
+  </si>
+  <si>
+    <t>alarm.new.warning.button</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>alarm.new.other.title</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.alert</t>
+  </si>
+  <si>
+    <t>Alert</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -725,6 +1143,10 @@
     <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
     <font/>
   </fonts>
@@ -760,7 +1182,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -797,7 +1219,10 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1080,7 +1505,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="6"/>
@@ -1104,7 +1529,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="6"/>
@@ -1116,7 +1541,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="6"/>
@@ -1128,12 +1553,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>17</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="7" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>6</v>
@@ -1141,47 +1566,47 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>21</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>23</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="s">
         <v>24</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>25</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>6</v>
@@ -1189,11 +1614,11 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>6</v>
@@ -1241,7 +1666,7 @@
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="7" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>6</v>
@@ -1249,11 +1674,11 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>6</v>
@@ -1261,11 +1686,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>6</v>
@@ -1273,11 +1698,11 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>6</v>
@@ -1285,23 +1710,23 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="7" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="5" t="s">
         <v>43</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>6</v>
@@ -1309,11 +1734,11 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="7" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>6</v>
@@ -1321,11 +1746,11 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>6</v>
@@ -1333,23 +1758,23 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="7" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>48</v>
+      <c r="A26" s="8" t="s">
+        <v>50</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="7" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>6</v>
@@ -1357,11 +1782,11 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="7" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>6</v>
@@ -1369,11 +1794,11 @@
     </row>
     <row r="28">
       <c r="A28" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>6</v>
@@ -1381,11 +1806,11 @@
     </row>
     <row r="29">
       <c r="A29" s="5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="7" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>6</v>
@@ -1393,11 +1818,11 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>6</v>
@@ -1405,11 +1830,11 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>6</v>
@@ -1417,11 +1842,11 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="7" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>6</v>
@@ -1429,11 +1854,11 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>6</v>
@@ -1441,11 +1866,11 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>6</v>
@@ -1453,11 +1878,11 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>6</v>
@@ -1469,7 +1894,7 @@
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>6</v>
@@ -1477,11 +1902,11 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>6</v>
@@ -1489,11 +1914,11 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>6</v>
@@ -1501,11 +1926,11 @@
     </row>
     <row r="39">
       <c r="A39" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="7" t="s">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>6</v>
@@ -1553,7 +1978,7 @@
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
-        <v>76</v>
+        <v>42</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>6</v>
@@ -1561,11 +1986,11 @@
     </row>
     <row r="44">
       <c r="A44" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>6</v>
@@ -1573,11 +1998,11 @@
     </row>
     <row r="45">
       <c r="A45" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>6</v>
@@ -1585,11 +2010,11 @@
     </row>
     <row r="46">
       <c r="A46" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>6</v>
@@ -1597,11 +2022,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>6</v>
@@ -1609,11 +2034,11 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>6</v>
@@ -1621,11 +2046,11 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>6</v>
@@ -1633,11 +2058,11 @@
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="7" t="s">
-        <v>24</v>
+        <v>89</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>6</v>
@@ -1661,7 +2086,7 @@
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="7" t="s">
-        <v>22</v>
+        <v>93</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>6</v>
@@ -1669,11 +2094,11 @@
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>6</v>
@@ -1681,11 +2106,11 @@
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
-        <v>74</v>
+        <v>31</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>6</v>
@@ -1693,11 +2118,11 @@
     </row>
     <row r="55">
       <c r="A55" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>6</v>
@@ -1705,11 +2130,11 @@
     </row>
     <row r="56">
       <c r="A56" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="7" t="s">
-        <v>99</v>
+        <v>29</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>6</v>
@@ -1733,7 +2158,7 @@
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="s">
-        <v>26</v>
+        <v>81</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -1764,24 +2189,26 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="10" t="s">
+      <c r="A61" s="5" t="s">
         <v>107</v>
       </c>
+      <c r="B61" s="6"/>
       <c r="C61" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="D61" s="10" t="s">
+      <c r="D61" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="10" t="s">
+      <c r="A62" s="5" t="s">
         <v>109</v>
       </c>
+      <c r="B62" s="6"/>
       <c r="C62" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D62" s="10" t="s">
+      <c r="D62" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1810,36 +2237,34 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="s">
+      <c r="A65" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="B65" s="6"/>
       <c r="C65" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D65" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="D65" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="s">
+      <c r="C66" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="6"/>
-      <c r="C66" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="D66" s="5" t="s">
+      <c r="D66" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B67" s="6"/>
       <c r="C67" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>6</v>
@@ -1847,11 +2272,11 @@
     </row>
     <row r="68">
       <c r="A68" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>6</v>
@@ -1859,11 +2284,11 @@
     </row>
     <row r="69">
       <c r="A69" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>6</v>
@@ -1871,11 +2296,11 @@
     </row>
     <row r="70">
       <c r="A70" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B70" s="6"/>
       <c r="C70" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D70" s="5" t="s">
         <v>6</v>
@@ -1883,35 +2308,35 @@
     </row>
     <row r="71">
       <c r="A71" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="D71" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="11" t="s">
+      <c r="B72" s="6"/>
+      <c r="C72" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B72" s="6"/>
-      <c r="C72" s="12" t="s">
+      <c r="D72" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="D72" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="11" t="s">
+      <c r="B73" s="6"/>
+      <c r="C73" s="7" t="s">
         <v>131</v>
-      </c>
-      <c r="B73" s="6"/>
-      <c r="C73" s="12" t="s">
-        <v>132</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>6</v>
@@ -1919,35 +2344,35 @@
     </row>
     <row r="74">
       <c r="A74" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B74" s="6"/>
       <c r="C74" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="D74" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="s">
-        <v>135</v>
       </c>
       <c r="B75" s="6"/>
       <c r="C75" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="D75" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="s">
-        <v>137</v>
       </c>
       <c r="B76" s="6"/>
       <c r="C76" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D76" s="5" t="s">
         <v>6</v>
@@ -1955,11 +2380,11 @@
     </row>
     <row r="77">
       <c r="A77" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B77" s="6"/>
       <c r="C77" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D77" s="5" t="s">
         <v>6</v>
@@ -1967,35 +2392,35 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B78" s="6"/>
       <c r="C78" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D78" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="s">
         <v>142</v>
-      </c>
-      <c r="D78" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="5" t="s">
-        <v>143</v>
       </c>
       <c r="B79" s="6"/>
       <c r="C79" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="s">
         <v>144</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="5" t="s">
-        <v>145</v>
       </c>
       <c r="B80" s="6"/>
       <c r="C80" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D80" s="5" t="s">
         <v>6</v>
@@ -2003,11 +2428,11 @@
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B81" s="6"/>
       <c r="C81" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>6</v>
@@ -2015,11 +2440,11 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B82" s="6"/>
       <c r="C82" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>6</v>
@@ -2027,11 +2452,11 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B83" s="6"/>
       <c r="C83" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>6</v>
@@ -2039,11 +2464,11 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B84" s="6"/>
       <c r="C84" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>6</v>
@@ -2051,11 +2476,11 @@
     </row>
     <row r="85">
       <c r="A85" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B85" s="6"/>
       <c r="C85" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>6</v>
@@ -2063,11 +2488,11 @@
     </row>
     <row r="86">
       <c r="A86" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B86" s="6"/>
       <c r="C86" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>6</v>
@@ -2075,11 +2500,11 @@
     </row>
     <row r="87">
       <c r="A87" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B87" s="6"/>
       <c r="C87" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D87" s="5" t="s">
         <v>6</v>
@@ -2087,11 +2512,11 @@
     </row>
     <row r="88">
       <c r="A88" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B88" s="6"/>
       <c r="C88" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>6</v>
@@ -2099,11 +2524,11 @@
     </row>
     <row r="89">
       <c r="A89" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B89" s="6"/>
       <c r="C89" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D89" s="5" t="s">
         <v>6</v>
@@ -2111,11 +2536,11 @@
     </row>
     <row r="90">
       <c r="A90" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B90" s="6"/>
       <c r="C90" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D90" s="5" t="s">
         <v>6</v>
@@ -2123,11 +2548,11 @@
     </row>
     <row r="91">
       <c r="A91" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B91" s="6"/>
       <c r="C91" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D91" s="5" t="s">
         <v>6</v>
@@ -2135,11 +2560,11 @@
     </row>
     <row r="92">
       <c r="A92" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B92" s="6"/>
       <c r="C92" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D92" s="5" t="s">
         <v>6</v>
@@ -2147,11 +2572,11 @@
     </row>
     <row r="93">
       <c r="A93" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B93" s="6"/>
       <c r="C93" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>6</v>
@@ -2159,11 +2584,11 @@
     </row>
     <row r="94">
       <c r="A94" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B94" s="6"/>
       <c r="C94" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D94" s="5" t="s">
         <v>6</v>
@@ -2171,11 +2596,11 @@
     </row>
     <row r="95">
       <c r="A95" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B95" s="6"/>
       <c r="C95" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D95" s="5" t="s">
         <v>6</v>
@@ -2183,11 +2608,11 @@
     </row>
     <row r="96">
       <c r="A96" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B96" s="6"/>
       <c r="C96" s="7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D96" s="5" t="s">
         <v>6</v>
@@ -2195,11 +2620,11 @@
     </row>
     <row r="97">
       <c r="A97" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B97" s="6"/>
       <c r="C97" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D97" s="5" t="s">
         <v>6</v>
@@ -2207,11 +2632,11 @@
     </row>
     <row r="98">
       <c r="A98" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B98" s="6"/>
       <c r="C98" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D98" s="5" t="s">
         <v>6</v>
@@ -2219,11 +2644,11 @@
     </row>
     <row r="99">
       <c r="A99" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B99" s="6"/>
       <c r="C99" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>6</v>
@@ -2231,11 +2656,11 @@
     </row>
     <row r="100">
       <c r="A100" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>6</v>
@@ -2243,11 +2668,11 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B101" s="6"/>
       <c r="C101" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>6</v>
@@ -2255,11 +2680,11 @@
     </row>
     <row r="102">
       <c r="A102" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B102" s="6"/>
       <c r="C102" s="7" t="s">
-        <v>24</v>
+        <v>189</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>6</v>
@@ -2271,7 +2696,7 @@
       </c>
       <c r="B103" s="6"/>
       <c r="C103" s="7" t="s">
-        <v>24</v>
+        <v>191</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>6</v>
@@ -2279,11 +2704,11 @@
     </row>
     <row r="104">
       <c r="A104" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B104" s="6"/>
       <c r="C104" s="7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>6</v>
@@ -2291,11 +2716,11 @@
     </row>
     <row r="105">
       <c r="A105" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="7" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D105" s="5" t="s">
         <v>6</v>
@@ -2303,11 +2728,11 @@
     </row>
     <row r="106">
       <c r="A106" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B106" s="6"/>
       <c r="C106" s="7" t="s">
-        <v>196</v>
+        <v>31</v>
       </c>
       <c r="D106" s="5" t="s">
         <v>6</v>
@@ -2319,7 +2744,7 @@
       </c>
       <c r="B107" s="6"/>
       <c r="C107" s="7" t="s">
-        <v>198</v>
+        <v>31</v>
       </c>
       <c r="D107" s="5" t="s">
         <v>6</v>
@@ -2327,11 +2752,11 @@
     </row>
     <row r="108">
       <c r="A108" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B108" s="6"/>
       <c r="C108" s="7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D108" s="5" t="s">
         <v>6</v>
@@ -2339,11 +2764,11 @@
     </row>
     <row r="109">
       <c r="A109" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B109" s="6"/>
       <c r="C109" s="7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>6</v>
@@ -2351,11 +2776,11 @@
     </row>
     <row r="110">
       <c r="A110" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B110" s="6"/>
       <c r="C110" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>6</v>
@@ -2363,11 +2788,11 @@
     </row>
     <row r="111">
       <c r="A111" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B111" s="6"/>
       <c r="C111" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>6</v>
@@ -2375,11 +2800,11 @@
     </row>
     <row r="112">
       <c r="A112" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B112" s="6"/>
       <c r="C112" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>6</v>
@@ -2387,11 +2812,11 @@
     </row>
     <row r="113">
       <c r="A113" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B113" s="6"/>
       <c r="C113" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>6</v>
@@ -2399,11 +2824,11 @@
     </row>
     <row r="114">
       <c r="A114" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B114" s="6"/>
       <c r="C114" s="7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>6</v>
@@ -2411,11 +2836,11 @@
     </row>
     <row r="115">
       <c r="A115" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B115" s="6"/>
       <c r="C115" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>6</v>
@@ -2423,11 +2848,11 @@
     </row>
     <row r="116">
       <c r="A116" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B116" s="6"/>
       <c r="C116" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D116" s="5" t="s">
         <v>6</v>
@@ -2435,459 +2860,867 @@
     </row>
     <row r="117">
       <c r="A117" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B117" s="6"/>
       <c r="C117" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="D117" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D117" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="11" t="s">
+      <c r="B118" s="6"/>
+      <c r="C118" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="B118" s="6"/>
-      <c r="C118" s="12" t="s">
+      <c r="D118" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="D118" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="11" t="s">
+      <c r="B119" s="6"/>
+      <c r="C119" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="B119" s="6"/>
-      <c r="C119" s="12" t="s">
+      <c r="D119" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="D119" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="11" t="s">
+      <c r="B120" s="6"/>
+      <c r="C120" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="B120" s="6"/>
-      <c r="C120" s="12" t="s">
+      <c r="D120" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="D120" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="6"/>
       <c r="B121" s="6"/>
-      <c r="C121" s="6"/>
-      <c r="D121" s="6"/>
+      <c r="C121" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="122">
-      <c r="A122" s="6"/>
+      <c r="A122" s="5" t="s">
+        <v>226</v>
+      </c>
       <c r="B122" s="6"/>
-      <c r="C122" s="6"/>
-      <c r="D122" s="6"/>
+      <c r="C122" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="123">
-      <c r="A123" s="6"/>
+      <c r="A123" s="5" t="s">
+        <v>228</v>
+      </c>
       <c r="B123" s="6"/>
-      <c r="C123" s="6"/>
-      <c r="D123" s="6"/>
+      <c r="C123" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="124">
-      <c r="A124" s="6"/>
+      <c r="A124" s="5" t="s">
+        <v>230</v>
+      </c>
       <c r="B124" s="6"/>
-      <c r="C124" s="6"/>
-      <c r="D124" s="6"/>
+      <c r="C124" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="D124" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="125">
-      <c r="A125" s="6"/>
+      <c r="A125" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="B125" s="6"/>
-      <c r="C125" s="6"/>
-      <c r="D125" s="6"/>
+      <c r="C125" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="126">
-      <c r="A126" s="6"/>
+      <c r="A126" s="5" t="s">
+        <v>234</v>
+      </c>
       <c r="B126" s="6"/>
-      <c r="C126" s="6"/>
-      <c r="D126" s="6"/>
+      <c r="C126" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="127">
-      <c r="A127" s="6"/>
+      <c r="A127" s="8" t="s">
+        <v>236</v>
+      </c>
       <c r="B127" s="6"/>
-      <c r="C127" s="6"/>
-      <c r="D127" s="6"/>
+      <c r="C127" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="128">
-      <c r="A128" s="6"/>
+      <c r="A128" s="8" t="s">
+        <v>238</v>
+      </c>
       <c r="B128" s="6"/>
-      <c r="C128" s="6"/>
-      <c r="D128" s="6"/>
+      <c r="C128" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" s="6"/>
+      <c r="A129" s="8" t="s">
+        <v>240</v>
+      </c>
       <c r="B129" s="6"/>
-      <c r="C129" s="6"/>
-      <c r="D129" s="6"/>
+      <c r="C129" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="130">
-      <c r="A130" s="6"/>
+      <c r="A130" s="5" t="s">
+        <v>242</v>
+      </c>
       <c r="B130" s="6"/>
-      <c r="C130" s="6"/>
-      <c r="D130" s="6"/>
+      <c r="C130" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" s="6"/>
+      <c r="A131" s="5" t="s">
+        <v>244</v>
+      </c>
       <c r="B131" s="6"/>
-      <c r="C131" s="6"/>
-      <c r="D131" s="6"/>
+      <c r="C131" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="6"/>
+      <c r="A132" s="5" t="s">
+        <v>246</v>
+      </c>
       <c r="B132" s="6"/>
-      <c r="C132" s="6"/>
-      <c r="D132" s="6"/>
+      <c r="C132" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="D132" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="133">
-      <c r="A133" s="6"/>
+      <c r="A133" s="5" t="s">
+        <v>248</v>
+      </c>
       <c r="B133" s="6"/>
-      <c r="C133" s="6"/>
-      <c r="D133" s="6"/>
+      <c r="C133" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="D133" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="134">
-      <c r="A134" s="6"/>
+      <c r="A134" s="5" t="s">
+        <v>250</v>
+      </c>
       <c r="B134" s="6"/>
-      <c r="C134" s="6"/>
-      <c r="D134" s="6"/>
+      <c r="C134" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="135">
-      <c r="A135" s="6"/>
+      <c r="A135" s="5" t="s">
+        <v>252</v>
+      </c>
       <c r="B135" s="6"/>
-      <c r="C135" s="6"/>
-      <c r="D135" s="6"/>
+      <c r="C135" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="136">
-      <c r="A136" s="6"/>
+      <c r="A136" s="5" t="s">
+        <v>254</v>
+      </c>
       <c r="B136" s="6"/>
-      <c r="C136" s="6"/>
-      <c r="D136" s="6"/>
+      <c r="C136" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="D136" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="137">
-      <c r="A137" s="6"/>
+      <c r="A137" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="B137" s="6"/>
-      <c r="C137" s="6"/>
-      <c r="D137" s="6"/>
+      <c r="C137" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="D137" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="138">
-      <c r="A138" s="6"/>
+      <c r="A138" s="11" t="s">
+        <v>258</v>
+      </c>
       <c r="B138" s="6"/>
-      <c r="C138" s="6"/>
-      <c r="D138" s="6"/>
+      <c r="C138" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="D138" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="139">
-      <c r="A139" s="6"/>
+      <c r="A139" s="5" t="s">
+        <v>260</v>
+      </c>
       <c r="B139" s="6"/>
-      <c r="C139" s="6"/>
-      <c r="D139" s="6"/>
+      <c r="C139" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="D139" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="140">
-      <c r="A140" s="6"/>
+      <c r="A140" s="5" t="s">
+        <v>262</v>
+      </c>
       <c r="B140" s="6"/>
-      <c r="C140" s="6"/>
-      <c r="D140" s="6"/>
+      <c r="C140" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="D140" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="141">
-      <c r="A141" s="6"/>
+      <c r="A141" s="5" t="s">
+        <v>264</v>
+      </c>
       <c r="B141" s="6"/>
-      <c r="C141" s="6"/>
-      <c r="D141" s="6"/>
+      <c r="C141" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="D141" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="142">
-      <c r="A142" s="6"/>
+      <c r="A142" s="5" t="s">
+        <v>266</v>
+      </c>
       <c r="B142" s="6"/>
-      <c r="C142" s="6"/>
-      <c r="D142" s="6"/>
+      <c r="C142" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="D142" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="143">
-      <c r="A143" s="6"/>
+      <c r="A143" s="8" t="s">
+        <v>268</v>
+      </c>
       <c r="B143" s="6"/>
-      <c r="C143" s="6"/>
-      <c r="D143" s="6"/>
+      <c r="C143" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="144">
-      <c r="A144" s="6"/>
+      <c r="A144" s="5" t="s">
+        <v>270</v>
+      </c>
       <c r="B144" s="6"/>
-      <c r="C144" s="6"/>
-      <c r="D144" s="6"/>
+      <c r="C144" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="D144" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="145">
-      <c r="A145" s="6"/>
+      <c r="A145" s="5" t="s">
+        <v>272</v>
+      </c>
       <c r="B145" s="6"/>
-      <c r="C145" s="6"/>
-      <c r="D145" s="6"/>
+      <c r="C145" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="D145" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="146">
-      <c r="A146" s="6"/>
+      <c r="A146" s="5" t="s">
+        <v>274</v>
+      </c>
       <c r="B146" s="6"/>
-      <c r="C146" s="6"/>
-      <c r="D146" s="6"/>
+      <c r="C146" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="D146" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="147">
-      <c r="A147" s="6"/>
+      <c r="A147" s="5" t="s">
+        <v>276</v>
+      </c>
       <c r="B147" s="6"/>
-      <c r="C147" s="6"/>
-      <c r="D147" s="6"/>
+      <c r="C147" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="D147" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="148">
-      <c r="A148" s="6"/>
+      <c r="A148" s="5" t="s">
+        <v>278</v>
+      </c>
       <c r="B148" s="6"/>
-      <c r="C148" s="6"/>
-      <c r="D148" s="6"/>
+      <c r="C148" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="D148" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="149">
-      <c r="A149" s="6"/>
+      <c r="A149" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="B149" s="6"/>
-      <c r="C149" s="6"/>
-      <c r="D149" s="6"/>
+      <c r="C149" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="D149" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="150">
-      <c r="A150" s="6"/>
+      <c r="A150" s="5" t="s">
+        <v>282</v>
+      </c>
       <c r="B150" s="6"/>
-      <c r="C150" s="6"/>
-      <c r="D150" s="6"/>
+      <c r="C150" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="D150" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="151">
-      <c r="A151" s="6"/>
+      <c r="A151" s="12" t="s">
+        <v>284</v>
+      </c>
       <c r="B151" s="6"/>
-      <c r="C151" s="6"/>
-      <c r="D151" s="6"/>
+      <c r="C151" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D151" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="152">
-      <c r="A152" s="6"/>
+      <c r="A152" s="12" t="s">
+        <v>286</v>
+      </c>
       <c r="B152" s="6"/>
-      <c r="C152" s="6"/>
-      <c r="D152" s="6"/>
+      <c r="C152" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="D152" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="153">
-      <c r="A153" s="6"/>
+      <c r="A153" s="5" t="s">
+        <v>288</v>
+      </c>
       <c r="B153" s="6"/>
-      <c r="C153" s="6"/>
-      <c r="D153" s="6"/>
+      <c r="C153" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="D153" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="154">
-      <c r="A154" s="6"/>
+      <c r="A154" s="5" t="s">
+        <v>290</v>
+      </c>
       <c r="B154" s="6"/>
-      <c r="C154" s="6"/>
-      <c r="D154" s="6"/>
+      <c r="C154" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="D154" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="155">
-      <c r="A155" s="6"/>
+      <c r="A155" s="5" t="s">
+        <v>292</v>
+      </c>
       <c r="B155" s="6"/>
-      <c r="C155" s="6"/>
-      <c r="D155" s="6"/>
+      <c r="C155" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="D155" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="156">
-      <c r="A156" s="6"/>
+      <c r="A156" s="5" t="s">
+        <v>294</v>
+      </c>
       <c r="B156" s="6"/>
-      <c r="C156" s="6"/>
-      <c r="D156" s="6"/>
+      <c r="C156" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="D156" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="157">
-      <c r="A157" s="6"/>
+      <c r="A157" s="5" t="s">
+        <v>296</v>
+      </c>
       <c r="B157" s="6"/>
-      <c r="C157" s="6"/>
-      <c r="D157" s="6"/>
+      <c r="C157" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="D157" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="158">
-      <c r="A158" s="6"/>
+      <c r="A158" s="12" t="s">
+        <v>298</v>
+      </c>
       <c r="B158" s="6"/>
-      <c r="C158" s="6"/>
-      <c r="D158" s="6"/>
+      <c r="C158" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="D158" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="159">
-      <c r="A159" s="6"/>
+      <c r="A159" s="10" t="s">
+        <v>300</v>
+      </c>
       <c r="B159" s="6"/>
-      <c r="C159" s="6"/>
-      <c r="D159" s="6"/>
+      <c r="C159" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="D159" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="160">
-      <c r="A160" s="6"/>
+      <c r="A160" s="10" t="s">
+        <v>302</v>
+      </c>
       <c r="B160" s="6"/>
-      <c r="C160" s="6"/>
-      <c r="D160" s="6"/>
+      <c r="C160" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="D160" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="161">
-      <c r="A161" s="6"/>
+      <c r="A161" s="10" t="s">
+        <v>304</v>
+      </c>
       <c r="B161" s="6"/>
-      <c r="C161" s="6"/>
-      <c r="D161" s="6"/>
+      <c r="C161" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="D161" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="162">
-      <c r="A162" s="6"/>
+      <c r="A162" s="10" t="s">
+        <v>306</v>
+      </c>
       <c r="B162" s="6"/>
-      <c r="C162" s="6"/>
-      <c r="D162" s="6"/>
+      <c r="C162" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="D162" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="163">
-      <c r="A163" s="6"/>
+      <c r="A163" s="10" t="s">
+        <v>308</v>
+      </c>
       <c r="B163" s="6"/>
-      <c r="C163" s="6"/>
-      <c r="D163" s="6"/>
+      <c r="C163" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="D163" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="164">
-      <c r="A164" s="6"/>
+      <c r="A164" s="10" t="s">
+        <v>310</v>
+      </c>
       <c r="B164" s="6"/>
-      <c r="C164" s="6"/>
-      <c r="D164" s="6"/>
+      <c r="C164" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="D164" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="165">
-      <c r="A165" s="6"/>
+      <c r="A165" s="5" t="s">
+        <v>312</v>
+      </c>
       <c r="B165" s="6"/>
-      <c r="C165" s="6"/>
-      <c r="D165" s="6"/>
+      <c r="C165" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="D165" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="166">
-      <c r="A166" s="6"/>
+      <c r="A166" s="5" t="s">
+        <v>314</v>
+      </c>
       <c r="B166" s="6"/>
-      <c r="C166" s="6"/>
-      <c r="D166" s="6"/>
+      <c r="C166" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="D166" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="167">
-      <c r="A167" s="6"/>
+      <c r="A167" s="5" t="s">
+        <v>316</v>
+      </c>
       <c r="B167" s="6"/>
-      <c r="C167" s="6"/>
-      <c r="D167" s="6"/>
+      <c r="C167" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="D167" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="168">
-      <c r="A168" s="6"/>
+      <c r="A168" s="5" t="s">
+        <v>318</v>
+      </c>
       <c r="B168" s="6"/>
-      <c r="C168" s="6"/>
-      <c r="D168" s="6"/>
+      <c r="C168" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="D168" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="169">
-      <c r="A169" s="6"/>
+      <c r="A169" s="5" t="s">
+        <v>320</v>
+      </c>
       <c r="B169" s="6"/>
-      <c r="C169" s="6"/>
-      <c r="D169" s="6"/>
+      <c r="C169" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="D169" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="170">
-      <c r="A170" s="6"/>
+      <c r="A170" s="5" t="s">
+        <v>322</v>
+      </c>
       <c r="B170" s="6"/>
-      <c r="C170" s="6"/>
-      <c r="D170" s="6"/>
+      <c r="C170" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="D170" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="171">
-      <c r="A171" s="6"/>
+      <c r="A171" s="5" t="s">
+        <v>324</v>
+      </c>
       <c r="B171" s="6"/>
-      <c r="C171" s="6"/>
-      <c r="D171" s="6"/>
+      <c r="C171" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="D171" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="172">
-      <c r="A172" s="6"/>
+      <c r="A172" s="5" t="s">
+        <v>326</v>
+      </c>
       <c r="B172" s="6"/>
-      <c r="C172" s="6"/>
-      <c r="D172" s="6"/>
+      <c r="C172" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="D172" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="173">
-      <c r="A173" s="6"/>
+      <c r="A173" s="5" t="s">
+        <v>328</v>
+      </c>
       <c r="B173" s="6"/>
-      <c r="C173" s="6"/>
-      <c r="D173" s="6"/>
+      <c r="C173" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="D173" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="174">
-      <c r="A174" s="6"/>
+      <c r="A174" s="5" t="s">
+        <v>330</v>
+      </c>
       <c r="B174" s="6"/>
-      <c r="C174" s="6"/>
-      <c r="D174" s="6"/>
+      <c r="C174" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="D174" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="175">
-      <c r="A175" s="6"/>
+      <c r="A175" s="5" t="s">
+        <v>332</v>
+      </c>
       <c r="B175" s="6"/>
-      <c r="C175" s="6"/>
-      <c r="D175" s="6"/>
+      <c r="C175" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="D175" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="176">
-      <c r="A176" s="6"/>
+      <c r="A176" s="5" t="s">
+        <v>334</v>
+      </c>
       <c r="B176" s="6"/>
-      <c r="C176" s="6"/>
-      <c r="D176" s="6"/>
+      <c r="C176" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="D176" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="177">
-      <c r="A177" s="6"/>
+      <c r="A177" s="5" t="s">
+        <v>336</v>
+      </c>
       <c r="B177" s="6"/>
-      <c r="C177" s="6"/>
-      <c r="D177" s="6"/>
+      <c r="C177" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="D177" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="178">
-      <c r="A178" s="6"/>
+      <c r="A178" s="5" t="s">
+        <v>338</v>
+      </c>
       <c r="B178" s="6"/>
-      <c r="C178" s="6"/>
-      <c r="D178" s="6"/>
+      <c r="C178" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="D178" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="179">
-      <c r="A179" s="6"/>
+      <c r="A179" s="5" t="s">
+        <v>340</v>
+      </c>
       <c r="B179" s="6"/>
-      <c r="C179" s="6"/>
-      <c r="D179" s="6"/>
+      <c r="C179" s="7" t="s">
+        <v>341</v>
+      </c>
+      <c r="D179" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="180">
-      <c r="A180" s="6"/>
+      <c r="A180" s="5" t="s">
+        <v>342</v>
+      </c>
       <c r="B180" s="6"/>
-      <c r="C180" s="6"/>
-      <c r="D180" s="6"/>
+      <c r="C180" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="D180" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="181">
-      <c r="A181" s="6"/>
+      <c r="A181" s="5" t="s">
+        <v>344</v>
+      </c>
       <c r="B181" s="6"/>
-      <c r="C181" s="6"/>
-      <c r="D181" s="6"/>
+      <c r="C181" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="D181" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="182">
-      <c r="A182" s="6"/>
+      <c r="A182" s="5" t="s">
+        <v>346</v>
+      </c>
       <c r="B182" s="6"/>
-      <c r="C182" s="6"/>
-      <c r="D182" s="6"/>
+      <c r="C182" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="D182" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="183">
-      <c r="A183" s="6"/>
+      <c r="A183" s="5" t="s">
+        <v>348</v>
+      </c>
       <c r="B183" s="6"/>
-      <c r="C183" s="6"/>
-      <c r="D183" s="6"/>
+      <c r="C183" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="D183" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="184">
-      <c r="A184" s="6"/>
+      <c r="A184" s="5" t="s">
+        <v>350</v>
+      </c>
       <c r="B184" s="6"/>
-      <c r="C184" s="6"/>
-      <c r="D184" s="6"/>
+      <c r="C184" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="D184" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="185">
-      <c r="A185" s="6"/>
+      <c r="A185" s="5" t="s">
+        <v>352</v>
+      </c>
       <c r="B185" s="6"/>
-      <c r="C185" s="6"/>
-      <c r="D185" s="6"/>
+      <c r="C185" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="D185" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="186">
-      <c r="A186" s="6"/>
+      <c r="A186" s="5" t="s">
+        <v>354</v>
+      </c>
       <c r="B186" s="6"/>
-      <c r="C186" s="6"/>
-      <c r="D186" s="6"/>
+      <c r="C186" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="D186" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="187">
-      <c r="A187" s="6"/>
+      <c r="A187" s="12" t="s">
+        <v>356</v>
+      </c>
       <c r="B187" s="6"/>
-      <c r="C187" s="6"/>
-      <c r="D187" s="6"/>
+      <c r="C187" s="13" t="s">
+        <v>357</v>
+      </c>
+      <c r="D187" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="188">
-      <c r="A188" s="6"/>
+      <c r="A188" s="12" t="s">
+        <v>358</v>
+      </c>
       <c r="B188" s="6"/>
-      <c r="C188" s="6"/>
-      <c r="D188" s="6"/>
+      <c r="C188" s="13" t="s">
+        <v>359</v>
+      </c>
+      <c r="D188" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="6"/>
@@ -8007,12 +8840,177 @@
       <c r="C1041" s="6"/>
       <c r="D1041" s="6"/>
     </row>
+    <row r="1042">
+      <c r="A1042" s="6"/>
+      <c r="B1042" s="6"/>
+      <c r="C1042" s="6"/>
+      <c r="D1042" s="6"/>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="6"/>
+      <c r="B1043" s="6"/>
+      <c r="C1043" s="6"/>
+      <c r="D1043" s="6"/>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="6"/>
+      <c r="B1044" s="6"/>
+      <c r="C1044" s="6"/>
+      <c r="D1044" s="6"/>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="6"/>
+      <c r="B1045" s="6"/>
+      <c r="C1045" s="6"/>
+      <c r="D1045" s="6"/>
+    </row>
+    <row r="1046">
+      <c r="A1046" s="6"/>
+      <c r="B1046" s="6"/>
+      <c r="C1046" s="6"/>
+      <c r="D1046" s="6"/>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="6"/>
+      <c r="B1047" s="6"/>
+      <c r="C1047" s="6"/>
+      <c r="D1047" s="6"/>
+    </row>
+    <row r="1048">
+      <c r="A1048" s="6"/>
+      <c r="B1048" s="6"/>
+      <c r="C1048" s="6"/>
+      <c r="D1048" s="6"/>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="6"/>
+      <c r="B1049" s="6"/>
+      <c r="C1049" s="6"/>
+      <c r="D1049" s="6"/>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="6"/>
+      <c r="B1050" s="6"/>
+      <c r="C1050" s="6"/>
+      <c r="D1050" s="6"/>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="6"/>
+      <c r="B1051" s="6"/>
+      <c r="C1051" s="6"/>
+      <c r="D1051" s="6"/>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="6"/>
+      <c r="B1052" s="6"/>
+      <c r="C1052" s="6"/>
+      <c r="D1052" s="6"/>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="6"/>
+      <c r="B1053" s="6"/>
+      <c r="C1053" s="6"/>
+      <c r="D1053" s="6"/>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="6"/>
+      <c r="B1054" s="6"/>
+      <c r="C1054" s="6"/>
+      <c r="D1054" s="6"/>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="6"/>
+      <c r="B1055" s="6"/>
+      <c r="C1055" s="6"/>
+      <c r="D1055" s="6"/>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="6"/>
+      <c r="B1056" s="6"/>
+      <c r="C1056" s="6"/>
+      <c r="D1056" s="6"/>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="6"/>
+      <c r="B1057" s="6"/>
+      <c r="C1057" s="6"/>
+      <c r="D1057" s="6"/>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="6"/>
+      <c r="B1058" s="6"/>
+      <c r="C1058" s="6"/>
+      <c r="D1058" s="6"/>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="6"/>
+      <c r="B1059" s="6"/>
+      <c r="C1059" s="6"/>
+      <c r="D1059" s="6"/>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="6"/>
+      <c r="B1060" s="6"/>
+      <c r="C1060" s="6"/>
+      <c r="D1060" s="6"/>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="6"/>
+      <c r="B1061" s="6"/>
+      <c r="C1061" s="6"/>
+      <c r="D1061" s="6"/>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="6"/>
+      <c r="B1062" s="6"/>
+      <c r="C1062" s="6"/>
+      <c r="D1062" s="6"/>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="6"/>
+      <c r="B1063" s="6"/>
+      <c r="C1063" s="6"/>
+      <c r="D1063" s="6"/>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="6"/>
+      <c r="B1064" s="6"/>
+      <c r="C1064" s="6"/>
+      <c r="D1064" s="6"/>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="6"/>
+      <c r="B1065" s="6"/>
+      <c r="C1065" s="6"/>
+      <c r="D1065" s="6"/>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="6"/>
+      <c r="B1066" s="6"/>
+      <c r="C1066" s="6"/>
+      <c r="D1066" s="6"/>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="6"/>
+      <c r="B1067" s="6"/>
+      <c r="C1067" s="6"/>
+      <c r="D1067" s="6"/>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="6"/>
+      <c r="B1068" s="6"/>
+      <c r="C1068" s="6"/>
+      <c r="D1068" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D120">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D188">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="A138"/>
+  </hyperlinks>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
WIP add modal for picking the alarm time
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="366">
   <si>
     <t>Key</t>
   </si>
@@ -1119,6 +1119,24 @@
   </si>
   <si>
     <t>Alert</t>
+  </si>
+  <si>
+    <t>banner.calibration.title</t>
+  </si>
+  <si>
+    <t>Calibration period</t>
+  </si>
+  <si>
+    <t>banner.calibration.message</t>
+  </si>
+  <si>
+    <t>Keep wearing your ring during the entirety of the 14 days calibration period for improved results!</t>
+  </si>
+  <si>
+    <t>alarm.new.time.edit</t>
+  </si>
+  <si>
+    <t>Edit alarm time</t>
   </si>
 </sst>
 </file>
@@ -3267,11 +3285,11 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="12" t="s">
+      <c r="A151" s="5" t="s">
         <v>284</v>
       </c>
       <c r="B151" s="6"/>
-      <c r="C151" s="13" t="s">
+      <c r="C151" s="7" t="s">
         <v>285</v>
       </c>
       <c r="D151" s="5" t="s">
@@ -3279,11 +3297,11 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="12" t="s">
+      <c r="A152" s="5" t="s">
         <v>286</v>
       </c>
       <c r="B152" s="6"/>
-      <c r="C152" s="13" t="s">
+      <c r="C152" s="7" t="s">
         <v>287</v>
       </c>
       <c r="D152" s="5" t="s">
@@ -3351,7 +3369,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="12" t="s">
+      <c r="A158" s="5" t="s">
         <v>298</v>
       </c>
       <c r="B158" s="6"/>
@@ -3699,11 +3717,11 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="12" t="s">
+      <c r="A187" s="5" t="s">
         <v>356</v>
       </c>
       <c r="B187" s="6"/>
-      <c r="C187" s="13" t="s">
+      <c r="C187" s="7" t="s">
         <v>357</v>
       </c>
       <c r="D187" s="5" t="s">
@@ -3711,11 +3729,11 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="12" t="s">
+      <c r="A188" s="5" t="s">
         <v>358</v>
       </c>
       <c r="B188" s="6"/>
-      <c r="C188" s="13" t="s">
+      <c r="C188" s="7" t="s">
         <v>359</v>
       </c>
       <c r="D188" s="5" t="s">
@@ -3723,22 +3741,40 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="6"/>
+      <c r="A189" s="5" t="s">
+        <v>360</v>
+      </c>
       <c r="B189" s="6"/>
-      <c r="C189" s="6"/>
-      <c r="D189" s="6"/>
+      <c r="C189" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="D189" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="190">
-      <c r="A190" s="6"/>
+      <c r="A190" s="5" t="s">
+        <v>362</v>
+      </c>
       <c r="B190" s="6"/>
-      <c r="C190" s="6"/>
-      <c r="D190" s="6"/>
+      <c r="C190" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="D190" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="191">
-      <c r="A191" s="6"/>
+      <c r="A191" s="12" t="s">
+        <v>364</v>
+      </c>
       <c r="B191" s="6"/>
-      <c r="C191" s="6"/>
-      <c r="D191" s="6"/>
+      <c r="C191" s="13" t="s">
+        <v>365</v>
+      </c>
+      <c r="D191" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="6"/>
@@ -9004,7 +9040,7 @@
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D188">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D191">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
display actual days left in wording
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="368">
   <si>
     <t>Key</t>
   </si>
@@ -923,6 +923,12 @@
     <t>Country is required.</t>
   </si>
   <si>
+    <t>onboarding.personal_info.error.born_date</t>
+  </si>
+  <si>
+    <t>Born date is required.</t>
+  </si>
+  <si>
     <t>alarm.new.edit_vibration.intensity</t>
   </si>
   <si>
@@ -1130,14 +1136,20 @@
     <t>banner.calibration.message</t>
   </si>
   <si>
-    <t>Keep wearing your ring during the entirety of the 14 days calibration period for improved results!</t>
+    <t>Keep wearing your ring during the entirety of the {days} days calibration period for improved results!</t>
+  </si>
+  <si>
+    <t>alarm.new.time.edit</t>
+  </si>
+  <si>
+    <t>Edit alarm time</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1160,6 +1172,7 @@
       <u/>
       <color rgb="FF0000FF"/>
     </font>
+    <font/>
   </fonts>
   <fills count="5">
     <fill>
@@ -1193,7 +1206,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1228,6 +1241,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3368,7 +3384,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="10" t="s">
+      <c r="A159" s="5" t="s">
         <v>300</v>
       </c>
       <c r="B159" s="6"/>
@@ -3440,7 +3456,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="5" t="s">
+      <c r="A165" s="10" t="s">
         <v>312</v>
       </c>
       <c r="B165" s="6"/>
@@ -3752,16 +3768,28 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="6"/>
+      <c r="A191" s="5" t="s">
+        <v>364</v>
+      </c>
       <c r="B191" s="6"/>
-      <c r="C191" s="6"/>
-      <c r="D191" s="6"/>
+      <c r="C191" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="D191" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="192">
-      <c r="A192" s="6"/>
+      <c r="A192" s="5" t="s">
+        <v>366</v>
+      </c>
       <c r="B192" s="6"/>
-      <c r="C192" s="6"/>
-      <c r="D192" s="6"/>
+      <c r="C192" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="D192" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="6"/>
@@ -9019,9 +9047,15 @@
       <c r="C1068" s="6"/>
       <c r="D1068" s="6"/>
     </row>
+    <row r="1069">
+      <c r="A1069" s="6"/>
+      <c r="B1069" s="6"/>
+      <c r="C1069" s="6"/>
+      <c r="D1069" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D190">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D192">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
merged and resolve some conflict
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="368">
   <si>
     <t>Key</t>
   </si>
@@ -923,6 +923,12 @@
     <t>Country is required.</t>
   </si>
   <si>
+    <t>onboarding.personal_info.error.born_date</t>
+  </si>
+  <si>
+    <t>Born date is required.</t>
+  </si>
+  <si>
     <t>alarm.new.edit_vibration.intensity</t>
   </si>
   <si>
@@ -1119,6 +1125,24 @@
   </si>
   <si>
     <t>Alert</t>
+  </si>
+  <si>
+    <t>banner.calibration.title</t>
+  </si>
+  <si>
+    <t>Calibration period</t>
+  </si>
+  <si>
+    <t>banner.calibration.message</t>
+  </si>
+  <si>
+    <t>Keep wearing your ring during the entirety of the 14 days calibration period for improved results!</t>
+  </si>
+  <si>
+    <t>alarm.new.time.edit</t>
+  </si>
+  <si>
+    <t>Edit alarm time</t>
   </si>
 </sst>
 </file>
@@ -3267,11 +3291,11 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="12" t="s">
+      <c r="A151" s="5" t="s">
         <v>284</v>
       </c>
       <c r="B151" s="6"/>
-      <c r="C151" s="13" t="s">
+      <c r="C151" s="7" t="s">
         <v>285</v>
       </c>
       <c r="D151" s="5" t="s">
@@ -3279,11 +3303,11 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="12" t="s">
+      <c r="A152" s="5" t="s">
         <v>286</v>
       </c>
       <c r="B152" s="6"/>
-      <c r="C152" s="13" t="s">
+      <c r="C152" s="7" t="s">
         <v>287</v>
       </c>
       <c r="D152" s="5" t="s">
@@ -3327,11 +3351,11 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="5" t="s">
+      <c r="A156" s="12" t="s">
         <v>294</v>
       </c>
       <c r="B156" s="6"/>
-      <c r="C156" s="7" t="s">
+      <c r="C156" s="13" t="s">
         <v>295</v>
       </c>
       <c r="D156" s="5" t="s">
@@ -3351,7 +3375,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="12" t="s">
+      <c r="A158" s="5" t="s">
         <v>298</v>
       </c>
       <c r="B158" s="6"/>
@@ -3363,7 +3387,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="10" t="s">
+      <c r="A159" s="5" t="s">
         <v>300</v>
       </c>
       <c r="B159" s="6"/>
@@ -3435,7 +3459,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="5" t="s">
+      <c r="A165" s="10" t="s">
         <v>312</v>
       </c>
       <c r="B165" s="6"/>
@@ -3699,11 +3723,11 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="12" t="s">
+      <c r="A187" s="5" t="s">
         <v>356</v>
       </c>
       <c r="B187" s="6"/>
-      <c r="C187" s="13" t="s">
+      <c r="C187" s="7" t="s">
         <v>357</v>
       </c>
       <c r="D187" s="5" t="s">
@@ -3711,11 +3735,11 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="12" t="s">
+      <c r="A188" s="5" t="s">
         <v>358</v>
       </c>
       <c r="B188" s="6"/>
-      <c r="C188" s="13" t="s">
+      <c r="C188" s="7" t="s">
         <v>359</v>
       </c>
       <c r="D188" s="5" t="s">
@@ -3723,28 +3747,52 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="6"/>
+      <c r="A189" s="5" t="s">
+        <v>360</v>
+      </c>
       <c r="B189" s="6"/>
-      <c r="C189" s="6"/>
-      <c r="D189" s="6"/>
+      <c r="C189" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="D189" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="190">
-      <c r="A190" s="6"/>
+      <c r="A190" s="5" t="s">
+        <v>362</v>
+      </c>
       <c r="B190" s="6"/>
-      <c r="C190" s="6"/>
-      <c r="D190" s="6"/>
+      <c r="C190" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="D190" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="191">
-      <c r="A191" s="6"/>
+      <c r="A191" s="5" t="s">
+        <v>364</v>
+      </c>
       <c r="B191" s="6"/>
-      <c r="C191" s="6"/>
-      <c r="D191" s="6"/>
+      <c r="C191" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="D191" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="192">
-      <c r="A192" s="6"/>
+      <c r="A192" s="5" t="s">
+        <v>366</v>
+      </c>
       <c r="B192" s="6"/>
-      <c r="C192" s="6"/>
-      <c r="D192" s="6"/>
+      <c r="C192" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="D192" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="6"/>
@@ -9002,9 +9050,15 @@
       <c r="C1068" s="6"/>
       <c r="D1068" s="6"/>
     </row>
+    <row r="1069">
+      <c r="A1069" s="6"/>
+      <c r="B1069" s="6"/>
+      <c r="C1069" s="6"/>
+      <c r="D1069" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D188">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D192">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Wake up score in alarm screen
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="372">
   <si>
     <t>Key</t>
   </si>
@@ -929,6 +929,15 @@
     <t>Born date is required.</t>
   </si>
   <si>
+    <t>onboarding.personal_info.error.born_date_invalid</t>
+  </si>
+  <si>
+    <t>Born date is invalid.</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.error.default</t>
+  </si>
+  <si>
     <t>alarm.new.edit_vibration.intensity</t>
   </si>
   <si>
@@ -1127,6 +1136,9 @@
     <t>Alert</t>
   </si>
   <si>
+    <t>alarm.wake_up_score</t>
+  </si>
+  <si>
     <t>banner.calibration.title</t>
   </si>
   <si>
@@ -1136,7 +1148,7 @@
     <t>banner.calibration.message</t>
   </si>
   <si>
-    <t>Keep wearing your ring during the entirety of the 14 days calibration period for improved results!</t>
+    <t>Keep wearing your ring during the entirety of the {days} days calibration period for improved results!</t>
   </si>
   <si>
     <t>alarm.new.time.edit</t>
@@ -3351,11 +3363,11 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="12" t="s">
+      <c r="A156" s="5" t="s">
         <v>294</v>
       </c>
       <c r="B156" s="6"/>
-      <c r="C156" s="13" t="s">
+      <c r="C156" s="7" t="s">
         <v>295</v>
       </c>
       <c r="D156" s="5" t="s">
@@ -3375,12 +3387,12 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="5" t="s">
+      <c r="A158" s="12" t="s">
         <v>298</v>
       </c>
       <c r="B158" s="6"/>
-      <c r="C158" s="7" t="s">
-        <v>299</v>
+      <c r="C158" s="13" t="s">
+        <v>42</v>
       </c>
       <c r="D158" s="5" t="s">
         <v>6</v>
@@ -3388,35 +3400,35 @@
     </row>
     <row r="159">
       <c r="A159" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="D159" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="s">
         <v>301</v>
-      </c>
-      <c r="D159" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="10" t="s">
-        <v>302</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="D160" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="s">
         <v>303</v>
-      </c>
-      <c r="D160" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="10" t="s">
-        <v>304</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="7" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D161" s="5" t="s">
         <v>6</v>
@@ -3424,11 +3436,11 @@
     </row>
     <row r="162">
       <c r="A162" s="10" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>6</v>
@@ -3436,11 +3448,11 @@
     </row>
     <row r="163">
       <c r="A163" s="10" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
@@ -3448,11 +3460,11 @@
     </row>
     <row r="164">
       <c r="A164" s="10" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
@@ -3460,35 +3472,35 @@
     </row>
     <row r="165">
       <c r="A165" s="10" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="D165" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="10" t="s">
         <v>313</v>
-      </c>
-      <c r="D165" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="5" t="s">
-        <v>314</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="D166" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="10" t="s">
         <v>315</v>
-      </c>
-      <c r="D166" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="5" t="s">
-        <v>316</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="7" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D167" s="5" t="s">
         <v>6</v>
@@ -3496,11 +3508,11 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
@@ -3508,11 +3520,11 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="7" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D169" s="5" t="s">
         <v>6</v>
@@ -3520,11 +3532,11 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D170" s="5" t="s">
         <v>6</v>
@@ -3532,11 +3544,11 @@
     </row>
     <row r="171">
       <c r="A171" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D171" s="5" t="s">
         <v>6</v>
@@ -3544,11 +3556,11 @@
     </row>
     <row r="172">
       <c r="A172" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D172" s="5" t="s">
         <v>6</v>
@@ -3556,11 +3568,11 @@
     </row>
     <row r="173">
       <c r="A173" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="7" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D173" s="5" t="s">
         <v>6</v>
@@ -3568,11 +3580,11 @@
     </row>
     <row r="174">
       <c r="A174" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
@@ -3580,11 +3592,11 @@
     </row>
     <row r="175">
       <c r="A175" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
@@ -3592,11 +3604,11 @@
     </row>
     <row r="176">
       <c r="A176" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
@@ -3604,11 +3616,11 @@
     </row>
     <row r="177">
       <c r="A177" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
@@ -3616,11 +3628,11 @@
     </row>
     <row r="178">
       <c r="A178" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
@@ -3628,11 +3640,11 @@
     </row>
     <row r="179">
       <c r="A179" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
@@ -3640,11 +3652,11 @@
     </row>
     <row r="180">
       <c r="A180" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
@@ -3652,11 +3664,11 @@
     </row>
     <row r="181">
       <c r="A181" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
@@ -3664,11 +3676,11 @@
     </row>
     <row r="182">
       <c r="A182" s="5" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="7" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>6</v>
@@ -3676,11 +3688,11 @@
     </row>
     <row r="183">
       <c r="A183" s="5" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="7" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>6</v>
@@ -3688,11 +3700,11 @@
     </row>
     <row r="184">
       <c r="A184" s="5" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="7" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D184" s="5" t="s">
         <v>6</v>
@@ -3700,11 +3712,11 @@
     </row>
     <row r="185">
       <c r="A185" s="5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="7" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D185" s="5" t="s">
         <v>6</v>
@@ -3712,11 +3724,11 @@
     </row>
     <row r="186">
       <c r="A186" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="7" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D186" s="5" t="s">
         <v>6</v>
@@ -3724,11 +3736,11 @@
     </row>
     <row r="187">
       <c r="A187" s="5" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>6</v>
@@ -3736,11 +3748,11 @@
     </row>
     <row r="188">
       <c r="A188" s="5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D188" s="5" t="s">
         <v>6</v>
@@ -3748,11 +3760,11 @@
     </row>
     <row r="189">
       <c r="A189" s="5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>6</v>
@@ -3760,11 +3772,11 @@
     </row>
     <row r="190">
       <c r="A190" s="5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>6</v>
@@ -3772,45 +3784,63 @@
     </row>
     <row r="191">
       <c r="A191" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="D191" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="12" t="s">
         <v>365</v>
       </c>
-      <c r="D191" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="5" t="s">
+      <c r="B192" s="6"/>
+      <c r="C192" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="D192" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="B192" s="6"/>
-      <c r="C192" s="7" t="s">
+      <c r="B193" s="6"/>
+      <c r="C193" s="7" t="s">
         <v>367</v>
       </c>
-      <c r="D192" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="6"/>
-      <c r="B193" s="6"/>
-      <c r="C193" s="6"/>
-      <c r="D193" s="6"/>
+      <c r="D193" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="194">
-      <c r="A194" s="6"/>
+      <c r="A194" s="5" t="s">
+        <v>368</v>
+      </c>
       <c r="B194" s="6"/>
-      <c r="C194" s="6"/>
-      <c r="D194" s="6"/>
+      <c r="C194" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="D194" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="195">
-      <c r="A195" s="6"/>
+      <c r="A195" s="5" t="s">
+        <v>370</v>
+      </c>
       <c r="B195" s="6"/>
-      <c r="C195" s="6"/>
-      <c r="D195" s="6"/>
+      <c r="C195" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="D195" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="6"/>
@@ -9056,9 +9086,27 @@
       <c r="C1069" s="6"/>
       <c r="D1069" s="6"/>
     </row>
+    <row r="1070">
+      <c r="A1070" s="6"/>
+      <c r="B1070" s="6"/>
+      <c r="C1070" s="6"/>
+      <c r="D1070" s="6"/>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="6"/>
+      <c r="B1071" s="6"/>
+      <c r="C1071" s="6"/>
+      <c r="D1071" s="6"/>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="6"/>
+      <c r="B1072" s="6"/>
+      <c r="C1072" s="6"/>
+      <c r="D1072" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D192">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D195">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
display alarms of the week under the screen
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="373">
   <si>
     <t>Key</t>
   </si>
@@ -929,6 +929,15 @@
     <t>Born date is required.</t>
   </si>
   <si>
+    <t>onboarding.personal_info.error.born_date_invalid</t>
+  </si>
+  <si>
+    <t>Born date is invalid.</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.error.default</t>
+  </si>
+  <si>
     <t>alarm.new.edit_vibration.intensity</t>
   </si>
   <si>
@@ -1127,6 +1136,18 @@
     <t>Alert</t>
   </si>
   <si>
+    <t>alarm.wake_up_score</t>
+  </si>
+  <si>
+    <t>alarm.new.time.edit</t>
+  </si>
+  <si>
+    <t>Edit alarm time</t>
+  </si>
+  <si>
+    <t>alarm.week_overview</t>
+  </si>
+  <si>
     <t>banner.calibration.title</t>
   </si>
   <si>
@@ -1136,20 +1157,14 @@
     <t>banner.calibration.message</t>
   </si>
   <si>
-    <t>Keep wearing your ring during the entirety of the 14 days calibration period for improved results!</t>
-  </si>
-  <si>
-    <t>alarm.new.time.edit</t>
-  </si>
-  <si>
-    <t>Edit alarm time</t>
+    <t>Keep wearing your ring during the entirety of the {days} days calibration period for improved results!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1172,7 +1187,6 @@
       <u/>
       <color rgb="FF0000FF"/>
     </font>
-    <font/>
   </fonts>
   <fills count="5">
     <fill>
@@ -1206,7 +1220,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1241,12 +1255,6 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3351,11 +3359,11 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="12" t="s">
+      <c r="A156" s="5" t="s">
         <v>294</v>
       </c>
       <c r="B156" s="6"/>
-      <c r="C156" s="13" t="s">
+      <c r="C156" s="7" t="s">
         <v>295</v>
       </c>
       <c r="D156" s="5" t="s">
@@ -3380,7 +3388,7 @@
       </c>
       <c r="B158" s="6"/>
       <c r="C158" s="7" t="s">
-        <v>299</v>
+        <v>42</v>
       </c>
       <c r="D158" s="5" t="s">
         <v>6</v>
@@ -3388,35 +3396,35 @@
     </row>
     <row r="159">
       <c r="A159" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="D159" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="s">
         <v>301</v>
-      </c>
-      <c r="D159" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="10" t="s">
-        <v>302</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="D160" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="s">
         <v>303</v>
-      </c>
-      <c r="D160" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="10" t="s">
-        <v>304</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="7" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D161" s="5" t="s">
         <v>6</v>
@@ -3424,11 +3432,11 @@
     </row>
     <row r="162">
       <c r="A162" s="10" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>6</v>
@@ -3436,11 +3444,11 @@
     </row>
     <row r="163">
       <c r="A163" s="10" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
@@ -3448,11 +3456,11 @@
     </row>
     <row r="164">
       <c r="A164" s="10" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
@@ -3460,35 +3468,35 @@
     </row>
     <row r="165">
       <c r="A165" s="10" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="D165" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="10" t="s">
         <v>313</v>
-      </c>
-      <c r="D165" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="5" t="s">
-        <v>314</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="D166" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="10" t="s">
         <v>315</v>
-      </c>
-      <c r="D166" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="5" t="s">
-        <v>316</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="7" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D167" s="5" t="s">
         <v>6</v>
@@ -3496,11 +3504,11 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
@@ -3508,11 +3516,11 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="7" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D169" s="5" t="s">
         <v>6</v>
@@ -3520,11 +3528,11 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D170" s="5" t="s">
         <v>6</v>
@@ -3532,11 +3540,11 @@
     </row>
     <row r="171">
       <c r="A171" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D171" s="5" t="s">
         <v>6</v>
@@ -3544,11 +3552,11 @@
     </row>
     <row r="172">
       <c r="A172" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D172" s="5" t="s">
         <v>6</v>
@@ -3556,11 +3564,11 @@
     </row>
     <row r="173">
       <c r="A173" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="7" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D173" s="5" t="s">
         <v>6</v>
@@ -3568,11 +3576,11 @@
     </row>
     <row r="174">
       <c r="A174" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
@@ -3580,11 +3588,11 @@
     </row>
     <row r="175">
       <c r="A175" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
@@ -3592,11 +3600,11 @@
     </row>
     <row r="176">
       <c r="A176" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
@@ -3604,11 +3612,11 @@
     </row>
     <row r="177">
       <c r="A177" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
@@ -3616,11 +3624,11 @@
     </row>
     <row r="178">
       <c r="A178" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
@@ -3628,11 +3636,11 @@
     </row>
     <row r="179">
       <c r="A179" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
@@ -3640,11 +3648,11 @@
     </row>
     <row r="180">
       <c r="A180" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
@@ -3652,11 +3660,11 @@
     </row>
     <row r="181">
       <c r="A181" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
@@ -3664,11 +3672,11 @@
     </row>
     <row r="182">
       <c r="A182" s="5" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="7" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>6</v>
@@ -3676,11 +3684,11 @@
     </row>
     <row r="183">
       <c r="A183" s="5" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="7" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>6</v>
@@ -3688,11 +3696,11 @@
     </row>
     <row r="184">
       <c r="A184" s="5" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="7" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D184" s="5" t="s">
         <v>6</v>
@@ -3700,11 +3708,11 @@
     </row>
     <row r="185">
       <c r="A185" s="5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="7" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D185" s="5" t="s">
         <v>6</v>
@@ -3712,11 +3720,11 @@
     </row>
     <row r="186">
       <c r="A186" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="7" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D186" s="5" t="s">
         <v>6</v>
@@ -3724,11 +3732,11 @@
     </row>
     <row r="187">
       <c r="A187" s="5" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>6</v>
@@ -3736,11 +3744,11 @@
     </row>
     <row r="188">
       <c r="A188" s="5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D188" s="5" t="s">
         <v>6</v>
@@ -3748,11 +3756,11 @@
     </row>
     <row r="189">
       <c r="A189" s="5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>6</v>
@@ -3760,11 +3768,11 @@
     </row>
     <row r="190">
       <c r="A190" s="5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>6</v>
@@ -3772,11 +3780,11 @@
     </row>
     <row r="191">
       <c r="A191" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>6</v>
@@ -3784,39 +3792,63 @@
     </row>
     <row r="192">
       <c r="A192" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="D192" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="B193" s="6"/>
+      <c r="C193" s="7" t="s">
         <v>367</v>
       </c>
-      <c r="D192" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="6"/>
-      <c r="B193" s="6"/>
-      <c r="C193" s="6"/>
-      <c r="D193" s="6"/>
+      <c r="D193" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="194">
-      <c r="A194" s="6"/>
+      <c r="A194" s="5" t="s">
+        <v>368</v>
+      </c>
       <c r="B194" s="6"/>
-      <c r="C194" s="6"/>
-      <c r="D194" s="6"/>
+      <c r="C194" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="D194" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="195">
-      <c r="A195" s="6"/>
+      <c r="A195" s="5" t="s">
+        <v>369</v>
+      </c>
       <c r="B195" s="6"/>
-      <c r="C195" s="6"/>
-      <c r="D195" s="6"/>
+      <c r="C195" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="D195" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="196">
-      <c r="A196" s="6"/>
+      <c r="A196" s="5" t="s">
+        <v>371</v>
+      </c>
       <c r="B196" s="6"/>
-      <c r="C196" s="6"/>
-      <c r="D196" s="6"/>
+      <c r="C196" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="D196" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="6"/>
@@ -9056,9 +9088,33 @@
       <c r="C1069" s="6"/>
       <c r="D1069" s="6"/>
     </row>
+    <row r="1070">
+      <c r="A1070" s="6"/>
+      <c r="B1070" s="6"/>
+      <c r="C1070" s="6"/>
+      <c r="D1070" s="6"/>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="6"/>
+      <c r="B1071" s="6"/>
+      <c r="C1071" s="6"/>
+      <c r="D1071" s="6"/>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="6"/>
+      <c r="B1072" s="6"/>
+      <c r="C1072" s="6"/>
+      <c r="D1072" s="6"/>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="6"/>
+      <c r="B1073" s="6"/>
+      <c r="C1073" s="6"/>
+      <c r="D1073" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D192">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D196">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Auth and sync user logic
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="372">
   <si>
     <t>Key</t>
   </si>
@@ -935,6 +935,9 @@
     <t>Born date is invalid.</t>
   </si>
   <si>
+    <t>onboarding.personal_info.error.default</t>
+  </si>
+  <si>
     <t>alarm.new.edit_vibration.intensity</t>
   </si>
   <si>
@@ -1131,6 +1134,9 @@
   </si>
   <si>
     <t>Alert</t>
+  </si>
+  <si>
+    <t>alarm.wake_up_score</t>
   </si>
   <si>
     <t>banner.calibration.title</t>
@@ -3369,11 +3375,11 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="12" t="s">
+      <c r="A157" s="5" t="s">
         <v>296</v>
       </c>
       <c r="B157" s="6"/>
-      <c r="C157" s="13" t="s">
+      <c r="C157" s="7" t="s">
         <v>297</v>
       </c>
       <c r="D157" s="5" t="s">
@@ -3381,12 +3387,12 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="5" t="s">
+      <c r="A158" s="12" t="s">
         <v>298</v>
       </c>
       <c r="B158" s="6"/>
-      <c r="C158" s="7" t="s">
-        <v>299</v>
+      <c r="C158" s="13" t="s">
+        <v>42</v>
       </c>
       <c r="D158" s="5" t="s">
         <v>6</v>
@@ -3394,11 +3400,11 @@
     </row>
     <row r="159">
       <c r="A159" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="7" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D159" s="5" t="s">
         <v>6</v>
@@ -3406,23 +3412,23 @@
     </row>
     <row r="160">
       <c r="A160" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="D160" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="s">
         <v>303</v>
-      </c>
-      <c r="D160" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="10" t="s">
-        <v>304</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="7" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D161" s="5" t="s">
         <v>6</v>
@@ -3430,11 +3436,11 @@
     </row>
     <row r="162">
       <c r="A162" s="10" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>6</v>
@@ -3442,11 +3448,11 @@
     </row>
     <row r="163">
       <c r="A163" s="10" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
@@ -3454,11 +3460,11 @@
     </row>
     <row r="164">
       <c r="A164" s="10" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
@@ -3466,11 +3472,11 @@
     </row>
     <row r="165">
       <c r="A165" s="10" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="7" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D165" s="5" t="s">
         <v>6</v>
@@ -3478,23 +3484,23 @@
     </row>
     <row r="166">
       <c r="A166" s="10" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="D166" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="10" t="s">
         <v>315</v>
-      </c>
-      <c r="D166" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="5" t="s">
-        <v>316</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="7" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D167" s="5" t="s">
         <v>6</v>
@@ -3502,11 +3508,11 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
@@ -3514,11 +3520,11 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="7" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D169" s="5" t="s">
         <v>6</v>
@@ -3526,11 +3532,11 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D170" s="5" t="s">
         <v>6</v>
@@ -3538,11 +3544,11 @@
     </row>
     <row r="171">
       <c r="A171" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D171" s="5" t="s">
         <v>6</v>
@@ -3550,11 +3556,11 @@
     </row>
     <row r="172">
       <c r="A172" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D172" s="5" t="s">
         <v>6</v>
@@ -3562,11 +3568,11 @@
     </row>
     <row r="173">
       <c r="A173" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="7" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D173" s="5" t="s">
         <v>6</v>
@@ -3574,11 +3580,11 @@
     </row>
     <row r="174">
       <c r="A174" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
@@ -3586,11 +3592,11 @@
     </row>
     <row r="175">
       <c r="A175" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
@@ -3598,11 +3604,11 @@
     </row>
     <row r="176">
       <c r="A176" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
@@ -3610,11 +3616,11 @@
     </row>
     <row r="177">
       <c r="A177" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
@@ -3622,11 +3628,11 @@
     </row>
     <row r="178">
       <c r="A178" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
@@ -3634,11 +3640,11 @@
     </row>
     <row r="179">
       <c r="A179" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
@@ -3646,11 +3652,11 @@
     </row>
     <row r="180">
       <c r="A180" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
@@ -3658,11 +3664,11 @@
     </row>
     <row r="181">
       <c r="A181" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
@@ -3670,11 +3676,11 @@
     </row>
     <row r="182">
       <c r="A182" s="5" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="7" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>6</v>
@@ -3682,11 +3688,11 @@
     </row>
     <row r="183">
       <c r="A183" s="5" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="7" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>6</v>
@@ -3694,11 +3700,11 @@
     </row>
     <row r="184">
       <c r="A184" s="5" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="7" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D184" s="5" t="s">
         <v>6</v>
@@ -3706,11 +3712,11 @@
     </row>
     <row r="185">
       <c r="A185" s="5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="7" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D185" s="5" t="s">
         <v>6</v>
@@ -3718,11 +3724,11 @@
     </row>
     <row r="186">
       <c r="A186" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="7" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D186" s="5" t="s">
         <v>6</v>
@@ -3730,11 +3736,11 @@
     </row>
     <row r="187">
       <c r="A187" s="5" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>6</v>
@@ -3742,11 +3748,11 @@
     </row>
     <row r="188">
       <c r="A188" s="5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D188" s="5" t="s">
         <v>6</v>
@@ -3754,11 +3760,11 @@
     </row>
     <row r="189">
       <c r="A189" s="5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>6</v>
@@ -3766,11 +3772,11 @@
     </row>
     <row r="190">
       <c r="A190" s="5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>6</v>
@@ -3778,23 +3784,23 @@
     </row>
     <row r="191">
       <c r="A191" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="D191" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="12" t="s">
         <v>365</v>
       </c>
-      <c r="D191" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="5" t="s">
-        <v>366</v>
-      </c>
       <c r="B192" s="6"/>
-      <c r="C192" s="7" t="s">
-        <v>367</v>
+      <c r="C192" s="13" t="s">
+        <v>149</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
@@ -3802,27 +3808,39 @@
     </row>
     <row r="193">
       <c r="A193" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="D193" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="B194" s="6"/>
+      <c r="C194" s="7" t="s">
         <v>369</v>
       </c>
-      <c r="D193" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" s="6"/>
-      <c r="B194" s="6"/>
-      <c r="C194" s="6"/>
-      <c r="D194" s="6"/>
+      <c r="D194" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="195">
-      <c r="A195" s="6"/>
+      <c r="A195" s="5" t="s">
+        <v>370</v>
+      </c>
       <c r="B195" s="6"/>
-      <c r="C195" s="6"/>
-      <c r="D195" s="6"/>
+      <c r="C195" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="D195" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="6"/>
@@ -9074,9 +9092,21 @@
       <c r="C1070" s="6"/>
       <c r="D1070" s="6"/>
     </row>
+    <row r="1071">
+      <c r="A1071" s="6"/>
+      <c r="B1071" s="6"/>
+      <c r="C1071" s="6"/>
+      <c r="D1071" s="6"/>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="6"/>
+      <c r="B1072" s="6"/>
+      <c r="C1072" s="6"/>
+      <c r="D1072" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D193">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D195">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Change navigation + Profile avatar
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="375">
   <si>
     <t>Key</t>
   </si>
@@ -626,6 +626,12 @@
   </si>
   <si>
     <t>PROFILE</t>
+  </si>
+  <si>
+    <t>profile.user_creation</t>
+  </si>
+  <si>
+    <t>User since {date}</t>
   </si>
   <si>
     <t>profile.logout</t>
@@ -1164,7 +1170,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1183,6 +1189,7 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -1220,7 +1227,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1255,6 +1262,12 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2795,11 +2808,11 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="5" t="s">
+      <c r="A109" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="B109" s="6"/>
-      <c r="C109" s="7" t="s">
+      <c r="B109" s="11"/>
+      <c r="C109" s="12" t="s">
         <v>201</v>
       </c>
       <c r="D109" s="5" t="s">
@@ -3011,7 +3024,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="8" t="s">
+      <c r="A127" s="5" t="s">
         <v>236</v>
       </c>
       <c r="B127" s="6"/>
@@ -3047,7 +3060,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="5" t="s">
+      <c r="A130" s="8" t="s">
         <v>242</v>
       </c>
       <c r="B130" s="6"/>
@@ -3143,7 +3156,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="11" t="s">
+      <c r="A138" s="5" t="s">
         <v>258</v>
       </c>
       <c r="B138" s="6"/>
@@ -3155,7 +3168,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="5" t="s">
+      <c r="A139" s="13" t="s">
         <v>260</v>
       </c>
       <c r="B139" s="6"/>
@@ -3203,7 +3216,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="8" t="s">
+      <c r="A143" s="5" t="s">
         <v>268</v>
       </c>
       <c r="B143" s="6"/>
@@ -3215,7 +3228,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="5" t="s">
+      <c r="A144" s="8" t="s">
         <v>270</v>
       </c>
       <c r="B144" s="6"/>
@@ -3388,7 +3401,7 @@
       </c>
       <c r="B158" s="6"/>
       <c r="C158" s="7" t="s">
-        <v>42</v>
+        <v>299</v>
       </c>
       <c r="D158" s="5" t="s">
         <v>6</v>
@@ -3396,11 +3409,11 @@
     </row>
     <row r="159">
       <c r="A159" s="5" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="7" t="s">
-        <v>300</v>
+        <v>42</v>
       </c>
       <c r="D159" s="5" t="s">
         <v>6</v>
@@ -3431,7 +3444,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="10" t="s">
+      <c r="A162" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B162" s="6"/>
@@ -3503,7 +3516,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="5" t="s">
+      <c r="A168" s="10" t="s">
         <v>317</v>
       </c>
       <c r="B168" s="6"/>
@@ -3796,7 +3809,7 @@
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
-        <v>149</v>
+        <v>366</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
@@ -3804,11 +3817,11 @@
     </row>
     <row r="193">
       <c r="A193" s="5" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>367</v>
+        <v>149</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
@@ -3820,7 +3833,7 @@
       </c>
       <c r="B194" s="6"/>
       <c r="C194" s="7" t="s">
-        <v>249</v>
+        <v>369</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>6</v>
@@ -3828,11 +3841,11 @@
     </row>
     <row r="195">
       <c r="A195" s="5" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B195" s="6"/>
       <c r="C195" s="7" t="s">
-        <v>370</v>
+        <v>251</v>
       </c>
       <c r="D195" s="5" t="s">
         <v>6</v>
@@ -3851,10 +3864,16 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="6"/>
+      <c r="A197" s="5" t="s">
+        <v>373</v>
+      </c>
       <c r="B197" s="6"/>
-      <c r="C197" s="6"/>
-      <c r="D197" s="6"/>
+      <c r="C197" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="D197" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="6"/>
@@ -9112,14 +9131,20 @@
       <c r="C1073" s="6"/>
       <c r="D1073" s="6"/>
     </row>
+    <row r="1074">
+      <c r="A1074" s="6"/>
+      <c r="B1074" s="6"/>
+      <c r="C1074" s="6"/>
+      <c r="D1074" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D196">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D197">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A138"/>
+    <hyperlink r:id="rId1" ref="A139"/>
   </hyperlinks>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
Display profile basic info + Edit name
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="398">
   <si>
     <t>Key</t>
   </si>
@@ -622,7 +622,7 @@
     <t>forgot_password.reset.confirm_password.placeholder</t>
   </si>
   <si>
-    <t>profile.header.title</t>
+    <t>header.profile</t>
   </si>
   <si>
     <t>PROFILE</t>
@@ -644,6 +644,81 @@
   </si>
   <si>
     <t>Global score</t>
+  </si>
+  <si>
+    <t>profile.list_header.profile</t>
+  </si>
+  <si>
+    <t>Profile</t>
+  </si>
+  <si>
+    <t>profile.list.profile_information</t>
+  </si>
+  <si>
+    <t>Profile Information</t>
+  </si>
+  <si>
+    <t>header.profile_information</t>
+  </si>
+  <si>
+    <t>profile_info.basic_info</t>
+  </si>
+  <si>
+    <t>Basic info</t>
+  </si>
+  <si>
+    <t>profile_info.name</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>profile_info.birthday</t>
+  </si>
+  <si>
+    <t>Birthday</t>
+  </si>
+  <si>
+    <t>profile_info.height</t>
+  </si>
+  <si>
+    <t>Height</t>
+  </si>
+  <si>
+    <t>profile_info.weight</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>profile_info.sex</t>
+  </si>
+  <si>
+    <t>Sex</t>
+  </si>
+  <si>
+    <t>profile_info.leaderboard</t>
+  </si>
+  <si>
+    <t>Participate in Leaderboards</t>
+  </si>
+  <si>
+    <t>profile_info.advanced_info</t>
+  </si>
+  <si>
+    <t>Advanced Information</t>
+  </si>
+  <si>
+    <t>profile_info.edit_name.title</t>
+  </si>
+  <si>
+    <t>Edit Name</t>
+  </si>
+  <si>
+    <t>profile_info.edit_name.save</t>
+  </si>
+  <si>
+    <t>Save</t>
   </si>
   <si>
     <t>header.live</t>
@@ -762,9 +837,6 @@
   </si>
   <si>
     <t>drawer.profile</t>
-  </si>
-  <si>
-    <t>Profile</t>
   </si>
   <si>
     <t>drawer.close</t>
@@ -999,9 +1071,6 @@
   </si>
   <si>
     <t>alarm.new.save_button</t>
-  </si>
-  <si>
-    <t>Save</t>
   </si>
   <si>
     <t>alarm.new.repeat.weekdays</t>
@@ -2796,7 +2865,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="5" t="s">
+      <c r="A108" s="11" t="s">
         <v>198</v>
       </c>
       <c r="B108" s="6"/>
@@ -2844,11 +2913,11 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="5" t="s">
+      <c r="A112" s="11" t="s">
         <v>206</v>
       </c>
       <c r="B112" s="6"/>
-      <c r="C112" s="7" t="s">
+      <c r="C112" s="12" t="s">
         <v>207</v>
       </c>
       <c r="D112" s="5" t="s">
@@ -2856,11 +2925,11 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="5" t="s">
+      <c r="A113" s="11" t="s">
         <v>208</v>
       </c>
       <c r="B113" s="6"/>
-      <c r="C113" s="7" t="s">
+      <c r="C113" s="12" t="s">
         <v>209</v>
       </c>
       <c r="D113" s="5" t="s">
@@ -2868,132 +2937,132 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="5" t="s">
+      <c r="A114" s="11" t="s">
         <v>210</v>
       </c>
       <c r="B114" s="6"/>
-      <c r="C114" s="7" t="s">
+      <c r="C114" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="D114" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="5" t="s">
+      <c r="B115" s="6"/>
+      <c r="C115" s="12" t="s">
         <v>212</v>
       </c>
-      <c r="B115" s="6"/>
-      <c r="C115" s="7" t="s">
+      <c r="D115" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="11" t="s">
         <v>213</v>
       </c>
-      <c r="D115" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="5" t="s">
+      <c r="B116" s="6"/>
+      <c r="C116" s="12" t="s">
         <v>214</v>
       </c>
-      <c r="B116" s="6"/>
-      <c r="C116" s="7" t="s">
+      <c r="D116" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="11" t="s">
         <v>215</v>
       </c>
-      <c r="D116" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="5" t="s">
+      <c r="B117" s="6"/>
+      <c r="C117" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="B117" s="6"/>
-      <c r="C117" s="7" t="s">
+      <c r="D117" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="s">
         <v>217</v>
       </c>
-      <c r="D117" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="5" t="s">
+      <c r="B118" s="6"/>
+      <c r="C118" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="B118" s="6"/>
-      <c r="C118" s="7" t="s">
+      <c r="D118" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="D118" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="5" t="s">
+      <c r="B119" s="6"/>
+      <c r="C119" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="B119" s="6"/>
-      <c r="C119" s="7" t="s">
+      <c r="D119" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="D119" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="5" t="s">
+      <c r="B120" s="6"/>
+      <c r="C120" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="B120" s="6"/>
-      <c r="C120" s="7" t="s">
+      <c r="D120" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="11" t="s">
         <v>223</v>
       </c>
-      <c r="D120" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="5" t="s">
+      <c r="B121" s="6"/>
+      <c r="C121" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="B121" s="6"/>
-      <c r="C121" s="7" t="s">
+      <c r="D121" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="D121" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="5" t="s">
+      <c r="B122" s="6"/>
+      <c r="C122" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="B122" s="6"/>
-      <c r="C122" s="7" t="s">
+      <c r="D122" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="11" t="s">
         <v>227</v>
       </c>
-      <c r="D122" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="5" t="s">
+      <c r="B123" s="6"/>
+      <c r="C123" s="12" t="s">
         <v>228</v>
       </c>
-      <c r="B123" s="6"/>
-      <c r="C123" s="7" t="s">
+      <c r="D123" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="s">
         <v>229</v>
       </c>
-      <c r="D123" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="5" t="s">
+      <c r="B124" s="6"/>
+      <c r="C124" s="12" t="s">
         <v>230</v>
-      </c>
-      <c r="B124" s="6"/>
-      <c r="C124" s="7" t="s">
-        <v>231</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -3001,11 +3070,11 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>6</v>
@@ -3013,11 +3082,11 @@
     </row>
     <row r="126">
       <c r="A126" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B126" s="6"/>
       <c r="C126" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D126" s="5" t="s">
         <v>6</v>
@@ -3025,47 +3094,47 @@
     </row>
     <row r="127">
       <c r="A127" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B127" s="6"/>
       <c r="C127" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="s">
         <v>237</v>
-      </c>
-      <c r="D127" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="8" t="s">
-        <v>238</v>
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="s">
         <v>239</v>
-      </c>
-      <c r="D128" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="8" t="s">
-        <v>240</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="s">
         <v>241</v>
-      </c>
-      <c r="D129" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="8" t="s">
-        <v>242</v>
       </c>
       <c r="B130" s="6"/>
       <c r="C130" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D130" s="5" t="s">
         <v>6</v>
@@ -3073,11 +3142,11 @@
     </row>
     <row r="131">
       <c r="A131" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B131" s="6"/>
       <c r="C131" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>6</v>
@@ -3085,11 +3154,11 @@
     </row>
     <row r="132">
       <c r="A132" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B132" s="6"/>
       <c r="C132" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D132" s="5" t="s">
         <v>6</v>
@@ -3097,11 +3166,11 @@
     </row>
     <row r="133">
       <c r="A133" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B133" s="6"/>
       <c r="C133" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>6</v>
@@ -3109,11 +3178,11 @@
     </row>
     <row r="134">
       <c r="A134" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B134" s="6"/>
       <c r="C134" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D134" s="5" t="s">
         <v>6</v>
@@ -3121,11 +3190,11 @@
     </row>
     <row r="135">
       <c r="A135" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B135" s="6"/>
       <c r="C135" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D135" s="5" t="s">
         <v>6</v>
@@ -3133,11 +3202,11 @@
     </row>
     <row r="136">
       <c r="A136" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B136" s="6"/>
       <c r="C136" s="7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D136" s="5" t="s">
         <v>6</v>
@@ -3145,11 +3214,11 @@
     </row>
     <row r="137">
       <c r="A137" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>6</v>
@@ -3157,23 +3226,23 @@
     </row>
     <row r="138">
       <c r="A138" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B138" s="6"/>
       <c r="C138" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="D138" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="s">
         <v>259</v>
-      </c>
-      <c r="D138" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="13" t="s">
-        <v>260</v>
       </c>
       <c r="B139" s="6"/>
       <c r="C139" s="7" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D139" s="5" t="s">
         <v>6</v>
@@ -3181,59 +3250,59 @@
     </row>
     <row r="140">
       <c r="A140" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B140" s="6"/>
       <c r="C140" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="D140" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="8" t="s">
         <v>263</v>
-      </c>
-      <c r="D140" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="5" t="s">
-        <v>264</v>
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="D141" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="8" t="s">
         <v>265</v>
-      </c>
-      <c r="D141" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="5" t="s">
-        <v>266</v>
       </c>
       <c r="B142" s="6"/>
       <c r="C142" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="D142" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="8" t="s">
         <v>267</v>
-      </c>
-      <c r="D142" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="5" t="s">
-        <v>268</v>
       </c>
       <c r="B143" s="6"/>
       <c r="C143" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="s">
         <v>269</v>
-      </c>
-      <c r="D143" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="8" t="s">
-        <v>270</v>
       </c>
       <c r="B144" s="6"/>
       <c r="C144" s="7" t="s">
-        <v>271</v>
+        <v>207</v>
       </c>
       <c r="D144" s="5" t="s">
         <v>6</v>
@@ -3241,11 +3310,11 @@
     </row>
     <row r="145">
       <c r="A145" s="5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B145" s="6"/>
       <c r="C145" s="7" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D145" s="5" t="s">
         <v>6</v>
@@ -3253,11 +3322,11 @@
     </row>
     <row r="146">
       <c r="A146" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B146" s="6"/>
       <c r="C146" s="7" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D146" s="5" t="s">
         <v>6</v>
@@ -3265,11 +3334,11 @@
     </row>
     <row r="147">
       <c r="A147" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B147" s="6"/>
       <c r="C147" s="7" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D147" s="5" t="s">
         <v>6</v>
@@ -3277,11 +3346,11 @@
     </row>
     <row r="148">
       <c r="A148" s="5" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B148" s="6"/>
       <c r="C148" s="7" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D148" s="5" t="s">
         <v>6</v>
@@ -3289,11 +3358,11 @@
     </row>
     <row r="149">
       <c r="A149" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B149" s="6"/>
       <c r="C149" s="7" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D149" s="5" t="s">
         <v>6</v>
@@ -3301,11 +3370,11 @@
     </row>
     <row r="150">
       <c r="A150" s="5" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B150" s="6"/>
       <c r="C150" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D150" s="5" t="s">
         <v>6</v>
@@ -3313,23 +3382,23 @@
     </row>
     <row r="151">
       <c r="A151" s="5" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B151" s="6"/>
       <c r="C151" s="7" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="D151" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="5" t="s">
-        <v>286</v>
+      <c r="A152" s="13" t="s">
+        <v>284</v>
       </c>
       <c r="B152" s="6"/>
       <c r="C152" s="7" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D152" s="5" t="s">
         <v>6</v>
@@ -3337,11 +3406,11 @@
     </row>
     <row r="153">
       <c r="A153" s="5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B153" s="6"/>
       <c r="C153" s="7" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D153" s="5" t="s">
         <v>6</v>
@@ -3349,11 +3418,11 @@
     </row>
     <row r="154">
       <c r="A154" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B154" s="6"/>
       <c r="C154" s="7" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D154" s="5" t="s">
         <v>6</v>
@@ -3361,11 +3430,11 @@
     </row>
     <row r="155">
       <c r="A155" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B155" s="6"/>
       <c r="C155" s="7" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D155" s="5" t="s">
         <v>6</v>
@@ -3373,23 +3442,23 @@
     </row>
     <row r="156">
       <c r="A156" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B156" s="6"/>
       <c r="C156" s="7" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="D156" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="5" t="s">
-        <v>296</v>
+      <c r="A157" s="8" t="s">
+        <v>294</v>
       </c>
       <c r="B157" s="6"/>
       <c r="C157" s="7" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D157" s="5" t="s">
         <v>6</v>
@@ -3397,11 +3466,11 @@
     </row>
     <row r="158">
       <c r="A158" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B158" s="6"/>
       <c r="C158" s="7" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D158" s="5" t="s">
         <v>6</v>
@@ -3409,11 +3478,11 @@
     </row>
     <row r="159">
       <c r="A159" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="7" t="s">
-        <v>42</v>
+        <v>299</v>
       </c>
       <c r="D159" s="5" t="s">
         <v>6</v>
@@ -3421,11 +3490,11 @@
     </row>
     <row r="160">
       <c r="A160" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D160" s="5" t="s">
         <v>6</v>
@@ -3433,11 +3502,11 @@
     </row>
     <row r="161">
       <c r="A161" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D161" s="5" t="s">
         <v>6</v>
@@ -3445,83 +3514,83 @@
     </row>
     <row r="162">
       <c r="A162" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="D162" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="s">
         <v>306</v>
-      </c>
-      <c r="D162" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="10" t="s">
-        <v>307</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="D163" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="s">
         <v>308</v>
-      </c>
-      <c r="D163" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="10" t="s">
-        <v>309</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="D164" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="s">
         <v>310</v>
-      </c>
-      <c r="D164" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="10" t="s">
-        <v>311</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="D165" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="s">
         <v>312</v>
-      </c>
-      <c r="D165" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="10" t="s">
-        <v>313</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="D166" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="s">
         <v>314</v>
-      </c>
-      <c r="D166" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="10" t="s">
-        <v>315</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="D167" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="s">
         <v>316</v>
-      </c>
-      <c r="D167" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="10" t="s">
-        <v>317</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
@@ -3529,11 +3598,11 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="7" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D169" s="5" t="s">
         <v>6</v>
@@ -3541,11 +3610,11 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="7" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D170" s="5" t="s">
         <v>6</v>
@@ -3553,11 +3622,11 @@
     </row>
     <row r="171">
       <c r="A171" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="7" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D171" s="5" t="s">
         <v>6</v>
@@ -3565,11 +3634,11 @@
     </row>
     <row r="172">
       <c r="A172" s="5" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="7" t="s">
-        <v>326</v>
+        <v>42</v>
       </c>
       <c r="D172" s="5" t="s">
         <v>6</v>
@@ -3577,11 +3646,11 @@
     </row>
     <row r="173">
       <c r="A173" s="5" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="7" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D173" s="5" t="s">
         <v>6</v>
@@ -3589,11 +3658,11 @@
     </row>
     <row r="174">
       <c r="A174" s="5" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
@@ -3601,83 +3670,83 @@
     </row>
     <row r="175">
       <c r="A175" s="5" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="5" t="s">
-        <v>333</v>
+      <c r="A176" s="10" t="s">
+        <v>331</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="5" t="s">
-        <v>335</v>
+      <c r="A177" s="10" t="s">
+        <v>333</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="5" t="s">
-        <v>337</v>
+      <c r="A178" s="10" t="s">
+        <v>335</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="5" t="s">
-        <v>339</v>
+      <c r="A179" s="10" t="s">
+        <v>337</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="5" t="s">
-        <v>341</v>
+      <c r="A180" s="10" t="s">
+        <v>339</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="5" t="s">
-        <v>343</v>
+      <c r="A181" s="10" t="s">
+        <v>341</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
@@ -3685,11 +3754,11 @@
     </row>
     <row r="182">
       <c r="A182" s="5" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="7" t="s">
-        <v>346</v>
+        <v>230</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>6</v>
@@ -3697,11 +3766,11 @@
     </row>
     <row r="183">
       <c r="A183" s="5" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="7" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>6</v>
@@ -3709,11 +3778,11 @@
     </row>
     <row r="184">
       <c r="A184" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="7" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="D184" s="5" t="s">
         <v>6</v>
@@ -3721,11 +3790,11 @@
     </row>
     <row r="185">
       <c r="A185" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="7" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="D185" s="5" t="s">
         <v>6</v>
@@ -3733,11 +3802,11 @@
     </row>
     <row r="186">
       <c r="A186" s="5" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="7" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="D186" s="5" t="s">
         <v>6</v>
@@ -3745,11 +3814,11 @@
     </row>
     <row r="187">
       <c r="A187" s="5" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>6</v>
@@ -3757,11 +3826,11 @@
     </row>
     <row r="188">
       <c r="A188" s="5" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="D188" s="5" t="s">
         <v>6</v>
@@ -3769,11 +3838,11 @@
     </row>
     <row r="189">
       <c r="A189" s="5" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="7" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>6</v>
@@ -3781,11 +3850,11 @@
     </row>
     <row r="190">
       <c r="A190" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>6</v>
@@ -3793,11 +3862,11 @@
     </row>
     <row r="191">
       <c r="A191" s="5" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>6</v>
@@ -3805,11 +3874,11 @@
     </row>
     <row r="192">
       <c r="A192" s="5" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
@@ -3817,11 +3886,11 @@
     </row>
     <row r="193">
       <c r="A193" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>149</v>
+        <v>365</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
@@ -3829,11 +3898,11 @@
     </row>
     <row r="194">
       <c r="A194" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B194" s="6"/>
       <c r="C194" s="7" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>6</v>
@@ -3841,11 +3910,11 @@
     </row>
     <row r="195">
       <c r="A195" s="5" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B195" s="6"/>
       <c r="C195" s="7" t="s">
-        <v>251</v>
+        <v>369</v>
       </c>
       <c r="D195" s="5" t="s">
         <v>6</v>
@@ -3853,11 +3922,11 @@
     </row>
     <row r="196">
       <c r="A196" s="5" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B196" s="6"/>
       <c r="C196" s="7" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D196" s="5" t="s">
         <v>6</v>
@@ -3865,93 +3934,171 @@
     </row>
     <row r="197">
       <c r="A197" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B197" s="6"/>
       <c r="C197" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="D197" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="D197" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" s="6"/>
       <c r="B198" s="6"/>
-      <c r="C198" s="6"/>
-      <c r="D198" s="6"/>
+      <c r="C198" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="D198" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="199">
-      <c r="A199" s="6"/>
+      <c r="A199" s="5" t="s">
+        <v>376</v>
+      </c>
       <c r="B199" s="6"/>
-      <c r="C199" s="6"/>
-      <c r="D199" s="6"/>
+      <c r="C199" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="D199" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="200">
-      <c r="A200" s="6"/>
+      <c r="A200" s="5" t="s">
+        <v>378</v>
+      </c>
       <c r="B200" s="6"/>
-      <c r="C200" s="6"/>
-      <c r="D200" s="6"/>
+      <c r="C200" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="D200" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="201">
-      <c r="A201" s="6"/>
+      <c r="A201" s="5" t="s">
+        <v>380</v>
+      </c>
       <c r="B201" s="6"/>
-      <c r="C201" s="6"/>
-      <c r="D201" s="6"/>
+      <c r="C201" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="D201" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="202">
-      <c r="A202" s="6"/>
+      <c r="A202" s="5" t="s">
+        <v>382</v>
+      </c>
       <c r="B202" s="6"/>
-      <c r="C202" s="6"/>
-      <c r="D202" s="6"/>
+      <c r="C202" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="D202" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="203">
-      <c r="A203" s="6"/>
+      <c r="A203" s="5" t="s">
+        <v>384</v>
+      </c>
       <c r="B203" s="6"/>
-      <c r="C203" s="6"/>
-      <c r="D203" s="6"/>
+      <c r="C203" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="D203" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="204">
-      <c r="A204" s="6"/>
+      <c r="A204" s="5" t="s">
+        <v>386</v>
+      </c>
       <c r="B204" s="6"/>
-      <c r="C204" s="6"/>
-      <c r="D204" s="6"/>
+      <c r="C204" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="D204" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="205">
-      <c r="A205" s="6"/>
+      <c r="A205" s="5" t="s">
+        <v>388</v>
+      </c>
       <c r="B205" s="6"/>
-      <c r="C205" s="6"/>
-      <c r="D205" s="6"/>
+      <c r="C205" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="D205" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="206">
-      <c r="A206" s="6"/>
+      <c r="A206" s="5" t="s">
+        <v>390</v>
+      </c>
       <c r="B206" s="6"/>
-      <c r="C206" s="6"/>
-      <c r="D206" s="6"/>
+      <c r="C206" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="D206" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="207">
-      <c r="A207" s="6"/>
+      <c r="A207" s="5" t="s">
+        <v>391</v>
+      </c>
       <c r="B207" s="6"/>
-      <c r="C207" s="6"/>
-      <c r="D207" s="6"/>
+      <c r="C207" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="D207" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="208">
-      <c r="A208" s="6"/>
+      <c r="A208" s="5" t="s">
+        <v>393</v>
+      </c>
       <c r="B208" s="6"/>
-      <c r="C208" s="6"/>
-      <c r="D208" s="6"/>
+      <c r="C208" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="D208" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="209">
-      <c r="A209" s="6"/>
+      <c r="A209" s="5" t="s">
+        <v>394</v>
+      </c>
       <c r="B209" s="6"/>
-      <c r="C209" s="6"/>
-      <c r="D209" s="6"/>
+      <c r="C209" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="D209" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="210">
-      <c r="A210" s="6"/>
+      <c r="A210" s="5" t="s">
+        <v>396</v>
+      </c>
       <c r="B210" s="6"/>
-      <c r="C210" s="6"/>
-      <c r="D210" s="6"/>
+      <c r="C210" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="D210" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="6"/>
@@ -9137,14 +9284,92 @@
       <c r="C1074" s="6"/>
       <c r="D1074" s="6"/>
     </row>
+    <row r="1075">
+      <c r="A1075" s="6"/>
+      <c r="B1075" s="6"/>
+      <c r="C1075" s="6"/>
+      <c r="D1075" s="6"/>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="6"/>
+      <c r="B1076" s="6"/>
+      <c r="C1076" s="6"/>
+      <c r="D1076" s="6"/>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="6"/>
+      <c r="B1077" s="6"/>
+      <c r="C1077" s="6"/>
+      <c r="D1077" s="6"/>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="6"/>
+      <c r="B1078" s="6"/>
+      <c r="C1078" s="6"/>
+      <c r="D1078" s="6"/>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="6"/>
+      <c r="B1079" s="6"/>
+      <c r="C1079" s="6"/>
+      <c r="D1079" s="6"/>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="6"/>
+      <c r="B1080" s="6"/>
+      <c r="C1080" s="6"/>
+      <c r="D1080" s="6"/>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="6"/>
+      <c r="B1081" s="6"/>
+      <c r="C1081" s="6"/>
+      <c r="D1081" s="6"/>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="6"/>
+      <c r="B1082" s="6"/>
+      <c r="C1082" s="6"/>
+      <c r="D1082" s="6"/>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="6"/>
+      <c r="B1083" s="6"/>
+      <c r="C1083" s="6"/>
+      <c r="D1083" s="6"/>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="6"/>
+      <c r="B1084" s="6"/>
+      <c r="C1084" s="6"/>
+      <c r="D1084" s="6"/>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="6"/>
+      <c r="B1085" s="6"/>
+      <c r="C1085" s="6"/>
+      <c r="D1085" s="6"/>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="6"/>
+      <c r="B1086" s="6"/>
+      <c r="C1086" s="6"/>
+      <c r="D1086" s="6"/>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="6"/>
+      <c r="B1087" s="6"/>
+      <c r="C1087" s="6"/>
+      <c r="D1087" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D197">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D210">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A139"/>
+    <hyperlink r:id="rId1" ref="A152"/>
   </hyperlinks>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
ask user location before scanning
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="407">
   <si>
     <t>Key</t>
   </si>
@@ -65,6 +65,21 @@
   </si>
   <si>
     <t>setup.scan.disabled.enable</t>
+  </si>
+  <si>
+    <t>setup.scan.location_disabled.title</t>
+  </si>
+  <si>
+    <t>Enable location</t>
+  </si>
+  <si>
+    <t>setup.scan.location_disabled.message</t>
+  </si>
+  <si>
+    <t>To be able to use bluetooth connection, Android needs your phone to enable location</t>
+  </si>
+  <si>
+    <t>setup.scan.location_disabled.enable</t>
   </si>
   <si>
     <t>setup.scan.enabled.title</t>
@@ -366,6 +381,21 @@
   </si>
   <si>
     <t>Next</t>
+  </si>
+  <si>
+    <t>global.cancel</t>
+  </si>
+  <si>
+    <t>Cancel</t>
+  </si>
+  <si>
+    <t>global.save</t>
+  </si>
+  <si>
+    <t>Save</t>
+  </si>
+  <si>
+    <t>global.continue</t>
   </si>
   <si>
     <t>home.sync.syncing</t>
@@ -622,12 +652,18 @@
     <t>forgot_password.reset.confirm_password.placeholder</t>
   </si>
   <si>
-    <t>profile.header.title</t>
+    <t>header.profile</t>
   </si>
   <si>
     <t>PROFILE</t>
   </si>
   <si>
+    <t>profile.user_creation</t>
+  </si>
+  <si>
+    <t>User since {date}</t>
+  </si>
+  <si>
     <t>profile.logout</t>
   </si>
   <si>
@@ -638,6 +674,75 @@
   </si>
   <si>
     <t>Global score</t>
+  </si>
+  <si>
+    <t>profile.list_header.profile</t>
+  </si>
+  <si>
+    <t>Profile</t>
+  </si>
+  <si>
+    <t>profile.list.profile_information</t>
+  </si>
+  <si>
+    <t>Profile Information</t>
+  </si>
+  <si>
+    <t>header.profile_information</t>
+  </si>
+  <si>
+    <t>profile_info.basic_info</t>
+  </si>
+  <si>
+    <t>Basic info</t>
+  </si>
+  <si>
+    <t>profile_info.name</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>profile_info.birthday</t>
+  </si>
+  <si>
+    <t>Birthday</t>
+  </si>
+  <si>
+    <t>profile_info.height</t>
+  </si>
+  <si>
+    <t>Height</t>
+  </si>
+  <si>
+    <t>profile_info.weight</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>profile_info.sex</t>
+  </si>
+  <si>
+    <t>Sex</t>
+  </si>
+  <si>
+    <t>profile_info.leaderboard</t>
+  </si>
+  <si>
+    <t>Participate in Leaderboards</t>
+  </si>
+  <si>
+    <t>profile_info.advanced_info</t>
+  </si>
+  <si>
+    <t>Advanced Information</t>
+  </si>
+  <si>
+    <t>profile_info.edit_name.title</t>
+  </si>
+  <si>
+    <t>Edit Name</t>
   </si>
   <si>
     <t>header.live</t>
@@ -756,9 +861,6 @@
   </si>
   <si>
     <t>drawer.profile</t>
-  </si>
-  <si>
-    <t>Profile</t>
   </si>
   <si>
     <t>drawer.close</t>
@@ -929,6 +1031,15 @@
     <t>Born date is required.</t>
   </si>
   <si>
+    <t>onboarding.personal_info.error.born_date_invalid</t>
+  </si>
+  <si>
+    <t>Born date is invalid.</t>
+  </si>
+  <si>
+    <t>onboarding.personal_info.error.default</t>
+  </si>
+  <si>
     <t>alarm.new.edit_vibration.intensity</t>
   </si>
   <si>
@@ -986,9 +1097,6 @@
     <t>alarm.new.save_button</t>
   </si>
   <si>
-    <t>Save</t>
-  </si>
-  <si>
     <t>alarm.new.repeat.weekdays</t>
   </si>
   <si>
@@ -1127,6 +1235,18 @@
     <t>Alert</t>
   </si>
   <si>
+    <t>alarm.wake_up_score</t>
+  </si>
+  <si>
+    <t>alarm.new.time.edit</t>
+  </si>
+  <si>
+    <t>Edit alarm time</t>
+  </si>
+  <si>
+    <t>alarm.week_overview</t>
+  </si>
+  <si>
     <t>banner.calibration.title</t>
   </si>
   <si>
@@ -1139,17 +1259,14 @@
     <t>Keep wearing your ring during the entirety of the {days} days calibration period for improved results!</t>
   </si>
   <si>
-    <t>alarm.new.time.edit</t>
-  </si>
-  <si>
-    <t>Edit alarm time</t>
+    <t>profile.header.title</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1168,11 +1285,20 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
     </font>
-    <font/>
+    <font>
+      <strike/>
+      <color rgb="FFFF0000"/>
+    </font>
+    <font>
+      <strike/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1206,7 +1332,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1234,6 +1360,9 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -1241,11 +1370,24 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1598,7 +1740,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="6"/>
@@ -1610,60 +1752,60 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="8" t="s">
         <v>22</v>
       </c>
       <c r="B11" s="6"/>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="s">
-        <v>24</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="s">
         <v>25</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="s">
         <v>27</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="s">
         <v>29</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>6</v>
@@ -1671,11 +1813,11 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>6</v>
@@ -1683,11 +1825,11 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>6</v>
@@ -1723,7 +1865,7 @@
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>6</v>
@@ -1731,11 +1873,11 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>6</v>
@@ -1743,11 +1885,11 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>6</v>
@@ -1755,11 +1897,11 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>6</v>
@@ -1767,11 +1909,11 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>6</v>
@@ -1779,23 +1921,23 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="7" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="5" t="s">
         <v>50</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>6</v>
@@ -1803,11 +1945,11 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="7" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>6</v>
@@ -1815,23 +1957,23 @@
     </row>
     <row r="28">
       <c r="A28" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="s">
-        <v>54</v>
+      <c r="A29" s="8" t="s">
+        <v>55</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="7" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>6</v>
@@ -1839,11 +1981,11 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>6</v>
@@ -1851,11 +1993,11 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>6</v>
@@ -1863,11 +2005,11 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>6</v>
@@ -1875,11 +2017,11 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>6</v>
@@ -1887,11 +2029,11 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>6</v>
@@ -1899,7 +2041,7 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
@@ -1911,11 +2053,11 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>6</v>
@@ -1923,11 +2065,11 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>6</v>
@@ -1935,11 +2077,11 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>6</v>
@@ -1951,7 +2093,7 @@
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="7" t="s">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>6</v>
@@ -1959,11 +2101,11 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>6</v>
@@ -1971,11 +2113,11 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>6</v>
@@ -1983,11 +2125,11 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>6</v>
@@ -1995,11 +2137,11 @@
     </row>
     <row r="43">
       <c r="A43" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>6</v>
@@ -2035,7 +2177,7 @@
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
-        <v>81</v>
+        <v>47</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>6</v>
@@ -2043,11 +2185,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>6</v>
@@ -2055,11 +2197,11 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>6</v>
@@ -2067,11 +2209,11 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>6</v>
@@ -2079,11 +2221,11 @@
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>6</v>
@@ -2091,11 +2233,11 @@
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>6</v>
@@ -2103,11 +2245,11 @@
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>6</v>
@@ -2115,11 +2257,11 @@
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>6</v>
@@ -2127,11 +2269,11 @@
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
-        <v>31</v>
+        <v>96</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>6</v>
@@ -2155,7 +2297,7 @@
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="7" t="s">
-        <v>29</v>
+        <v>100</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>6</v>
@@ -2163,11 +2305,11 @@
     </row>
     <row r="57">
       <c r="A57" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
-        <v>101</v>
+        <v>36</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>6</v>
@@ -2179,7 +2321,7 @@
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -2187,11 +2329,11 @@
     </row>
     <row r="59">
       <c r="A59" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B59" s="6"/>
       <c r="C59" s="7" t="s">
-        <v>104</v>
+        <v>34</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>6</v>
@@ -2215,7 +2357,7 @@
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="7" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>6</v>
@@ -2223,11 +2365,11 @@
     </row>
     <row r="62">
       <c r="A62" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B62" s="6"/>
       <c r="C62" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>6</v>
@@ -2235,11 +2377,11 @@
     </row>
     <row r="63">
       <c r="A63" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>6</v>
@@ -2247,35 +2389,37 @@
     </row>
     <row r="64">
       <c r="A64" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="D64" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="10" t="s">
+      <c r="B65" s="6"/>
+      <c r="C65" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="C65" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D65" s="10" t="s">
+      <c r="D65" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="10" t="s">
+      <c r="A66" s="5" t="s">
         <v>116</v>
       </c>
+      <c r="B66" s="6"/>
       <c r="C66" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="D66" s="10" t="s">
+      <c r="D66" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2292,72 +2436,67 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="s">
+      <c r="A68" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D68" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="D68" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="s">
+      <c r="C69" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="B69" s="6"/>
-      <c r="C69" s="7" t="s">
+      <c r="D69" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="D69" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="s">
+      <c r="C70" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B70" s="6"/>
-      <c r="C70" s="7" t="s">
+      <c r="D70" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="D70" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="s">
+      <c r="C71" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="B71" s="6"/>
-      <c r="C71" s="7" t="s">
+      <c r="D71" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="D71" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="B72" s="6"/>
-      <c r="C72" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="D72" s="5" t="s">
+      <c r="C72" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D72" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B73" s="6"/>
       <c r="C73" s="7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>6</v>
@@ -2365,11 +2504,11 @@
     </row>
     <row r="74">
       <c r="A74" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B74" s="6"/>
       <c r="C74" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D74" s="5" t="s">
         <v>6</v>
@@ -2377,11 +2516,11 @@
     </row>
     <row r="75">
       <c r="A75" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B75" s="6"/>
       <c r="C75" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D75" s="5" t="s">
         <v>6</v>
@@ -2389,11 +2528,11 @@
     </row>
     <row r="76">
       <c r="A76" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B76" s="6"/>
       <c r="C76" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D76" s="5" t="s">
         <v>6</v>
@@ -2401,11 +2540,11 @@
     </row>
     <row r="77">
       <c r="A77" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B77" s="6"/>
       <c r="C77" s="7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D77" s="5" t="s">
         <v>6</v>
@@ -2413,35 +2552,35 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B78" s="6"/>
       <c r="C78" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D78" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="s">
-        <v>142</v>
+      <c r="A79" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="B79" s="6"/>
       <c r="C79" s="7" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D79" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="s">
-        <v>144</v>
+      <c r="A80" s="5" t="s">
+        <v>142</v>
       </c>
       <c r="B80" s="6"/>
       <c r="C80" s="7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D80" s="5" t="s">
         <v>6</v>
@@ -2449,11 +2588,11 @@
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B81" s="6"/>
       <c r="C81" s="7" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>6</v>
@@ -2461,11 +2600,11 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B82" s="6"/>
       <c r="C82" s="7" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>6</v>
@@ -2473,11 +2612,11 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B83" s="6"/>
       <c r="C83" s="7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>6</v>
@@ -2485,35 +2624,35 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B84" s="6"/>
       <c r="C84" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="5" t="s">
-        <v>154</v>
+      <c r="A85" s="8" t="s">
+        <v>152</v>
       </c>
       <c r="B85" s="6"/>
       <c r="C85" s="7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="5" t="s">
-        <v>156</v>
+      <c r="A86" s="8" t="s">
+        <v>154</v>
       </c>
       <c r="B86" s="6"/>
       <c r="C86" s="7" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>6</v>
@@ -2521,11 +2660,11 @@
     </row>
     <row r="87">
       <c r="A87" s="5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B87" s="6"/>
       <c r="C87" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D87" s="5" t="s">
         <v>6</v>
@@ -2533,11 +2672,11 @@
     </row>
     <row r="88">
       <c r="A88" s="5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B88" s="6"/>
       <c r="C88" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>6</v>
@@ -2545,11 +2684,11 @@
     </row>
     <row r="89">
       <c r="A89" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B89" s="6"/>
       <c r="C89" s="7" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D89" s="5" t="s">
         <v>6</v>
@@ -2557,11 +2696,11 @@
     </row>
     <row r="90">
       <c r="A90" s="5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B90" s="6"/>
       <c r="C90" s="7" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D90" s="5" t="s">
         <v>6</v>
@@ -2569,11 +2708,11 @@
     </row>
     <row r="91">
       <c r="A91" s="5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B91" s="6"/>
       <c r="C91" s="7" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D91" s="5" t="s">
         <v>6</v>
@@ -2581,11 +2720,11 @@
     </row>
     <row r="92">
       <c r="A92" s="5" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B92" s="6"/>
       <c r="C92" s="7" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D92" s="5" t="s">
         <v>6</v>
@@ -2593,11 +2732,11 @@
     </row>
     <row r="93">
       <c r="A93" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B93" s="6"/>
       <c r="C93" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>6</v>
@@ -2605,11 +2744,11 @@
     </row>
     <row r="94">
       <c r="A94" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B94" s="6"/>
       <c r="C94" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D94" s="5" t="s">
         <v>6</v>
@@ -2617,11 +2756,11 @@
     </row>
     <row r="95">
       <c r="A95" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B95" s="6"/>
       <c r="C95" s="7" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D95" s="5" t="s">
         <v>6</v>
@@ -2629,11 +2768,11 @@
     </row>
     <row r="96">
       <c r="A96" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B96" s="6"/>
       <c r="C96" s="7" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D96" s="5" t="s">
         <v>6</v>
@@ -2641,11 +2780,11 @@
     </row>
     <row r="97">
       <c r="A97" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B97" s="6"/>
       <c r="C97" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D97" s="5" t="s">
         <v>6</v>
@@ -2653,11 +2792,11 @@
     </row>
     <row r="98">
       <c r="A98" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B98" s="6"/>
       <c r="C98" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D98" s="5" t="s">
         <v>6</v>
@@ -2665,11 +2804,11 @@
     </row>
     <row r="99">
       <c r="A99" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B99" s="6"/>
       <c r="C99" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>6</v>
@@ -2677,11 +2816,11 @@
     </row>
     <row r="100">
       <c r="A100" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>6</v>
@@ -2689,11 +2828,11 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B101" s="6"/>
       <c r="C101" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>6</v>
@@ -2701,11 +2840,11 @@
     </row>
     <row r="102">
       <c r="A102" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B102" s="6"/>
       <c r="C102" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>6</v>
@@ -2713,11 +2852,11 @@
     </row>
     <row r="103">
       <c r="A103" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B103" s="6"/>
       <c r="C103" s="7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>6</v>
@@ -2725,11 +2864,11 @@
     </row>
     <row r="104">
       <c r="A104" s="5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B104" s="6"/>
       <c r="C104" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>6</v>
@@ -2737,11 +2876,11 @@
     </row>
     <row r="105">
       <c r="A105" s="5" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D105" s="5" t="s">
         <v>6</v>
@@ -2749,11 +2888,11 @@
     </row>
     <row r="106">
       <c r="A106" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B106" s="6"/>
       <c r="C106" s="7" t="s">
-        <v>31</v>
+        <v>195</v>
       </c>
       <c r="D106" s="5" t="s">
         <v>6</v>
@@ -2761,11 +2900,11 @@
     </row>
     <row r="107">
       <c r="A107" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B107" s="6"/>
       <c r="C107" s="7" t="s">
-        <v>31</v>
+        <v>197</v>
       </c>
       <c r="D107" s="5" t="s">
         <v>6</v>
@@ -2825,7 +2964,7 @@
       </c>
       <c r="B112" s="6"/>
       <c r="C112" s="7" t="s">
-        <v>207</v>
+        <v>36</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>6</v>
@@ -2833,11 +2972,11 @@
     </row>
     <row r="113">
       <c r="A113" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B113" s="6"/>
       <c r="C113" s="7" t="s">
-        <v>209</v>
+        <v>36</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>6</v>
@@ -2845,11 +2984,11 @@
     </row>
     <row r="114">
       <c r="A114" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B114" s="6"/>
       <c r="C114" s="7" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>6</v>
@@ -2857,11 +2996,11 @@
     </row>
     <row r="115">
       <c r="A115" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="B115" s="6"/>
+        <v>210</v>
+      </c>
+      <c r="B115" s="5"/>
       <c r="C115" s="7" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>6</v>
@@ -2869,11 +3008,11 @@
     </row>
     <row r="116">
       <c r="A116" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B116" s="6"/>
       <c r="C116" s="7" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D116" s="5" t="s">
         <v>6</v>
@@ -2881,11 +3020,11 @@
     </row>
     <row r="117">
       <c r="A117" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B117" s="6"/>
       <c r="C117" s="7" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>6</v>
@@ -2893,11 +3032,11 @@
     </row>
     <row r="118">
       <c r="A118" s="5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B118" s="6"/>
       <c r="C118" s="7" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>6</v>
@@ -2905,11 +3044,11 @@
     </row>
     <row r="119">
       <c r="A119" s="5" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B119" s="6"/>
       <c r="C119" s="7" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>6</v>
@@ -2917,11 +3056,11 @@
     </row>
     <row r="120">
       <c r="A120" s="5" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B120" s="6"/>
       <c r="C120" s="7" t="s">
-        <v>223</v>
+        <v>209</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>6</v>
@@ -2929,11 +3068,11 @@
     </row>
     <row r="121">
       <c r="A121" s="5" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B121" s="6"/>
       <c r="C121" s="7" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>6</v>
@@ -2941,11 +3080,11 @@
     </row>
     <row r="122">
       <c r="A122" s="5" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B122" s="6"/>
       <c r="C122" s="7" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>6</v>
@@ -2953,11 +3092,11 @@
     </row>
     <row r="123">
       <c r="A123" s="5" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B123" s="6"/>
       <c r="C123" s="7" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>6</v>
@@ -2965,11 +3104,11 @@
     </row>
     <row r="124">
       <c r="A124" s="5" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -2977,59 +3116,59 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="5" t="s">
-        <v>234</v>
+      <c r="A126" s="8" t="s">
+        <v>231</v>
       </c>
       <c r="B126" s="6"/>
       <c r="C126" s="7" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D126" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="8" t="s">
-        <v>236</v>
+      <c r="A127" s="5" t="s">
+        <v>233</v>
       </c>
       <c r="B127" s="6"/>
       <c r="C127" s="7" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D127" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="8" t="s">
-        <v>238</v>
+      <c r="A128" s="5" t="s">
+        <v>235</v>
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="8" t="s">
-        <v>240</v>
+      <c r="A129" s="5" t="s">
+        <v>237</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="D129" s="5" t="s">
         <v>6</v>
@@ -3037,11 +3176,11 @@
     </row>
     <row r="130">
       <c r="A130" s="5" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B130" s="6"/>
       <c r="C130" s="7" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D130" s="5" t="s">
         <v>6</v>
@@ -3049,11 +3188,11 @@
     </row>
     <row r="131">
       <c r="A131" s="5" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B131" s="6"/>
       <c r="C131" s="7" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>6</v>
@@ -3061,11 +3200,11 @@
     </row>
     <row r="132">
       <c r="A132" s="5" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B132" s="6"/>
       <c r="C132" s="7" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D132" s="5" t="s">
         <v>6</v>
@@ -3073,11 +3212,11 @@
     </row>
     <row r="133">
       <c r="A133" s="5" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B133" s="6"/>
       <c r="C133" s="7" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>6</v>
@@ -3085,11 +3224,11 @@
     </row>
     <row r="134">
       <c r="A134" s="5" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B134" s="6"/>
       <c r="C134" s="7" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D134" s="5" t="s">
         <v>6</v>
@@ -3097,11 +3236,11 @@
     </row>
     <row r="135">
       <c r="A135" s="5" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B135" s="6"/>
       <c r="C135" s="7" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D135" s="5" t="s">
         <v>6</v>
@@ -3109,11 +3248,11 @@
     </row>
     <row r="136">
       <c r="A136" s="5" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B136" s="6"/>
       <c r="C136" s="7" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D136" s="5" t="s">
         <v>6</v>
@@ -3121,23 +3260,23 @@
     </row>
     <row r="137">
       <c r="A137" s="5" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="11" t="s">
-        <v>258</v>
+      <c r="A138" s="5" t="s">
+        <v>255</v>
       </c>
       <c r="B138" s="6"/>
       <c r="C138" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>6</v>
@@ -3145,11 +3284,11 @@
     </row>
     <row r="139">
       <c r="A139" s="5" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B139" s="6"/>
       <c r="C139" s="7" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D139" s="5" t="s">
         <v>6</v>
@@ -3157,11 +3296,11 @@
     </row>
     <row r="140">
       <c r="A140" s="5" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B140" s="6"/>
       <c r="C140" s="7" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D140" s="5" t="s">
         <v>6</v>
@@ -3169,11 +3308,11 @@
     </row>
     <row r="141">
       <c r="A141" s="5" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="7" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D141" s="5" t="s">
         <v>6</v>
@@ -3181,23 +3320,23 @@
     </row>
     <row r="142">
       <c r="A142" s="5" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B142" s="6"/>
       <c r="C142" s="7" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D142" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="8" t="s">
-        <v>268</v>
+      <c r="A143" s="5" t="s">
+        <v>265</v>
       </c>
       <c r="B143" s="6"/>
       <c r="C143" s="7" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D143" s="5" t="s">
         <v>6</v>
@@ -3205,11 +3344,11 @@
     </row>
     <row r="144">
       <c r="A144" s="5" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B144" s="6"/>
       <c r="C144" s="7" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D144" s="5" t="s">
         <v>6</v>
@@ -3217,47 +3356,47 @@
     </row>
     <row r="145">
       <c r="A145" s="5" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B145" s="6"/>
       <c r="C145" s="7" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D145" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="5" t="s">
-        <v>274</v>
+      <c r="A146" s="8" t="s">
+        <v>271</v>
       </c>
       <c r="B146" s="6"/>
       <c r="C146" s="7" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D146" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="5" t="s">
-        <v>276</v>
+      <c r="A147" s="8" t="s">
+        <v>273</v>
       </c>
       <c r="B147" s="6"/>
       <c r="C147" s="7" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D147" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="5" t="s">
-        <v>278</v>
+      <c r="A148" s="8" t="s">
+        <v>275</v>
       </c>
       <c r="B148" s="6"/>
       <c r="C148" s="7" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D148" s="5" t="s">
         <v>6</v>
@@ -3265,11 +3404,11 @@
     </row>
     <row r="149">
       <c r="A149" s="5" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B149" s="6"/>
       <c r="C149" s="7" t="s">
-        <v>281</v>
+        <v>217</v>
       </c>
       <c r="D149" s="5" t="s">
         <v>6</v>
@@ -3277,11 +3416,11 @@
     </row>
     <row r="150">
       <c r="A150" s="5" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="B150" s="6"/>
       <c r="C150" s="7" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="D150" s="5" t="s">
         <v>6</v>
@@ -3289,11 +3428,11 @@
     </row>
     <row r="151">
       <c r="A151" s="5" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="B151" s="6"/>
       <c r="C151" s="7" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="D151" s="5" t="s">
         <v>6</v>
@@ -3301,11 +3440,11 @@
     </row>
     <row r="152">
       <c r="A152" s="5" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="B152" s="6"/>
       <c r="C152" s="7" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="D152" s="5" t="s">
         <v>6</v>
@@ -3313,11 +3452,11 @@
     </row>
     <row r="153">
       <c r="A153" s="5" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="B153" s="6"/>
       <c r="C153" s="7" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="D153" s="5" t="s">
         <v>6</v>
@@ -3325,11 +3464,11 @@
     </row>
     <row r="154">
       <c r="A154" s="5" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="B154" s="6"/>
       <c r="C154" s="7" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D154" s="5" t="s">
         <v>6</v>
@@ -3337,11 +3476,11 @@
     </row>
     <row r="155">
       <c r="A155" s="5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B155" s="6"/>
       <c r="C155" s="7" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="D155" s="5" t="s">
         <v>6</v>
@@ -3349,23 +3488,23 @@
     </row>
     <row r="156">
       <c r="A156" s="5" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="B156" s="6"/>
       <c r="C156" s="7" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="D156" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="5" t="s">
-        <v>296</v>
+      <c r="A157" s="13" t="s">
+        <v>292</v>
       </c>
       <c r="B157" s="6"/>
       <c r="C157" s="7" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="D157" s="5" t="s">
         <v>6</v>
@@ -3373,11 +3512,11 @@
     </row>
     <row r="158">
       <c r="A158" s="5" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B158" s="6"/>
       <c r="C158" s="7" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D158" s="5" t="s">
         <v>6</v>
@@ -3385,83 +3524,83 @@
     </row>
     <row r="159">
       <c r="A159" s="5" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D159" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="10" t="s">
-        <v>302</v>
+      <c r="A160" s="5" t="s">
+        <v>298</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="7" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="D160" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="10" t="s">
-        <v>304</v>
+      <c r="A161" s="5" t="s">
+        <v>300</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="7" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D161" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="10" t="s">
-        <v>306</v>
+      <c r="A162" s="8" t="s">
+        <v>302</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="7" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="10" t="s">
-        <v>308</v>
+      <c r="A163" s="5" t="s">
+        <v>304</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="10" t="s">
-        <v>310</v>
+      <c r="A164" s="5" t="s">
+        <v>306</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="10" t="s">
-        <v>312</v>
+      <c r="A165" s="5" t="s">
+        <v>308</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="7" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D165" s="5" t="s">
         <v>6</v>
@@ -3469,11 +3608,11 @@
     </row>
     <row r="166">
       <c r="A166" s="5" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="7" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="D166" s="5" t="s">
         <v>6</v>
@@ -3481,11 +3620,11 @@
     </row>
     <row r="167">
       <c r="A167" s="5" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="7" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D167" s="5" t="s">
         <v>6</v>
@@ -3493,11 +3632,11 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
@@ -3505,11 +3644,11 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="7" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="D169" s="5" t="s">
         <v>6</v>
@@ -3517,11 +3656,11 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="7" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="D170" s="5" t="s">
         <v>6</v>
@@ -3529,11 +3668,11 @@
     </row>
     <row r="171">
       <c r="A171" s="5" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="7" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D171" s="5" t="s">
         <v>6</v>
@@ -3541,11 +3680,11 @@
     </row>
     <row r="172">
       <c r="A172" s="5" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="7" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="D172" s="5" t="s">
         <v>6</v>
@@ -3553,11 +3692,11 @@
     </row>
     <row r="173">
       <c r="A173" s="5" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="7" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="D173" s="5" t="s">
         <v>6</v>
@@ -3565,11 +3704,11 @@
     </row>
     <row r="174">
       <c r="A174" s="5" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
@@ -3577,11 +3716,11 @@
     </row>
     <row r="175">
       <c r="A175" s="5" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
@@ -3589,11 +3728,11 @@
     </row>
     <row r="176">
       <c r="A176" s="5" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
@@ -3601,11 +3740,11 @@
     </row>
     <row r="177">
       <c r="A177" s="5" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>337</v>
+        <v>47</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
@@ -3613,11 +3752,11 @@
     </row>
     <row r="178">
       <c r="A178" s="5" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
@@ -3625,11 +3764,11 @@
     </row>
     <row r="179">
       <c r="A179" s="5" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
@@ -3637,83 +3776,83 @@
     </row>
     <row r="180">
       <c r="A180" s="5" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="5" t="s">
-        <v>344</v>
+      <c r="A181" s="11" t="s">
+        <v>339</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="5" t="s">
-        <v>346</v>
+      <c r="A182" s="11" t="s">
+        <v>341</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="7" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="5" t="s">
-        <v>348</v>
+      <c r="A183" s="11" t="s">
+        <v>343</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="7" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="5" t="s">
-        <v>350</v>
+      <c r="A184" s="11" t="s">
+        <v>345</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="7" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D184" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="5" t="s">
-        <v>352</v>
+      <c r="A185" s="11" t="s">
+        <v>347</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="7" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D185" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="5" t="s">
-        <v>354</v>
+      <c r="A186" s="11" t="s">
+        <v>349</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="7" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="D186" s="5" t="s">
         <v>6</v>
@@ -3721,11 +3860,11 @@
     </row>
     <row r="187">
       <c r="A187" s="5" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
-        <v>357</v>
+        <v>126</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>6</v>
@@ -3733,11 +3872,11 @@
     </row>
     <row r="188">
       <c r="A188" s="5" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
       <c r="D188" s="5" t="s">
         <v>6</v>
@@ -3745,11 +3884,11 @@
     </row>
     <row r="189">
       <c r="A189" s="5" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="7" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>6</v>
@@ -3757,11 +3896,11 @@
     </row>
     <row r="190">
       <c r="A190" s="5" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>6</v>
@@ -3769,11 +3908,11 @@
     </row>
     <row r="191">
       <c r="A191" s="5" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="B191" s="6"/>
-      <c r="C191" s="12" t="s">
-        <v>365</v>
+      <c r="C191" s="7" t="s">
+        <v>359</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>6</v>
@@ -3781,159 +3920,325 @@
     </row>
     <row r="192">
       <c r="A192" s="5" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="D192" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="B193" s="6"/>
+      <c r="C193" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="D193" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="B194" s="6"/>
+      <c r="C194" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="D194" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="B195" s="6"/>
+      <c r="C195" s="7" t="s">
         <v>367</v>
       </c>
-      <c r="D192" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="6"/>
-      <c r="B193" s="6"/>
-      <c r="C193" s="6"/>
-      <c r="D193" s="6"/>
-    </row>
-    <row r="194">
-      <c r="A194" s="6"/>
-      <c r="B194" s="6"/>
-      <c r="C194" s="6"/>
-      <c r="D194" s="6"/>
-    </row>
-    <row r="195">
-      <c r="A195" s="6"/>
-      <c r="B195" s="6"/>
-      <c r="C195" s="6"/>
-      <c r="D195" s="6"/>
+      <c r="D195" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="196">
-      <c r="A196" s="6"/>
+      <c r="A196" s="5" t="s">
+        <v>368</v>
+      </c>
       <c r="B196" s="6"/>
-      <c r="C196" s="6"/>
-      <c r="D196" s="6"/>
+      <c r="C196" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="D196" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="197">
-      <c r="A197" s="6"/>
+      <c r="A197" s="5" t="s">
+        <v>370</v>
+      </c>
       <c r="B197" s="6"/>
-      <c r="C197" s="6"/>
-      <c r="D197" s="6"/>
+      <c r="C197" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="D197" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="198">
-      <c r="A198" s="6"/>
+      <c r="A198" s="5" t="s">
+        <v>372</v>
+      </c>
       <c r="B198" s="6"/>
-      <c r="C198" s="6"/>
-      <c r="D198" s="6"/>
+      <c r="C198" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="D198" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="199">
-      <c r="A199" s="6"/>
+      <c r="A199" s="5" t="s">
+        <v>374</v>
+      </c>
       <c r="B199" s="6"/>
-      <c r="C199" s="6"/>
-      <c r="D199" s="6"/>
+      <c r="C199" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="D199" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="200">
-      <c r="A200" s="6"/>
+      <c r="A200" s="5" t="s">
+        <v>376</v>
+      </c>
       <c r="B200" s="6"/>
-      <c r="C200" s="6"/>
-      <c r="D200" s="6"/>
+      <c r="C200" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="D200" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="201">
-      <c r="A201" s="6"/>
+      <c r="A201" s="5" t="s">
+        <v>378</v>
+      </c>
       <c r="B201" s="6"/>
-      <c r="C201" s="6"/>
-      <c r="D201" s="6"/>
+      <c r="C201" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="D201" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="202">
-      <c r="A202" s="6"/>
+      <c r="A202" s="5" t="s">
+        <v>380</v>
+      </c>
       <c r="B202" s="6"/>
-      <c r="C202" s="6"/>
-      <c r="D202" s="6"/>
+      <c r="C202" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="D202" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="203">
-      <c r="A203" s="6"/>
+      <c r="A203" s="5" t="s">
+        <v>382</v>
+      </c>
       <c r="B203" s="6"/>
-      <c r="C203" s="6"/>
-      <c r="D203" s="6"/>
+      <c r="C203" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="D203" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="204">
-      <c r="A204" s="6"/>
+      <c r="A204" s="5" t="s">
+        <v>384</v>
+      </c>
       <c r="B204" s="6"/>
-      <c r="C204" s="6"/>
-      <c r="D204" s="6"/>
+      <c r="C204" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="D204" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="205">
-      <c r="A205" s="6"/>
+      <c r="A205" s="5" t="s">
+        <v>386</v>
+      </c>
       <c r="B205" s="6"/>
-      <c r="C205" s="6"/>
-      <c r="D205" s="6"/>
+      <c r="C205" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="D205" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="206">
-      <c r="A206" s="6"/>
+      <c r="A206" s="5" t="s">
+        <v>388</v>
+      </c>
       <c r="B206" s="6"/>
-      <c r="C206" s="6"/>
-      <c r="D206" s="6"/>
+      <c r="C206" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="D206" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="207">
-      <c r="A207" s="6"/>
+      <c r="A207" s="5" t="s">
+        <v>390</v>
+      </c>
       <c r="B207" s="6"/>
-      <c r="C207" s="6"/>
-      <c r="D207" s="6"/>
+      <c r="C207" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="D207" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="208">
-      <c r="A208" s="6"/>
+      <c r="A208" s="5" t="s">
+        <v>392</v>
+      </c>
       <c r="B208" s="6"/>
-      <c r="C208" s="6"/>
-      <c r="D208" s="6"/>
+      <c r="C208" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="D208" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="209">
-      <c r="A209" s="6"/>
+      <c r="A209" s="5" t="s">
+        <v>394</v>
+      </c>
       <c r="B209" s="6"/>
-      <c r="C209" s="6"/>
-      <c r="D209" s="6"/>
+      <c r="C209" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="D209" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="210">
-      <c r="A210" s="6"/>
+      <c r="A210" s="5" t="s">
+        <v>396</v>
+      </c>
       <c r="B210" s="6"/>
-      <c r="C210" s="6"/>
-      <c r="D210" s="6"/>
+      <c r="C210" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="D210" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="211">
-      <c r="A211" s="6"/>
+      <c r="A211" s="5" t="s">
+        <v>398</v>
+      </c>
       <c r="B211" s="6"/>
-      <c r="C211" s="6"/>
-      <c r="D211" s="6"/>
+      <c r="C211" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="D211" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="212">
-      <c r="A212" s="6"/>
+      <c r="A212" s="5" t="s">
+        <v>399</v>
+      </c>
       <c r="B212" s="6"/>
-      <c r="C212" s="6"/>
-      <c r="D212" s="6"/>
+      <c r="C212" s="7" t="s">
+        <v>400</v>
+      </c>
+      <c r="D212" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="213">
-      <c r="A213" s="6"/>
+      <c r="A213" s="5" t="s">
+        <v>401</v>
+      </c>
       <c r="B213" s="6"/>
-      <c r="C213" s="6"/>
-      <c r="D213" s="6"/>
+      <c r="C213" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="D213" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="214">
-      <c r="A214" s="6"/>
+      <c r="A214" s="5" t="s">
+        <v>402</v>
+      </c>
       <c r="B214" s="6"/>
-      <c r="C214" s="6"/>
-      <c r="D214" s="6"/>
+      <c r="C214" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="D214" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="215">
-      <c r="A215" s="6"/>
+      <c r="A215" s="5" t="s">
+        <v>404</v>
+      </c>
       <c r="B215" s="6"/>
-      <c r="C215" s="6"/>
-      <c r="D215" s="6"/>
+      <c r="C215" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="D215" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="216">
-      <c r="A216" s="6"/>
-      <c r="B216" s="6"/>
-      <c r="C216" s="6"/>
-      <c r="D216" s="6"/>
+      <c r="A216" s="14" t="s">
+        <v>406</v>
+      </c>
+      <c r="B216" s="15"/>
+      <c r="C216" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="D216" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E216" s="18"/>
+      <c r="F216" s="18"/>
+      <c r="G216" s="18"/>
+      <c r="H216" s="18"/>
+      <c r="I216" s="18"/>
+      <c r="J216" s="18"/>
+      <c r="K216" s="18"/>
+      <c r="L216" s="18"/>
+      <c r="M216" s="18"/>
+      <c r="N216" s="18"/>
+      <c r="O216" s="18"/>
+      <c r="P216" s="18"/>
+      <c r="Q216" s="18"/>
+      <c r="R216" s="18"/>
+      <c r="S216" s="18"/>
+      <c r="T216" s="18"/>
+      <c r="U216" s="18"/>
+      <c r="V216" s="18"/>
+      <c r="W216" s="18"/>
+      <c r="X216" s="18"/>
+      <c r="Y216" s="18"/>
+      <c r="Z216" s="18"/>
     </row>
     <row r="217">
       <c r="A217" s="6"/>
@@ -9053,14 +9358,152 @@
       <c r="C1069" s="6"/>
       <c r="D1069" s="6"/>
     </row>
+    <row r="1070">
+      <c r="A1070" s="6"/>
+      <c r="B1070" s="6"/>
+      <c r="C1070" s="6"/>
+      <c r="D1070" s="6"/>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="6"/>
+      <c r="B1071" s="6"/>
+      <c r="C1071" s="6"/>
+      <c r="D1071" s="6"/>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="6"/>
+      <c r="B1072" s="6"/>
+      <c r="C1072" s="6"/>
+      <c r="D1072" s="6"/>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="6"/>
+      <c r="B1073" s="6"/>
+      <c r="C1073" s="6"/>
+      <c r="D1073" s="6"/>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="6"/>
+      <c r="B1074" s="6"/>
+      <c r="C1074" s="6"/>
+      <c r="D1074" s="6"/>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="6"/>
+      <c r="B1075" s="6"/>
+      <c r="C1075" s="6"/>
+      <c r="D1075" s="6"/>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="6"/>
+      <c r="B1076" s="6"/>
+      <c r="C1076" s="6"/>
+      <c r="D1076" s="6"/>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="6"/>
+      <c r="B1077" s="6"/>
+      <c r="C1077" s="6"/>
+      <c r="D1077" s="6"/>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="6"/>
+      <c r="B1078" s="6"/>
+      <c r="C1078" s="6"/>
+      <c r="D1078" s="6"/>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="6"/>
+      <c r="B1079" s="6"/>
+      <c r="C1079" s="6"/>
+      <c r="D1079" s="6"/>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="6"/>
+      <c r="B1080" s="6"/>
+      <c r="C1080" s="6"/>
+      <c r="D1080" s="6"/>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="6"/>
+      <c r="B1081" s="6"/>
+      <c r="C1081" s="6"/>
+      <c r="D1081" s="6"/>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="6"/>
+      <c r="B1082" s="6"/>
+      <c r="C1082" s="6"/>
+      <c r="D1082" s="6"/>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="6"/>
+      <c r="B1083" s="6"/>
+      <c r="C1083" s="6"/>
+      <c r="D1083" s="6"/>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="6"/>
+      <c r="B1084" s="6"/>
+      <c r="C1084" s="6"/>
+      <c r="D1084" s="6"/>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="6"/>
+      <c r="B1085" s="6"/>
+      <c r="C1085" s="6"/>
+      <c r="D1085" s="6"/>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="6"/>
+      <c r="B1086" s="6"/>
+      <c r="C1086" s="6"/>
+      <c r="D1086" s="6"/>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="6"/>
+      <c r="B1087" s="6"/>
+      <c r="C1087" s="6"/>
+      <c r="D1087" s="6"/>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="6"/>
+      <c r="B1088" s="6"/>
+      <c r="C1088" s="6"/>
+      <c r="D1088" s="6"/>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="6"/>
+      <c r="B1089" s="6"/>
+      <c r="C1089" s="6"/>
+      <c r="D1089" s="6"/>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="6"/>
+      <c r="B1090" s="6"/>
+      <c r="C1090" s="6"/>
+      <c r="D1090" s="6"/>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="6"/>
+      <c r="B1091" s="6"/>
+      <c r="C1091" s="6"/>
+      <c r="D1091" s="6"/>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="6"/>
+      <c r="B1092" s="6"/>
+      <c r="C1092" s="6"/>
+      <c r="D1092" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D192">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D216">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A138"/>
+    <hyperlink r:id="rId1" ref="A157"/>
   </hyperlinks>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
Edit height, weight and sex
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="417">
   <si>
     <t>Key</t>
   </si>
@@ -65,6 +65,21 @@
   </si>
   <si>
     <t>setup.scan.disabled.enable</t>
+  </si>
+  <si>
+    <t>setup.scan.location_disabled.title</t>
+  </si>
+  <si>
+    <t>Enable location</t>
+  </si>
+  <si>
+    <t>setup.scan.location_disabled.message</t>
+  </si>
+  <si>
+    <t>To be able to use bluetooth connection, Android needs your phone to enable location</t>
+  </si>
+  <si>
+    <t>setup.scan.location_disabled.enable</t>
   </si>
   <si>
     <t>setup.scan.enabled.title</t>
@@ -366,6 +381,24 @@
   </si>
   <si>
     <t>Next</t>
+  </si>
+  <si>
+    <t>global.cancel</t>
+  </si>
+  <si>
+    <t>Cancel</t>
+  </si>
+  <si>
+    <t>global.save</t>
+  </si>
+  <si>
+    <t>Save</t>
+  </si>
+  <si>
+    <t>global.continue</t>
+  </si>
+  <si>
+    <t>global.default_error</t>
   </si>
   <si>
     <t>home.sync.syncing</t>
@@ -685,18 +718,43 @@
     <t>Height</t>
   </si>
   <si>
+    <t>profile_info.bottom_sheet.height</t>
+  </si>
+  <si>
+    <t>Select your Height</t>
+  </si>
+  <si>
     <t>profile_info.weight</t>
   </si>
   <si>
     <t>Weight</t>
   </si>
   <si>
+    <t>profile_info.bottom_sheet.weight</t>
+  </si>
+  <si>
+    <t>Select your Weight</t>
+  </si>
+  <si>
     <t>profile_info.sex</t>
   </si>
   <si>
     <t>Sex</t>
   </si>
   <si>
+    <t>profile_info.bottom_sheet.sex.title</t>
+  </si>
+  <si>
+    <t>Please Confirm</t>
+  </si>
+  <si>
+    <t>profile_info.bottom_sheet.sex.description</t>
+  </si>
+  <si>
+    <t>Confirm that you want to change your sex.
+By doing so, many of your profile parameters will be modified.</t>
+  </si>
+  <si>
     <t>profile_info.leaderboard</t>
   </si>
   <si>
@@ -716,9 +774,6 @@
   </si>
   <si>
     <t>profile_info.edit_name.save</t>
-  </si>
-  <si>
-    <t>Save</t>
   </si>
   <si>
     <t>header.live</t>
@@ -1234,12 +1289,15 @@
   <si>
     <t>Keep wearing your ring during the entirety of the {days} days calibration period for improved results!</t>
   </si>
+  <si>
+    <t>profile.header.title</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1263,8 +1321,17 @@
       <u/>
       <color rgb="FF0000FF"/>
     </font>
+    <font>
+      <strike/>
+      <color rgb="FFFF0000"/>
+    </font>
+    <font>
+      <strike/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1289,6 +1356,12 @@
         <bgColor rgb="FFFFA500"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -1296,7 +1369,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1324,6 +1397,9 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -1331,14 +1407,36 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1691,7 +1789,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="6"/>
@@ -1703,60 +1801,60 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="8" t="s">
         <v>22</v>
       </c>
       <c r="B11" s="6"/>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="s">
-        <v>24</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="s">
         <v>25</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="s">
         <v>27</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="s">
         <v>29</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>6</v>
@@ -1764,11 +1862,11 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>6</v>
@@ -1776,11 +1874,11 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>6</v>
@@ -1816,7 +1914,7 @@
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>6</v>
@@ -1824,11 +1922,11 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>6</v>
@@ -1836,11 +1934,11 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>6</v>
@@ -1848,11 +1946,11 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>6</v>
@@ -1860,11 +1958,11 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>6</v>
@@ -1872,23 +1970,23 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="7" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="5" t="s">
         <v>50</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>6</v>
@@ -1896,11 +1994,11 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="7" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>6</v>
@@ -1908,23 +2006,23 @@
     </row>
     <row r="28">
       <c r="A28" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="s">
-        <v>54</v>
+      <c r="A29" s="8" t="s">
+        <v>55</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="7" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>6</v>
@@ -1932,11 +2030,11 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>6</v>
@@ -1944,11 +2042,11 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>6</v>
@@ -1956,11 +2054,11 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>6</v>
@@ -1968,11 +2066,11 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>6</v>
@@ -1980,11 +2078,11 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>6</v>
@@ -1992,7 +2090,7 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
@@ -2004,11 +2102,11 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>6</v>
@@ -2016,11 +2114,11 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>6</v>
@@ -2028,11 +2126,11 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>6</v>
@@ -2044,7 +2142,7 @@
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="7" t="s">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>6</v>
@@ -2052,11 +2150,11 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>6</v>
@@ -2064,11 +2162,11 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>6</v>
@@ -2076,11 +2174,11 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>6</v>
@@ -2088,11 +2186,11 @@
     </row>
     <row r="43">
       <c r="A43" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>6</v>
@@ -2128,7 +2226,7 @@
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
-        <v>81</v>
+        <v>47</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>6</v>
@@ -2136,11 +2234,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>6</v>
@@ -2148,11 +2246,11 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>6</v>
@@ -2160,11 +2258,11 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>6</v>
@@ -2172,11 +2270,11 @@
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>6</v>
@@ -2184,11 +2282,11 @@
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>6</v>
@@ -2196,11 +2294,11 @@
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>6</v>
@@ -2208,11 +2306,11 @@
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>6</v>
@@ -2220,11 +2318,11 @@
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
-        <v>31</v>
+        <v>96</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>6</v>
@@ -2248,7 +2346,7 @@
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="7" t="s">
-        <v>29</v>
+        <v>100</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>6</v>
@@ -2256,11 +2354,11 @@
     </row>
     <row r="57">
       <c r="A57" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
-        <v>101</v>
+        <v>36</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>6</v>
@@ -2272,7 +2370,7 @@
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -2280,11 +2378,11 @@
     </row>
     <row r="59">
       <c r="A59" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B59" s="6"/>
       <c r="C59" s="7" t="s">
-        <v>104</v>
+        <v>34</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>6</v>
@@ -2308,7 +2406,7 @@
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="7" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>6</v>
@@ -2316,11 +2414,11 @@
     </row>
     <row r="62">
       <c r="A62" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B62" s="6"/>
       <c r="C62" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>6</v>
@@ -2328,11 +2426,11 @@
     </row>
     <row r="63">
       <c r="A63" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>6</v>
@@ -2340,35 +2438,37 @@
     </row>
     <row r="64">
       <c r="A64" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="D64" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="10" t="s">
+      <c r="B65" s="6"/>
+      <c r="C65" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="C65" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D65" s="10" t="s">
+      <c r="D65" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="10" t="s">
+      <c r="A66" s="5" t="s">
         <v>116</v>
       </c>
+      <c r="B66" s="6"/>
       <c r="C66" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="D66" s="10" t="s">
+      <c r="D66" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2385,84 +2485,78 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="s">
+      <c r="A68" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D68" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="D68" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="s">
+      <c r="C69" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="B69" s="6"/>
-      <c r="C69" s="7" t="s">
+      <c r="D69" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="D69" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="s">
+      <c r="C70" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B70" s="6"/>
-      <c r="C70" s="7" t="s">
+      <c r="D70" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="D70" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="s">
+      <c r="C71" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="B71" s="6"/>
-      <c r="C71" s="7" t="s">
+      <c r="D71" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="D71" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="s">
+      <c r="C72" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D72" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="B72" s="6"/>
-      <c r="C72" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="D72" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="B73" s="6"/>
-      <c r="C73" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="D73" s="5" t="s">
+      <c r="C73" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D73" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B74" s="6"/>
       <c r="C74" s="7" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D74" s="5" t="s">
         <v>6</v>
@@ -2470,11 +2564,11 @@
     </row>
     <row r="75">
       <c r="A75" s="5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B75" s="6"/>
       <c r="C75" s="7" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D75" s="5" t="s">
         <v>6</v>
@@ -2482,11 +2576,11 @@
     </row>
     <row r="76">
       <c r="A76" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B76" s="6"/>
       <c r="C76" s="7" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D76" s="5" t="s">
         <v>6</v>
@@ -2494,11 +2588,11 @@
     </row>
     <row r="77">
       <c r="A77" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B77" s="6"/>
       <c r="C77" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D77" s="5" t="s">
         <v>6</v>
@@ -2506,35 +2600,35 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B78" s="6"/>
       <c r="C78" s="7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D78" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="s">
-        <v>142</v>
+      <c r="A79" s="5" t="s">
+        <v>139</v>
       </c>
       <c r="B79" s="6"/>
       <c r="C79" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D79" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="s">
-        <v>144</v>
+      <c r="A80" s="5" t="s">
+        <v>141</v>
       </c>
       <c r="B80" s="6"/>
       <c r="C80" s="7" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D80" s="5" t="s">
         <v>6</v>
@@ -2542,11 +2636,11 @@
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B81" s="6"/>
       <c r="C81" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>6</v>
@@ -2554,11 +2648,11 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B82" s="6"/>
       <c r="C82" s="7" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>6</v>
@@ -2566,11 +2660,11 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B83" s="6"/>
       <c r="C83" s="7" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>6</v>
@@ -2578,11 +2672,11 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B84" s="6"/>
       <c r="C84" s="7" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>6</v>
@@ -2590,35 +2684,35 @@
     </row>
     <row r="85">
       <c r="A85" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B85" s="6"/>
       <c r="C85" s="7" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="5" t="s">
-        <v>156</v>
+      <c r="A86" s="8" t="s">
+        <v>153</v>
       </c>
       <c r="B86" s="6"/>
       <c r="C86" s="7" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="5" t="s">
-        <v>158</v>
+      <c r="A87" s="8" t="s">
+        <v>155</v>
       </c>
       <c r="B87" s="6"/>
       <c r="C87" s="7" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D87" s="5" t="s">
         <v>6</v>
@@ -2626,11 +2720,11 @@
     </row>
     <row r="88">
       <c r="A88" s="5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B88" s="6"/>
       <c r="C88" s="7" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>6</v>
@@ -2638,11 +2732,11 @@
     </row>
     <row r="89">
       <c r="A89" s="5" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B89" s="6"/>
       <c r="C89" s="7" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D89" s="5" t="s">
         <v>6</v>
@@ -2650,11 +2744,11 @@
     </row>
     <row r="90">
       <c r="A90" s="5" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B90" s="6"/>
       <c r="C90" s="7" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D90" s="5" t="s">
         <v>6</v>
@@ -2662,11 +2756,11 @@
     </row>
     <row r="91">
       <c r="A91" s="5" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B91" s="6"/>
       <c r="C91" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D91" s="5" t="s">
         <v>6</v>
@@ -2674,11 +2768,11 @@
     </row>
     <row r="92">
       <c r="A92" s="5" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B92" s="6"/>
       <c r="C92" s="7" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D92" s="5" t="s">
         <v>6</v>
@@ -2686,11 +2780,11 @@
     </row>
     <row r="93">
       <c r="A93" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B93" s="6"/>
       <c r="C93" s="7" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>6</v>
@@ -2698,11 +2792,11 @@
     </row>
     <row r="94">
       <c r="A94" s="5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B94" s="6"/>
       <c r="C94" s="7" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D94" s="5" t="s">
         <v>6</v>
@@ -2710,11 +2804,11 @@
     </row>
     <row r="95">
       <c r="A95" s="5" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B95" s="6"/>
       <c r="C95" s="7" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D95" s="5" t="s">
         <v>6</v>
@@ -2722,11 +2816,11 @@
     </row>
     <row r="96">
       <c r="A96" s="5" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B96" s="6"/>
       <c r="C96" s="7" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D96" s="5" t="s">
         <v>6</v>
@@ -2734,11 +2828,11 @@
     </row>
     <row r="97">
       <c r="A97" s="5" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B97" s="6"/>
       <c r="C97" s="7" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D97" s="5" t="s">
         <v>6</v>
@@ -2746,11 +2840,11 @@
     </row>
     <row r="98">
       <c r="A98" s="5" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B98" s="6"/>
       <c r="C98" s="7" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D98" s="5" t="s">
         <v>6</v>
@@ -2758,11 +2852,11 @@
     </row>
     <row r="99">
       <c r="A99" s="5" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B99" s="6"/>
       <c r="C99" s="7" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>6</v>
@@ -2770,11 +2864,11 @@
     </row>
     <row r="100">
       <c r="A100" s="5" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>6</v>
@@ -2782,11 +2876,11 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B101" s="6"/>
       <c r="C101" s="7" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>6</v>
@@ -2794,11 +2888,11 @@
     </row>
     <row r="102">
       <c r="A102" s="5" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B102" s="6"/>
       <c r="C102" s="7" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>6</v>
@@ -2806,11 +2900,11 @@
     </row>
     <row r="103">
       <c r="A103" s="5" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B103" s="6"/>
       <c r="C103" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>6</v>
@@ -2818,11 +2912,11 @@
     </row>
     <row r="104">
       <c r="A104" s="5" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B104" s="6"/>
       <c r="C104" s="7" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>6</v>
@@ -2830,11 +2924,11 @@
     </row>
     <row r="105">
       <c r="A105" s="5" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="7" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D105" s="5" t="s">
         <v>6</v>
@@ -2842,11 +2936,11 @@
     </row>
     <row r="106">
       <c r="A106" s="5" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B106" s="6"/>
       <c r="C106" s="7" t="s">
-        <v>31</v>
+        <v>194</v>
       </c>
       <c r="D106" s="5" t="s">
         <v>6</v>
@@ -2854,35 +2948,35 @@
     </row>
     <row r="107">
       <c r="A107" s="5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B107" s="6"/>
       <c r="C107" s="7" t="s">
-        <v>31</v>
+        <v>196</v>
       </c>
       <c r="D107" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="11" t="s">
-        <v>198</v>
+      <c r="A108" s="5" t="s">
+        <v>197</v>
       </c>
       <c r="B108" s="6"/>
       <c r="C108" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="D108" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="11" t="s">
+      <c r="B109" s="6"/>
+      <c r="C109" s="7" t="s">
         <v>200</v>
-      </c>
-      <c r="B109" s="11"/>
-      <c r="C109" s="12" t="s">
-        <v>201</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>6</v>
@@ -2890,11 +2984,11 @@
     </row>
     <row r="110">
       <c r="A110" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B110" s="6"/>
       <c r="C110" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>6</v>
@@ -2902,167 +2996,167 @@
     </row>
     <row r="111">
       <c r="A111" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B111" s="6"/>
       <c r="C111" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="D111" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="11" t="s">
+      <c r="B112" s="6"/>
+      <c r="C112" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="B112" s="6"/>
-      <c r="C112" s="12" t="s">
+      <c r="D112" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="D112" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="11" t="s">
+      <c r="B113" s="6"/>
+      <c r="C113" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D113" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="B113" s="6"/>
-      <c r="C113" s="12" t="s">
+      <c r="B114" s="6"/>
+      <c r="C114" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="D113" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="11" t="s">
+      <c r="B115" s="6"/>
+      <c r="C115" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="B114" s="6"/>
-      <c r="C114" s="12" t="s">
-        <v>199</v>
-      </c>
-      <c r="D114" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="11" t="s">
+      <c r="D115" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="B115" s="6"/>
-      <c r="C115" s="12" t="s">
+      <c r="B116" s="5"/>
+      <c r="C116" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="D115" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="11" t="s">
+      <c r="D116" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="B116" s="6"/>
-      <c r="C116" s="12" t="s">
+      <c r="B117" s="6"/>
+      <c r="C117" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="D116" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="11" t="s">
+      <c r="D117" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B117" s="6"/>
-      <c r="C117" s="12" t="s">
+      <c r="B118" s="6"/>
+      <c r="C118" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="D117" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="11" t="s">
+      <c r="D118" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="B118" s="6"/>
-      <c r="C118" s="12" t="s">
+      <c r="B119" s="6"/>
+      <c r="C119" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="D118" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="11" t="s">
+      <c r="D119" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="B119" s="6"/>
-      <c r="C119" s="12" t="s">
+      <c r="B120" s="6"/>
+      <c r="C120" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="D119" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="8" t="s">
+      <c r="D120" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="B120" s="6"/>
-      <c r="C120" s="12" t="s">
+      <c r="B121" s="6"/>
+      <c r="C121" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="D120" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="11" t="s">
+      <c r="B122" s="6"/>
+      <c r="C122" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="B121" s="6"/>
-      <c r="C121" s="12" t="s">
+      <c r="D122" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="D121" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="11" t="s">
+      <c r="B123" s="6"/>
+      <c r="C123" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="B122" s="6"/>
-      <c r="C122" s="12" t="s">
+      <c r="D123" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="D122" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="11" t="s">
+      <c r="B124" s="6"/>
+      <c r="C124" s="7" t="s">
         <v>227</v>
-      </c>
-      <c r="B123" s="6"/>
-      <c r="C123" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="D123" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="B124" s="6"/>
-      <c r="C124" s="12" t="s">
-        <v>230</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -3070,23 +3164,23 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="5" t="s">
-        <v>233</v>
+      <c r="A126" s="13" t="s">
+        <v>230</v>
       </c>
       <c r="B126" s="6"/>
-      <c r="C126" s="7" t="s">
-        <v>234</v>
+      <c r="C126" s="9" t="s">
+        <v>231</v>
       </c>
       <c r="D126" s="5" t="s">
         <v>6</v>
@@ -3094,59 +3188,59 @@
     </row>
     <row r="127">
       <c r="A127" s="5" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B127" s="6"/>
       <c r="C127" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="B128" s="6"/>
+      <c r="C128" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="s">
         <v>236</v>
-      </c>
-      <c r="D127" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="B128" s="6"/>
-      <c r="C128" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="D128" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="5" t="s">
-        <v>239</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="B130" s="6"/>
+      <c r="C130" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="D129" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="5" t="s">
+      <c r="B131" s="6"/>
+      <c r="C131" s="9" t="s">
         <v>241</v>
-      </c>
-      <c r="B130" s="6"/>
-      <c r="C130" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="D130" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="B131" s="6"/>
-      <c r="C131" s="7" t="s">
-        <v>244</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>6</v>
@@ -3154,11 +3248,11 @@
     </row>
     <row r="132">
       <c r="A132" s="5" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B132" s="6"/>
       <c r="C132" s="7" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D132" s="5" t="s">
         <v>6</v>
@@ -3166,11 +3260,11 @@
     </row>
     <row r="133">
       <c r="A133" s="5" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B133" s="6"/>
       <c r="C133" s="7" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>6</v>
@@ -3178,35 +3272,35 @@
     </row>
     <row r="134">
       <c r="A134" s="5" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B134" s="6"/>
       <c r="C134" s="7" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D134" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="B135" s="6"/>
-      <c r="C135" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="D135" s="5" t="s">
+      <c r="A135" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="B135" s="15"/>
+      <c r="C135" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="D135" s="16" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B136" s="6"/>
       <c r="C136" s="7" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="D136" s="5" t="s">
         <v>6</v>
@@ -3214,11 +3308,11 @@
     </row>
     <row r="137">
       <c r="A137" s="5" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>6</v>
@@ -3226,11 +3320,11 @@
     </row>
     <row r="138">
       <c r="A138" s="5" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B138" s="6"/>
       <c r="C138" s="7" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>6</v>
@@ -3238,11 +3332,11 @@
     </row>
     <row r="139">
       <c r="A139" s="5" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="B139" s="6"/>
       <c r="C139" s="7" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="D139" s="5" t="s">
         <v>6</v>
@@ -3250,47 +3344,47 @@
     </row>
     <row r="140">
       <c r="A140" s="5" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B140" s="6"/>
       <c r="C140" s="7" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D140" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="8" t="s">
-        <v>263</v>
+      <c r="A141" s="5" t="s">
+        <v>259</v>
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="7" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="D141" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="8" t="s">
-        <v>265</v>
+      <c r="A142" s="5" t="s">
+        <v>261</v>
       </c>
       <c r="B142" s="6"/>
       <c r="C142" s="7" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="D142" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="8" t="s">
-        <v>267</v>
+      <c r="A143" s="5" t="s">
+        <v>263</v>
       </c>
       <c r="B143" s="6"/>
       <c r="C143" s="7" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="D143" s="5" t="s">
         <v>6</v>
@@ -3298,11 +3392,11 @@
     </row>
     <row r="144">
       <c r="A144" s="5" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="B144" s="6"/>
       <c r="C144" s="7" t="s">
-        <v>207</v>
+        <v>266</v>
       </c>
       <c r="D144" s="5" t="s">
         <v>6</v>
@@ -3310,11 +3404,11 @@
     </row>
     <row r="145">
       <c r="A145" s="5" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B145" s="6"/>
       <c r="C145" s="7" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D145" s="5" t="s">
         <v>6</v>
@@ -3322,11 +3416,11 @@
     </row>
     <row r="146">
       <c r="A146" s="5" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B146" s="6"/>
       <c r="C146" s="7" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D146" s="5" t="s">
         <v>6</v>
@@ -3334,11 +3428,11 @@
     </row>
     <row r="147">
       <c r="A147" s="5" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="B147" s="6"/>
       <c r="C147" s="7" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D147" s="5" t="s">
         <v>6</v>
@@ -3346,11 +3440,11 @@
     </row>
     <row r="148">
       <c r="A148" s="5" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B148" s="6"/>
       <c r="C148" s="7" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D148" s="5" t="s">
         <v>6</v>
@@ -3358,11 +3452,11 @@
     </row>
     <row r="149">
       <c r="A149" s="5" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B149" s="6"/>
       <c r="C149" s="7" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D149" s="5" t="s">
         <v>6</v>
@@ -3370,11 +3464,11 @@
     </row>
     <row r="150">
       <c r="A150" s="5" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B150" s="6"/>
       <c r="C150" s="7" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="D150" s="5" t="s">
         <v>6</v>
@@ -3382,47 +3476,47 @@
     </row>
     <row r="151">
       <c r="A151" s="5" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B151" s="6"/>
       <c r="C151" s="7" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D151" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="13" t="s">
-        <v>284</v>
+      <c r="A152" s="8" t="s">
+        <v>281</v>
       </c>
       <c r="B152" s="6"/>
       <c r="C152" s="7" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="D152" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="5" t="s">
-        <v>286</v>
+      <c r="A153" s="8" t="s">
+        <v>283</v>
       </c>
       <c r="B153" s="6"/>
       <c r="C153" s="7" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="D153" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="5" t="s">
-        <v>288</v>
+      <c r="A154" s="8" t="s">
+        <v>285</v>
       </c>
       <c r="B154" s="6"/>
       <c r="C154" s="7" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D154" s="5" t="s">
         <v>6</v>
@@ -3430,11 +3524,11 @@
     </row>
     <row r="155">
       <c r="A155" s="5" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="B155" s="6"/>
       <c r="C155" s="7" t="s">
-        <v>291</v>
+        <v>218</v>
       </c>
       <c r="D155" s="5" t="s">
         <v>6</v>
@@ -3442,23 +3536,23 @@
     </row>
     <row r="156">
       <c r="A156" s="5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B156" s="6"/>
       <c r="C156" s="7" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="D156" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="8" t="s">
-        <v>294</v>
+      <c r="A157" s="5" t="s">
+        <v>290</v>
       </c>
       <c r="B157" s="6"/>
       <c r="C157" s="7" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="D157" s="5" t="s">
         <v>6</v>
@@ -3466,11 +3560,11 @@
     </row>
     <row r="158">
       <c r="A158" s="5" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B158" s="6"/>
       <c r="C158" s="7" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="D158" s="5" t="s">
         <v>6</v>
@@ -3478,11 +3572,11 @@
     </row>
     <row r="159">
       <c r="A159" s="5" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="7" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D159" s="5" t="s">
         <v>6</v>
@@ -3490,11 +3584,11 @@
     </row>
     <row r="160">
       <c r="A160" s="5" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D160" s="5" t="s">
         <v>6</v>
@@ -3502,11 +3596,11 @@
     </row>
     <row r="161">
       <c r="A161" s="5" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="7" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="D161" s="5" t="s">
         <v>6</v>
@@ -3514,23 +3608,23 @@
     </row>
     <row r="162">
       <c r="A162" s="5" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="7" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="5" t="s">
-        <v>306</v>
+      <c r="A163" s="17" t="s">
+        <v>302</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
@@ -3538,11 +3632,11 @@
     </row>
     <row r="164">
       <c r="A164" s="5" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
@@ -3550,11 +3644,11 @@
     </row>
     <row r="165">
       <c r="A165" s="5" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="7" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="D165" s="5" t="s">
         <v>6</v>
@@ -3562,11 +3656,11 @@
     </row>
     <row r="166">
       <c r="A166" s="5" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="7" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D166" s="5" t="s">
         <v>6</v>
@@ -3574,23 +3668,23 @@
     </row>
     <row r="167">
       <c r="A167" s="5" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="7" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="D167" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="5" t="s">
-        <v>316</v>
+      <c r="A168" s="8" t="s">
+        <v>312</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
@@ -3598,11 +3692,11 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="7" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="D169" s="5" t="s">
         <v>6</v>
@@ -3610,11 +3704,11 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="7" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="D170" s="5" t="s">
         <v>6</v>
@@ -3622,11 +3716,11 @@
     </row>
     <row r="171">
       <c r="A171" s="5" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="7" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="D171" s="5" t="s">
         <v>6</v>
@@ -3634,11 +3728,11 @@
     </row>
     <row r="172">
       <c r="A172" s="5" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="7" t="s">
-        <v>42</v>
+        <v>321</v>
       </c>
       <c r="D172" s="5" t="s">
         <v>6</v>
@@ -3646,11 +3740,11 @@
     </row>
     <row r="173">
       <c r="A173" s="5" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="7" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="D173" s="5" t="s">
         <v>6</v>
@@ -3658,11 +3752,11 @@
     </row>
     <row r="174">
       <c r="A174" s="5" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
@@ -3670,83 +3764,83 @@
     </row>
     <row r="175">
       <c r="A175" s="5" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="10" t="s">
-        <v>331</v>
+      <c r="A176" s="5" t="s">
+        <v>328</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="10" t="s">
-        <v>333</v>
+      <c r="A177" s="5" t="s">
+        <v>330</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="10" t="s">
-        <v>335</v>
+      <c r="A178" s="5" t="s">
+        <v>332</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="10" t="s">
-        <v>337</v>
+      <c r="A179" s="5" t="s">
+        <v>334</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="10" t="s">
-        <v>339</v>
+      <c r="A180" s="5" t="s">
+        <v>336</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="10" t="s">
-        <v>341</v>
+      <c r="A181" s="5" t="s">
+        <v>338</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
@@ -3754,11 +3848,11 @@
     </row>
     <row r="182">
       <c r="A182" s="5" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="7" t="s">
-        <v>230</v>
+        <v>341</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>6</v>
@@ -3766,11 +3860,11 @@
     </row>
     <row r="183">
       <c r="A183" s="5" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="7" t="s">
-        <v>345</v>
+        <v>47</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>6</v>
@@ -3778,11 +3872,11 @@
     </row>
     <row r="184">
       <c r="A184" s="5" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="7" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="D184" s="5" t="s">
         <v>6</v>
@@ -3790,11 +3884,11 @@
     </row>
     <row r="185">
       <c r="A185" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="7" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="D185" s="5" t="s">
         <v>6</v>
@@ -3802,83 +3896,83 @@
     </row>
     <row r="186">
       <c r="A186" s="5" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="7" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="D186" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="5" t="s">
-        <v>352</v>
+      <c r="A187" s="11" t="s">
+        <v>349</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="5" t="s">
-        <v>354</v>
+      <c r="A188" s="11" t="s">
+        <v>351</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="D188" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="5" t="s">
-        <v>356</v>
+      <c r="A189" s="11" t="s">
+        <v>353</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="7" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="5" t="s">
-        <v>358</v>
+      <c r="A190" s="11" t="s">
+        <v>355</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="5" t="s">
-        <v>360</v>
+      <c r="A191" s="11" t="s">
+        <v>357</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="5" t="s">
-        <v>362</v>
+      <c r="A192" s="11" t="s">
+        <v>359</v>
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
@@ -3886,11 +3980,11 @@
     </row>
     <row r="193">
       <c r="A193" s="5" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>365</v>
+        <v>126</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
@@ -3898,11 +3992,11 @@
     </row>
     <row r="194">
       <c r="A194" s="5" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="B194" s="6"/>
       <c r="C194" s="7" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>6</v>
@@ -3910,11 +4004,11 @@
     </row>
     <row r="195">
       <c r="A195" s="5" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="B195" s="6"/>
       <c r="C195" s="7" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="D195" s="5" t="s">
         <v>6</v>
@@ -3922,11 +4016,11 @@
     </row>
     <row r="196">
       <c r="A196" s="5" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="B196" s="6"/>
       <c r="C196" s="7" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="D196" s="5" t="s">
         <v>6</v>
@@ -3934,11 +4028,11 @@
     </row>
     <row r="197">
       <c r="A197" s="5" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="B197" s="6"/>
       <c r="C197" s="7" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="D197" s="5" t="s">
         <v>6</v>
@@ -3946,11 +4040,11 @@
     </row>
     <row r="198">
       <c r="A198" s="5" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="B198" s="6"/>
       <c r="C198" s="7" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="D198" s="5" t="s">
         <v>6</v>
@@ -3958,11 +4052,11 @@
     </row>
     <row r="199">
       <c r="A199" s="5" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="B199" s="6"/>
       <c r="C199" s="7" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="D199" s="5" t="s">
         <v>6</v>
@@ -3970,11 +4064,11 @@
     </row>
     <row r="200">
       <c r="A200" s="5" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="B200" s="6"/>
       <c r="C200" s="7" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="D200" s="5" t="s">
         <v>6</v>
@@ -3982,11 +4076,11 @@
     </row>
     <row r="201">
       <c r="A201" s="5" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="B201" s="6"/>
       <c r="C201" s="7" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="D201" s="5" t="s">
         <v>6</v>
@@ -3994,11 +4088,11 @@
     </row>
     <row r="202">
       <c r="A202" s="5" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="B202" s="6"/>
       <c r="C202" s="7" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D202" s="5" t="s">
         <v>6</v>
@@ -4006,11 +4100,11 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="B203" s="6"/>
       <c r="C203" s="7" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="D203" s="5" t="s">
         <v>6</v>
@@ -4018,11 +4112,11 @@
     </row>
     <row r="204">
       <c r="A204" s="5" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="B204" s="6"/>
       <c r="C204" s="7" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="D204" s="5" t="s">
         <v>6</v>
@@ -4030,11 +4124,11 @@
     </row>
     <row r="205">
       <c r="A205" s="5" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="B205" s="6"/>
       <c r="C205" s="7" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="D205" s="5" t="s">
         <v>6</v>
@@ -4042,11 +4136,11 @@
     </row>
     <row r="206">
       <c r="A206" s="5" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="B206" s="6"/>
       <c r="C206" s="7" t="s">
-        <v>149</v>
+        <v>387</v>
       </c>
       <c r="D206" s="5" t="s">
         <v>6</v>
@@ -4054,11 +4148,11 @@
     </row>
     <row r="207">
       <c r="A207" s="5" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="B207" s="6"/>
       <c r="C207" s="7" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="D207" s="5" t="s">
         <v>6</v>
@@ -4066,11 +4160,11 @@
     </row>
     <row r="208">
       <c r="A208" s="5" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="B208" s="6"/>
       <c r="C208" s="7" t="s">
-        <v>275</v>
+        <v>391</v>
       </c>
       <c r="D208" s="5" t="s">
         <v>6</v>
@@ -4078,11 +4172,11 @@
     </row>
     <row r="209">
       <c r="A209" s="5" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B209" s="6"/>
       <c r="C209" s="7" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D209" s="5" t="s">
         <v>6</v>
@@ -4090,87 +4184,181 @@
     </row>
     <row r="210">
       <c r="A210" s="5" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B210" s="6"/>
       <c r="C210" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="D210" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="B211" s="6"/>
+      <c r="C211" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="D210" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" s="6"/>
-      <c r="B211" s="6"/>
-      <c r="C211" s="6"/>
-      <c r="D211" s="6"/>
+      <c r="D211" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="212">
-      <c r="A212" s="6"/>
+      <c r="A212" s="5" t="s">
+        <v>398</v>
+      </c>
       <c r="B212" s="6"/>
-      <c r="C212" s="6"/>
-      <c r="D212" s="6"/>
+      <c r="C212" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="D212" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="213">
-      <c r="A213" s="6"/>
+      <c r="A213" s="5" t="s">
+        <v>400</v>
+      </c>
       <c r="B213" s="6"/>
-      <c r="C213" s="6"/>
-      <c r="D213" s="6"/>
+      <c r="C213" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="D213" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="214">
-      <c r="A214" s="6"/>
+      <c r="A214" s="5" t="s">
+        <v>402</v>
+      </c>
       <c r="B214" s="6"/>
-      <c r="C214" s="6"/>
-      <c r="D214" s="6"/>
+      <c r="C214" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="D214" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="215">
-      <c r="A215" s="6"/>
+      <c r="A215" s="5" t="s">
+        <v>404</v>
+      </c>
       <c r="B215" s="6"/>
-      <c r="C215" s="6"/>
-      <c r="D215" s="6"/>
+      <c r="C215" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="D215" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="216">
-      <c r="A216" s="6"/>
+      <c r="A216" s="5" t="s">
+        <v>406</v>
+      </c>
       <c r="B216" s="6"/>
-      <c r="C216" s="6"/>
-      <c r="D216" s="6"/>
+      <c r="C216" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="D216" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="217">
-      <c r="A217" s="6"/>
+      <c r="A217" s="5" t="s">
+        <v>408</v>
+      </c>
       <c r="B217" s="6"/>
-      <c r="C217" s="6"/>
-      <c r="D217" s="6"/>
+      <c r="C217" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D217" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="218">
-      <c r="A218" s="6"/>
+      <c r="A218" s="5" t="s">
+        <v>409</v>
+      </c>
       <c r="B218" s="6"/>
-      <c r="C218" s="6"/>
-      <c r="D218" s="6"/>
+      <c r="C218" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="D218" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="219">
-      <c r="A219" s="6"/>
+      <c r="A219" s="5" t="s">
+        <v>411</v>
+      </c>
       <c r="B219" s="6"/>
-      <c r="C219" s="6"/>
-      <c r="D219" s="6"/>
+      <c r="C219" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="D219" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="220">
-      <c r="A220" s="6"/>
+      <c r="A220" s="5" t="s">
+        <v>412</v>
+      </c>
       <c r="B220" s="6"/>
-      <c r="C220" s="6"/>
-      <c r="D220" s="6"/>
+      <c r="C220" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D220" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="221">
-      <c r="A221" s="6"/>
+      <c r="A221" s="5" t="s">
+        <v>414</v>
+      </c>
       <c r="B221" s="6"/>
-      <c r="C221" s="6"/>
-      <c r="D221" s="6"/>
+      <c r="C221" s="7" t="s">
+        <v>415</v>
+      </c>
+      <c r="D221" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="222">
-      <c r="A222" s="6"/>
-      <c r="B222" s="6"/>
-      <c r="C222" s="6"/>
-      <c r="D222" s="6"/>
+      <c r="A222" s="18" t="s">
+        <v>416</v>
+      </c>
+      <c r="B222" s="19"/>
+      <c r="C222" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="D222" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E222" s="22"/>
+      <c r="F222" s="22"/>
+      <c r="G222" s="22"/>
+      <c r="H222" s="22"/>
+      <c r="I222" s="22"/>
+      <c r="J222" s="22"/>
+      <c r="K222" s="22"/>
+      <c r="L222" s="22"/>
+      <c r="M222" s="22"/>
+      <c r="N222" s="22"/>
+      <c r="O222" s="22"/>
+      <c r="P222" s="22"/>
+      <c r="Q222" s="22"/>
+      <c r="R222" s="22"/>
+      <c r="S222" s="22"/>
+      <c r="T222" s="22"/>
+      <c r="U222" s="22"/>
+      <c r="V222" s="22"/>
+      <c r="W222" s="22"/>
+      <c r="X222" s="22"/>
+      <c r="Y222" s="22"/>
+      <c r="Z222" s="22"/>
     </row>
     <row r="223">
       <c r="A223" s="6"/>
@@ -9362,14 +9550,80 @@
       <c r="C1087" s="6"/>
       <c r="D1087" s="6"/>
     </row>
+    <row r="1088">
+      <c r="A1088" s="6"/>
+      <c r="B1088" s="6"/>
+      <c r="C1088" s="6"/>
+      <c r="D1088" s="6"/>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="6"/>
+      <c r="B1089" s="6"/>
+      <c r="C1089" s="6"/>
+      <c r="D1089" s="6"/>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="6"/>
+      <c r="B1090" s="6"/>
+      <c r="C1090" s="6"/>
+      <c r="D1090" s="6"/>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="6"/>
+      <c r="B1091" s="6"/>
+      <c r="C1091" s="6"/>
+      <c r="D1091" s="6"/>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="6"/>
+      <c r="B1092" s="6"/>
+      <c r="C1092" s="6"/>
+      <c r="D1092" s="6"/>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="6"/>
+      <c r="B1093" s="6"/>
+      <c r="C1093" s="6"/>
+      <c r="D1093" s="6"/>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="6"/>
+      <c r="B1094" s="6"/>
+      <c r="C1094" s="6"/>
+      <c r="D1094" s="6"/>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="6"/>
+      <c r="B1095" s="6"/>
+      <c r="C1095" s="6"/>
+      <c r="D1095" s="6"/>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="6"/>
+      <c r="B1096" s="6"/>
+      <c r="C1096" s="6"/>
+      <c r="D1096" s="6"/>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="6"/>
+      <c r="B1097" s="6"/>
+      <c r="C1097" s="6"/>
+      <c r="D1097" s="6"/>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="6"/>
+      <c r="B1098" s="6"/>
+      <c r="C1098" s="6"/>
+      <c r="D1098" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D210">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D222">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A152"/>
+    <hyperlink r:id="rId1" ref="A163"/>
   </hyperlinks>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
Advanced information base screen
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="433">
   <si>
     <t>Key</t>
   </si>
@@ -1089,7 +1089,7 @@
     <t>Vibration type</t>
   </si>
   <si>
-    <t>alarm.new.edit_vibration.type.alert_default</t>
+    <t>alarm.new.edit_vibration.type.alert</t>
   </si>
   <si>
     <t>Alert (default)</t>
@@ -1297,6 +1297,48 @@
   </si>
   <si>
     <t>profile.header.title</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.discharge</t>
+  </si>
+  <si>
+    <t>Discharge</t>
+  </si>
+  <si>
+    <t>header.profile_advanced_information</t>
+  </si>
+  <si>
+    <t>ADVANCED INFORMATION</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.about_you</t>
+  </si>
+  <si>
+    <t>About you</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.lifestyle_info</t>
+  </si>
+  <si>
+    <t>Lifestyle information</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.title</t>
+  </si>
+  <si>
+    <t>Work Time</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.day</t>
+  </si>
+  <si>
+    <t>Day Worker</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.night</t>
+  </si>
+  <si>
+    <t>Night Worker</t>
   </si>
 </sst>
 </file>
@@ -1322,11 +1364,11 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
     </font>
+    <font/>
     <font>
       <strike/>
       <color rgb="FFFF0000"/>
@@ -1405,17 +1447,14 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
@@ -1430,6 +1469,9 @@
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -3276,11 +3318,11 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="11" t="s">
+      <c r="A135" s="5" t="s">
         <v>248</v>
       </c>
       <c r="B135" s="6"/>
-      <c r="C135" s="12" t="s">
+      <c r="C135" s="7" t="s">
         <v>249</v>
       </c>
       <c r="D135" s="5" t="s">
@@ -3288,14 +3330,14 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="13" t="s">
+      <c r="A136" s="11" t="s">
         <v>250</v>
       </c>
-      <c r="B136" s="14"/>
-      <c r="C136" s="13" t="s">
+      <c r="B136" s="12"/>
+      <c r="C136" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="D136" s="13" t="s">
+      <c r="D136" s="11" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3624,7 +3666,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="15" t="s">
+      <c r="A164" s="13" t="s">
         <v>304</v>
       </c>
       <c r="B164" s="6"/>
@@ -3900,7 +3942,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="5" t="s">
+      <c r="A187" s="14" t="s">
         <v>349</v>
       </c>
       <c r="B187" s="6"/>
@@ -4332,80 +4374,122 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="16" t="s">
+      <c r="A223" s="15" t="s">
         <v>418</v>
       </c>
-      <c r="B223" s="17"/>
-      <c r="C223" s="18" t="s">
+      <c r="B223" s="16"/>
+      <c r="C223" s="17" t="s">
         <v>218</v>
       </c>
-      <c r="D223" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="E223" s="19"/>
-      <c r="F223" s="19"/>
-      <c r="G223" s="19"/>
-      <c r="H223" s="19"/>
-      <c r="I223" s="19"/>
-      <c r="J223" s="19"/>
-      <c r="K223" s="19"/>
-      <c r="L223" s="19"/>
-      <c r="M223" s="19"/>
-      <c r="N223" s="19"/>
-      <c r="O223" s="19"/>
-      <c r="P223" s="19"/>
-      <c r="Q223" s="19"/>
-      <c r="R223" s="19"/>
-      <c r="S223" s="19"/>
-      <c r="T223" s="19"/>
-      <c r="U223" s="19"/>
-      <c r="V223" s="19"/>
-      <c r="W223" s="19"/>
-      <c r="X223" s="19"/>
-      <c r="Y223" s="19"/>
-      <c r="Z223" s="19"/>
+      <c r="D223" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E223" s="18"/>
+      <c r="F223" s="18"/>
+      <c r="G223" s="18"/>
+      <c r="H223" s="18"/>
+      <c r="I223" s="18"/>
+      <c r="J223" s="18"/>
+      <c r="K223" s="18"/>
+      <c r="L223" s="18"/>
+      <c r="M223" s="18"/>
+      <c r="N223" s="18"/>
+      <c r="O223" s="18"/>
+      <c r="P223" s="18"/>
+      <c r="Q223" s="18"/>
+      <c r="R223" s="18"/>
+      <c r="S223" s="18"/>
+      <c r="T223" s="18"/>
+      <c r="U223" s="18"/>
+      <c r="V223" s="18"/>
+      <c r="W223" s="18"/>
+      <c r="X223" s="18"/>
+      <c r="Y223" s="18"/>
+      <c r="Z223" s="18"/>
     </row>
     <row r="224">
-      <c r="A224" s="6"/>
+      <c r="A224" s="14" t="s">
+        <v>419</v>
+      </c>
       <c r="B224" s="6"/>
-      <c r="C224" s="6"/>
-      <c r="D224" s="6"/>
+      <c r="C224" s="19" t="s">
+        <v>420</v>
+      </c>
+      <c r="D224" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="225">
-      <c r="A225" s="6"/>
+      <c r="A225" s="14" t="s">
+        <v>421</v>
+      </c>
       <c r="B225" s="6"/>
-      <c r="C225" s="6"/>
-      <c r="D225" s="6"/>
+      <c r="C225" s="19" t="s">
+        <v>422</v>
+      </c>
+      <c r="D225" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="226">
-      <c r="A226" s="6"/>
+      <c r="A226" s="14" t="s">
+        <v>423</v>
+      </c>
       <c r="B226" s="6"/>
-      <c r="C226" s="6"/>
-      <c r="D226" s="6"/>
+      <c r="C226" s="19" t="s">
+        <v>424</v>
+      </c>
+      <c r="D226" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="227">
-      <c r="A227" s="6"/>
+      <c r="A227" s="14" t="s">
+        <v>425</v>
+      </c>
       <c r="B227" s="6"/>
-      <c r="C227" s="6"/>
-      <c r="D227" s="6"/>
+      <c r="C227" s="19" t="s">
+        <v>426</v>
+      </c>
+      <c r="D227" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="228">
-      <c r="A228" s="6"/>
+      <c r="A228" s="14" t="s">
+        <v>427</v>
+      </c>
       <c r="B228" s="6"/>
-      <c r="C228" s="6"/>
-      <c r="D228" s="6"/>
+      <c r="C228" s="19" t="s">
+        <v>428</v>
+      </c>
+      <c r="D228" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="229">
-      <c r="A229" s="6"/>
+      <c r="A229" s="14" t="s">
+        <v>429</v>
+      </c>
       <c r="B229" s="6"/>
-      <c r="C229" s="6"/>
-      <c r="D229" s="6"/>
+      <c r="C229" s="19" t="s">
+        <v>430</v>
+      </c>
+      <c r="D229" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="230">
-      <c r="A230" s="6"/>
+      <c r="A230" s="14" t="s">
+        <v>431</v>
+      </c>
       <c r="B230" s="6"/>
-      <c r="C230" s="6"/>
-      <c r="D230" s="6"/>
+      <c r="C230" s="19" t="s">
+        <v>432</v>
+      </c>
+      <c r="D230" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="6"/>
@@ -9623,7 +9707,7 @@
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D223">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D230">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
WIP alarm clock creation, add vibration bottom sheet
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="421">
   <si>
     <t>Key</t>
   </si>
@@ -65,6 +65,21 @@
   </si>
   <si>
     <t>setup.scan.disabled.enable</t>
+  </si>
+  <si>
+    <t>setup.scan.location_disabled.title</t>
+  </si>
+  <si>
+    <t>Enable location</t>
+  </si>
+  <si>
+    <t>setup.scan.location_disabled.message</t>
+  </si>
+  <si>
+    <t>To be able to use bluetooth connection, Android needs your phone to enable location</t>
+  </si>
+  <si>
+    <t>setup.scan.location_disabled.enable</t>
   </si>
   <si>
     <t>setup.scan.enabled.title</t>
@@ -366,6 +381,24 @@
   </si>
   <si>
     <t>Next</t>
+  </si>
+  <si>
+    <t>global.cancel</t>
+  </si>
+  <si>
+    <t>Cancel</t>
+  </si>
+  <si>
+    <t>global.save</t>
+  </si>
+  <si>
+    <t>Save</t>
+  </si>
+  <si>
+    <t>global.continue</t>
+  </si>
+  <si>
+    <t>global.default_error</t>
   </si>
   <si>
     <t>home.sync.syncing</t>
@@ -622,12 +655,18 @@
     <t>forgot_password.reset.confirm_password.placeholder</t>
   </si>
   <si>
-    <t>profile.header.title</t>
+    <t>header.profile</t>
   </si>
   <si>
     <t>PROFILE</t>
   </si>
   <si>
+    <t>profile.user_creation</t>
+  </si>
+  <si>
+    <t>User since {date}</t>
+  </si>
+  <si>
     <t>profile.logout</t>
   </si>
   <si>
@@ -638,6 +677,109 @@
   </si>
   <si>
     <t>Global score</t>
+  </si>
+  <si>
+    <t>profile.list_header.profile</t>
+  </si>
+  <si>
+    <t>Profile</t>
+  </si>
+  <si>
+    <t>profile.list.profile_information</t>
+  </si>
+  <si>
+    <t>Profile Information</t>
+  </si>
+  <si>
+    <t>header.profile_information</t>
+  </si>
+  <si>
+    <t>profile_info.basic_info</t>
+  </si>
+  <si>
+    <t>Basic info</t>
+  </si>
+  <si>
+    <t>profile_info.name</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>profile_info.birthday</t>
+  </si>
+  <si>
+    <t>Birthday</t>
+  </si>
+  <si>
+    <t>profile_info.height</t>
+  </si>
+  <si>
+    <t>Height</t>
+  </si>
+  <si>
+    <t>profile_info.bottom_sheet.height</t>
+  </si>
+  <si>
+    <t>Select your Height</t>
+  </si>
+  <si>
+    <t>profile_info.weight</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>profile_info.bottom_sheet.weight</t>
+  </si>
+  <si>
+    <t>Select your Weight</t>
+  </si>
+  <si>
+    <t>profile_info.sex</t>
+  </si>
+  <si>
+    <t>Sex</t>
+  </si>
+  <si>
+    <t>profile_info.bottom_sheet.sex.title</t>
+  </si>
+  <si>
+    <t>Please Confirm</t>
+  </si>
+  <si>
+    <t>profile_info.bottom_sheet.sex.description</t>
+  </si>
+  <si>
+    <t>Confirm that you want to change your sex.
+By doing so, many of your profile parameters will be modified.</t>
+  </si>
+  <si>
+    <t>profile_info.leaderboard</t>
+  </si>
+  <si>
+    <t>Participate in Leaderboards</t>
+  </si>
+  <si>
+    <t>profile_info.advanced_info</t>
+  </si>
+  <si>
+    <t>Advanced Information</t>
+  </si>
+  <si>
+    <t>profile_info.edit_name.title</t>
+  </si>
+  <si>
+    <t>Edit Name</t>
+  </si>
+  <si>
+    <t>profile_info.edit_birthday.title</t>
+  </si>
+  <si>
+    <t>Edit Birthday</t>
+  </si>
+  <si>
+    <t>profile_info.edit_name.save</t>
   </si>
   <si>
     <t>header.live</t>
@@ -756,9 +898,6 @@
   </si>
   <si>
     <t>drawer.profile</t>
-  </si>
-  <si>
-    <t>Profile</t>
   </si>
   <si>
     <t>drawer.close</t>
@@ -950,7 +1089,7 @@
     <t>Vibration type</t>
   </si>
   <si>
-    <t>alarm.new.edit_vibration.type.alert_default</t>
+    <t>alarm.new.edit_vibration.type.alert</t>
   </si>
   <si>
     <t>Alert (default)</t>
@@ -995,9 +1134,6 @@
     <t>alarm.new.save_button</t>
   </si>
   <si>
-    <t>Save</t>
-  </si>
-  <si>
     <t>alarm.new.repeat.weekdays</t>
   </si>
   <si>
@@ -1139,6 +1275,15 @@
     <t>alarm.wake_up_score</t>
   </si>
   <si>
+    <t>alarm.new.time.edit</t>
+  </si>
+  <si>
+    <t>Edit alarm time</t>
+  </si>
+  <si>
+    <t>alarm.week_overview</t>
+  </si>
+  <si>
     <t>banner.calibration.title</t>
   </si>
   <si>
@@ -1151,17 +1296,20 @@
     <t>Keep wearing your ring during the entirety of the {days} days calibration period for improved results!</t>
   </si>
   <si>
-    <t>alarm.new.time.edit</t>
-  </si>
-  <si>
-    <t>Edit alarm time</t>
+    <t>profile.header.title</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.discharge</t>
+  </si>
+  <si>
+    <t>Discharge</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1185,8 +1333,13 @@
       <color rgb="FF0000FF"/>
     </font>
     <font/>
+    <font>
+      <strike/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1211,6 +1364,12 @@
         <bgColor rgb="FFFFA500"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -1218,7 +1377,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1252,12 +1411,28 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -1613,7 +1788,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="6"/>
@@ -1625,60 +1800,60 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="8" t="s">
         <v>22</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="s">
-        <v>24</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="s">
         <v>25</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="s">
         <v>27</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="s">
         <v>29</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>6</v>
@@ -1686,11 +1861,11 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>6</v>
@@ -1698,11 +1873,11 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>6</v>
@@ -1738,7 +1913,7 @@
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>6</v>
@@ -1746,11 +1921,11 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>6</v>
@@ -1758,11 +1933,11 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>6</v>
@@ -1770,11 +1945,11 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>6</v>
@@ -1782,11 +1957,11 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>6</v>
@@ -1794,23 +1969,23 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="7" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="5" t="s">
         <v>50</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>6</v>
@@ -1818,11 +1993,11 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="7" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>6</v>
@@ -1830,23 +2005,23 @@
     </row>
     <row r="28">
       <c r="A28" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="s">
-        <v>54</v>
+      <c r="A29" s="8" t="s">
+        <v>55</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="7" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>6</v>
@@ -1854,11 +2029,11 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>6</v>
@@ -1866,11 +2041,11 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>6</v>
@@ -1878,11 +2053,11 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>6</v>
@@ -1890,11 +2065,11 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>6</v>
@@ -1902,11 +2077,11 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>6</v>
@@ -1914,7 +2089,7 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
@@ -1926,11 +2101,11 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>6</v>
@@ -1938,11 +2113,11 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>6</v>
@@ -1950,11 +2125,11 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>6</v>
@@ -1966,7 +2141,7 @@
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="7" t="s">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>6</v>
@@ -1974,11 +2149,11 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>6</v>
@@ -1986,11 +2161,11 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>6</v>
@@ -1998,11 +2173,11 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>6</v>
@@ -2010,11 +2185,11 @@
     </row>
     <row r="43">
       <c r="A43" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>6</v>
@@ -2050,7 +2225,7 @@
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
-        <v>81</v>
+        <v>47</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>6</v>
@@ -2058,11 +2233,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>6</v>
@@ -2070,11 +2245,11 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>6</v>
@@ -2082,11 +2257,11 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>6</v>
@@ -2094,11 +2269,11 @@
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>6</v>
@@ -2106,11 +2281,11 @@
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>6</v>
@@ -2118,11 +2293,11 @@
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>6</v>
@@ -2130,11 +2305,11 @@
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>6</v>
@@ -2142,11 +2317,11 @@
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
-        <v>31</v>
+        <v>96</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>6</v>
@@ -2170,7 +2345,7 @@
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="7" t="s">
-        <v>29</v>
+        <v>100</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>6</v>
@@ -2178,11 +2353,11 @@
     </row>
     <row r="57">
       <c r="A57" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
-        <v>101</v>
+        <v>36</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>6</v>
@@ -2194,7 +2369,7 @@
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -2202,11 +2377,11 @@
     </row>
     <row r="59">
       <c r="A59" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B59" s="6"/>
       <c r="C59" s="7" t="s">
-        <v>104</v>
+        <v>34</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>6</v>
@@ -2230,7 +2405,7 @@
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="7" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>6</v>
@@ -2238,11 +2413,11 @@
     </row>
     <row r="62">
       <c r="A62" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B62" s="6"/>
       <c r="C62" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>6</v>
@@ -2250,11 +2425,11 @@
     </row>
     <row r="63">
       <c r="A63" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>6</v>
@@ -2262,35 +2437,37 @@
     </row>
     <row r="64">
       <c r="A64" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="D64" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="10" t="s">
+      <c r="B65" s="6"/>
+      <c r="C65" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="C65" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D65" s="10" t="s">
+      <c r="D65" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="10" t="s">
+      <c r="A66" s="5" t="s">
         <v>116</v>
       </c>
+      <c r="B66" s="6"/>
       <c r="C66" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="D66" s="10" t="s">
+      <c r="D66" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2307,84 +2484,78 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="s">
+      <c r="A68" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D68" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="D68" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="s">
+      <c r="C69" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="B69" s="6"/>
-      <c r="C69" s="7" t="s">
+      <c r="D69" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="D69" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="s">
+      <c r="C70" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="B70" s="6"/>
-      <c r="C70" s="7" t="s">
+      <c r="D70" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="D70" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="s">
+      <c r="C71" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="B71" s="6"/>
-      <c r="C71" s="7" t="s">
+      <c r="D71" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="D71" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="s">
+      <c r="C72" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D72" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="B72" s="6"/>
-      <c r="C72" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="D72" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="B73" s="6"/>
       <c r="C73" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="D73" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D73" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B74" s="6"/>
       <c r="C74" s="7" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D74" s="5" t="s">
         <v>6</v>
@@ -2392,11 +2563,11 @@
     </row>
     <row r="75">
       <c r="A75" s="5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B75" s="6"/>
       <c r="C75" s="7" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D75" s="5" t="s">
         <v>6</v>
@@ -2404,11 +2575,11 @@
     </row>
     <row r="76">
       <c r="A76" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B76" s="6"/>
       <c r="C76" s="7" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D76" s="5" t="s">
         <v>6</v>
@@ -2416,11 +2587,11 @@
     </row>
     <row r="77">
       <c r="A77" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B77" s="6"/>
       <c r="C77" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D77" s="5" t="s">
         <v>6</v>
@@ -2428,35 +2599,35 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B78" s="6"/>
       <c r="C78" s="7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D78" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="s">
-        <v>142</v>
+      <c r="A79" s="5" t="s">
+        <v>139</v>
       </c>
       <c r="B79" s="6"/>
       <c r="C79" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D79" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="s">
-        <v>144</v>
+      <c r="A80" s="5" t="s">
+        <v>141</v>
       </c>
       <c r="B80" s="6"/>
       <c r="C80" s="7" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D80" s="5" t="s">
         <v>6</v>
@@ -2464,11 +2635,11 @@
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B81" s="6"/>
       <c r="C81" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>6</v>
@@ -2476,11 +2647,11 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B82" s="6"/>
       <c r="C82" s="7" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>6</v>
@@ -2488,11 +2659,11 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B83" s="6"/>
       <c r="C83" s="7" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>6</v>
@@ -2500,11 +2671,11 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B84" s="6"/>
       <c r="C84" s="7" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>6</v>
@@ -2512,35 +2683,35 @@
     </row>
     <row r="85">
       <c r="A85" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B85" s="6"/>
       <c r="C85" s="7" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="5" t="s">
-        <v>156</v>
+      <c r="A86" s="8" t="s">
+        <v>153</v>
       </c>
       <c r="B86" s="6"/>
       <c r="C86" s="7" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="5" t="s">
-        <v>158</v>
+      <c r="A87" s="8" t="s">
+        <v>155</v>
       </c>
       <c r="B87" s="6"/>
       <c r="C87" s="7" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D87" s="5" t="s">
         <v>6</v>
@@ -2548,11 +2719,11 @@
     </row>
     <row r="88">
       <c r="A88" s="5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B88" s="6"/>
       <c r="C88" s="7" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>6</v>
@@ -2560,11 +2731,11 @@
     </row>
     <row r="89">
       <c r="A89" s="5" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B89" s="6"/>
       <c r="C89" s="7" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D89" s="5" t="s">
         <v>6</v>
@@ -2572,11 +2743,11 @@
     </row>
     <row r="90">
       <c r="A90" s="5" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B90" s="6"/>
       <c r="C90" s="7" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D90" s="5" t="s">
         <v>6</v>
@@ -2584,11 +2755,11 @@
     </row>
     <row r="91">
       <c r="A91" s="5" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B91" s="6"/>
       <c r="C91" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D91" s="5" t="s">
         <v>6</v>
@@ -2596,11 +2767,11 @@
     </row>
     <row r="92">
       <c r="A92" s="5" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B92" s="6"/>
       <c r="C92" s="7" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D92" s="5" t="s">
         <v>6</v>
@@ -2608,11 +2779,11 @@
     </row>
     <row r="93">
       <c r="A93" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B93" s="6"/>
       <c r="C93" s="7" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>6</v>
@@ -2620,11 +2791,11 @@
     </row>
     <row r="94">
       <c r="A94" s="5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B94" s="6"/>
       <c r="C94" s="7" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D94" s="5" t="s">
         <v>6</v>
@@ -2632,11 +2803,11 @@
     </row>
     <row r="95">
       <c r="A95" s="5" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B95" s="6"/>
       <c r="C95" s="7" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D95" s="5" t="s">
         <v>6</v>
@@ -2644,11 +2815,11 @@
     </row>
     <row r="96">
       <c r="A96" s="5" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B96" s="6"/>
       <c r="C96" s="7" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D96" s="5" t="s">
         <v>6</v>
@@ -2656,11 +2827,11 @@
     </row>
     <row r="97">
       <c r="A97" s="5" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B97" s="6"/>
       <c r="C97" s="7" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D97" s="5" t="s">
         <v>6</v>
@@ -2668,11 +2839,11 @@
     </row>
     <row r="98">
       <c r="A98" s="5" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B98" s="6"/>
       <c r="C98" s="7" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D98" s="5" t="s">
         <v>6</v>
@@ -2680,11 +2851,11 @@
     </row>
     <row r="99">
       <c r="A99" s="5" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B99" s="6"/>
       <c r="C99" s="7" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>6</v>
@@ -2692,11 +2863,11 @@
     </row>
     <row r="100">
       <c r="A100" s="5" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B100" s="6"/>
       <c r="C100" s="7" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>6</v>
@@ -2704,11 +2875,11 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B101" s="6"/>
       <c r="C101" s="7" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>6</v>
@@ -2716,11 +2887,11 @@
     </row>
     <row r="102">
       <c r="A102" s="5" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B102" s="6"/>
       <c r="C102" s="7" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>6</v>
@@ -2728,11 +2899,11 @@
     </row>
     <row r="103">
       <c r="A103" s="5" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B103" s="6"/>
       <c r="C103" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>6</v>
@@ -2740,11 +2911,11 @@
     </row>
     <row r="104">
       <c r="A104" s="5" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B104" s="6"/>
       <c r="C104" s="7" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>6</v>
@@ -2752,11 +2923,11 @@
     </row>
     <row r="105">
       <c r="A105" s="5" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="7" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D105" s="5" t="s">
         <v>6</v>
@@ -2764,11 +2935,11 @@
     </row>
     <row r="106">
       <c r="A106" s="5" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B106" s="6"/>
       <c r="C106" s="7" t="s">
-        <v>31</v>
+        <v>194</v>
       </c>
       <c r="D106" s="5" t="s">
         <v>6</v>
@@ -2776,11 +2947,11 @@
     </row>
     <row r="107">
       <c r="A107" s="5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B107" s="6"/>
       <c r="C107" s="7" t="s">
-        <v>31</v>
+        <v>196</v>
       </c>
       <c r="D107" s="5" t="s">
         <v>6</v>
@@ -2788,11 +2959,11 @@
     </row>
     <row r="108">
       <c r="A108" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B108" s="6"/>
       <c r="C108" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D108" s="5" t="s">
         <v>6</v>
@@ -2800,11 +2971,11 @@
     </row>
     <row r="109">
       <c r="A109" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B109" s="6"/>
       <c r="C109" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>6</v>
@@ -2812,11 +2983,11 @@
     </row>
     <row r="110">
       <c r="A110" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B110" s="6"/>
       <c r="C110" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>6</v>
@@ -2824,11 +2995,11 @@
     </row>
     <row r="111">
       <c r="A111" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B111" s="6"/>
       <c r="C111" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>6</v>
@@ -2836,11 +3007,11 @@
     </row>
     <row r="112">
       <c r="A112" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B112" s="6"/>
       <c r="C112" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>6</v>
@@ -2848,11 +3019,11 @@
     </row>
     <row r="113">
       <c r="A113" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B113" s="6"/>
       <c r="C113" s="7" t="s">
-        <v>209</v>
+        <v>36</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>6</v>
@@ -2860,11 +3031,11 @@
     </row>
     <row r="114">
       <c r="A114" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B114" s="6"/>
       <c r="C114" s="7" t="s">
-        <v>211</v>
+        <v>36</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>6</v>
@@ -2872,11 +3043,11 @@
     </row>
     <row r="115">
       <c r="A115" s="5" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B115" s="6"/>
       <c r="C115" s="7" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>6</v>
@@ -2884,11 +3055,11 @@
     </row>
     <row r="116">
       <c r="A116" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="B116" s="6"/>
+        <v>211</v>
+      </c>
+      <c r="B116" s="5"/>
       <c r="C116" s="7" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D116" s="5" t="s">
         <v>6</v>
@@ -2896,11 +3067,11 @@
     </row>
     <row r="117">
       <c r="A117" s="5" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B117" s="6"/>
       <c r="C117" s="7" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>6</v>
@@ -2908,11 +3079,11 @@
     </row>
     <row r="118">
       <c r="A118" s="5" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B118" s="6"/>
       <c r="C118" s="7" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>6</v>
@@ -2920,11 +3091,11 @@
     </row>
     <row r="119">
       <c r="A119" s="5" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B119" s="6"/>
       <c r="C119" s="7" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>6</v>
@@ -2932,11 +3103,11 @@
     </row>
     <row r="120">
       <c r="A120" s="5" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B120" s="6"/>
       <c r="C120" s="7" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>6</v>
@@ -2944,11 +3115,11 @@
     </row>
     <row r="121">
       <c r="A121" s="5" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B121" s="6"/>
       <c r="C121" s="7" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>6</v>
@@ -2956,11 +3127,11 @@
     </row>
     <row r="122">
       <c r="A122" s="5" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B122" s="6"/>
       <c r="C122" s="7" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>6</v>
@@ -2968,11 +3139,11 @@
     </row>
     <row r="123">
       <c r="A123" s="5" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B123" s="6"/>
       <c r="C123" s="7" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>6</v>
@@ -2980,11 +3151,11 @@
     </row>
     <row r="124">
       <c r="A124" s="5" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -2992,11 +3163,11 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>6</v>
@@ -3004,35 +3175,35 @@
     </row>
     <row r="126">
       <c r="A126" s="5" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B126" s="6"/>
       <c r="C126" s="7" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="D126" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="8" t="s">
-        <v>236</v>
+      <c r="A127" s="5" t="s">
+        <v>232</v>
       </c>
       <c r="B127" s="6"/>
       <c r="C127" s="7" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="D127" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="8" t="s">
-        <v>238</v>
+      <c r="A128" s="5" t="s">
+        <v>234</v>
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>6</v>
@@ -3040,35 +3211,35 @@
     </row>
     <row r="129">
       <c r="A129" s="8" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D129" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="5" t="s">
-        <v>242</v>
+      <c r="A130" s="8" t="s">
+        <v>238</v>
       </c>
       <c r="B130" s="6"/>
       <c r="C130" s="7" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D130" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="5" t="s">
-        <v>244</v>
+      <c r="A131" s="8" t="s">
+        <v>240</v>
       </c>
       <c r="B131" s="6"/>
       <c r="C131" s="7" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>6</v>
@@ -3076,11 +3247,11 @@
     </row>
     <row r="132">
       <c r="A132" s="5" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="B132" s="6"/>
       <c r="C132" s="7" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="D132" s="5" t="s">
         <v>6</v>
@@ -3088,11 +3259,11 @@
     </row>
     <row r="133">
       <c r="A133" s="5" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="B133" s="6"/>
       <c r="C133" s="7" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>6</v>
@@ -3100,11 +3271,11 @@
     </row>
     <row r="134">
       <c r="A134" s="5" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="B134" s="6"/>
       <c r="C134" s="7" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D134" s="5" t="s">
         <v>6</v>
@@ -3112,47 +3283,47 @@
     </row>
     <row r="135">
       <c r="A135" s="5" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="B135" s="6"/>
       <c r="C135" s="7" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D135" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="B136" s="6"/>
-      <c r="C136" s="7" t="s">
-        <v>255</v>
-      </c>
-      <c r="D136" s="5" t="s">
+      <c r="A136" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="B136" s="12"/>
+      <c r="C136" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="D136" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="11" t="s">
-        <v>258</v>
+      <c r="A138" s="5" t="s">
+        <v>253</v>
       </c>
       <c r="B138" s="6"/>
       <c r="C138" s="7" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>6</v>
@@ -3160,11 +3331,11 @@
     </row>
     <row r="139">
       <c r="A139" s="5" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="B139" s="6"/>
       <c r="C139" s="7" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="D139" s="5" t="s">
         <v>6</v>
@@ -3172,11 +3343,11 @@
     </row>
     <row r="140">
       <c r="A140" s="5" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B140" s="6"/>
       <c r="C140" s="7" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="D140" s="5" t="s">
         <v>6</v>
@@ -3184,11 +3355,11 @@
     </row>
     <row r="141">
       <c r="A141" s="5" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="7" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D141" s="5" t="s">
         <v>6</v>
@@ -3196,23 +3367,23 @@
     </row>
     <row r="142">
       <c r="A142" s="5" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B142" s="6"/>
       <c r="C142" s="7" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="D142" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="8" t="s">
-        <v>268</v>
+      <c r="A143" s="5" t="s">
+        <v>263</v>
       </c>
       <c r="B143" s="6"/>
       <c r="C143" s="7" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D143" s="5" t="s">
         <v>6</v>
@@ -3220,11 +3391,11 @@
     </row>
     <row r="144">
       <c r="A144" s="5" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B144" s="6"/>
       <c r="C144" s="7" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="D144" s="5" t="s">
         <v>6</v>
@@ -3232,11 +3403,11 @@
     </row>
     <row r="145">
       <c r="A145" s="5" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="B145" s="6"/>
       <c r="C145" s="7" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="D145" s="5" t="s">
         <v>6</v>
@@ -3244,11 +3415,11 @@
     </row>
     <row r="146">
       <c r="A146" s="5" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B146" s="6"/>
       <c r="C146" s="7" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="D146" s="5" t="s">
         <v>6</v>
@@ -3256,11 +3427,11 @@
     </row>
     <row r="147">
       <c r="A147" s="5" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="B147" s="6"/>
       <c r="C147" s="7" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="D147" s="5" t="s">
         <v>6</v>
@@ -3268,11 +3439,11 @@
     </row>
     <row r="148">
       <c r="A148" s="5" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="B148" s="6"/>
       <c r="C148" s="7" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="D148" s="5" t="s">
         <v>6</v>
@@ -3280,11 +3451,11 @@
     </row>
     <row r="149">
       <c r="A149" s="5" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="B149" s="6"/>
       <c r="C149" s="7" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="D149" s="5" t="s">
         <v>6</v>
@@ -3292,11 +3463,11 @@
     </row>
     <row r="150">
       <c r="A150" s="5" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="B150" s="6"/>
       <c r="C150" s="7" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="D150" s="5" t="s">
         <v>6</v>
@@ -3304,11 +3475,11 @@
     </row>
     <row r="151">
       <c r="A151" s="5" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="B151" s="6"/>
       <c r="C151" s="7" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="D151" s="5" t="s">
         <v>6</v>
@@ -3316,47 +3487,47 @@
     </row>
     <row r="152">
       <c r="A152" s="5" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="B152" s="6"/>
       <c r="C152" s="7" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="D152" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="5" t="s">
-        <v>288</v>
+      <c r="A153" s="8" t="s">
+        <v>283</v>
       </c>
       <c r="B153" s="6"/>
       <c r="C153" s="7" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="D153" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="5" t="s">
-        <v>290</v>
+      <c r="A154" s="8" t="s">
+        <v>285</v>
       </c>
       <c r="B154" s="6"/>
       <c r="C154" s="7" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="D154" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="5" t="s">
-        <v>292</v>
+      <c r="A155" s="8" t="s">
+        <v>287</v>
       </c>
       <c r="B155" s="6"/>
       <c r="C155" s="7" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="D155" s="5" t="s">
         <v>6</v>
@@ -3364,11 +3535,11 @@
     </row>
     <row r="156">
       <c r="A156" s="5" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="B156" s="6"/>
       <c r="C156" s="7" t="s">
-        <v>295</v>
+        <v>218</v>
       </c>
       <c r="D156" s="5" t="s">
         <v>6</v>
@@ -3376,23 +3547,23 @@
     </row>
     <row r="157">
       <c r="A157" s="5" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="B157" s="6"/>
       <c r="C157" s="7" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="D157" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="12" t="s">
-        <v>298</v>
+      <c r="A158" s="5" t="s">
+        <v>292</v>
       </c>
       <c r="B158" s="6"/>
-      <c r="C158" s="13" t="s">
-        <v>42</v>
+      <c r="C158" s="7" t="s">
+        <v>293</v>
       </c>
       <c r="D158" s="5" t="s">
         <v>6</v>
@@ -3400,11 +3571,11 @@
     </row>
     <row r="159">
       <c r="A159" s="5" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="7" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="D159" s="5" t="s">
         <v>6</v>
@@ -3412,11 +3583,11 @@
     </row>
     <row r="160">
       <c r="A160" s="5" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="7" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="D160" s="5" t="s">
         <v>6</v>
@@ -3424,83 +3595,83 @@
     </row>
     <row r="161">
       <c r="A161" s="5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="7" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D161" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="10" t="s">
-        <v>305</v>
+      <c r="A162" s="5" t="s">
+        <v>300</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="7" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="10" t="s">
-        <v>307</v>
+      <c r="A163" s="5" t="s">
+        <v>302</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="10" t="s">
-        <v>309</v>
+      <c r="A164" s="13" t="s">
+        <v>304</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="10" t="s">
-        <v>311</v>
+      <c r="A165" s="5" t="s">
+        <v>306</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="7" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="D165" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="10" t="s">
-        <v>313</v>
+      <c r="A166" s="5" t="s">
+        <v>308</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="7" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="D166" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="10" t="s">
-        <v>315</v>
+      <c r="A167" s="5" t="s">
+        <v>310</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="7" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="D167" s="5" t="s">
         <v>6</v>
@@ -3508,23 +3679,23 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="5" t="s">
-        <v>319</v>
+      <c r="A169" s="8" t="s">
+        <v>314</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="7" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="D169" s="5" t="s">
         <v>6</v>
@@ -3532,11 +3703,11 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="7" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D170" s="5" t="s">
         <v>6</v>
@@ -3544,11 +3715,11 @@
     </row>
     <row r="171">
       <c r="A171" s="5" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="7" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="D171" s="5" t="s">
         <v>6</v>
@@ -3556,11 +3727,11 @@
     </row>
     <row r="172">
       <c r="A172" s="5" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="7" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="D172" s="5" t="s">
         <v>6</v>
@@ -3568,11 +3739,11 @@
     </row>
     <row r="173">
       <c r="A173" s="5" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="7" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="D173" s="5" t="s">
         <v>6</v>
@@ -3580,11 +3751,11 @@
     </row>
     <row r="174">
       <c r="A174" s="5" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
@@ -3592,11 +3763,11 @@
     </row>
     <row r="175">
       <c r="A175" s="5" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
@@ -3604,11 +3775,11 @@
     </row>
     <row r="176">
       <c r="A176" s="5" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
@@ -3616,11 +3787,11 @@
     </row>
     <row r="177">
       <c r="A177" s="5" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
@@ -3628,11 +3799,11 @@
     </row>
     <row r="178">
       <c r="A178" s="5" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
@@ -3640,11 +3811,11 @@
     </row>
     <row r="179">
       <c r="A179" s="5" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
@@ -3652,11 +3823,11 @@
     </row>
     <row r="180">
       <c r="A180" s="5" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
@@ -3664,11 +3835,11 @@
     </row>
     <row r="181">
       <c r="A181" s="5" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
@@ -3676,11 +3847,11 @@
     </row>
     <row r="182">
       <c r="A182" s="5" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="7" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>6</v>
@@ -3688,11 +3859,11 @@
     </row>
     <row r="183">
       <c r="A183" s="5" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="7" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>6</v>
@@ -3700,11 +3871,11 @@
     </row>
     <row r="184">
       <c r="A184" s="5" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="7" t="s">
-        <v>350</v>
+        <v>47</v>
       </c>
       <c r="D184" s="5" t="s">
         <v>6</v>
@@ -3712,11 +3883,11 @@
     </row>
     <row r="185">
       <c r="A185" s="5" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="7" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="D185" s="5" t="s">
         <v>6</v>
@@ -3724,95 +3895,95 @@
     </row>
     <row r="186">
       <c r="A186" s="5" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="7" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="D186" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="5" t="s">
-        <v>355</v>
+      <c r="A187" s="14" t="s">
+        <v>349</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="5" t="s">
-        <v>357</v>
+      <c r="A188" s="10" t="s">
+        <v>351</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="D188" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="5" t="s">
-        <v>359</v>
+      <c r="A189" s="10" t="s">
+        <v>353</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="7" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="5" t="s">
-        <v>361</v>
+      <c r="A190" s="10" t="s">
+        <v>355</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="5" t="s">
-        <v>363</v>
+      <c r="A191" s="10" t="s">
+        <v>357</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="12" t="s">
-        <v>365</v>
+      <c r="A192" s="10" t="s">
+        <v>359</v>
       </c>
       <c r="B192" s="6"/>
-      <c r="C192" s="13" t="s">
-        <v>149</v>
+      <c r="C192" s="7" t="s">
+        <v>360</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="5" t="s">
-        <v>366</v>
+      <c r="A193" s="10" t="s">
+        <v>361</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
@@ -3820,11 +3991,11 @@
     </row>
     <row r="194">
       <c r="A194" s="5" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="B194" s="6"/>
       <c r="C194" s="7" t="s">
-        <v>369</v>
+        <v>126</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>6</v>
@@ -3832,189 +4003,385 @@
     </row>
     <row r="195">
       <c r="A195" s="5" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="B195" s="6"/>
       <c r="C195" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="D195" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="B196" s="6"/>
+      <c r="C196" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="D196" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="B197" s="6"/>
+      <c r="C197" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="D197" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="B198" s="6"/>
+      <c r="C198" s="7" t="s">
         <v>371</v>
       </c>
-      <c r="D195" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" s="6"/>
-      <c r="B196" s="6"/>
-      <c r="C196" s="6"/>
-      <c r="D196" s="6"/>
-    </row>
-    <row r="197">
-      <c r="A197" s="6"/>
-      <c r="B197" s="6"/>
-      <c r="C197" s="6"/>
-      <c r="D197" s="6"/>
-    </row>
-    <row r="198">
-      <c r="A198" s="6"/>
-      <c r="B198" s="6"/>
-      <c r="C198" s="6"/>
-      <c r="D198" s="6"/>
+      <c r="D198" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="199">
-      <c r="A199" s="6"/>
+      <c r="A199" s="5" t="s">
+        <v>372</v>
+      </c>
       <c r="B199" s="6"/>
-      <c r="C199" s="6"/>
-      <c r="D199" s="6"/>
+      <c r="C199" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="D199" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="200">
-      <c r="A200" s="6"/>
+      <c r="A200" s="5" t="s">
+        <v>374</v>
+      </c>
       <c r="B200" s="6"/>
-      <c r="C200" s="6"/>
-      <c r="D200" s="6"/>
+      <c r="C200" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="D200" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="201">
-      <c r="A201" s="6"/>
+      <c r="A201" s="5" t="s">
+        <v>376</v>
+      </c>
       <c r="B201" s="6"/>
-      <c r="C201" s="6"/>
-      <c r="D201" s="6"/>
+      <c r="C201" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="D201" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="202">
-      <c r="A202" s="6"/>
+      <c r="A202" s="5" t="s">
+        <v>378</v>
+      </c>
       <c r="B202" s="6"/>
-      <c r="C202" s="6"/>
-      <c r="D202" s="6"/>
+      <c r="C202" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="D202" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="203">
-      <c r="A203" s="6"/>
+      <c r="A203" s="5" t="s">
+        <v>380</v>
+      </c>
       <c r="B203" s="6"/>
-      <c r="C203" s="6"/>
-      <c r="D203" s="6"/>
+      <c r="C203" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="D203" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="204">
-      <c r="A204" s="6"/>
+      <c r="A204" s="5" t="s">
+        <v>382</v>
+      </c>
       <c r="B204" s="6"/>
-      <c r="C204" s="6"/>
-      <c r="D204" s="6"/>
+      <c r="C204" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="D204" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="205">
-      <c r="A205" s="6"/>
+      <c r="A205" s="5" t="s">
+        <v>384</v>
+      </c>
       <c r="B205" s="6"/>
-      <c r="C205" s="6"/>
-      <c r="D205" s="6"/>
+      <c r="C205" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="D205" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="206">
-      <c r="A206" s="6"/>
+      <c r="A206" s="5" t="s">
+        <v>386</v>
+      </c>
       <c r="B206" s="6"/>
-      <c r="C206" s="6"/>
-      <c r="D206" s="6"/>
+      <c r="C206" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="D206" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="207">
-      <c r="A207" s="6"/>
+      <c r="A207" s="5" t="s">
+        <v>388</v>
+      </c>
       <c r="B207" s="6"/>
-      <c r="C207" s="6"/>
-      <c r="D207" s="6"/>
+      <c r="C207" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="D207" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="208">
-      <c r="A208" s="6"/>
+      <c r="A208" s="5" t="s">
+        <v>390</v>
+      </c>
       <c r="B208" s="6"/>
-      <c r="C208" s="6"/>
-      <c r="D208" s="6"/>
+      <c r="C208" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="D208" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="209">
-      <c r="A209" s="6"/>
+      <c r="A209" s="5" t="s">
+        <v>392</v>
+      </c>
       <c r="B209" s="6"/>
-      <c r="C209" s="6"/>
-      <c r="D209" s="6"/>
+      <c r="C209" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="D209" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="210">
-      <c r="A210" s="6"/>
+      <c r="A210" s="5" t="s">
+        <v>394</v>
+      </c>
       <c r="B210" s="6"/>
-      <c r="C210" s="6"/>
-      <c r="D210" s="6"/>
+      <c r="C210" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="D210" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="211">
-      <c r="A211" s="6"/>
+      <c r="A211" s="5" t="s">
+        <v>396</v>
+      </c>
       <c r="B211" s="6"/>
-      <c r="C211" s="6"/>
-      <c r="D211" s="6"/>
+      <c r="C211" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="D211" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="212">
-      <c r="A212" s="6"/>
+      <c r="A212" s="5" t="s">
+        <v>398</v>
+      </c>
       <c r="B212" s="6"/>
-      <c r="C212" s="6"/>
-      <c r="D212" s="6"/>
+      <c r="C212" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="D212" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="213">
-      <c r="A213" s="6"/>
+      <c r="A213" s="5" t="s">
+        <v>400</v>
+      </c>
       <c r="B213" s="6"/>
-      <c r="C213" s="6"/>
-      <c r="D213" s="6"/>
+      <c r="C213" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="D213" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="214">
-      <c r="A214" s="6"/>
+      <c r="A214" s="5" t="s">
+        <v>402</v>
+      </c>
       <c r="B214" s="6"/>
-      <c r="C214" s="6"/>
-      <c r="D214" s="6"/>
+      <c r="C214" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="D214" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="215">
-      <c r="A215" s="6"/>
+      <c r="A215" s="5" t="s">
+        <v>404</v>
+      </c>
       <c r="B215" s="6"/>
-      <c r="C215" s="6"/>
-      <c r="D215" s="6"/>
+      <c r="C215" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="D215" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="216">
-      <c r="A216" s="6"/>
+      <c r="A216" s="5" t="s">
+        <v>406</v>
+      </c>
       <c r="B216" s="6"/>
-      <c r="C216" s="6"/>
-      <c r="D216" s="6"/>
+      <c r="C216" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="D216" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="217">
-      <c r="A217" s="6"/>
+      <c r="A217" s="5" t="s">
+        <v>408</v>
+      </c>
       <c r="B217" s="6"/>
-      <c r="C217" s="6"/>
-      <c r="D217" s="6"/>
+      <c r="C217" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="D217" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="218">
-      <c r="A218" s="6"/>
+      <c r="A218" s="5" t="s">
+        <v>410</v>
+      </c>
       <c r="B218" s="6"/>
-      <c r="C218" s="6"/>
-      <c r="D218" s="6"/>
+      <c r="C218" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D218" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="219">
-      <c r="A219" s="6"/>
+      <c r="A219" s="5" t="s">
+        <v>411</v>
+      </c>
       <c r="B219" s="6"/>
-      <c r="C219" s="6"/>
-      <c r="D219" s="6"/>
+      <c r="C219" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D219" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="220">
-      <c r="A220" s="6"/>
+      <c r="A220" s="5" t="s">
+        <v>413</v>
+      </c>
       <c r="B220" s="6"/>
-      <c r="C220" s="6"/>
-      <c r="D220" s="6"/>
+      <c r="C220" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="D220" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="221">
-      <c r="A221" s="6"/>
+      <c r="A221" s="5" t="s">
+        <v>414</v>
+      </c>
       <c r="B221" s="6"/>
-      <c r="C221" s="6"/>
-      <c r="D221" s="6"/>
+      <c r="C221" s="7" t="s">
+        <v>415</v>
+      </c>
+      <c r="D221" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="222">
-      <c r="A222" s="6"/>
+      <c r="A222" s="5" t="s">
+        <v>416</v>
+      </c>
       <c r="B222" s="6"/>
-      <c r="C222" s="6"/>
-      <c r="D222" s="6"/>
+      <c r="C222" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="D222" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="223">
-      <c r="A223" s="6"/>
-      <c r="B223" s="6"/>
-      <c r="C223" s="6"/>
-      <c r="D223" s="6"/>
+      <c r="A223" s="15" t="s">
+        <v>418</v>
+      </c>
+      <c r="B223" s="16"/>
+      <c r="C223" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="D223" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E223" s="18"/>
+      <c r="F223" s="18"/>
+      <c r="G223" s="18"/>
+      <c r="H223" s="18"/>
+      <c r="I223" s="18"/>
+      <c r="J223" s="18"/>
+      <c r="K223" s="18"/>
+      <c r="L223" s="18"/>
+      <c r="M223" s="18"/>
+      <c r="N223" s="18"/>
+      <c r="O223" s="18"/>
+      <c r="P223" s="18"/>
+      <c r="Q223" s="18"/>
+      <c r="R223" s="18"/>
+      <c r="S223" s="18"/>
+      <c r="T223" s="18"/>
+      <c r="U223" s="18"/>
+      <c r="V223" s="18"/>
+      <c r="W223" s="18"/>
+      <c r="X223" s="18"/>
+      <c r="Y223" s="18"/>
+      <c r="Z223" s="18"/>
     </row>
     <row r="224">
-      <c r="A224" s="6"/>
+      <c r="A224" s="14" t="s">
+        <v>419</v>
+      </c>
       <c r="B224" s="6"/>
-      <c r="C224" s="6"/>
-      <c r="D224" s="6"/>
+      <c r="C224" s="19" t="s">
+        <v>420</v>
+      </c>
+      <c r="D224" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="6"/>
@@ -9104,14 +9471,176 @@
       <c r="C1072" s="6"/>
       <c r="D1072" s="6"/>
     </row>
+    <row r="1073">
+      <c r="A1073" s="6"/>
+      <c r="B1073" s="6"/>
+      <c r="C1073" s="6"/>
+      <c r="D1073" s="6"/>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="6"/>
+      <c r="B1074" s="6"/>
+      <c r="C1074" s="6"/>
+      <c r="D1074" s="6"/>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="6"/>
+      <c r="B1075" s="6"/>
+      <c r="C1075" s="6"/>
+      <c r="D1075" s="6"/>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="6"/>
+      <c r="B1076" s="6"/>
+      <c r="C1076" s="6"/>
+      <c r="D1076" s="6"/>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="6"/>
+      <c r="B1077" s="6"/>
+      <c r="C1077" s="6"/>
+      <c r="D1077" s="6"/>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="6"/>
+      <c r="B1078" s="6"/>
+      <c r="C1078" s="6"/>
+      <c r="D1078" s="6"/>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="6"/>
+      <c r="B1079" s="6"/>
+      <c r="C1079" s="6"/>
+      <c r="D1079" s="6"/>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="6"/>
+      <c r="B1080" s="6"/>
+      <c r="C1080" s="6"/>
+      <c r="D1080" s="6"/>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="6"/>
+      <c r="B1081" s="6"/>
+      <c r="C1081" s="6"/>
+      <c r="D1081" s="6"/>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="6"/>
+      <c r="B1082" s="6"/>
+      <c r="C1082" s="6"/>
+      <c r="D1082" s="6"/>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="6"/>
+      <c r="B1083" s="6"/>
+      <c r="C1083" s="6"/>
+      <c r="D1083" s="6"/>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="6"/>
+      <c r="B1084" s="6"/>
+      <c r="C1084" s="6"/>
+      <c r="D1084" s="6"/>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="6"/>
+      <c r="B1085" s="6"/>
+      <c r="C1085" s="6"/>
+      <c r="D1085" s="6"/>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="6"/>
+      <c r="B1086" s="6"/>
+      <c r="C1086" s="6"/>
+      <c r="D1086" s="6"/>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="6"/>
+      <c r="B1087" s="6"/>
+      <c r="C1087" s="6"/>
+      <c r="D1087" s="6"/>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="6"/>
+      <c r="B1088" s="6"/>
+      <c r="C1088" s="6"/>
+      <c r="D1088" s="6"/>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="6"/>
+      <c r="B1089" s="6"/>
+      <c r="C1089" s="6"/>
+      <c r="D1089" s="6"/>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="6"/>
+      <c r="B1090" s="6"/>
+      <c r="C1090" s="6"/>
+      <c r="D1090" s="6"/>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="6"/>
+      <c r="B1091" s="6"/>
+      <c r="C1091" s="6"/>
+      <c r="D1091" s="6"/>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="6"/>
+      <c r="B1092" s="6"/>
+      <c r="C1092" s="6"/>
+      <c r="D1092" s="6"/>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="6"/>
+      <c r="B1093" s="6"/>
+      <c r="C1093" s="6"/>
+      <c r="D1093" s="6"/>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="6"/>
+      <c r="B1094" s="6"/>
+      <c r="C1094" s="6"/>
+      <c r="D1094" s="6"/>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="6"/>
+      <c r="B1095" s="6"/>
+      <c r="C1095" s="6"/>
+      <c r="D1095" s="6"/>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="6"/>
+      <c r="B1096" s="6"/>
+      <c r="C1096" s="6"/>
+      <c r="D1096" s="6"/>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="6"/>
+      <c r="B1097" s="6"/>
+      <c r="C1097" s="6"/>
+      <c r="D1097" s="6"/>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="6"/>
+      <c r="B1098" s="6"/>
+      <c r="C1098" s="6"/>
+      <c r="D1098" s="6"/>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="6"/>
+      <c r="B1099" s="6"/>
+      <c r="C1099" s="6"/>
+      <c r="D1099" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D195">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D224">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A138"/>
+    <hyperlink r:id="rId1" ref="A164"/>
   </hyperlinks>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
Adds bottom to confirm logout
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="439">
   <si>
     <t>Key</t>
   </si>
@@ -673,6 +673,22 @@
     <t>Log out</t>
   </si>
   <si>
+    <t>profile.logout_bottom_sheet.title</t>
+  </si>
+  <si>
+    <t>Please Confirm</t>
+  </si>
+  <si>
+    <t>profile.logout_bottom_sheet.description</t>
+  </si>
+  <si>
+    <t>Are you sure you want to log out from your account?
+Your Circular ring &lt;strong&gt;won’t synch&lt;/strong&gt; to your account during the time that you are offline.</t>
+  </si>
+  <si>
+    <t>profile.logout_bottom_sheet.logout</t>
+  </si>
+  <si>
     <t>profile.global_score.label</t>
   </si>
   <si>
@@ -743,9 +759,6 @@
   </si>
   <si>
     <t>profile_info.bottom_sheet.sex.title</t>
-  </si>
-  <si>
-    <t>Please Confirm</t>
   </si>
   <si>
     <t>profile_info.bottom_sheet.sex.description</t>
@@ -771,6 +784,12 @@
   </si>
   <si>
     <t>Edit Name</t>
+  </si>
+  <si>
+    <t>profile_info.edit_birthday.title</t>
+  </si>
+  <si>
+    <t>Edit Birthday</t>
   </si>
   <si>
     <t>profile_info.edit_name.save</t>
@@ -1083,7 +1102,7 @@
     <t>Vibration type</t>
   </si>
   <si>
-    <t>alarm.new.edit_vibration.type.alert_default</t>
+    <t>alarm.new.edit_vibration.type.alert</t>
   </si>
   <si>
     <t>Alert (default)</t>
@@ -1291,13 +1310,61 @@
   </si>
   <si>
     <t>profile.header.title</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.discharge</t>
+  </si>
+  <si>
+    <t>Discharge</t>
+  </si>
+  <si>
+    <t>header.profile_advanced_information</t>
+  </si>
+  <si>
+    <t>ADVANCED INFORMATION</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.about_you</t>
+  </si>
+  <si>
+    <t>About you</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.lifestyle_info</t>
+  </si>
+  <si>
+    <t>Lifestyle information</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.title</t>
+  </si>
+  <si>
+    <t>Work Time</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.day</t>
+  </si>
+  <si>
+    <t>Day Worker</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.night</t>
+  </si>
+  <si>
+    <t>Night Worker</t>
+  </si>
+  <si>
+    <t>alarm.new.label.placeholder</t>
+  </si>
+  <si>
+    <t>Enter label here</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1320,10 +1387,6 @@
     <font>
       <u/>
       <color rgb="FF0000FF"/>
-    </font>
-    <font>
-      <strike/>
-      <color rgb="FFFF0000"/>
     </font>
     <font>
       <strike/>
@@ -1369,7 +1432,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="20">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1397,9 +1460,6 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -1407,19 +1467,16 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
+    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
@@ -1431,9 +1488,6 @@
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
@@ -1805,7 +1859,7 @@
         <v>22</v>
       </c>
       <c r="B11" s="6"/>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="7" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="5" t="s">
@@ -1825,7 +1879,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="9" t="s">
         <v>25</v>
       </c>
       <c r="B13" s="6"/>
@@ -1837,7 +1891,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="9" t="s">
         <v>27</v>
       </c>
       <c r="B14" s="6"/>
@@ -1849,7 +1903,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="9" t="s">
         <v>29</v>
       </c>
       <c r="B15" s="6"/>
@@ -2485,68 +2539,68 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="11" t="s">
+      <c r="A68" s="10" t="s">
         <v>120</v>
       </c>
       <c r="C68" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D68" s="11" t="s">
+      <c r="D68" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="11" t="s">
+      <c r="A69" s="10" t="s">
         <v>121</v>
       </c>
       <c r="C69" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="D69" s="11" t="s">
+      <c r="D69" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="12" t="s">
+      <c r="A70" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="C70" s="9" t="s">
+      <c r="C70" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="D70" s="11" t="s">
+      <c r="D70" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="12" t="s">
+      <c r="A71" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="C71" s="9" t="s">
+      <c r="C71" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="D71" s="11" t="s">
+      <c r="D71" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="12" t="s">
+      <c r="A72" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="C72" s="9" t="s">
+      <c r="C72" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D72" s="11" t="s">
+      <c r="D72" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="12" t="s">
+      <c r="A73" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D73" s="11" t="s">
+      <c r="D73" s="10" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3079,11 +3133,11 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="5" t="s">
+      <c r="A118" s="11" t="s">
         <v>215</v>
       </c>
       <c r="B118" s="6"/>
-      <c r="C118" s="7" t="s">
+      <c r="C118" s="12" t="s">
         <v>216</v>
       </c>
       <c r="D118" s="5" t="s">
@@ -3091,11 +3145,11 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="5" t="s">
+      <c r="A119" s="11" t="s">
         <v>217</v>
       </c>
       <c r="B119" s="6"/>
-      <c r="C119" s="7" t="s">
+      <c r="C119" s="12" t="s">
         <v>218</v>
       </c>
       <c r="D119" s="5" t="s">
@@ -3103,12 +3157,12 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="5" t="s">
+      <c r="A120" s="11" t="s">
         <v>219</v>
       </c>
       <c r="B120" s="6"/>
-      <c r="C120" s="7" t="s">
-        <v>220</v>
+      <c r="C120" s="12" t="s">
+        <v>214</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>6</v>
@@ -3116,11 +3170,11 @@
     </row>
     <row r="121">
       <c r="A121" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B121" s="6"/>
       <c r="C121" s="7" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>6</v>
@@ -3156,7 +3210,7 @@
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>227</v>
+        <v>210</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -3164,23 +3218,23 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D125" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="13" t="s">
+      <c r="B126" s="6"/>
+      <c r="C126" s="7" t="s">
         <v>230</v>
-      </c>
-      <c r="B126" s="6"/>
-      <c r="C126" s="9" t="s">
-        <v>231</v>
       </c>
       <c r="D126" s="5" t="s">
         <v>6</v>
@@ -3188,119 +3242,119 @@
     </row>
     <row r="127">
       <c r="A127" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B127" s="6"/>
       <c r="C127" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="D127" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="13" t="s">
+      <c r="B128" s="6"/>
+      <c r="C128" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="B128" s="6"/>
-      <c r="C128" s="9" t="s">
+      <c r="D128" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="s">
         <v>235</v>
-      </c>
-      <c r="D128" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="8" t="s">
-        <v>236</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="D129" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="8" t="s">
+      <c r="B130" s="6"/>
+      <c r="C130" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="B130" s="6"/>
-      <c r="C130" s="9" t="s">
+      <c r="D130" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="D130" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="8" t="s">
+      <c r="B131" s="6"/>
+      <c r="C131" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="B131" s="6"/>
-      <c r="C131" s="9" t="s">
+      <c r="D131" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="8" t="s">
         <v>241</v>
-      </c>
-      <c r="D131" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="5" t="s">
-        <v>242</v>
       </c>
       <c r="B132" s="6"/>
       <c r="C132" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D132" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="8" t="s">
         <v>243</v>
-      </c>
-      <c r="D132" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="5" t="s">
-        <v>244</v>
       </c>
       <c r="B133" s="6"/>
       <c r="C133" s="7" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="5" t="s">
-        <v>246</v>
+      <c r="A134" s="8" t="s">
+        <v>244</v>
       </c>
       <c r="B134" s="6"/>
       <c r="C134" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="B135" s="6"/>
+      <c r="C135" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="D134" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="14" t="s">
-        <v>248</v>
-      </c>
-      <c r="B135" s="15"/>
-      <c r="C135" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="D135" s="16" t="s">
+      <c r="D135" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B136" s="6"/>
       <c r="C136" s="7" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D136" s="5" t="s">
         <v>6</v>
@@ -3308,11 +3362,11 @@
     </row>
     <row r="137">
       <c r="A137" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>6</v>
@@ -3320,35 +3374,35 @@
     </row>
     <row r="138">
       <c r="A138" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B138" s="6"/>
       <c r="C138" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="D138" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="13" t="s">
         <v>254</v>
       </c>
-      <c r="D138" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="B139" s="6"/>
-      <c r="C139" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="D139" s="5" t="s">
+      <c r="B139" s="14"/>
+      <c r="C139" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="D139" s="13" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B140" s="6"/>
       <c r="C140" s="7" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D140" s="5" t="s">
         <v>6</v>
@@ -3356,11 +3410,11 @@
     </row>
     <row r="141">
       <c r="A141" s="5" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="7" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D141" s="5" t="s">
         <v>6</v>
@@ -3368,11 +3422,11 @@
     </row>
     <row r="142">
       <c r="A142" s="5" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B142" s="6"/>
       <c r="C142" s="7" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="D142" s="5" t="s">
         <v>6</v>
@@ -3380,11 +3434,11 @@
     </row>
     <row r="143">
       <c r="A143" s="5" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B143" s="6"/>
       <c r="C143" s="7" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D143" s="5" t="s">
         <v>6</v>
@@ -3392,11 +3446,11 @@
     </row>
     <row r="144">
       <c r="A144" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B144" s="6"/>
       <c r="C144" s="7" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D144" s="5" t="s">
         <v>6</v>
@@ -3404,11 +3458,11 @@
     </row>
     <row r="145">
       <c r="A145" s="5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B145" s="6"/>
       <c r="C145" s="7" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D145" s="5" t="s">
         <v>6</v>
@@ -3416,11 +3470,11 @@
     </row>
     <row r="146">
       <c r="A146" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B146" s="6"/>
       <c r="C146" s="7" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D146" s="5" t="s">
         <v>6</v>
@@ -3428,11 +3482,11 @@
     </row>
     <row r="147">
       <c r="A147" s="5" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B147" s="6"/>
       <c r="C147" s="7" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D147" s="5" t="s">
         <v>6</v>
@@ -3440,11 +3494,11 @@
     </row>
     <row r="148">
       <c r="A148" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B148" s="6"/>
       <c r="C148" s="7" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D148" s="5" t="s">
         <v>6</v>
@@ -3452,11 +3506,11 @@
     </row>
     <row r="149">
       <c r="A149" s="5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B149" s="6"/>
       <c r="C149" s="7" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D149" s="5" t="s">
         <v>6</v>
@@ -3464,11 +3518,11 @@
     </row>
     <row r="150">
       <c r="A150" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B150" s="6"/>
       <c r="C150" s="7" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D150" s="5" t="s">
         <v>6</v>
@@ -3476,47 +3530,47 @@
     </row>
     <row r="151">
       <c r="A151" s="5" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B151" s="6"/>
       <c r="C151" s="7" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D151" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="8" t="s">
-        <v>281</v>
+      <c r="A152" s="5" t="s">
+        <v>279</v>
       </c>
       <c r="B152" s="6"/>
       <c r="C152" s="7" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="D152" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="8" t="s">
-        <v>283</v>
+      <c r="A153" s="5" t="s">
+        <v>281</v>
       </c>
       <c r="B153" s="6"/>
       <c r="C153" s="7" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D153" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="8" t="s">
-        <v>285</v>
+      <c r="A154" s="5" t="s">
+        <v>283</v>
       </c>
       <c r="B154" s="6"/>
       <c r="C154" s="7" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D154" s="5" t="s">
         <v>6</v>
@@ -3524,47 +3578,47 @@
     </row>
     <row r="155">
       <c r="A155" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B155" s="6"/>
       <c r="C155" s="7" t="s">
-        <v>218</v>
+        <v>286</v>
       </c>
       <c r="D155" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="5" t="s">
-        <v>288</v>
+      <c r="A156" s="8" t="s">
+        <v>287</v>
       </c>
       <c r="B156" s="6"/>
       <c r="C156" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="D156" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="8" t="s">
         <v>289</v>
-      </c>
-      <c r="D156" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="5" t="s">
-        <v>290</v>
       </c>
       <c r="B157" s="6"/>
       <c r="C157" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="D157" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="8" t="s">
         <v>291</v>
-      </c>
-      <c r="D157" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="5" t="s">
-        <v>292</v>
       </c>
       <c r="B158" s="6"/>
       <c r="C158" s="7" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D158" s="5" t="s">
         <v>6</v>
@@ -3572,11 +3626,11 @@
     </row>
     <row r="159">
       <c r="A159" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="7" t="s">
-        <v>295</v>
+        <v>223</v>
       </c>
       <c r="D159" s="5" t="s">
         <v>6</v>
@@ -3584,11 +3638,11 @@
     </row>
     <row r="160">
       <c r="A160" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="7" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D160" s="5" t="s">
         <v>6</v>
@@ -3596,11 +3650,11 @@
     </row>
     <row r="161">
       <c r="A161" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="7" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D161" s="5" t="s">
         <v>6</v>
@@ -3608,23 +3662,23 @@
     </row>
     <row r="162">
       <c r="A162" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="7" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="17" t="s">
-        <v>302</v>
+      <c r="A163" s="5" t="s">
+        <v>300</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
@@ -3632,11 +3686,11 @@
     </row>
     <row r="164">
       <c r="A164" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
@@ -3644,11 +3698,11 @@
     </row>
     <row r="165">
       <c r="A165" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="7" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D165" s="5" t="s">
         <v>6</v>
@@ -3656,35 +3710,35 @@
     </row>
     <row r="166">
       <c r="A166" s="5" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="7" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D166" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="5" t="s">
-        <v>310</v>
+      <c r="A167" s="15" t="s">
+        <v>308</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="7" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D167" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="8" t="s">
-        <v>312</v>
+      <c r="A168" s="5" t="s">
+        <v>310</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
@@ -3692,11 +3746,11 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="7" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D169" s="5" t="s">
         <v>6</v>
@@ -3704,11 +3758,11 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="7" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D170" s="5" t="s">
         <v>6</v>
@@ -3716,23 +3770,23 @@
     </row>
     <row r="171">
       <c r="A171" s="5" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="7" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D171" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="5" t="s">
-        <v>320</v>
+      <c r="A172" s="8" t="s">
+        <v>318</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="7" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D172" s="5" t="s">
         <v>6</v>
@@ -3740,11 +3794,11 @@
     </row>
     <row r="173">
       <c r="A173" s="5" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="7" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D173" s="5" t="s">
         <v>6</v>
@@ -3752,11 +3806,11 @@
     </row>
     <row r="174">
       <c r="A174" s="5" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
@@ -3764,11 +3818,11 @@
     </row>
     <row r="175">
       <c r="A175" s="5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
@@ -3776,11 +3830,11 @@
     </row>
     <row r="176">
       <c r="A176" s="5" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
@@ -3788,11 +3842,11 @@
     </row>
     <row r="177">
       <c r="A177" s="5" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
@@ -3800,11 +3854,11 @@
     </row>
     <row r="178">
       <c r="A178" s="5" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
@@ -3812,11 +3866,11 @@
     </row>
     <row r="179">
       <c r="A179" s="5" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
@@ -3824,11 +3878,11 @@
     </row>
     <row r="180">
       <c r="A180" s="5" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
@@ -3836,11 +3890,11 @@
     </row>
     <row r="181">
       <c r="A181" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
@@ -3848,11 +3902,11 @@
     </row>
     <row r="182">
       <c r="A182" s="5" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="7" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>6</v>
@@ -3860,11 +3914,11 @@
     </row>
     <row r="183">
       <c r="A183" s="5" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="7" t="s">
-        <v>47</v>
+        <v>341</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>6</v>
@@ -3872,11 +3926,11 @@
     </row>
     <row r="184">
       <c r="A184" s="5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D184" s="5" t="s">
         <v>6</v>
@@ -3884,11 +3938,11 @@
     </row>
     <row r="185">
       <c r="A185" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="7" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D185" s="5" t="s">
         <v>6</v>
@@ -3896,131 +3950,131 @@
     </row>
     <row r="186">
       <c r="A186" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="D186" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="s">
         <v>348</v>
-      </c>
-      <c r="D186" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="11" t="s">
-        <v>349</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
-        <v>350</v>
+        <v>47</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="11" t="s">
-        <v>351</v>
+      <c r="A188" s="5" t="s">
+        <v>349</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D188" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="11" t="s">
-        <v>353</v>
+      <c r="A189" s="5" t="s">
+        <v>351</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="7" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="11" t="s">
-        <v>355</v>
+      <c r="A190" s="5" t="s">
+        <v>353</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="11" t="s">
-        <v>357</v>
+      <c r="A191" s="10" t="s">
+        <v>355</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="11" t="s">
-        <v>359</v>
+      <c r="A192" s="10" t="s">
+        <v>357</v>
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="5" t="s">
-        <v>361</v>
+      <c r="A193" s="10" t="s">
+        <v>359</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>126</v>
+        <v>360</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="5" t="s">
-        <v>362</v>
+      <c r="A194" s="10" t="s">
+        <v>361</v>
       </c>
       <c r="B194" s="6"/>
       <c r="C194" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="D194" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="10" t="s">
         <v>363</v>
-      </c>
-      <c r="D194" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" s="5" t="s">
-        <v>364</v>
       </c>
       <c r="B195" s="6"/>
       <c r="C195" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="D195" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="10" t="s">
         <v>365</v>
-      </c>
-      <c r="D195" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" s="5" t="s">
-        <v>366</v>
       </c>
       <c r="B196" s="6"/>
       <c r="C196" s="7" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D196" s="5" t="s">
         <v>6</v>
@@ -4028,11 +4082,11 @@
     </row>
     <row r="197">
       <c r="A197" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B197" s="6"/>
       <c r="C197" s="7" t="s">
-        <v>369</v>
+        <v>126</v>
       </c>
       <c r="D197" s="5" t="s">
         <v>6</v>
@@ -4040,11 +4094,11 @@
     </row>
     <row r="198">
       <c r="A198" s="5" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B198" s="6"/>
       <c r="C198" s="7" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D198" s="5" t="s">
         <v>6</v>
@@ -4052,11 +4106,11 @@
     </row>
     <row r="199">
       <c r="A199" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B199" s="6"/>
       <c r="C199" s="7" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="D199" s="5" t="s">
         <v>6</v>
@@ -4064,11 +4118,11 @@
     </row>
     <row r="200">
       <c r="A200" s="5" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B200" s="6"/>
       <c r="C200" s="7" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D200" s="5" t="s">
         <v>6</v>
@@ -4076,11 +4130,11 @@
     </row>
     <row r="201">
       <c r="A201" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B201" s="6"/>
       <c r="C201" s="7" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="D201" s="5" t="s">
         <v>6</v>
@@ -4088,11 +4142,11 @@
     </row>
     <row r="202">
       <c r="A202" s="5" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B202" s="6"/>
       <c r="C202" s="7" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D202" s="5" t="s">
         <v>6</v>
@@ -4100,11 +4154,11 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B203" s="6"/>
       <c r="C203" s="7" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D203" s="5" t="s">
         <v>6</v>
@@ -4112,11 +4166,11 @@
     </row>
     <row r="204">
       <c r="A204" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B204" s="6"/>
       <c r="C204" s="7" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D204" s="5" t="s">
         <v>6</v>
@@ -4124,11 +4178,11 @@
     </row>
     <row r="205">
       <c r="A205" s="5" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B205" s="6"/>
       <c r="C205" s="7" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D205" s="5" t="s">
         <v>6</v>
@@ -4136,11 +4190,11 @@
     </row>
     <row r="206">
       <c r="A206" s="5" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B206" s="6"/>
       <c r="C206" s="7" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D206" s="5" t="s">
         <v>6</v>
@@ -4148,11 +4202,11 @@
     </row>
     <row r="207">
       <c r="A207" s="5" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B207" s="6"/>
       <c r="C207" s="7" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D207" s="5" t="s">
         <v>6</v>
@@ -4160,11 +4214,11 @@
     </row>
     <row r="208">
       <c r="A208" s="5" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B208" s="6"/>
       <c r="C208" s="7" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D208" s="5" t="s">
         <v>6</v>
@@ -4172,11 +4226,11 @@
     </row>
     <row r="209">
       <c r="A209" s="5" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B209" s="6"/>
       <c r="C209" s="7" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="D209" s="5" t="s">
         <v>6</v>
@@ -4184,11 +4238,11 @@
     </row>
     <row r="210">
       <c r="A210" s="5" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B210" s="6"/>
       <c r="C210" s="7" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D210" s="5" t="s">
         <v>6</v>
@@ -4196,11 +4250,11 @@
     </row>
     <row r="211">
       <c r="A211" s="5" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B211" s="6"/>
       <c r="C211" s="7" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D211" s="5" t="s">
         <v>6</v>
@@ -4208,11 +4262,11 @@
     </row>
     <row r="212">
       <c r="A212" s="5" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B212" s="6"/>
       <c r="C212" s="7" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D212" s="5" t="s">
         <v>6</v>
@@ -4220,11 +4274,11 @@
     </row>
     <row r="213">
       <c r="A213" s="5" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B213" s="6"/>
       <c r="C213" s="7" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="D213" s="5" t="s">
         <v>6</v>
@@ -4232,11 +4286,11 @@
     </row>
     <row r="214">
       <c r="A214" s="5" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B214" s="6"/>
       <c r="C214" s="7" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="D214" s="5" t="s">
         <v>6</v>
@@ -4244,11 +4298,11 @@
     </row>
     <row r="215">
       <c r="A215" s="5" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B215" s="6"/>
       <c r="C215" s="7" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="D215" s="5" t="s">
         <v>6</v>
@@ -4256,11 +4310,11 @@
     </row>
     <row r="216">
       <c r="A216" s="5" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B216" s="6"/>
       <c r="C216" s="7" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="D216" s="5" t="s">
         <v>6</v>
@@ -4268,11 +4322,11 @@
     </row>
     <row r="217">
       <c r="A217" s="5" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B217" s="6"/>
       <c r="C217" s="7" t="s">
-        <v>160</v>
+        <v>407</v>
       </c>
       <c r="D217" s="5" t="s">
         <v>6</v>
@@ -4280,11 +4334,11 @@
     </row>
     <row r="218">
       <c r="A218" s="5" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B218" s="6"/>
       <c r="C218" s="7" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="D218" s="5" t="s">
         <v>6</v>
@@ -4292,11 +4346,11 @@
     </row>
     <row r="219">
       <c r="A219" s="5" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B219" s="6"/>
       <c r="C219" s="7" t="s">
-        <v>293</v>
+        <v>411</v>
       </c>
       <c r="D219" s="5" t="s">
         <v>6</v>
@@ -4320,117 +4374,190 @@
       </c>
       <c r="B221" s="6"/>
       <c r="C221" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D221" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="5" t="s">
         <v>415</v>
       </c>
-      <c r="D221" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" s="18" t="s">
+      <c r="B222" s="6"/>
+      <c r="C222" s="7" t="s">
         <v>416</v>
       </c>
-      <c r="B222" s="19"/>
-      <c r="C222" s="20" t="s">
-        <v>218</v>
-      </c>
-      <c r="D222" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="E222" s="22"/>
-      <c r="F222" s="22"/>
-      <c r="G222" s="22"/>
-      <c r="H222" s="22"/>
-      <c r="I222" s="22"/>
-      <c r="J222" s="22"/>
-      <c r="K222" s="22"/>
-      <c r="L222" s="22"/>
-      <c r="M222" s="22"/>
-      <c r="N222" s="22"/>
-      <c r="O222" s="22"/>
-      <c r="P222" s="22"/>
-      <c r="Q222" s="22"/>
-      <c r="R222" s="22"/>
-      <c r="S222" s="22"/>
-      <c r="T222" s="22"/>
-      <c r="U222" s="22"/>
-      <c r="V222" s="22"/>
-      <c r="W222" s="22"/>
-      <c r="X222" s="22"/>
-      <c r="Y222" s="22"/>
-      <c r="Z222" s="22"/>
+      <c r="D222" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="223">
-      <c r="A223" s="6"/>
+      <c r="A223" s="5" t="s">
+        <v>417</v>
+      </c>
       <c r="B223" s="6"/>
-      <c r="C223" s="6"/>
-      <c r="D223" s="6"/>
+      <c r="C223" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="D223" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="224">
-      <c r="A224" s="6"/>
+      <c r="A224" s="5" t="s">
+        <v>418</v>
+      </c>
       <c r="B224" s="6"/>
-      <c r="C224" s="6"/>
-      <c r="D224" s="6"/>
+      <c r="C224" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="D224" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="225">
-      <c r="A225" s="6"/>
+      <c r="A225" s="5" t="s">
+        <v>420</v>
+      </c>
       <c r="B225" s="6"/>
-      <c r="C225" s="6"/>
-      <c r="D225" s="6"/>
+      <c r="C225" s="7" t="s">
+        <v>421</v>
+      </c>
+      <c r="D225" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="226">
-      <c r="A226" s="6"/>
-      <c r="B226" s="6"/>
-      <c r="C226" s="6"/>
-      <c r="D226" s="6"/>
+      <c r="A226" s="16" t="s">
+        <v>422</v>
+      </c>
+      <c r="B226" s="17"/>
+      <c r="C226" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="D226" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E226" s="19"/>
+      <c r="F226" s="19"/>
+      <c r="G226" s="19"/>
+      <c r="H226" s="19"/>
+      <c r="I226" s="19"/>
+      <c r="J226" s="19"/>
+      <c r="K226" s="19"/>
+      <c r="L226" s="19"/>
+      <c r="M226" s="19"/>
+      <c r="N226" s="19"/>
+      <c r="O226" s="19"/>
+      <c r="P226" s="19"/>
+      <c r="Q226" s="19"/>
+      <c r="R226" s="19"/>
+      <c r="S226" s="19"/>
+      <c r="T226" s="19"/>
+      <c r="U226" s="19"/>
+      <c r="V226" s="19"/>
+      <c r="W226" s="19"/>
+      <c r="X226" s="19"/>
+      <c r="Y226" s="19"/>
+      <c r="Z226" s="19"/>
     </row>
     <row r="227">
-      <c r="A227" s="6"/>
+      <c r="A227" s="5" t="s">
+        <v>423</v>
+      </c>
       <c r="B227" s="6"/>
-      <c r="C227" s="6"/>
-      <c r="D227" s="6"/>
+      <c r="C227" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="D227" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="228">
-      <c r="A228" s="6"/>
+      <c r="A228" s="5" t="s">
+        <v>425</v>
+      </c>
       <c r="B228" s="6"/>
-      <c r="C228" s="6"/>
-      <c r="D228" s="6"/>
+      <c r="C228" s="7" t="s">
+        <v>426</v>
+      </c>
+      <c r="D228" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="229">
-      <c r="A229" s="6"/>
+      <c r="A229" s="5" t="s">
+        <v>427</v>
+      </c>
       <c r="B229" s="6"/>
-      <c r="C229" s="6"/>
-      <c r="D229" s="6"/>
+      <c r="C229" s="7" t="s">
+        <v>428</v>
+      </c>
+      <c r="D229" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="230">
-      <c r="A230" s="6"/>
+      <c r="A230" s="5" t="s">
+        <v>429</v>
+      </c>
       <c r="B230" s="6"/>
-      <c r="C230" s="6"/>
-      <c r="D230" s="6"/>
+      <c r="C230" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="D230" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="231">
-      <c r="A231" s="6"/>
+      <c r="A231" s="5" t="s">
+        <v>431</v>
+      </c>
       <c r="B231" s="6"/>
-      <c r="C231" s="6"/>
-      <c r="D231" s="6"/>
+      <c r="C231" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="D231" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="232">
-      <c r="A232" s="6"/>
+      <c r="A232" s="5" t="s">
+        <v>433</v>
+      </c>
       <c r="B232" s="6"/>
-      <c r="C232" s="6"/>
-      <c r="D232" s="6"/>
+      <c r="C232" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="D232" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="233">
-      <c r="A233" s="6"/>
+      <c r="A233" s="5" t="s">
+        <v>435</v>
+      </c>
       <c r="B233" s="6"/>
-      <c r="C233" s="6"/>
-      <c r="D233" s="6"/>
+      <c r="C233" s="7" t="s">
+        <v>436</v>
+      </c>
+      <c r="D233" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="234">
-      <c r="A234" s="6"/>
-      <c r="B234" s="6"/>
-      <c r="C234" s="6"/>
-      <c r="D234" s="6"/>
+      <c r="A234" s="16" t="s">
+        <v>437</v>
+      </c>
+      <c r="B234" s="17"/>
+      <c r="C234" s="18" t="s">
+        <v>438</v>
+      </c>
+      <c r="D234" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E234" s="19"/>
     </row>
     <row r="235">
       <c r="A235" s="6"/>
@@ -9616,14 +9743,38 @@
       <c r="C1098" s="6"/>
       <c r="D1098" s="6"/>
     </row>
+    <row r="1099">
+      <c r="A1099" s="6"/>
+      <c r="B1099" s="6"/>
+      <c r="C1099" s="6"/>
+      <c r="D1099" s="6"/>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="6"/>
+      <c r="B1100" s="6"/>
+      <c r="C1100" s="6"/>
+      <c r="D1100" s="6"/>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="6"/>
+      <c r="B1101" s="6"/>
+      <c r="C1101" s="6"/>
+      <c r="D1101" s="6"/>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="6"/>
+      <c r="B1102" s="6"/>
+      <c r="C1102" s="6"/>
+      <c r="D1102" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D222">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D234">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A163"/>
+    <hyperlink r:id="rId1" ref="A167"/>
   </hyperlinks>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
CIRC-153 Add ring to account CIRC-154 Handle pairing error
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="510">
   <si>
     <t>Key</t>
   </si>
@@ -104,6 +104,19 @@
   </si>
   <si>
     <t>Success !</t>
+  </si>
+  <si>
+    <t>setup.pairing.failed.title</t>
+  </si>
+  <si>
+    <t>Pairing Failed</t>
+  </si>
+  <si>
+    <t>setup.pairing.failed.message</t>
+  </si>
+  <si>
+    <t>This ring is currently associated to an already existing Circular account.
+&lt;strong&gt;Unpair it&lt;/strong&gt; from your other account by going into the ‘My Ring’ menu and clicking on the red cross. An email has been sent to the currently associated account.</t>
   </si>
   <si>
     <t>login.title</t>
@@ -399,6 +412,18 @@
   </si>
   <si>
     <t>global.default_error</t>
+  </si>
+  <si>
+    <t>global.yes</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>global.no</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
   <si>
     <t>home.sync.syncing</t>
@@ -1342,6 +1367,12 @@
     <t>Work Time</t>
   </si>
   <si>
+    <t>alarm.new.label.placeholder</t>
+  </si>
+  <si>
+    <t>Enter label here</t>
+  </si>
+  <si>
     <t>profile_advanced_info.work_time.day</t>
   </si>
   <si>
@@ -1354,17 +1385,200 @@
     <t>Night Worker</t>
   </si>
   <si>
-    <t>alarm.new.label.placeholder</t>
-  </si>
-  <si>
-    <t>Enter label here</t>
+    <t>profile_advanced_info.chrono_type.morning</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.solar</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.night</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.morning_erratic</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.solar_erratic</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.night_erratic</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.title</t>
+  </si>
+  <si>
+    <t>Physical Disabilities</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.none</t>
+  </si>
+  <si>
+    <t>No physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.moderate</t>
+  </si>
+  <si>
+    <t>Moderate physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.total</t>
+  </si>
+  <si>
+    <t>Total physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.title</t>
+  </si>
+  <si>
+    <t>Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.none</t>
+  </si>
+  <si>
+    <t>No Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.insomnia</t>
+  </si>
+  <si>
+    <t>Insomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.hypersomnia</t>
+  </si>
+  <si>
+    <t>Hypersomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.other</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.title</t>
+  </si>
+  <si>
+    <t>Sleep Aid</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.none</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.daily</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.weekly</t>
+  </si>
+  <si>
+    <t>Weekly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.monthly</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.title</t>
+  </si>
+  <si>
+    <t>Sleep supplements</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.none</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.daily</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.weekly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.monthly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeper_type.light</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeper_type.night</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.menstrual_cycle</t>
+  </si>
+  <si>
+    <t>Menstrual cycle</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.menopause</t>
+  </si>
+  <si>
+    <t>Menopause</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.perimenopause</t>
+  </si>
+  <si>
+    <t>Perimenopause</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.none</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.pills</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.condoms</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.vaginal_ring</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.patch</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.iud</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.implant</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.fertility_awareness</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.other</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_28</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_24</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_21</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.open_for_napping.title</t>
+  </si>
+  <si>
+    <t>Open for Napping</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.unknown_option</t>
+  </si>
+  <si>
+    <t>Unknown option</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1384,6 +1598,10 @@
       <name val="Arial"/>
     </font>
     <font/>
+    <font>
+      <u/>
+      <color rgb="FF1155CC"/>
+    </font>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -1432,7 +1650,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1467,10 +1685,13 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
@@ -1478,19 +1699,22 @@
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1915,7 +2139,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B16" s="6"/>
@@ -1927,7 +2151,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="9" t="s">
         <v>33</v>
       </c>
       <c r="B17" s="6"/>
@@ -1968,7 +2192,7 @@
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>6</v>
@@ -1976,11 +2200,11 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>6</v>
@@ -1988,11 +2212,11 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>6</v>
@@ -2064,19 +2288,19 @@
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>55</v>
+      <c r="A29" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="7" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>6</v>
@@ -2084,23 +2308,23 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="s">
-        <v>57</v>
+      <c r="A31" s="8" t="s">
+        <v>59</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>6</v>
@@ -2108,11 +2332,11 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="7" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>6</v>
@@ -2120,11 +2344,11 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>6</v>
@@ -2132,7 +2356,7 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
@@ -2144,11 +2368,11 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>6</v>
@@ -2156,11 +2380,11 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>6</v>
@@ -2168,11 +2392,11 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>6</v>
@@ -2180,11 +2404,11 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>6</v>
@@ -2192,11 +2416,11 @@
     </row>
     <row r="39">
       <c r="A39" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="7" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>6</v>
@@ -2204,11 +2428,11 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>6</v>
@@ -2216,11 +2440,11 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>6</v>
@@ -2280,7 +2504,7 @@
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
-        <v>47</v>
+        <v>81</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>6</v>
@@ -2288,11 +2512,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>6</v>
@@ -2300,11 +2524,11 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>6</v>
@@ -2412,7 +2636,7 @@
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
-        <v>36</v>
+        <v>102</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>6</v>
@@ -2420,11 +2644,11 @@
     </row>
     <row r="58">
       <c r="A58" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -2432,11 +2656,11 @@
     </row>
     <row r="59">
       <c r="A59" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B59" s="6"/>
       <c r="C59" s="7" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>6</v>
@@ -2444,11 +2668,11 @@
     </row>
     <row r="60">
       <c r="A60" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>6</v>
@@ -2456,11 +2680,11 @@
     </row>
     <row r="61">
       <c r="A61" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="7" t="s">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>6</v>
@@ -2468,11 +2692,11 @@
     </row>
     <row r="62">
       <c r="A62" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B62" s="6"/>
       <c r="C62" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>6</v>
@@ -2480,11 +2704,11 @@
     </row>
     <row r="63">
       <c r="A63" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="7" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>6</v>
@@ -2539,33 +2763,35 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="10" t="s">
+      <c r="A68" s="5" t="s">
         <v>120</v>
       </c>
+      <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D68" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D68" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="10" t="s">
-        <v>121</v>
-      </c>
+      <c r="A69" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B69" s="6"/>
       <c r="C69" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D69" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="D69" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>124</v>
+        <v>10</v>
       </c>
       <c r="D70" s="10" t="s">
         <v>6</v>
@@ -2587,7 +2813,7 @@
         <v>127</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>12</v>
+        <v>128</v>
       </c>
       <c r="D72" s="10" t="s">
         <v>6</v>
@@ -2595,60 +2821,56 @@
     </row>
     <row r="73">
       <c r="A73" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>47</v>
+        <v>130</v>
       </c>
       <c r="D73" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="B74" s="6"/>
+      <c r="A74" s="10" t="s">
+        <v>131</v>
+      </c>
       <c r="C74" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="D74" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D74" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="B75" s="6"/>
+      <c r="A75" s="10" t="s">
+        <v>132</v>
+      </c>
       <c r="C75" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="D75" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D75" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="5" t="s">
+      <c r="A76" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="B76" s="6"/>
-      <c r="C76" s="7" t="s">
+      <c r="C76" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="D76" s="5" t="s">
+      <c r="D76" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="5" t="s">
+      <c r="A77" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="B77" s="6"/>
-      <c r="C77" s="7" t="s">
+      <c r="C77" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="D77" s="5" t="s">
+      <c r="D77" s="10" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2749,7 +2971,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="8" t="s">
+      <c r="A86" s="5" t="s">
         <v>153</v>
       </c>
       <c r="B86" s="6"/>
@@ -2761,7 +2983,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="8" t="s">
+      <c r="A87" s="5" t="s">
         <v>155</v>
       </c>
       <c r="B87" s="6"/>
@@ -2797,7 +3019,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="5" t="s">
+      <c r="A90" s="8" t="s">
         <v>161</v>
       </c>
       <c r="B90" s="6"/>
@@ -2809,7 +3031,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="s">
+      <c r="A91" s="8" t="s">
         <v>163</v>
       </c>
       <c r="B91" s="6"/>
@@ -3078,7 +3300,7 @@
       </c>
       <c r="B113" s="6"/>
       <c r="C113" s="7" t="s">
-        <v>36</v>
+        <v>208</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>6</v>
@@ -3086,11 +3308,11 @@
     </row>
     <row r="114">
       <c r="A114" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B114" s="6"/>
       <c r="C114" s="7" t="s">
-        <v>36</v>
+        <v>210</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>6</v>
@@ -3098,11 +3320,11 @@
     </row>
     <row r="115">
       <c r="A115" s="5" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B115" s="6"/>
       <c r="C115" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>6</v>
@@ -3110,11 +3332,11 @@
     </row>
     <row r="116">
       <c r="A116" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="B116" s="5"/>
+        <v>213</v>
+      </c>
+      <c r="B116" s="6"/>
       <c r="C116" s="7" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D116" s="5" t="s">
         <v>6</v>
@@ -3122,34 +3344,34 @@
     </row>
     <row r="117">
       <c r="A117" s="5" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B117" s="6"/>
       <c r="C117" s="7" t="s">
-        <v>214</v>
+        <v>40</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="11" t="s">
-        <v>215</v>
+      <c r="A118" s="5" t="s">
+        <v>216</v>
       </c>
       <c r="B118" s="6"/>
-      <c r="C118" s="12" t="s">
-        <v>216</v>
+      <c r="C118" s="7" t="s">
+        <v>40</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="11" t="s">
+      <c r="A119" s="5" t="s">
         <v>217</v>
       </c>
       <c r="B119" s="6"/>
-      <c r="C119" s="12" t="s">
+      <c r="C119" s="7" t="s">
         <v>218</v>
       </c>
       <c r="D119" s="5" t="s">
@@ -3157,12 +3379,12 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="11" t="s">
+      <c r="A120" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="B120" s="6"/>
-      <c r="C120" s="12" t="s">
-        <v>214</v>
+      <c r="B120" s="5"/>
+      <c r="C120" s="7" t="s">
+        <v>220</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>6</v>
@@ -3170,11 +3392,11 @@
     </row>
     <row r="121">
       <c r="A121" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B121" s="6"/>
       <c r="C121" s="7" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>6</v>
@@ -3182,11 +3404,11 @@
     </row>
     <row r="122">
       <c r="A122" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B122" s="6"/>
       <c r="C122" s="7" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>6</v>
@@ -3194,11 +3416,11 @@
     </row>
     <row r="123">
       <c r="A123" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B123" s="6"/>
       <c r="C123" s="7" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>6</v>
@@ -3206,11 +3428,11 @@
     </row>
     <row r="124">
       <c r="A124" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -3218,11 +3440,11 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>6</v>
@@ -3230,11 +3452,11 @@
     </row>
     <row r="126">
       <c r="A126" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B126" s="6"/>
       <c r="C126" s="7" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D126" s="5" t="s">
         <v>6</v>
@@ -3242,11 +3464,11 @@
     </row>
     <row r="127">
       <c r="A127" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B127" s="6"/>
       <c r="C127" s="7" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D127" s="5" t="s">
         <v>6</v>
@@ -3254,11 +3476,11 @@
     </row>
     <row r="128">
       <c r="A128" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
-        <v>234</v>
+        <v>218</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>6</v>
@@ -3301,7 +3523,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="8" t="s">
+      <c r="A132" s="5" t="s">
         <v>241</v>
       </c>
       <c r="B132" s="6"/>
@@ -3313,24 +3535,24 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="8" t="s">
+      <c r="A133" s="5" t="s">
         <v>243</v>
       </c>
       <c r="B133" s="6"/>
       <c r="C133" s="7" t="s">
-        <v>216</v>
+        <v>244</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="8" t="s">
-        <v>244</v>
+      <c r="A134" s="5" t="s">
+        <v>245</v>
       </c>
       <c r="B134" s="6"/>
       <c r="C134" s="7" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D134" s="5" t="s">
         <v>6</v>
@@ -3338,42 +3560,42 @@
     </row>
     <row r="135">
       <c r="A135" s="5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B135" s="6"/>
       <c r="C135" s="7" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D135" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="5" t="s">
-        <v>248</v>
+      <c r="A136" s="8" t="s">
+        <v>249</v>
       </c>
       <c r="B136" s="6"/>
       <c r="C136" s="7" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D136" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="5" t="s">
-        <v>250</v>
+      <c r="A137" s="8" t="s">
+        <v>251</v>
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
-        <v>251</v>
+        <v>224</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="5" t="s">
+      <c r="A138" s="8" t="s">
         <v>252</v>
       </c>
       <c r="B138" s="6"/>
@@ -3385,24 +3607,24 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="13" t="s">
+      <c r="A139" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="B139" s="14"/>
-      <c r="C139" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="D139" s="13" t="s">
+      <c r="B139" s="6"/>
+      <c r="C139" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="D139" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B140" s="6"/>
       <c r="C140" s="7" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D140" s="5" t="s">
         <v>6</v>
@@ -3410,11 +3632,11 @@
     </row>
     <row r="141">
       <c r="A141" s="5" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="7" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D141" s="5" t="s">
         <v>6</v>
@@ -3422,25 +3644,25 @@
     </row>
     <row r="142">
       <c r="A142" s="5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B142" s="6"/>
       <c r="C142" s="7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D142" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="B143" s="6"/>
-      <c r="C143" s="7" t="s">
+      <c r="A143" s="14" t="s">
         <v>262</v>
       </c>
-      <c r="D143" s="5" t="s">
+      <c r="B143" s="15"/>
+      <c r="C143" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="D143" s="14" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3589,7 +3811,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="8" t="s">
+      <c r="A156" s="5" t="s">
         <v>287</v>
       </c>
       <c r="B156" s="6"/>
@@ -3601,7 +3823,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="8" t="s">
+      <c r="A157" s="5" t="s">
         <v>289</v>
       </c>
       <c r="B157" s="6"/>
@@ -3613,7 +3835,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="8" t="s">
+      <c r="A158" s="5" t="s">
         <v>291</v>
       </c>
       <c r="B158" s="6"/>
@@ -3630,43 +3852,43 @@
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="7" t="s">
-        <v>223</v>
+        <v>294</v>
       </c>
       <c r="D159" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="5" t="s">
-        <v>294</v>
+      <c r="A160" s="8" t="s">
+        <v>295</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="7" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D160" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="5" t="s">
-        <v>296</v>
+      <c r="A161" s="8" t="s">
+        <v>297</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D161" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="5" t="s">
-        <v>298</v>
+      <c r="A162" s="8" t="s">
+        <v>299</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>6</v>
@@ -3674,11 +3896,11 @@
     </row>
     <row r="163">
       <c r="A163" s="5" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>301</v>
+        <v>231</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
@@ -3721,7 +3943,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="15" t="s">
+      <c r="A167" s="5" t="s">
         <v>308</v>
       </c>
       <c r="B167" s="6"/>
@@ -3769,7 +3991,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="5" t="s">
+      <c r="A171" s="16" t="s">
         <v>316</v>
       </c>
       <c r="B171" s="6"/>
@@ -3781,7 +4003,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="8" t="s">
+      <c r="A172" s="5" t="s">
         <v>318</v>
       </c>
       <c r="B172" s="6"/>
@@ -3829,7 +4051,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="5" t="s">
+      <c r="A176" s="8" t="s">
         <v>326</v>
       </c>
       <c r="B176" s="6"/>
@@ -3966,7 +4188,7 @@
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
-        <v>47</v>
+        <v>349</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>6</v>
@@ -3974,11 +4196,11 @@
     </row>
     <row r="188">
       <c r="A188" s="5" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D188" s="5" t="s">
         <v>6</v>
@@ -3986,11 +4208,11 @@
     </row>
     <row r="189">
       <c r="A189" s="5" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="7" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>6</v>
@@ -3998,30 +4220,30 @@
     </row>
     <row r="190">
       <c r="A190" s="5" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="10" t="s">
-        <v>355</v>
+      <c r="A191" s="5" t="s">
+        <v>356</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
-        <v>356</v>
+        <v>51</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="10" t="s">
+      <c r="A192" s="5" t="s">
         <v>357</v>
       </c>
       <c r="B192" s="6"/>
@@ -4033,7 +4255,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="10" t="s">
+      <c r="A193" s="5" t="s">
         <v>359</v>
       </c>
       <c r="B193" s="6"/>
@@ -4045,7 +4267,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="10" t="s">
+      <c r="A194" s="5" t="s">
         <v>361</v>
       </c>
       <c r="B194" s="6"/>
@@ -4081,48 +4303,48 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="5" t="s">
+      <c r="A197" s="10" t="s">
         <v>367</v>
       </c>
       <c r="B197" s="6"/>
       <c r="C197" s="7" t="s">
-        <v>126</v>
+        <v>368</v>
       </c>
       <c r="D197" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="5" t="s">
-        <v>368</v>
+      <c r="A198" s="10" t="s">
+        <v>369</v>
       </c>
       <c r="B198" s="6"/>
       <c r="C198" s="7" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D198" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="5" t="s">
-        <v>370</v>
+      <c r="A199" s="10" t="s">
+        <v>371</v>
       </c>
       <c r="B199" s="6"/>
       <c r="C199" s="7" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D199" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="5" t="s">
-        <v>372</v>
+      <c r="A200" s="10" t="s">
+        <v>373</v>
       </c>
       <c r="B200" s="6"/>
       <c r="C200" s="7" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D200" s="5" t="s">
         <v>6</v>
@@ -4130,11 +4352,11 @@
     </row>
     <row r="201">
       <c r="A201" s="5" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B201" s="6"/>
       <c r="C201" s="7" t="s">
-        <v>375</v>
+        <v>130</v>
       </c>
       <c r="D201" s="5" t="s">
         <v>6</v>
@@ -4374,7 +4596,7 @@
       </c>
       <c r="B221" s="6"/>
       <c r="C221" s="7" t="s">
-        <v>160</v>
+        <v>415</v>
       </c>
       <c r="D221" s="5" t="s">
         <v>6</v>
@@ -4382,11 +4604,11 @@
     </row>
     <row r="222">
       <c r="A222" s="5" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B222" s="6"/>
       <c r="C222" s="7" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D222" s="5" t="s">
         <v>6</v>
@@ -4394,11 +4616,11 @@
     </row>
     <row r="223">
       <c r="A223" s="5" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B223" s="6"/>
       <c r="C223" s="7" t="s">
-        <v>299</v>
+        <v>419</v>
       </c>
       <c r="D223" s="5" t="s">
         <v>6</v>
@@ -4406,11 +4628,11 @@
     </row>
     <row r="224">
       <c r="A224" s="5" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B224" s="6"/>
       <c r="C224" s="7" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D224" s="5" t="s">
         <v>6</v>
@@ -4418,57 +4640,35 @@
     </row>
     <row r="225">
       <c r="A225" s="5" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B225" s="6"/>
       <c r="C225" s="7" t="s">
-        <v>421</v>
+        <v>168</v>
       </c>
       <c r="D225" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="16" t="s">
-        <v>422</v>
-      </c>
-      <c r="B226" s="17"/>
-      <c r="C226" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D226" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="E226" s="19"/>
-      <c r="F226" s="19"/>
-      <c r="G226" s="19"/>
-      <c r="H226" s="19"/>
-      <c r="I226" s="19"/>
-      <c r="J226" s="19"/>
-      <c r="K226" s="19"/>
-      <c r="L226" s="19"/>
-      <c r="M226" s="19"/>
-      <c r="N226" s="19"/>
-      <c r="O226" s="19"/>
-      <c r="P226" s="19"/>
-      <c r="Q226" s="19"/>
-      <c r="R226" s="19"/>
-      <c r="S226" s="19"/>
-      <c r="T226" s="19"/>
-      <c r="U226" s="19"/>
-      <c r="V226" s="19"/>
-      <c r="W226" s="19"/>
-      <c r="X226" s="19"/>
-      <c r="Y226" s="19"/>
-      <c r="Z226" s="19"/>
+      <c r="A226" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="B226" s="6"/>
+      <c r="C226" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="D226" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="5" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B227" s="6"/>
       <c r="C227" s="7" t="s">
-        <v>424</v>
+        <v>307</v>
       </c>
       <c r="D227" s="5" t="s">
         <v>6</v>
@@ -4476,11 +4676,11 @@
     </row>
     <row r="228">
       <c r="A228" s="5" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B228" s="6"/>
       <c r="C228" s="7" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D228" s="5" t="s">
         <v>6</v>
@@ -4488,27 +4688,49 @@
     </row>
     <row r="229">
       <c r="A229" s="5" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B229" s="6"/>
       <c r="C229" s="7" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D229" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="B230" s="6"/>
-      <c r="C230" s="7" t="s">
+      <c r="A230" s="17" t="s">
         <v>430</v>
       </c>
-      <c r="D230" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="B230" s="18"/>
+      <c r="C230" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="D230" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E230" s="20"/>
+      <c r="F230" s="20"/>
+      <c r="G230" s="20"/>
+      <c r="H230" s="20"/>
+      <c r="I230" s="20"/>
+      <c r="J230" s="20"/>
+      <c r="K230" s="20"/>
+      <c r="L230" s="20"/>
+      <c r="M230" s="20"/>
+      <c r="N230" s="20"/>
+      <c r="O230" s="20"/>
+      <c r="P230" s="20"/>
+      <c r="Q230" s="20"/>
+      <c r="R230" s="20"/>
+      <c r="S230" s="20"/>
+      <c r="T230" s="20"/>
+      <c r="U230" s="20"/>
+      <c r="V230" s="20"/>
+      <c r="W230" s="20"/>
+      <c r="X230" s="20"/>
+      <c r="Y230" s="20"/>
+      <c r="Z230" s="20"/>
     </row>
     <row r="231">
       <c r="A231" s="5" t="s">
@@ -4547,305 +4769,513 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="16" t="s">
+      <c r="A234" s="5" t="s">
         <v>437</v>
       </c>
-      <c r="B234" s="17"/>
-      <c r="C234" s="18" t="s">
+      <c r="B234" s="6"/>
+      <c r="C234" s="7" t="s">
         <v>438</v>
       </c>
-      <c r="D234" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="E234" s="19"/>
+      <c r="D234" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="235">
-      <c r="A235" s="6"/>
+      <c r="A235" s="5" t="s">
+        <v>439</v>
+      </c>
       <c r="B235" s="6"/>
-      <c r="C235" s="6"/>
-      <c r="D235" s="6"/>
+      <c r="C235" s="7" t="s">
+        <v>440</v>
+      </c>
+      <c r="D235" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="236">
-      <c r="A236" s="6"/>
-      <c r="B236" s="6"/>
-      <c r="C236" s="6"/>
-      <c r="D236" s="6"/>
+      <c r="A236" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="B236" s="18"/>
+      <c r="C236" s="19" t="s">
+        <v>442</v>
+      </c>
+      <c r="D236" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E236" s="20"/>
     </row>
     <row r="237">
-      <c r="A237" s="6"/>
+      <c r="A237" s="21" t="s">
+        <v>443</v>
+      </c>
       <c r="B237" s="6"/>
-      <c r="C237" s="6"/>
-      <c r="D237" s="6"/>
+      <c r="C237" s="12" t="s">
+        <v>444</v>
+      </c>
+      <c r="D237" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="238">
-      <c r="A238" s="6"/>
+      <c r="A238" s="21" t="s">
+        <v>445</v>
+      </c>
       <c r="B238" s="6"/>
-      <c r="C238" s="6"/>
-      <c r="D238" s="6"/>
+      <c r="C238" s="12" t="s">
+        <v>446</v>
+      </c>
+      <c r="D238" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="239">
-      <c r="A239" s="6"/>
+      <c r="A239" s="21" t="s">
+        <v>447</v>
+      </c>
       <c r="B239" s="6"/>
       <c r="C239" s="6"/>
       <c r="D239" s="6"/>
     </row>
     <row r="240">
-      <c r="A240" s="6"/>
+      <c r="A240" s="21" t="s">
+        <v>448</v>
+      </c>
       <c r="B240" s="6"/>
       <c r="C240" s="6"/>
       <c r="D240" s="6"/>
     </row>
     <row r="241">
-      <c r="A241" s="6"/>
+      <c r="A241" s="21" t="s">
+        <v>449</v>
+      </c>
       <c r="B241" s="6"/>
       <c r="C241" s="6"/>
       <c r="D241" s="6"/>
     </row>
     <row r="242">
-      <c r="A242" s="6"/>
+      <c r="A242" s="21" t="s">
+        <v>450</v>
+      </c>
       <c r="B242" s="6"/>
       <c r="C242" s="6"/>
       <c r="D242" s="6"/>
     </row>
     <row r="243">
-      <c r="A243" s="6"/>
+      <c r="A243" s="21" t="s">
+        <v>451</v>
+      </c>
       <c r="B243" s="6"/>
       <c r="C243" s="6"/>
       <c r="D243" s="6"/>
     </row>
     <row r="244">
-      <c r="A244" s="6"/>
+      <c r="A244" s="21" t="s">
+        <v>452</v>
+      </c>
       <c r="B244" s="6"/>
       <c r="C244" s="6"/>
       <c r="D244" s="6"/>
     </row>
     <row r="245">
-      <c r="A245" s="6"/>
+      <c r="A245" s="21" t="s">
+        <v>453</v>
+      </c>
       <c r="B245" s="6"/>
-      <c r="C245" s="6"/>
-      <c r="D245" s="6"/>
+      <c r="C245" s="12" t="s">
+        <v>454</v>
+      </c>
+      <c r="D245" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="246">
-      <c r="A246" s="6"/>
+      <c r="A246" s="21" t="s">
+        <v>455</v>
+      </c>
       <c r="B246" s="6"/>
-      <c r="C246" s="6"/>
-      <c r="D246" s="6"/>
+      <c r="C246" s="12" t="s">
+        <v>456</v>
+      </c>
+      <c r="D246" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="247">
-      <c r="A247" s="6"/>
+      <c r="A247" s="21" t="s">
+        <v>457</v>
+      </c>
       <c r="B247" s="6"/>
-      <c r="C247" s="6"/>
-      <c r="D247" s="6"/>
+      <c r="C247" s="12" t="s">
+        <v>458</v>
+      </c>
+      <c r="D247" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="248">
-      <c r="A248" s="6"/>
+      <c r="A248" s="21" t="s">
+        <v>459</v>
+      </c>
       <c r="B248" s="6"/>
-      <c r="C248" s="6"/>
-      <c r="D248" s="6"/>
+      <c r="C248" s="12" t="s">
+        <v>460</v>
+      </c>
+      <c r="D248" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="249">
-      <c r="A249" s="6"/>
+      <c r="A249" s="21" t="s">
+        <v>461</v>
+      </c>
       <c r="B249" s="6"/>
-      <c r="C249" s="6"/>
-      <c r="D249" s="6"/>
+      <c r="C249" s="12" t="s">
+        <v>462</v>
+      </c>
+      <c r="D249" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="250">
-      <c r="A250" s="6"/>
+      <c r="A250" s="21" t="s">
+        <v>463</v>
+      </c>
       <c r="B250" s="6"/>
-      <c r="C250" s="6"/>
-      <c r="D250" s="6"/>
+      <c r="C250" s="12" t="s">
+        <v>464</v>
+      </c>
+      <c r="D250" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="251">
-      <c r="A251" s="6"/>
+      <c r="A251" s="21" t="s">
+        <v>465</v>
+      </c>
       <c r="B251" s="6"/>
-      <c r="C251" s="6"/>
-      <c r="D251" s="6"/>
+      <c r="C251" s="12" t="s">
+        <v>466</v>
+      </c>
+      <c r="D251" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="252">
-      <c r="A252" s="6"/>
+      <c r="A252" s="21" t="s">
+        <v>467</v>
+      </c>
       <c r="B252" s="6"/>
-      <c r="C252" s="6"/>
-      <c r="D252" s="6"/>
+      <c r="C252" s="12" t="s">
+        <v>468</v>
+      </c>
+      <c r="D252" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="253">
-      <c r="A253" s="6"/>
+      <c r="A253" s="21" t="s">
+        <v>469</v>
+      </c>
       <c r="B253" s="6"/>
-      <c r="C253" s="6"/>
-      <c r="D253" s="6"/>
+      <c r="C253" s="12" t="s">
+        <v>419</v>
+      </c>
+      <c r="D253" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="254">
-      <c r="A254" s="6"/>
+      <c r="A254" s="21" t="s">
+        <v>470</v>
+      </c>
       <c r="B254" s="6"/>
-      <c r="C254" s="6"/>
-      <c r="D254" s="6"/>
+      <c r="C254" s="12" t="s">
+        <v>471</v>
+      </c>
+      <c r="D254" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="255">
-      <c r="A255" s="6"/>
+      <c r="A255" s="21" t="s">
+        <v>472</v>
+      </c>
       <c r="B255" s="6"/>
-      <c r="C255" s="6"/>
-      <c r="D255" s="6"/>
+      <c r="C255" s="12" t="s">
+        <v>473</v>
+      </c>
+      <c r="D255" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="256">
-      <c r="A256" s="6"/>
+      <c r="A256" s="21" t="s">
+        <v>474</v>
+      </c>
       <c r="B256" s="6"/>
-      <c r="C256" s="6"/>
-      <c r="D256" s="6"/>
+      <c r="C256" s="12" t="s">
+        <v>475</v>
+      </c>
+      <c r="D256" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="257">
-      <c r="A257" s="6"/>
+      <c r="A257" s="21" t="s">
+        <v>476</v>
+      </c>
       <c r="B257" s="6"/>
-      <c r="C257" s="6"/>
-      <c r="D257" s="6"/>
+      <c r="C257" s="12" t="s">
+        <v>477</v>
+      </c>
+      <c r="D257" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="258">
-      <c r="A258" s="6"/>
+      <c r="A258" s="21" t="s">
+        <v>478</v>
+      </c>
       <c r="B258" s="6"/>
-      <c r="C258" s="6"/>
-      <c r="D258" s="6"/>
+      <c r="C258" s="12" t="s">
+        <v>479</v>
+      </c>
+      <c r="D258" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="259">
-      <c r="A259" s="6"/>
+      <c r="A259" s="21" t="s">
+        <v>480</v>
+      </c>
       <c r="B259" s="6"/>
-      <c r="C259" s="6"/>
-      <c r="D259" s="6"/>
+      <c r="C259" s="12" t="s">
+        <v>481</v>
+      </c>
+      <c r="D259" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="260">
-      <c r="A260" s="6"/>
+      <c r="A260" s="21" t="s">
+        <v>482</v>
+      </c>
       <c r="B260" s="6"/>
-      <c r="C260" s="6"/>
-      <c r="D260" s="6"/>
+      <c r="C260" s="12" t="s">
+        <v>473</v>
+      </c>
+      <c r="D260" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="261">
-      <c r="A261" s="6"/>
+      <c r="A261" s="21" t="s">
+        <v>483</v>
+      </c>
       <c r="B261" s="6"/>
-      <c r="C261" s="6"/>
-      <c r="D261" s="6"/>
+      <c r="C261" s="12" t="s">
+        <v>475</v>
+      </c>
+      <c r="D261" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="262">
-      <c r="A262" s="6"/>
+      <c r="A262" s="21" t="s">
+        <v>484</v>
+      </c>
       <c r="B262" s="6"/>
-      <c r="C262" s="6"/>
-      <c r="D262" s="6"/>
+      <c r="C262" s="12" t="s">
+        <v>477</v>
+      </c>
+      <c r="D262" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="263">
-      <c r="A263" s="6"/>
+      <c r="A263" s="21" t="s">
+        <v>485</v>
+      </c>
       <c r="B263" s="6"/>
-      <c r="C263" s="6"/>
-      <c r="D263" s="6"/>
+      <c r="C263" s="12" t="s">
+        <v>479</v>
+      </c>
+      <c r="D263" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="264">
-      <c r="A264" s="6"/>
+      <c r="A264" s="21" t="s">
+        <v>486</v>
+      </c>
       <c r="B264" s="6"/>
       <c r="C264" s="6"/>
       <c r="D264" s="6"/>
     </row>
     <row r="265">
-      <c r="A265" s="6"/>
+      <c r="A265" s="21" t="s">
+        <v>487</v>
+      </c>
       <c r="B265" s="6"/>
       <c r="C265" s="6"/>
       <c r="D265" s="6"/>
     </row>
     <row r="266">
-      <c r="A266" s="6"/>
+      <c r="A266" s="21" t="s">
+        <v>488</v>
+      </c>
       <c r="B266" s="6"/>
-      <c r="C266" s="6"/>
-      <c r="D266" s="6"/>
+      <c r="C266" s="12" t="s">
+        <v>489</v>
+      </c>
+      <c r="D266" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="267">
-      <c r="A267" s="6"/>
+      <c r="A267" s="21" t="s">
+        <v>490</v>
+      </c>
       <c r="B267" s="6"/>
-      <c r="C267" s="6"/>
-      <c r="D267" s="6"/>
+      <c r="C267" s="12" t="s">
+        <v>491</v>
+      </c>
+      <c r="D267" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="268">
-      <c r="A268" s="6"/>
+      <c r="A268" s="21" t="s">
+        <v>492</v>
+      </c>
       <c r="B268" s="6"/>
-      <c r="C268" s="6"/>
-      <c r="D268" s="6"/>
+      <c r="C268" s="12" t="s">
+        <v>493</v>
+      </c>
+      <c r="D268" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="269">
-      <c r="A269" s="6"/>
+      <c r="A269" s="21" t="s">
+        <v>494</v>
+      </c>
       <c r="B269" s="6"/>
       <c r="C269" s="6"/>
       <c r="D269" s="6"/>
     </row>
     <row r="270">
-      <c r="A270" s="6"/>
+      <c r="A270" s="21" t="s">
+        <v>495</v>
+      </c>
       <c r="B270" s="6"/>
       <c r="C270" s="6"/>
       <c r="D270" s="6"/>
     </row>
     <row r="271">
-      <c r="A271" s="6"/>
+      <c r="A271" s="21" t="s">
+        <v>496</v>
+      </c>
       <c r="B271" s="6"/>
       <c r="C271" s="6"/>
       <c r="D271" s="6"/>
     </row>
     <row r="272">
-      <c r="A272" s="6"/>
+      <c r="A272" s="21" t="s">
+        <v>497</v>
+      </c>
       <c r="B272" s="6"/>
       <c r="C272" s="6"/>
       <c r="D272" s="6"/>
     </row>
     <row r="273">
-      <c r="A273" s="6"/>
+      <c r="A273" s="21" t="s">
+        <v>498</v>
+      </c>
       <c r="B273" s="6"/>
       <c r="C273" s="6"/>
       <c r="D273" s="6"/>
     </row>
     <row r="274">
-      <c r="A274" s="6"/>
+      <c r="A274" s="21" t="s">
+        <v>499</v>
+      </c>
       <c r="B274" s="6"/>
       <c r="C274" s="6"/>
       <c r="D274" s="6"/>
     </row>
     <row r="275">
-      <c r="A275" s="6"/>
+      <c r="A275" s="21" t="s">
+        <v>500</v>
+      </c>
       <c r="B275" s="6"/>
       <c r="C275" s="6"/>
       <c r="D275" s="6"/>
     </row>
     <row r="276">
-      <c r="A276" s="6"/>
+      <c r="A276" s="21" t="s">
+        <v>501</v>
+      </c>
       <c r="B276" s="6"/>
       <c r="C276" s="6"/>
       <c r="D276" s="6"/>
     </row>
     <row r="277">
-      <c r="A277" s="6"/>
+      <c r="A277" s="21" t="s">
+        <v>502</v>
+      </c>
       <c r="B277" s="6"/>
       <c r="C277" s="6"/>
       <c r="D277" s="6"/>
     </row>
     <row r="278">
-      <c r="A278" s="6"/>
+      <c r="A278" s="21" t="s">
+        <v>503</v>
+      </c>
       <c r="B278" s="6"/>
       <c r="C278" s="6"/>
       <c r="D278" s="6"/>
     </row>
     <row r="279">
-      <c r="A279" s="6"/>
+      <c r="A279" s="21" t="s">
+        <v>504</v>
+      </c>
       <c r="B279" s="6"/>
       <c r="C279" s="6"/>
       <c r="D279" s="6"/>
     </row>
     <row r="280">
-      <c r="A280" s="6"/>
+      <c r="A280" s="21" t="s">
+        <v>505</v>
+      </c>
       <c r="B280" s="6"/>
       <c r="C280" s="6"/>
       <c r="D280" s="6"/>
     </row>
     <row r="281">
-      <c r="A281" s="6"/>
+      <c r="A281" s="21" t="s">
+        <v>506</v>
+      </c>
       <c r="B281" s="6"/>
-      <c r="C281" s="6"/>
-      <c r="D281" s="6"/>
+      <c r="C281" s="12" t="s">
+        <v>507</v>
+      </c>
+      <c r="D281" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="282">
-      <c r="A282" s="6"/>
+      <c r="A282" s="21" t="s">
+        <v>508</v>
+      </c>
       <c r="B282" s="6"/>
-      <c r="C282" s="6"/>
-      <c r="D282" s="6"/>
+      <c r="C282" s="12" t="s">
+        <v>509</v>
+      </c>
+      <c r="D282" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="6"/>
@@ -9767,15 +10197,58 @@
       <c r="C1102" s="6"/>
       <c r="D1102" s="6"/>
     </row>
+    <row r="1103">
+      <c r="A1103" s="6"/>
+      <c r="B1103" s="6"/>
+      <c r="C1103" s="6"/>
+      <c r="D1103" s="6"/>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="6"/>
+      <c r="B1104" s="6"/>
+      <c r="C1104" s="6"/>
+      <c r="D1104" s="6"/>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="6"/>
+      <c r="B1105" s="6"/>
+      <c r="C1105" s="6"/>
+      <c r="D1105" s="6"/>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="6"/>
+      <c r="B1106" s="6"/>
+      <c r="C1106" s="6"/>
+      <c r="D1106" s="6"/>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="6"/>
+      <c r="B1107" s="6"/>
+      <c r="C1107" s="6"/>
+      <c r="D1107" s="6"/>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="6"/>
+      <c r="B1108" s="6"/>
+      <c r="C1108" s="6"/>
+      <c r="D1108" s="6"/>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="6"/>
+      <c r="B1109" s="6"/>
+      <c r="C1109" s="6"/>
+      <c r="D1109" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D234">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D238 D245:D263 D266:D268 D281:D282">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A167"/>
+    <hyperlink r:id="rId1" ref="A77"/>
+    <hyperlink r:id="rId2" ref="A171"/>
   </hyperlinks>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
WIP creation of an alarm
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="520">
   <si>
     <t>Key</t>
   </si>
@@ -104,6 +104,19 @@
   </si>
   <si>
     <t>Success !</t>
+  </si>
+  <si>
+    <t>setup.pairing.failed.title</t>
+  </si>
+  <si>
+    <t>Pairing Failed</t>
+  </si>
+  <si>
+    <t>setup.pairing.failed.message</t>
+  </si>
+  <si>
+    <t>This ring is currently associated to an already existing Circular account.
+&lt;strong&gt;Unpair it&lt;/strong&gt; from your other account by going into the ‘My Ring’ menu and clicking on the red cross. An email has been sent to the currently associated account.</t>
   </si>
   <si>
     <t>login.title</t>
@@ -399,6 +412,18 @@
   </si>
   <si>
     <t>global.default_error</t>
+  </si>
+  <si>
+    <t>global.yes</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>global.no</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
   <si>
     <t>home.sync.syncing</t>
@@ -673,6 +698,22 @@
     <t>Log out</t>
   </si>
   <si>
+    <t>profile.logout_bottom_sheet.title</t>
+  </si>
+  <si>
+    <t>Please Confirm</t>
+  </si>
+  <si>
+    <t>profile.logout_bottom_sheet.description</t>
+  </si>
+  <si>
+    <t>Are you sure you want to log out from your account?
+Your Circular ring &lt;strong&gt;won’t synch&lt;/strong&gt; to your account during the time that you are offline.</t>
+  </si>
+  <si>
+    <t>profile.logout_bottom_sheet.logout</t>
+  </si>
+  <si>
     <t>profile.global_score.label</t>
   </si>
   <si>
@@ -743,9 +784,6 @@
   </si>
   <si>
     <t>profile_info.bottom_sheet.sex.title</t>
-  </si>
-  <si>
-    <t>Please Confirm</t>
   </si>
   <si>
     <t>profile_info.bottom_sheet.sex.description</t>
@@ -934,6 +972,12 @@
   </si>
   <si>
     <t>Repeat</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.description</t>
+  </si>
+  <si>
+    <t>Choose on what day(s) you want this alarm to go off.</t>
   </si>
   <si>
     <t>onboarding.wear.title</t>
@@ -1200,6 +1244,12 @@
     <t>Snooze</t>
   </si>
   <si>
+    <t>alarm.new.snooze.description</t>
+  </si>
+  <si>
+    <t>Time interval between each snooze. Press the ring’s button once to snooze. Press it twice to completely stop the vibrations.</t>
+  </si>
+  <si>
     <t>alarm.new.snooze.screen_title</t>
   </si>
   <si>
@@ -1236,12 +1286,30 @@
     <t>Smart Snooze</t>
   </si>
   <si>
+    <t>alarm.new.smart_snooze.description</t>
+  </si>
+  <si>
+    <t>Time interval between each snooze. Vibrations will stop automatically once the ring has detected that you’re up and walking.</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.smart_switch</t>
+  </si>
+  <si>
+    <t>Make it smart</t>
+  </si>
+  <si>
     <t>alarm.new.smart_alarm.title</t>
   </si>
   <si>
     <t>Smart Alarm</t>
   </si>
   <si>
+    <t>alarm.new.smart_alarm.description</t>
+  </si>
+  <si>
+    <t>Maximum time window for smart alarm to ring before selected wake up time. More time means more chances to get the lightest wake up.</t>
+  </si>
+  <si>
     <t>alarm.new.warning.title</t>
   </si>
   <si>
@@ -1303,13 +1371,244 @@
   </si>
   <si>
     <t>Discharge</t>
+  </si>
+  <si>
+    <t>header.profile_advanced_information</t>
+  </si>
+  <si>
+    <t>ADVANCED INFORMATION</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.about_you</t>
+  </si>
+  <si>
+    <t>About you</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.lifestyle_info</t>
+  </si>
+  <si>
+    <t>Lifestyle information</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.title</t>
+  </si>
+  <si>
+    <t>Work Time</t>
+  </si>
+  <si>
+    <t>alarm.new.label.placeholder</t>
+  </si>
+  <si>
+    <t>Enter label here</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.day</t>
+  </si>
+  <si>
+    <t>Day Worker</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.night</t>
+  </si>
+  <si>
+    <t>Night Worker</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.morning</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.solar</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.night</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.morning_erratic</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.solar_erratic</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.night_erratic</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.title</t>
+  </si>
+  <si>
+    <t>Physical Disabilities</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.none</t>
+  </si>
+  <si>
+    <t>No physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.moderate</t>
+  </si>
+  <si>
+    <t>Moderate physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.total</t>
+  </si>
+  <si>
+    <t>Total physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.title</t>
+  </si>
+  <si>
+    <t>Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.none</t>
+  </si>
+  <si>
+    <t>No Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.insomnia</t>
+  </si>
+  <si>
+    <t>Insomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.hypersomnia</t>
+  </si>
+  <si>
+    <t>Hypersomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.other</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.title</t>
+  </si>
+  <si>
+    <t>Sleep Aid</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.none</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.daily</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.weekly</t>
+  </si>
+  <si>
+    <t>Weekly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.monthly</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.title</t>
+  </si>
+  <si>
+    <t>Sleep supplements</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.none</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.daily</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.weekly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.monthly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeper_type.light</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeper_type.night</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.menstrual_cycle</t>
+  </si>
+  <si>
+    <t>Menstrual cycle</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.menopause</t>
+  </si>
+  <si>
+    <t>Menopause</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.perimenopause</t>
+  </si>
+  <si>
+    <t>Perimenopause</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.none</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.pills</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.condoms</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.vaginal_ring</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.patch</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.iud</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.implant</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.fertility_awareness</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.other</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_28</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_24</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_21</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.open_for_napping.title</t>
+  </si>
+  <si>
+    <t>Open for Napping</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.unknown_option</t>
+  </si>
+  <si>
+    <t>Unknown option</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1330,9 +1629,17 @@
     </font>
     <font>
       <u/>
+      <color rgb="FF1155CC"/>
+    </font>
+    <font>
+      <u/>
       <color rgb="FF0000FF"/>
     </font>
     <font/>
+    <font>
+      <strike/>
+      <color rgb="FFFF0000"/>
+    </font>
     <font>
       <strike/>
       <color rgb="FFFF0000"/>
@@ -1377,7 +1684,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1411,14 +1718,14 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
@@ -1426,16 +1733,28 @@
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1860,7 +2179,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B16" s="6"/>
@@ -1872,7 +2191,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="9" t="s">
         <v>33</v>
       </c>
       <c r="B17" s="6"/>
@@ -1913,7 +2232,7 @@
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>6</v>
@@ -1921,11 +2240,11 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>6</v>
@@ -1933,11 +2252,11 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>6</v>
@@ -2009,19 +2328,19 @@
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>55</v>
+      <c r="A29" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="7" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>6</v>
@@ -2029,23 +2348,23 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="s">
-        <v>57</v>
+      <c r="A31" s="8" t="s">
+        <v>59</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>6</v>
@@ -2053,11 +2372,11 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="7" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>6</v>
@@ -2065,11 +2384,11 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>6</v>
@@ -2077,7 +2396,7 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
@@ -2089,11 +2408,11 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>6</v>
@@ -2101,11 +2420,11 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>6</v>
@@ -2113,11 +2432,11 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>6</v>
@@ -2125,11 +2444,11 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>6</v>
@@ -2137,11 +2456,11 @@
     </row>
     <row r="39">
       <c r="A39" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="7" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>6</v>
@@ -2149,11 +2468,11 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>6</v>
@@ -2161,11 +2480,11 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>6</v>
@@ -2225,7 +2544,7 @@
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
-        <v>47</v>
+        <v>81</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>6</v>
@@ -2233,11 +2552,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>6</v>
@@ -2245,11 +2564,11 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>6</v>
@@ -2357,7 +2676,7 @@
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
-        <v>36</v>
+        <v>102</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>6</v>
@@ -2365,11 +2684,11 @@
     </row>
     <row r="58">
       <c r="A58" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -2377,11 +2696,11 @@
     </row>
     <row r="59">
       <c r="A59" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B59" s="6"/>
       <c r="C59" s="7" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>6</v>
@@ -2389,11 +2708,11 @@
     </row>
     <row r="60">
       <c r="A60" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>6</v>
@@ -2401,11 +2720,11 @@
     </row>
     <row r="61">
       <c r="A61" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="7" t="s">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>6</v>
@@ -2413,11 +2732,11 @@
     </row>
     <row r="62">
       <c r="A62" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B62" s="6"/>
       <c r="C62" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>6</v>
@@ -2425,11 +2744,11 @@
     </row>
     <row r="63">
       <c r="A63" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="7" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>6</v>
@@ -2484,33 +2803,35 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="10" t="s">
+      <c r="A68" s="5" t="s">
         <v>120</v>
       </c>
+      <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D68" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D68" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="10" t="s">
-        <v>121</v>
-      </c>
+      <c r="A69" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B69" s="6"/>
       <c r="C69" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D69" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="D69" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>124</v>
+        <v>10</v>
       </c>
       <c r="D70" s="10" t="s">
         <v>6</v>
@@ -2532,7 +2853,7 @@
         <v>127</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>12</v>
+        <v>128</v>
       </c>
       <c r="D72" s="10" t="s">
         <v>6</v>
@@ -2540,60 +2861,56 @@
     </row>
     <row r="73">
       <c r="A73" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>47</v>
+        <v>130</v>
       </c>
       <c r="D73" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="B74" s="6"/>
+      <c r="A74" s="10" t="s">
+        <v>131</v>
+      </c>
       <c r="C74" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="D74" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D74" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="B75" s="6"/>
+      <c r="A75" s="10" t="s">
+        <v>132</v>
+      </c>
       <c r="C75" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="D75" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D75" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="5" t="s">
+      <c r="A76" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="B76" s="6"/>
       <c r="C76" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="D76" s="5" t="s">
+      <c r="D76" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="5" t="s">
+      <c r="A77" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="B77" s="6"/>
       <c r="C77" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="D77" s="5" t="s">
+      <c r="D77" s="10" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2694,7 +3011,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="8" t="s">
+      <c r="A86" s="5" t="s">
         <v>153</v>
       </c>
       <c r="B86" s="6"/>
@@ -2706,7 +3023,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="8" t="s">
+      <c r="A87" s="5" t="s">
         <v>155</v>
       </c>
       <c r="B87" s="6"/>
@@ -2742,7 +3059,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="5" t="s">
+      <c r="A90" s="8" t="s">
         <v>161</v>
       </c>
       <c r="B90" s="6"/>
@@ -2754,7 +3071,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="s">
+      <c r="A91" s="8" t="s">
         <v>163</v>
       </c>
       <c r="B91" s="6"/>
@@ -3023,7 +3340,7 @@
       </c>
       <c r="B113" s="6"/>
       <c r="C113" s="7" t="s">
-        <v>36</v>
+        <v>208</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>6</v>
@@ -3031,11 +3348,11 @@
     </row>
     <row r="114">
       <c r="A114" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B114" s="6"/>
       <c r="C114" s="7" t="s">
-        <v>36</v>
+        <v>210</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>6</v>
@@ -3043,11 +3360,11 @@
     </row>
     <row r="115">
       <c r="A115" s="5" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B115" s="6"/>
       <c r="C115" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>6</v>
@@ -3055,11 +3372,11 @@
     </row>
     <row r="116">
       <c r="A116" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="B116" s="5"/>
+        <v>213</v>
+      </c>
+      <c r="B116" s="6"/>
       <c r="C116" s="7" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D116" s="5" t="s">
         <v>6</v>
@@ -3067,11 +3384,11 @@
     </row>
     <row r="117">
       <c r="A117" s="5" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B117" s="6"/>
       <c r="C117" s="7" t="s">
-        <v>214</v>
+        <v>40</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>6</v>
@@ -3079,11 +3396,11 @@
     </row>
     <row r="118">
       <c r="A118" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B118" s="6"/>
       <c r="C118" s="7" t="s">
-        <v>216</v>
+        <v>40</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>6</v>
@@ -3105,7 +3422,7 @@
       <c r="A120" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="B120" s="6"/>
+      <c r="B120" s="5"/>
       <c r="C120" s="7" t="s">
         <v>220</v>
       </c>
@@ -3119,7 +3436,7 @@
       </c>
       <c r="B121" s="6"/>
       <c r="C121" s="7" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>6</v>
@@ -3127,11 +3444,11 @@
     </row>
     <row r="122">
       <c r="A122" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B122" s="6"/>
       <c r="C122" s="7" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>6</v>
@@ -3139,11 +3456,11 @@
     </row>
     <row r="123">
       <c r="A123" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B123" s="6"/>
       <c r="C123" s="7" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>6</v>
@@ -3151,11 +3468,11 @@
     </row>
     <row r="124">
       <c r="A124" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -3203,43 +3520,43 @@
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="s">
         <v>235</v>
-      </c>
-      <c r="D128" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="8" t="s">
-        <v>236</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="s">
         <v>237</v>
-      </c>
-      <c r="D129" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="8" t="s">
-        <v>238</v>
       </c>
       <c r="B130" s="6"/>
       <c r="C130" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="s">
         <v>239</v>
-      </c>
-      <c r="D130" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="8" t="s">
-        <v>240</v>
       </c>
       <c r="B131" s="6"/>
       <c r="C131" s="7" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>6</v>
@@ -3247,11 +3564,11 @@
     </row>
     <row r="132">
       <c r="A132" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B132" s="6"/>
       <c r="C132" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D132" s="5" t="s">
         <v>6</v>
@@ -3259,11 +3576,11 @@
     </row>
     <row r="133">
       <c r="A133" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B133" s="6"/>
       <c r="C133" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>6</v>
@@ -3271,11 +3588,11 @@
     </row>
     <row r="134">
       <c r="A134" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B134" s="6"/>
       <c r="C134" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D134" s="5" t="s">
         <v>6</v>
@@ -3283,47 +3600,47 @@
     </row>
     <row r="135">
       <c r="A135" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B135" s="6"/>
       <c r="C135" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="8" t="s">
         <v>249</v>
       </c>
-      <c r="D135" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="11" t="s">
+      <c r="B136" s="6"/>
+      <c r="C136" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="B136" s="12"/>
-      <c r="C136" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D136" s="11" t="s">
+      <c r="D136" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="5" t="s">
+      <c r="A137" s="8" t="s">
         <v>251</v>
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="D137" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="8" t="s">
         <v>252</v>
-      </c>
-      <c r="D137" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="5" t="s">
-        <v>253</v>
       </c>
       <c r="B138" s="6"/>
       <c r="C138" s="7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>6</v>
@@ -3331,11 +3648,11 @@
     </row>
     <row r="139">
       <c r="A139" s="5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B139" s="6"/>
       <c r="C139" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D139" s="5" t="s">
         <v>6</v>
@@ -3343,11 +3660,11 @@
     </row>
     <row r="140">
       <c r="A140" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B140" s="6"/>
       <c r="C140" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D140" s="5" t="s">
         <v>6</v>
@@ -3355,11 +3672,11 @@
     </row>
     <row r="141">
       <c r="A141" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="7" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D141" s="5" t="s">
         <v>6</v>
@@ -3367,35 +3684,35 @@
     </row>
     <row r="142">
       <c r="A142" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B142" s="6"/>
       <c r="C142" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="D142" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="12" t="s">
         <v>262</v>
       </c>
-      <c r="D142" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="B143" s="6"/>
-      <c r="C143" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="D143" s="5" t="s">
+      <c r="B143" s="13"/>
+      <c r="C143" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D143" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B144" s="6"/>
       <c r="C144" s="7" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D144" s="5" t="s">
         <v>6</v>
@@ -3403,11 +3720,11 @@
     </row>
     <row r="145">
       <c r="A145" s="5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B145" s="6"/>
       <c r="C145" s="7" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D145" s="5" t="s">
         <v>6</v>
@@ -3415,11 +3732,11 @@
     </row>
     <row r="146">
       <c r="A146" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B146" s="6"/>
       <c r="C146" s="7" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D146" s="5" t="s">
         <v>6</v>
@@ -3427,11 +3744,11 @@
     </row>
     <row r="147">
       <c r="A147" s="5" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B147" s="6"/>
       <c r="C147" s="7" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D147" s="5" t="s">
         <v>6</v>
@@ -3439,11 +3756,11 @@
     </row>
     <row r="148">
       <c r="A148" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B148" s="6"/>
       <c r="C148" s="7" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D148" s="5" t="s">
         <v>6</v>
@@ -3451,11 +3768,11 @@
     </row>
     <row r="149">
       <c r="A149" s="5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B149" s="6"/>
       <c r="C149" s="7" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D149" s="5" t="s">
         <v>6</v>
@@ -3463,11 +3780,11 @@
     </row>
     <row r="150">
       <c r="A150" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B150" s="6"/>
       <c r="C150" s="7" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D150" s="5" t="s">
         <v>6</v>
@@ -3475,11 +3792,11 @@
     </row>
     <row r="151">
       <c r="A151" s="5" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B151" s="6"/>
       <c r="C151" s="7" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D151" s="5" t="s">
         <v>6</v>
@@ -3487,47 +3804,47 @@
     </row>
     <row r="152">
       <c r="A152" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B152" s="6"/>
       <c r="C152" s="7" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="D152" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="8" t="s">
-        <v>283</v>
+      <c r="A153" s="5" t="s">
+        <v>281</v>
       </c>
       <c r="B153" s="6"/>
       <c r="C153" s="7" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D153" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="8" t="s">
-        <v>285</v>
+      <c r="A154" s="5" t="s">
+        <v>283</v>
       </c>
       <c r="B154" s="6"/>
       <c r="C154" s="7" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D154" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="8" t="s">
-        <v>287</v>
+      <c r="A155" s="5" t="s">
+        <v>285</v>
       </c>
       <c r="B155" s="6"/>
       <c r="C155" s="7" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D155" s="5" t="s">
         <v>6</v>
@@ -3535,11 +3852,11 @@
     </row>
     <row r="156">
       <c r="A156" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B156" s="6"/>
       <c r="C156" s="7" t="s">
-        <v>218</v>
+        <v>288</v>
       </c>
       <c r="D156" s="5" t="s">
         <v>6</v>
@@ -3547,11 +3864,11 @@
     </row>
     <row r="157">
       <c r="A157" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B157" s="6"/>
       <c r="C157" s="7" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D157" s="5" t="s">
         <v>6</v>
@@ -3559,11 +3876,11 @@
     </row>
     <row r="158">
       <c r="A158" s="5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B158" s="6"/>
       <c r="C158" s="7" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D158" s="5" t="s">
         <v>6</v>
@@ -3571,47 +3888,47 @@
     </row>
     <row r="159">
       <c r="A159" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="D159" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="8" t="s">
         <v>295</v>
-      </c>
-      <c r="D159" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="5" t="s">
-        <v>296</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="D160" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="8" t="s">
         <v>297</v>
-      </c>
-      <c r="D160" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="5" t="s">
-        <v>298</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="D161" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="8" t="s">
         <v>299</v>
-      </c>
-      <c r="D161" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="5" t="s">
-        <v>300</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="7" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>6</v>
@@ -3619,23 +3936,23 @@
     </row>
     <row r="163">
       <c r="A163" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>303</v>
+        <v>231</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="13" t="s">
-        <v>304</v>
+      <c r="A164" s="5" t="s">
+        <v>302</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
@@ -3643,11 +3960,11 @@
     </row>
     <row r="165">
       <c r="A165" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="7" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D165" s="5" t="s">
         <v>6</v>
@@ -3655,11 +3972,11 @@
     </row>
     <row r="166">
       <c r="A166" s="5" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="7" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D166" s="5" t="s">
         <v>6</v>
@@ -3667,11 +3984,11 @@
     </row>
     <row r="167">
       <c r="A167" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="7" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D167" s="5" t="s">
         <v>6</v>
@@ -3679,23 +3996,23 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="8" t="s">
-        <v>314</v>
+      <c r="A169" s="5" t="s">
+        <v>312</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="7" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D169" s="5" t="s">
         <v>6</v>
@@ -3703,11 +4020,11 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="7" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D170" s="5" t="s">
         <v>6</v>
@@ -3715,23 +4032,23 @@
     </row>
     <row r="171">
       <c r="A171" s="5" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="7" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D171" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="5" t="s">
-        <v>320</v>
+      <c r="A172" s="14" t="s">
+        <v>318</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="7" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D172" s="5" t="s">
         <v>6</v>
@@ -3739,11 +4056,11 @@
     </row>
     <row r="173">
       <c r="A173" s="5" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="7" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D173" s="5" t="s">
         <v>6</v>
@@ -3751,11 +4068,11 @@
     </row>
     <row r="174">
       <c r="A174" s="5" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
@@ -3763,11 +4080,11 @@
     </row>
     <row r="175">
       <c r="A175" s="5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
@@ -3775,23 +4092,23 @@
     </row>
     <row r="176">
       <c r="A176" s="5" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="5" t="s">
-        <v>330</v>
+      <c r="A177" s="8" t="s">
+        <v>328</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
@@ -3799,11 +4116,11 @@
     </row>
     <row r="178">
       <c r="A178" s="5" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
@@ -3811,11 +4128,11 @@
     </row>
     <row r="179">
       <c r="A179" s="5" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
@@ -3823,11 +4140,11 @@
     </row>
     <row r="180">
       <c r="A180" s="5" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
@@ -3835,11 +4152,11 @@
     </row>
     <row r="181">
       <c r="A181" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
@@ -3847,11 +4164,11 @@
     </row>
     <row r="182">
       <c r="A182" s="5" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="7" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>6</v>
@@ -3859,11 +4176,11 @@
     </row>
     <row r="183">
       <c r="A183" s="5" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="7" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>6</v>
@@ -3871,11 +4188,11 @@
     </row>
     <row r="184">
       <c r="A184" s="5" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="7" t="s">
-        <v>47</v>
+        <v>343</v>
       </c>
       <c r="D184" s="5" t="s">
         <v>6</v>
@@ -3883,11 +4200,11 @@
     </row>
     <row r="185">
       <c r="A185" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="7" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D185" s="5" t="s">
         <v>6</v>
@@ -3895,95 +4212,95 @@
     </row>
     <row r="186">
       <c r="A186" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="D186" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="s">
         <v>348</v>
-      </c>
-      <c r="D186" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="14" t="s">
-        <v>349</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="D187" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="5" t="s">
         <v>350</v>
-      </c>
-      <c r="D187" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="10" t="s">
-        <v>351</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="D188" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="D188" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" s="10" t="s">
-        <v>353</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="D189" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="5" t="s">
         <v>354</v>
-      </c>
-      <c r="D189" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="10" t="s">
-        <v>355</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="D190" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="s">
         <v>356</v>
-      </c>
-      <c r="D190" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" s="10" t="s">
-        <v>357</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="D191" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="5" t="s">
         <v>358</v>
-      </c>
-      <c r="D191" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="10" t="s">
-        <v>359</v>
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
-        <v>360</v>
+        <v>51</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="10" t="s">
-        <v>361</v>
+      <c r="A193" s="5" t="s">
+        <v>359</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
@@ -3991,11 +4308,11 @@
     </row>
     <row r="194">
       <c r="A194" s="5" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B194" s="6"/>
       <c r="C194" s="7" t="s">
-        <v>126</v>
+        <v>362</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>6</v>
@@ -4003,83 +4320,83 @@
     </row>
     <row r="195">
       <c r="A195" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B195" s="6"/>
       <c r="C195" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="D195" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="10" t="s">
         <v>365</v>
-      </c>
-      <c r="D195" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" s="5" t="s">
-        <v>366</v>
       </c>
       <c r="B196" s="6"/>
       <c r="C196" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="D196" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="10" t="s">
         <v>367</v>
-      </c>
-      <c r="D196" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" s="5" t="s">
-        <v>368</v>
       </c>
       <c r="B197" s="6"/>
       <c r="C197" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="D197" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="10" t="s">
         <v>369</v>
-      </c>
-      <c r="D197" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" s="5" t="s">
-        <v>370</v>
       </c>
       <c r="B198" s="6"/>
       <c r="C198" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="D198" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="10" t="s">
         <v>371</v>
-      </c>
-      <c r="D198" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" s="5" t="s">
-        <v>372</v>
       </c>
       <c r="B199" s="6"/>
       <c r="C199" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="D199" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="10" t="s">
         <v>373</v>
-      </c>
-      <c r="D199" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" s="5" t="s">
-        <v>374</v>
       </c>
       <c r="B200" s="6"/>
       <c r="C200" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="D200" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="10" t="s">
         <v>375</v>
-      </c>
-      <c r="D200" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" s="5" t="s">
-        <v>376</v>
       </c>
       <c r="B201" s="6"/>
       <c r="C201" s="7" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D201" s="5" t="s">
         <v>6</v>
@@ -4087,11 +4404,11 @@
     </row>
     <row r="202">
       <c r="A202" s="5" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B202" s="6"/>
       <c r="C202" s="7" t="s">
-        <v>379</v>
+        <v>130</v>
       </c>
       <c r="D202" s="5" t="s">
         <v>6</v>
@@ -4099,11 +4416,11 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B203" s="6"/>
       <c r="C203" s="7" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D203" s="5" t="s">
         <v>6</v>
@@ -4111,11 +4428,11 @@
     </row>
     <row r="204">
       <c r="A204" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B204" s="6"/>
       <c r="C204" s="7" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D204" s="5" t="s">
         <v>6</v>
@@ -4123,11 +4440,11 @@
     </row>
     <row r="205">
       <c r="A205" s="5" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B205" s="6"/>
       <c r="C205" s="7" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D205" s="5" t="s">
         <v>6</v>
@@ -4135,11 +4452,11 @@
     </row>
     <row r="206">
       <c r="A206" s="5" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B206" s="6"/>
       <c r="C206" s="7" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D206" s="5" t="s">
         <v>6</v>
@@ -4147,11 +4464,11 @@
     </row>
     <row r="207">
       <c r="A207" s="5" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B207" s="6"/>
       <c r="C207" s="7" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D207" s="5" t="s">
         <v>6</v>
@@ -4159,11 +4476,11 @@
     </row>
     <row r="208">
       <c r="A208" s="5" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B208" s="6"/>
       <c r="C208" s="7" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D208" s="5" t="s">
         <v>6</v>
@@ -4171,11 +4488,11 @@
     </row>
     <row r="209">
       <c r="A209" s="5" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B209" s="6"/>
       <c r="C209" s="7" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="D209" s="5" t="s">
         <v>6</v>
@@ -4183,11 +4500,11 @@
     </row>
     <row r="210">
       <c r="A210" s="5" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B210" s="6"/>
       <c r="C210" s="7" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D210" s="5" t="s">
         <v>6</v>
@@ -4195,11 +4512,11 @@
     </row>
     <row r="211">
       <c r="A211" s="5" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B211" s="6"/>
       <c r="C211" s="7" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D211" s="5" t="s">
         <v>6</v>
@@ -4207,11 +4524,11 @@
     </row>
     <row r="212">
       <c r="A212" s="5" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B212" s="6"/>
       <c r="C212" s="7" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D212" s="5" t="s">
         <v>6</v>
@@ -4219,47 +4536,47 @@
     </row>
     <row r="213">
       <c r="A213" s="5" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B213" s="6"/>
       <c r="C213" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="D213" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="15" t="s">
+        <v>400</v>
+      </c>
+      <c r="B214" s="6"/>
+      <c r="C214" s="16" t="s">
         <v>401</v>
       </c>
-      <c r="D213" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" s="5" t="s">
+      <c r="D214" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="17" t="s">
         <v>402</v>
       </c>
-      <c r="B214" s="6"/>
-      <c r="C214" s="7" t="s">
+      <c r="B215" s="18"/>
+      <c r="C215" s="19" t="s">
         <v>403</v>
       </c>
-      <c r="D214" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" s="5" t="s">
-        <v>404</v>
-      </c>
-      <c r="B215" s="6"/>
-      <c r="C215" s="7" t="s">
-        <v>405</v>
-      </c>
-      <c r="D215" s="5" t="s">
+      <c r="D215" s="20" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="5" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B216" s="6"/>
       <c r="C216" s="7" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="D216" s="5" t="s">
         <v>6</v>
@@ -4267,11 +4584,11 @@
     </row>
     <row r="217">
       <c r="A217" s="5" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B217" s="6"/>
       <c r="C217" s="7" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="D217" s="5" t="s">
         <v>6</v>
@@ -4279,11 +4596,11 @@
     </row>
     <row r="218">
       <c r="A218" s="5" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B218" s="6"/>
       <c r="C218" s="7" t="s">
-        <v>160</v>
+        <v>409</v>
       </c>
       <c r="D218" s="5" t="s">
         <v>6</v>
@@ -4291,11 +4608,11 @@
     </row>
     <row r="219">
       <c r="A219" s="5" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B219" s="6"/>
       <c r="C219" s="7" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D219" s="5" t="s">
         <v>6</v>
@@ -4303,22 +4620,22 @@
     </row>
     <row r="220">
       <c r="A220" s="5" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B220" s="6"/>
       <c r="C220" s="7" t="s">
-        <v>295</v>
+        <v>413</v>
       </c>
       <c r="D220" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="5" t="s">
+      <c r="A221" s="15" t="s">
         <v>414</v>
       </c>
       <c r="B221" s="6"/>
-      <c r="C221" s="7" t="s">
+      <c r="C221" s="16" t="s">
         <v>415</v>
       </c>
       <c r="D221" s="5" t="s">
@@ -4326,11 +4643,11 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="5" t="s">
+      <c r="A222" s="15" t="s">
         <v>416</v>
       </c>
       <c r="B222" s="6"/>
-      <c r="C222" s="7" t="s">
+      <c r="C222" s="16" t="s">
         <v>417</v>
       </c>
       <c r="D222" s="5" t="s">
@@ -4338,428 +4655,727 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="15" t="s">
+      <c r="A223" s="5" t="s">
         <v>418</v>
       </c>
-      <c r="B223" s="16"/>
-      <c r="C223" s="17" t="s">
-        <v>218</v>
-      </c>
-      <c r="D223" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E223" s="18"/>
-      <c r="F223" s="18"/>
-      <c r="G223" s="18"/>
-      <c r="H223" s="18"/>
-      <c r="I223" s="18"/>
-      <c r="J223" s="18"/>
-      <c r="K223" s="18"/>
-      <c r="L223" s="18"/>
-      <c r="M223" s="18"/>
-      <c r="N223" s="18"/>
-      <c r="O223" s="18"/>
-      <c r="P223" s="18"/>
-      <c r="Q223" s="18"/>
-      <c r="R223" s="18"/>
-      <c r="S223" s="18"/>
-      <c r="T223" s="18"/>
-      <c r="U223" s="18"/>
-      <c r="V223" s="18"/>
-      <c r="W223" s="18"/>
-      <c r="X223" s="18"/>
-      <c r="Y223" s="18"/>
-      <c r="Z223" s="18"/>
+      <c r="B223" s="6"/>
+      <c r="C223" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="D223" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="224">
-      <c r="A224" s="14" t="s">
-        <v>419</v>
+      <c r="A224" s="15" t="s">
+        <v>420</v>
       </c>
       <c r="B224" s="6"/>
-      <c r="C224" s="19" t="s">
-        <v>420</v>
+      <c r="C224" s="16" t="s">
+        <v>421</v>
       </c>
       <c r="D224" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="6"/>
+      <c r="A225" s="5" t="s">
+        <v>422</v>
+      </c>
       <c r="B225" s="6"/>
-      <c r="C225" s="6"/>
-      <c r="D225" s="6"/>
+      <c r="C225" s="7" t="s">
+        <v>423</v>
+      </c>
+      <c r="D225" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="226">
-      <c r="A226" s="6"/>
+      <c r="A226" s="5" t="s">
+        <v>424</v>
+      </c>
       <c r="B226" s="6"/>
-      <c r="C226" s="6"/>
-      <c r="D226" s="6"/>
+      <c r="C226" s="7" t="s">
+        <v>425</v>
+      </c>
+      <c r="D226" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="227">
-      <c r="A227" s="6"/>
+      <c r="A227" s="5" t="s">
+        <v>426</v>
+      </c>
       <c r="B227" s="6"/>
-      <c r="C227" s="6"/>
-      <c r="D227" s="6"/>
+      <c r="C227" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="D227" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="228">
-      <c r="A228" s="6"/>
+      <c r="A228" s="5" t="s">
+        <v>428</v>
+      </c>
       <c r="B228" s="6"/>
-      <c r="C228" s="6"/>
-      <c r="D228" s="6"/>
+      <c r="C228" s="7" t="s">
+        <v>429</v>
+      </c>
+      <c r="D228" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="229">
-      <c r="A229" s="6"/>
+      <c r="A229" s="5" t="s">
+        <v>430</v>
+      </c>
       <c r="B229" s="6"/>
-      <c r="C229" s="6"/>
-      <c r="D229" s="6"/>
+      <c r="C229" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="D229" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="230">
-      <c r="A230" s="6"/>
+      <c r="A230" s="5" t="s">
+        <v>432</v>
+      </c>
       <c r="B230" s="6"/>
-      <c r="C230" s="6"/>
-      <c r="D230" s="6"/>
+      <c r="C230" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="D230" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="231">
-      <c r="A231" s="6"/>
+      <c r="A231" s="5" t="s">
+        <v>433</v>
+      </c>
       <c r="B231" s="6"/>
-      <c r="C231" s="6"/>
-      <c r="D231" s="6"/>
+      <c r="C231" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="D231" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="232">
-      <c r="A232" s="6"/>
+      <c r="A232" s="5" t="s">
+        <v>435</v>
+      </c>
       <c r="B232" s="6"/>
-      <c r="C232" s="6"/>
-      <c r="D232" s="6"/>
+      <c r="C232" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="D232" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="233">
-      <c r="A233" s="6"/>
+      <c r="A233" s="5" t="s">
+        <v>436</v>
+      </c>
       <c r="B233" s="6"/>
-      <c r="C233" s="6"/>
-      <c r="D233" s="6"/>
+      <c r="C233" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="D233" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="234">
-      <c r="A234" s="6"/>
+      <c r="A234" s="5" t="s">
+        <v>438</v>
+      </c>
       <c r="B234" s="6"/>
-      <c r="C234" s="6"/>
-      <c r="D234" s="6"/>
+      <c r="C234" s="7" t="s">
+        <v>439</v>
+      </c>
+      <c r="D234" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="235">
-      <c r="A235" s="6"/>
-      <c r="B235" s="6"/>
-      <c r="C235" s="6"/>
-      <c r="D235" s="6"/>
+      <c r="A235" s="20" t="s">
+        <v>440</v>
+      </c>
+      <c r="B235" s="21"/>
+      <c r="C235" s="22" t="s">
+        <v>231</v>
+      </c>
+      <c r="D235" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E235" s="23"/>
+      <c r="F235" s="23"/>
+      <c r="G235" s="23"/>
+      <c r="H235" s="23"/>
+      <c r="I235" s="23"/>
+      <c r="J235" s="23"/>
+      <c r="K235" s="23"/>
+      <c r="L235" s="23"/>
+      <c r="M235" s="23"/>
+      <c r="N235" s="23"/>
+      <c r="O235" s="23"/>
+      <c r="P235" s="23"/>
+      <c r="Q235" s="23"/>
+      <c r="R235" s="23"/>
+      <c r="S235" s="23"/>
+      <c r="T235" s="23"/>
+      <c r="U235" s="23"/>
+      <c r="V235" s="23"/>
+      <c r="W235" s="23"/>
+      <c r="X235" s="23"/>
+      <c r="Y235" s="23"/>
+      <c r="Z235" s="23"/>
     </row>
     <row r="236">
-      <c r="A236" s="6"/>
+      <c r="A236" s="5" t="s">
+        <v>441</v>
+      </c>
       <c r="B236" s="6"/>
-      <c r="C236" s="6"/>
-      <c r="D236" s="6"/>
+      <c r="C236" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="D236" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="237">
-      <c r="A237" s="6"/>
+      <c r="A237" s="5" t="s">
+        <v>443</v>
+      </c>
       <c r="B237" s="6"/>
-      <c r="C237" s="6"/>
-      <c r="D237" s="6"/>
+      <c r="C237" s="7" t="s">
+        <v>444</v>
+      </c>
+      <c r="D237" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="238">
-      <c r="A238" s="6"/>
+      <c r="A238" s="5" t="s">
+        <v>445</v>
+      </c>
       <c r="B238" s="6"/>
-      <c r="C238" s="6"/>
-      <c r="D238" s="6"/>
+      <c r="C238" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="D238" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="239">
-      <c r="A239" s="6"/>
+      <c r="A239" s="5" t="s">
+        <v>447</v>
+      </c>
       <c r="B239" s="6"/>
-      <c r="C239" s="6"/>
-      <c r="D239" s="6"/>
+      <c r="C239" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="D239" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="240">
-      <c r="A240" s="6"/>
+      <c r="A240" s="5" t="s">
+        <v>449</v>
+      </c>
       <c r="B240" s="6"/>
-      <c r="C240" s="6"/>
-      <c r="D240" s="6"/>
+      <c r="C240" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="D240" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="241">
-      <c r="A241" s="6"/>
-      <c r="B241" s="6"/>
-      <c r="C241" s="6"/>
-      <c r="D241" s="6"/>
+      <c r="A241" s="20" t="s">
+        <v>451</v>
+      </c>
+      <c r="B241" s="21"/>
+      <c r="C241" s="22" t="s">
+        <v>452</v>
+      </c>
+      <c r="D241" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E241" s="23"/>
     </row>
     <row r="242">
-      <c r="A242" s="6"/>
+      <c r="A242" s="5" t="s">
+        <v>453</v>
+      </c>
       <c r="B242" s="6"/>
-      <c r="C242" s="6"/>
-      <c r="D242" s="6"/>
+      <c r="C242" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="D242" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="243">
-      <c r="A243" s="6"/>
+      <c r="A243" s="5" t="s">
+        <v>455</v>
+      </c>
       <c r="B243" s="6"/>
-      <c r="C243" s="6"/>
-      <c r="D243" s="6"/>
+      <c r="C243" s="7" t="s">
+        <v>456</v>
+      </c>
+      <c r="D243" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="244">
-      <c r="A244" s="6"/>
+      <c r="A244" s="5" t="s">
+        <v>457</v>
+      </c>
       <c r="B244" s="6"/>
       <c r="C244" s="6"/>
       <c r="D244" s="6"/>
     </row>
     <row r="245">
-      <c r="A245" s="6"/>
+      <c r="A245" s="5" t="s">
+        <v>458</v>
+      </c>
       <c r="B245" s="6"/>
       <c r="C245" s="6"/>
       <c r="D245" s="6"/>
     </row>
     <row r="246">
-      <c r="A246" s="6"/>
+      <c r="A246" s="5" t="s">
+        <v>459</v>
+      </c>
       <c r="B246" s="6"/>
       <c r="C246" s="6"/>
       <c r="D246" s="6"/>
     </row>
     <row r="247">
-      <c r="A247" s="6"/>
+      <c r="A247" s="5" t="s">
+        <v>460</v>
+      </c>
       <c r="B247" s="6"/>
       <c r="C247" s="6"/>
       <c r="D247" s="6"/>
     </row>
     <row r="248">
-      <c r="A248" s="6"/>
+      <c r="A248" s="5" t="s">
+        <v>461</v>
+      </c>
       <c r="B248" s="6"/>
       <c r="C248" s="6"/>
       <c r="D248" s="6"/>
     </row>
     <row r="249">
-      <c r="A249" s="6"/>
+      <c r="A249" s="5" t="s">
+        <v>462</v>
+      </c>
       <c r="B249" s="6"/>
       <c r="C249" s="6"/>
       <c r="D249" s="6"/>
     </row>
     <row r="250">
-      <c r="A250" s="6"/>
+      <c r="A250" s="5" t="s">
+        <v>463</v>
+      </c>
       <c r="B250" s="6"/>
-      <c r="C250" s="6"/>
-      <c r="D250" s="6"/>
+      <c r="C250" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="D250" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="251">
-      <c r="A251" s="6"/>
+      <c r="A251" s="5" t="s">
+        <v>465</v>
+      </c>
       <c r="B251" s="6"/>
-      <c r="C251" s="6"/>
-      <c r="D251" s="6"/>
+      <c r="C251" s="7" t="s">
+        <v>466</v>
+      </c>
+      <c r="D251" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="252">
-      <c r="A252" s="6"/>
+      <c r="A252" s="5" t="s">
+        <v>467</v>
+      </c>
       <c r="B252" s="6"/>
-      <c r="C252" s="6"/>
-      <c r="D252" s="6"/>
+      <c r="C252" s="7" t="s">
+        <v>468</v>
+      </c>
+      <c r="D252" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="253">
-      <c r="A253" s="6"/>
+      <c r="A253" s="5" t="s">
+        <v>469</v>
+      </c>
       <c r="B253" s="6"/>
-      <c r="C253" s="6"/>
-      <c r="D253" s="6"/>
+      <c r="C253" s="7" t="s">
+        <v>470</v>
+      </c>
+      <c r="D253" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="254">
-      <c r="A254" s="6"/>
+      <c r="A254" s="5" t="s">
+        <v>471</v>
+      </c>
       <c r="B254" s="6"/>
-      <c r="C254" s="6"/>
-      <c r="D254" s="6"/>
+      <c r="C254" s="7" t="s">
+        <v>472</v>
+      </c>
+      <c r="D254" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="255">
-      <c r="A255" s="6"/>
+      <c r="A255" s="5" t="s">
+        <v>473</v>
+      </c>
       <c r="B255" s="6"/>
-      <c r="C255" s="6"/>
-      <c r="D255" s="6"/>
+      <c r="C255" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="D255" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="256">
-      <c r="A256" s="6"/>
+      <c r="A256" s="5" t="s">
+        <v>475</v>
+      </c>
       <c r="B256" s="6"/>
-      <c r="C256" s="6"/>
-      <c r="D256" s="6"/>
+      <c r="C256" s="7" t="s">
+        <v>476</v>
+      </c>
+      <c r="D256" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="257">
-      <c r="A257" s="6"/>
+      <c r="A257" s="5" t="s">
+        <v>477</v>
+      </c>
       <c r="B257" s="6"/>
-      <c r="C257" s="6"/>
-      <c r="D257" s="6"/>
+      <c r="C257" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="D257" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="258">
-      <c r="A258" s="6"/>
+      <c r="A258" s="5" t="s">
+        <v>479</v>
+      </c>
       <c r="B258" s="6"/>
-      <c r="C258" s="6"/>
-      <c r="D258" s="6"/>
+      <c r="C258" s="7" t="s">
+        <v>429</v>
+      </c>
+      <c r="D258" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="259">
-      <c r="A259" s="6"/>
+      <c r="A259" s="5" t="s">
+        <v>480</v>
+      </c>
       <c r="B259" s="6"/>
-      <c r="C259" s="6"/>
-      <c r="D259" s="6"/>
+      <c r="C259" s="7" t="s">
+        <v>481</v>
+      </c>
+      <c r="D259" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="260">
-      <c r="A260" s="6"/>
+      <c r="A260" s="5" t="s">
+        <v>482</v>
+      </c>
       <c r="B260" s="6"/>
-      <c r="C260" s="6"/>
-      <c r="D260" s="6"/>
+      <c r="C260" s="7" t="s">
+        <v>483</v>
+      </c>
+      <c r="D260" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="261">
-      <c r="A261" s="6"/>
+      <c r="A261" s="5" t="s">
+        <v>484</v>
+      </c>
       <c r="B261" s="6"/>
-      <c r="C261" s="6"/>
-      <c r="D261" s="6"/>
+      <c r="C261" s="7" t="s">
+        <v>485</v>
+      </c>
+      <c r="D261" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="262">
-      <c r="A262" s="6"/>
+      <c r="A262" s="5" t="s">
+        <v>486</v>
+      </c>
       <c r="B262" s="6"/>
-      <c r="C262" s="6"/>
-      <c r="D262" s="6"/>
+      <c r="C262" s="7" t="s">
+        <v>487</v>
+      </c>
+      <c r="D262" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="263">
-      <c r="A263" s="6"/>
+      <c r="A263" s="5" t="s">
+        <v>488</v>
+      </c>
       <c r="B263" s="6"/>
-      <c r="C263" s="6"/>
-      <c r="D263" s="6"/>
+      <c r="C263" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="D263" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="264">
-      <c r="A264" s="6"/>
+      <c r="A264" s="5" t="s">
+        <v>490</v>
+      </c>
       <c r="B264" s="6"/>
-      <c r="C264" s="6"/>
-      <c r="D264" s="6"/>
+      <c r="C264" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="D264" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="265">
-      <c r="A265" s="6"/>
+      <c r="A265" s="5" t="s">
+        <v>492</v>
+      </c>
       <c r="B265" s="6"/>
-      <c r="C265" s="6"/>
-      <c r="D265" s="6"/>
+      <c r="C265" s="7" t="s">
+        <v>483</v>
+      </c>
+      <c r="D265" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="266">
-      <c r="A266" s="6"/>
+      <c r="A266" s="5" t="s">
+        <v>493</v>
+      </c>
       <c r="B266" s="6"/>
-      <c r="C266" s="6"/>
-      <c r="D266" s="6"/>
+      <c r="C266" s="7" t="s">
+        <v>485</v>
+      </c>
+      <c r="D266" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="267">
-      <c r="A267" s="6"/>
+      <c r="A267" s="5" t="s">
+        <v>494</v>
+      </c>
       <c r="B267" s="6"/>
-      <c r="C267" s="6"/>
-      <c r="D267" s="6"/>
+      <c r="C267" s="7" t="s">
+        <v>487</v>
+      </c>
+      <c r="D267" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="268">
-      <c r="A268" s="6"/>
+      <c r="A268" s="5" t="s">
+        <v>495</v>
+      </c>
       <c r="B268" s="6"/>
-      <c r="C268" s="6"/>
-      <c r="D268" s="6"/>
+      <c r="C268" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="D268" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="269">
-      <c r="A269" s="6"/>
+      <c r="A269" s="5" t="s">
+        <v>496</v>
+      </c>
       <c r="B269" s="6"/>
       <c r="C269" s="6"/>
       <c r="D269" s="6"/>
     </row>
     <row r="270">
-      <c r="A270" s="6"/>
+      <c r="A270" s="5" t="s">
+        <v>497</v>
+      </c>
       <c r="B270" s="6"/>
       <c r="C270" s="6"/>
       <c r="D270" s="6"/>
     </row>
     <row r="271">
-      <c r="A271" s="6"/>
+      <c r="A271" s="5" t="s">
+        <v>498</v>
+      </c>
       <c r="B271" s="6"/>
-      <c r="C271" s="6"/>
-      <c r="D271" s="6"/>
+      <c r="C271" s="7" t="s">
+        <v>499</v>
+      </c>
+      <c r="D271" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="272">
-      <c r="A272" s="6"/>
+      <c r="A272" s="5" t="s">
+        <v>500</v>
+      </c>
       <c r="B272" s="6"/>
-      <c r="C272" s="6"/>
-      <c r="D272" s="6"/>
+      <c r="C272" s="7" t="s">
+        <v>501</v>
+      </c>
+      <c r="D272" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="273">
-      <c r="A273" s="6"/>
+      <c r="A273" s="5" t="s">
+        <v>502</v>
+      </c>
       <c r="B273" s="6"/>
-      <c r="C273" s="6"/>
-      <c r="D273" s="6"/>
+      <c r="C273" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="D273" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="274">
-      <c r="A274" s="6"/>
+      <c r="A274" s="5" t="s">
+        <v>504</v>
+      </c>
       <c r="B274" s="6"/>
       <c r="C274" s="6"/>
       <c r="D274" s="6"/>
     </row>
     <row r="275">
-      <c r="A275" s="6"/>
+      <c r="A275" s="5" t="s">
+        <v>505</v>
+      </c>
       <c r="B275" s="6"/>
       <c r="C275" s="6"/>
       <c r="D275" s="6"/>
     </row>
     <row r="276">
-      <c r="A276" s="6"/>
+      <c r="A276" s="5" t="s">
+        <v>506</v>
+      </c>
       <c r="B276" s="6"/>
       <c r="C276" s="6"/>
       <c r="D276" s="6"/>
     </row>
     <row r="277">
-      <c r="A277" s="6"/>
+      <c r="A277" s="5" t="s">
+        <v>507</v>
+      </c>
       <c r="B277" s="6"/>
       <c r="C277" s="6"/>
       <c r="D277" s="6"/>
     </row>
     <row r="278">
-      <c r="A278" s="6"/>
+      <c r="A278" s="5" t="s">
+        <v>508</v>
+      </c>
       <c r="B278" s="6"/>
       <c r="C278" s="6"/>
       <c r="D278" s="6"/>
     </row>
     <row r="279">
-      <c r="A279" s="6"/>
+      <c r="A279" s="5" t="s">
+        <v>509</v>
+      </c>
       <c r="B279" s="6"/>
       <c r="C279" s="6"/>
       <c r="D279" s="6"/>
     </row>
     <row r="280">
-      <c r="A280" s="6"/>
+      <c r="A280" s="5" t="s">
+        <v>510</v>
+      </c>
       <c r="B280" s="6"/>
       <c r="C280" s="6"/>
       <c r="D280" s="6"/>
     </row>
     <row r="281">
-      <c r="A281" s="6"/>
+      <c r="A281" s="5" t="s">
+        <v>511</v>
+      </c>
       <c r="B281" s="6"/>
       <c r="C281" s="6"/>
       <c r="D281" s="6"/>
     </row>
     <row r="282">
-      <c r="A282" s="6"/>
+      <c r="A282" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="B282" s="6"/>
       <c r="C282" s="6"/>
       <c r="D282" s="6"/>
     </row>
     <row r="283">
-      <c r="A283" s="6"/>
+      <c r="A283" s="5" t="s">
+        <v>513</v>
+      </c>
       <c r="B283" s="6"/>
       <c r="C283" s="6"/>
       <c r="D283" s="6"/>
     </row>
     <row r="284">
-      <c r="A284" s="6"/>
+      <c r="A284" s="5" t="s">
+        <v>514</v>
+      </c>
       <c r="B284" s="6"/>
       <c r="C284" s="6"/>
       <c r="D284" s="6"/>
     </row>
     <row r="285">
-      <c r="A285" s="6"/>
+      <c r="A285" s="5" t="s">
+        <v>515</v>
+      </c>
       <c r="B285" s="6"/>
       <c r="C285" s="6"/>
       <c r="D285" s="6"/>
     </row>
     <row r="286">
-      <c r="A286" s="6"/>
+      <c r="A286" s="5" t="s">
+        <v>516</v>
+      </c>
       <c r="B286" s="6"/>
-      <c r="C286" s="6"/>
-      <c r="D286" s="6"/>
+      <c r="C286" s="7" t="s">
+        <v>517</v>
+      </c>
+      <c r="D286" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="287">
-      <c r="A287" s="6"/>
+      <c r="A287" s="5" t="s">
+        <v>518</v>
+      </c>
       <c r="B287" s="6"/>
-      <c r="C287" s="6"/>
-      <c r="D287" s="6"/>
+      <c r="C287" s="7" t="s">
+        <v>519</v>
+      </c>
+      <c r="D287" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="6"/>
@@ -9633,15 +10249,106 @@
       <c r="C1099" s="6"/>
       <c r="D1099" s="6"/>
     </row>
+    <row r="1100">
+      <c r="A1100" s="6"/>
+      <c r="B1100" s="6"/>
+      <c r="C1100" s="6"/>
+      <c r="D1100" s="6"/>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="6"/>
+      <c r="B1101" s="6"/>
+      <c r="C1101" s="6"/>
+      <c r="D1101" s="6"/>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="6"/>
+      <c r="B1102" s="6"/>
+      <c r="C1102" s="6"/>
+      <c r="D1102" s="6"/>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="6"/>
+      <c r="B1103" s="6"/>
+      <c r="C1103" s="6"/>
+      <c r="D1103" s="6"/>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="6"/>
+      <c r="B1104" s="6"/>
+      <c r="C1104" s="6"/>
+      <c r="D1104" s="6"/>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="6"/>
+      <c r="B1105" s="6"/>
+      <c r="C1105" s="6"/>
+      <c r="D1105" s="6"/>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="6"/>
+      <c r="B1106" s="6"/>
+      <c r="C1106" s="6"/>
+      <c r="D1106" s="6"/>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="6"/>
+      <c r="B1107" s="6"/>
+      <c r="C1107" s="6"/>
+      <c r="D1107" s="6"/>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="6"/>
+      <c r="B1108" s="6"/>
+      <c r="C1108" s="6"/>
+      <c r="D1108" s="6"/>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="6"/>
+      <c r="B1109" s="6"/>
+      <c r="C1109" s="6"/>
+      <c r="D1109" s="6"/>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="6"/>
+      <c r="B1110" s="6"/>
+      <c r="C1110" s="6"/>
+      <c r="D1110" s="6"/>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="6"/>
+      <c r="B1111" s="6"/>
+      <c r="C1111" s="6"/>
+      <c r="D1111" s="6"/>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="6"/>
+      <c r="B1112" s="6"/>
+      <c r="C1112" s="6"/>
+      <c r="D1112" s="6"/>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="6"/>
+      <c r="B1113" s="6"/>
+      <c r="C1113" s="6"/>
+      <c r="D1113" s="6"/>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="6"/>
+      <c r="B1114" s="6"/>
+      <c r="C1114" s="6"/>
+      <c r="D1114" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D224">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D243 D250:D268 D271:D273 D286:D287">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A164"/>
+    <hyperlink r:id="rId1" ref="A77"/>
+    <hyperlink r:id="rId2" ref="A172"/>
   </hyperlinks>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
WIP create alarm (work but some problemes)
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="524">
   <si>
     <t>Key</t>
   </si>
@@ -1490,6 +1490,12 @@
     <t>Sleep Aid</t>
   </si>
   <si>
+    <t>profile_advanced_info.sleeping_pills.description</t>
+  </si>
+  <si>
+    <t>Sleeping pills include any prescription sleep drugs.</t>
+  </si>
+  <si>
     <t>profile_advanced_info.sleeping_pills.none</t>
   </si>
   <si>
@@ -1518,6 +1524,12 @@
   </si>
   <si>
     <t>Sleep supplements</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.description</t>
+  </si>
+  <si>
+    <t>Dietary supplements include melatonin, herbs, magnesium, etc...</t>
   </si>
   <si>
     <t>profile_advanced_info.dietary_supplements.none</t>
@@ -1608,7 +1620,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1635,16 +1647,12 @@
       <u/>
       <color rgb="FF0000FF"/>
     </font>
-    <font/>
-    <font>
-      <strike/>
-      <color rgb="FFFF0000"/>
-    </font>
     <font>
       <strike/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
     </font>
+    <font/>
   </fonts>
   <fills count="6">
     <fill>
@@ -1684,7 +1692,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1733,28 +1741,19 @@
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -4547,11 +4546,11 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="15" t="s">
+      <c r="A214" s="5" t="s">
         <v>400</v>
       </c>
       <c r="B214" s="6"/>
-      <c r="C214" s="16" t="s">
+      <c r="C214" s="7" t="s">
         <v>401</v>
       </c>
       <c r="D214" s="5" t="s">
@@ -4559,14 +4558,14 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="17" t="s">
+      <c r="A215" s="15" t="s">
         <v>402</v>
       </c>
-      <c r="B215" s="18"/>
-      <c r="C215" s="19" t="s">
+      <c r="B215" s="16"/>
+      <c r="C215" s="17" t="s">
         <v>403</v>
       </c>
-      <c r="D215" s="20" t="s">
+      <c r="D215" s="15" t="s">
         <v>6</v>
       </c>
     </row>
@@ -4631,11 +4630,11 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="15" t="s">
+      <c r="A221" s="5" t="s">
         <v>414</v>
       </c>
       <c r="B221" s="6"/>
-      <c r="C221" s="16" t="s">
+      <c r="C221" s="7" t="s">
         <v>415</v>
       </c>
       <c r="D221" s="5" t="s">
@@ -4643,11 +4642,11 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="15" t="s">
+      <c r="A222" s="5" t="s">
         <v>416</v>
       </c>
       <c r="B222" s="6"/>
-      <c r="C222" s="16" t="s">
+      <c r="C222" s="7" t="s">
         <v>417</v>
       </c>
       <c r="D222" s="5" t="s">
@@ -4667,11 +4666,11 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="15" t="s">
+      <c r="A224" s="5" t="s">
         <v>420</v>
       </c>
       <c r="B224" s="6"/>
-      <c r="C224" s="16" t="s">
+      <c r="C224" s="7" t="s">
         <v>421</v>
       </c>
       <c r="D224" s="5" t="s">
@@ -4799,38 +4798,38 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="20" t="s">
+      <c r="A235" s="15" t="s">
         <v>440</v>
       </c>
-      <c r="B235" s="21"/>
-      <c r="C235" s="22" t="s">
+      <c r="B235" s="16"/>
+      <c r="C235" s="17" t="s">
         <v>231</v>
       </c>
-      <c r="D235" s="20" t="s">
-        <v>6</v>
-      </c>
-      <c r="E235" s="23"/>
-      <c r="F235" s="23"/>
-      <c r="G235" s="23"/>
-      <c r="H235" s="23"/>
-      <c r="I235" s="23"/>
-      <c r="J235" s="23"/>
-      <c r="K235" s="23"/>
-      <c r="L235" s="23"/>
-      <c r="M235" s="23"/>
-      <c r="N235" s="23"/>
-      <c r="O235" s="23"/>
-      <c r="P235" s="23"/>
-      <c r="Q235" s="23"/>
-      <c r="R235" s="23"/>
-      <c r="S235" s="23"/>
-      <c r="T235" s="23"/>
-      <c r="U235" s="23"/>
-      <c r="V235" s="23"/>
-      <c r="W235" s="23"/>
-      <c r="X235" s="23"/>
-      <c r="Y235" s="23"/>
-      <c r="Z235" s="23"/>
+      <c r="D235" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E235" s="18"/>
+      <c r="F235" s="18"/>
+      <c r="G235" s="18"/>
+      <c r="H235" s="18"/>
+      <c r="I235" s="18"/>
+      <c r="J235" s="18"/>
+      <c r="K235" s="18"/>
+      <c r="L235" s="18"/>
+      <c r="M235" s="18"/>
+      <c r="N235" s="18"/>
+      <c r="O235" s="18"/>
+      <c r="P235" s="18"/>
+      <c r="Q235" s="18"/>
+      <c r="R235" s="18"/>
+      <c r="S235" s="18"/>
+      <c r="T235" s="18"/>
+      <c r="U235" s="18"/>
+      <c r="V235" s="18"/>
+      <c r="W235" s="18"/>
+      <c r="X235" s="18"/>
+      <c r="Y235" s="18"/>
+      <c r="Z235" s="18"/>
     </row>
     <row r="236">
       <c r="A236" s="5" t="s">
@@ -4893,17 +4892,17 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="20" t="s">
+      <c r="A241" s="15" t="s">
         <v>451</v>
       </c>
-      <c r="B241" s="21"/>
-      <c r="C241" s="22" t="s">
+      <c r="B241" s="16"/>
+      <c r="C241" s="17" t="s">
         <v>452</v>
       </c>
-      <c r="D241" s="20" t="s">
-        <v>6</v>
-      </c>
-      <c r="E241" s="23"/>
+      <c r="D241" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E241" s="18"/>
     </row>
     <row r="242">
       <c r="A242" s="5" t="s">
@@ -5098,11 +5097,11 @@
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="5" t="s">
+      <c r="A260" s="19" t="s">
         <v>482</v>
       </c>
       <c r="B260" s="6"/>
-      <c r="C260" s="7" t="s">
+      <c r="C260" s="20" t="s">
         <v>483</v>
       </c>
       <c r="D260" s="5" t="s">
@@ -5163,19 +5162,19 @@
       </c>
       <c r="B265" s="6"/>
       <c r="C265" s="7" t="s">
-        <v>483</v>
+        <v>493</v>
       </c>
       <c r="D265" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="266">
-      <c r="A266" s="5" t="s">
-        <v>493</v>
+      <c r="A266" s="19" t="s">
+        <v>494</v>
       </c>
       <c r="B266" s="6"/>
-      <c r="C266" s="7" t="s">
-        <v>485</v>
+      <c r="C266" s="20" t="s">
+        <v>495</v>
       </c>
       <c r="D266" s="5" t="s">
         <v>6</v>
@@ -5183,11 +5182,11 @@
     </row>
     <row r="267">
       <c r="A267" s="5" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B267" s="6"/>
       <c r="C267" s="7" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="D267" s="5" t="s">
         <v>6</v>
@@ -5195,11 +5194,11 @@
     </row>
     <row r="268">
       <c r="A268" s="5" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B268" s="6"/>
       <c r="C268" s="7" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="D268" s="5" t="s">
         <v>6</v>
@@ -5207,43 +5206,43 @@
     </row>
     <row r="269">
       <c r="A269" s="5" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B269" s="6"/>
-      <c r="C269" s="6"/>
-      <c r="D269" s="6"/>
+      <c r="C269" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="D269" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="5" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B270" s="6"/>
-      <c r="C270" s="6"/>
-      <c r="D270" s="6"/>
+      <c r="C270" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="D270" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="5" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B271" s="6"/>
-      <c r="C271" s="7" t="s">
-        <v>499</v>
-      </c>
-      <c r="D271" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C271" s="6"/>
+      <c r="D271" s="6"/>
     </row>
     <row r="272">
       <c r="A272" s="5" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B272" s="6"/>
-      <c r="C272" s="7" t="s">
-        <v>501</v>
-      </c>
-      <c r="D272" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C272" s="6"/>
+      <c r="D272" s="6"/>
     </row>
     <row r="273">
       <c r="A273" s="5" t="s">
@@ -5262,20 +5261,28 @@
         <v>504</v>
       </c>
       <c r="B274" s="6"/>
-      <c r="C274" s="6"/>
-      <c r="D274" s="6"/>
+      <c r="C274" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="D274" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="5" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B275" s="6"/>
-      <c r="C275" s="6"/>
-      <c r="D275" s="6"/>
+      <c r="C275" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="D275" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="5" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B276" s="6"/>
       <c r="C276" s="6"/>
@@ -5283,7 +5290,7 @@
     </row>
     <row r="277">
       <c r="A277" s="5" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B277" s="6"/>
       <c r="C277" s="6"/>
@@ -5291,7 +5298,7 @@
     </row>
     <row r="278">
       <c r="A278" s="5" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B278" s="6"/>
       <c r="C278" s="6"/>
@@ -5299,7 +5306,7 @@
     </row>
     <row r="279">
       <c r="A279" s="5" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B279" s="6"/>
       <c r="C279" s="6"/>
@@ -5307,7 +5314,7 @@
     </row>
     <row r="280">
       <c r="A280" s="5" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B280" s="6"/>
       <c r="C280" s="6"/>
@@ -5315,7 +5322,7 @@
     </row>
     <row r="281">
       <c r="A281" s="5" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B281" s="6"/>
       <c r="C281" s="6"/>
@@ -5323,7 +5330,7 @@
     </row>
     <row r="282">
       <c r="A282" s="5" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B282" s="6"/>
       <c r="C282" s="6"/>
@@ -5331,7 +5338,7 @@
     </row>
     <row r="283">
       <c r="A283" s="5" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B283" s="6"/>
       <c r="C283" s="6"/>
@@ -5339,7 +5346,7 @@
     </row>
     <row r="284">
       <c r="A284" s="5" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B284" s="6"/>
       <c r="C284" s="6"/>
@@ -5347,7 +5354,7 @@
     </row>
     <row r="285">
       <c r="A285" s="5" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B285" s="6"/>
       <c r="C285" s="6"/>
@@ -5355,39 +5362,43 @@
     </row>
     <row r="286">
       <c r="A286" s="5" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B286" s="6"/>
-      <c r="C286" s="7" t="s">
-        <v>517</v>
-      </c>
-      <c r="D286" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C286" s="6"/>
+      <c r="D286" s="6"/>
     </row>
     <row r="287">
       <c r="A287" s="5" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B287" s="6"/>
-      <c r="C287" s="7" t="s">
-        <v>519</v>
-      </c>
-      <c r="D287" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C287" s="6"/>
+      <c r="D287" s="6"/>
     </row>
     <row r="288">
-      <c r="A288" s="6"/>
+      <c r="A288" s="5" t="s">
+        <v>520</v>
+      </c>
       <c r="B288" s="6"/>
-      <c r="C288" s="6"/>
-      <c r="D288" s="6"/>
+      <c r="C288" s="7" t="s">
+        <v>521</v>
+      </c>
+      <c r="D288" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="289">
-      <c r="A289" s="6"/>
+      <c r="A289" s="5" t="s">
+        <v>522</v>
+      </c>
       <c r="B289" s="6"/>
-      <c r="C289" s="6"/>
-      <c r="D289" s="6"/>
+      <c r="C289" s="7" t="s">
+        <v>523</v>
+      </c>
+      <c r="D289" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="6"/>
@@ -10339,9 +10350,21 @@
       <c r="C1114" s="6"/>
       <c r="D1114" s="6"/>
     </row>
+    <row r="1115">
+      <c r="A1115" s="6"/>
+      <c r="B1115" s="6"/>
+      <c r="C1115" s="6"/>
+      <c r="D1115" s="6"/>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="6"/>
+      <c r="B1116" s="6"/>
+      <c r="C1116" s="6"/>
+      <c r="D1116" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D243 D250:D268 D271:D273 D286:D287">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D243 D250:D270 D273:D275 D288:D289">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Format day + improve style
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="552">
   <si>
     <t>Key</t>
   </si>
@@ -424,6 +424,12 @@
   </si>
   <si>
     <t>no</t>
+  </si>
+  <si>
+    <t>global.not_enough_data</t>
+  </si>
+  <si>
+    <t>Not enough information</t>
   </si>
   <si>
     <t>home.sync.syncing</t>
@@ -1415,212 +1421,290 @@
     <t>Night Worker</t>
   </si>
   <si>
+    <t>profile_advanced_info.physical_disability.title</t>
+  </si>
+  <si>
+    <t>Physical Disabilities</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.none</t>
+  </si>
+  <si>
+    <t>No physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.moderate</t>
+  </si>
+  <si>
+    <t>Moderate physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.total</t>
+  </si>
+  <si>
+    <t>Total physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.title</t>
+  </si>
+  <si>
+    <t>Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.none</t>
+  </si>
+  <si>
+    <t>No Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.insomnia</t>
+  </si>
+  <si>
+    <t>Insomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.hypersomnia</t>
+  </si>
+  <si>
+    <t>Hypersomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.other</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.title</t>
+  </si>
+  <si>
+    <t>Sleep Aid</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.description</t>
+  </si>
+  <si>
+    <t>Sleeping pills include any prescription sleep drugs.</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.none</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.daily</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.weekly</t>
+  </si>
+  <si>
+    <t>Weekly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.monthly</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.title</t>
+  </si>
+  <si>
+    <t>Sleep supplements</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.description</t>
+  </si>
+  <si>
+    <t>Dietary supplements include melatonin, herbs, magnesium, etc...</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.none</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.daily</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.weekly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.monthly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeper_type.light</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeper_type.night</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.menstrual_cycle</t>
+  </si>
+  <si>
+    <t>Menstrual cycle</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.menopause</t>
+  </si>
+  <si>
+    <t>Menopause</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.perimenopause</t>
+  </si>
+  <si>
+    <t>Perimenopause</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.none</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.pills</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.condoms</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.vaginal_ring</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.patch</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.iud</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.implant</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.fertility_awareness</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.other</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_28</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_24</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_21</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.open_for_napping.title</t>
+  </si>
+  <si>
+    <t>Open for Napping</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.unknown_option</t>
+  </si>
+  <si>
+    <t>Unknown option</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.title</t>
+  </si>
+  <si>
+    <t>Heart Rate</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.maximum</t>
+  </si>
+  <si>
+    <t>🔝 Maximum</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.sport_target</t>
+  </si>
+  <si>
+    <t>🎯 Sport Target</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.comparative_title</t>
+  </si>
+  <si>
+    <t>Comparative Info</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.rhr</t>
+  </si>
+  <si>
+    <t>😴 RHR</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.vo2_max</t>
+  </si>
+  <si>
+    <t>😮‍💨 VO2 Max</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.bmi.title</t>
+  </si>
+  <si>
+    <t>Body Mass Index</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.title</t>
+  </si>
+  <si>
+    <t>Chronotype</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.morning</t>
   </si>
   <si>
+    <t>Morning type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.solar</t>
   </si>
   <si>
+    <t>Solar type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.night</t>
   </si>
   <si>
+    <t>Night type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.morning_erratic</t>
   </si>
   <si>
+    <t>Morning erratic type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.solar_erratic</t>
   </si>
   <si>
+    <t>Solar erratic type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.night_erratic</t>
   </si>
   <si>
-    <t>profile_advanced_info.physical_disability.title</t>
-  </si>
-  <si>
-    <t>Physical Disabilities</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.none</t>
-  </si>
-  <si>
-    <t>No physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.moderate</t>
-  </si>
-  <si>
-    <t>Moderate physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.total</t>
-  </si>
-  <si>
-    <t>Total physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.title</t>
-  </si>
-  <si>
-    <t>Sleep Disorder</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.none</t>
-  </si>
-  <si>
-    <t>No Sleep Disorder</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.insomnia</t>
-  </si>
-  <si>
-    <t>Insomnia</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.hypersomnia</t>
-  </si>
-  <si>
-    <t>Hypersomnia</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.other</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.title</t>
-  </si>
-  <si>
-    <t>Sleep Aid</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.description</t>
-  </si>
-  <si>
-    <t>Sleeping pills include any prescription sleep drugs.</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.none</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.daily</t>
-  </si>
-  <si>
-    <t>Daily</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.weekly</t>
-  </si>
-  <si>
-    <t>Weekly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.monthly</t>
-  </si>
-  <si>
-    <t>Monthly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.title</t>
-  </si>
-  <si>
-    <t>Sleep supplements</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.description</t>
-  </si>
-  <si>
-    <t>Dietary supplements include melatonin, herbs, magnesium, etc...</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.none</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.daily</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.weekly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.monthly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeper_type.light</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeper_type.night</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.fertility_state.menstrual_cycle</t>
-  </si>
-  <si>
-    <t>Menstrual cycle</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.fertility_state.menopause</t>
-  </si>
-  <si>
-    <t>Menopause</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.fertility_state.perimenopause</t>
-  </si>
-  <si>
-    <t>Perimenopause</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.none</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.pills</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.condoms</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.vaginal_ring</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.patch</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.iud</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.implant</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.fertility_awareness</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.other</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.pill_pack_format.days_28</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.pill_pack_format.days_24</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.pill_pack_format.days_21</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.open_for_napping.title</t>
-  </si>
-  <si>
-    <t>Open for Napping</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.unknown_option</t>
-  </si>
-  <si>
-    <t>Unknown option</t>
+    <t>Night erratic type</t>
+  </si>
+  <si>
+    <t>alarm.weekdays</t>
+  </si>
+  <si>
+    <t>Weekdays</t>
+  </si>
+  <si>
+    <t>alarm.everydays</t>
+  </si>
+  <si>
+    <t>Every day</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1643,6 +1727,7 @@
       <u/>
       <color rgb="FF1155CC"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -1652,7 +1737,9 @@
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
     </font>
-    <font/>
+    <font>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1692,7 +1779,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1729,30 +1816,36 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2914,14 +3007,13 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="5" t="s">
+      <c r="A78" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="B78" s="6"/>
-      <c r="C78" s="7" t="s">
+      <c r="C78" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="D78" s="5" t="s">
+      <c r="D78" s="10" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3058,7 +3150,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="8" t="s">
+      <c r="A90" s="5" t="s">
         <v>161</v>
       </c>
       <c r="B90" s="6"/>
@@ -3082,7 +3174,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="5" t="s">
+      <c r="A92" s="8" t="s">
         <v>165</v>
       </c>
       <c r="B92" s="6"/>
@@ -3387,7 +3479,7 @@
       </c>
       <c r="B117" s="6"/>
       <c r="C117" s="7" t="s">
-        <v>40</v>
+        <v>216</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>6</v>
@@ -3395,7 +3487,7 @@
     </row>
     <row r="118">
       <c r="A118" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B118" s="6"/>
       <c r="C118" s="7" t="s">
@@ -3407,11 +3499,11 @@
     </row>
     <row r="119">
       <c r="A119" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B119" s="6"/>
       <c r="C119" s="7" t="s">
-        <v>218</v>
+        <v>40</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>6</v>
@@ -3421,7 +3513,7 @@
       <c r="A120" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="B120" s="5"/>
+      <c r="B120" s="6"/>
       <c r="C120" s="7" t="s">
         <v>220</v>
       </c>
@@ -3433,7 +3525,7 @@
       <c r="A121" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="B121" s="6"/>
+      <c r="B121" s="5"/>
       <c r="C121" s="7" t="s">
         <v>222</v>
       </c>
@@ -3471,7 +3563,7 @@
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -3479,11 +3571,11 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>6</v>
@@ -3519,7 +3611,7 @@
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>6</v>
@@ -3527,11 +3619,11 @@
     </row>
     <row r="129">
       <c r="A129" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="D129" s="5" t="s">
         <v>6</v>
@@ -3610,7 +3702,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="8" t="s">
+      <c r="A136" s="5" t="s">
         <v>249</v>
       </c>
       <c r="B136" s="6"/>
@@ -3627,7 +3719,7 @@
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
-        <v>224</v>
+        <v>252</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>6</v>
@@ -3635,18 +3727,18 @@
     </row>
     <row r="138">
       <c r="A138" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B138" s="6"/>
       <c r="C138" s="7" t="s">
-        <v>253</v>
+        <v>226</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="5" t="s">
+      <c r="A139" s="8" t="s">
         <v>254</v>
       </c>
       <c r="B139" s="6"/>
@@ -3694,26 +3786,26 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="12" t="s">
+      <c r="A143" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="B143" s="13"/>
-      <c r="C143" s="12" t="s">
+      <c r="B143" s="6"/>
+      <c r="C143" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="B144" s="14"/>
+      <c r="C144" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="D143" s="12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="B144" s="6"/>
-      <c r="C144" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="D144" s="5" t="s">
+      <c r="D144" s="13" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3898,7 +3990,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="8" t="s">
+      <c r="A160" s="5" t="s">
         <v>295</v>
       </c>
       <c r="B160" s="6"/>
@@ -3934,12 +4026,12 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="5" t="s">
+      <c r="A163" s="8" t="s">
         <v>301</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>231</v>
+        <v>302</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
@@ -3947,11 +4039,11 @@
     </row>
     <row r="164">
       <c r="A164" s="5" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>303</v>
+        <v>233</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
@@ -4042,7 +4134,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="14" t="s">
+      <c r="A172" s="5" t="s">
         <v>318</v>
       </c>
       <c r="B172" s="6"/>
@@ -4054,7 +4146,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="5" t="s">
+      <c r="A173" s="15" t="s">
         <v>320</v>
       </c>
       <c r="B173" s="6"/>
@@ -4102,7 +4194,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="8" t="s">
+      <c r="A177" s="5" t="s">
         <v>328</v>
       </c>
       <c r="B177" s="6"/>
@@ -4114,7 +4206,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="5" t="s">
+      <c r="A178" s="8" t="s">
         <v>330</v>
       </c>
       <c r="B178" s="6"/>
@@ -4287,7 +4379,7 @@
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
-        <v>51</v>
+        <v>359</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
@@ -4295,11 +4387,11 @@
     </row>
     <row r="193">
       <c r="A193" s="5" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>360</v>
+        <v>51</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
@@ -4330,7 +4422,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="10" t="s">
+      <c r="A196" s="5" t="s">
         <v>365</v>
       </c>
       <c r="B196" s="6"/>
@@ -4402,12 +4494,12 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="5" t="s">
+      <c r="A202" s="10" t="s">
         <v>377</v>
       </c>
       <c r="B202" s="6"/>
       <c r="C202" s="7" t="s">
-        <v>130</v>
+        <v>378</v>
       </c>
       <c r="D202" s="5" t="s">
         <v>6</v>
@@ -4415,11 +4507,11 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B203" s="6"/>
       <c r="C203" s="7" t="s">
-        <v>379</v>
+        <v>130</v>
       </c>
       <c r="D203" s="5" t="s">
         <v>6</v>
@@ -4558,26 +4650,26 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="15" t="s">
+      <c r="A215" s="5" t="s">
         <v>402</v>
       </c>
-      <c r="B215" s="16"/>
-      <c r="C215" s="17" t="s">
+      <c r="B215" s="6"/>
+      <c r="C215" s="7" t="s">
         <v>403</v>
       </c>
-      <c r="D215" s="15" t="s">
+      <c r="D215" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="5" t="s">
+      <c r="A216" s="16" t="s">
         <v>404</v>
       </c>
-      <c r="B216" s="6"/>
-      <c r="C216" s="7" t="s">
+      <c r="B216" s="17"/>
+      <c r="C216" s="18" t="s">
         <v>405</v>
       </c>
-      <c r="D216" s="5" t="s">
+      <c r="D216" s="16" t="s">
         <v>6</v>
       </c>
     </row>
@@ -4743,7 +4835,7 @@
       </c>
       <c r="B230" s="6"/>
       <c r="C230" s="7" t="s">
-        <v>168</v>
+        <v>433</v>
       </c>
       <c r="D230" s="5" t="s">
         <v>6</v>
@@ -4751,11 +4843,11 @@
     </row>
     <row r="231">
       <c r="A231" s="5" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B231" s="6"/>
       <c r="C231" s="7" t="s">
-        <v>434</v>
+        <v>170</v>
       </c>
       <c r="D231" s="5" t="s">
         <v>6</v>
@@ -4767,7 +4859,7 @@
       </c>
       <c r="B232" s="6"/>
       <c r="C232" s="7" t="s">
-        <v>307</v>
+        <v>436</v>
       </c>
       <c r="D232" s="5" t="s">
         <v>6</v>
@@ -4775,11 +4867,11 @@
     </row>
     <row r="233">
       <c r="A233" s="5" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B233" s="6"/>
       <c r="C233" s="7" t="s">
-        <v>437</v>
+        <v>309</v>
       </c>
       <c r="D233" s="5" t="s">
         <v>6</v>
@@ -4798,50 +4890,50 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="15" t="s">
+      <c r="A235" s="5" t="s">
         <v>440</v>
       </c>
-      <c r="B235" s="16"/>
-      <c r="C235" s="17" t="s">
-        <v>231</v>
-      </c>
-      <c r="D235" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E235" s="18"/>
-      <c r="F235" s="18"/>
-      <c r="G235" s="18"/>
-      <c r="H235" s="18"/>
-      <c r="I235" s="18"/>
-      <c r="J235" s="18"/>
-      <c r="K235" s="18"/>
-      <c r="L235" s="18"/>
-      <c r="M235" s="18"/>
-      <c r="N235" s="18"/>
-      <c r="O235" s="18"/>
-      <c r="P235" s="18"/>
-      <c r="Q235" s="18"/>
-      <c r="R235" s="18"/>
-      <c r="S235" s="18"/>
-      <c r="T235" s="18"/>
-      <c r="U235" s="18"/>
-      <c r="V235" s="18"/>
-      <c r="W235" s="18"/>
-      <c r="X235" s="18"/>
-      <c r="Y235" s="18"/>
-      <c r="Z235" s="18"/>
+      <c r="B235" s="6"/>
+      <c r="C235" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="D235" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="236">
-      <c r="A236" s="5" t="s">
-        <v>441</v>
-      </c>
-      <c r="B236" s="6"/>
-      <c r="C236" s="7" t="s">
+      <c r="A236" s="16" t="s">
         <v>442</v>
       </c>
-      <c r="D236" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="B236" s="17"/>
+      <c r="C236" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="D236" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E236" s="19"/>
+      <c r="F236" s="19"/>
+      <c r="G236" s="19"/>
+      <c r="H236" s="19"/>
+      <c r="I236" s="19"/>
+      <c r="J236" s="19"/>
+      <c r="K236" s="19"/>
+      <c r="L236" s="19"/>
+      <c r="M236" s="19"/>
+      <c r="N236" s="19"/>
+      <c r="O236" s="19"/>
+      <c r="P236" s="19"/>
+      <c r="Q236" s="19"/>
+      <c r="R236" s="19"/>
+      <c r="S236" s="19"/>
+      <c r="T236" s="19"/>
+      <c r="U236" s="19"/>
+      <c r="V236" s="19"/>
+      <c r="W236" s="19"/>
+      <c r="X236" s="19"/>
+      <c r="Y236" s="19"/>
+      <c r="Z236" s="19"/>
     </row>
     <row r="237">
       <c r="A237" s="5" t="s">
@@ -4892,29 +4984,29 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="15" t="s">
+      <c r="A241" s="5" t="s">
         <v>451</v>
       </c>
-      <c r="B241" s="16"/>
-      <c r="C241" s="17" t="s">
+      <c r="B241" s="6"/>
+      <c r="C241" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="D241" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E241" s="18"/>
+      <c r="D241" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="242">
-      <c r="A242" s="5" t="s">
+      <c r="A242" s="16" t="s">
         <v>453</v>
       </c>
-      <c r="B242" s="6"/>
-      <c r="C242" s="7" t="s">
+      <c r="B242" s="17"/>
+      <c r="C242" s="18" t="s">
         <v>454</v>
       </c>
-      <c r="D242" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="D242" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E242" s="19"/>
     </row>
     <row r="243">
       <c r="A243" s="5" t="s">
@@ -4933,56 +5025,80 @@
         <v>457</v>
       </c>
       <c r="B244" s="6"/>
-      <c r="C244" s="6"/>
-      <c r="D244" s="6"/>
+      <c r="C244" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="D244" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="5" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B245" s="6"/>
-      <c r="C245" s="6"/>
-      <c r="D245" s="6"/>
+      <c r="C245" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="D245" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="5" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B246" s="6"/>
-      <c r="C246" s="6"/>
-      <c r="D246" s="6"/>
+      <c r="C246" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="D246" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="5" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B247" s="6"/>
-      <c r="C247" s="6"/>
-      <c r="D247" s="6"/>
+      <c r="C247" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="D247" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="5" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B248" s="6"/>
-      <c r="C248" s="6"/>
-      <c r="D248" s="6"/>
+      <c r="C248" s="7" t="s">
+        <v>466</v>
+      </c>
+      <c r="D248" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="5" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="B249" s="6"/>
-      <c r="C249" s="6"/>
-      <c r="D249" s="6"/>
+      <c r="C249" s="7" t="s">
+        <v>468</v>
+      </c>
+      <c r="D249" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="5" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="B250" s="6"/>
       <c r="C250" s="7" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="D250" s="5" t="s">
         <v>6</v>
@@ -4990,11 +5106,11 @@
     </row>
     <row r="251">
       <c r="A251" s="5" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="B251" s="6"/>
       <c r="C251" s="7" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="D251" s="5" t="s">
         <v>6</v>
@@ -5002,11 +5118,11 @@
     </row>
     <row r="252">
       <c r="A252" s="5" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="B252" s="6"/>
       <c r="C252" s="7" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="D252" s="5" t="s">
         <v>6</v>
@@ -5014,11 +5130,11 @@
     </row>
     <row r="253">
       <c r="A253" s="5" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B253" s="6"/>
       <c r="C253" s="7" t="s">
-        <v>470</v>
+        <v>431</v>
       </c>
       <c r="D253" s="5" t="s">
         <v>6</v>
@@ -5026,11 +5142,11 @@
     </row>
     <row r="254">
       <c r="A254" s="5" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="B254" s="6"/>
       <c r="C254" s="7" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="D254" s="5" t="s">
         <v>6</v>
@@ -5038,11 +5154,11 @@
     </row>
     <row r="255">
       <c r="A255" s="5" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="B255" s="6"/>
       <c r="C255" s="7" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="D255" s="5" t="s">
         <v>6</v>
@@ -5050,11 +5166,11 @@
     </row>
     <row r="256">
       <c r="A256" s="5" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="B256" s="6"/>
       <c r="C256" s="7" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="D256" s="5" t="s">
         <v>6</v>
@@ -5062,11 +5178,11 @@
     </row>
     <row r="257">
       <c r="A257" s="5" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="B257" s="6"/>
       <c r="C257" s="7" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="D257" s="5" t="s">
         <v>6</v>
@@ -5074,11 +5190,11 @@
     </row>
     <row r="258">
       <c r="A258" s="5" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="B258" s="6"/>
       <c r="C258" s="7" t="s">
-        <v>429</v>
+        <v>485</v>
       </c>
       <c r="D258" s="5" t="s">
         <v>6</v>
@@ -5086,23 +5202,23 @@
     </row>
     <row r="259">
       <c r="A259" s="5" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="B259" s="6"/>
       <c r="C259" s="7" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="D259" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="19" t="s">
-        <v>482</v>
+      <c r="A260" s="5" t="s">
+        <v>488</v>
       </c>
       <c r="B260" s="6"/>
-      <c r="C260" s="20" t="s">
-        <v>483</v>
+      <c r="C260" s="7" t="s">
+        <v>489</v>
       </c>
       <c r="D260" s="5" t="s">
         <v>6</v>
@@ -5110,11 +5226,11 @@
     </row>
     <row r="261">
       <c r="A261" s="5" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="B261" s="6"/>
       <c r="C261" s="7" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="D261" s="5" t="s">
         <v>6</v>
@@ -5122,11 +5238,11 @@
     </row>
     <row r="262">
       <c r="A262" s="5" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="B262" s="6"/>
       <c r="C262" s="7" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="D262" s="5" t="s">
         <v>6</v>
@@ -5134,11 +5250,11 @@
     </row>
     <row r="263">
       <c r="A263" s="5" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="B263" s="6"/>
       <c r="C263" s="7" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
       <c r="D263" s="5" t="s">
         <v>6</v>
@@ -5146,11 +5262,11 @@
     </row>
     <row r="264">
       <c r="A264" s="5" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="B264" s="6"/>
       <c r="C264" s="7" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D264" s="5" t="s">
         <v>6</v>
@@ -5158,47 +5274,39 @@
     </row>
     <row r="265">
       <c r="A265" s="5" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="B265" s="6"/>
       <c r="C265" s="7" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="D265" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="266">
-      <c r="A266" s="19" t="s">
-        <v>494</v>
+      <c r="A266" s="5" t="s">
+        <v>496</v>
       </c>
       <c r="B266" s="6"/>
-      <c r="C266" s="20" t="s">
-        <v>495</v>
-      </c>
-      <c r="D266" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C266" s="6"/>
+      <c r="D266" s="6"/>
     </row>
     <row r="267">
       <c r="A267" s="5" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B267" s="6"/>
-      <c r="C267" s="7" t="s">
-        <v>485</v>
-      </c>
-      <c r="D267" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C267" s="6"/>
+      <c r="D267" s="6"/>
     </row>
     <row r="268">
       <c r="A268" s="5" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B268" s="6"/>
       <c r="C268" s="7" t="s">
-        <v>487</v>
+        <v>499</v>
       </c>
       <c r="D268" s="5" t="s">
         <v>6</v>
@@ -5206,11 +5314,11 @@
     </row>
     <row r="269">
       <c r="A269" s="5" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B269" s="6"/>
       <c r="C269" s="7" t="s">
-        <v>489</v>
+        <v>501</v>
       </c>
       <c r="D269" s="5" t="s">
         <v>6</v>
@@ -5218,11 +5326,11 @@
     </row>
     <row r="270">
       <c r="A270" s="5" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="B270" s="6"/>
       <c r="C270" s="7" t="s">
-        <v>491</v>
+        <v>503</v>
       </c>
       <c r="D270" s="5" t="s">
         <v>6</v>
@@ -5230,7 +5338,7 @@
     </row>
     <row r="271">
       <c r="A271" s="5" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="B271" s="6"/>
       <c r="C271" s="6"/>
@@ -5238,7 +5346,7 @@
     </row>
     <row r="272">
       <c r="A272" s="5" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="B272" s="6"/>
       <c r="C272" s="6"/>
@@ -5246,43 +5354,31 @@
     </row>
     <row r="273">
       <c r="A273" s="5" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="B273" s="6"/>
-      <c r="C273" s="7" t="s">
-        <v>503</v>
-      </c>
-      <c r="D273" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C273" s="6"/>
+      <c r="D273" s="6"/>
     </row>
     <row r="274">
       <c r="A274" s="5" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="B274" s="6"/>
-      <c r="C274" s="7" t="s">
-        <v>505</v>
-      </c>
-      <c r="D274" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C274" s="6"/>
+      <c r="D274" s="6"/>
     </row>
     <row r="275">
       <c r="A275" s="5" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B275" s="6"/>
-      <c r="C275" s="7" t="s">
-        <v>507</v>
-      </c>
-      <c r="D275" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C275" s="6"/>
+      <c r="D275" s="6"/>
     </row>
     <row r="276">
       <c r="A276" s="5" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B276" s="6"/>
       <c r="C276" s="6"/>
@@ -5290,7 +5386,7 @@
     </row>
     <row r="277">
       <c r="A277" s="5" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B277" s="6"/>
       <c r="C277" s="6"/>
@@ -5298,7 +5394,7 @@
     </row>
     <row r="278">
       <c r="A278" s="5" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B278" s="6"/>
       <c r="C278" s="6"/>
@@ -5306,7 +5402,7 @@
     </row>
     <row r="279">
       <c r="A279" s="5" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B279" s="6"/>
       <c r="C279" s="6"/>
@@ -5314,7 +5410,7 @@
     </row>
     <row r="280">
       <c r="A280" s="5" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B280" s="6"/>
       <c r="C280" s="6"/>
@@ -5322,7 +5418,7 @@
     </row>
     <row r="281">
       <c r="A281" s="5" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B281" s="6"/>
       <c r="C281" s="6"/>
@@ -5330,7 +5426,7 @@
     </row>
     <row r="282">
       <c r="A282" s="5" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B282" s="6"/>
       <c r="C282" s="6"/>
@@ -5338,133 +5434,219 @@
     </row>
     <row r="283">
       <c r="A283" s="5" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B283" s="6"/>
-      <c r="C283" s="6"/>
-      <c r="D283" s="6"/>
+      <c r="C283" s="7" t="s">
+        <v>517</v>
+      </c>
+      <c r="D283" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="5" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B284" s="6"/>
-      <c r="C284" s="6"/>
-      <c r="D284" s="6"/>
+      <c r="C284" s="7" t="s">
+        <v>519</v>
+      </c>
+      <c r="D284" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="285">
-      <c r="A285" s="5" t="s">
-        <v>517</v>
+      <c r="A285" s="20" t="s">
+        <v>520</v>
       </c>
       <c r="B285" s="6"/>
-      <c r="C285" s="6"/>
-      <c r="D285" s="6"/>
+      <c r="C285" s="12" t="s">
+        <v>521</v>
+      </c>
+      <c r="D285" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="286">
-      <c r="A286" s="5" t="s">
-        <v>518</v>
+      <c r="A286" s="20" t="s">
+        <v>522</v>
       </c>
       <c r="B286" s="6"/>
-      <c r="C286" s="6"/>
-      <c r="D286" s="6"/>
+      <c r="C286" s="12" t="s">
+        <v>523</v>
+      </c>
+      <c r="D286" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="287">
-      <c r="A287" s="5" t="s">
-        <v>519</v>
+      <c r="A287" s="20" t="s">
+        <v>524</v>
       </c>
       <c r="B287" s="6"/>
-      <c r="C287" s="6"/>
-      <c r="D287" s="6"/>
+      <c r="C287" s="12" t="s">
+        <v>525</v>
+      </c>
+      <c r="D287" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="288">
-      <c r="A288" s="5" t="s">
-        <v>520</v>
+      <c r="A288" s="20" t="s">
+        <v>526</v>
       </c>
       <c r="B288" s="6"/>
-      <c r="C288" s="7" t="s">
-        <v>521</v>
+      <c r="C288" s="12" t="s">
+        <v>527</v>
       </c>
       <c r="D288" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="289">
-      <c r="A289" s="5" t="s">
-        <v>522</v>
+      <c r="A289" s="20" t="s">
+        <v>528</v>
       </c>
       <c r="B289" s="6"/>
-      <c r="C289" s="7" t="s">
-        <v>523</v>
+      <c r="C289" s="12" t="s">
+        <v>529</v>
       </c>
       <c r="D289" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="290">
-      <c r="A290" s="6"/>
+      <c r="A290" s="20" t="s">
+        <v>530</v>
+      </c>
       <c r="B290" s="6"/>
-      <c r="C290" s="6"/>
-      <c r="D290" s="6"/>
+      <c r="C290" s="12" t="s">
+        <v>531</v>
+      </c>
+      <c r="D290" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="291">
-      <c r="A291" s="6"/>
+      <c r="A291" s="20" t="s">
+        <v>532</v>
+      </c>
       <c r="B291" s="6"/>
-      <c r="C291" s="6"/>
-      <c r="D291" s="6"/>
+      <c r="C291" s="12" t="s">
+        <v>533</v>
+      </c>
+      <c r="D291" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="292">
-      <c r="A292" s="6"/>
+      <c r="A292" s="20" t="s">
+        <v>534</v>
+      </c>
       <c r="B292" s="6"/>
-      <c r="C292" s="6"/>
-      <c r="D292" s="6"/>
+      <c r="C292" s="12" t="s">
+        <v>535</v>
+      </c>
+      <c r="D292" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="293">
-      <c r="A293" s="6"/>
+      <c r="A293" s="21" t="s">
+        <v>536</v>
+      </c>
       <c r="B293" s="6"/>
-      <c r="C293" s="6"/>
-      <c r="D293" s="6"/>
+      <c r="C293" s="12" t="s">
+        <v>537</v>
+      </c>
+      <c r="D293" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="294">
-      <c r="A294" s="6"/>
+      <c r="A294" s="22" t="s">
+        <v>538</v>
+      </c>
       <c r="B294" s="6"/>
-      <c r="C294" s="6"/>
-      <c r="D294" s="6"/>
+      <c r="C294" s="12" t="s">
+        <v>539</v>
+      </c>
+      <c r="D294" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="295">
-      <c r="A295" s="6"/>
+      <c r="A295" s="22" t="s">
+        <v>540</v>
+      </c>
       <c r="B295" s="6"/>
-      <c r="C295" s="6"/>
-      <c r="D295" s="6"/>
+      <c r="C295" s="12" t="s">
+        <v>541</v>
+      </c>
+      <c r="D295" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="296">
-      <c r="A296" s="6"/>
+      <c r="A296" s="22" t="s">
+        <v>542</v>
+      </c>
       <c r="B296" s="6"/>
-      <c r="C296" s="6"/>
-      <c r="D296" s="6"/>
+      <c r="C296" s="12" t="s">
+        <v>543</v>
+      </c>
+      <c r="D296" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="297">
-      <c r="A297" s="6"/>
+      <c r="A297" s="22" t="s">
+        <v>544</v>
+      </c>
       <c r="B297" s="6"/>
-      <c r="C297" s="6"/>
-      <c r="D297" s="6"/>
+      <c r="C297" s="12" t="s">
+        <v>545</v>
+      </c>
+      <c r="D297" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="298">
-      <c r="A298" s="6"/>
+      <c r="A298" s="22" t="s">
+        <v>546</v>
+      </c>
       <c r="B298" s="6"/>
-      <c r="C298" s="6"/>
-      <c r="D298" s="6"/>
+      <c r="C298" s="12" t="s">
+        <v>547</v>
+      </c>
+      <c r="D298" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="299">
-      <c r="A299" s="6"/>
+      <c r="A299" s="20" t="s">
+        <v>548</v>
+      </c>
       <c r="B299" s="6"/>
-      <c r="C299" s="6"/>
-      <c r="D299" s="6"/>
+      <c r="C299" s="12" t="s">
+        <v>549</v>
+      </c>
+      <c r="D299" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="300">
-      <c r="A300" s="6"/>
+      <c r="A300" s="20" t="s">
+        <v>550</v>
+      </c>
       <c r="B300" s="6"/>
-      <c r="C300" s="6"/>
-      <c r="D300" s="6"/>
+      <c r="C300" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="D300" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="6"/>
@@ -10350,27 +10532,15 @@
       <c r="C1114" s="6"/>
       <c r="D1114" s="6"/>
     </row>
-    <row r="1115">
-      <c r="A1115" s="6"/>
-      <c r="B1115" s="6"/>
-      <c r="C1115" s="6"/>
-      <c r="D1115" s="6"/>
-    </row>
-    <row r="1116">
-      <c r="A1116" s="6"/>
-      <c r="B1116" s="6"/>
-      <c r="C1116" s="6"/>
-      <c r="D1116" s="6"/>
-    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D243 D250:D270 D273:D275 D288:D289">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D265 D268:D270 D283:D300">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="A77"/>
-    <hyperlink r:id="rId2" ref="A172"/>
+    <hyperlink r:id="rId2" ref="A173"/>
   </hyperlinks>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
HRate BMI and ChronoType cards
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="552">
   <si>
     <t>Key</t>
   </si>
@@ -424,6 +424,12 @@
   </si>
   <si>
     <t>no</t>
+  </si>
+  <si>
+    <t>global.not_enough_data</t>
+  </si>
+  <si>
+    <t>Not enough information</t>
   </si>
   <si>
     <t>home.sync.syncing</t>
@@ -1415,212 +1421,290 @@
     <t>Night Worker</t>
   </si>
   <si>
+    <t>profile_advanced_info.physical_disability.title</t>
+  </si>
+  <si>
+    <t>Physical Disabilities</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.none</t>
+  </si>
+  <si>
+    <t>No physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.moderate</t>
+  </si>
+  <si>
+    <t>Moderate physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.total</t>
+  </si>
+  <si>
+    <t>Total physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.title</t>
+  </si>
+  <si>
+    <t>Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.none</t>
+  </si>
+  <si>
+    <t>No Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.insomnia</t>
+  </si>
+  <si>
+    <t>Insomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.hypersomnia</t>
+  </si>
+  <si>
+    <t>Hypersomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.other</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.title</t>
+  </si>
+  <si>
+    <t>Sleep Aid</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.description</t>
+  </si>
+  <si>
+    <t>Sleeping pills include any prescription sleep drugs.</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.none</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.daily</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.weekly</t>
+  </si>
+  <si>
+    <t>Weekly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.monthly</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.title</t>
+  </si>
+  <si>
+    <t>Sleep supplements</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.description</t>
+  </si>
+  <si>
+    <t>Dietary supplements include melatonin, herbs, magnesium, etc...</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.none</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.daily</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.weekly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.monthly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeper_type.light</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeper_type.night</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.menstrual_cycle</t>
+  </si>
+  <si>
+    <t>Menstrual cycle</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.menopause</t>
+  </si>
+  <si>
+    <t>Menopause</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.perimenopause</t>
+  </si>
+  <si>
+    <t>Perimenopause</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.none</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.pills</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.condoms</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.vaginal_ring</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.patch</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.iud</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.implant</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.fertility_awareness</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.other</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_28</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_24</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_21</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.open_for_napping.title</t>
+  </si>
+  <si>
+    <t>Open for Napping</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.unknown_option</t>
+  </si>
+  <si>
+    <t>Unknown option</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.title</t>
+  </si>
+  <si>
+    <t>Heart Rate</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.maximum</t>
+  </si>
+  <si>
+    <t>🔝 Maximum</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.sport_target</t>
+  </si>
+  <si>
+    <t>🎯 Sport Target</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.comparative_title</t>
+  </si>
+  <si>
+    <t>Comparative Info</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.rhr</t>
+  </si>
+  <si>
+    <t>😴 RHR</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.vo2_max</t>
+  </si>
+  <si>
+    <t>😮‍💨 VO2 Max</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.bmi.title</t>
+  </si>
+  <si>
+    <t>Body Mass Index</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.title</t>
+  </si>
+  <si>
+    <t>Chronotype</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.morning</t>
   </si>
   <si>
+    <t>Morning type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.solar</t>
   </si>
   <si>
+    <t>Solar type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.night</t>
   </si>
   <si>
+    <t>Night type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.morning_erratic</t>
   </si>
   <si>
+    <t>Morning erratic type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.solar_erratic</t>
   </si>
   <si>
+    <t>Solar erratic type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.night_erratic</t>
   </si>
   <si>
-    <t>profile_advanced_info.physical_disability.title</t>
-  </si>
-  <si>
-    <t>Physical Disabilities</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.none</t>
-  </si>
-  <si>
-    <t>No physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.moderate</t>
-  </si>
-  <si>
-    <t>Moderate physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.total</t>
-  </si>
-  <si>
-    <t>Total physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.title</t>
-  </si>
-  <si>
-    <t>Sleep Disorder</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.none</t>
-  </si>
-  <si>
-    <t>No Sleep Disorder</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.insomnia</t>
-  </si>
-  <si>
-    <t>Insomnia</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.hypersomnia</t>
-  </si>
-  <si>
-    <t>Hypersomnia</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.other</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.title</t>
-  </si>
-  <si>
-    <t>Sleep Aid</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.description</t>
-  </si>
-  <si>
-    <t>Sleeping pills include any prescription sleep drugs.</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.none</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.daily</t>
-  </si>
-  <si>
-    <t>Daily</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.weekly</t>
-  </si>
-  <si>
-    <t>Weekly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.monthly</t>
-  </si>
-  <si>
-    <t>Monthly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.title</t>
-  </si>
-  <si>
-    <t>Sleep supplements</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.description</t>
-  </si>
-  <si>
-    <t>Dietary supplements include melatonin, herbs, magnesium, etc...</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.none</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.daily</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.weekly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.monthly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeper_type.light</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeper_type.night</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.fertility_state.menstrual_cycle</t>
-  </si>
-  <si>
-    <t>Menstrual cycle</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.fertility_state.menopause</t>
-  </si>
-  <si>
-    <t>Menopause</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.fertility_state.perimenopause</t>
-  </si>
-  <si>
-    <t>Perimenopause</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.none</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.pills</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.condoms</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.vaginal_ring</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.patch</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.iud</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.implant</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.fertility_awareness</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.other</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.pill_pack_format.days_28</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.pill_pack_format.days_24</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.pill_pack_format.days_21</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.open_for_napping.title</t>
-  </si>
-  <si>
-    <t>Open for Napping</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.unknown_option</t>
-  </si>
-  <si>
-    <t>Unknown option</t>
+    <t>Night erratic type</t>
+  </si>
+  <si>
+    <t>alarm.weekdays</t>
+  </si>
+  <si>
+    <t>Weekdays</t>
+  </si>
+  <si>
+    <t>alarm.everydays</t>
+  </si>
+  <si>
+    <t>Every day</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1643,6 +1727,7 @@
       <u/>
       <color rgb="FF1155CC"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -1652,7 +1737,9 @@
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
     </font>
-    <font/>
+    <font>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1692,7 +1779,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1729,30 +1816,36 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2914,14 +3007,13 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="5" t="s">
+      <c r="A78" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="B78" s="6"/>
-      <c r="C78" s="7" t="s">
+      <c r="C78" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="D78" s="5" t="s">
+      <c r="D78" s="10" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3058,7 +3150,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="8" t="s">
+      <c r="A90" s="5" t="s">
         <v>161</v>
       </c>
       <c r="B90" s="6"/>
@@ -3082,7 +3174,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="5" t="s">
+      <c r="A92" s="8" t="s">
         <v>165</v>
       </c>
       <c r="B92" s="6"/>
@@ -3387,7 +3479,7 @@
       </c>
       <c r="B117" s="6"/>
       <c r="C117" s="7" t="s">
-        <v>40</v>
+        <v>216</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>6</v>
@@ -3395,7 +3487,7 @@
     </row>
     <row r="118">
       <c r="A118" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B118" s="6"/>
       <c r="C118" s="7" t="s">
@@ -3407,11 +3499,11 @@
     </row>
     <row r="119">
       <c r="A119" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B119" s="6"/>
       <c r="C119" s="7" t="s">
-        <v>218</v>
+        <v>40</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>6</v>
@@ -3421,7 +3513,7 @@
       <c r="A120" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="B120" s="5"/>
+      <c r="B120" s="6"/>
       <c r="C120" s="7" t="s">
         <v>220</v>
       </c>
@@ -3433,7 +3525,7 @@
       <c r="A121" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="B121" s="6"/>
+      <c r="B121" s="5"/>
       <c r="C121" s="7" t="s">
         <v>222</v>
       </c>
@@ -3471,7 +3563,7 @@
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -3479,11 +3571,11 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>6</v>
@@ -3519,7 +3611,7 @@
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>6</v>
@@ -3527,11 +3619,11 @@
     </row>
     <row r="129">
       <c r="A129" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="D129" s="5" t="s">
         <v>6</v>
@@ -3610,7 +3702,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="8" t="s">
+      <c r="A136" s="5" t="s">
         <v>249</v>
       </c>
       <c r="B136" s="6"/>
@@ -3627,7 +3719,7 @@
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
-        <v>224</v>
+        <v>252</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>6</v>
@@ -3635,18 +3727,18 @@
     </row>
     <row r="138">
       <c r="A138" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B138" s="6"/>
       <c r="C138" s="7" t="s">
-        <v>253</v>
+        <v>226</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="5" t="s">
+      <c r="A139" s="8" t="s">
         <v>254</v>
       </c>
       <c r="B139" s="6"/>
@@ -3694,26 +3786,26 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="12" t="s">
+      <c r="A143" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="B143" s="13"/>
-      <c r="C143" s="12" t="s">
+      <c r="B143" s="6"/>
+      <c r="C143" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="B144" s="14"/>
+      <c r="C144" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="D143" s="12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="B144" s="6"/>
-      <c r="C144" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="D144" s="5" t="s">
+      <c r="D144" s="13" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3898,7 +3990,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="8" t="s">
+      <c r="A160" s="5" t="s">
         <v>295</v>
       </c>
       <c r="B160" s="6"/>
@@ -3934,12 +4026,12 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="5" t="s">
+      <c r="A163" s="8" t="s">
         <v>301</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>231</v>
+        <v>302</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
@@ -3947,11 +4039,11 @@
     </row>
     <row r="164">
       <c r="A164" s="5" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>303</v>
+        <v>233</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
@@ -4042,7 +4134,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="14" t="s">
+      <c r="A172" s="5" t="s">
         <v>318</v>
       </c>
       <c r="B172" s="6"/>
@@ -4054,7 +4146,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="5" t="s">
+      <c r="A173" s="15" t="s">
         <v>320</v>
       </c>
       <c r="B173" s="6"/>
@@ -4102,7 +4194,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="8" t="s">
+      <c r="A177" s="5" t="s">
         <v>328</v>
       </c>
       <c r="B177" s="6"/>
@@ -4114,7 +4206,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="5" t="s">
+      <c r="A178" s="8" t="s">
         <v>330</v>
       </c>
       <c r="B178" s="6"/>
@@ -4287,7 +4379,7 @@
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
-        <v>51</v>
+        <v>359</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
@@ -4295,11 +4387,11 @@
     </row>
     <row r="193">
       <c r="A193" s="5" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>360</v>
+        <v>51</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
@@ -4330,7 +4422,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="10" t="s">
+      <c r="A196" s="5" t="s">
         <v>365</v>
       </c>
       <c r="B196" s="6"/>
@@ -4402,12 +4494,12 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="5" t="s">
+      <c r="A202" s="10" t="s">
         <v>377</v>
       </c>
       <c r="B202" s="6"/>
       <c r="C202" s="7" t="s">
-        <v>130</v>
+        <v>378</v>
       </c>
       <c r="D202" s="5" t="s">
         <v>6</v>
@@ -4415,11 +4507,11 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B203" s="6"/>
       <c r="C203" s="7" t="s">
-        <v>379</v>
+        <v>130</v>
       </c>
       <c r="D203" s="5" t="s">
         <v>6</v>
@@ -4558,26 +4650,26 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="15" t="s">
+      <c r="A215" s="5" t="s">
         <v>402</v>
       </c>
-      <c r="B215" s="16"/>
-      <c r="C215" s="17" t="s">
+      <c r="B215" s="6"/>
+      <c r="C215" s="7" t="s">
         <v>403</v>
       </c>
-      <c r="D215" s="15" t="s">
+      <c r="D215" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="5" t="s">
+      <c r="A216" s="16" t="s">
         <v>404</v>
       </c>
-      <c r="B216" s="6"/>
-      <c r="C216" s="7" t="s">
+      <c r="B216" s="17"/>
+      <c r="C216" s="18" t="s">
         <v>405</v>
       </c>
-      <c r="D216" s="5" t="s">
+      <c r="D216" s="16" t="s">
         <v>6</v>
       </c>
     </row>
@@ -4743,7 +4835,7 @@
       </c>
       <c r="B230" s="6"/>
       <c r="C230" s="7" t="s">
-        <v>168</v>
+        <v>433</v>
       </c>
       <c r="D230" s="5" t="s">
         <v>6</v>
@@ -4751,11 +4843,11 @@
     </row>
     <row r="231">
       <c r="A231" s="5" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B231" s="6"/>
       <c r="C231" s="7" t="s">
-        <v>434</v>
+        <v>170</v>
       </c>
       <c r="D231" s="5" t="s">
         <v>6</v>
@@ -4767,7 +4859,7 @@
       </c>
       <c r="B232" s="6"/>
       <c r="C232" s="7" t="s">
-        <v>307</v>
+        <v>436</v>
       </c>
       <c r="D232" s="5" t="s">
         <v>6</v>
@@ -4775,11 +4867,11 @@
     </row>
     <row r="233">
       <c r="A233" s="5" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B233" s="6"/>
       <c r="C233" s="7" t="s">
-        <v>437</v>
+        <v>309</v>
       </c>
       <c r="D233" s="5" t="s">
         <v>6</v>
@@ -4798,50 +4890,50 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="15" t="s">
+      <c r="A235" s="5" t="s">
         <v>440</v>
       </c>
-      <c r="B235" s="16"/>
-      <c r="C235" s="17" t="s">
-        <v>231</v>
-      </c>
-      <c r="D235" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E235" s="18"/>
-      <c r="F235" s="18"/>
-      <c r="G235" s="18"/>
-      <c r="H235" s="18"/>
-      <c r="I235" s="18"/>
-      <c r="J235" s="18"/>
-      <c r="K235" s="18"/>
-      <c r="L235" s="18"/>
-      <c r="M235" s="18"/>
-      <c r="N235" s="18"/>
-      <c r="O235" s="18"/>
-      <c r="P235" s="18"/>
-      <c r="Q235" s="18"/>
-      <c r="R235" s="18"/>
-      <c r="S235" s="18"/>
-      <c r="T235" s="18"/>
-      <c r="U235" s="18"/>
-      <c r="V235" s="18"/>
-      <c r="W235" s="18"/>
-      <c r="X235" s="18"/>
-      <c r="Y235" s="18"/>
-      <c r="Z235" s="18"/>
+      <c r="B235" s="6"/>
+      <c r="C235" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="D235" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="236">
-      <c r="A236" s="5" t="s">
-        <v>441</v>
-      </c>
-      <c r="B236" s="6"/>
-      <c r="C236" s="7" t="s">
+      <c r="A236" s="16" t="s">
         <v>442</v>
       </c>
-      <c r="D236" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="B236" s="17"/>
+      <c r="C236" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="D236" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E236" s="19"/>
+      <c r="F236" s="19"/>
+      <c r="G236" s="19"/>
+      <c r="H236" s="19"/>
+      <c r="I236" s="19"/>
+      <c r="J236" s="19"/>
+      <c r="K236" s="19"/>
+      <c r="L236" s="19"/>
+      <c r="M236" s="19"/>
+      <c r="N236" s="19"/>
+      <c r="O236" s="19"/>
+      <c r="P236" s="19"/>
+      <c r="Q236" s="19"/>
+      <c r="R236" s="19"/>
+      <c r="S236" s="19"/>
+      <c r="T236" s="19"/>
+      <c r="U236" s="19"/>
+      <c r="V236" s="19"/>
+      <c r="W236" s="19"/>
+      <c r="X236" s="19"/>
+      <c r="Y236" s="19"/>
+      <c r="Z236" s="19"/>
     </row>
     <row r="237">
       <c r="A237" s="5" t="s">
@@ -4892,29 +4984,29 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="15" t="s">
+      <c r="A241" s="5" t="s">
         <v>451</v>
       </c>
-      <c r="B241" s="16"/>
-      <c r="C241" s="17" t="s">
+      <c r="B241" s="6"/>
+      <c r="C241" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="D241" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E241" s="18"/>
+      <c r="D241" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="242">
-      <c r="A242" s="5" t="s">
+      <c r="A242" s="16" t="s">
         <v>453</v>
       </c>
-      <c r="B242" s="6"/>
-      <c r="C242" s="7" t="s">
+      <c r="B242" s="17"/>
+      <c r="C242" s="18" t="s">
         <v>454</v>
       </c>
-      <c r="D242" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="D242" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E242" s="19"/>
     </row>
     <row r="243">
       <c r="A243" s="5" t="s">
@@ -4933,56 +5025,80 @@
         <v>457</v>
       </c>
       <c r="B244" s="6"/>
-      <c r="C244" s="6"/>
-      <c r="D244" s="6"/>
+      <c r="C244" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="D244" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="5" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B245" s="6"/>
-      <c r="C245" s="6"/>
-      <c r="D245" s="6"/>
+      <c r="C245" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="D245" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="5" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B246" s="6"/>
-      <c r="C246" s="6"/>
-      <c r="D246" s="6"/>
+      <c r="C246" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="D246" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="5" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B247" s="6"/>
-      <c r="C247" s="6"/>
-      <c r="D247" s="6"/>
+      <c r="C247" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="D247" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="5" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B248" s="6"/>
-      <c r="C248" s="6"/>
-      <c r="D248" s="6"/>
+      <c r="C248" s="7" t="s">
+        <v>466</v>
+      </c>
+      <c r="D248" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="5" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="B249" s="6"/>
-      <c r="C249" s="6"/>
-      <c r="D249" s="6"/>
+      <c r="C249" s="7" t="s">
+        <v>468</v>
+      </c>
+      <c r="D249" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="5" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="B250" s="6"/>
       <c r="C250" s="7" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="D250" s="5" t="s">
         <v>6</v>
@@ -4990,11 +5106,11 @@
     </row>
     <row r="251">
       <c r="A251" s="5" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="B251" s="6"/>
       <c r="C251" s="7" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="D251" s="5" t="s">
         <v>6</v>
@@ -5002,11 +5118,11 @@
     </row>
     <row r="252">
       <c r="A252" s="5" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="B252" s="6"/>
       <c r="C252" s="7" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="D252" s="5" t="s">
         <v>6</v>
@@ -5014,11 +5130,11 @@
     </row>
     <row r="253">
       <c r="A253" s="5" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B253" s="6"/>
       <c r="C253" s="7" t="s">
-        <v>470</v>
+        <v>431</v>
       </c>
       <c r="D253" s="5" t="s">
         <v>6</v>
@@ -5026,11 +5142,11 @@
     </row>
     <row r="254">
       <c r="A254" s="5" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="B254" s="6"/>
       <c r="C254" s="7" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="D254" s="5" t="s">
         <v>6</v>
@@ -5038,11 +5154,11 @@
     </row>
     <row r="255">
       <c r="A255" s="5" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="B255" s="6"/>
       <c r="C255" s="7" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="D255" s="5" t="s">
         <v>6</v>
@@ -5050,11 +5166,11 @@
     </row>
     <row r="256">
       <c r="A256" s="5" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="B256" s="6"/>
       <c r="C256" s="7" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="D256" s="5" t="s">
         <v>6</v>
@@ -5062,11 +5178,11 @@
     </row>
     <row r="257">
       <c r="A257" s="5" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="B257" s="6"/>
       <c r="C257" s="7" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="D257" s="5" t="s">
         <v>6</v>
@@ -5074,11 +5190,11 @@
     </row>
     <row r="258">
       <c r="A258" s="5" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="B258" s="6"/>
       <c r="C258" s="7" t="s">
-        <v>429</v>
+        <v>485</v>
       </c>
       <c r="D258" s="5" t="s">
         <v>6</v>
@@ -5086,23 +5202,23 @@
     </row>
     <row r="259">
       <c r="A259" s="5" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="B259" s="6"/>
       <c r="C259" s="7" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="D259" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="19" t="s">
-        <v>482</v>
+      <c r="A260" s="5" t="s">
+        <v>488</v>
       </c>
       <c r="B260" s="6"/>
-      <c r="C260" s="20" t="s">
-        <v>483</v>
+      <c r="C260" s="7" t="s">
+        <v>489</v>
       </c>
       <c r="D260" s="5" t="s">
         <v>6</v>
@@ -5110,11 +5226,11 @@
     </row>
     <row r="261">
       <c r="A261" s="5" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="B261" s="6"/>
       <c r="C261" s="7" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="D261" s="5" t="s">
         <v>6</v>
@@ -5122,11 +5238,11 @@
     </row>
     <row r="262">
       <c r="A262" s="5" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="B262" s="6"/>
       <c r="C262" s="7" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="D262" s="5" t="s">
         <v>6</v>
@@ -5134,11 +5250,11 @@
     </row>
     <row r="263">
       <c r="A263" s="5" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="B263" s="6"/>
       <c r="C263" s="7" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
       <c r="D263" s="5" t="s">
         <v>6</v>
@@ -5146,11 +5262,11 @@
     </row>
     <row r="264">
       <c r="A264" s="5" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="B264" s="6"/>
       <c r="C264" s="7" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D264" s="5" t="s">
         <v>6</v>
@@ -5158,47 +5274,39 @@
     </row>
     <row r="265">
       <c r="A265" s="5" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="B265" s="6"/>
       <c r="C265" s="7" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="D265" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="266">
-      <c r="A266" s="19" t="s">
-        <v>494</v>
+      <c r="A266" s="5" t="s">
+        <v>496</v>
       </c>
       <c r="B266" s="6"/>
-      <c r="C266" s="20" t="s">
-        <v>495</v>
-      </c>
-      <c r="D266" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C266" s="6"/>
+      <c r="D266" s="6"/>
     </row>
     <row r="267">
       <c r="A267" s="5" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B267" s="6"/>
-      <c r="C267" s="7" t="s">
-        <v>485</v>
-      </c>
-      <c r="D267" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C267" s="6"/>
+      <c r="D267" s="6"/>
     </row>
     <row r="268">
       <c r="A268" s="5" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B268" s="6"/>
       <c r="C268" s="7" t="s">
-        <v>487</v>
+        <v>499</v>
       </c>
       <c r="D268" s="5" t="s">
         <v>6</v>
@@ -5206,11 +5314,11 @@
     </row>
     <row r="269">
       <c r="A269" s="5" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B269" s="6"/>
       <c r="C269" s="7" t="s">
-        <v>489</v>
+        <v>501</v>
       </c>
       <c r="D269" s="5" t="s">
         <v>6</v>
@@ -5218,11 +5326,11 @@
     </row>
     <row r="270">
       <c r="A270" s="5" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="B270" s="6"/>
       <c r="C270" s="7" t="s">
-        <v>491</v>
+        <v>503</v>
       </c>
       <c r="D270" s="5" t="s">
         <v>6</v>
@@ -5230,7 +5338,7 @@
     </row>
     <row r="271">
       <c r="A271" s="5" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="B271" s="6"/>
       <c r="C271" s="6"/>
@@ -5238,7 +5346,7 @@
     </row>
     <row r="272">
       <c r="A272" s="5" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="B272" s="6"/>
       <c r="C272" s="6"/>
@@ -5246,43 +5354,31 @@
     </row>
     <row r="273">
       <c r="A273" s="5" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="B273" s="6"/>
-      <c r="C273" s="7" t="s">
-        <v>503</v>
-      </c>
-      <c r="D273" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C273" s="6"/>
+      <c r="D273" s="6"/>
     </row>
     <row r="274">
       <c r="A274" s="5" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="B274" s="6"/>
-      <c r="C274" s="7" t="s">
-        <v>505</v>
-      </c>
-      <c r="D274" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C274" s="6"/>
+      <c r="D274" s="6"/>
     </row>
     <row r="275">
       <c r="A275" s="5" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B275" s="6"/>
-      <c r="C275" s="7" t="s">
-        <v>507</v>
-      </c>
-      <c r="D275" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C275" s="6"/>
+      <c r="D275" s="6"/>
     </row>
     <row r="276">
       <c r="A276" s="5" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B276" s="6"/>
       <c r="C276" s="6"/>
@@ -5290,7 +5386,7 @@
     </row>
     <row r="277">
       <c r="A277" s="5" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B277" s="6"/>
       <c r="C277" s="6"/>
@@ -5298,7 +5394,7 @@
     </row>
     <row r="278">
       <c r="A278" s="5" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B278" s="6"/>
       <c r="C278" s="6"/>
@@ -5306,7 +5402,7 @@
     </row>
     <row r="279">
       <c r="A279" s="5" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B279" s="6"/>
       <c r="C279" s="6"/>
@@ -5314,7 +5410,7 @@
     </row>
     <row r="280">
       <c r="A280" s="5" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B280" s="6"/>
       <c r="C280" s="6"/>
@@ -5322,7 +5418,7 @@
     </row>
     <row r="281">
       <c r="A281" s="5" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B281" s="6"/>
       <c r="C281" s="6"/>
@@ -5330,7 +5426,7 @@
     </row>
     <row r="282">
       <c r="A282" s="5" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B282" s="6"/>
       <c r="C282" s="6"/>
@@ -5338,133 +5434,219 @@
     </row>
     <row r="283">
       <c r="A283" s="5" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B283" s="6"/>
-      <c r="C283" s="6"/>
-      <c r="D283" s="6"/>
+      <c r="C283" s="7" t="s">
+        <v>517</v>
+      </c>
+      <c r="D283" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="5" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B284" s="6"/>
-      <c r="C284" s="6"/>
-      <c r="D284" s="6"/>
+      <c r="C284" s="7" t="s">
+        <v>519</v>
+      </c>
+      <c r="D284" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="285">
-      <c r="A285" s="5" t="s">
-        <v>517</v>
+      <c r="A285" s="20" t="s">
+        <v>520</v>
       </c>
       <c r="B285" s="6"/>
-      <c r="C285" s="6"/>
-      <c r="D285" s="6"/>
+      <c r="C285" s="12" t="s">
+        <v>521</v>
+      </c>
+      <c r="D285" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="286">
-      <c r="A286" s="5" t="s">
-        <v>518</v>
+      <c r="A286" s="20" t="s">
+        <v>522</v>
       </c>
       <c r="B286" s="6"/>
-      <c r="C286" s="6"/>
-      <c r="D286" s="6"/>
+      <c r="C286" s="12" t="s">
+        <v>523</v>
+      </c>
+      <c r="D286" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="287">
-      <c r="A287" s="5" t="s">
-        <v>519</v>
+      <c r="A287" s="20" t="s">
+        <v>524</v>
       </c>
       <c r="B287" s="6"/>
-      <c r="C287" s="6"/>
-      <c r="D287" s="6"/>
+      <c r="C287" s="12" t="s">
+        <v>525</v>
+      </c>
+      <c r="D287" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="288">
-      <c r="A288" s="5" t="s">
-        <v>520</v>
+      <c r="A288" s="20" t="s">
+        <v>526</v>
       </c>
       <c r="B288" s="6"/>
-      <c r="C288" s="7" t="s">
-        <v>521</v>
+      <c r="C288" s="12" t="s">
+        <v>527</v>
       </c>
       <c r="D288" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="289">
-      <c r="A289" s="5" t="s">
-        <v>522</v>
+      <c r="A289" s="20" t="s">
+        <v>528</v>
       </c>
       <c r="B289" s="6"/>
-      <c r="C289" s="7" t="s">
-        <v>523</v>
+      <c r="C289" s="12" t="s">
+        <v>529</v>
       </c>
       <c r="D289" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="290">
-      <c r="A290" s="6"/>
+      <c r="A290" s="20" t="s">
+        <v>530</v>
+      </c>
       <c r="B290" s="6"/>
-      <c r="C290" s="6"/>
-      <c r="D290" s="6"/>
+      <c r="C290" s="12" t="s">
+        <v>531</v>
+      </c>
+      <c r="D290" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="291">
-      <c r="A291" s="6"/>
+      <c r="A291" s="20" t="s">
+        <v>532</v>
+      </c>
       <c r="B291" s="6"/>
-      <c r="C291" s="6"/>
-      <c r="D291" s="6"/>
+      <c r="C291" s="12" t="s">
+        <v>533</v>
+      </c>
+      <c r="D291" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="292">
-      <c r="A292" s="6"/>
+      <c r="A292" s="20" t="s">
+        <v>534</v>
+      </c>
       <c r="B292" s="6"/>
-      <c r="C292" s="6"/>
-      <c r="D292" s="6"/>
+      <c r="C292" s="12" t="s">
+        <v>535</v>
+      </c>
+      <c r="D292" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="293">
-      <c r="A293" s="6"/>
+      <c r="A293" s="21" t="s">
+        <v>536</v>
+      </c>
       <c r="B293" s="6"/>
-      <c r="C293" s="6"/>
-      <c r="D293" s="6"/>
+      <c r="C293" s="12" t="s">
+        <v>537</v>
+      </c>
+      <c r="D293" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="294">
-      <c r="A294" s="6"/>
+      <c r="A294" s="22" t="s">
+        <v>538</v>
+      </c>
       <c r="B294" s="6"/>
-      <c r="C294" s="6"/>
-      <c r="D294" s="6"/>
+      <c r="C294" s="12" t="s">
+        <v>539</v>
+      </c>
+      <c r="D294" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="295">
-      <c r="A295" s="6"/>
+      <c r="A295" s="22" t="s">
+        <v>540</v>
+      </c>
       <c r="B295" s="6"/>
-      <c r="C295" s="6"/>
-      <c r="D295" s="6"/>
+      <c r="C295" s="12" t="s">
+        <v>541</v>
+      </c>
+      <c r="D295" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="296">
-      <c r="A296" s="6"/>
+      <c r="A296" s="22" t="s">
+        <v>542</v>
+      </c>
       <c r="B296" s="6"/>
-      <c r="C296" s="6"/>
-      <c r="D296" s="6"/>
+      <c r="C296" s="12" t="s">
+        <v>543</v>
+      </c>
+      <c r="D296" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="297">
-      <c r="A297" s="6"/>
+      <c r="A297" s="22" t="s">
+        <v>544</v>
+      </c>
       <c r="B297" s="6"/>
-      <c r="C297" s="6"/>
-      <c r="D297" s="6"/>
+      <c r="C297" s="12" t="s">
+        <v>545</v>
+      </c>
+      <c r="D297" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="298">
-      <c r="A298" s="6"/>
+      <c r="A298" s="22" t="s">
+        <v>546</v>
+      </c>
       <c r="B298" s="6"/>
-      <c r="C298" s="6"/>
-      <c r="D298" s="6"/>
+      <c r="C298" s="12" t="s">
+        <v>547</v>
+      </c>
+      <c r="D298" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="299">
-      <c r="A299" s="6"/>
+      <c r="A299" s="20" t="s">
+        <v>548</v>
+      </c>
       <c r="B299" s="6"/>
-      <c r="C299" s="6"/>
-      <c r="D299" s="6"/>
+      <c r="C299" s="12" t="s">
+        <v>549</v>
+      </c>
+      <c r="D299" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="300">
-      <c r="A300" s="6"/>
+      <c r="A300" s="20" t="s">
+        <v>550</v>
+      </c>
       <c r="B300" s="6"/>
-      <c r="C300" s="6"/>
-      <c r="D300" s="6"/>
+      <c r="C300" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="D300" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="6"/>
@@ -10350,27 +10532,15 @@
       <c r="C1114" s="6"/>
       <c r="D1114" s="6"/>
     </row>
-    <row r="1115">
-      <c r="A1115" s="6"/>
-      <c r="B1115" s="6"/>
-      <c r="C1115" s="6"/>
-      <c r="D1115" s="6"/>
-    </row>
-    <row r="1116">
-      <c r="A1116" s="6"/>
-      <c r="B1116" s="6"/>
-      <c r="C1116" s="6"/>
-      <c r="D1116" s="6"/>
-    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D243 D250:D270 D273:D275 D288:D289">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D265 D268:D270 D283:D300">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="A77"/>
-    <hyperlink r:id="rId2" ref="A172"/>
+    <hyperlink r:id="rId2" ref="A173"/>
   </hyperlinks>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
(WIP) female info edition
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="580">
   <si>
     <t>Key</t>
   </si>
@@ -1427,6 +1427,12 @@
     <t>Physical Disabilities</t>
   </si>
   <si>
+    <t>profile_advanced_info.physical_disability.description</t>
+  </si>
+  <si>
+    <t>If you suffer from any disability, Circular will calibrate more realistic goals to account for your condition.</t>
+  </si>
+  <si>
     <t>profile_advanced_info.physical_disability.none</t>
   </si>
   <si>
@@ -1538,6 +1544,18 @@
     <t>profile_advanced_info.sleeper_type.night</t>
   </si>
   <si>
+    <t>profile_advanced_info.period_tracking_info</t>
+  </si>
+  <si>
+    <t>Period tracking</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.title</t>
+  </si>
+  <si>
+    <t>Fertility State</t>
+  </si>
+  <si>
     <t>profile_advanced_info.fertility_state.menstrual_cycle</t>
   </si>
   <si>
@@ -1556,40 +1574,107 @@
     <t>Perimenopause</t>
   </si>
   <si>
+    <t>profile_advanced_info.cycle_length.title</t>
+  </si>
+  <si>
+    <t>Cycle Length</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.title</t>
+  </si>
+  <si>
+    <t>Birth Control Type</t>
+  </si>
+  <si>
+    <t>header.birth_control</t>
+  </si>
+  <si>
+    <t>BIRTH CONTROL TYPE</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.selection_invitation</t>
+  </si>
+  <si>
+    <t>What is your birth control type?
+Select from below:</t>
+  </si>
+  <si>
     <t>profile_advanced_info.birth_control.none</t>
   </si>
   <si>
     <t>profile_advanced_info.birth_control.pills</t>
   </si>
   <si>
+    <t>Pills</t>
+  </si>
+  <si>
     <t>profile_advanced_info.birth_control.condoms</t>
   </si>
   <si>
+    <t>Condoms</t>
+  </si>
+  <si>
     <t>profile_advanced_info.birth_control.vaginal_ring</t>
   </si>
   <si>
+    <t>Vaginal Ring</t>
+  </si>
+  <si>
     <t>profile_advanced_info.birth_control.patch</t>
   </si>
   <si>
+    <t>Patch</t>
+  </si>
+  <si>
     <t>profile_advanced_info.birth_control.iud</t>
   </si>
   <si>
+    <t>IUD</t>
+  </si>
+  <si>
     <t>profile_advanced_info.birth_control.implant</t>
   </si>
   <si>
+    <t>Implant</t>
+  </si>
+  <si>
     <t>profile_advanced_info.birth_control.fertility_awareness</t>
   </si>
   <si>
+    <t>Fertility Awareness Method</t>
+  </si>
+  <si>
     <t>profile_advanced_info.birth_control.other</t>
   </si>
   <si>
+    <t>profile_advanced_info.pill_pack_format.title</t>
+  </si>
+  <si>
+    <t>Pill Pack Format</t>
+  </si>
+  <si>
     <t>profile_advanced_info.pill_pack_format.days_28</t>
   </si>
   <si>
+    <t>28 days regimen</t>
+  </si>
+  <si>
     <t>profile_advanced_info.pill_pack_format.days_24</t>
   </si>
   <si>
+    <t>24 days regimen</t>
+  </si>
+  <si>
     <t>profile_advanced_info.pill_pack_format.days_21</t>
+  </si>
+  <si>
+    <t>21 days regimen</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.conceiving.title</t>
+  </si>
+  <si>
+    <t>Conceiving?</t>
   </si>
   <si>
     <t>profile_advanced_info.open_for_napping.title</t>
@@ -1779,7 +1864,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1840,6 +1925,9 @@
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
@@ -5045,11 +5133,11 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="5" t="s">
+      <c r="A246" s="20" t="s">
         <v>461</v>
       </c>
-      <c r="B246" s="6"/>
-      <c r="C246" s="7" t="s">
+      <c r="B246" s="21"/>
+      <c r="C246" s="12" t="s">
         <v>462</v>
       </c>
       <c r="D246" s="5" t="s">
@@ -5134,7 +5222,7 @@
       </c>
       <c r="B253" s="6"/>
       <c r="C253" s="7" t="s">
-        <v>431</v>
+        <v>476</v>
       </c>
       <c r="D253" s="5" t="s">
         <v>6</v>
@@ -5142,11 +5230,11 @@
     </row>
     <row r="254">
       <c r="A254" s="5" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B254" s="6"/>
       <c r="C254" s="7" t="s">
-        <v>477</v>
+        <v>431</v>
       </c>
       <c r="D254" s="5" t="s">
         <v>6</v>
@@ -5242,7 +5330,7 @@
       </c>
       <c r="B262" s="6"/>
       <c r="C262" s="7" t="s">
-        <v>481</v>
+        <v>493</v>
       </c>
       <c r="D262" s="5" t="s">
         <v>6</v>
@@ -5250,7 +5338,7 @@
     </row>
     <row r="263">
       <c r="A263" s="5" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B263" s="6"/>
       <c r="C263" s="7" t="s">
@@ -5262,7 +5350,7 @@
     </row>
     <row r="264">
       <c r="A264" s="5" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B264" s="6"/>
       <c r="C264" s="7" t="s">
@@ -5274,7 +5362,7 @@
     </row>
     <row r="265">
       <c r="A265" s="5" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B265" s="6"/>
       <c r="C265" s="7" t="s">
@@ -5286,15 +5374,19 @@
     </row>
     <row r="266">
       <c r="A266" s="5" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B266" s="6"/>
-      <c r="C266" s="6"/>
-      <c r="D266" s="6"/>
+      <c r="C266" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="D266" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="5" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B267" s="6"/>
       <c r="C267" s="6"/>
@@ -5302,22 +5394,18 @@
     </row>
     <row r="268">
       <c r="A268" s="5" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B268" s="6"/>
-      <c r="C268" s="7" t="s">
-        <v>499</v>
-      </c>
-      <c r="D268" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C268" s="6"/>
+      <c r="D268" s="6"/>
     </row>
     <row r="269">
-      <c r="A269" s="5" t="s">
+      <c r="A269" s="20" t="s">
         <v>500</v>
       </c>
       <c r="B269" s="6"/>
-      <c r="C269" s="7" t="s">
+      <c r="C269" s="12" t="s">
         <v>501</v>
       </c>
       <c r="D269" s="5" t="s">
@@ -5325,11 +5413,11 @@
       </c>
     </row>
     <row r="270">
-      <c r="A270" s="5" t="s">
+      <c r="A270" s="20" t="s">
         <v>502</v>
       </c>
       <c r="B270" s="6"/>
-      <c r="C270" s="7" t="s">
+      <c r="C270" s="12" t="s">
         <v>503</v>
       </c>
       <c r="D270" s="5" t="s">
@@ -5341,104 +5429,152 @@
         <v>504</v>
       </c>
       <c r="B271" s="6"/>
-      <c r="C271" s="6"/>
-      <c r="D271" s="6"/>
+      <c r="C271" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="D271" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="5" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B272" s="6"/>
-      <c r="C272" s="6"/>
-      <c r="D272" s="6"/>
+      <c r="C272" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="D272" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="5" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B273" s="6"/>
-      <c r="C273" s="6"/>
-      <c r="D273" s="6"/>
+      <c r="C273" s="7" t="s">
+        <v>509</v>
+      </c>
+      <c r="D273" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="274">
-      <c r="A274" s="5" t="s">
-        <v>507</v>
+      <c r="A274" s="20" t="s">
+        <v>510</v>
       </c>
       <c r="B274" s="6"/>
-      <c r="C274" s="6"/>
-      <c r="D274" s="6"/>
+      <c r="C274" s="12" t="s">
+        <v>511</v>
+      </c>
+      <c r="D274" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="275">
-      <c r="A275" s="5" t="s">
-        <v>508</v>
+      <c r="A275" s="20" t="s">
+        <v>512</v>
       </c>
       <c r="B275" s="6"/>
-      <c r="C275" s="6"/>
-      <c r="D275" s="6"/>
+      <c r="C275" s="12" t="s">
+        <v>513</v>
+      </c>
+      <c r="D275" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="276">
-      <c r="A276" s="5" t="s">
-        <v>509</v>
+      <c r="A276" s="20" t="s">
+        <v>514</v>
       </c>
       <c r="B276" s="6"/>
-      <c r="C276" s="6"/>
-      <c r="D276" s="6"/>
+      <c r="C276" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="D276" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="277">
-      <c r="A277" s="5" t="s">
-        <v>510</v>
+      <c r="A277" s="20" t="s">
+        <v>516</v>
       </c>
       <c r="B277" s="6"/>
-      <c r="C277" s="6"/>
-      <c r="D277" s="6"/>
+      <c r="C277" s="12" t="s">
+        <v>517</v>
+      </c>
+      <c r="D277" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="5" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="B278" s="6"/>
-      <c r="C278" s="6"/>
-      <c r="D278" s="6"/>
+      <c r="C278" s="12" t="s">
+        <v>483</v>
+      </c>
+      <c r="D278" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="5" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
       <c r="B279" s="6"/>
-      <c r="C279" s="6"/>
-      <c r="D279" s="6"/>
+      <c r="C279" s="12" t="s">
+        <v>520</v>
+      </c>
+      <c r="D279" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="5" t="s">
-        <v>513</v>
+        <v>521</v>
       </c>
       <c r="B280" s="6"/>
-      <c r="C280" s="6"/>
-      <c r="D280" s="6"/>
+      <c r="C280" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="D280" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="5" t="s">
-        <v>514</v>
+        <v>523</v>
       </c>
       <c r="B281" s="6"/>
-      <c r="C281" s="6"/>
-      <c r="D281" s="6"/>
+      <c r="C281" s="12" t="s">
+        <v>524</v>
+      </c>
+      <c r="D281" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="5" t="s">
-        <v>515</v>
+        <v>525</v>
       </c>
       <c r="B282" s="6"/>
-      <c r="C282" s="6"/>
-      <c r="D282" s="6"/>
+      <c r="C282" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D282" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="5" t="s">
-        <v>516</v>
+        <v>527</v>
       </c>
       <c r="B283" s="6"/>
-      <c r="C283" s="7" t="s">
-        <v>517</v>
+      <c r="C283" s="12" t="s">
+        <v>528</v>
       </c>
       <c r="D283" s="5" t="s">
         <v>6</v>
@@ -5446,35 +5582,35 @@
     </row>
     <row r="284">
       <c r="A284" s="5" t="s">
-        <v>518</v>
+        <v>529</v>
       </c>
       <c r="B284" s="6"/>
-      <c r="C284" s="7" t="s">
-        <v>519</v>
+      <c r="C284" s="12" t="s">
+        <v>530</v>
       </c>
       <c r="D284" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="285">
-      <c r="A285" s="20" t="s">
-        <v>520</v>
+      <c r="A285" s="5" t="s">
+        <v>531</v>
       </c>
       <c r="B285" s="6"/>
       <c r="C285" s="12" t="s">
-        <v>521</v>
+        <v>532</v>
       </c>
       <c r="D285" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="286">
-      <c r="A286" s="20" t="s">
-        <v>522</v>
+      <c r="A286" s="5" t="s">
+        <v>533</v>
       </c>
       <c r="B286" s="6"/>
       <c r="C286" s="12" t="s">
-        <v>523</v>
+        <v>431</v>
       </c>
       <c r="D286" s="5" t="s">
         <v>6</v>
@@ -5482,47 +5618,47 @@
     </row>
     <row r="287">
       <c r="A287" s="20" t="s">
-        <v>524</v>
+        <v>534</v>
       </c>
       <c r="B287" s="6"/>
       <c r="C287" s="12" t="s">
-        <v>525</v>
+        <v>535</v>
       </c>
       <c r="D287" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="288">
-      <c r="A288" s="20" t="s">
-        <v>526</v>
+      <c r="A288" s="5" t="s">
+        <v>536</v>
       </c>
       <c r="B288" s="6"/>
       <c r="C288" s="12" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="D288" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="289">
-      <c r="A289" s="20" t="s">
-        <v>528</v>
+      <c r="A289" s="5" t="s">
+        <v>538</v>
       </c>
       <c r="B289" s="6"/>
       <c r="C289" s="12" t="s">
-        <v>529</v>
+        <v>539</v>
       </c>
       <c r="D289" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="290">
-      <c r="A290" s="20" t="s">
-        <v>530</v>
+      <c r="A290" s="5" t="s">
+        <v>540</v>
       </c>
       <c r="B290" s="6"/>
       <c r="C290" s="12" t="s">
-        <v>531</v>
+        <v>541</v>
       </c>
       <c r="D290" s="5" t="s">
         <v>6</v>
@@ -5530,95 +5666,95 @@
     </row>
     <row r="291">
       <c r="A291" s="20" t="s">
-        <v>532</v>
+        <v>542</v>
       </c>
       <c r="B291" s="6"/>
       <c r="C291" s="12" t="s">
-        <v>533</v>
+        <v>543</v>
       </c>
       <c r="D291" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="292">
-      <c r="A292" s="20" t="s">
-        <v>534</v>
+      <c r="A292" s="5" t="s">
+        <v>544</v>
       </c>
       <c r="B292" s="6"/>
-      <c r="C292" s="12" t="s">
-        <v>535</v>
+      <c r="C292" s="7" t="s">
+        <v>545</v>
       </c>
       <c r="D292" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="21" t="s">
-        <v>536</v>
+      <c r="A293" s="5" t="s">
+        <v>546</v>
       </c>
       <c r="B293" s="6"/>
-      <c r="C293" s="12" t="s">
-        <v>537</v>
+      <c r="C293" s="7" t="s">
+        <v>547</v>
       </c>
       <c r="D293" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="294">
-      <c r="A294" s="22" t="s">
-        <v>538</v>
+      <c r="A294" s="20" t="s">
+        <v>548</v>
       </c>
       <c r="B294" s="6"/>
       <c r="C294" s="12" t="s">
-        <v>539</v>
+        <v>549</v>
       </c>
       <c r="D294" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="22" t="s">
-        <v>540</v>
+      <c r="A295" s="20" t="s">
+        <v>550</v>
       </c>
       <c r="B295" s="6"/>
       <c r="C295" s="12" t="s">
-        <v>541</v>
+        <v>551</v>
       </c>
       <c r="D295" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="296">
-      <c r="A296" s="22" t="s">
-        <v>542</v>
+      <c r="A296" s="20" t="s">
+        <v>552</v>
       </c>
       <c r="B296" s="6"/>
       <c r="C296" s="12" t="s">
-        <v>543</v>
+        <v>553</v>
       </c>
       <c r="D296" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="297">
-      <c r="A297" s="22" t="s">
-        <v>544</v>
+      <c r="A297" s="20" t="s">
+        <v>554</v>
       </c>
       <c r="B297" s="6"/>
       <c r="C297" s="12" t="s">
-        <v>545</v>
+        <v>555</v>
       </c>
       <c r="D297" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="298">
-      <c r="A298" s="22" t="s">
-        <v>546</v>
+      <c r="A298" s="20" t="s">
+        <v>556</v>
       </c>
       <c r="B298" s="6"/>
       <c r="C298" s="12" t="s">
-        <v>547</v>
+        <v>557</v>
       </c>
       <c r="D298" s="5" t="s">
         <v>6</v>
@@ -5626,11 +5762,11 @@
     </row>
     <row r="299">
       <c r="A299" s="20" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="B299" s="6"/>
       <c r="C299" s="12" t="s">
-        <v>549</v>
+        <v>559</v>
       </c>
       <c r="D299" s="5" t="s">
         <v>6</v>
@@ -5638,69 +5774,123 @@
     </row>
     <row r="300">
       <c r="A300" s="20" t="s">
-        <v>550</v>
+        <v>560</v>
       </c>
       <c r="B300" s="6"/>
       <c r="C300" s="12" t="s">
-        <v>551</v>
+        <v>561</v>
       </c>
       <c r="D300" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="301">
-      <c r="A301" s="6"/>
+      <c r="A301" s="20" t="s">
+        <v>562</v>
+      </c>
       <c r="B301" s="6"/>
-      <c r="C301" s="6"/>
-      <c r="D301" s="6"/>
+      <c r="C301" s="12" t="s">
+        <v>563</v>
+      </c>
+      <c r="D301" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="302">
-      <c r="A302" s="6"/>
+      <c r="A302" s="22" t="s">
+        <v>564</v>
+      </c>
       <c r="B302" s="6"/>
-      <c r="C302" s="6"/>
-      <c r="D302" s="6"/>
+      <c r="C302" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="D302" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="303">
-      <c r="A303" s="6"/>
+      <c r="A303" s="23" t="s">
+        <v>566</v>
+      </c>
       <c r="B303" s="6"/>
-      <c r="C303" s="6"/>
-      <c r="D303" s="6"/>
+      <c r="C303" s="12" t="s">
+        <v>567</v>
+      </c>
+      <c r="D303" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="304">
-      <c r="A304" s="6"/>
+      <c r="A304" s="23" t="s">
+        <v>568</v>
+      </c>
       <c r="B304" s="6"/>
-      <c r="C304" s="6"/>
-      <c r="D304" s="6"/>
+      <c r="C304" s="12" t="s">
+        <v>569</v>
+      </c>
+      <c r="D304" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="305">
-      <c r="A305" s="6"/>
+      <c r="A305" s="23" t="s">
+        <v>570</v>
+      </c>
       <c r="B305" s="6"/>
-      <c r="C305" s="6"/>
-      <c r="D305" s="6"/>
+      <c r="C305" s="12" t="s">
+        <v>571</v>
+      </c>
+      <c r="D305" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="306">
-      <c r="A306" s="6"/>
+      <c r="A306" s="23" t="s">
+        <v>572</v>
+      </c>
       <c r="B306" s="6"/>
-      <c r="C306" s="6"/>
-      <c r="D306" s="6"/>
+      <c r="C306" s="12" t="s">
+        <v>573</v>
+      </c>
+      <c r="D306" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="307">
-      <c r="A307" s="6"/>
+      <c r="A307" s="23" t="s">
+        <v>574</v>
+      </c>
       <c r="B307" s="6"/>
-      <c r="C307" s="6"/>
-      <c r="D307" s="6"/>
+      <c r="C307" s="12" t="s">
+        <v>575</v>
+      </c>
+      <c r="D307" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="308">
-      <c r="A308" s="6"/>
+      <c r="A308" s="20" t="s">
+        <v>576</v>
+      </c>
       <c r="B308" s="6"/>
-      <c r="C308" s="6"/>
-      <c r="D308" s="6"/>
+      <c r="C308" s="12" t="s">
+        <v>577</v>
+      </c>
+      <c r="D308" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="309">
-      <c r="A309" s="6"/>
+      <c r="A309" s="20" t="s">
+        <v>578</v>
+      </c>
       <c r="B309" s="6"/>
-      <c r="C309" s="6"/>
-      <c r="D309" s="6"/>
+      <c r="C309" s="12" t="s">
+        <v>579</v>
+      </c>
+      <c r="D309" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="6"/>
@@ -10532,9 +10722,63 @@
       <c r="C1114" s="6"/>
       <c r="D1114" s="6"/>
     </row>
+    <row r="1115">
+      <c r="A1115" s="6"/>
+      <c r="B1115" s="6"/>
+      <c r="C1115" s="6"/>
+      <c r="D1115" s="6"/>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="6"/>
+      <c r="B1116" s="6"/>
+      <c r="C1116" s="6"/>
+      <c r="D1116" s="6"/>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="6"/>
+      <c r="B1117" s="6"/>
+      <c r="C1117" s="6"/>
+      <c r="D1117" s="6"/>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="6"/>
+      <c r="B1118" s="6"/>
+      <c r="C1118" s="6"/>
+      <c r="D1118" s="6"/>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="6"/>
+      <c r="B1119" s="6"/>
+      <c r="C1119" s="6"/>
+      <c r="D1119" s="6"/>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="6"/>
+      <c r="B1120" s="6"/>
+      <c r="C1120" s="6"/>
+      <c r="D1120" s="6"/>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="6"/>
+      <c r="B1121" s="6"/>
+      <c r="C1121" s="6"/>
+      <c r="D1121" s="6"/>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="6"/>
+      <c r="B1122" s="6"/>
+      <c r="C1122" s="6"/>
+      <c r="D1122" s="6"/>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="6"/>
+      <c r="B1123" s="6"/>
+      <c r="C1123" s="6"/>
+      <c r="D1123" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D265 D268:D270 D283:D300">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D266 D269:D309">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
BirthControl edition + Comparative info bottom sheet
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="933" uniqueCount="585">
   <si>
     <t>Key</t>
   </si>
@@ -1725,6 +1725,16 @@
     <t>😮‍💨 VO2 Max</t>
   </si>
   <si>
+    <t>profile_advanced_info.comparative_info.title</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.comparative_info.description</t>
+  </si>
+  <si>
+    <t>In this section, you can see comparative information. The values you can read are healthy and average values for your physiology. This information takes into account your gender, age and condition. You can compare to these values to evaluate where you position yourself. 
+⚠️ However, please note that relying on population-level averages has its limits. That’s because metrics vary significantly between different people. What’s normal and healthy for one individual may not be for another.</t>
+  </si>
+  <si>
     <t>profile_advanced_info.bmi.title</t>
   </si>
   <si>
@@ -1771,6 +1781,12 @@
   </si>
   <si>
     <t>Night erratic type</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.stride.title</t>
+  </si>
+  <si>
+    <t>Stride</t>
   </si>
   <si>
     <t>alarm.weekdays</t>
@@ -1864,7 +1880,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1934,6 +1950,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5778,7 +5797,7 @@
       </c>
       <c r="B300" s="6"/>
       <c r="C300" s="12" t="s">
-        <v>561</v>
+        <v>555</v>
       </c>
       <c r="D300" s="5" t="s">
         <v>6</v>
@@ -5786,47 +5805,47 @@
     </row>
     <row r="301">
       <c r="A301" s="20" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B301" s="6"/>
       <c r="C301" s="12" t="s">
+        <v>562</v>
+      </c>
+      <c r="D301" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="20" t="s">
         <v>563</v>
-      </c>
-      <c r="D301" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" s="22" t="s">
-        <v>564</v>
       </c>
       <c r="B302" s="6"/>
       <c r="C302" s="12" t="s">
+        <v>564</v>
+      </c>
+      <c r="D302" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="20" t="s">
         <v>565</v>
-      </c>
-      <c r="D302" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" s="23" t="s">
-        <v>566</v>
       </c>
       <c r="B303" s="6"/>
       <c r="C303" s="12" t="s">
+        <v>566</v>
+      </c>
+      <c r="D303" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="22" t="s">
         <v>567</v>
-      </c>
-      <c r="D303" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" s="23" t="s">
-        <v>568</v>
       </c>
       <c r="B304" s="6"/>
       <c r="C304" s="12" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="D304" s="5" t="s">
         <v>6</v>
@@ -5834,11 +5853,11 @@
     </row>
     <row r="305">
       <c r="A305" s="23" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B305" s="6"/>
       <c r="C305" s="12" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D305" s="5" t="s">
         <v>6</v>
@@ -5846,11 +5865,11 @@
     </row>
     <row r="306">
       <c r="A306" s="23" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B306" s="6"/>
       <c r="C306" s="12" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D306" s="5" t="s">
         <v>6</v>
@@ -5858,57 +5877,75 @@
     </row>
     <row r="307">
       <c r="A307" s="23" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B307" s="6"/>
       <c r="C307" s="12" t="s">
+        <v>574</v>
+      </c>
+      <c r="D307" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="23" t="s">
         <v>575</v>
-      </c>
-      <c r="D307" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" s="20" t="s">
-        <v>576</v>
       </c>
       <c r="B308" s="6"/>
       <c r="C308" s="12" t="s">
+        <v>576</v>
+      </c>
+      <c r="D308" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="23" t="s">
         <v>577</v>
-      </c>
-      <c r="D308" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" s="20" t="s">
-        <v>578</v>
       </c>
       <c r="B309" s="6"/>
       <c r="C309" s="12" t="s">
+        <v>578</v>
+      </c>
+      <c r="D309" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="24" t="s">
         <v>579</v>
       </c>
-      <c r="D309" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" s="6"/>
       <c r="B310" s="6"/>
-      <c r="C310" s="6"/>
-      <c r="D310" s="6"/>
+      <c r="C310" s="12" t="s">
+        <v>580</v>
+      </c>
+      <c r="D310" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="311">
-      <c r="A311" s="6"/>
+      <c r="A311" s="20" t="s">
+        <v>581</v>
+      </c>
       <c r="B311" s="6"/>
-      <c r="C311" s="6"/>
-      <c r="D311" s="6"/>
+      <c r="C311" s="12" t="s">
+        <v>582</v>
+      </c>
+      <c r="D311" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="312">
-      <c r="A312" s="6"/>
+      <c r="A312" s="20" t="s">
+        <v>583</v>
+      </c>
       <c r="B312" s="6"/>
-      <c r="C312" s="6"/>
-      <c r="D312" s="6"/>
+      <c r="C312" s="12" t="s">
+        <v>584</v>
+      </c>
+      <c r="D312" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="6"/>
@@ -10776,9 +10813,27 @@
       <c r="C1123" s="6"/>
       <c r="D1123" s="6"/>
     </row>
+    <row r="1124">
+      <c r="A1124" s="6"/>
+      <c r="B1124" s="6"/>
+      <c r="C1124" s="6"/>
+      <c r="D1124" s="6"/>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="6"/>
+      <c r="B1125" s="6"/>
+      <c r="C1125" s="6"/>
+      <c r="D1125" s="6"/>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="6"/>
+      <c r="B1126" s="6"/>
+      <c r="C1126" s="6"/>
+      <c r="D1126" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D266 D269:D309">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D266 D269:D312">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
merge master and resolve conflict
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="510">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="580">
   <si>
     <t>Key</t>
   </si>
@@ -424,6 +424,12 @@
   </si>
   <si>
     <t>no</t>
+  </si>
+  <si>
+    <t>global.not_enough_data</t>
+  </si>
+  <si>
+    <t>Not enough information</t>
   </si>
   <si>
     <t>home.sync.syncing</t>
@@ -972,6 +978,12 @@
   </si>
   <si>
     <t>Repeat</t>
+  </si>
+  <si>
+    <t>alarm.new.repeat.description</t>
+  </si>
+  <si>
+    <t>Choose on what day(s) you want this alarm to go off.</t>
   </si>
   <si>
     <t>onboarding.wear.title</t>
@@ -1238,6 +1250,12 @@
     <t>Snooze</t>
   </si>
   <si>
+    <t>alarm.new.snooze.description</t>
+  </si>
+  <si>
+    <t>Time interval between each snooze. Press the ring’s button once to snooze. Press it twice to completely stop the vibrations.</t>
+  </si>
+  <si>
     <t>alarm.new.snooze.screen_title</t>
   </si>
   <si>
@@ -1274,12 +1292,30 @@
     <t>Smart Snooze</t>
   </si>
   <si>
+    <t>alarm.new.smart_snooze.description</t>
+  </si>
+  <si>
+    <t>Time interval between each snooze. Vibrations will stop automatically once the ring has detected that you’re up and walking.</t>
+  </si>
+  <si>
+    <t>alarm.new.snooze.smart_switch</t>
+  </si>
+  <si>
+    <t>Make it smart</t>
+  </si>
+  <si>
     <t>alarm.new.smart_alarm.title</t>
   </si>
   <si>
     <t>Smart Alarm</t>
   </si>
   <si>
+    <t>alarm.new.smart_alarm.description</t>
+  </si>
+  <si>
+    <t>Maximum time window for smart alarm to ring before selected wake up time. More time means more chances to get the lightest wake up.</t>
+  </si>
+  <si>
     <t>alarm.new.warning.title</t>
   </si>
   <si>
@@ -1385,200 +1421,375 @@
     <t>Night Worker</t>
   </si>
   <si>
+    <t>profile_advanced_info.physical_disability.title</t>
+  </si>
+  <si>
+    <t>Physical Disabilities</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.description</t>
+  </si>
+  <si>
+    <t>If you suffer from any disability, Circular will calibrate more realistic goals to account for your condition.</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.none</t>
+  </si>
+  <si>
+    <t>No physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.moderate</t>
+  </si>
+  <si>
+    <t>Moderate physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.total</t>
+  </si>
+  <si>
+    <t>Total physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.title</t>
+  </si>
+  <si>
+    <t>Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.none</t>
+  </si>
+  <si>
+    <t>No Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.insomnia</t>
+  </si>
+  <si>
+    <t>Insomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.hypersomnia</t>
+  </si>
+  <si>
+    <t>Hypersomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.other</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.title</t>
+  </si>
+  <si>
+    <t>Sleep Aid</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.description</t>
+  </si>
+  <si>
+    <t>Sleeping pills include any prescription sleep drugs.</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.none</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.daily</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.weekly</t>
+  </si>
+  <si>
+    <t>Weekly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeping_pills.monthly</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.title</t>
+  </si>
+  <si>
+    <t>Sleep supplements</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.description</t>
+  </si>
+  <si>
+    <t>Dietary supplements include melatonin, herbs, magnesium, etc...</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.none</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.daily</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.weekly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.dietary_supplements.monthly</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeper_type.light</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleeper_type.night</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.period_tracking_info</t>
+  </si>
+  <si>
+    <t>Period tracking</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.title</t>
+  </si>
+  <si>
+    <t>Fertility State</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.menstrual_cycle</t>
+  </si>
+  <si>
+    <t>Menstrual cycle</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.menopause</t>
+  </si>
+  <si>
+    <t>Menopause</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.fertility_state.perimenopause</t>
+  </si>
+  <si>
+    <t>Perimenopause</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.cycle_length.title</t>
+  </si>
+  <si>
+    <t>Cycle Length</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.title</t>
+  </si>
+  <si>
+    <t>Birth Control Type</t>
+  </si>
+  <si>
+    <t>header.birth_control</t>
+  </si>
+  <si>
+    <t>BIRTH CONTROL TYPE</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.selection_invitation</t>
+  </si>
+  <si>
+    <t>What is your birth control type?
+Select from below:</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.none</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.pills</t>
+  </si>
+  <si>
+    <t>Pills</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.condoms</t>
+  </si>
+  <si>
+    <t>Condoms</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.vaginal_ring</t>
+  </si>
+  <si>
+    <t>Vaginal Ring</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.patch</t>
+  </si>
+  <si>
+    <t>Patch</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.iud</t>
+  </si>
+  <si>
+    <t>IUD</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.implant</t>
+  </si>
+  <si>
+    <t>Implant</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.fertility_awareness</t>
+  </si>
+  <si>
+    <t>Fertility Awareness Method</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.birth_control.other</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.title</t>
+  </si>
+  <si>
+    <t>Pill Pack Format</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_28</t>
+  </si>
+  <si>
+    <t>28 days regimen</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_24</t>
+  </si>
+  <si>
+    <t>24 days regimen</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.pill_pack_format.days_21</t>
+  </si>
+  <si>
+    <t>21 days regimen</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.conceiving.title</t>
+  </si>
+  <si>
+    <t>Conceiving?</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.open_for_napping.title</t>
+  </si>
+  <si>
+    <t>Open for Napping</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.unknown_option</t>
+  </si>
+  <si>
+    <t>Unknown option</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.title</t>
+  </si>
+  <si>
+    <t>Heart Rate</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.maximum</t>
+  </si>
+  <si>
+    <t>🔝 Maximum</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.sport_target</t>
+  </si>
+  <si>
+    <t>🎯 Sport Target</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.comparative_title</t>
+  </si>
+  <si>
+    <t>Comparative Info</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.rhr</t>
+  </si>
+  <si>
+    <t>😴 RHR</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.heart_rate.vo2_max</t>
+  </si>
+  <si>
+    <t>😮‍💨 VO2 Max</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.bmi.title</t>
+  </si>
+  <si>
+    <t>Body Mass Index</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.chrono_type.title</t>
+  </si>
+  <si>
+    <t>Chronotype</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.morning</t>
   </si>
   <si>
+    <t>Morning type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.solar</t>
   </si>
   <si>
+    <t>Solar type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.night</t>
   </si>
   <si>
+    <t>Night type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.morning_erratic</t>
   </si>
   <si>
+    <t>Morning erratic type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.solar_erratic</t>
   </si>
   <si>
+    <t>Solar erratic type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.chrono_type.night_erratic</t>
   </si>
   <si>
-    <t>profile_advanced_info.physical_disability.title</t>
-  </si>
-  <si>
-    <t>Physical Disabilities</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.none</t>
-  </si>
-  <si>
-    <t>No physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.moderate</t>
-  </si>
-  <si>
-    <t>Moderate physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.total</t>
-  </si>
-  <si>
-    <t>Total physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.title</t>
-  </si>
-  <si>
-    <t>Sleep Disorder</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.none</t>
-  </si>
-  <si>
-    <t>No Sleep Disorder</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.insomnia</t>
-  </si>
-  <si>
-    <t>Insomnia</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.hypersomnia</t>
-  </si>
-  <si>
-    <t>Hypersomnia</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.other</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.title</t>
-  </si>
-  <si>
-    <t>Sleep Aid</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.none</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.daily</t>
-  </si>
-  <si>
-    <t>Daily</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.weekly</t>
-  </si>
-  <si>
-    <t>Weekly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeping_pills.monthly</t>
-  </si>
-  <si>
-    <t>Monthly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.title</t>
-  </si>
-  <si>
-    <t>Sleep supplements</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.none</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.daily</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.weekly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.dietary_supplements.monthly</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeper_type.light</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleeper_type.night</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.fertility_state.menstrual_cycle</t>
-  </si>
-  <si>
-    <t>Menstrual cycle</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.fertility_state.menopause</t>
-  </si>
-  <si>
-    <t>Menopause</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.fertility_state.perimenopause</t>
-  </si>
-  <si>
-    <t>Perimenopause</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.none</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.pills</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.condoms</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.vaginal_ring</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.patch</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.iud</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.implant</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.fertility_awareness</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.birth_control.other</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.pill_pack_format.days_28</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.pill_pack_format.days_24</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.pill_pack_format.days_21</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.open_for_napping.title</t>
-  </si>
-  <si>
-    <t>Open for Napping</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.unknown_option</t>
-  </si>
-  <si>
-    <t>Unknown option</t>
+    <t>Night erratic type</t>
+  </si>
+  <si>
+    <t>alarm.weekdays</t>
+  </si>
+  <si>
+    <t>Weekdays</t>
+  </si>
+  <si>
+    <t>alarm.everydays</t>
+  </si>
+  <si>
+    <t>Every day</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1597,11 +1808,11 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <u/>
       <color rgb="FF1155CC"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -1609,6 +1820,9 @@
     <font>
       <strike/>
       <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -1650,7 +1864,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1687,11 +1901,8 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
@@ -1712,8 +1923,17 @@
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2853,10 +3073,10 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="11" t="s">
+      <c r="A76" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="C76" s="12" t="s">
+      <c r="C76" s="7" t="s">
         <v>134</v>
       </c>
       <c r="D76" s="10" t="s">
@@ -2864,10 +3084,10 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="13" t="s">
+      <c r="A77" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="C77" s="12" t="s">
+      <c r="C77" s="7" t="s">
         <v>136</v>
       </c>
       <c r="D77" s="10" t="s">
@@ -2875,14 +3095,13 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="5" t="s">
+      <c r="A78" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="B78" s="6"/>
-      <c r="C78" s="7" t="s">
+      <c r="C78" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="D78" s="5" t="s">
+      <c r="D78" s="10" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3019,7 +3238,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="8" t="s">
+      <c r="A90" s="5" t="s">
         <v>161</v>
       </c>
       <c r="B90" s="6"/>
@@ -3043,7 +3262,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="5" t="s">
+      <c r="A92" s="8" t="s">
         <v>165</v>
       </c>
       <c r="B92" s="6"/>
@@ -3348,7 +3567,7 @@
       </c>
       <c r="B117" s="6"/>
       <c r="C117" s="7" t="s">
-        <v>40</v>
+        <v>216</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>6</v>
@@ -3356,7 +3575,7 @@
     </row>
     <row r="118">
       <c r="A118" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B118" s="6"/>
       <c r="C118" s="7" t="s">
@@ -3368,11 +3587,11 @@
     </row>
     <row r="119">
       <c r="A119" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B119" s="6"/>
       <c r="C119" s="7" t="s">
-        <v>218</v>
+        <v>40</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>6</v>
@@ -3382,7 +3601,7 @@
       <c r="A120" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="B120" s="5"/>
+      <c r="B120" s="6"/>
       <c r="C120" s="7" t="s">
         <v>220</v>
       </c>
@@ -3394,7 +3613,7 @@
       <c r="A121" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="B121" s="6"/>
+      <c r="B121" s="5"/>
       <c r="C121" s="7" t="s">
         <v>222</v>
       </c>
@@ -3432,7 +3651,7 @@
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -3440,11 +3659,11 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>6</v>
@@ -3480,7 +3699,7 @@
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>6</v>
@@ -3488,11 +3707,11 @@
     </row>
     <row r="129">
       <c r="A129" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="D129" s="5" t="s">
         <v>6</v>
@@ -3571,7 +3790,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="8" t="s">
+      <c r="A136" s="5" t="s">
         <v>249</v>
       </c>
       <c r="B136" s="6"/>
@@ -3588,7 +3807,7 @@
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
-        <v>224</v>
+        <v>252</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>6</v>
@@ -3596,18 +3815,18 @@
     </row>
     <row r="138">
       <c r="A138" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B138" s="6"/>
       <c r="C138" s="7" t="s">
-        <v>253</v>
+        <v>226</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="5" t="s">
+      <c r="A139" s="8" t="s">
         <v>254</v>
       </c>
       <c r="B139" s="6"/>
@@ -3655,26 +3874,26 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="14" t="s">
+      <c r="A143" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="B143" s="15"/>
-      <c r="C143" s="14" t="s">
+      <c r="B143" s="6"/>
+      <c r="C143" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="B144" s="14"/>
+      <c r="C144" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="D143" s="14" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="B144" s="6"/>
-      <c r="C144" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="D144" s="5" t="s">
+      <c r="D144" s="13" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3859,7 +4078,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="8" t="s">
+      <c r="A160" s="5" t="s">
         <v>295</v>
       </c>
       <c r="B160" s="6"/>
@@ -3895,12 +4114,12 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="5" t="s">
+      <c r="A163" s="8" t="s">
         <v>301</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>231</v>
+        <v>302</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
@@ -3908,11 +4127,11 @@
     </row>
     <row r="164">
       <c r="A164" s="5" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>303</v>
+        <v>233</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
@@ -3991,7 +4210,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="16" t="s">
+      <c r="A171" s="5" t="s">
         <v>316</v>
       </c>
       <c r="B171" s="6"/>
@@ -4015,7 +4234,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="5" t="s">
+      <c r="A173" s="15" t="s">
         <v>320</v>
       </c>
       <c r="B173" s="6"/>
@@ -4051,7 +4270,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="8" t="s">
+      <c r="A176" s="5" t="s">
         <v>326</v>
       </c>
       <c r="B176" s="6"/>
@@ -4075,7 +4294,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="5" t="s">
+      <c r="A178" s="8" t="s">
         <v>330</v>
       </c>
       <c r="B178" s="6"/>
@@ -4236,7 +4455,7 @@
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
-        <v>51</v>
+        <v>357</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>6</v>
@@ -4244,11 +4463,11 @@
     </row>
     <row r="192">
       <c r="A192" s="5" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
@@ -4256,11 +4475,11 @@
     </row>
     <row r="193">
       <c r="A193" s="5" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>360</v>
+        <v>51</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
@@ -4279,7 +4498,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="10" t="s">
+      <c r="A195" s="5" t="s">
         <v>363</v>
       </c>
       <c r="B195" s="6"/>
@@ -4291,7 +4510,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="10" t="s">
+      <c r="A196" s="5" t="s">
         <v>365</v>
       </c>
       <c r="B196" s="6"/>
@@ -4351,24 +4570,24 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="5" t="s">
+      <c r="A201" s="10" t="s">
         <v>375</v>
       </c>
       <c r="B201" s="6"/>
       <c r="C201" s="7" t="s">
-        <v>130</v>
+        <v>376</v>
       </c>
       <c r="D201" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="5" t="s">
-        <v>376</v>
+      <c r="A202" s="10" t="s">
+        <v>377</v>
       </c>
       <c r="B202" s="6"/>
       <c r="C202" s="7" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D202" s="5" t="s">
         <v>6</v>
@@ -4376,11 +4595,11 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B203" s="6"/>
       <c r="C203" s="7" t="s">
-        <v>379</v>
+        <v>130</v>
       </c>
       <c r="D203" s="5" t="s">
         <v>6</v>
@@ -4531,14 +4750,14 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="5" t="s">
+      <c r="A216" s="16" t="s">
         <v>404</v>
       </c>
-      <c r="B216" s="6"/>
-      <c r="C216" s="7" t="s">
+      <c r="B216" s="17"/>
+      <c r="C216" s="18" t="s">
         <v>405</v>
       </c>
-      <c r="D216" s="5" t="s">
+      <c r="D216" s="16" t="s">
         <v>6</v>
       </c>
     </row>
@@ -4644,7 +4863,7 @@
       </c>
       <c r="B225" s="6"/>
       <c r="C225" s="7" t="s">
-        <v>168</v>
+        <v>423</v>
       </c>
       <c r="D225" s="5" t="s">
         <v>6</v>
@@ -4652,11 +4871,11 @@
     </row>
     <row r="226">
       <c r="A226" s="5" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B226" s="6"/>
       <c r="C226" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D226" s="5" t="s">
         <v>6</v>
@@ -4664,11 +4883,11 @@
     </row>
     <row r="227">
       <c r="A227" s="5" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B227" s="6"/>
       <c r="C227" s="7" t="s">
-        <v>307</v>
+        <v>427</v>
       </c>
       <c r="D227" s="5" t="s">
         <v>6</v>
@@ -4676,11 +4895,11 @@
     </row>
     <row r="228">
       <c r="A228" s="5" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B228" s="6"/>
       <c r="C228" s="7" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="D228" s="5" t="s">
         <v>6</v>
@@ -4688,57 +4907,35 @@
     </row>
     <row r="229">
       <c r="A229" s="5" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B229" s="6"/>
       <c r="C229" s="7" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="D229" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="17" t="s">
-        <v>430</v>
-      </c>
-      <c r="B230" s="18"/>
-      <c r="C230" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="D230" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E230" s="20"/>
-      <c r="F230" s="20"/>
-      <c r="G230" s="20"/>
-      <c r="H230" s="20"/>
-      <c r="I230" s="20"/>
-      <c r="J230" s="20"/>
-      <c r="K230" s="20"/>
-      <c r="L230" s="20"/>
-      <c r="M230" s="20"/>
-      <c r="N230" s="20"/>
-      <c r="O230" s="20"/>
-      <c r="P230" s="20"/>
-      <c r="Q230" s="20"/>
-      <c r="R230" s="20"/>
-      <c r="S230" s="20"/>
-      <c r="T230" s="20"/>
-      <c r="U230" s="20"/>
-      <c r="V230" s="20"/>
-      <c r="W230" s="20"/>
-      <c r="X230" s="20"/>
-      <c r="Y230" s="20"/>
-      <c r="Z230" s="20"/>
+      <c r="A230" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="B230" s="6"/>
+      <c r="C230" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="D230" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="5" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="B231" s="6"/>
       <c r="C231" s="7" t="s">
-        <v>432</v>
+        <v>170</v>
       </c>
       <c r="D231" s="5" t="s">
         <v>6</v>
@@ -4746,11 +4943,11 @@
     </row>
     <row r="232">
       <c r="A232" s="5" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B232" s="6"/>
       <c r="C232" s="7" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D232" s="5" t="s">
         <v>6</v>
@@ -4758,11 +4955,11 @@
     </row>
     <row r="233">
       <c r="A233" s="5" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B233" s="6"/>
       <c r="C233" s="7" t="s">
-        <v>436</v>
+        <v>309</v>
       </c>
       <c r="D233" s="5" t="s">
         <v>6</v>
@@ -4770,11 +4967,11 @@
     </row>
     <row r="234">
       <c r="A234" s="5" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B234" s="6"/>
       <c r="C234" s="7" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D234" s="5" t="s">
         <v>6</v>
@@ -4782,35 +4979,56 @@
     </row>
     <row r="235">
       <c r="A235" s="5" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B235" s="6"/>
       <c r="C235" s="7" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D235" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="17" t="s">
-        <v>441</v>
-      </c>
-      <c r="B236" s="18"/>
-      <c r="C236" s="19" t="s">
+      <c r="A236" s="16" t="s">
         <v>442</v>
       </c>
-      <c r="D236" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E236" s="20"/>
+      <c r="B236" s="17"/>
+      <c r="C236" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="D236" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E236" s="19"/>
+      <c r="F236" s="19"/>
+      <c r="G236" s="19"/>
+      <c r="H236" s="19"/>
+      <c r="I236" s="19"/>
+      <c r="J236" s="19"/>
+      <c r="K236" s="19"/>
+      <c r="L236" s="19"/>
+      <c r="M236" s="19"/>
+      <c r="N236" s="19"/>
+      <c r="O236" s="19"/>
+      <c r="P236" s="19"/>
+      <c r="Q236" s="19"/>
+      <c r="R236" s="19"/>
+      <c r="S236" s="19"/>
+      <c r="T236" s="19"/>
+      <c r="U236" s="19"/>
+      <c r="V236" s="19"/>
+      <c r="W236" s="19"/>
+      <c r="X236" s="19"/>
+      <c r="Y236" s="19"/>
+      <c r="Z236" s="19"/>
     </row>
     <row r="237">
-      <c r="A237" s="21" t="s">
+      <c r="A237" s="5" t="s">
         <v>443</v>
       </c>
       <c r="B237" s="6"/>
-      <c r="C237" s="12" t="s">
+      <c r="C237" s="7" t="s">
         <v>444</v>
       </c>
       <c r="D237" s="5" t="s">
@@ -4818,11 +5036,11 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="21" t="s">
+      <c r="A238" s="5" t="s">
         <v>445</v>
       </c>
       <c r="B238" s="6"/>
-      <c r="C238" s="12" t="s">
+      <c r="C238" s="7" t="s">
         <v>446</v>
       </c>
       <c r="D238" s="5" t="s">
@@ -4830,303 +5048,336 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="21" t="s">
+      <c r="A239" s="5" t="s">
         <v>447</v>
       </c>
       <c r="B239" s="6"/>
-      <c r="C239" s="6"/>
-      <c r="D239" s="6"/>
+      <c r="C239" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="D239" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="240">
-      <c r="A240" s="21" t="s">
-        <v>448</v>
+      <c r="A240" s="5" t="s">
+        <v>449</v>
       </c>
       <c r="B240" s="6"/>
-      <c r="C240" s="6"/>
-      <c r="D240" s="6"/>
+      <c r="C240" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="D240" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="241">
-      <c r="A241" s="21" t="s">
-        <v>449</v>
+      <c r="A241" s="5" t="s">
+        <v>451</v>
       </c>
       <c r="B241" s="6"/>
-      <c r="C241" s="6"/>
-      <c r="D241" s="6"/>
+      <c r="C241" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="D241" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="242">
-      <c r="A242" s="21" t="s">
-        <v>450</v>
-      </c>
-      <c r="B242" s="6"/>
-      <c r="C242" s="6"/>
-      <c r="D242" s="6"/>
+      <c r="A242" s="16" t="s">
+        <v>453</v>
+      </c>
+      <c r="B242" s="17"/>
+      <c r="C242" s="18" t="s">
+        <v>454</v>
+      </c>
+      <c r="D242" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E242" s="19"/>
     </row>
     <row r="243">
-      <c r="A243" s="21" t="s">
-        <v>451</v>
+      <c r="A243" s="5" t="s">
+        <v>455</v>
       </c>
       <c r="B243" s="6"/>
-      <c r="C243" s="6"/>
-      <c r="D243" s="6"/>
+      <c r="C243" s="7" t="s">
+        <v>456</v>
+      </c>
+      <c r="D243" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="244">
-      <c r="A244" s="21" t="s">
-        <v>452</v>
+      <c r="A244" s="5" t="s">
+        <v>457</v>
       </c>
       <c r="B244" s="6"/>
-      <c r="C244" s="6"/>
-      <c r="D244" s="6"/>
+      <c r="C244" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="D244" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="245">
-      <c r="A245" s="21" t="s">
-        <v>453</v>
+      <c r="A245" s="5" t="s">
+        <v>459</v>
       </c>
       <c r="B245" s="6"/>
-      <c r="C245" s="12" t="s">
-        <v>454</v>
+      <c r="C245" s="7" t="s">
+        <v>460</v>
       </c>
       <c r="D245" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="21" t="s">
-        <v>455</v>
-      </c>
-      <c r="B246" s="6"/>
+      <c r="A246" s="20" t="s">
+        <v>461</v>
+      </c>
+      <c r="B246" s="21"/>
       <c r="C246" s="12" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="D246" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="21" t="s">
-        <v>457</v>
+      <c r="A247" s="5" t="s">
+        <v>463</v>
       </c>
       <c r="B247" s="6"/>
-      <c r="C247" s="12" t="s">
-        <v>458</v>
+      <c r="C247" s="7" t="s">
+        <v>464</v>
       </c>
       <c r="D247" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="21" t="s">
-        <v>459</v>
+      <c r="A248" s="5" t="s">
+        <v>465</v>
       </c>
       <c r="B248" s="6"/>
-      <c r="C248" s="12" t="s">
-        <v>460</v>
+      <c r="C248" s="7" t="s">
+        <v>466</v>
       </c>
       <c r="D248" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="21" t="s">
-        <v>461</v>
+      <c r="A249" s="5" t="s">
+        <v>467</v>
       </c>
       <c r="B249" s="6"/>
-      <c r="C249" s="12" t="s">
-        <v>462</v>
+      <c r="C249" s="7" t="s">
+        <v>468</v>
       </c>
       <c r="D249" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="21" t="s">
-        <v>463</v>
+      <c r="A250" s="5" t="s">
+        <v>469</v>
       </c>
       <c r="B250" s="6"/>
-      <c r="C250" s="12" t="s">
-        <v>464</v>
+      <c r="C250" s="7" t="s">
+        <v>470</v>
       </c>
       <c r="D250" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="21" t="s">
-        <v>465</v>
+      <c r="A251" s="5" t="s">
+        <v>471</v>
       </c>
       <c r="B251" s="6"/>
-      <c r="C251" s="12" t="s">
-        <v>466</v>
+      <c r="C251" s="7" t="s">
+        <v>472</v>
       </c>
       <c r="D251" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="21" t="s">
-        <v>467</v>
+      <c r="A252" s="5" t="s">
+        <v>473</v>
       </c>
       <c r="B252" s="6"/>
-      <c r="C252" s="12" t="s">
-        <v>468</v>
+      <c r="C252" s="7" t="s">
+        <v>474</v>
       </c>
       <c r="D252" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="21" t="s">
-        <v>469</v>
+      <c r="A253" s="5" t="s">
+        <v>475</v>
       </c>
       <c r="B253" s="6"/>
-      <c r="C253" s="12" t="s">
-        <v>419</v>
+      <c r="C253" s="7" t="s">
+        <v>476</v>
       </c>
       <c r="D253" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="21" t="s">
-        <v>470</v>
+      <c r="A254" s="5" t="s">
+        <v>477</v>
       </c>
       <c r="B254" s="6"/>
-      <c r="C254" s="12" t="s">
-        <v>471</v>
+      <c r="C254" s="7" t="s">
+        <v>431</v>
       </c>
       <c r="D254" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="21" t="s">
-        <v>472</v>
+      <c r="A255" s="5" t="s">
+        <v>478</v>
       </c>
       <c r="B255" s="6"/>
-      <c r="C255" s="12" t="s">
-        <v>473</v>
+      <c r="C255" s="7" t="s">
+        <v>479</v>
       </c>
       <c r="D255" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="21" t="s">
-        <v>474</v>
+      <c r="A256" s="5" t="s">
+        <v>480</v>
       </c>
       <c r="B256" s="6"/>
-      <c r="C256" s="12" t="s">
-        <v>475</v>
+      <c r="C256" s="7" t="s">
+        <v>481</v>
       </c>
       <c r="D256" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="257">
-      <c r="A257" s="21" t="s">
-        <v>476</v>
+      <c r="A257" s="5" t="s">
+        <v>482</v>
       </c>
       <c r="B257" s="6"/>
-      <c r="C257" s="12" t="s">
-        <v>477</v>
+      <c r="C257" s="7" t="s">
+        <v>483</v>
       </c>
       <c r="D257" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="21" t="s">
-        <v>478</v>
+      <c r="A258" s="5" t="s">
+        <v>484</v>
       </c>
       <c r="B258" s="6"/>
-      <c r="C258" s="12" t="s">
-        <v>479</v>
+      <c r="C258" s="7" t="s">
+        <v>485</v>
       </c>
       <c r="D258" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="259">
-      <c r="A259" s="21" t="s">
-        <v>480</v>
+      <c r="A259" s="5" t="s">
+        <v>486</v>
       </c>
       <c r="B259" s="6"/>
-      <c r="C259" s="12" t="s">
-        <v>481</v>
+      <c r="C259" s="7" t="s">
+        <v>487</v>
       </c>
       <c r="D259" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="21" t="s">
-        <v>482</v>
+      <c r="A260" s="5" t="s">
+        <v>488</v>
       </c>
       <c r="B260" s="6"/>
-      <c r="C260" s="12" t="s">
-        <v>473</v>
+      <c r="C260" s="7" t="s">
+        <v>489</v>
       </c>
       <c r="D260" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="261">
-      <c r="A261" s="21" t="s">
+      <c r="A261" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B261" s="6"/>
+      <c r="C261" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="D261" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B262" s="6"/>
+      <c r="C262" s="7" t="s">
+        <v>493</v>
+      </c>
+      <c r="D262" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="B263" s="6"/>
+      <c r="C263" s="7" t="s">
         <v>483</v>
       </c>
-      <c r="B261" s="6"/>
-      <c r="C261" s="12" t="s">
-        <v>475</v>
-      </c>
-      <c r="D261" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" s="21" t="s">
-        <v>484</v>
-      </c>
-      <c r="B262" s="6"/>
-      <c r="C262" s="12" t="s">
-        <v>477</v>
-      </c>
-      <c r="D262" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" s="21" t="s">
+      <c r="D263" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="B264" s="6"/>
+      <c r="C264" s="7" t="s">
         <v>485</v>
       </c>
-      <c r="B263" s="6"/>
-      <c r="C263" s="12" t="s">
-        <v>479</v>
-      </c>
-      <c r="D263" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" s="21" t="s">
-        <v>486</v>
-      </c>
-      <c r="B264" s="6"/>
-      <c r="C264" s="6"/>
-      <c r="D264" s="6"/>
+      <c r="D264" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="265">
-      <c r="A265" s="21" t="s">
+      <c r="A265" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="B265" s="6"/>
+      <c r="C265" s="7" t="s">
         <v>487</v>
       </c>
-      <c r="B265" s="6"/>
-      <c r="C265" s="6"/>
-      <c r="D265" s="6"/>
+      <c r="D265" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="266">
-      <c r="A266" s="21" t="s">
-        <v>488</v>
+      <c r="A266" s="5" t="s">
+        <v>497</v>
       </c>
       <c r="B266" s="6"/>
-      <c r="C266" s="12" t="s">
+      <c r="C266" s="7" t="s">
         <v>489</v>
       </c>
       <c r="D266" s="5" t="s">
@@ -5134,310 +5385,512 @@
       </c>
     </row>
     <row r="267">
-      <c r="A267" s="21" t="s">
-        <v>490</v>
+      <c r="A267" s="5" t="s">
+        <v>498</v>
       </c>
       <c r="B267" s="6"/>
-      <c r="C267" s="12" t="s">
-        <v>491</v>
-      </c>
-      <c r="D267" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C267" s="6"/>
+      <c r="D267" s="6"/>
     </row>
     <row r="268">
-      <c r="A268" s="21" t="s">
-        <v>492</v>
+      <c r="A268" s="5" t="s">
+        <v>499</v>
       </c>
       <c r="B268" s="6"/>
-      <c r="C268" s="12" t="s">
-        <v>493</v>
-      </c>
-      <c r="D268" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C268" s="6"/>
+      <c r="D268" s="6"/>
     </row>
     <row r="269">
-      <c r="A269" s="21" t="s">
-        <v>494</v>
+      <c r="A269" s="20" t="s">
+        <v>500</v>
       </c>
       <c r="B269" s="6"/>
-      <c r="C269" s="6"/>
-      <c r="D269" s="6"/>
+      <c r="C269" s="12" t="s">
+        <v>501</v>
+      </c>
+      <c r="D269" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="270">
-      <c r="A270" s="21" t="s">
-        <v>495</v>
+      <c r="A270" s="20" t="s">
+        <v>502</v>
       </c>
       <c r="B270" s="6"/>
-      <c r="C270" s="6"/>
-      <c r="D270" s="6"/>
+      <c r="C270" s="12" t="s">
+        <v>503</v>
+      </c>
+      <c r="D270" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="271">
-      <c r="A271" s="21" t="s">
-        <v>496</v>
+      <c r="A271" s="5" t="s">
+        <v>504</v>
       </c>
       <c r="B271" s="6"/>
-      <c r="C271" s="6"/>
-      <c r="D271" s="6"/>
+      <c r="C271" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="D271" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="272">
-      <c r="A272" s="21" t="s">
-        <v>497</v>
+      <c r="A272" s="5" t="s">
+        <v>506</v>
       </c>
       <c r="B272" s="6"/>
-      <c r="C272" s="6"/>
-      <c r="D272" s="6"/>
+      <c r="C272" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="D272" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="273">
-      <c r="A273" s="21" t="s">
-        <v>498</v>
+      <c r="A273" s="5" t="s">
+        <v>508</v>
       </c>
       <c r="B273" s="6"/>
-      <c r="C273" s="6"/>
-      <c r="D273" s="6"/>
+      <c r="C273" s="7" t="s">
+        <v>509</v>
+      </c>
+      <c r="D273" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="274">
-      <c r="A274" s="21" t="s">
-        <v>499</v>
+      <c r="A274" s="20" t="s">
+        <v>510</v>
       </c>
       <c r="B274" s="6"/>
-      <c r="C274" s="6"/>
-      <c r="D274" s="6"/>
+      <c r="C274" s="12" t="s">
+        <v>511</v>
+      </c>
+      <c r="D274" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="275">
-      <c r="A275" s="21" t="s">
-        <v>500</v>
+      <c r="A275" s="20" t="s">
+        <v>512</v>
       </c>
       <c r="B275" s="6"/>
-      <c r="C275" s="6"/>
-      <c r="D275" s="6"/>
+      <c r="C275" s="12" t="s">
+        <v>513</v>
+      </c>
+      <c r="D275" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="276">
-      <c r="A276" s="21" t="s">
-        <v>501</v>
+      <c r="A276" s="20" t="s">
+        <v>514</v>
       </c>
       <c r="B276" s="6"/>
-      <c r="C276" s="6"/>
-      <c r="D276" s="6"/>
+      <c r="C276" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="D276" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="277">
-      <c r="A277" s="21" t="s">
-        <v>502</v>
+      <c r="A277" s="20" t="s">
+        <v>516</v>
       </c>
       <c r="B277" s="6"/>
-      <c r="C277" s="6"/>
-      <c r="D277" s="6"/>
+      <c r="C277" s="12" t="s">
+        <v>517</v>
+      </c>
+      <c r="D277" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="278">
-      <c r="A278" s="21" t="s">
-        <v>503</v>
+      <c r="A278" s="5" t="s">
+        <v>518</v>
       </c>
       <c r="B278" s="6"/>
-      <c r="C278" s="6"/>
-      <c r="D278" s="6"/>
+      <c r="C278" s="12" t="s">
+        <v>483</v>
+      </c>
+      <c r="D278" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="279">
-      <c r="A279" s="21" t="s">
-        <v>504</v>
+      <c r="A279" s="5" t="s">
+        <v>519</v>
       </c>
       <c r="B279" s="6"/>
-      <c r="C279" s="6"/>
-      <c r="D279" s="6"/>
+      <c r="C279" s="12" t="s">
+        <v>520</v>
+      </c>
+      <c r="D279" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="280">
-      <c r="A280" s="21" t="s">
-        <v>505</v>
+      <c r="A280" s="5" t="s">
+        <v>521</v>
       </c>
       <c r="B280" s="6"/>
-      <c r="C280" s="6"/>
-      <c r="D280" s="6"/>
+      <c r="C280" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="D280" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="281">
-      <c r="A281" s="21" t="s">
-        <v>506</v>
+      <c r="A281" s="5" t="s">
+        <v>523</v>
       </c>
       <c r="B281" s="6"/>
       <c r="C281" s="12" t="s">
-        <v>507</v>
+        <v>524</v>
       </c>
       <c r="D281" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="282">
-      <c r="A282" s="21" t="s">
-        <v>508</v>
+      <c r="A282" s="5" t="s">
+        <v>525</v>
       </c>
       <c r="B282" s="6"/>
       <c r="C282" s="12" t="s">
-        <v>509</v>
+        <v>526</v>
       </c>
       <c r="D282" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="283">
-      <c r="A283" s="6"/>
+      <c r="A283" s="5" t="s">
+        <v>527</v>
+      </c>
       <c r="B283" s="6"/>
-      <c r="C283" s="6"/>
-      <c r="D283" s="6"/>
+      <c r="C283" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="D283" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="284">
-      <c r="A284" s="6"/>
+      <c r="A284" s="5" t="s">
+        <v>529</v>
+      </c>
       <c r="B284" s="6"/>
-      <c r="C284" s="6"/>
-      <c r="D284" s="6"/>
+      <c r="C284" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="D284" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="285">
-      <c r="A285" s="6"/>
+      <c r="A285" s="5" t="s">
+        <v>531</v>
+      </c>
       <c r="B285" s="6"/>
-      <c r="C285" s="6"/>
-      <c r="D285" s="6"/>
+      <c r="C285" s="12" t="s">
+        <v>532</v>
+      </c>
+      <c r="D285" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="286">
-      <c r="A286" s="6"/>
+      <c r="A286" s="5" t="s">
+        <v>533</v>
+      </c>
       <c r="B286" s="6"/>
-      <c r="C286" s="6"/>
-      <c r="D286" s="6"/>
+      <c r="C286" s="12" t="s">
+        <v>431</v>
+      </c>
+      <c r="D286" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="287">
-      <c r="A287" s="6"/>
+      <c r="A287" s="20" t="s">
+        <v>534</v>
+      </c>
       <c r="B287" s="6"/>
-      <c r="C287" s="6"/>
-      <c r="D287" s="6"/>
+      <c r="C287" s="12" t="s">
+        <v>535</v>
+      </c>
+      <c r="D287" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="288">
-      <c r="A288" s="6"/>
+      <c r="A288" s="5" t="s">
+        <v>536</v>
+      </c>
       <c r="B288" s="6"/>
-      <c r="C288" s="6"/>
-      <c r="D288" s="6"/>
+      <c r="C288" s="12" t="s">
+        <v>537</v>
+      </c>
+      <c r="D288" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="289">
-      <c r="A289" s="6"/>
+      <c r="A289" s="5" t="s">
+        <v>538</v>
+      </c>
       <c r="B289" s="6"/>
-      <c r="C289" s="6"/>
-      <c r="D289" s="6"/>
+      <c r="C289" s="12" t="s">
+        <v>539</v>
+      </c>
+      <c r="D289" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="290">
-      <c r="A290" s="6"/>
+      <c r="A290" s="5" t="s">
+        <v>540</v>
+      </c>
       <c r="B290" s="6"/>
-      <c r="C290" s="6"/>
-      <c r="D290" s="6"/>
+      <c r="C290" s="12" t="s">
+        <v>541</v>
+      </c>
+      <c r="D290" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="291">
-      <c r="A291" s="6"/>
+      <c r="A291" s="20" t="s">
+        <v>542</v>
+      </c>
       <c r="B291" s="6"/>
-      <c r="C291" s="6"/>
-      <c r="D291" s="6"/>
+      <c r="C291" s="12" t="s">
+        <v>543</v>
+      </c>
+      <c r="D291" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="292">
-      <c r="A292" s="6"/>
+      <c r="A292" s="5" t="s">
+        <v>544</v>
+      </c>
       <c r="B292" s="6"/>
-      <c r="C292" s="6"/>
-      <c r="D292" s="6"/>
+      <c r="C292" s="7" t="s">
+        <v>545</v>
+      </c>
+      <c r="D292" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="293">
-      <c r="A293" s="6"/>
+      <c r="A293" s="5" t="s">
+        <v>546</v>
+      </c>
       <c r="B293" s="6"/>
-      <c r="C293" s="6"/>
-      <c r="D293" s="6"/>
+      <c r="C293" s="7" t="s">
+        <v>547</v>
+      </c>
+      <c r="D293" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="294">
-      <c r="A294" s="6"/>
+      <c r="A294" s="20" t="s">
+        <v>548</v>
+      </c>
       <c r="B294" s="6"/>
-      <c r="C294" s="6"/>
-      <c r="D294" s="6"/>
+      <c r="C294" s="12" t="s">
+        <v>549</v>
+      </c>
+      <c r="D294" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="295">
-      <c r="A295" s="6"/>
+      <c r="A295" s="20" t="s">
+        <v>550</v>
+      </c>
       <c r="B295" s="6"/>
-      <c r="C295" s="6"/>
-      <c r="D295" s="6"/>
+      <c r="C295" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="D295" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="296">
-      <c r="A296" s="6"/>
+      <c r="A296" s="20" t="s">
+        <v>552</v>
+      </c>
       <c r="B296" s="6"/>
-      <c r="C296" s="6"/>
-      <c r="D296" s="6"/>
+      <c r="C296" s="12" t="s">
+        <v>553</v>
+      </c>
+      <c r="D296" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="297">
-      <c r="A297" s="6"/>
+      <c r="A297" s="20" t="s">
+        <v>554</v>
+      </c>
       <c r="B297" s="6"/>
-      <c r="C297" s="6"/>
-      <c r="D297" s="6"/>
+      <c r="C297" s="12" t="s">
+        <v>555</v>
+      </c>
+      <c r="D297" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="298">
-      <c r="A298" s="6"/>
+      <c r="A298" s="20" t="s">
+        <v>556</v>
+      </c>
       <c r="B298" s="6"/>
-      <c r="C298" s="6"/>
-      <c r="D298" s="6"/>
+      <c r="C298" s="12" t="s">
+        <v>557</v>
+      </c>
+      <c r="D298" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="299">
-      <c r="A299" s="6"/>
+      <c r="A299" s="20" t="s">
+        <v>558</v>
+      </c>
       <c r="B299" s="6"/>
-      <c r="C299" s="6"/>
-      <c r="D299" s="6"/>
+      <c r="C299" s="12" t="s">
+        <v>559</v>
+      </c>
+      <c r="D299" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="300">
-      <c r="A300" s="6"/>
+      <c r="A300" s="20" t="s">
+        <v>560</v>
+      </c>
       <c r="B300" s="6"/>
-      <c r="C300" s="6"/>
-      <c r="D300" s="6"/>
+      <c r="C300" s="12" t="s">
+        <v>561</v>
+      </c>
+      <c r="D300" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="301">
-      <c r="A301" s="6"/>
+      <c r="A301" s="20" t="s">
+        <v>562</v>
+      </c>
       <c r="B301" s="6"/>
-      <c r="C301" s="6"/>
-      <c r="D301" s="6"/>
+      <c r="C301" s="12" t="s">
+        <v>563</v>
+      </c>
+      <c r="D301" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="302">
-      <c r="A302" s="6"/>
+      <c r="A302" s="22" t="s">
+        <v>564</v>
+      </c>
       <c r="B302" s="6"/>
-      <c r="C302" s="6"/>
-      <c r="D302" s="6"/>
+      <c r="C302" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="D302" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="303">
-      <c r="A303" s="6"/>
+      <c r="A303" s="23" t="s">
+        <v>566</v>
+      </c>
       <c r="B303" s="6"/>
-      <c r="C303" s="6"/>
-      <c r="D303" s="6"/>
+      <c r="C303" s="12" t="s">
+        <v>567</v>
+      </c>
+      <c r="D303" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="304">
-      <c r="A304" s="6"/>
+      <c r="A304" s="23" t="s">
+        <v>568</v>
+      </c>
       <c r="B304" s="6"/>
-      <c r="C304" s="6"/>
-      <c r="D304" s="6"/>
+      <c r="C304" s="12" t="s">
+        <v>569</v>
+      </c>
+      <c r="D304" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="305">
-      <c r="A305" s="6"/>
+      <c r="A305" s="23" t="s">
+        <v>570</v>
+      </c>
       <c r="B305" s="6"/>
-      <c r="C305" s="6"/>
-      <c r="D305" s="6"/>
+      <c r="C305" s="12" t="s">
+        <v>571</v>
+      </c>
+      <c r="D305" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="306">
-      <c r="A306" s="6"/>
+      <c r="A306" s="23" t="s">
+        <v>572</v>
+      </c>
       <c r="B306" s="6"/>
-      <c r="C306" s="6"/>
-      <c r="D306" s="6"/>
+      <c r="C306" s="12" t="s">
+        <v>573</v>
+      </c>
+      <c r="D306" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="307">
-      <c r="A307" s="6"/>
+      <c r="A307" s="23" t="s">
+        <v>574</v>
+      </c>
       <c r="B307" s="6"/>
-      <c r="C307" s="6"/>
-      <c r="D307" s="6"/>
+      <c r="C307" s="12" t="s">
+        <v>575</v>
+      </c>
+      <c r="D307" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="308">
-      <c r="A308" s="6"/>
+      <c r="A308" s="20" t="s">
+        <v>576</v>
+      </c>
       <c r="B308" s="6"/>
-      <c r="C308" s="6"/>
-      <c r="D308" s="6"/>
+      <c r="C308" s="12" t="s">
+        <v>577</v>
+      </c>
+      <c r="D308" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="309">
-      <c r="A309" s="6"/>
+      <c r="A309" s="20" t="s">
+        <v>578</v>
+      </c>
       <c r="B309" s="6"/>
-      <c r="C309" s="6"/>
-      <c r="D309" s="6"/>
+      <c r="C309" s="12" t="s">
+        <v>579</v>
+      </c>
+      <c r="D309" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="6"/>
@@ -10239,15 +10692,99 @@
       <c r="C1109" s="6"/>
       <c r="D1109" s="6"/>
     </row>
+    <row r="1110">
+      <c r="A1110" s="6"/>
+      <c r="B1110" s="6"/>
+      <c r="C1110" s="6"/>
+      <c r="D1110" s="6"/>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="6"/>
+      <c r="B1111" s="6"/>
+      <c r="C1111" s="6"/>
+      <c r="D1111" s="6"/>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="6"/>
+      <c r="B1112" s="6"/>
+      <c r="C1112" s="6"/>
+      <c r="D1112" s="6"/>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="6"/>
+      <c r="B1113" s="6"/>
+      <c r="C1113" s="6"/>
+      <c r="D1113" s="6"/>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="6"/>
+      <c r="B1114" s="6"/>
+      <c r="C1114" s="6"/>
+      <c r="D1114" s="6"/>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="6"/>
+      <c r="B1115" s="6"/>
+      <c r="C1115" s="6"/>
+      <c r="D1115" s="6"/>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="6"/>
+      <c r="B1116" s="6"/>
+      <c r="C1116" s="6"/>
+      <c r="D1116" s="6"/>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="6"/>
+      <c r="B1117" s="6"/>
+      <c r="C1117" s="6"/>
+      <c r="D1117" s="6"/>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="6"/>
+      <c r="B1118" s="6"/>
+      <c r="C1118" s="6"/>
+      <c r="D1118" s="6"/>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="6"/>
+      <c r="B1119" s="6"/>
+      <c r="C1119" s="6"/>
+      <c r="D1119" s="6"/>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="6"/>
+      <c r="B1120" s="6"/>
+      <c r="C1120" s="6"/>
+      <c r="D1120" s="6"/>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="6"/>
+      <c r="B1121" s="6"/>
+      <c r="C1121" s="6"/>
+      <c r="D1121" s="6"/>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="6"/>
+      <c r="B1122" s="6"/>
+      <c r="C1122" s="6"/>
+      <c r="D1122" s="6"/>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="6"/>
+      <c r="B1123" s="6"/>
+      <c r="C1123" s="6"/>
+      <c r="D1123" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D238 D245:D263 D266:D268 D281:D282">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D266 D269:D309">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="A77"/>
-    <hyperlink r:id="rId2" ref="A171"/>
+    <hyperlink r:id="rId2" ref="A173"/>
   </hyperlinks>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
cycle length bottom sheet
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="939" uniqueCount="589">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="593">
   <si>
     <t>Key</t>
   </si>
@@ -1795,6 +1795,18 @@
     <t>Select Stride</t>
   </si>
   <si>
+    <t>profile_advanced_info.cycle_length.bottom_sheet.title</t>
+  </si>
+  <si>
+    <t>Select your Cycle Length</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.cycle_length.days</t>
+  </si>
+  <si>
+    <t>{count} days</t>
+  </si>
+  <si>
     <t>profile_advanced_info.stride.reset</t>
   </si>
   <si>
@@ -1817,7 +1829,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1840,7 +1852,11 @@
       <u/>
       <color rgb="FF1155CC"/>
     </font>
-    <font/>
+    <font>
+      <u/>
+      <color rgb="FF1155CC"/>
+      <name val="Arial"/>
+    </font>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -1853,6 +1869,7 @@
     <font>
       <name val="Arial"/>
     </font>
+    <font/>
   </fonts>
   <fills count="6">
     <fill>
@@ -1929,8 +1946,8 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
@@ -1951,20 +1968,20 @@
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3126,10 +3143,10 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="11" t="s">
+      <c r="A78" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="C78" s="12" t="s">
+      <c r="C78" s="7" t="s">
         <v>138</v>
       </c>
       <c r="D78" s="10" t="s">
@@ -5164,11 +5181,11 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="20" t="s">
+      <c r="A246" s="5" t="s">
         <v>461</v>
       </c>
-      <c r="B246" s="21"/>
-      <c r="C246" s="12" t="s">
+      <c r="B246" s="6"/>
+      <c r="C246" s="7" t="s">
         <v>462</v>
       </c>
       <c r="D246" s="5" t="s">
@@ -5432,11 +5449,11 @@
       <c r="D268" s="6"/>
     </row>
     <row r="269">
-      <c r="A269" s="20" t="s">
+      <c r="A269" s="5" t="s">
         <v>500</v>
       </c>
       <c r="B269" s="6"/>
-      <c r="C269" s="12" t="s">
+      <c r="C269" s="7" t="s">
         <v>501</v>
       </c>
       <c r="D269" s="5" t="s">
@@ -5444,11 +5461,11 @@
       </c>
     </row>
     <row r="270">
-      <c r="A270" s="20" t="s">
+      <c r="A270" s="5" t="s">
         <v>502</v>
       </c>
       <c r="B270" s="6"/>
-      <c r="C270" s="12" t="s">
+      <c r="C270" s="7" t="s">
         <v>503</v>
       </c>
       <c r="D270" s="5" t="s">
@@ -5492,11 +5509,11 @@
       </c>
     </row>
     <row r="274">
-      <c r="A274" s="20" t="s">
+      <c r="A274" s="5" t="s">
         <v>510</v>
       </c>
       <c r="B274" s="6"/>
-      <c r="C274" s="12" t="s">
+      <c r="C274" s="7" t="s">
         <v>511</v>
       </c>
       <c r="D274" s="5" t="s">
@@ -5504,11 +5521,11 @@
       </c>
     </row>
     <row r="275">
-      <c r="A275" s="20" t="s">
+      <c r="A275" s="5" t="s">
         <v>512</v>
       </c>
       <c r="B275" s="6"/>
-      <c r="C275" s="12" t="s">
+      <c r="C275" s="7" t="s">
         <v>513</v>
       </c>
       <c r="D275" s="5" t="s">
@@ -5516,11 +5533,11 @@
       </c>
     </row>
     <row r="276">
-      <c r="A276" s="20" t="s">
+      <c r="A276" s="5" t="s">
         <v>514</v>
       </c>
       <c r="B276" s="6"/>
-      <c r="C276" s="12" t="s">
+      <c r="C276" s="7" t="s">
         <v>515</v>
       </c>
       <c r="D276" s="5" t="s">
@@ -5528,11 +5545,11 @@
       </c>
     </row>
     <row r="277">
-      <c r="A277" s="20" t="s">
+      <c r="A277" s="5" t="s">
         <v>516</v>
       </c>
       <c r="B277" s="6"/>
-      <c r="C277" s="12" t="s">
+      <c r="C277" s="7" t="s">
         <v>517</v>
       </c>
       <c r="D277" s="5" t="s">
@@ -5544,7 +5561,7 @@
         <v>518</v>
       </c>
       <c r="B278" s="6"/>
-      <c r="C278" s="12" t="s">
+      <c r="C278" s="7" t="s">
         <v>483</v>
       </c>
       <c r="D278" s="5" t="s">
@@ -5556,7 +5573,7 @@
         <v>519</v>
       </c>
       <c r="B279" s="6"/>
-      <c r="C279" s="12" t="s">
+      <c r="C279" s="7" t="s">
         <v>520</v>
       </c>
       <c r="D279" s="5" t="s">
@@ -5568,7 +5585,7 @@
         <v>521</v>
       </c>
       <c r="B280" s="6"/>
-      <c r="C280" s="12" t="s">
+      <c r="C280" s="7" t="s">
         <v>522</v>
       </c>
       <c r="D280" s="5" t="s">
@@ -5580,7 +5597,7 @@
         <v>523</v>
       </c>
       <c r="B281" s="6"/>
-      <c r="C281" s="12" t="s">
+      <c r="C281" s="7" t="s">
         <v>524</v>
       </c>
       <c r="D281" s="5" t="s">
@@ -5592,7 +5609,7 @@
         <v>525</v>
       </c>
       <c r="B282" s="6"/>
-      <c r="C282" s="12" t="s">
+      <c r="C282" s="7" t="s">
         <v>526</v>
       </c>
       <c r="D282" s="5" t="s">
@@ -5604,7 +5621,7 @@
         <v>527</v>
       </c>
       <c r="B283" s="6"/>
-      <c r="C283" s="12" t="s">
+      <c r="C283" s="7" t="s">
         <v>528</v>
       </c>
       <c r="D283" s="5" t="s">
@@ -5616,7 +5633,7 @@
         <v>529</v>
       </c>
       <c r="B284" s="6"/>
-      <c r="C284" s="12" t="s">
+      <c r="C284" s="7" t="s">
         <v>530</v>
       </c>
       <c r="D284" s="5" t="s">
@@ -5628,7 +5645,7 @@
         <v>531</v>
       </c>
       <c r="B285" s="6"/>
-      <c r="C285" s="12" t="s">
+      <c r="C285" s="7" t="s">
         <v>532</v>
       </c>
       <c r="D285" s="5" t="s">
@@ -5640,7 +5657,7 @@
         <v>533</v>
       </c>
       <c r="B286" s="6"/>
-      <c r="C286" s="12" t="s">
+      <c r="C286" s="7" t="s">
         <v>431</v>
       </c>
       <c r="D286" s="5" t="s">
@@ -5648,11 +5665,11 @@
       </c>
     </row>
     <row r="287">
-      <c r="A287" s="20" t="s">
+      <c r="A287" s="5" t="s">
         <v>534</v>
       </c>
       <c r="B287" s="6"/>
-      <c r="C287" s="12" t="s">
+      <c r="C287" s="7" t="s">
         <v>535</v>
       </c>
       <c r="D287" s="5" t="s">
@@ -5664,7 +5681,7 @@
         <v>536</v>
       </c>
       <c r="B288" s="6"/>
-      <c r="C288" s="12" t="s">
+      <c r="C288" s="7" t="s">
         <v>537</v>
       </c>
       <c r="D288" s="5" t="s">
@@ -5676,7 +5693,7 @@
         <v>538</v>
       </c>
       <c r="B289" s="6"/>
-      <c r="C289" s="12" t="s">
+      <c r="C289" s="7" t="s">
         <v>539</v>
       </c>
       <c r="D289" s="5" t="s">
@@ -5688,7 +5705,7 @@
         <v>540</v>
       </c>
       <c r="B290" s="6"/>
-      <c r="C290" s="12" t="s">
+      <c r="C290" s="7" t="s">
         <v>541</v>
       </c>
       <c r="D290" s="5" t="s">
@@ -5696,11 +5713,11 @@
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="20" t="s">
+      <c r="A291" s="5" t="s">
         <v>542</v>
       </c>
       <c r="B291" s="6"/>
-      <c r="C291" s="12" t="s">
+      <c r="C291" s="7" t="s">
         <v>543</v>
       </c>
       <c r="D291" s="5" t="s">
@@ -5732,11 +5749,11 @@
       </c>
     </row>
     <row r="294">
-      <c r="A294" s="20" t="s">
+      <c r="A294" s="5" t="s">
         <v>548</v>
       </c>
       <c r="B294" s="6"/>
-      <c r="C294" s="12" t="s">
+      <c r="C294" s="7" t="s">
         <v>549</v>
       </c>
       <c r="D294" s="5" t="s">
@@ -5744,11 +5761,11 @@
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="20" t="s">
+      <c r="A295" s="5" t="s">
         <v>550</v>
       </c>
       <c r="B295" s="6"/>
-      <c r="C295" s="12" t="s">
+      <c r="C295" s="7" t="s">
         <v>551</v>
       </c>
       <c r="D295" s="5" t="s">
@@ -5756,11 +5773,11 @@
       </c>
     </row>
     <row r="296">
-      <c r="A296" s="20" t="s">
+      <c r="A296" s="5" t="s">
         <v>552</v>
       </c>
       <c r="B296" s="6"/>
-      <c r="C296" s="12" t="s">
+      <c r="C296" s="7" t="s">
         <v>553</v>
       </c>
       <c r="D296" s="5" t="s">
@@ -5768,11 +5785,11 @@
       </c>
     </row>
     <row r="297">
-      <c r="A297" s="20" t="s">
+      <c r="A297" s="5" t="s">
         <v>554</v>
       </c>
       <c r="B297" s="6"/>
-      <c r="C297" s="12" t="s">
+      <c r="C297" s="7" t="s">
         <v>555</v>
       </c>
       <c r="D297" s="5" t="s">
@@ -5780,11 +5797,11 @@
       </c>
     </row>
     <row r="298">
-      <c r="A298" s="20" t="s">
+      <c r="A298" s="5" t="s">
         <v>556</v>
       </c>
       <c r="B298" s="6"/>
-      <c r="C298" s="12" t="s">
+      <c r="C298" s="7" t="s">
         <v>557</v>
       </c>
       <c r="D298" s="5" t="s">
@@ -5792,11 +5809,11 @@
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="20" t="s">
+      <c r="A299" s="5" t="s">
         <v>558</v>
       </c>
       <c r="B299" s="6"/>
-      <c r="C299" s="12" t="s">
+      <c r="C299" s="7" t="s">
         <v>559</v>
       </c>
       <c r="D299" s="5" t="s">
@@ -5804,11 +5821,11 @@
       </c>
     </row>
     <row r="300">
-      <c r="A300" s="20" t="s">
+      <c r="A300" s="5" t="s">
         <v>560</v>
       </c>
       <c r="B300" s="6"/>
-      <c r="C300" s="12" t="s">
+      <c r="C300" s="7" t="s">
         <v>555</v>
       </c>
       <c r="D300" s="5" t="s">
@@ -5816,11 +5833,11 @@
       </c>
     </row>
     <row r="301">
-      <c r="A301" s="20" t="s">
+      <c r="A301" s="5" t="s">
         <v>561</v>
       </c>
       <c r="B301" s="6"/>
-      <c r="C301" s="12" t="s">
+      <c r="C301" s="7" t="s">
         <v>562</v>
       </c>
       <c r="D301" s="5" t="s">
@@ -5828,11 +5845,11 @@
       </c>
     </row>
     <row r="302">
-      <c r="A302" s="20" t="s">
+      <c r="A302" s="5" t="s">
         <v>563</v>
       </c>
       <c r="B302" s="6"/>
-      <c r="C302" s="12" t="s">
+      <c r="C302" s="7" t="s">
         <v>564</v>
       </c>
       <c r="D302" s="5" t="s">
@@ -5840,11 +5857,11 @@
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="20" t="s">
+      <c r="A303" s="5" t="s">
         <v>565</v>
       </c>
       <c r="B303" s="6"/>
-      <c r="C303" s="12" t="s">
+      <c r="C303" s="7" t="s">
         <v>566</v>
       </c>
       <c r="D303" s="5" t="s">
@@ -5852,11 +5869,11 @@
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="22" t="s">
+      <c r="A304" s="20" t="s">
         <v>567</v>
       </c>
       <c r="B304" s="6"/>
-      <c r="C304" s="12" t="s">
+      <c r="C304" s="7" t="s">
         <v>568</v>
       </c>
       <c r="D304" s="5" t="s">
@@ -5864,11 +5881,11 @@
       </c>
     </row>
     <row r="305">
-      <c r="A305" s="23" t="s">
+      <c r="A305" s="21" t="s">
         <v>569</v>
       </c>
       <c r="B305" s="6"/>
-      <c r="C305" s="12" t="s">
+      <c r="C305" s="7" t="s">
         <v>570</v>
       </c>
       <c r="D305" s="5" t="s">
@@ -5876,11 +5893,11 @@
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="23" t="s">
+      <c r="A306" s="21" t="s">
         <v>571</v>
       </c>
       <c r="B306" s="6"/>
-      <c r="C306" s="12" t="s">
+      <c r="C306" s="7" t="s">
         <v>572</v>
       </c>
       <c r="D306" s="5" t="s">
@@ -5888,11 +5905,11 @@
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="23" t="s">
+      <c r="A307" s="21" t="s">
         <v>573</v>
       </c>
       <c r="B307" s="6"/>
-      <c r="C307" s="12" t="s">
+      <c r="C307" s="7" t="s">
         <v>574</v>
       </c>
       <c r="D307" s="5" t="s">
@@ -5900,11 +5917,11 @@
       </c>
     </row>
     <row r="308">
-      <c r="A308" s="23" t="s">
+      <c r="A308" s="21" t="s">
         <v>575</v>
       </c>
       <c r="B308" s="6"/>
-      <c r="C308" s="12" t="s">
+      <c r="C308" s="7" t="s">
         <v>576</v>
       </c>
       <c r="D308" s="5" t="s">
@@ -5912,11 +5929,11 @@
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="23" t="s">
+      <c r="A309" s="21" t="s">
         <v>577</v>
       </c>
       <c r="B309" s="6"/>
-      <c r="C309" s="12" t="s">
+      <c r="C309" s="7" t="s">
         <v>578</v>
       </c>
       <c r="D309" s="5" t="s">
@@ -5924,11 +5941,11 @@
       </c>
     </row>
     <row r="310">
-      <c r="A310" s="24" t="s">
+      <c r="A310" s="22" t="s">
         <v>579</v>
       </c>
       <c r="B310" s="6"/>
-      <c r="C310" s="12" t="s">
+      <c r="C310" s="7" t="s">
         <v>580</v>
       </c>
       <c r="D310" s="5" t="s">
@@ -5936,11 +5953,11 @@
       </c>
     </row>
     <row r="311">
-      <c r="A311" s="24" t="s">
+      <c r="A311" s="22" t="s">
         <v>581</v>
       </c>
-      <c r="B311" s="21"/>
-      <c r="C311" s="12" t="s">
+      <c r="B311" s="6"/>
+      <c r="C311" s="7" t="s">
         <v>582</v>
       </c>
       <c r="D311" s="5" t="s">
@@ -5948,11 +5965,11 @@
       </c>
     </row>
     <row r="312">
-      <c r="A312" s="24" t="s">
+      <c r="A312" s="23" t="s">
         <v>583</v>
       </c>
       <c r="B312" s="6"/>
-      <c r="C312" s="12" t="s">
+      <c r="C312" s="24" t="s">
         <v>584</v>
       </c>
       <c r="D312" s="5" t="s">
@@ -5960,11 +5977,11 @@
       </c>
     </row>
     <row r="313">
-      <c r="A313" s="20" t="s">
+      <c r="A313" s="23" t="s">
         <v>585</v>
       </c>
       <c r="B313" s="6"/>
-      <c r="C313" s="12" t="s">
+      <c r="C313" s="24" t="s">
         <v>586</v>
       </c>
       <c r="D313" s="5" t="s">
@@ -5972,11 +5989,11 @@
       </c>
     </row>
     <row r="314">
-      <c r="A314" s="20" t="s">
+      <c r="A314" s="22" t="s">
         <v>587</v>
       </c>
       <c r="B314" s="6"/>
-      <c r="C314" s="12" t="s">
+      <c r="C314" s="7" t="s">
         <v>588</v>
       </c>
       <c r="D314" s="5" t="s">
@@ -5984,16 +6001,28 @@
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="6"/>
+      <c r="A315" s="5" t="s">
+        <v>589</v>
+      </c>
       <c r="B315" s="6"/>
-      <c r="C315" s="6"/>
-      <c r="D315" s="6"/>
+      <c r="C315" s="7" t="s">
+        <v>590</v>
+      </c>
+      <c r="D315" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="316">
-      <c r="A316" s="6"/>
+      <c r="A316" s="5" t="s">
+        <v>591</v>
+      </c>
       <c r="B316" s="6"/>
-      <c r="C316" s="6"/>
-      <c r="D316" s="6"/>
+      <c r="C316" s="7" t="s">
+        <v>592</v>
+      </c>
+      <c r="D316" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="6"/>
@@ -10867,9 +10896,21 @@
       <c r="C1128" s="6"/>
       <c r="D1128" s="6"/>
     </row>
+    <row r="1129">
+      <c r="A1129" s="6"/>
+      <c r="B1129" s="6"/>
+      <c r="C1129" s="6"/>
+      <c r="D1129" s="6"/>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="6"/>
+      <c r="B1130" s="6"/>
+      <c r="C1130" s="6"/>
+      <c r="D1130" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D266 D269:D314">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D266 D269:D316">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
properly words cycle length slider
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="593">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="595">
   <si>
     <t>Key</t>
   </si>
@@ -1805,6 +1805,12 @@
   </si>
   <si>
     <t>{count} days</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.cycle_length.label</t>
+  </si>
+  <si>
+    <t>Days</t>
   </si>
   <si>
     <t>profile_advanced_info.stride.reset</t>
@@ -5989,11 +5995,11 @@
       </c>
     </row>
     <row r="314">
-      <c r="A314" s="22" t="s">
+      <c r="A314" s="23" t="s">
         <v>587</v>
       </c>
       <c r="B314" s="6"/>
-      <c r="C314" s="7" t="s">
+      <c r="C314" s="24" t="s">
         <v>588</v>
       </c>
       <c r="D314" s="5" t="s">
@@ -6001,7 +6007,7 @@
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="5" t="s">
+      <c r="A315" s="22" t="s">
         <v>589</v>
       </c>
       <c r="B315" s="6"/>
@@ -6025,10 +6031,16 @@
       </c>
     </row>
     <row r="317">
-      <c r="A317" s="6"/>
+      <c r="A317" s="5" t="s">
+        <v>593</v>
+      </c>
       <c r="B317" s="6"/>
-      <c r="C317" s="6"/>
-      <c r="D317" s="6"/>
+      <c r="C317" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="D317" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="6"/>
@@ -10908,9 +10920,15 @@
       <c r="C1130" s="6"/>
       <c r="D1130" s="6"/>
     </row>
+    <row r="1131">
+      <c r="A1131" s="6"/>
+      <c r="B1131" s="6"/>
+      <c r="C1131" s="6"/>
+      <c r="D1131" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D266 D269:D316">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D266 D269:D317">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
edit and remove alarms
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="597">
   <si>
     <t>Key</t>
   </si>
@@ -984,6 +984,12 @@
   </si>
   <si>
     <t>Choose on what day(s) you want this alarm to go off.</t>
+  </si>
+  <si>
+    <t>alarm.delete</t>
+  </si>
+  <si>
+    <t>Delete Alarm</t>
   </si>
   <si>
     <t>onboarding.wear.title</t>
@@ -1835,7 +1841,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1863,6 +1869,7 @@
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -1872,10 +1879,6 @@
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <name val="Arial"/>
-    </font>
-    <font/>
   </fonts>
   <fills count="6">
     <fill>
@@ -1964,16 +1967,22 @@
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
@@ -1982,12 +1991,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4276,11 +4279,11 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="5" t="s">
+      <c r="A172" s="15" t="s">
         <v>318</v>
       </c>
       <c r="B172" s="6"/>
-      <c r="C172" s="7" t="s">
+      <c r="C172" s="16" t="s">
         <v>319</v>
       </c>
       <c r="D172" s="5" t="s">
@@ -4288,7 +4291,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="15" t="s">
+      <c r="A173" s="5" t="s">
         <v>320</v>
       </c>
       <c r="B173" s="6"/>
@@ -4300,7 +4303,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="5" t="s">
+      <c r="A174" s="17" t="s">
         <v>322</v>
       </c>
       <c r="B174" s="6"/>
@@ -4348,7 +4351,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="8" t="s">
+      <c r="A178" s="5" t="s">
         <v>330</v>
       </c>
       <c r="B178" s="6"/>
@@ -4360,7 +4363,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="5" t="s">
+      <c r="A179" s="8" t="s">
         <v>332</v>
       </c>
       <c r="B179" s="6"/>
@@ -4533,7 +4536,7 @@
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>51</v>
+        <v>361</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
@@ -4541,11 +4544,11 @@
     </row>
     <row r="194">
       <c r="A194" s="5" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B194" s="6"/>
       <c r="C194" s="7" t="s">
-        <v>362</v>
+        <v>51</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>6</v>
@@ -4576,7 +4579,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="10" t="s">
+      <c r="A197" s="5" t="s">
         <v>367</v>
       </c>
       <c r="B197" s="6"/>
@@ -4648,12 +4651,12 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="5" t="s">
+      <c r="A203" s="10" t="s">
         <v>379</v>
       </c>
       <c r="B203" s="6"/>
       <c r="C203" s="7" t="s">
-        <v>130</v>
+        <v>380</v>
       </c>
       <c r="D203" s="5" t="s">
         <v>6</v>
@@ -4661,11 +4664,11 @@
     </row>
     <row r="204">
       <c r="A204" s="5" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B204" s="6"/>
       <c r="C204" s="7" t="s">
-        <v>381</v>
+        <v>130</v>
       </c>
       <c r="D204" s="5" t="s">
         <v>6</v>
@@ -4804,26 +4807,26 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="16" t="s">
+      <c r="A216" s="5" t="s">
         <v>404</v>
       </c>
-      <c r="B216" s="17"/>
-      <c r="C216" s="18" t="s">
+      <c r="B216" s="6"/>
+      <c r="C216" s="7" t="s">
         <v>405</v>
       </c>
-      <c r="D216" s="16" t="s">
+      <c r="D216" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="5" t="s">
+      <c r="A217" s="18" t="s">
         <v>406</v>
       </c>
-      <c r="B217" s="6"/>
-      <c r="C217" s="7" t="s">
+      <c r="B217" s="19"/>
+      <c r="C217" s="20" t="s">
         <v>407</v>
       </c>
-      <c r="D217" s="5" t="s">
+      <c r="D217" s="18" t="s">
         <v>6</v>
       </c>
     </row>
@@ -4989,7 +4992,7 @@
       </c>
       <c r="B231" s="6"/>
       <c r="C231" s="7" t="s">
-        <v>170</v>
+        <v>435</v>
       </c>
       <c r="D231" s="5" t="s">
         <v>6</v>
@@ -4997,11 +5000,11 @@
     </row>
     <row r="232">
       <c r="A232" s="5" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B232" s="6"/>
       <c r="C232" s="7" t="s">
-        <v>436</v>
+        <v>170</v>
       </c>
       <c r="D232" s="5" t="s">
         <v>6</v>
@@ -5013,7 +5016,7 @@
       </c>
       <c r="B233" s="6"/>
       <c r="C233" s="7" t="s">
-        <v>309</v>
+        <v>438</v>
       </c>
       <c r="D233" s="5" t="s">
         <v>6</v>
@@ -5021,11 +5024,11 @@
     </row>
     <row r="234">
       <c r="A234" s="5" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B234" s="6"/>
       <c r="C234" s="7" t="s">
-        <v>439</v>
+        <v>309</v>
       </c>
       <c r="D234" s="5" t="s">
         <v>6</v>
@@ -5044,50 +5047,50 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="16" t="s">
+      <c r="A236" s="5" t="s">
         <v>442</v>
       </c>
-      <c r="B236" s="17"/>
-      <c r="C236" s="18" t="s">
+      <c r="B236" s="6"/>
+      <c r="C236" s="7" t="s">
+        <v>443</v>
+      </c>
+      <c r="D236" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="18" t="s">
+        <v>444</v>
+      </c>
+      <c r="B237" s="19"/>
+      <c r="C237" s="20" t="s">
         <v>233</v>
       </c>
-      <c r="D236" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="E236" s="19"/>
-      <c r="F236" s="19"/>
-      <c r="G236" s="19"/>
-      <c r="H236" s="19"/>
-      <c r="I236" s="19"/>
-      <c r="J236" s="19"/>
-      <c r="K236" s="19"/>
-      <c r="L236" s="19"/>
-      <c r="M236" s="19"/>
-      <c r="N236" s="19"/>
-      <c r="O236" s="19"/>
-      <c r="P236" s="19"/>
-      <c r="Q236" s="19"/>
-      <c r="R236" s="19"/>
-      <c r="S236" s="19"/>
-      <c r="T236" s="19"/>
-      <c r="U236" s="19"/>
-      <c r="V236" s="19"/>
-      <c r="W236" s="19"/>
-      <c r="X236" s="19"/>
-      <c r="Y236" s="19"/>
-      <c r="Z236" s="19"/>
-    </row>
-    <row r="237">
-      <c r="A237" s="5" t="s">
-        <v>443</v>
-      </c>
-      <c r="B237" s="6"/>
-      <c r="C237" s="7" t="s">
-        <v>444</v>
-      </c>
-      <c r="D237" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="D237" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="E237" s="21"/>
+      <c r="F237" s="21"/>
+      <c r="G237" s="21"/>
+      <c r="H237" s="21"/>
+      <c r="I237" s="21"/>
+      <c r="J237" s="21"/>
+      <c r="K237" s="21"/>
+      <c r="L237" s="21"/>
+      <c r="M237" s="21"/>
+      <c r="N237" s="21"/>
+      <c r="O237" s="21"/>
+      <c r="P237" s="21"/>
+      <c r="Q237" s="21"/>
+      <c r="R237" s="21"/>
+      <c r="S237" s="21"/>
+      <c r="T237" s="21"/>
+      <c r="U237" s="21"/>
+      <c r="V237" s="21"/>
+      <c r="W237" s="21"/>
+      <c r="X237" s="21"/>
+      <c r="Y237" s="21"/>
+      <c r="Z237" s="21"/>
     </row>
     <row r="238">
       <c r="A238" s="5" t="s">
@@ -5138,29 +5141,29 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="16" t="s">
+      <c r="A242" s="5" t="s">
         <v>453</v>
       </c>
-      <c r="B242" s="17"/>
-      <c r="C242" s="18" t="s">
+      <c r="B242" s="6"/>
+      <c r="C242" s="7" t="s">
         <v>454</v>
       </c>
-      <c r="D242" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="E242" s="19"/>
+      <c r="D242" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="243">
-      <c r="A243" s="5" t="s">
+      <c r="A243" s="18" t="s">
         <v>455</v>
       </c>
-      <c r="B243" s="6"/>
-      <c r="C243" s="7" t="s">
+      <c r="B243" s="19"/>
+      <c r="C243" s="20" t="s">
         <v>456</v>
       </c>
-      <c r="D243" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="D243" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="E243" s="21"/>
     </row>
     <row r="244">
       <c r="A244" s="5" t="s">
@@ -5288,7 +5291,7 @@
       </c>
       <c r="B254" s="6"/>
       <c r="C254" s="7" t="s">
-        <v>431</v>
+        <v>478</v>
       </c>
       <c r="D254" s="5" t="s">
         <v>6</v>
@@ -5296,11 +5299,11 @@
     </row>
     <row r="255">
       <c r="A255" s="5" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B255" s="6"/>
       <c r="C255" s="7" t="s">
-        <v>479</v>
+        <v>433</v>
       </c>
       <c r="D255" s="5" t="s">
         <v>6</v>
@@ -5396,7 +5399,7 @@
       </c>
       <c r="B263" s="6"/>
       <c r="C263" s="7" t="s">
-        <v>483</v>
+        <v>495</v>
       </c>
       <c r="D263" s="5" t="s">
         <v>6</v>
@@ -5404,7 +5407,7 @@
     </row>
     <row r="264">
       <c r="A264" s="5" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B264" s="6"/>
       <c r="C264" s="7" t="s">
@@ -5416,7 +5419,7 @@
     </row>
     <row r="265">
       <c r="A265" s="5" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B265" s="6"/>
       <c r="C265" s="7" t="s">
@@ -5428,7 +5431,7 @@
     </row>
     <row r="266">
       <c r="A266" s="5" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B266" s="6"/>
       <c r="C266" s="7" t="s">
@@ -5440,15 +5443,19 @@
     </row>
     <row r="267">
       <c r="A267" s="5" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B267" s="6"/>
-      <c r="C267" s="6"/>
-      <c r="D267" s="6"/>
+      <c r="C267" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="D267" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="5" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B268" s="6"/>
       <c r="C268" s="6"/>
@@ -5456,15 +5463,11 @@
     </row>
     <row r="269">
       <c r="A269" s="5" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B269" s="6"/>
-      <c r="C269" s="7" t="s">
-        <v>501</v>
-      </c>
-      <c r="D269" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C269" s="6"/>
+      <c r="D269" s="6"/>
     </row>
     <row r="270">
       <c r="A270" s="5" t="s">
@@ -5568,7 +5571,7 @@
       </c>
       <c r="B278" s="6"/>
       <c r="C278" s="7" t="s">
-        <v>483</v>
+        <v>519</v>
       </c>
       <c r="D278" s="5" t="s">
         <v>6</v>
@@ -5576,11 +5579,11 @@
     </row>
     <row r="279">
       <c r="A279" s="5" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B279" s="6"/>
       <c r="C279" s="7" t="s">
-        <v>520</v>
+        <v>485</v>
       </c>
       <c r="D279" s="5" t="s">
         <v>6</v>
@@ -5664,7 +5667,7 @@
       </c>
       <c r="B286" s="6"/>
       <c r="C286" s="7" t="s">
-        <v>431</v>
+        <v>534</v>
       </c>
       <c r="D286" s="5" t="s">
         <v>6</v>
@@ -5672,11 +5675,11 @@
     </row>
     <row r="287">
       <c r="A287" s="5" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B287" s="6"/>
       <c r="C287" s="7" t="s">
-        <v>535</v>
+        <v>433</v>
       </c>
       <c r="D287" s="5" t="s">
         <v>6</v>
@@ -5832,7 +5835,7 @@
       </c>
       <c r="B300" s="6"/>
       <c r="C300" s="7" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="D300" s="5" t="s">
         <v>6</v>
@@ -5840,11 +5843,11 @@
     </row>
     <row r="301">
       <c r="A301" s="5" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B301" s="6"/>
       <c r="C301" s="7" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="D301" s="5" t="s">
         <v>6</v>
@@ -5875,7 +5878,7 @@
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="20" t="s">
+      <c r="A304" s="5" t="s">
         <v>567</v>
       </c>
       <c r="B304" s="6"/>
@@ -5887,7 +5890,7 @@
       </c>
     </row>
     <row r="305">
-      <c r="A305" s="21" t="s">
+      <c r="A305" s="22" t="s">
         <v>569</v>
       </c>
       <c r="B305" s="6"/>
@@ -5899,7 +5902,7 @@
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="21" t="s">
+      <c r="A306" s="23" t="s">
         <v>571</v>
       </c>
       <c r="B306" s="6"/>
@@ -5911,7 +5914,7 @@
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="21" t="s">
+      <c r="A307" s="23" t="s">
         <v>573</v>
       </c>
       <c r="B307" s="6"/>
@@ -5923,7 +5926,7 @@
       </c>
     </row>
     <row r="308">
-      <c r="A308" s="21" t="s">
+      <c r="A308" s="23" t="s">
         <v>575</v>
       </c>
       <c r="B308" s="6"/>
@@ -5935,7 +5938,7 @@
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="21" t="s">
+      <c r="A309" s="23" t="s">
         <v>577</v>
       </c>
       <c r="B309" s="6"/>
@@ -5947,7 +5950,7 @@
       </c>
     </row>
     <row r="310">
-      <c r="A310" s="22" t="s">
+      <c r="A310" s="23" t="s">
         <v>579</v>
       </c>
       <c r="B310" s="6"/>
@@ -5959,7 +5962,7 @@
       </c>
     </row>
     <row r="311">
-      <c r="A311" s="22" t="s">
+      <c r="A311" s="24" t="s">
         <v>581</v>
       </c>
       <c r="B311" s="6"/>
@@ -5971,11 +5974,11 @@
       </c>
     </row>
     <row r="312">
-      <c r="A312" s="23" t="s">
+      <c r="A312" s="24" t="s">
         <v>583</v>
       </c>
       <c r="B312" s="6"/>
-      <c r="C312" s="24" t="s">
+      <c r="C312" s="7" t="s">
         <v>584</v>
       </c>
       <c r="D312" s="5" t="s">
@@ -5983,11 +5986,11 @@
       </c>
     </row>
     <row r="313">
-      <c r="A313" s="23" t="s">
+      <c r="A313" s="24" t="s">
         <v>585</v>
       </c>
       <c r="B313" s="6"/>
-      <c r="C313" s="24" t="s">
+      <c r="C313" s="7" t="s">
         <v>586</v>
       </c>
       <c r="D313" s="5" t="s">
@@ -5995,11 +5998,11 @@
       </c>
     </row>
     <row r="314">
-      <c r="A314" s="23" t="s">
+      <c r="A314" s="24" t="s">
         <v>587</v>
       </c>
       <c r="B314" s="6"/>
-      <c r="C314" s="24" t="s">
+      <c r="C314" s="7" t="s">
         <v>588</v>
       </c>
       <c r="D314" s="5" t="s">
@@ -6007,7 +6010,7 @@
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="22" t="s">
+      <c r="A315" s="24" t="s">
         <v>589</v>
       </c>
       <c r="B315" s="6"/>
@@ -6019,7 +6022,7 @@
       </c>
     </row>
     <row r="316">
-      <c r="A316" s="5" t="s">
+      <c r="A316" s="24" t="s">
         <v>591</v>
       </c>
       <c r="B316" s="6"/>
@@ -6043,10 +6046,16 @@
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="6"/>
+      <c r="A318" s="5" t="s">
+        <v>595</v>
+      </c>
       <c r="B318" s="6"/>
-      <c r="C318" s="6"/>
-      <c r="D318" s="6"/>
+      <c r="C318" s="7" t="s">
+        <v>596</v>
+      </c>
+      <c r="D318" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="6"/>
@@ -10926,15 +10935,21 @@
       <c r="C1131" s="6"/>
       <c r="D1131" s="6"/>
     </row>
+    <row r="1132">
+      <c r="A1132" s="6"/>
+      <c r="B1132" s="6"/>
+      <c r="C1132" s="6"/>
+      <c r="D1132" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D266 D269:D317">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D267 D270:D318">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="A77"/>
-    <hyperlink r:id="rId2" ref="A173"/>
+    <hyperlink r:id="rId2" ref="A174"/>
   </hyperlinks>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
"My Ring" in header right only on Home page
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -180,7 +180,7 @@
     <t>header.activity</t>
   </si>
   <si>
-    <t>Activity Analysis</t>
+    <t>ACTIVITY ANALYSIS</t>
   </si>
   <si>
     <t>ring.battery.label</t>
@@ -1860,6 +1860,7 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF1155CC"/>
@@ -1869,7 +1870,6 @@
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -1918,7 +1918,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1949,13 +1949,16 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -1963,12 +1966,6 @@
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
@@ -2564,7 +2561,7 @@
         <v>54</v>
       </c>
       <c r="B28" s="6"/>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="10" t="s">
         <v>55</v>
       </c>
       <c r="D28" s="5" t="s">
@@ -3064,101 +3061,101 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="10" t="s">
+      <c r="A70" s="11" t="s">
         <v>124</v>
       </c>
       <c r="C70" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D70" s="10" t="s">
+      <c r="D70" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="10" t="s">
+      <c r="A71" s="11" t="s">
         <v>125</v>
       </c>
       <c r="C71" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="D71" s="10" t="s">
+      <c r="D71" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="10" t="s">
+      <c r="A72" s="11" t="s">
         <v>127</v>
       </c>
       <c r="C72" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="D72" s="10" t="s">
+      <c r="D72" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="10" t="s">
+      <c r="A73" s="11" t="s">
         <v>129</v>
       </c>
       <c r="C73" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="D73" s="10" t="s">
+      <c r="D73" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="10" t="s">
+      <c r="A74" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C74" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D74" s="10" t="s">
+      <c r="D74" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="10" t="s">
+      <c r="A75" s="11" t="s">
         <v>132</v>
       </c>
       <c r="C75" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D75" s="10" t="s">
+      <c r="D75" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="10" t="s">
+      <c r="A76" s="11" t="s">
         <v>133</v>
       </c>
       <c r="C76" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="D76" s="10" t="s">
+      <c r="D76" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="11" t="s">
+      <c r="A77" s="12" t="s">
         <v>135</v>
       </c>
       <c r="C77" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="D77" s="10" t="s">
+      <c r="D77" s="11" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="12" t="s">
+      <c r="A78" s="13" t="s">
         <v>137</v>
       </c>
       <c r="C78" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="D78" s="10" t="s">
+      <c r="D78" s="11" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3943,14 +3940,14 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="13" t="s">
+      <c r="A144" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="B144" s="14"/>
-      <c r="C144" s="13" t="s">
+      <c r="B144" s="15"/>
+      <c r="C144" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="D144" s="13" t="s">
+      <c r="D144" s="14" t="s">
         <v>6</v>
       </c>
     </row>
@@ -4279,11 +4276,11 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="15" t="s">
+      <c r="A172" s="5" t="s">
         <v>318</v>
       </c>
       <c r="B172" s="6"/>
-      <c r="C172" s="16" t="s">
+      <c r="C172" s="7" t="s">
         <v>319</v>
       </c>
       <c r="D172" s="5" t="s">
@@ -4303,7 +4300,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="17" t="s">
+      <c r="A174" s="16" t="s">
         <v>322</v>
       </c>
       <c r="B174" s="6"/>
@@ -4591,7 +4588,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="10" t="s">
+      <c r="A198" s="11" t="s">
         <v>369</v>
       </c>
       <c r="B198" s="6"/>
@@ -4603,7 +4600,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="10" t="s">
+      <c r="A199" s="11" t="s">
         <v>371</v>
       </c>
       <c r="B199" s="6"/>
@@ -4615,7 +4612,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="10" t="s">
+      <c r="A200" s="11" t="s">
         <v>373</v>
       </c>
       <c r="B200" s="6"/>
@@ -4627,7 +4624,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="10" t="s">
+      <c r="A201" s="11" t="s">
         <v>375</v>
       </c>
       <c r="B201" s="6"/>
@@ -4639,7 +4636,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="10" t="s">
+      <c r="A202" s="11" t="s">
         <v>377</v>
       </c>
       <c r="B202" s="6"/>
@@ -4651,7 +4648,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="10" t="s">
+      <c r="A203" s="11" t="s">
         <v>379</v>
       </c>
       <c r="B203" s="6"/>
@@ -4819,14 +4816,14 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="18" t="s">
+      <c r="A217" s="17" t="s">
         <v>406</v>
       </c>
-      <c r="B217" s="19"/>
-      <c r="C217" s="20" t="s">
+      <c r="B217" s="18"/>
+      <c r="C217" s="19" t="s">
         <v>407</v>
       </c>
-      <c r="D217" s="18" t="s">
+      <c r="D217" s="17" t="s">
         <v>6</v>
       </c>
     </row>
@@ -5059,38 +5056,38 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="18" t="s">
+      <c r="A237" s="17" t="s">
         <v>444</v>
       </c>
-      <c r="B237" s="19"/>
-      <c r="C237" s="20" t="s">
+      <c r="B237" s="18"/>
+      <c r="C237" s="19" t="s">
         <v>233</v>
       </c>
-      <c r="D237" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="E237" s="21"/>
-      <c r="F237" s="21"/>
-      <c r="G237" s="21"/>
-      <c r="H237" s="21"/>
-      <c r="I237" s="21"/>
-      <c r="J237" s="21"/>
-      <c r="K237" s="21"/>
-      <c r="L237" s="21"/>
-      <c r="M237" s="21"/>
-      <c r="N237" s="21"/>
-      <c r="O237" s="21"/>
-      <c r="P237" s="21"/>
-      <c r="Q237" s="21"/>
-      <c r="R237" s="21"/>
-      <c r="S237" s="21"/>
-      <c r="T237" s="21"/>
-      <c r="U237" s="21"/>
-      <c r="V237" s="21"/>
-      <c r="W237" s="21"/>
-      <c r="X237" s="21"/>
-      <c r="Y237" s="21"/>
-      <c r="Z237" s="21"/>
+      <c r="D237" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E237" s="20"/>
+      <c r="F237" s="20"/>
+      <c r="G237" s="20"/>
+      <c r="H237" s="20"/>
+      <c r="I237" s="20"/>
+      <c r="J237" s="20"/>
+      <c r="K237" s="20"/>
+      <c r="L237" s="20"/>
+      <c r="M237" s="20"/>
+      <c r="N237" s="20"/>
+      <c r="O237" s="20"/>
+      <c r="P237" s="20"/>
+      <c r="Q237" s="20"/>
+      <c r="R237" s="20"/>
+      <c r="S237" s="20"/>
+      <c r="T237" s="20"/>
+      <c r="U237" s="20"/>
+      <c r="V237" s="20"/>
+      <c r="W237" s="20"/>
+      <c r="X237" s="20"/>
+      <c r="Y237" s="20"/>
+      <c r="Z237" s="20"/>
     </row>
     <row r="238">
       <c r="A238" s="5" t="s">
@@ -5153,17 +5150,17 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="18" t="s">
+      <c r="A243" s="17" t="s">
         <v>455</v>
       </c>
-      <c r="B243" s="19"/>
-      <c r="C243" s="20" t="s">
+      <c r="B243" s="18"/>
+      <c r="C243" s="19" t="s">
         <v>456</v>
       </c>
-      <c r="D243" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="E243" s="21"/>
+      <c r="D243" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E243" s="20"/>
     </row>
     <row r="244">
       <c r="A244" s="5" t="s">
@@ -5890,7 +5887,7 @@
       </c>
     </row>
     <row r="305">
-      <c r="A305" s="22" t="s">
+      <c r="A305" s="21" t="s">
         <v>569</v>
       </c>
       <c r="B305" s="6"/>
@@ -5902,7 +5899,7 @@
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="23" t="s">
+      <c r="A306" s="22" t="s">
         <v>571</v>
       </c>
       <c r="B306" s="6"/>
@@ -5914,7 +5911,7 @@
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="23" t="s">
+      <c r="A307" s="22" t="s">
         <v>573</v>
       </c>
       <c r="B307" s="6"/>
@@ -5926,7 +5923,7 @@
       </c>
     </row>
     <row r="308">
-      <c r="A308" s="23" t="s">
+      <c r="A308" s="22" t="s">
         <v>575</v>
       </c>
       <c r="B308" s="6"/>
@@ -5938,7 +5935,7 @@
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="23" t="s">
+      <c r="A309" s="22" t="s">
         <v>577</v>
       </c>
       <c r="B309" s="6"/>
@@ -5950,7 +5947,7 @@
       </c>
     </row>
     <row r="310">
-      <c r="A310" s="23" t="s">
+      <c r="A310" s="22" t="s">
         <v>579</v>
       </c>
       <c r="B310" s="6"/>
@@ -5962,7 +5959,7 @@
       </c>
     </row>
     <row r="311">
-      <c r="A311" s="24" t="s">
+      <c r="A311" s="23" t="s">
         <v>581</v>
       </c>
       <c r="B311" s="6"/>
@@ -5974,7 +5971,7 @@
       </c>
     </row>
     <row r="312">
-      <c r="A312" s="24" t="s">
+      <c r="A312" s="23" t="s">
         <v>583</v>
       </c>
       <c r="B312" s="6"/>
@@ -5986,7 +5983,7 @@
       </c>
     </row>
     <row r="313">
-      <c r="A313" s="24" t="s">
+      <c r="A313" s="23" t="s">
         <v>585</v>
       </c>
       <c r="B313" s="6"/>
@@ -5998,7 +5995,7 @@
       </c>
     </row>
     <row r="314">
-      <c r="A314" s="24" t="s">
+      <c r="A314" s="23" t="s">
         <v>587</v>
       </c>
       <c r="B314" s="6"/>
@@ -6010,7 +6007,7 @@
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="24" t="s">
+      <c r="A315" s="23" t="s">
         <v>589</v>
       </c>
       <c r="B315" s="6"/>
@@ -6022,7 +6019,7 @@
       </c>
     </row>
     <row r="316">
-      <c r="A316" s="24" t="s">
+      <c r="A316" s="23" t="s">
         <v>591</v>
       </c>
       <c r="B316" s="6"/>

</xml_diff>

<commit_message>
no more tsc error
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="607">
   <si>
     <t>Key</t>
   </si>
@@ -1843,16 +1843,28 @@
     <t>Every day</t>
   </si>
   <si>
+    <t>alarm.weekends</t>
+  </si>
+  <si>
+    <t>Weekends</t>
+  </si>
+  <si>
     <t>header.manage_my_rings</t>
   </si>
   <si>
     <t>MANAGE MY RINGS</t>
   </si>
   <si>
-    <t>alarm.weekends</t>
-  </si>
-  <si>
-    <t>Weekends</t>
+    <t>manage_rings.general</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>manage_rings.paired_rings_title</t>
+  </si>
+  <si>
+    <t>Rings paired to your account</t>
   </si>
 </sst>
 </file>
@@ -6100,11 +6112,11 @@
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="11" t="s">
+      <c r="A321" s="5" t="s">
         <v>601</v>
       </c>
       <c r="B321" s="6"/>
-      <c r="C321" s="10" t="s">
+      <c r="C321" s="7" t="s">
         <v>602</v>
       </c>
       <c r="D321" s="5" t="s">
@@ -6112,22 +6124,34 @@
       </c>
     </row>
     <row r="322">
-      <c r="A322" s="6"/>
+      <c r="A322" s="11" t="s">
+        <v>603</v>
+      </c>
       <c r="B322" s="6"/>
-      <c r="C322" s="6"/>
-      <c r="D322" s="6"/>
+      <c r="C322" s="10" t="s">
+        <v>604</v>
+      </c>
+      <c r="D322" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="323">
-      <c r="A323" s="6"/>
+      <c r="A323" s="5"/>
       <c r="B323" s="6"/>
-      <c r="C323" s="6"/>
-      <c r="D323" s="6"/>
+      <c r="C323" s="7"/>
+      <c r="D323" s="5"/>
     </row>
     <row r="324">
-      <c r="A324" s="6"/>
+      <c r="A324" s="11" t="s">
+        <v>605</v>
+      </c>
       <c r="B324" s="6"/>
-      <c r="C324" s="6"/>
-      <c r="D324" s="6"/>
+      <c r="C324" s="10" t="s">
+        <v>606</v>
+      </c>
+      <c r="D324" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="6"/>
@@ -10983,9 +11007,15 @@
       <c r="C1133" s="6"/>
       <c r="D1133" s="6"/>
     </row>
+    <row r="1134">
+      <c r="A1134" s="6"/>
+      <c r="B1134" s="6"/>
+      <c r="C1134" s="6"/>
+      <c r="D1134" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D268 D271:D321">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D268 D271:D324">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
reuse score component accross circle screens
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="667">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="669">
   <si>
     <t>Key</t>
   </si>
@@ -460,6 +460,12 @@
   </si>
   <si>
     <t>Sync success</t>
+  </si>
+  <si>
+    <t>activity.energy_score</t>
+  </si>
+  <si>
+    <t>Energy score</t>
   </si>
   <si>
     <t>activity.score.daily_metrics</t>
@@ -2095,6 +2101,7 @@
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -2104,7 +2111,6 @@
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
     </font>
-    <font/>
   </fonts>
   <fills count="6">
     <fill>
@@ -2184,25 +2190,31 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
@@ -2211,12 +2223,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3449,11 +3455,11 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="5" t="s">
+      <c r="A84" s="13" t="s">
         <v>149</v>
       </c>
       <c r="B84" s="6"/>
-      <c r="C84" s="7" t="s">
+      <c r="C84" s="14" t="s">
         <v>150</v>
       </c>
       <c r="D84" s="5" t="s">
@@ -3569,7 +3575,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="s">
+      <c r="A94" s="5" t="s">
         <v>169</v>
       </c>
       <c r="B94" s="6"/>
@@ -3593,7 +3599,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="5" t="s">
+      <c r="A96" s="8" t="s">
         <v>173</v>
       </c>
       <c r="B96" s="6"/>
@@ -3898,7 +3904,7 @@
       </c>
       <c r="B121" s="6"/>
       <c r="C121" s="7" t="s">
-        <v>40</v>
+        <v>224</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>6</v>
@@ -3906,7 +3912,7 @@
     </row>
     <row r="122">
       <c r="A122" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B122" s="6"/>
       <c r="C122" s="7" t="s">
@@ -3918,11 +3924,11 @@
     </row>
     <row r="123">
       <c r="A123" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B123" s="6"/>
       <c r="C123" s="7" t="s">
-        <v>226</v>
+        <v>40</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>6</v>
@@ -3932,7 +3938,7 @@
       <c r="A124" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="B124" s="5"/>
+      <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
         <v>228</v>
       </c>
@@ -3944,7 +3950,7 @@
       <c r="A125" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="B125" s="6"/>
+      <c r="B125" s="5"/>
       <c r="C125" s="7" t="s">
         <v>230</v>
       </c>
@@ -3982,7 +3988,7 @@
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>6</v>
@@ -3990,11 +3996,11 @@
     </row>
     <row r="129">
       <c r="A129" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="D129" s="5" t="s">
         <v>6</v>
@@ -4030,7 +4036,7 @@
       </c>
       <c r="B132" s="6"/>
       <c r="C132" s="7" t="s">
-        <v>226</v>
+        <v>243</v>
       </c>
       <c r="D132" s="5" t="s">
         <v>6</v>
@@ -4038,11 +4044,11 @@
     </row>
     <row r="133">
       <c r="A133" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B133" s="6"/>
       <c r="C133" s="7" t="s">
-        <v>244</v>
+        <v>228</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>6</v>
@@ -4121,7 +4127,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="8" t="s">
+      <c r="A140" s="5" t="s">
         <v>257</v>
       </c>
       <c r="B140" s="6"/>
@@ -4138,7 +4144,7 @@
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="7" t="s">
-        <v>232</v>
+        <v>260</v>
       </c>
       <c r="D141" s="5" t="s">
         <v>6</v>
@@ -4146,18 +4152,18 @@
     </row>
     <row r="142">
       <c r="A142" s="8" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B142" s="6"/>
       <c r="C142" s="7" t="s">
-        <v>261</v>
+        <v>234</v>
       </c>
       <c r="D142" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="5" t="s">
+      <c r="A143" s="8" t="s">
         <v>262</v>
       </c>
       <c r="B143" s="6"/>
@@ -4205,26 +4211,26 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="13" t="s">
+      <c r="A147" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="B147" s="14"/>
-      <c r="C147" s="13" t="s">
+      <c r="B147" s="6"/>
+      <c r="C147" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="D147" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="B148" s="16"/>
+      <c r="C148" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="D147" s="13" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="B148" s="6"/>
-      <c r="C148" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="D148" s="5" t="s">
+      <c r="D148" s="15" t="s">
         <v>6</v>
       </c>
     </row>
@@ -4409,7 +4415,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="8" t="s">
+      <c r="A164" s="5" t="s">
         <v>303</v>
       </c>
       <c r="B164" s="6"/>
@@ -4445,12 +4451,12 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="5" t="s">
+      <c r="A167" s="8" t="s">
         <v>309</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="7" t="s">
-        <v>239</v>
+        <v>310</v>
       </c>
       <c r="D167" s="5" t="s">
         <v>6</v>
@@ -4458,11 +4464,11 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>311</v>
+        <v>241</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
@@ -4565,7 +4571,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="15" t="s">
+      <c r="A177" s="5" t="s">
         <v>328</v>
       </c>
       <c r="B177" s="6"/>
@@ -4577,7 +4583,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="5" t="s">
+      <c r="A178" s="17" t="s">
         <v>330</v>
       </c>
       <c r="B178" s="6"/>
@@ -4625,7 +4631,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="8" t="s">
+      <c r="A182" s="5" t="s">
         <v>338</v>
       </c>
       <c r="B182" s="6"/>
@@ -4637,7 +4643,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="5" t="s">
+      <c r="A183" s="8" t="s">
         <v>340</v>
       </c>
       <c r="B183" s="6"/>
@@ -4810,7 +4816,7 @@
       </c>
       <c r="B197" s="6"/>
       <c r="C197" s="7" t="s">
-        <v>51</v>
+        <v>369</v>
       </c>
       <c r="D197" s="5" t="s">
         <v>6</v>
@@ -4818,11 +4824,11 @@
     </row>
     <row r="198">
       <c r="A198" s="5" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B198" s="6"/>
       <c r="C198" s="7" t="s">
-        <v>370</v>
+        <v>51</v>
       </c>
       <c r="D198" s="5" t="s">
         <v>6</v>
@@ -4853,7 +4859,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="10" t="s">
+      <c r="A201" s="5" t="s">
         <v>375</v>
       </c>
       <c r="B201" s="6"/>
@@ -4925,12 +4931,12 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="5" t="s">
+      <c r="A207" s="10" t="s">
         <v>387</v>
       </c>
       <c r="B207" s="6"/>
       <c r="C207" s="7" t="s">
-        <v>134</v>
+        <v>388</v>
       </c>
       <c r="D207" s="5" t="s">
         <v>6</v>
@@ -4938,11 +4944,11 @@
     </row>
     <row r="208">
       <c r="A208" s="5" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B208" s="6"/>
       <c r="C208" s="7" t="s">
-        <v>389</v>
+        <v>134</v>
       </c>
       <c r="D208" s="5" t="s">
         <v>6</v>
@@ -5081,26 +5087,26 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="16" t="s">
+      <c r="A220" s="5" t="s">
         <v>412</v>
       </c>
-      <c r="B220" s="17"/>
-      <c r="C220" s="18" t="s">
+      <c r="B220" s="6"/>
+      <c r="C220" s="7" t="s">
         <v>413</v>
       </c>
-      <c r="D220" s="16" t="s">
+      <c r="D220" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="5" t="s">
+      <c r="A221" s="18" t="s">
         <v>414</v>
       </c>
-      <c r="B221" s="6"/>
-      <c r="C221" s="7" t="s">
+      <c r="B221" s="19"/>
+      <c r="C221" s="20" t="s">
         <v>415</v>
       </c>
-      <c r="D221" s="5" t="s">
+      <c r="D221" s="18" t="s">
         <v>6</v>
       </c>
     </row>
@@ -5266,7 +5272,7 @@
       </c>
       <c r="B235" s="6"/>
       <c r="C235" s="7" t="s">
-        <v>176</v>
+        <v>443</v>
       </c>
       <c r="D235" s="5" t="s">
         <v>6</v>
@@ -5274,11 +5280,11 @@
     </row>
     <row r="236">
       <c r="A236" s="5" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B236" s="6"/>
       <c r="C236" s="7" t="s">
-        <v>444</v>
+        <v>178</v>
       </c>
       <c r="D236" s="5" t="s">
         <v>6</v>
@@ -5290,7 +5296,7 @@
       </c>
       <c r="B237" s="6"/>
       <c r="C237" s="7" t="s">
-        <v>315</v>
+        <v>446</v>
       </c>
       <c r="D237" s="5" t="s">
         <v>6</v>
@@ -5298,11 +5304,11 @@
     </row>
     <row r="238">
       <c r="A238" s="5" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B238" s="6"/>
       <c r="C238" s="7" t="s">
-        <v>447</v>
+        <v>317</v>
       </c>
       <c r="D238" s="5" t="s">
         <v>6</v>
@@ -5321,50 +5327,50 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="16" t="s">
+      <c r="A240" s="5" t="s">
         <v>450</v>
       </c>
-      <c r="B240" s="17"/>
-      <c r="C240" s="18" t="s">
-        <v>239</v>
-      </c>
-      <c r="D240" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="E240" s="19"/>
-      <c r="F240" s="19"/>
-      <c r="G240" s="19"/>
-      <c r="H240" s="19"/>
-      <c r="I240" s="19"/>
-      <c r="J240" s="19"/>
-      <c r="K240" s="19"/>
-      <c r="L240" s="19"/>
-      <c r="M240" s="19"/>
-      <c r="N240" s="19"/>
-      <c r="O240" s="19"/>
-      <c r="P240" s="19"/>
-      <c r="Q240" s="19"/>
-      <c r="R240" s="19"/>
-      <c r="S240" s="19"/>
-      <c r="T240" s="19"/>
-      <c r="U240" s="19"/>
-      <c r="V240" s="19"/>
-      <c r="W240" s="19"/>
-      <c r="X240" s="19"/>
-      <c r="Y240" s="19"/>
-      <c r="Z240" s="19"/>
+      <c r="B240" s="6"/>
+      <c r="C240" s="7" t="s">
+        <v>451</v>
+      </c>
+      <c r="D240" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="241">
-      <c r="A241" s="5" t="s">
-        <v>451</v>
-      </c>
-      <c r="B241" s="6"/>
-      <c r="C241" s="7" t="s">
+      <c r="A241" s="18" t="s">
         <v>452</v>
       </c>
-      <c r="D241" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="B241" s="19"/>
+      <c r="C241" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="D241" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="E241" s="21"/>
+      <c r="F241" s="21"/>
+      <c r="G241" s="21"/>
+      <c r="H241" s="21"/>
+      <c r="I241" s="21"/>
+      <c r="J241" s="21"/>
+      <c r="K241" s="21"/>
+      <c r="L241" s="21"/>
+      <c r="M241" s="21"/>
+      <c r="N241" s="21"/>
+      <c r="O241" s="21"/>
+      <c r="P241" s="21"/>
+      <c r="Q241" s="21"/>
+      <c r="R241" s="21"/>
+      <c r="S241" s="21"/>
+      <c r="T241" s="21"/>
+      <c r="U241" s="21"/>
+      <c r="V241" s="21"/>
+      <c r="W241" s="21"/>
+      <c r="X241" s="21"/>
+      <c r="Y241" s="21"/>
+      <c r="Z241" s="21"/>
     </row>
     <row r="242">
       <c r="A242" s="5" t="s">
@@ -5415,29 +5421,29 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="16" t="s">
+      <c r="A246" s="5" t="s">
         <v>461</v>
       </c>
-      <c r="B246" s="17"/>
-      <c r="C246" s="18" t="s">
+      <c r="B246" s="6"/>
+      <c r="C246" s="7" t="s">
         <v>462</v>
       </c>
-      <c r="D246" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="E246" s="19"/>
+      <c r="D246" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="247">
-      <c r="A247" s="5" t="s">
+      <c r="A247" s="18" t="s">
         <v>463</v>
       </c>
-      <c r="B247" s="6"/>
-      <c r="C247" s="7" t="s">
+      <c r="B247" s="19"/>
+      <c r="C247" s="20" t="s">
         <v>464</v>
       </c>
-      <c r="D247" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="D247" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="E247" s="21"/>
     </row>
     <row r="248">
       <c r="A248" s="5" t="s">
@@ -5565,7 +5571,7 @@
       </c>
       <c r="B258" s="6"/>
       <c r="C258" s="7" t="s">
-        <v>439</v>
+        <v>486</v>
       </c>
       <c r="D258" s="5" t="s">
         <v>6</v>
@@ -5573,11 +5579,11 @@
     </row>
     <row r="259">
       <c r="A259" s="5" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B259" s="6"/>
       <c r="C259" s="7" t="s">
-        <v>487</v>
+        <v>441</v>
       </c>
       <c r="D259" s="5" t="s">
         <v>6</v>
@@ -5673,7 +5679,7 @@
       </c>
       <c r="B267" s="6"/>
       <c r="C267" s="7" t="s">
-        <v>491</v>
+        <v>503</v>
       </c>
       <c r="D267" s="5" t="s">
         <v>6</v>
@@ -5681,7 +5687,7 @@
     </row>
     <row r="268">
       <c r="A268" s="5" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B268" s="6"/>
       <c r="C268" s="7" t="s">
@@ -5693,7 +5699,7 @@
     </row>
     <row r="269">
       <c r="A269" s="5" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B269" s="6"/>
       <c r="C269" s="7" t="s">
@@ -5705,7 +5711,7 @@
     </row>
     <row r="270">
       <c r="A270" s="5" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B270" s="6"/>
       <c r="C270" s="7" t="s">
@@ -5717,15 +5723,19 @@
     </row>
     <row r="271">
       <c r="A271" s="5" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B271" s="6"/>
-      <c r="C271" s="6"/>
-      <c r="D271" s="6"/>
+      <c r="C271" s="7" t="s">
+        <v>499</v>
+      </c>
+      <c r="D271" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="5" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B272" s="6"/>
       <c r="C272" s="6"/>
@@ -5733,15 +5743,11 @@
     </row>
     <row r="273">
       <c r="A273" s="5" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B273" s="6"/>
-      <c r="C273" s="7" t="s">
-        <v>509</v>
-      </c>
-      <c r="D273" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C273" s="6"/>
+      <c r="D273" s="6"/>
     </row>
     <row r="274">
       <c r="A274" s="5" t="s">
@@ -5845,7 +5851,7 @@
       </c>
       <c r="B282" s="6"/>
       <c r="C282" s="7" t="s">
-        <v>491</v>
+        <v>527</v>
       </c>
       <c r="D282" s="5" t="s">
         <v>6</v>
@@ -5853,11 +5859,11 @@
     </row>
     <row r="283">
       <c r="A283" s="5" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B283" s="6"/>
       <c r="C283" s="7" t="s">
-        <v>528</v>
+        <v>493</v>
       </c>
       <c r="D283" s="5" t="s">
         <v>6</v>
@@ -5941,7 +5947,7 @@
       </c>
       <c r="B290" s="6"/>
       <c r="C290" s="7" t="s">
-        <v>439</v>
+        <v>542</v>
       </c>
       <c r="D290" s="5" t="s">
         <v>6</v>
@@ -5949,11 +5955,11 @@
     </row>
     <row r="291">
       <c r="A291" s="5" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B291" s="6"/>
       <c r="C291" s="7" t="s">
-        <v>543</v>
+        <v>441</v>
       </c>
       <c r="D291" s="5" t="s">
         <v>6</v>
@@ -6109,7 +6115,7 @@
       </c>
       <c r="B304" s="6"/>
       <c r="C304" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D304" s="5" t="s">
         <v>6</v>
@@ -6117,11 +6123,11 @@
     </row>
     <row r="305">
       <c r="A305" s="5" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B305" s="6"/>
       <c r="C305" s="7" t="s">
-        <v>570</v>
+        <v>565</v>
       </c>
       <c r="D305" s="5" t="s">
         <v>6</v>
@@ -6152,7 +6158,7 @@
       </c>
     </row>
     <row r="308">
-      <c r="A308" s="20" t="s">
+      <c r="A308" s="5" t="s">
         <v>575</v>
       </c>
       <c r="B308" s="6"/>
@@ -6164,7 +6170,7 @@
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="21" t="s">
+      <c r="A309" s="22" t="s">
         <v>577</v>
       </c>
       <c r="B309" s="6"/>
@@ -6176,7 +6182,7 @@
       </c>
     </row>
     <row r="310">
-      <c r="A310" s="21" t="s">
+      <c r="A310" s="23" t="s">
         <v>579</v>
       </c>
       <c r="B310" s="6"/>
@@ -6188,7 +6194,7 @@
       </c>
     </row>
     <row r="311">
-      <c r="A311" s="21" t="s">
+      <c r="A311" s="23" t="s">
         <v>581</v>
       </c>
       <c r="B311" s="6"/>
@@ -6200,7 +6206,7 @@
       </c>
     </row>
     <row r="312">
-      <c r="A312" s="21" t="s">
+      <c r="A312" s="23" t="s">
         <v>583</v>
       </c>
       <c r="B312" s="6"/>
@@ -6212,7 +6218,7 @@
       </c>
     </row>
     <row r="313">
-      <c r="A313" s="21" t="s">
+      <c r="A313" s="23" t="s">
         <v>585</v>
       </c>
       <c r="B313" s="6"/>
@@ -6224,7 +6230,7 @@
       </c>
     </row>
     <row r="314">
-      <c r="A314" s="22" t="s">
+      <c r="A314" s="23" t="s">
         <v>587</v>
       </c>
       <c r="B314" s="6"/>
@@ -6236,7 +6242,7 @@
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="22" t="s">
+      <c r="A315" s="24" t="s">
         <v>589</v>
       </c>
       <c r="B315" s="6"/>
@@ -6248,7 +6254,7 @@
       </c>
     </row>
     <row r="316">
-      <c r="A316" s="22" t="s">
+      <c r="A316" s="24" t="s">
         <v>591</v>
       </c>
       <c r="B316" s="6"/>
@@ -6260,7 +6266,7 @@
       </c>
     </row>
     <row r="317">
-      <c r="A317" s="22" t="s">
+      <c r="A317" s="24" t="s">
         <v>593</v>
       </c>
       <c r="B317" s="6"/>
@@ -6272,7 +6278,7 @@
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="22" t="s">
+      <c r="A318" s="24" t="s">
         <v>595</v>
       </c>
       <c r="B318" s="6"/>
@@ -6284,7 +6290,7 @@
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="22" t="s">
+      <c r="A319" s="24" t="s">
         <v>597</v>
       </c>
       <c r="B319" s="6"/>
@@ -6296,7 +6302,7 @@
       </c>
     </row>
     <row r="320">
-      <c r="A320" s="5" t="s">
+      <c r="A320" s="24" t="s">
         <v>599</v>
       </c>
       <c r="B320" s="6"/>
@@ -6452,11 +6458,11 @@
       </c>
     </row>
     <row r="333">
-      <c r="A333" s="23" t="s">
+      <c r="A333" s="5" t="s">
         <v>625</v>
       </c>
       <c r="B333" s="6"/>
-      <c r="C333" s="24" t="s">
+      <c r="C333" s="7" t="s">
         <v>626</v>
       </c>
       <c r="D333" s="5" t="s">
@@ -6464,11 +6470,11 @@
       </c>
     </row>
     <row r="334">
-      <c r="A334" s="5" t="s">
+      <c r="A334" s="13" t="s">
         <v>627</v>
       </c>
       <c r="B334" s="6"/>
-      <c r="C334" s="7" t="s">
+      <c r="C334" s="14" t="s">
         <v>628</v>
       </c>
       <c r="D334" s="5" t="s">
@@ -6668,11 +6674,11 @@
       </c>
     </row>
     <row r="351">
-      <c r="A351" s="23" t="s">
+      <c r="A351" s="5" t="s">
         <v>661</v>
       </c>
       <c r="B351" s="6"/>
-      <c r="C351" s="24" t="s">
+      <c r="C351" s="7" t="s">
         <v>662</v>
       </c>
       <c r="D351" s="5" t="s">
@@ -6680,11 +6686,11 @@
       </c>
     </row>
     <row r="352">
-      <c r="A352" s="23" t="s">
+      <c r="A352" s="13" t="s">
         <v>663</v>
       </c>
       <c r="B352" s="6"/>
-      <c r="C352" s="24" t="s">
+      <c r="C352" s="14" t="s">
         <v>664</v>
       </c>
       <c r="D352" s="5" t="s">
@@ -6692,11 +6698,11 @@
       </c>
     </row>
     <row r="353">
-      <c r="A353" s="23" t="s">
+      <c r="A353" s="13" t="s">
         <v>665</v>
       </c>
       <c r="B353" s="6"/>
-      <c r="C353" s="24" t="s">
+      <c r="C353" s="14" t="s">
         <v>666</v>
       </c>
       <c r="D353" s="5" t="s">
@@ -6704,13 +6710,19 @@
       </c>
     </row>
     <row r="354">
-      <c r="A354" s="23"/>
+      <c r="A354" s="13" t="s">
+        <v>667</v>
+      </c>
       <c r="B354" s="6"/>
-      <c r="C354" s="6"/>
-      <c r="D354" s="6"/>
+      <c r="C354" s="14" t="s">
+        <v>668</v>
+      </c>
+      <c r="D354" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="355">
-      <c r="A355" s="6"/>
+      <c r="A355" s="13"/>
       <c r="B355" s="6"/>
       <c r="C355" s="6"/>
       <c r="D355" s="6"/>
@@ -11443,15 +11455,21 @@
       <c r="C1143" s="6"/>
       <c r="D1143" s="6"/>
     </row>
+    <row r="1144">
+      <c r="A1144" s="6"/>
+      <c r="B1144" s="6"/>
+      <c r="C1144" s="6"/>
+      <c r="D1144" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D270 D273:D353">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D271 D274:D354">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="A79"/>
-    <hyperlink r:id="rId2" ref="A177"/>
+    <hyperlink r:id="rId2" ref="A178"/>
   </hyperlinks>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
Bottom sheet to confirm ring deletion
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1158" uniqueCount="731">
   <si>
     <t>Key</t>
   </si>
@@ -50,6 +50,24 @@
   </si>
   <si>
     <t>Continue</t>
+  </si>
+  <si>
+    <t>url.terms_and_conditions</t>
+  </si>
+  <si>
+    <t>https://www.circular.xyz/en/terms-of-use</t>
+  </si>
+  <si>
+    <t>url.privacy</t>
+  </si>
+  <si>
+    <t>https://www.circular.xyz/en/privacy-policy</t>
+  </si>
+  <si>
+    <t>url.faq</t>
+  </si>
+  <si>
+    <t>https://www.circular.xyz/en/help#FAQ</t>
   </si>
   <si>
     <t>setup.scan.disabled.title</t>
@@ -189,6 +207,12 @@
     <t>ACTIVITY ANALYSIS</t>
   </si>
   <si>
+    <t>header.settings</t>
+  </si>
+  <si>
+    <t>Settings</t>
+  </si>
+  <si>
     <t>ring.battery.label</t>
   </si>
   <si>
@@ -442,6 +466,12 @@
   </si>
   <si>
     <t>Not enough information</t>
+  </si>
+  <si>
+    <t>global.done</t>
+  </si>
+  <si>
+    <t>Done</t>
   </si>
   <si>
     <t>home.sync.syncing</t>
@@ -969,9 +999,6 @@
   </si>
   <si>
     <t>drawer.settings</t>
-  </si>
-  <si>
-    <t>Settings</t>
   </si>
   <si>
     <t>drawer.close</t>
@@ -1933,6 +1960,34 @@
     <t>MAC address:</t>
   </si>
   <si>
+    <t>manage_rings.delete.validation.title</t>
+  </si>
+  <si>
+    <t>manage_rings.delete.validation.subtitle</t>
+  </si>
+  <si>
+    <t>Are you sure that you want to dissociate this ring from your account?</t>
+  </si>
+  <si>
+    <t>manage_rings.delete.validation.description</t>
+  </si>
+  <si>
+    <t>This will delete the configuration of your ring. 
+Please keep your ring and phone close to each other during this process if you wish to continue.</t>
+  </si>
+  <si>
+    <t>manage_rings.delete.validation.dissociate</t>
+  </si>
+  <si>
+    <t>Dissociate</t>
+  </si>
+  <si>
+    <t>manage_rings.delete.success.title</t>
+  </si>
+  <si>
+    <t>Ring successfully dissociated</t>
+  </si>
+  <si>
     <t>sleep.quality_score</t>
   </si>
   <si>
@@ -2086,13 +2141,127 @@
   <si>
     <t>I've noticed that you do not have any circle installed 🧐.
 Install circles through the add a circle menu to start using your ring and receive recommendations from me.</t>
+  </si>
+  <si>
+    <t>settings.general</t>
+  </si>
+  <si>
+    <t>settings.notifications.title</t>
+  </si>
+  <si>
+    <t>Notifications</t>
+  </si>
+  <si>
+    <t>settings.date_format.title</t>
+  </si>
+  <si>
+    <t>Date Format</t>
+  </si>
+  <si>
+    <t>settings.date_format.label</t>
+  </si>
+  <si>
+    <t>Date format to appear through your app.</t>
+  </si>
+  <si>
+    <t>settings.time_format</t>
+  </si>
+  <si>
+    <t>Time Format</t>
+  </si>
+  <si>
+    <t>settings.height_format</t>
+  </si>
+  <si>
+    <t>Height Format</t>
+  </si>
+  <si>
+    <t>settings.weight_format</t>
+  </si>
+  <si>
+    <t>Weight Format</t>
+  </si>
+  <si>
+    <t>settings.temperature_format</t>
+  </si>
+  <si>
+    <t>Temperature Format</t>
+  </si>
+  <si>
+    <t>settings.dark_mode</t>
+  </si>
+  <si>
+    <t>Dark Mode</t>
+  </si>
+  <si>
+    <t>settings.security</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>settings.logged_in</t>
+  </si>
+  <si>
+    <t>Logged in with</t>
+  </si>
+  <si>
+    <t>settings.2fa</t>
+  </si>
+  <si>
+    <t>Two Factor Authentification</t>
+  </si>
+  <si>
+    <t>settings.other</t>
+  </si>
+  <si>
+    <t>settings.clear_history</t>
+  </si>
+  <si>
+    <t>Clear data history</t>
+  </si>
+  <si>
+    <t>settings.terms</t>
+  </si>
+  <si>
+    <t>Terms &amp; Conditions</t>
+  </si>
+  <si>
+    <t>settings.privacy</t>
+  </si>
+  <si>
+    <t>Privacy &amp; Terms of Use</t>
+  </si>
+  <si>
+    <t>settings.app_version</t>
+  </si>
+  <si>
+    <t>App Version</t>
+  </si>
+  <si>
+    <t>settings.help</t>
+  </si>
+  <si>
+    <t>Help</t>
+  </si>
+  <si>
+    <t>settings.faq</t>
+  </si>
+  <si>
+    <t>FAQ</t>
+  </si>
+  <si>
+    <t>settings.support.title</t>
+  </si>
+  <si>
+    <t>Contact support</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -2106,6 +2275,14 @@
     <font>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF1155CC"/>
     </font>
     <font>
       <color rgb="FF000000"/>
@@ -2129,6 +2306,7 @@
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
     </font>
+    <font/>
   </fonts>
   <fills count="6">
     <fill>
@@ -2168,7 +2346,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2193,19 +2371,25 @@
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -2214,19 +2398,19 @@
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
@@ -2236,8 +2420,11 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2547,7 +2734,7 @@
         <v>13</v>
       </c>
       <c r="B6" s="6"/>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="5" t="s">
@@ -2559,7 +2746,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="6"/>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="9" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="5" t="s">
@@ -2567,12 +2754,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="5" t="s">
         <v>17</v>
       </c>
       <c r="B8" s="6"/>
-      <c r="C8" s="7" t="s">
-        <v>14</v>
+      <c r="C8" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>6</v>
@@ -2580,35 +2767,35 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>20</v>
+      <c r="A10" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>22</v>
+      <c r="A11" s="10" t="s">
+        <v>23</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>6</v>
@@ -2616,42 +2803,42 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="s">
-        <v>25</v>
+      <c r="A13" s="10" t="s">
+        <v>26</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="s">
-        <v>27</v>
+      <c r="A14" s="10" t="s">
+        <v>28</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="5" t="s">
         <v>29</v>
       </c>
       <c r="B15" s="6"/>
@@ -2663,7 +2850,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B16" s="6"/>
@@ -2675,7 +2862,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="11" t="s">
         <v>33</v>
       </c>
       <c r="B17" s="6"/>
@@ -2687,7 +2874,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="11" t="s">
         <v>35</v>
       </c>
       <c r="B18" s="6"/>
@@ -2699,7 +2886,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="11" t="s">
         <v>37</v>
       </c>
       <c r="B19" s="6"/>
@@ -2711,7 +2898,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="11" t="s">
         <v>39</v>
       </c>
       <c r="B20" s="6"/>
@@ -2740,7 +2927,7 @@
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>6</v>
@@ -2748,11 +2935,11 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>6</v>
@@ -2760,11 +2947,11 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>6</v>
@@ -2772,11 +2959,11 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="7" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>6</v>
@@ -2860,19 +3047,19 @@
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="7" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="s">
-        <v>63</v>
+      <c r="A33" s="5" t="s">
+        <v>64</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>6</v>
@@ -2880,11 +3067,11 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>6</v>
@@ -2892,11 +3079,11 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>6</v>
@@ -2904,23 +3091,23 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="s">
-        <v>68</v>
+      <c r="A37" s="10" t="s">
+        <v>71</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>6</v>
@@ -2928,11 +3115,11 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>6</v>
@@ -2940,11 +3127,11 @@
     </row>
     <row r="39">
       <c r="A39" s="5" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="7" t="s">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>6</v>
@@ -2952,11 +3139,11 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>6</v>
@@ -2964,11 +3151,11 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>6</v>
@@ -2976,11 +3163,11 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="7" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>6</v>
@@ -2988,11 +3175,11 @@
     </row>
     <row r="43">
       <c r="A43" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>6</v>
@@ -3000,11 +3187,11 @@
     </row>
     <row r="44">
       <c r="A44" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="7" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>6</v>
@@ -3012,11 +3199,11 @@
     </row>
     <row r="45">
       <c r="A45" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="7" t="s">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>6</v>
@@ -3024,11 +3211,11 @@
     </row>
     <row r="46">
       <c r="A46" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>6</v>
@@ -3036,11 +3223,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>83</v>
+        <v>42</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>6</v>
@@ -3076,7 +3263,7 @@
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="7" t="s">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>6</v>
@@ -3084,11 +3271,11 @@
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>6</v>
@@ -3096,11 +3283,11 @@
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>6</v>
@@ -3108,11 +3295,11 @@
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>6</v>
@@ -3120,11 +3307,11 @@
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
-        <v>96</v>
+        <v>57</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>6</v>
@@ -3208,7 +3395,7 @@
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="7" t="s">
-        <v>40</v>
+        <v>110</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>6</v>
@@ -3216,11 +3403,11 @@
     </row>
     <row r="62">
       <c r="A62" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B62" s="6"/>
       <c r="C62" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>6</v>
@@ -3228,11 +3415,11 @@
     </row>
     <row r="63">
       <c r="A63" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="7" t="s">
-        <v>38</v>
+        <v>114</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>6</v>
@@ -3240,11 +3427,11 @@
     </row>
     <row r="64">
       <c r="A64" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>6</v>
@@ -3252,11 +3439,11 @@
     </row>
     <row r="65">
       <c r="A65" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="6"/>
       <c r="C65" s="7" t="s">
-        <v>94</v>
+        <v>46</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>6</v>
@@ -3264,11 +3451,11 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="6"/>
       <c r="C66" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>6</v>
@@ -3276,11 +3463,11 @@
     </row>
     <row r="67">
       <c r="A67" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B67" s="6"/>
       <c r="C67" s="7" t="s">
-        <v>119</v>
+        <v>44</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>6</v>
@@ -3288,11 +3475,11 @@
     </row>
     <row r="68">
       <c r="A68" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>6</v>
@@ -3300,11 +3487,11 @@
     </row>
     <row r="69">
       <c r="A69" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" s="7" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>6</v>
@@ -3335,161 +3522,160 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="10" t="s">
+      <c r="A72" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="B72" s="6"/>
       <c r="C72" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B73" s="6"/>
+      <c r="C73" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D73" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B74" s="6"/>
+      <c r="C74" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="B75" s="6"/>
+      <c r="C75" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="C76" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D72" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="C73" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="D73" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="C74" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="D74" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C75" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="D75" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="C76" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D76" s="10" t="s">
+      <c r="D76" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="10" t="s">
-        <v>136</v>
+      <c r="A77" s="12" t="s">
+        <v>137</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D77" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D77" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="10" t="s">
-        <v>137</v>
+      <c r="A78" s="12" t="s">
+        <v>139</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="D78" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="D78" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="11" t="s">
-        <v>139</v>
+      <c r="A79" s="12" t="s">
+        <v>141</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="D79" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="D79" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="12" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="D80" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D80" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="B81" s="6"/>
+      <c r="A81" s="12" t="s">
+        <v>144</v>
+      </c>
       <c r="C81" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="D81" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D81" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="5" t="s">
+      <c r="A82" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="B82" s="6"/>
       <c r="C82" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="D82" s="5" t="s">
+      <c r="D82" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="5" t="s">
+      <c r="A83" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="B83" s="6"/>
       <c r="C83" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="D83" s="5" t="s">
+      <c r="D83" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="5" t="s">
+      <c r="A84" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="B84" s="6"/>
       <c r="C84" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="D84" s="5" t="s">
+      <c r="D84" s="12" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="5" t="s">
+      <c r="A85" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="B85" s="6"/>
       <c r="C85" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="D85" s="5" t="s">
+      <c r="D85" s="12" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3602,7 +3788,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="8" t="s">
+      <c r="A95" s="5" t="s">
         <v>171</v>
       </c>
       <c r="B95" s="6"/>
@@ -3614,7 +3800,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="8" t="s">
+      <c r="A96" s="5" t="s">
         <v>173</v>
       </c>
       <c r="B96" s="6"/>
@@ -3662,7 +3848,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="5" t="s">
+      <c r="A100" s="10" t="s">
         <v>181</v>
       </c>
       <c r="B100" s="6"/>
@@ -3674,7 +3860,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="s">
+      <c r="A101" s="10" t="s">
         <v>183</v>
       </c>
       <c r="B101" s="6"/>
@@ -3931,7 +4117,7 @@
       </c>
       <c r="B122" s="6"/>
       <c r="C122" s="7" t="s">
-        <v>40</v>
+        <v>226</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>6</v>
@@ -3939,11 +4125,11 @@
     </row>
     <row r="123">
       <c r="A123" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B123" s="6"/>
       <c r="C123" s="7" t="s">
-        <v>40</v>
+        <v>228</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>6</v>
@@ -3951,11 +4137,11 @@
     </row>
     <row r="124">
       <c r="A124" s="5" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B124" s="6"/>
       <c r="C124" s="7" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>6</v>
@@ -3963,11 +4149,11 @@
     </row>
     <row r="125">
       <c r="A125" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="B125" s="5"/>
+        <v>231</v>
+      </c>
+      <c r="B125" s="6"/>
       <c r="C125" s="7" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>6</v>
@@ -3975,11 +4161,11 @@
     </row>
     <row r="126">
       <c r="A126" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B126" s="6"/>
       <c r="C126" s="7" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D126" s="5" t="s">
         <v>6</v>
@@ -3987,11 +4173,11 @@
     </row>
     <row r="127">
       <c r="A127" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B127" s="6"/>
       <c r="C127" s="7" t="s">
-        <v>234</v>
+        <v>46</v>
       </c>
       <c r="D127" s="5" t="s">
         <v>6</v>
@@ -3999,11 +4185,11 @@
     </row>
     <row r="128">
       <c r="A128" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
-        <v>236</v>
+        <v>46</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>6</v>
@@ -4015,7 +4201,7 @@
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="D129" s="5" t="s">
         <v>6</v>
@@ -4023,11 +4209,11 @@
     </row>
     <row r="130">
       <c r="A130" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="B130" s="6"/>
+        <v>239</v>
+      </c>
+      <c r="B130" s="5"/>
       <c r="C130" s="7" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D130" s="5" t="s">
         <v>6</v>
@@ -4035,11 +4221,11 @@
     </row>
     <row r="131">
       <c r="A131" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B131" s="6"/>
       <c r="C131" s="7" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>6</v>
@@ -4047,11 +4233,11 @@
     </row>
     <row r="132">
       <c r="A132" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B132" s="6"/>
       <c r="C132" s="7" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D132" s="5" t="s">
         <v>6</v>
@@ -4059,11 +4245,11 @@
     </row>
     <row r="133">
       <c r="A133" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B133" s="6"/>
       <c r="C133" s="7" t="s">
-        <v>228</v>
+        <v>246</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>6</v>
@@ -4071,11 +4257,11 @@
     </row>
     <row r="134">
       <c r="A134" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B134" s="6"/>
       <c r="C134" s="7" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="D134" s="5" t="s">
         <v>6</v>
@@ -4083,11 +4269,11 @@
     </row>
     <row r="135">
       <c r="A135" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B135" s="6"/>
       <c r="C135" s="7" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D135" s="5" t="s">
         <v>6</v>
@@ -4095,11 +4281,11 @@
     </row>
     <row r="136">
       <c r="A136" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B136" s="6"/>
       <c r="C136" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D136" s="5" t="s">
         <v>6</v>
@@ -4107,11 +4293,11 @@
     </row>
     <row r="137">
       <c r="A137" s="5" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>6</v>
@@ -4119,11 +4305,11 @@
     </row>
     <row r="138">
       <c r="A138" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B138" s="6"/>
       <c r="C138" s="7" t="s">
-        <v>254</v>
+        <v>238</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>6</v>
@@ -4154,7 +4340,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="8" t="s">
+      <c r="A141" s="5" t="s">
         <v>259</v>
       </c>
       <c r="B141" s="6"/>
@@ -4166,24 +4352,24 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="8" t="s">
+      <c r="A142" s="5" t="s">
         <v>261</v>
       </c>
       <c r="B142" s="6"/>
       <c r="C142" s="7" t="s">
-        <v>234</v>
+        <v>262</v>
       </c>
       <c r="D142" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="8" t="s">
-        <v>262</v>
+      <c r="A143" s="5" t="s">
+        <v>263</v>
       </c>
       <c r="B143" s="6"/>
       <c r="C143" s="7" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D143" s="5" t="s">
         <v>6</v>
@@ -4191,11 +4377,11 @@
     </row>
     <row r="144">
       <c r="A144" s="5" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B144" s="6"/>
       <c r="C144" s="7" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D144" s="5" t="s">
         <v>6</v>
@@ -4203,59 +4389,59 @@
     </row>
     <row r="145">
       <c r="A145" s="5" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B145" s="6"/>
       <c r="C145" s="7" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D145" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="5" t="s">
-        <v>268</v>
+      <c r="A146" s="10" t="s">
+        <v>269</v>
       </c>
       <c r="B146" s="6"/>
       <c r="C146" s="7" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D146" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="5" t="s">
-        <v>270</v>
+      <c r="A147" s="10" t="s">
+        <v>271</v>
       </c>
       <c r="B147" s="6"/>
       <c r="C147" s="7" t="s">
-        <v>271</v>
+        <v>244</v>
       </c>
       <c r="D147" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="13" t="s">
+      <c r="A148" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="B148" s="14"/>
-      <c r="C148" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="D148" s="13" t="s">
+      <c r="B148" s="6"/>
+      <c r="C148" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="D148" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B149" s="6"/>
       <c r="C149" s="7" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D149" s="5" t="s">
         <v>6</v>
@@ -4263,11 +4449,11 @@
     </row>
     <row r="150">
       <c r="A150" s="5" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B150" s="6"/>
       <c r="C150" s="7" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D150" s="5" t="s">
         <v>6</v>
@@ -4275,11 +4461,11 @@
     </row>
     <row r="151">
       <c r="A151" s="5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B151" s="6"/>
       <c r="C151" s="7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D151" s="5" t="s">
         <v>6</v>
@@ -4287,25 +4473,25 @@
     </row>
     <row r="152">
       <c r="A152" s="5" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B152" s="6"/>
       <c r="C152" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D152" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="5" t="s">
-        <v>281</v>
-      </c>
-      <c r="B153" s="6"/>
-      <c r="C153" s="7" t="s">
+      <c r="A153" s="15" t="s">
         <v>282</v>
       </c>
-      <c r="D153" s="5" t="s">
+      <c r="B153" s="16"/>
+      <c r="C153" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="D153" s="15" t="s">
         <v>6</v>
       </c>
     </row>
@@ -4442,7 +4628,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="8" t="s">
+      <c r="A165" s="5" t="s">
         <v>305</v>
       </c>
       <c r="B165" s="6"/>
@@ -4454,7 +4640,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="8" t="s">
+      <c r="A166" s="5" t="s">
         <v>307</v>
       </c>
       <c r="B166" s="6"/>
@@ -4466,7 +4652,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="8" t="s">
+      <c r="A167" s="5" t="s">
         <v>309</v>
       </c>
       <c r="B167" s="6"/>
@@ -4483,7 +4669,7 @@
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>241</v>
+        <v>312</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
@@ -4491,47 +4677,47 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="7" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D169" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="5" t="s">
-        <v>314</v>
+      <c r="A170" s="10" t="s">
+        <v>315</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D170" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="5" t="s">
-        <v>316</v>
+      <c r="A171" s="10" t="s">
+        <v>317</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="7" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D171" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="5" t="s">
-        <v>318</v>
+      <c r="A172" s="10" t="s">
+        <v>319</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="7" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D172" s="5" t="s">
         <v>6</v>
@@ -4539,11 +4725,11 @@
     </row>
     <row r="173">
       <c r="A173" s="5" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="7" t="s">
-        <v>321</v>
+        <v>251</v>
       </c>
       <c r="D173" s="5" t="s">
         <v>6</v>
@@ -4555,7 +4741,7 @@
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>323</v>
+        <v>65</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
@@ -4563,11 +4749,11 @@
     </row>
     <row r="175">
       <c r="A175" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
@@ -4575,11 +4761,11 @@
     </row>
     <row r="176">
       <c r="A176" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
@@ -4587,11 +4773,11 @@
     </row>
     <row r="177">
       <c r="A177" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
@@ -4599,23 +4785,23 @@
     </row>
     <row r="178">
       <c r="A178" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="D178" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="s">
         <v>331</v>
-      </c>
-      <c r="D178" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="15" t="s">
-        <v>332</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
@@ -4623,11 +4809,11 @@
     </row>
     <row r="180">
       <c r="A180" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
@@ -4635,11 +4821,11 @@
     </row>
     <row r="181">
       <c r="A181" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
@@ -4647,11 +4833,11 @@
     </row>
     <row r="182">
       <c r="A182" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>6</v>
@@ -4659,23 +4845,23 @@
     </row>
     <row r="183">
       <c r="A183" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="D183" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="17" t="s">
         <v>341</v>
-      </c>
-      <c r="D183" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="8" t="s">
-        <v>342</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D184" s="5" t="s">
         <v>6</v>
@@ -4683,11 +4869,11 @@
     </row>
     <row r="185">
       <c r="A185" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D185" s="5" t="s">
         <v>6</v>
@@ -4695,11 +4881,11 @@
     </row>
     <row r="186">
       <c r="A186" s="5" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="7" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D186" s="5" t="s">
         <v>6</v>
@@ -4707,11 +4893,11 @@
     </row>
     <row r="187">
       <c r="A187" s="5" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>6</v>
@@ -4719,23 +4905,23 @@
     </row>
     <row r="188">
       <c r="A188" s="5" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="D188" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="10" t="s">
         <v>351</v>
-      </c>
-      <c r="D188" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" s="5" t="s">
-        <v>352</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="7" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>6</v>
@@ -4743,11 +4929,11 @@
     </row>
     <row r="190">
       <c r="A190" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>6</v>
@@ -4755,11 +4941,11 @@
     </row>
     <row r="191">
       <c r="A191" s="5" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>6</v>
@@ -4767,11 +4953,11 @@
     </row>
     <row r="192">
       <c r="A192" s="5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
@@ -4779,11 +4965,11 @@
     </row>
     <row r="193">
       <c r="A193" s="5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
@@ -4791,11 +4977,11 @@
     </row>
     <row r="194">
       <c r="A194" s="5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B194" s="6"/>
       <c r="C194" s="7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>6</v>
@@ -4803,11 +4989,11 @@
     </row>
     <row r="195">
       <c r="A195" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B195" s="6"/>
       <c r="C195" s="7" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D195" s="5" t="s">
         <v>6</v>
@@ -4815,11 +5001,11 @@
     </row>
     <row r="196">
       <c r="A196" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B196" s="6"/>
       <c r="C196" s="7" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D196" s="5" t="s">
         <v>6</v>
@@ -4827,11 +5013,11 @@
     </row>
     <row r="197">
       <c r="A197" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B197" s="6"/>
       <c r="C197" s="7" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="D197" s="5" t="s">
         <v>6</v>
@@ -4839,11 +5025,11 @@
     </row>
     <row r="198">
       <c r="A198" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B198" s="6"/>
       <c r="C198" s="7" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="D198" s="5" t="s">
         <v>6</v>
@@ -4851,11 +5037,11 @@
     </row>
     <row r="199">
       <c r="A199" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B199" s="6"/>
       <c r="C199" s="7" t="s">
-        <v>51</v>
+        <v>372</v>
       </c>
       <c r="D199" s="5" t="s">
         <v>6</v>
@@ -4898,7 +5084,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="10" t="s">
+      <c r="A203" s="5" t="s">
         <v>379</v>
       </c>
       <c r="B203" s="6"/>
@@ -4910,79 +5096,79 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="10" t="s">
+      <c r="A204" s="5" t="s">
         <v>381</v>
       </c>
       <c r="B204" s="6"/>
       <c r="C204" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D204" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="5" t="s">
         <v>382</v>
-      </c>
-      <c r="D204" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" s="10" t="s">
-        <v>383</v>
       </c>
       <c r="B205" s="6"/>
       <c r="C205" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="D205" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="5" t="s">
         <v>384</v>
-      </c>
-      <c r="D205" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" s="10" t="s">
-        <v>385</v>
       </c>
       <c r="B206" s="6"/>
       <c r="C206" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="D206" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="5" t="s">
         <v>386</v>
-      </c>
-      <c r="D206" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" s="10" t="s">
-        <v>387</v>
       </c>
       <c r="B207" s="6"/>
       <c r="C207" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="D207" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="12" t="s">
         <v>388</v>
-      </c>
-      <c r="D207" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" s="10" t="s">
-        <v>389</v>
       </c>
       <c r="B208" s="6"/>
       <c r="C208" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="D208" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="12" t="s">
         <v>390</v>
-      </c>
-      <c r="D208" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" s="5" t="s">
-        <v>391</v>
       </c>
       <c r="B209" s="6"/>
       <c r="C209" s="7" t="s">
-        <v>134</v>
+        <v>391</v>
       </c>
       <c r="D209" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="5" t="s">
+      <c r="A210" s="12" t="s">
         <v>392</v>
       </c>
       <c r="B210" s="6"/>
@@ -4994,7 +5180,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="5" t="s">
+      <c r="A211" s="12" t="s">
         <v>394</v>
       </c>
       <c r="B211" s="6"/>
@@ -5006,7 +5192,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="5" t="s">
+      <c r="A212" s="12" t="s">
         <v>396</v>
       </c>
       <c r="B212" s="6"/>
@@ -5018,7 +5204,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="5" t="s">
+      <c r="A213" s="12" t="s">
         <v>398</v>
       </c>
       <c r="B213" s="6"/>
@@ -5035,7 +5221,7 @@
       </c>
       <c r="B214" s="6"/>
       <c r="C214" s="7" t="s">
-        <v>401</v>
+        <v>142</v>
       </c>
       <c r="D214" s="5" t="s">
         <v>6</v>
@@ -5043,11 +5229,11 @@
     </row>
     <row r="215">
       <c r="A215" s="5" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B215" s="6"/>
       <c r="C215" s="7" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D215" s="5" t="s">
         <v>6</v>
@@ -5055,11 +5241,11 @@
     </row>
     <row r="216">
       <c r="A216" s="5" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B216" s="6"/>
       <c r="C216" s="7" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D216" s="5" t="s">
         <v>6</v>
@@ -5067,11 +5253,11 @@
     </row>
     <row r="217">
       <c r="A217" s="5" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B217" s="6"/>
       <c r="C217" s="7" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="D217" s="5" t="s">
         <v>6</v>
@@ -5079,11 +5265,11 @@
     </row>
     <row r="218">
       <c r="A218" s="5" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B218" s="6"/>
       <c r="C218" s="7" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="D218" s="5" t="s">
         <v>6</v>
@@ -5091,11 +5277,11 @@
     </row>
     <row r="219">
       <c r="A219" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B219" s="6"/>
       <c r="C219" s="7" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D219" s="5" t="s">
         <v>6</v>
@@ -5103,11 +5289,11 @@
     </row>
     <row r="220">
       <c r="A220" s="5" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B220" s="6"/>
       <c r="C220" s="7" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="D220" s="5" t="s">
         <v>6</v>
@@ -5115,35 +5301,35 @@
     </row>
     <row r="221">
       <c r="A221" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B221" s="6"/>
       <c r="C221" s="7" t="s">
+        <v>414</v>
+      </c>
+      <c r="D221" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="5" t="s">
         <v>415</v>
       </c>
-      <c r="D221" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" s="16" t="s">
+      <c r="B222" s="6"/>
+      <c r="C222" s="7" t="s">
         <v>416</v>
       </c>
-      <c r="B222" s="17"/>
-      <c r="C222" s="18" t="s">
-        <v>417</v>
-      </c>
-      <c r="D222" s="16" t="s">
+      <c r="D222" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="5" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B223" s="6"/>
       <c r="C223" s="7" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="D223" s="5" t="s">
         <v>6</v>
@@ -5151,11 +5337,11 @@
     </row>
     <row r="224">
       <c r="A224" s="5" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B224" s="6"/>
       <c r="C224" s="7" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D224" s="5" t="s">
         <v>6</v>
@@ -5163,11 +5349,11 @@
     </row>
     <row r="225">
       <c r="A225" s="5" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B225" s="6"/>
       <c r="C225" s="7" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D225" s="5" t="s">
         <v>6</v>
@@ -5175,35 +5361,35 @@
     </row>
     <row r="226">
       <c r="A226" s="5" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B226" s="6"/>
       <c r="C226" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="D226" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="18" t="s">
         <v>425</v>
       </c>
-      <c r="D226" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" s="5" t="s">
+      <c r="B227" s="19"/>
+      <c r="C227" s="20" t="s">
         <v>426</v>
       </c>
-      <c r="B227" s="6"/>
-      <c r="C227" s="7" t="s">
-        <v>427</v>
-      </c>
-      <c r="D227" s="5" t="s">
+      <c r="D227" s="18" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="5" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B228" s="6"/>
       <c r="C228" s="7" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D228" s="5" t="s">
         <v>6</v>
@@ -5211,11 +5397,11 @@
     </row>
     <row r="229">
       <c r="A229" s="5" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B229" s="6"/>
       <c r="C229" s="7" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="D229" s="5" t="s">
         <v>6</v>
@@ -5223,11 +5409,11 @@
     </row>
     <row r="230">
       <c r="A230" s="5" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B230" s="6"/>
       <c r="C230" s="7" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D230" s="5" t="s">
         <v>6</v>
@@ -5235,11 +5421,11 @@
     </row>
     <row r="231">
       <c r="A231" s="5" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B231" s="6"/>
       <c r="C231" s="7" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="D231" s="5" t="s">
         <v>6</v>
@@ -5247,11 +5433,11 @@
     </row>
     <row r="232">
       <c r="A232" s="5" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B232" s="6"/>
       <c r="C232" s="7" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="D232" s="5" t="s">
         <v>6</v>
@@ -5259,11 +5445,11 @@
     </row>
     <row r="233">
       <c r="A233" s="5" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B233" s="6"/>
       <c r="C233" s="7" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="D233" s="5" t="s">
         <v>6</v>
@@ -5271,11 +5457,11 @@
     </row>
     <row r="234">
       <c r="A234" s="5" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B234" s="6"/>
       <c r="C234" s="7" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="D234" s="5" t="s">
         <v>6</v>
@@ -5283,11 +5469,11 @@
     </row>
     <row r="235">
       <c r="A235" s="5" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B235" s="6"/>
       <c r="C235" s="7" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="D235" s="5" t="s">
         <v>6</v>
@@ -5295,11 +5481,11 @@
     </row>
     <row r="236">
       <c r="A236" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B236" s="6"/>
       <c r="C236" s="7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D236" s="5" t="s">
         <v>6</v>
@@ -5307,11 +5493,11 @@
     </row>
     <row r="237">
       <c r="A237" s="5" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B237" s="6"/>
       <c r="C237" s="7" t="s">
-        <v>178</v>
+        <v>446</v>
       </c>
       <c r="D237" s="5" t="s">
         <v>6</v>
@@ -5335,7 +5521,7 @@
       </c>
       <c r="B239" s="6"/>
       <c r="C239" s="7" t="s">
-        <v>319</v>
+        <v>450</v>
       </c>
       <c r="D239" s="5" t="s">
         <v>6</v>
@@ -5343,11 +5529,11 @@
     </row>
     <row r="240">
       <c r="A240" s="5" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B240" s="6"/>
       <c r="C240" s="7" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D240" s="5" t="s">
         <v>6</v>
@@ -5355,57 +5541,35 @@
     </row>
     <row r="241">
       <c r="A241" s="5" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B241" s="6"/>
       <c r="C241" s="7" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D241" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="16" t="s">
-        <v>454</v>
-      </c>
-      <c r="B242" s="17"/>
-      <c r="C242" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="D242" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="E242" s="19"/>
-      <c r="F242" s="19"/>
-      <c r="G242" s="19"/>
-      <c r="H242" s="19"/>
-      <c r="I242" s="19"/>
-      <c r="J242" s="19"/>
-      <c r="K242" s="19"/>
-      <c r="L242" s="19"/>
-      <c r="M242" s="19"/>
-      <c r="N242" s="19"/>
-      <c r="O242" s="19"/>
-      <c r="P242" s="19"/>
-      <c r="Q242" s="19"/>
-      <c r="R242" s="19"/>
-      <c r="S242" s="19"/>
-      <c r="T242" s="19"/>
-      <c r="U242" s="19"/>
-      <c r="V242" s="19"/>
-      <c r="W242" s="19"/>
-      <c r="X242" s="19"/>
-      <c r="Y242" s="19"/>
-      <c r="Z242" s="19"/>
+      <c r="A242" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B242" s="6"/>
+      <c r="C242" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D242" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="5" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B243" s="6"/>
       <c r="C243" s="7" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D243" s="5" t="s">
         <v>6</v>
@@ -5413,11 +5577,11 @@
     </row>
     <row r="244">
       <c r="A244" s="5" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B244" s="6"/>
       <c r="C244" s="7" t="s">
-        <v>458</v>
+        <v>328</v>
       </c>
       <c r="D244" s="5" t="s">
         <v>6</v>
@@ -5448,37 +5612,58 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="5" t="s">
+      <c r="A247" s="18" t="s">
         <v>463</v>
       </c>
-      <c r="B247" s="6"/>
-      <c r="C247" s="7" t="s">
+      <c r="B247" s="19"/>
+      <c r="C247" s="20" t="s">
+        <v>251</v>
+      </c>
+      <c r="D247" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="E247" s="21"/>
+      <c r="F247" s="21"/>
+      <c r="G247" s="21"/>
+      <c r="H247" s="21"/>
+      <c r="I247" s="21"/>
+      <c r="J247" s="21"/>
+      <c r="K247" s="21"/>
+      <c r="L247" s="21"/>
+      <c r="M247" s="21"/>
+      <c r="N247" s="21"/>
+      <c r="O247" s="21"/>
+      <c r="P247" s="21"/>
+      <c r="Q247" s="21"/>
+      <c r="R247" s="21"/>
+      <c r="S247" s="21"/>
+      <c r="T247" s="21"/>
+      <c r="U247" s="21"/>
+      <c r="V247" s="21"/>
+      <c r="W247" s="21"/>
+      <c r="X247" s="21"/>
+      <c r="Y247" s="21"/>
+      <c r="Z247" s="21"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="5" t="s">
         <v>464</v>
       </c>
-      <c r="D247" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" s="16" t="s">
+      <c r="B248" s="6"/>
+      <c r="C248" s="7" t="s">
         <v>465</v>
       </c>
-      <c r="B248" s="17"/>
-      <c r="C248" s="18" t="s">
-        <v>466</v>
-      </c>
-      <c r="D248" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="E248" s="19"/>
+      <c r="D248" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="5" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B249" s="6"/>
       <c r="C249" s="7" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D249" s="5" t="s">
         <v>6</v>
@@ -5486,11 +5671,11 @@
     </row>
     <row r="250">
       <c r="A250" s="5" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B250" s="6"/>
       <c r="C250" s="7" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="D250" s="5" t="s">
         <v>6</v>
@@ -5498,11 +5683,11 @@
     </row>
     <row r="251">
       <c r="A251" s="5" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B251" s="6"/>
       <c r="C251" s="7" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D251" s="5" t="s">
         <v>6</v>
@@ -5510,35 +5695,36 @@
     </row>
     <row r="252">
       <c r="A252" s="5" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B252" s="6"/>
       <c r="C252" s="7" t="s">
+        <v>473</v>
+      </c>
+      <c r="D252" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="18" t="s">
         <v>474</v>
       </c>
-      <c r="D252" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" s="5" t="s">
+      <c r="B253" s="19"/>
+      <c r="C253" s="20" t="s">
         <v>475</v>
       </c>
-      <c r="B253" s="6"/>
-      <c r="C253" s="7" t="s">
-        <v>476</v>
-      </c>
-      <c r="D253" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="D253" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="E253" s="21"/>
     </row>
     <row r="254">
       <c r="A254" s="5" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B254" s="6"/>
       <c r="C254" s="7" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D254" s="5" t="s">
         <v>6</v>
@@ -5546,11 +5732,11 @@
     </row>
     <row r="255">
       <c r="A255" s="5" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B255" s="6"/>
       <c r="C255" s="7" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="D255" s="5" t="s">
         <v>6</v>
@@ -5558,11 +5744,11 @@
     </row>
     <row r="256">
       <c r="A256" s="5" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B256" s="6"/>
       <c r="C256" s="7" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="D256" s="5" t="s">
         <v>6</v>
@@ -5570,11 +5756,11 @@
     </row>
     <row r="257">
       <c r="A257" s="5" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B257" s="6"/>
       <c r="C257" s="7" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="D257" s="5" t="s">
         <v>6</v>
@@ -5582,11 +5768,11 @@
     </row>
     <row r="258">
       <c r="A258" s="5" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B258" s="6"/>
       <c r="C258" s="7" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D258" s="5" t="s">
         <v>6</v>
@@ -5594,11 +5780,11 @@
     </row>
     <row r="259">
       <c r="A259" s="5" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B259" s="6"/>
       <c r="C259" s="7" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D259" s="5" t="s">
         <v>6</v>
@@ -5606,11 +5792,11 @@
     </row>
     <row r="260">
       <c r="A260" s="5" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B260" s="6"/>
       <c r="C260" s="7" t="s">
-        <v>443</v>
+        <v>489</v>
       </c>
       <c r="D260" s="5" t="s">
         <v>6</v>
@@ -5670,7 +5856,7 @@
       </c>
       <c r="B265" s="6"/>
       <c r="C265" s="7" t="s">
-        <v>499</v>
+        <v>452</v>
       </c>
       <c r="D265" s="5" t="s">
         <v>6</v>
@@ -5678,11 +5864,11 @@
     </row>
     <row r="266">
       <c r="A266" s="5" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B266" s="6"/>
       <c r="C266" s="7" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D266" s="5" t="s">
         <v>6</v>
@@ -5690,11 +5876,11 @@
     </row>
     <row r="267">
       <c r="A267" s="5" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B267" s="6"/>
       <c r="C267" s="7" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D267" s="5" t="s">
         <v>6</v>
@@ -5702,11 +5888,11 @@
     </row>
     <row r="268">
       <c r="A268" s="5" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B268" s="6"/>
       <c r="C268" s="7" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="D268" s="5" t="s">
         <v>6</v>
@@ -5714,11 +5900,11 @@
     </row>
     <row r="269">
       <c r="A269" s="5" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B269" s="6"/>
       <c r="C269" s="7" t="s">
-        <v>495</v>
+        <v>506</v>
       </c>
       <c r="D269" s="5" t="s">
         <v>6</v>
@@ -5730,7 +5916,7 @@
       </c>
       <c r="B270" s="6"/>
       <c r="C270" s="7" t="s">
-        <v>497</v>
+        <v>508</v>
       </c>
       <c r="D270" s="5" t="s">
         <v>6</v>
@@ -5738,11 +5924,11 @@
     </row>
     <row r="271">
       <c r="A271" s="5" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B271" s="6"/>
       <c r="C271" s="7" t="s">
-        <v>499</v>
+        <v>510</v>
       </c>
       <c r="D271" s="5" t="s">
         <v>6</v>
@@ -5750,11 +5936,11 @@
     </row>
     <row r="272">
       <c r="A272" s="5" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B272" s="6"/>
       <c r="C272" s="7" t="s">
-        <v>501</v>
+        <v>512</v>
       </c>
       <c r="D272" s="5" t="s">
         <v>6</v>
@@ -5762,27 +5948,35 @@
     </row>
     <row r="273">
       <c r="A273" s="5" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="B273" s="6"/>
-      <c r="C273" s="6"/>
-      <c r="D273" s="6"/>
+      <c r="C273" s="7" t="s">
+        <v>514</v>
+      </c>
+      <c r="D273" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="5" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="B274" s="6"/>
-      <c r="C274" s="6"/>
-      <c r="D274" s="6"/>
+      <c r="C274" s="7" t="s">
+        <v>504</v>
+      </c>
+      <c r="D274" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="5" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="B275" s="6"/>
       <c r="C275" s="7" t="s">
-        <v>513</v>
+        <v>506</v>
       </c>
       <c r="D275" s="5" t="s">
         <v>6</v>
@@ -5790,11 +5984,11 @@
     </row>
     <row r="276">
       <c r="A276" s="5" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="B276" s="6"/>
       <c r="C276" s="7" t="s">
-        <v>515</v>
+        <v>508</v>
       </c>
       <c r="D276" s="5" t="s">
         <v>6</v>
@@ -5802,11 +5996,11 @@
     </row>
     <row r="277">
       <c r="A277" s="5" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B277" s="6"/>
       <c r="C277" s="7" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="D277" s="5" t="s">
         <v>6</v>
@@ -5814,35 +6008,27 @@
     </row>
     <row r="278">
       <c r="A278" s="5" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B278" s="6"/>
-      <c r="C278" s="7" t="s">
-        <v>519</v>
-      </c>
-      <c r="D278" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C278" s="6"/>
+      <c r="D278" s="6"/>
     </row>
     <row r="279">
       <c r="A279" s="5" t="s">
         <v>520</v>
       </c>
       <c r="B279" s="6"/>
-      <c r="C279" s="7" t="s">
-        <v>521</v>
-      </c>
-      <c r="D279" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C279" s="6"/>
+      <c r="D279" s="6"/>
     </row>
     <row r="280">
       <c r="A280" s="5" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B280" s="6"/>
       <c r="C280" s="7" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D280" s="5" t="s">
         <v>6</v>
@@ -5850,11 +6036,11 @@
     </row>
     <row r="281">
       <c r="A281" s="5" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B281" s="6"/>
       <c r="C281" s="7" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="D281" s="5" t="s">
         <v>6</v>
@@ -5862,11 +6048,11 @@
     </row>
     <row r="282">
       <c r="A282" s="5" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B282" s="6"/>
       <c r="C282" s="7" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="D282" s="5" t="s">
         <v>6</v>
@@ -5874,11 +6060,11 @@
     </row>
     <row r="283">
       <c r="A283" s="5" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B283" s="6"/>
       <c r="C283" s="7" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="D283" s="5" t="s">
         <v>6</v>
@@ -5886,11 +6072,11 @@
     </row>
     <row r="284">
       <c r="A284" s="5" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B284" s="6"/>
       <c r="C284" s="7" t="s">
-        <v>495</v>
+        <v>530</v>
       </c>
       <c r="D284" s="5" t="s">
         <v>6</v>
@@ -5950,7 +6136,7 @@
       </c>
       <c r="B289" s="6"/>
       <c r="C289" s="7" t="s">
-        <v>540</v>
+        <v>504</v>
       </c>
       <c r="D289" s="5" t="s">
         <v>6</v>
@@ -5958,11 +6144,11 @@
     </row>
     <row r="290">
       <c r="A290" s="5" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B290" s="6"/>
       <c r="C290" s="7" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="D290" s="5" t="s">
         <v>6</v>
@@ -5970,11 +6156,11 @@
     </row>
     <row r="291">
       <c r="A291" s="5" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B291" s="6"/>
       <c r="C291" s="7" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="D291" s="5" t="s">
         <v>6</v>
@@ -5982,11 +6168,11 @@
     </row>
     <row r="292">
       <c r="A292" s="5" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B292" s="6"/>
       <c r="C292" s="7" t="s">
-        <v>443</v>
+        <v>545</v>
       </c>
       <c r="D292" s="5" t="s">
         <v>6</v>
@@ -6046,7 +6232,7 @@
       </c>
       <c r="B297" s="6"/>
       <c r="C297" s="7" t="s">
-        <v>555</v>
+        <v>452</v>
       </c>
       <c r="D297" s="5" t="s">
         <v>6</v>
@@ -6054,11 +6240,11 @@
     </row>
     <row r="298">
       <c r="A298" s="5" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B298" s="6"/>
       <c r="C298" s="7" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D298" s="5" t="s">
         <v>6</v>
@@ -6066,11 +6252,11 @@
     </row>
     <row r="299">
       <c r="A299" s="5" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B299" s="6"/>
       <c r="C299" s="7" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="D299" s="5" t="s">
         <v>6</v>
@@ -6078,11 +6264,11 @@
     </row>
     <row r="300">
       <c r="A300" s="5" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B300" s="6"/>
       <c r="C300" s="7" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="D300" s="5" t="s">
         <v>6</v>
@@ -6090,11 +6276,11 @@
     </row>
     <row r="301">
       <c r="A301" s="5" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B301" s="6"/>
       <c r="C301" s="7" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="D301" s="5" t="s">
         <v>6</v>
@@ -6102,11 +6288,11 @@
     </row>
     <row r="302">
       <c r="A302" s="5" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B302" s="6"/>
       <c r="C302" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D302" s="5" t="s">
         <v>6</v>
@@ -6114,11 +6300,11 @@
     </row>
     <row r="303">
       <c r="A303" s="5" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B303" s="6"/>
       <c r="C303" s="7" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="D303" s="5" t="s">
         <v>6</v>
@@ -6126,11 +6312,11 @@
     </row>
     <row r="304">
       <c r="A304" s="5" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B304" s="6"/>
       <c r="C304" s="7" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="D304" s="5" t="s">
         <v>6</v>
@@ -6138,11 +6324,11 @@
     </row>
     <row r="305">
       <c r="A305" s="5" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B305" s="6"/>
       <c r="C305" s="7" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D305" s="5" t="s">
         <v>6</v>
@@ -6150,11 +6336,11 @@
     </row>
     <row r="306">
       <c r="A306" s="5" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B306" s="6"/>
       <c r="C306" s="7" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="D306" s="5" t="s">
         <v>6</v>
@@ -6197,7 +6383,7 @@
       </c>
     </row>
     <row r="310">
-      <c r="A310" s="20" t="s">
+      <c r="A310" s="5" t="s">
         <v>579</v>
       </c>
       <c r="B310" s="6"/>
@@ -6209,192 +6395,192 @@
       </c>
     </row>
     <row r="311">
-      <c r="A311" s="21" t="s">
+      <c r="A311" s="5" t="s">
         <v>581</v>
       </c>
       <c r="B311" s="6"/>
       <c r="C311" s="7" t="s">
+        <v>576</v>
+      </c>
+      <c r="D311" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="5" t="s">
         <v>582</v>
-      </c>
-      <c r="D311" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" s="21" t="s">
-        <v>583</v>
       </c>
       <c r="B312" s="6"/>
       <c r="C312" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="D312" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="5" t="s">
         <v>584</v>
-      </c>
-      <c r="D312" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" s="21" t="s">
-        <v>585</v>
       </c>
       <c r="B313" s="6"/>
       <c r="C313" s="7" t="s">
+        <v>585</v>
+      </c>
+      <c r="D313" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="5" t="s">
         <v>586</v>
-      </c>
-      <c r="D313" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" s="21" t="s">
-        <v>587</v>
       </c>
       <c r="B314" s="6"/>
       <c r="C314" s="7" t="s">
+        <v>587</v>
+      </c>
+      <c r="D314" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="22" t="s">
         <v>588</v>
-      </c>
-      <c r="D314" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" s="21" t="s">
-        <v>589</v>
       </c>
       <c r="B315" s="6"/>
       <c r="C315" s="7" t="s">
+        <v>589</v>
+      </c>
+      <c r="D315" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="23" t="s">
         <v>590</v>
-      </c>
-      <c r="D315" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" s="22" t="s">
-        <v>591</v>
       </c>
       <c r="B316" s="6"/>
       <c r="C316" s="7" t="s">
+        <v>591</v>
+      </c>
+      <c r="D316" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="23" t="s">
         <v>592</v>
-      </c>
-      <c r="D316" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" s="22" t="s">
-        <v>593</v>
       </c>
       <c r="B317" s="6"/>
       <c r="C317" s="7" t="s">
+        <v>593</v>
+      </c>
+      <c r="D317" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="23" t="s">
         <v>594</v>
-      </c>
-      <c r="D317" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" s="22" t="s">
-        <v>595</v>
       </c>
       <c r="B318" s="6"/>
       <c r="C318" s="7" t="s">
+        <v>595</v>
+      </c>
+      <c r="D318" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="23" t="s">
         <v>596</v>
-      </c>
-      <c r="D318" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" s="22" t="s">
-        <v>597</v>
       </c>
       <c r="B319" s="6"/>
       <c r="C319" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="D319" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="23" t="s">
         <v>598</v>
-      </c>
-      <c r="D319" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" s="22" t="s">
-        <v>599</v>
       </c>
       <c r="B320" s="6"/>
       <c r="C320" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="D320" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="24" t="s">
         <v>600</v>
-      </c>
-      <c r="D320" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" s="22" t="s">
-        <v>601</v>
       </c>
       <c r="B321" s="6"/>
       <c r="C321" s="7" t="s">
+        <v>601</v>
+      </c>
+      <c r="D321" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="24" t="s">
         <v>602</v>
-      </c>
-      <c r="D321" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" s="5" t="s">
-        <v>603</v>
       </c>
       <c r="B322" s="6"/>
       <c r="C322" s="7" t="s">
+        <v>603</v>
+      </c>
+      <c r="D322" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="24" t="s">
         <v>604</v>
-      </c>
-      <c r="D322" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" s="5" t="s">
-        <v>605</v>
       </c>
       <c r="B323" s="6"/>
       <c r="C323" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="D323" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="24" t="s">
         <v>606</v>
-      </c>
-      <c r="D323" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" s="5" t="s">
-        <v>607</v>
       </c>
       <c r="B324" s="6"/>
       <c r="C324" s="7" t="s">
+        <v>607</v>
+      </c>
+      <c r="D324" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="24" t="s">
         <v>608</v>
-      </c>
-      <c r="D324" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" s="5" t="s">
-        <v>609</v>
       </c>
       <c r="B325" s="6"/>
       <c r="C325" s="7" t="s">
+        <v>609</v>
+      </c>
+      <c r="D325" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="24" t="s">
         <v>610</v>
-      </c>
-      <c r="D325" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" s="5" t="s">
-        <v>611</v>
       </c>
       <c r="B326" s="6"/>
       <c r="C326" s="7" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D326" s="5" t="s">
         <v>6</v>
@@ -6402,11 +6588,11 @@
     </row>
     <row r="327">
       <c r="A327" s="5" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B327" s="6"/>
       <c r="C327" s="7" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D327" s="5" t="s">
         <v>6</v>
@@ -6414,11 +6600,11 @@
     </row>
     <row r="328">
       <c r="A328" s="5" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B328" s="6"/>
       <c r="C328" s="7" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D328" s="5" t="s">
         <v>6</v>
@@ -6426,11 +6612,11 @@
     </row>
     <row r="329">
       <c r="A329" s="5" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B329" s="6"/>
       <c r="C329" s="7" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D329" s="5" t="s">
         <v>6</v>
@@ -6438,11 +6624,11 @@
     </row>
     <row r="330">
       <c r="A330" s="5" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B330" s="6"/>
       <c r="C330" s="7" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D330" s="5" t="s">
         <v>6</v>
@@ -6450,11 +6636,11 @@
     </row>
     <row r="331">
       <c r="A331" s="5" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B331" s="6"/>
       <c r="C331" s="7" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D331" s="5" t="s">
         <v>6</v>
@@ -6462,11 +6648,11 @@
     </row>
     <row r="332">
       <c r="A332" s="5" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B332" s="6"/>
       <c r="C332" s="7" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D332" s="5" t="s">
         <v>6</v>
@@ -6474,11 +6660,11 @@
     </row>
     <row r="333">
       <c r="A333" s="5" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B333" s="6"/>
       <c r="C333" s="7" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D333" s="5" t="s">
         <v>6</v>
@@ -6486,11 +6672,11 @@
     </row>
     <row r="334">
       <c r="A334" s="5" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B334" s="6"/>
       <c r="C334" s="7" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D334" s="5" t="s">
         <v>6</v>
@@ -6498,11 +6684,11 @@
     </row>
     <row r="335">
       <c r="A335" s="5" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B335" s="6"/>
       <c r="C335" s="7" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D335" s="5" t="s">
         <v>6</v>
@@ -6510,11 +6696,11 @@
     </row>
     <row r="336">
       <c r="A336" s="5" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B336" s="6"/>
       <c r="C336" s="7" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D336" s="5" t="s">
         <v>6</v>
@@ -6522,11 +6708,11 @@
     </row>
     <row r="337">
       <c r="A337" s="5" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B337" s="6"/>
       <c r="C337" s="7" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D337" s="5" t="s">
         <v>6</v>
@@ -6534,11 +6720,11 @@
     </row>
     <row r="338">
       <c r="A338" s="5" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B338" s="6"/>
       <c r="C338" s="7" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D338" s="5" t="s">
         <v>6</v>
@@ -6546,11 +6732,11 @@
     </row>
     <row r="339">
       <c r="A339" s="5" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B339" s="6"/>
       <c r="C339" s="7" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D339" s="5" t="s">
         <v>6</v>
@@ -6558,11 +6744,11 @@
     </row>
     <row r="340">
       <c r="A340" s="5" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B340" s="6"/>
       <c r="C340" s="7" t="s">
-        <v>640</v>
+        <v>446</v>
       </c>
       <c r="D340" s="5" t="s">
         <v>6</v>
@@ -6570,11 +6756,11 @@
     </row>
     <row r="341">
       <c r="A341" s="5" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="B341" s="6"/>
       <c r="C341" s="7" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="D341" s="5" t="s">
         <v>6</v>
@@ -6582,11 +6768,11 @@
     </row>
     <row r="342">
       <c r="A342" s="5" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B342" s="6"/>
       <c r="C342" s="7" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="D342" s="5" t="s">
         <v>6</v>
@@ -6594,11 +6780,11 @@
     </row>
     <row r="343">
       <c r="A343" s="5" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B343" s="6"/>
       <c r="C343" s="7" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="D343" s="5" t="s">
         <v>6</v>
@@ -6606,11 +6792,11 @@
     </row>
     <row r="344">
       <c r="A344" s="5" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="B344" s="6"/>
       <c r="C344" s="7" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="D344" s="5" t="s">
         <v>6</v>
@@ -6618,11 +6804,11 @@
     </row>
     <row r="345">
       <c r="A345" s="5" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B345" s="6"/>
       <c r="C345" s="7" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="D345" s="5" t="s">
         <v>6</v>
@@ -6630,11 +6816,11 @@
     </row>
     <row r="346">
       <c r="A346" s="5" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B346" s="6"/>
       <c r="C346" s="7" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D346" s="5" t="s">
         <v>6</v>
@@ -6642,11 +6828,11 @@
     </row>
     <row r="347">
       <c r="A347" s="5" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="B347" s="6"/>
       <c r="C347" s="7" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D347" s="5" t="s">
         <v>6</v>
@@ -6654,11 +6840,11 @@
     </row>
     <row r="348">
       <c r="A348" s="5" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="B348" s="6"/>
       <c r="C348" s="7" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D348" s="5" t="s">
         <v>6</v>
@@ -6666,11 +6852,11 @@
     </row>
     <row r="349">
       <c r="A349" s="5" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B349" s="6"/>
       <c r="C349" s="7" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D349" s="5" t="s">
         <v>6</v>
@@ -6678,11 +6864,11 @@
     </row>
     <row r="350">
       <c r="A350" s="5" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="B350" s="6"/>
       <c r="C350" s="7" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="D350" s="5" t="s">
         <v>6</v>
@@ -6690,11 +6876,11 @@
     </row>
     <row r="351">
       <c r="A351" s="5" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="B351" s="6"/>
       <c r="C351" s="7" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D351" s="5" t="s">
         <v>6</v>
@@ -6702,11 +6888,11 @@
     </row>
     <row r="352">
       <c r="A352" s="5" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="B352" s="6"/>
       <c r="C352" s="7" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D352" s="5" t="s">
         <v>6</v>
@@ -6714,11 +6900,11 @@
     </row>
     <row r="353">
       <c r="A353" s="5" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="B353" s="6"/>
       <c r="C353" s="7" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="D353" s="5" t="s">
         <v>6</v>
@@ -6726,11 +6912,11 @@
     </row>
     <row r="354">
       <c r="A354" s="5" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="B354" s="6"/>
       <c r="C354" s="7" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="D354" s="5" t="s">
         <v>6</v>
@@ -6738,11 +6924,11 @@
     </row>
     <row r="355">
       <c r="A355" s="5" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="B355" s="6"/>
       <c r="C355" s="7" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="D355" s="5" t="s">
         <v>6</v>
@@ -6750,11 +6936,11 @@
     </row>
     <row r="356">
       <c r="A356" s="5" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B356" s="6"/>
       <c r="C356" s="7" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="D356" s="5" t="s">
         <v>6</v>
@@ -6762,199 +6948,375 @@
     </row>
     <row r="357">
       <c r="A357" s="5" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B357" s="6"/>
       <c r="C357" s="7" t="s">
+        <v>672</v>
+      </c>
+      <c r="D357" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="5" t="s">
+        <v>673</v>
+      </c>
+      <c r="B358" s="6"/>
+      <c r="C358" s="7" t="s">
         <v>674</v>
       </c>
-      <c r="D357" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="358">
-      <c r="A358" s="6"/>
-      <c r="B358" s="6"/>
-      <c r="C358" s="23"/>
       <c r="D358" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="359">
-      <c r="A359" s="6"/>
+      <c r="A359" s="5" t="s">
+        <v>675</v>
+      </c>
       <c r="B359" s="6"/>
-      <c r="C359" s="7"/>
+      <c r="C359" s="7" t="s">
+        <v>676</v>
+      </c>
       <c r="D359" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="360">
-      <c r="A360" s="6"/>
+      <c r="A360" s="5" t="s">
+        <v>677</v>
+      </c>
       <c r="B360" s="6"/>
-      <c r="C360" s="6"/>
-      <c r="D360" s="6"/>
+      <c r="C360" s="7" t="s">
+        <v>678</v>
+      </c>
+      <c r="D360" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="361">
-      <c r="A361" s="6"/>
+      <c r="A361" s="5" t="s">
+        <v>679</v>
+      </c>
       <c r="B361" s="6"/>
-      <c r="C361" s="6"/>
-      <c r="D361" s="6"/>
+      <c r="C361" s="7" t="s">
+        <v>680</v>
+      </c>
+      <c r="D361" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="362">
-      <c r="A362" s="6"/>
+      <c r="A362" s="5" t="s">
+        <v>681</v>
+      </c>
       <c r="B362" s="6"/>
-      <c r="C362" s="6"/>
-      <c r="D362" s="6"/>
+      <c r="C362" s="7" t="s">
+        <v>682</v>
+      </c>
+      <c r="D362" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="363">
-      <c r="A363" s="6"/>
+      <c r="A363" s="5" t="s">
+        <v>683</v>
+      </c>
       <c r="B363" s="6"/>
-      <c r="C363" s="6"/>
-      <c r="D363" s="6"/>
+      <c r="C363" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="D363" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="364">
-      <c r="A364" s="6"/>
+      <c r="A364" s="5" t="s">
+        <v>685</v>
+      </c>
       <c r="B364" s="6"/>
-      <c r="C364" s="6"/>
-      <c r="D364" s="6"/>
+      <c r="C364" s="7" t="s">
+        <v>686</v>
+      </c>
+      <c r="D364" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="365">
-      <c r="A365" s="6"/>
+      <c r="A365" s="5" t="s">
+        <v>687</v>
+      </c>
       <c r="B365" s="6"/>
-      <c r="C365" s="6"/>
-      <c r="D365" s="6"/>
+      <c r="C365" s="7" t="s">
+        <v>688</v>
+      </c>
+      <c r="D365" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="366">
-      <c r="A366" s="6"/>
+      <c r="A366" s="5" t="s">
+        <v>689</v>
+      </c>
       <c r="B366" s="6"/>
-      <c r="C366" s="6"/>
-      <c r="D366" s="6"/>
+      <c r="C366" s="7" t="s">
+        <v>690</v>
+      </c>
+      <c r="D366" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="367">
-      <c r="A367" s="6"/>
+      <c r="A367" s="5" t="s">
+        <v>691</v>
+      </c>
       <c r="B367" s="6"/>
-      <c r="C367" s="6"/>
-      <c r="D367" s="6"/>
+      <c r="C367" s="7" t="s">
+        <v>692</v>
+      </c>
+      <c r="D367" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="368">
-      <c r="A368" s="6"/>
+      <c r="A368" s="5" t="s">
+        <v>693</v>
+      </c>
       <c r="B368" s="6"/>
-      <c r="C368" s="6"/>
-      <c r="D368" s="6"/>
+      <c r="C368" s="7" t="s">
+        <v>621</v>
+      </c>
+      <c r="D368" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="369">
-      <c r="A369" s="6"/>
+      <c r="A369" s="5" t="s">
+        <v>694</v>
+      </c>
       <c r="B369" s="6"/>
-      <c r="C369" s="6"/>
-      <c r="D369" s="6"/>
+      <c r="C369" s="7" t="s">
+        <v>695</v>
+      </c>
+      <c r="D369" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="370">
-      <c r="A370" s="6"/>
+      <c r="A370" s="25" t="s">
+        <v>696</v>
+      </c>
       <c r="B370" s="6"/>
-      <c r="C370" s="6"/>
-      <c r="D370" s="6"/>
+      <c r="C370" s="7" t="s">
+        <v>697</v>
+      </c>
+      <c r="D370" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="371">
-      <c r="A371" s="6"/>
+      <c r="A371" s="25" t="s">
+        <v>698</v>
+      </c>
       <c r="B371" s="6"/>
-      <c r="C371" s="6"/>
-      <c r="D371" s="6"/>
+      <c r="C371" s="26" t="s">
+        <v>699</v>
+      </c>
+      <c r="D371" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="372">
-      <c r="A372" s="6"/>
+      <c r="A372" s="5" t="s">
+        <v>700</v>
+      </c>
       <c r="B372" s="6"/>
-      <c r="C372" s="6"/>
-      <c r="D372" s="6"/>
+      <c r="C372" s="7" t="s">
+        <v>701</v>
+      </c>
+      <c r="D372" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="373">
-      <c r="A373" s="6"/>
+      <c r="A373" s="5" t="s">
+        <v>702</v>
+      </c>
       <c r="B373" s="6"/>
-      <c r="C373" s="6"/>
-      <c r="D373" s="6"/>
+      <c r="C373" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="D373" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="374">
-      <c r="A374" s="6"/>
+      <c r="A374" s="5" t="s">
+        <v>704</v>
+      </c>
       <c r="B374" s="6"/>
-      <c r="C374" s="6"/>
-      <c r="D374" s="6"/>
+      <c r="C374" s="7" t="s">
+        <v>705</v>
+      </c>
+      <c r="D374" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="375">
-      <c r="A375" s="6"/>
+      <c r="A375" s="5" t="s">
+        <v>706</v>
+      </c>
       <c r="B375" s="6"/>
-      <c r="C375" s="6"/>
-      <c r="D375" s="6"/>
+      <c r="C375" s="7" t="s">
+        <v>707</v>
+      </c>
+      <c r="D375" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="376">
-      <c r="A376" s="6"/>
+      <c r="A376" s="5" t="s">
+        <v>708</v>
+      </c>
       <c r="B376" s="6"/>
-      <c r="C376" s="6"/>
-      <c r="D376" s="6"/>
+      <c r="C376" s="7" t="s">
+        <v>709</v>
+      </c>
+      <c r="D376" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="377">
-      <c r="A377" s="6"/>
+      <c r="A377" s="5" t="s">
+        <v>710</v>
+      </c>
       <c r="B377" s="6"/>
-      <c r="C377" s="6"/>
-      <c r="D377" s="6"/>
+      <c r="C377" s="7" t="s">
+        <v>711</v>
+      </c>
+      <c r="D377" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="378">
-      <c r="A378" s="6"/>
+      <c r="A378" s="5" t="s">
+        <v>712</v>
+      </c>
       <c r="B378" s="6"/>
-      <c r="C378" s="6"/>
-      <c r="D378" s="6"/>
+      <c r="C378" s="7" t="s">
+        <v>713</v>
+      </c>
+      <c r="D378" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="379">
-      <c r="A379" s="6"/>
+      <c r="A379" s="5" t="s">
+        <v>714</v>
+      </c>
       <c r="B379" s="6"/>
-      <c r="C379" s="6"/>
-      <c r="D379" s="6"/>
+      <c r="C379" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="D379" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="380">
-      <c r="A380" s="6"/>
+      <c r="A380" s="5" t="s">
+        <v>716</v>
+      </c>
       <c r="B380" s="6"/>
-      <c r="C380" s="6"/>
-      <c r="D380" s="6"/>
+      <c r="C380" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="D380" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="381">
-      <c r="A381" s="6"/>
+      <c r="A381" s="5" t="s">
+        <v>717</v>
+      </c>
       <c r="B381" s="6"/>
-      <c r="C381" s="6"/>
-      <c r="D381" s="6"/>
+      <c r="C381" s="7" t="s">
+        <v>718</v>
+      </c>
+      <c r="D381" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="382">
-      <c r="A382" s="6"/>
+      <c r="A382" s="5" t="s">
+        <v>719</v>
+      </c>
       <c r="B382" s="6"/>
-      <c r="C382" s="6"/>
-      <c r="D382" s="6"/>
+      <c r="C382" s="7" t="s">
+        <v>720</v>
+      </c>
+      <c r="D382" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="383">
-      <c r="A383" s="6"/>
+      <c r="A383" s="10" t="s">
+        <v>721</v>
+      </c>
       <c r="B383" s="6"/>
-      <c r="C383" s="6"/>
-      <c r="D383" s="6"/>
+      <c r="C383" s="7" t="s">
+        <v>722</v>
+      </c>
+      <c r="D383" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="384">
-      <c r="A384" s="6"/>
+      <c r="A384" s="10" t="s">
+        <v>723</v>
+      </c>
       <c r="B384" s="6"/>
-      <c r="C384" s="6"/>
-      <c r="D384" s="6"/>
+      <c r="C384" s="7" t="s">
+        <v>724</v>
+      </c>
+      <c r="D384" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="385">
-      <c r="A385" s="6"/>
+      <c r="A385" s="10" t="s">
+        <v>725</v>
+      </c>
       <c r="B385" s="6"/>
-      <c r="C385" s="6"/>
-      <c r="D385" s="6"/>
+      <c r="C385" s="7" t="s">
+        <v>726</v>
+      </c>
+      <c r="D385" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="386">
-      <c r="A386" s="6"/>
+      <c r="A386" s="5" t="s">
+        <v>727</v>
+      </c>
       <c r="B386" s="6"/>
-      <c r="C386" s="6"/>
-      <c r="D386" s="6"/>
+      <c r="C386" s="7" t="s">
+        <v>728</v>
+      </c>
+      <c r="D386" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="387">
-      <c r="A387" s="6"/>
+      <c r="A387" s="10" t="s">
+        <v>729</v>
+      </c>
       <c r="B387" s="6"/>
-      <c r="C387" s="6"/>
-      <c r="D387" s="6"/>
+      <c r="C387" s="7" t="s">
+        <v>730</v>
+      </c>
+      <c r="D387" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="6"/>
@@ -11504,19 +11866,85 @@
       <c r="C1145" s="6"/>
       <c r="D1145" s="6"/>
     </row>
+    <row r="1146">
+      <c r="A1146" s="6"/>
+      <c r="B1146" s="6"/>
+      <c r="C1146" s="6"/>
+      <c r="D1146" s="6"/>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="6"/>
+      <c r="B1147" s="6"/>
+      <c r="C1147" s="6"/>
+      <c r="D1147" s="6"/>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="6"/>
+      <c r="B1148" s="6"/>
+      <c r="C1148" s="6"/>
+      <c r="D1148" s="6"/>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="6"/>
+      <c r="B1149" s="6"/>
+      <c r="C1149" s="6"/>
+      <c r="D1149" s="6"/>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="6"/>
+      <c r="B1150" s="6"/>
+      <c r="C1150" s="6"/>
+      <c r="D1150" s="6"/>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="6"/>
+      <c r="B1151" s="6"/>
+      <c r="C1151" s="6"/>
+      <c r="D1151" s="6"/>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="6"/>
+      <c r="B1152" s="6"/>
+      <c r="C1152" s="6"/>
+      <c r="D1152" s="6"/>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="6"/>
+      <c r="B1153" s="6"/>
+      <c r="C1153" s="6"/>
+      <c r="D1153" s="6"/>
+    </row>
+    <row r="1154">
+      <c r="A1154" s="6"/>
+      <c r="B1154" s="6"/>
+      <c r="C1154" s="6"/>
+      <c r="D1154" s="6"/>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="6"/>
+      <c r="B1155" s="6"/>
+      <c r="C1155" s="6"/>
+      <c r="D1155" s="6"/>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="6"/>
+      <c r="B1156" s="6"/>
+      <c r="C1156" s="6"/>
+      <c r="D1156" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D272 D275:D357">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D277 D280:D387">
       <formula1>"Validé,A valider"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D358:D359">
-      <formula1>"A valider"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A79"/>
-    <hyperlink r:id="rId2" ref="A179"/>
+    <hyperlink r:id="rId1" ref="C6"/>
+    <hyperlink r:id="rId2" ref="C7"/>
+    <hyperlink r:id="rId3" ref="C8"/>
+    <hyperlink r:id="rId4" ref="A83"/>
+    <hyperlink r:id="rId5" ref="A184"/>
   </hyperlinks>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Correctly dissociate ring from account and locally
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -1954,10 +1954,10 @@
     <t>Version</t>
   </si>
   <si>
-    <t>manage_rings.ring.mac_address_prefix</t>
-  </si>
-  <si>
-    <t>MAC address:</t>
+    <t>manage_rings.ring.snu_prefix</t>
+  </si>
+  <si>
+    <t>SNU:</t>
   </si>
   <si>
     <t>manage_rings.delete.validation.title</t>
@@ -6731,11 +6731,11 @@
       </c>
     </row>
     <row r="339">
-      <c r="A339" s="5" t="s">
+      <c r="A339" s="25" t="s">
         <v>636</v>
       </c>
       <c r="B339" s="6"/>
-      <c r="C339" s="7" t="s">
+      <c r="C339" s="26" t="s">
         <v>637</v>
       </c>
       <c r="D339" s="5" t="s">
@@ -7103,7 +7103,7 @@
       </c>
     </row>
     <row r="370">
-      <c r="A370" s="25" t="s">
+      <c r="A370" s="5" t="s">
         <v>696</v>
       </c>
       <c r="B370" s="6"/>
@@ -7115,11 +7115,11 @@
       </c>
     </row>
     <row r="371">
-      <c r="A371" s="25" t="s">
+      <c r="A371" s="5" t="s">
         <v>698</v>
       </c>
       <c r="B371" s="6"/>
-      <c r="C371" s="26" t="s">
+      <c r="C371" s="7" t="s">
         <v>699</v>
       </c>
       <c r="D371" s="5" t="s">

</xml_diff>

<commit_message>
i18n on default ring name
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1158" uniqueCount="731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1161" uniqueCount="733">
   <si>
     <t>Key</t>
   </si>
@@ -531,7 +531,7 @@
     <t>home.circles.live.label</t>
   </si>
   <si>
-    <t>Live</t>
+    <t>Live measurement</t>
   </si>
   <si>
     <t>home.circles.alarm.label</t>
@@ -1400,145 +1400,145 @@
     <t>alarm.new.other.title</t>
   </si>
   <si>
+    <t>alarm.new.edit_vibration.alert</t>
+  </si>
+  <si>
+    <t>Alert</t>
+  </si>
+  <si>
+    <t>alarm.wake_up_score</t>
+  </si>
+  <si>
+    <t>alarm.new.time.edit</t>
+  </si>
+  <si>
+    <t>Edit alarm time</t>
+  </si>
+  <si>
+    <t>alarm.week_overview</t>
+  </si>
+  <si>
+    <t>banner.calibration.title</t>
+  </si>
+  <si>
+    <t>Calibration period</t>
+  </si>
+  <si>
+    <t>banner.calibration.message</t>
+  </si>
+  <si>
+    <t>Keep wearing your ring during the entirety of the {days} days calibration period for improved results!</t>
+  </si>
+  <si>
+    <t>profile.header.title</t>
+  </si>
+  <si>
+    <t>alarm.new.edit_vibration.type.discharge</t>
+  </si>
+  <si>
+    <t>Discharge</t>
+  </si>
+  <si>
+    <t>header.profile_advanced_information</t>
+  </si>
+  <si>
+    <t>ADVANCED INFORMATION</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.about_you</t>
+  </si>
+  <si>
+    <t>About you</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.lifestyle_info</t>
+  </si>
+  <si>
+    <t>Lifestyle information</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.title</t>
+  </si>
+  <si>
+    <t>Work Time</t>
+  </si>
+  <si>
+    <t>alarm.new.label.placeholder</t>
+  </si>
+  <si>
+    <t>Enter label here</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.day</t>
+  </si>
+  <si>
+    <t>Day Worker</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.work_time.night</t>
+  </si>
+  <si>
+    <t>Night Worker</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.title</t>
+  </si>
+  <si>
+    <t>Physical Disabilities</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.description</t>
+  </si>
+  <si>
+    <t>If you suffer from any disability, Circular will calibrate more realistic goals to account for your condition.</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.none</t>
+  </si>
+  <si>
+    <t>No physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.moderate</t>
+  </si>
+  <si>
+    <t>Moderate physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.physical_disability.total</t>
+  </si>
+  <si>
+    <t>Total physical disability</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.title</t>
+  </si>
+  <si>
+    <t>Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.none</t>
+  </si>
+  <si>
+    <t>No Sleep Disorder</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.insomnia</t>
+  </si>
+  <si>
+    <t>Insomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.hypersomnia</t>
+  </si>
+  <si>
+    <t>Hypersomnia</t>
+  </si>
+  <si>
+    <t>profile_advanced_info.sleep_disorder.other</t>
+  </si>
+  <si>
     <t>Other</t>
-  </si>
-  <si>
-    <t>alarm.new.edit_vibration.alert</t>
-  </si>
-  <si>
-    <t>Alert</t>
-  </si>
-  <si>
-    <t>alarm.wake_up_score</t>
-  </si>
-  <si>
-    <t>alarm.new.time.edit</t>
-  </si>
-  <si>
-    <t>Edit alarm time</t>
-  </si>
-  <si>
-    <t>alarm.week_overview</t>
-  </si>
-  <si>
-    <t>banner.calibration.title</t>
-  </si>
-  <si>
-    <t>Calibration period</t>
-  </si>
-  <si>
-    <t>banner.calibration.message</t>
-  </si>
-  <si>
-    <t>Keep wearing your ring during the entirety of the {days} days calibration period for improved results!</t>
-  </si>
-  <si>
-    <t>profile.header.title</t>
-  </si>
-  <si>
-    <t>alarm.new.edit_vibration.type.discharge</t>
-  </si>
-  <si>
-    <t>Discharge</t>
-  </si>
-  <si>
-    <t>header.profile_advanced_information</t>
-  </si>
-  <si>
-    <t>ADVANCED INFORMATION</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.about_you</t>
-  </si>
-  <si>
-    <t>About you</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.lifestyle_info</t>
-  </si>
-  <si>
-    <t>Lifestyle information</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.work_time.title</t>
-  </si>
-  <si>
-    <t>Work Time</t>
-  </si>
-  <si>
-    <t>alarm.new.label.placeholder</t>
-  </si>
-  <si>
-    <t>Enter label here</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.work_time.day</t>
-  </si>
-  <si>
-    <t>Day Worker</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.work_time.night</t>
-  </si>
-  <si>
-    <t>Night Worker</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.title</t>
-  </si>
-  <si>
-    <t>Physical Disabilities</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.description</t>
-  </si>
-  <si>
-    <t>If you suffer from any disability, Circular will calibrate more realistic goals to account for your condition.</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.none</t>
-  </si>
-  <si>
-    <t>No physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.moderate</t>
-  </si>
-  <si>
-    <t>Moderate physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.physical_disability.total</t>
-  </si>
-  <si>
-    <t>Total physical disability</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.title</t>
-  </si>
-  <si>
-    <t>Sleep Disorder</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.none</t>
-  </si>
-  <si>
-    <t>No Sleep Disorder</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.insomnia</t>
-  </si>
-  <si>
-    <t>Insomnia</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.hypersomnia</t>
-  </si>
-  <si>
-    <t>Hypersomnia</t>
-  </si>
-  <si>
-    <t>profile_advanced_info.sleep_disorder.other</t>
   </si>
   <si>
     <t>profile_advanced_info.sleeping_pills.title</t>
@@ -1940,6 +1940,12 @@
   </si>
   <si>
     <t>Vibrate</t>
+  </si>
+  <si>
+    <t>manage_rings.ring.default_name</t>
+  </si>
+  <si>
+    <t>Circular</t>
   </si>
   <si>
     <t>manage_rings.ring.sync_date_prefix</t>
@@ -5533,7 +5539,7 @@
       </c>
       <c r="B240" s="6"/>
       <c r="C240" s="7" t="s">
-        <v>452</v>
+        <v>65</v>
       </c>
       <c r="D240" s="5" t="s">
         <v>6</v>
@@ -5541,11 +5547,11 @@
     </row>
     <row r="241">
       <c r="A241" s="5" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B241" s="6"/>
       <c r="C241" s="7" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="D241" s="5" t="s">
         <v>6</v>
@@ -5553,7 +5559,7 @@
     </row>
     <row r="242">
       <c r="A242" s="5" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B242" s="6"/>
       <c r="C242" s="7" t="s">
@@ -5565,11 +5571,11 @@
     </row>
     <row r="243">
       <c r="A243" s="5" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B243" s="6"/>
       <c r="C243" s="7" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D243" s="5" t="s">
         <v>6</v>
@@ -5577,7 +5583,7 @@
     </row>
     <row r="244">
       <c r="A244" s="5" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B244" s="6"/>
       <c r="C244" s="7" t="s">
@@ -5589,11 +5595,11 @@
     </row>
     <row r="245">
       <c r="A245" s="5" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B245" s="6"/>
       <c r="C245" s="7" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="D245" s="5" t="s">
         <v>6</v>
@@ -5601,11 +5607,11 @@
     </row>
     <row r="246">
       <c r="A246" s="5" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B246" s="6"/>
       <c r="C246" s="7" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D246" s="5" t="s">
         <v>6</v>
@@ -5613,7 +5619,7 @@
     </row>
     <row r="247">
       <c r="A247" s="18" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B247" s="19"/>
       <c r="C247" s="20" t="s">
@@ -5647,11 +5653,11 @@
     </row>
     <row r="248">
       <c r="A248" s="5" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B248" s="6"/>
       <c r="C248" s="7" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D248" s="5" t="s">
         <v>6</v>
@@ -5659,11 +5665,11 @@
     </row>
     <row r="249">
       <c r="A249" s="5" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B249" s="6"/>
       <c r="C249" s="7" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="D249" s="5" t="s">
         <v>6</v>
@@ -5671,11 +5677,11 @@
     </row>
     <row r="250">
       <c r="A250" s="5" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B250" s="6"/>
       <c r="C250" s="7" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="D250" s="5" t="s">
         <v>6</v>
@@ -5683,11 +5689,11 @@
     </row>
     <row r="251">
       <c r="A251" s="5" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B251" s="6"/>
       <c r="C251" s="7" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D251" s="5" t="s">
         <v>6</v>
@@ -5695,11 +5701,11 @@
     </row>
     <row r="252">
       <c r="A252" s="5" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B252" s="6"/>
       <c r="C252" s="7" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="D252" s="5" t="s">
         <v>6</v>
@@ -5707,11 +5713,11 @@
     </row>
     <row r="253">
       <c r="A253" s="18" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B253" s="19"/>
       <c r="C253" s="20" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="D253" s="18" t="s">
         <v>6</v>
@@ -5720,11 +5726,11 @@
     </row>
     <row r="254">
       <c r="A254" s="5" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B254" s="6"/>
       <c r="C254" s="7" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="D254" s="5" t="s">
         <v>6</v>
@@ -5732,11 +5738,11 @@
     </row>
     <row r="255">
       <c r="A255" s="5" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B255" s="6"/>
       <c r="C255" s="7" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="D255" s="5" t="s">
         <v>6</v>
@@ -5744,11 +5750,11 @@
     </row>
     <row r="256">
       <c r="A256" s="5" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B256" s="6"/>
       <c r="C256" s="7" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="D256" s="5" t="s">
         <v>6</v>
@@ -5756,11 +5762,11 @@
     </row>
     <row r="257">
       <c r="A257" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B257" s="6"/>
       <c r="C257" s="7" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="D257" s="5" t="s">
         <v>6</v>
@@ -5768,11 +5774,11 @@
     </row>
     <row r="258">
       <c r="A258" s="5" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B258" s="6"/>
       <c r="C258" s="7" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="D258" s="5" t="s">
         <v>6</v>
@@ -5780,11 +5786,11 @@
     </row>
     <row r="259">
       <c r="A259" s="5" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B259" s="6"/>
       <c r="C259" s="7" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="D259" s="5" t="s">
         <v>6</v>
@@ -5792,11 +5798,11 @@
     </row>
     <row r="260">
       <c r="A260" s="5" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B260" s="6"/>
       <c r="C260" s="7" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D260" s="5" t="s">
         <v>6</v>
@@ -5804,11 +5810,11 @@
     </row>
     <row r="261">
       <c r="A261" s="5" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B261" s="6"/>
       <c r="C261" s="7" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D261" s="5" t="s">
         <v>6</v>
@@ -5816,11 +5822,11 @@
     </row>
     <row r="262">
       <c r="A262" s="5" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B262" s="6"/>
       <c r="C262" s="7" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="D262" s="5" t="s">
         <v>6</v>
@@ -5828,11 +5834,11 @@
     </row>
     <row r="263">
       <c r="A263" s="5" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B263" s="6"/>
       <c r="C263" s="7" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="D263" s="5" t="s">
         <v>6</v>
@@ -5840,11 +5846,11 @@
     </row>
     <row r="264">
       <c r="A264" s="5" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B264" s="6"/>
       <c r="C264" s="7" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="D264" s="5" t="s">
         <v>6</v>
@@ -5852,11 +5858,11 @@
     </row>
     <row r="265">
       <c r="A265" s="5" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B265" s="6"/>
       <c r="C265" s="7" t="s">
-        <v>452</v>
+        <v>498</v>
       </c>
       <c r="D265" s="5" t="s">
         <v>6</v>
@@ -6232,7 +6238,7 @@
       </c>
       <c r="B297" s="6"/>
       <c r="C297" s="7" t="s">
-        <v>452</v>
+        <v>498</v>
       </c>
       <c r="D297" s="5" t="s">
         <v>6</v>
@@ -6707,11 +6713,11 @@
       </c>
     </row>
     <row r="337">
-      <c r="A337" s="5" t="s">
+      <c r="A337" s="25" t="s">
         <v>632</v>
       </c>
       <c r="B337" s="6"/>
-      <c r="C337" s="7" t="s">
+      <c r="C337" s="26" t="s">
         <v>633</v>
       </c>
       <c r="D337" s="5" t="s">
@@ -6731,11 +6737,11 @@
       </c>
     </row>
     <row r="339">
-      <c r="A339" s="25" t="s">
+      <c r="A339" s="5" t="s">
         <v>636</v>
       </c>
       <c r="B339" s="6"/>
-      <c r="C339" s="26" t="s">
+      <c r="C339" s="7" t="s">
         <v>637</v>
       </c>
       <c r="D339" s="5" t="s">
@@ -6748,7 +6754,7 @@
       </c>
       <c r="B340" s="6"/>
       <c r="C340" s="7" t="s">
-        <v>446</v>
+        <v>639</v>
       </c>
       <c r="D340" s="5" t="s">
         <v>6</v>
@@ -6756,11 +6762,11 @@
     </row>
     <row r="341">
       <c r="A341" s="5" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B341" s="6"/>
       <c r="C341" s="7" t="s">
-        <v>640</v>
+        <v>446</v>
       </c>
       <c r="D341" s="5" t="s">
         <v>6</v>
@@ -7084,7 +7090,7 @@
       </c>
       <c r="B368" s="6"/>
       <c r="C368" s="7" t="s">
-        <v>621</v>
+        <v>694</v>
       </c>
       <c r="D368" s="5" t="s">
         <v>6</v>
@@ -7092,11 +7098,11 @@
     </row>
     <row r="369">
       <c r="A369" s="5" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B369" s="6"/>
       <c r="C369" s="7" t="s">
-        <v>695</v>
+        <v>621</v>
       </c>
       <c r="D369" s="5" t="s">
         <v>6</v>
@@ -7228,7 +7234,7 @@
       </c>
       <c r="B380" s="6"/>
       <c r="C380" s="7" t="s">
-        <v>452</v>
+        <v>717</v>
       </c>
       <c r="D380" s="5" t="s">
         <v>6</v>
@@ -7236,11 +7242,11 @@
     </row>
     <row r="381">
       <c r="A381" s="5" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B381" s="6"/>
       <c r="C381" s="7" t="s">
-        <v>718</v>
+        <v>498</v>
       </c>
       <c r="D381" s="5" t="s">
         <v>6</v>
@@ -7259,7 +7265,7 @@
       </c>
     </row>
     <row r="383">
-      <c r="A383" s="10" t="s">
+      <c r="A383" s="5" t="s">
         <v>721</v>
       </c>
       <c r="B383" s="6"/>
@@ -7295,7 +7301,7 @@
       </c>
     </row>
     <row r="386">
-      <c r="A386" s="5" t="s">
+      <c r="A386" s="10" t="s">
         <v>727</v>
       </c>
       <c r="B386" s="6"/>
@@ -7307,7 +7313,7 @@
       </c>
     </row>
     <row r="387">
-      <c r="A387" s="10" t="s">
+      <c r="A387" s="5" t="s">
         <v>729</v>
       </c>
       <c r="B387" s="6"/>
@@ -7319,10 +7325,16 @@
       </c>
     </row>
     <row r="388">
-      <c r="A388" s="6"/>
+      <c r="A388" s="10" t="s">
+        <v>731</v>
+      </c>
       <c r="B388" s="6"/>
-      <c r="C388" s="6"/>
-      <c r="D388" s="6"/>
+      <c r="C388" s="7" t="s">
+        <v>732</v>
+      </c>
+      <c r="D388" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="389">
       <c r="A389" s="6"/>
@@ -11932,9 +11944,15 @@
       <c r="C1156" s="6"/>
       <c r="D1156" s="6"/>
     </row>
+    <row r="1157">
+      <c r="A1157" s="6"/>
+      <c r="B1157" s="6"/>
+      <c r="C1157" s="6"/>
+      <c r="D1157" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D277 D280:D387">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D277 D280:D388">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Factory reset process (ble command not implemented)
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="747">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1195" uniqueCount="753">
   <si>
     <t>Key</t>
   </si>
@@ -230,6 +230,24 @@
   </si>
   <si>
     <t>Manage my Rings</t>
+  </si>
+  <si>
+    <t>ring.factory_reset</t>
+  </si>
+  <si>
+    <t>Factory Reset</t>
+  </si>
+  <si>
+    <t>ring.factory_reset_confirm.title</t>
+  </si>
+  <si>
+    <t>Do you confirm that you wish to factory reset your ring?</t>
+  </si>
+  <si>
+    <t>ring.factory_reset_confirm.description</t>
+  </si>
+  <si>
+    <t>You will go back to factory settings and all of the data in your ring will be erased.</t>
   </si>
   <si>
     <t>signin_signup.signin</t>
@@ -2310,7 +2328,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -2337,6 +2355,7 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF1155CC"/>
@@ -2394,7 +2413,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2431,13 +2450,19 @@
     <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -2446,19 +2471,19 @@
     <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
@@ -3151,36 +3176,36 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="12" t="s">
         <v>72</v>
       </c>
       <c r="B37" s="6"/>
-      <c r="C37" s="7" t="s">
-        <v>42</v>
+      <c r="C37" s="13" t="s">
+        <v>73</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="s">
-        <v>73</v>
+      <c r="A38" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="B38" s="6"/>
-      <c r="C38" s="7" t="s">
-        <v>53</v>
+      <c r="C38" s="13" t="s">
+        <v>75</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="s">
-        <v>74</v>
+      <c r="A39" s="12" t="s">
+        <v>76</v>
       </c>
       <c r="B39" s="6"/>
-      <c r="C39" s="7" t="s">
-        <v>53</v>
+      <c r="C39" s="13" t="s">
+        <v>77</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>6</v>
@@ -3188,23 +3213,23 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="7" t="s">
-        <v>76</v>
+        <v>42</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="s">
-        <v>77</v>
+      <c r="A41" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>6</v>
@@ -3212,11 +3237,11 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="7" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>6</v>
@@ -3224,11 +3249,11 @@
     </row>
     <row r="43">
       <c r="A43" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>6</v>
@@ -3236,11 +3261,11 @@
     </row>
     <row r="44">
       <c r="A44" s="5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>6</v>
@@ -3248,11 +3273,11 @@
     </row>
     <row r="45">
       <c r="A45" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="7" t="s">
-        <v>82</v>
+        <v>46</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>6</v>
@@ -3260,11 +3285,11 @@
     </row>
     <row r="46">
       <c r="A46" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>6</v>
@@ -3272,11 +3297,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>6</v>
@@ -3284,11 +3309,11 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>6</v>
@@ -3296,11 +3321,11 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
-        <v>87</v>
+        <v>46</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>6</v>
@@ -3308,11 +3333,11 @@
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="7" t="s">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>6</v>
@@ -3320,11 +3345,11 @@
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="7" t="s">
-        <v>91</v>
+        <v>42</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>6</v>
@@ -3372,7 +3397,7 @@
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="7" t="s">
-        <v>57</v>
+        <v>99</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>6</v>
@@ -3380,11 +3405,11 @@
     </row>
     <row r="56">
       <c r="A56" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>6</v>
@@ -3392,11 +3417,11 @@
     </row>
     <row r="57">
       <c r="A57" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>6</v>
@@ -3404,11 +3429,11 @@
     </row>
     <row r="58">
       <c r="A58" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="s">
-        <v>104</v>
+        <v>57</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>6</v>
@@ -3504,7 +3529,7 @@
       </c>
       <c r="B66" s="6"/>
       <c r="C66" s="7" t="s">
-        <v>46</v>
+        <v>120</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>6</v>
@@ -3512,11 +3537,11 @@
     </row>
     <row r="67">
       <c r="A67" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B67" s="6"/>
       <c r="C67" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>6</v>
@@ -3524,11 +3549,11 @@
     </row>
     <row r="68">
       <c r="A68" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B68" s="6"/>
       <c r="C68" s="7" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>6</v>
@@ -3536,11 +3561,11 @@
     </row>
     <row r="69">
       <c r="A69" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" s="7" t="s">
-        <v>124</v>
+        <v>46</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>6</v>
@@ -3548,11 +3573,11 @@
     </row>
     <row r="70">
       <c r="A70" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B70" s="6"/>
       <c r="C70" s="7" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="D70" s="5" t="s">
         <v>6</v>
@@ -3560,11 +3585,11 @@
     </row>
     <row r="71">
       <c r="A71" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" s="7" t="s">
-        <v>127</v>
+        <v>44</v>
       </c>
       <c r="D71" s="5" t="s">
         <v>6</v>
@@ -3572,11 +3597,11 @@
     </row>
     <row r="72">
       <c r="A72" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B72" s="6"/>
       <c r="C72" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>6</v>
@@ -3584,11 +3609,11 @@
     </row>
     <row r="73">
       <c r="A73" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B73" s="6"/>
       <c r="C73" s="7" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>6</v>
@@ -3631,101 +3656,104 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="12" t="s">
+      <c r="A77" s="5" t="s">
         <v>138</v>
       </c>
+      <c r="B77" s="6"/>
       <c r="C77" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="B78" s="6"/>
+      <c r="C78" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D78" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B79" s="6"/>
+      <c r="C79" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="C80" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D77" s="12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="C78" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="D78" s="12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="C79" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="D79" s="12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="C80" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="D80" s="12" t="s">
+      <c r="D80" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="12" t="s">
+      <c r="A81" s="14" t="s">
         <v>145</v>
       </c>
       <c r="C81" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="D81" s="14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="C82" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="D82" s="14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="D83" s="14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="C84" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D81" s="12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="C82" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="D82" s="12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="C83" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="D83" s="12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="C84" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="D84" s="12" t="s">
+      <c r="D84" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="14" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="D85" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D85" s="14" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3736,43 +3764,40 @@
       <c r="C86" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="D86" s="12" t="s">
+      <c r="D86" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="5" t="s">
+      <c r="A87" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="B87" s="6"/>
       <c r="C87" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="D87" s="5" t="s">
+      <c r="D87" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="5" t="s">
+      <c r="A88" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="B88" s="6"/>
       <c r="C88" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="D88" s="5" t="s">
+      <c r="D88" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="5" t="s">
+      <c r="A89" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="B89" s="6"/>
       <c r="C89" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="D89" s="5" t="s">
+      <c r="D89" s="14" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3909,7 +3934,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="10" t="s">
+      <c r="A101" s="5" t="s">
         <v>183</v>
       </c>
       <c r="B101" s="6"/>
@@ -3921,7 +3946,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="10" t="s">
+      <c r="A102" s="5" t="s">
         <v>185</v>
       </c>
       <c r="B102" s="6"/>
@@ -3945,7 +3970,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="5" t="s">
+      <c r="A104" s="10" t="s">
         <v>189</v>
       </c>
       <c r="B104" s="6"/>
@@ -3957,7 +3982,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="5" t="s">
+      <c r="A105" s="10" t="s">
         <v>191</v>
       </c>
       <c r="B105" s="6"/>
@@ -4238,7 +4263,7 @@
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7" t="s">
-        <v>46</v>
+        <v>238</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>6</v>
@@ -4246,11 +4271,11 @@
     </row>
     <row r="129">
       <c r="A129" s="5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B129" s="6"/>
       <c r="C129" s="7" t="s">
-        <v>46</v>
+        <v>240</v>
       </c>
       <c r="D129" s="5" t="s">
         <v>6</v>
@@ -4258,11 +4283,11 @@
     </row>
     <row r="130">
       <c r="A130" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B130" s="6"/>
       <c r="C130" s="7" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D130" s="5" t="s">
         <v>6</v>
@@ -4270,11 +4295,11 @@
     </row>
     <row r="131">
       <c r="A131" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="B131" s="5"/>
+        <v>243</v>
+      </c>
+      <c r="B131" s="6"/>
       <c r="C131" s="7" t="s">
-        <v>242</v>
+        <v>46</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>6</v>
@@ -4282,11 +4307,11 @@
     </row>
     <row r="132">
       <c r="A132" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B132" s="6"/>
       <c r="C132" s="7" t="s">
-        <v>244</v>
+        <v>46</v>
       </c>
       <c r="D132" s="5" t="s">
         <v>6</v>
@@ -4308,7 +4333,7 @@
       <c r="A134" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="B134" s="6"/>
+      <c r="B134" s="5"/>
       <c r="C134" s="7" t="s">
         <v>248</v>
       </c>
@@ -4322,7 +4347,7 @@
       </c>
       <c r="B135" s="6"/>
       <c r="C135" s="7" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="D135" s="5" t="s">
         <v>6</v>
@@ -4330,11 +4355,11 @@
     </row>
     <row r="136">
       <c r="A136" s="5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B136" s="6"/>
       <c r="C136" s="7" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D136" s="5" t="s">
         <v>6</v>
@@ -4342,11 +4367,11 @@
     </row>
     <row r="137">
       <c r="A137" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B137" s="6"/>
       <c r="C137" s="7" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>6</v>
@@ -4354,11 +4379,11 @@
     </row>
     <row r="138">
       <c r="A138" s="5" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B138" s="6"/>
       <c r="C138" s="7" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>6</v>
@@ -4370,7 +4395,7 @@
       </c>
       <c r="B139" s="6"/>
       <c r="C139" s="7" t="s">
-        <v>240</v>
+        <v>257</v>
       </c>
       <c r="D139" s="5" t="s">
         <v>6</v>
@@ -4378,11 +4403,11 @@
     </row>
     <row r="140">
       <c r="A140" s="5" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B140" s="6"/>
       <c r="C140" s="7" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D140" s="5" t="s">
         <v>6</v>
@@ -4390,11 +4415,11 @@
     </row>
     <row r="141">
       <c r="A141" s="5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D141" s="5" t="s">
         <v>6</v>
@@ -4402,11 +4427,11 @@
     </row>
     <row r="142">
       <c r="A142" s="5" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B142" s="6"/>
       <c r="C142" s="7" t="s">
-        <v>262</v>
+        <v>246</v>
       </c>
       <c r="D142" s="5" t="s">
         <v>6</v>
@@ -4461,7 +4486,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="10" t="s">
+      <c r="A147" s="5" t="s">
         <v>271</v>
       </c>
       <c r="B147" s="6"/>
@@ -4473,55 +4498,55 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="10" t="s">
+      <c r="A148" s="5" t="s">
         <v>273</v>
       </c>
       <c r="B148" s="6"/>
       <c r="C148" s="7" t="s">
-        <v>246</v>
+        <v>274</v>
       </c>
       <c r="D148" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="10" t="s">
-        <v>274</v>
+      <c r="A149" s="5" t="s">
+        <v>275</v>
       </c>
       <c r="B149" s="6"/>
       <c r="C149" s="7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D149" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="5" t="s">
-        <v>276</v>
+      <c r="A150" s="10" t="s">
+        <v>277</v>
       </c>
       <c r="B150" s="6"/>
       <c r="C150" s="7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D150" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="5" t="s">
-        <v>278</v>
+      <c r="A151" s="10" t="s">
+        <v>279</v>
       </c>
       <c r="B151" s="6"/>
       <c r="C151" s="7" t="s">
-        <v>279</v>
+        <v>252</v>
       </c>
       <c r="D151" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="5" t="s">
+      <c r="A152" s="10" t="s">
         <v>280</v>
       </c>
       <c r="B152" s="6"/>
@@ -4545,24 +4570,24 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="15" t="s">
+      <c r="A154" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="B154" s="16"/>
-      <c r="C154" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="D154" s="15" t="s">
+      <c r="B154" s="6"/>
+      <c r="C154" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="D154" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B155" s="6"/>
       <c r="C155" s="7" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D155" s="5" t="s">
         <v>6</v>
@@ -4570,25 +4595,25 @@
     </row>
     <row r="156">
       <c r="A156" s="5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B156" s="6"/>
       <c r="C156" s="7" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D156" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="5" t="s">
-        <v>289</v>
-      </c>
-      <c r="B157" s="6"/>
-      <c r="C157" s="7" t="s">
+      <c r="A157" s="17" t="s">
         <v>290</v>
       </c>
-      <c r="D157" s="5" t="s">
+      <c r="B157" s="18"/>
+      <c r="C157" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="D157" s="17" t="s">
         <v>6</v>
       </c>
     </row>
@@ -4749,7 +4774,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="10" t="s">
+      <c r="A171" s="5" t="s">
         <v>317</v>
       </c>
       <c r="B171" s="6"/>
@@ -4761,7 +4786,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="10" t="s">
+      <c r="A172" s="5" t="s">
         <v>319</v>
       </c>
       <c r="B172" s="6"/>
@@ -4773,7 +4798,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="10" t="s">
+      <c r="A173" s="5" t="s">
         <v>321</v>
       </c>
       <c r="B173" s="6"/>
@@ -4785,36 +4810,36 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="5" t="s">
+      <c r="A174" s="10" t="s">
         <v>323</v>
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>253</v>
+        <v>324</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="5" t="s">
-        <v>324</v>
+      <c r="A175" s="10" t="s">
+        <v>325</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="5" t="s">
-        <v>326</v>
+      <c r="A176" s="10" t="s">
+        <v>327</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>67</v>
+        <v>328</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
@@ -4822,11 +4847,11 @@
     </row>
     <row r="177">
       <c r="A177" s="5" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>328</v>
+        <v>259</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
@@ -4834,11 +4859,11 @@
     </row>
     <row r="178">
       <c r="A178" s="5" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
@@ -4846,11 +4871,11 @@
     </row>
     <row r="179">
       <c r="A179" s="5" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>332</v>
+        <v>67</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
@@ -4929,7 +4954,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="17" t="s">
+      <c r="A186" s="5" t="s">
         <v>345</v>
       </c>
       <c r="B186" s="6"/>
@@ -4965,7 +4990,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="5" t="s">
+      <c r="A189" s="19" t="s">
         <v>351</v>
       </c>
       <c r="B189" s="6"/>
@@ -4989,7 +5014,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="10" t="s">
+      <c r="A191" s="5" t="s">
         <v>355</v>
       </c>
       <c r="B191" s="6"/>
@@ -5025,7 +5050,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="5" t="s">
+      <c r="A194" s="10" t="s">
         <v>361</v>
       </c>
       <c r="B194" s="6"/>
@@ -5174,7 +5199,7 @@
       </c>
       <c r="B206" s="6"/>
       <c r="C206" s="7" t="s">
-        <v>57</v>
+        <v>386</v>
       </c>
       <c r="D206" s="5" t="s">
         <v>6</v>
@@ -5182,11 +5207,11 @@
     </row>
     <row r="207">
       <c r="A207" s="5" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B207" s="6"/>
       <c r="C207" s="7" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D207" s="5" t="s">
         <v>6</v>
@@ -5194,11 +5219,11 @@
     </row>
     <row r="208">
       <c r="A208" s="5" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B208" s="6"/>
       <c r="C208" s="7" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D208" s="5" t="s">
         <v>6</v>
@@ -5206,18 +5231,18 @@
     </row>
     <row r="209">
       <c r="A209" s="5" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B209" s="6"/>
       <c r="C209" s="7" t="s">
-        <v>391</v>
+        <v>57</v>
       </c>
       <c r="D209" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="12" t="s">
+      <c r="A210" s="5" t="s">
         <v>392</v>
       </c>
       <c r="B210" s="6"/>
@@ -5229,7 +5254,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="12" t="s">
+      <c r="A211" s="5" t="s">
         <v>394</v>
       </c>
       <c r="B211" s="6"/>
@@ -5241,7 +5266,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="12" t="s">
+      <c r="A212" s="5" t="s">
         <v>396</v>
       </c>
       <c r="B212" s="6"/>
@@ -5253,7 +5278,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="12" t="s">
+      <c r="A213" s="14" t="s">
         <v>398</v>
       </c>
       <c r="B213" s="6"/>
@@ -5265,7 +5290,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="12" t="s">
+      <c r="A214" s="14" t="s">
         <v>400</v>
       </c>
       <c r="B214" s="6"/>
@@ -5277,7 +5302,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="12" t="s">
+      <c r="A215" s="14" t="s">
         <v>402</v>
       </c>
       <c r="B215" s="6"/>
@@ -5289,36 +5314,36 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="5" t="s">
+      <c r="A216" s="14" t="s">
         <v>404</v>
       </c>
       <c r="B216" s="6"/>
       <c r="C216" s="7" t="s">
-        <v>144</v>
+        <v>405</v>
       </c>
       <c r="D216" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="5" t="s">
-        <v>405</v>
+      <c r="A217" s="14" t="s">
+        <v>406</v>
       </c>
       <c r="B217" s="6"/>
       <c r="C217" s="7" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D217" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="5" t="s">
-        <v>407</v>
+      <c r="A218" s="14" t="s">
+        <v>408</v>
       </c>
       <c r="B218" s="6"/>
       <c r="C218" s="7" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D218" s="5" t="s">
         <v>6</v>
@@ -5326,11 +5351,11 @@
     </row>
     <row r="219">
       <c r="A219" s="5" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B219" s="6"/>
       <c r="C219" s="7" t="s">
-        <v>410</v>
+        <v>150</v>
       </c>
       <c r="D219" s="5" t="s">
         <v>6</v>
@@ -5445,14 +5470,14 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="18" t="s">
+      <c r="A229" s="5" t="s">
         <v>429</v>
       </c>
-      <c r="B229" s="19"/>
-      <c r="C229" s="20" t="s">
+      <c r="B229" s="6"/>
+      <c r="C229" s="7" t="s">
         <v>430</v>
       </c>
-      <c r="D229" s="18" t="s">
+      <c r="D229" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -5481,14 +5506,14 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="5" t="s">
+      <c r="A232" s="20" t="s">
         <v>435</v>
       </c>
-      <c r="B232" s="6"/>
-      <c r="C232" s="7" t="s">
+      <c r="B232" s="21"/>
+      <c r="C232" s="22" t="s">
         <v>436</v>
       </c>
-      <c r="D232" s="5" t="s">
+      <c r="D232" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -5606,7 +5631,7 @@
       </c>
       <c r="B242" s="6"/>
       <c r="C242" s="7" t="s">
-        <v>67</v>
+        <v>456</v>
       </c>
       <c r="D242" s="5" t="s">
         <v>6</v>
@@ -5614,11 +5639,11 @@
     </row>
     <row r="243">
       <c r="A243" s="5" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B243" s="6"/>
       <c r="C243" s="7" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D243" s="5" t="s">
         <v>6</v>
@@ -5626,11 +5651,11 @@
     </row>
     <row r="244">
       <c r="A244" s="5" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B244" s="6"/>
       <c r="C244" s="7" t="s">
-        <v>190</v>
+        <v>460</v>
       </c>
       <c r="D244" s="5" t="s">
         <v>6</v>
@@ -5638,11 +5663,11 @@
     </row>
     <row r="245">
       <c r="A245" s="5" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B245" s="6"/>
       <c r="C245" s="7" t="s">
-        <v>460</v>
+        <v>67</v>
       </c>
       <c r="D245" s="5" t="s">
         <v>6</v>
@@ -5650,11 +5675,11 @@
     </row>
     <row r="246">
       <c r="A246" s="5" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B246" s="6"/>
       <c r="C246" s="7" t="s">
-        <v>332</v>
+        <v>463</v>
       </c>
       <c r="D246" s="5" t="s">
         <v>6</v>
@@ -5662,11 +5687,11 @@
     </row>
     <row r="247">
       <c r="A247" s="5" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B247" s="6"/>
       <c r="C247" s="7" t="s">
-        <v>463</v>
+        <v>196</v>
       </c>
       <c r="D247" s="5" t="s">
         <v>6</v>
@@ -5674,57 +5699,35 @@
     </row>
     <row r="248">
       <c r="A248" s="5" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B248" s="6"/>
       <c r="C248" s="7" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D248" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="18" t="s">
-        <v>466</v>
-      </c>
-      <c r="B249" s="19"/>
-      <c r="C249" s="20" t="s">
-        <v>253</v>
-      </c>
-      <c r="D249" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="E249" s="21"/>
-      <c r="F249" s="21"/>
-      <c r="G249" s="21"/>
-      <c r="H249" s="21"/>
-      <c r="I249" s="21"/>
-      <c r="J249" s="21"/>
-      <c r="K249" s="21"/>
-      <c r="L249" s="21"/>
-      <c r="M249" s="21"/>
-      <c r="N249" s="21"/>
-      <c r="O249" s="21"/>
-      <c r="P249" s="21"/>
-      <c r="Q249" s="21"/>
-      <c r="R249" s="21"/>
-      <c r="S249" s="21"/>
-      <c r="T249" s="21"/>
-      <c r="U249" s="21"/>
-      <c r="V249" s="21"/>
-      <c r="W249" s="21"/>
-      <c r="X249" s="21"/>
-      <c r="Y249" s="21"/>
-      <c r="Z249" s="21"/>
+      <c r="A249" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="B249" s="6"/>
+      <c r="C249" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="D249" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="5" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B250" s="6"/>
       <c r="C250" s="7" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D250" s="5" t="s">
         <v>6</v>
@@ -5732,27 +5735,49 @@
     </row>
     <row r="251">
       <c r="A251" s="5" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B251" s="6"/>
       <c r="C251" s="7" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D251" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="5" t="s">
-        <v>471</v>
-      </c>
-      <c r="B252" s="6"/>
-      <c r="C252" s="7" t="s">
+      <c r="A252" s="20" t="s">
         <v>472</v>
       </c>
-      <c r="D252" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="B252" s="21"/>
+      <c r="C252" s="22" t="s">
+        <v>259</v>
+      </c>
+      <c r="D252" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E252" s="23"/>
+      <c r="F252" s="23"/>
+      <c r="G252" s="23"/>
+      <c r="H252" s="23"/>
+      <c r="I252" s="23"/>
+      <c r="J252" s="23"/>
+      <c r="K252" s="23"/>
+      <c r="L252" s="23"/>
+      <c r="M252" s="23"/>
+      <c r="N252" s="23"/>
+      <c r="O252" s="23"/>
+      <c r="P252" s="23"/>
+      <c r="Q252" s="23"/>
+      <c r="R252" s="23"/>
+      <c r="S252" s="23"/>
+      <c r="T252" s="23"/>
+      <c r="U252" s="23"/>
+      <c r="V252" s="23"/>
+      <c r="W252" s="23"/>
+      <c r="X252" s="23"/>
+      <c r="Y252" s="23"/>
+      <c r="Z252" s="23"/>
     </row>
     <row r="253">
       <c r="A253" s="5" t="s">
@@ -5779,17 +5804,16 @@
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="18" t="s">
+      <c r="A255" s="5" t="s">
         <v>477</v>
       </c>
-      <c r="B255" s="19"/>
-      <c r="C255" s="20" t="s">
+      <c r="B255" s="6"/>
+      <c r="C255" s="7" t="s">
         <v>478</v>
       </c>
-      <c r="D255" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="E255" s="21"/>
+      <c r="D255" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="5" t="s">
@@ -5816,16 +5840,17 @@
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="5" t="s">
+      <c r="A258" s="20" t="s">
         <v>483</v>
       </c>
-      <c r="B258" s="6"/>
-      <c r="C258" s="7" t="s">
+      <c r="B258" s="21"/>
+      <c r="C258" s="22" t="s">
         <v>484</v>
       </c>
-      <c r="D258" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="D258" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E258" s="23"/>
     </row>
     <row r="259">
       <c r="A259" s="5" t="s">
@@ -6037,7 +6062,7 @@
       </c>
       <c r="B276" s="6"/>
       <c r="C276" s="7" t="s">
-        <v>508</v>
+        <v>520</v>
       </c>
       <c r="D276" s="5" t="s">
         <v>6</v>
@@ -6045,11 +6070,11 @@
     </row>
     <row r="277">
       <c r="A277" s="5" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B277" s="6"/>
       <c r="C277" s="7" t="s">
-        <v>510</v>
+        <v>522</v>
       </c>
       <c r="D277" s="5" t="s">
         <v>6</v>
@@ -6057,11 +6082,11 @@
     </row>
     <row r="278">
       <c r="A278" s="5" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B278" s="6"/>
       <c r="C278" s="7" t="s">
-        <v>512</v>
+        <v>524</v>
       </c>
       <c r="D278" s="5" t="s">
         <v>6</v>
@@ -6069,7 +6094,7 @@
     </row>
     <row r="279">
       <c r="A279" s="5" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B279" s="6"/>
       <c r="C279" s="7" t="s">
@@ -6081,27 +6106,35 @@
     </row>
     <row r="280">
       <c r="A280" s="5" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="B280" s="6"/>
-      <c r="C280" s="6"/>
-      <c r="D280" s="6"/>
+      <c r="C280" s="7" t="s">
+        <v>516</v>
+      </c>
+      <c r="D280" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="5" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="B281" s="6"/>
-      <c r="C281" s="6"/>
-      <c r="D281" s="6"/>
+      <c r="C281" s="7" t="s">
+        <v>518</v>
+      </c>
+      <c r="D281" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="5" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="B282" s="6"/>
       <c r="C282" s="7" t="s">
-        <v>526</v>
+        <v>520</v>
       </c>
       <c r="D282" s="5" t="s">
         <v>6</v>
@@ -6109,27 +6142,19 @@
     </row>
     <row r="283">
       <c r="A283" s="5" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B283" s="6"/>
-      <c r="C283" s="7" t="s">
-        <v>528</v>
-      </c>
-      <c r="D283" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C283" s="6"/>
+      <c r="D283" s="6"/>
     </row>
     <row r="284">
       <c r="A284" s="5" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B284" s="6"/>
-      <c r="C284" s="7" t="s">
-        <v>530</v>
-      </c>
-      <c r="D284" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="C284" s="6"/>
+      <c r="D284" s="6"/>
     </row>
     <row r="285">
       <c r="A285" s="5" t="s">
@@ -6209,7 +6234,7 @@
       </c>
       <c r="B291" s="6"/>
       <c r="C291" s="7" t="s">
-        <v>508</v>
+        <v>544</v>
       </c>
       <c r="D291" s="5" t="s">
         <v>6</v>
@@ -6217,11 +6242,11 @@
     </row>
     <row r="292">
       <c r="A292" s="5" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B292" s="6"/>
       <c r="C292" s="7" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D292" s="5" t="s">
         <v>6</v>
@@ -6229,11 +6254,11 @@
     </row>
     <row r="293">
       <c r="A293" s="5" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B293" s="6"/>
       <c r="C293" s="7" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="D293" s="5" t="s">
         <v>6</v>
@@ -6241,11 +6266,11 @@
     </row>
     <row r="294">
       <c r="A294" s="5" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B294" s="6"/>
       <c r="C294" s="7" t="s">
-        <v>549</v>
+        <v>514</v>
       </c>
       <c r="D294" s="5" t="s">
         <v>6</v>
@@ -6305,7 +6330,7 @@
       </c>
       <c r="B299" s="6"/>
       <c r="C299" s="7" t="s">
-        <v>502</v>
+        <v>559</v>
       </c>
       <c r="D299" s="5" t="s">
         <v>6</v>
@@ -6313,11 +6338,11 @@
     </row>
     <row r="300">
       <c r="A300" s="5" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B300" s="6"/>
       <c r="C300" s="7" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="D300" s="5" t="s">
         <v>6</v>
@@ -6325,11 +6350,11 @@
     </row>
     <row r="301">
       <c r="A301" s="5" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B301" s="6"/>
       <c r="C301" s="7" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="D301" s="5" t="s">
         <v>6</v>
@@ -6337,11 +6362,11 @@
     </row>
     <row r="302">
       <c r="A302" s="5" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B302" s="6"/>
       <c r="C302" s="7" t="s">
-        <v>564</v>
+        <v>508</v>
       </c>
       <c r="D302" s="5" t="s">
         <v>6</v>
@@ -6473,7 +6498,7 @@
       </c>
       <c r="B313" s="6"/>
       <c r="C313" s="7" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="D313" s="5" t="s">
         <v>6</v>
@@ -6481,11 +6506,11 @@
     </row>
     <row r="314">
       <c r="A314" s="5" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B314" s="6"/>
       <c r="C314" s="7" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="D314" s="5" t="s">
         <v>6</v>
@@ -6493,11 +6518,11 @@
     </row>
     <row r="315">
       <c r="A315" s="5" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B315" s="6"/>
       <c r="C315" s="7" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="D315" s="5" t="s">
         <v>6</v>
@@ -6505,18 +6530,18 @@
     </row>
     <row r="316">
       <c r="A316" s="5" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B316" s="6"/>
       <c r="C316" s="7" t="s">
-        <v>591</v>
+        <v>586</v>
       </c>
       <c r="D316" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="317">
-      <c r="A317" s="22" t="s">
+      <c r="A317" s="5" t="s">
         <v>592</v>
       </c>
       <c r="B317" s="6"/>
@@ -6528,7 +6553,7 @@
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="23" t="s">
+      <c r="A318" s="5" t="s">
         <v>594</v>
       </c>
       <c r="B318" s="6"/>
@@ -6540,7 +6565,7 @@
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="23" t="s">
+      <c r="A319" s="5" t="s">
         <v>596</v>
       </c>
       <c r="B319" s="6"/>
@@ -6552,7 +6577,7 @@
       </c>
     </row>
     <row r="320">
-      <c r="A320" s="23" t="s">
+      <c r="A320" s="24" t="s">
         <v>598</v>
       </c>
       <c r="B320" s="6"/>
@@ -6564,7 +6589,7 @@
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="23" t="s">
+      <c r="A321" s="25" t="s">
         <v>600</v>
       </c>
       <c r="B321" s="6"/>
@@ -6576,7 +6601,7 @@
       </c>
     </row>
     <row r="322">
-      <c r="A322" s="23" t="s">
+      <c r="A322" s="25" t="s">
         <v>602</v>
       </c>
       <c r="B322" s="6"/>
@@ -6588,7 +6613,7 @@
       </c>
     </row>
     <row r="323">
-      <c r="A323" s="24" t="s">
+      <c r="A323" s="25" t="s">
         <v>604</v>
       </c>
       <c r="B323" s="6"/>
@@ -6600,7 +6625,7 @@
       </c>
     </row>
     <row r="324">
-      <c r="A324" s="24" t="s">
+      <c r="A324" s="25" t="s">
         <v>606</v>
       </c>
       <c r="B324" s="6"/>
@@ -6612,7 +6637,7 @@
       </c>
     </row>
     <row r="325">
-      <c r="A325" s="24" t="s">
+      <c r="A325" s="25" t="s">
         <v>608</v>
       </c>
       <c r="B325" s="6"/>
@@ -6624,7 +6649,7 @@
       </c>
     </row>
     <row r="326">
-      <c r="A326" s="24" t="s">
+      <c r="A326" s="26" t="s">
         <v>610</v>
       </c>
       <c r="B326" s="6"/>
@@ -6636,7 +6661,7 @@
       </c>
     </row>
     <row r="327">
-      <c r="A327" s="24" t="s">
+      <c r="A327" s="26" t="s">
         <v>612</v>
       </c>
       <c r="B327" s="6"/>
@@ -6648,7 +6673,7 @@
       </c>
     </row>
     <row r="328">
-      <c r="A328" s="24" t="s">
+      <c r="A328" s="26" t="s">
         <v>614</v>
       </c>
       <c r="B328" s="6"/>
@@ -6660,7 +6685,7 @@
       </c>
     </row>
     <row r="329">
-      <c r="A329" s="5" t="s">
+      <c r="A329" s="26" t="s">
         <v>616</v>
       </c>
       <c r="B329" s="6"/>
@@ -6672,7 +6697,7 @@
       </c>
     </row>
     <row r="330">
-      <c r="A330" s="5" t="s">
+      <c r="A330" s="26" t="s">
         <v>618</v>
       </c>
       <c r="B330" s="6"/>
@@ -6684,7 +6709,7 @@
       </c>
     </row>
     <row r="331">
-      <c r="A331" s="5" t="s">
+      <c r="A331" s="26" t="s">
         <v>620</v>
       </c>
       <c r="B331" s="6"/>
@@ -6833,7 +6858,7 @@
       </c>
       <c r="B343" s="6"/>
       <c r="C343" s="7" t="s">
-        <v>450</v>
+        <v>645</v>
       </c>
       <c r="D343" s="5" t="s">
         <v>6</v>
@@ -6841,11 +6866,11 @@
     </row>
     <row r="344">
       <c r="A344" s="5" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B344" s="6"/>
       <c r="C344" s="7" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="D344" s="5" t="s">
         <v>6</v>
@@ -6853,11 +6878,11 @@
     </row>
     <row r="345">
       <c r="A345" s="5" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B345" s="6"/>
       <c r="C345" s="7" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="D345" s="5" t="s">
         <v>6</v>
@@ -6865,11 +6890,11 @@
     </row>
     <row r="346">
       <c r="A346" s="5" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B346" s="6"/>
       <c r="C346" s="7" t="s">
-        <v>650</v>
+        <v>456</v>
       </c>
       <c r="D346" s="5" t="s">
         <v>6</v>
@@ -7169,7 +7194,7 @@
       </c>
       <c r="B371" s="6"/>
       <c r="C371" s="7" t="s">
-        <v>625</v>
+        <v>700</v>
       </c>
       <c r="D371" s="5" t="s">
         <v>6</v>
@@ -7177,11 +7202,11 @@
     </row>
     <row r="372">
       <c r="A372" s="5" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B372" s="6"/>
       <c r="C372" s="7" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="D372" s="5" t="s">
         <v>6</v>
@@ -7189,11 +7214,11 @@
     </row>
     <row r="373">
       <c r="A373" s="5" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B373" s="6"/>
       <c r="C373" s="7" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="D373" s="5" t="s">
         <v>6</v>
@@ -7201,11 +7226,11 @@
     </row>
     <row r="374">
       <c r="A374" s="5" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B374" s="6"/>
       <c r="C374" s="7" t="s">
-        <v>705</v>
+        <v>631</v>
       </c>
       <c r="D374" s="5" t="s">
         <v>6</v>
@@ -7313,7 +7338,7 @@
       </c>
       <c r="B383" s="6"/>
       <c r="C383" s="7" t="s">
-        <v>502</v>
+        <v>723</v>
       </c>
       <c r="D383" s="5" t="s">
         <v>6</v>
@@ -7321,11 +7346,11 @@
     </row>
     <row r="384">
       <c r="A384" s="5" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B384" s="6"/>
       <c r="C384" s="7" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="D384" s="5" t="s">
         <v>6</v>
@@ -7333,30 +7358,30 @@
     </row>
     <row r="385">
       <c r="A385" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B385" s="6"/>
       <c r="C385" s="7" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="D385" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="386">
-      <c r="A386" s="10" t="s">
-        <v>727</v>
+      <c r="A386" s="5" t="s">
+        <v>728</v>
       </c>
       <c r="B386" s="6"/>
       <c r="C386" s="7" t="s">
-        <v>728</v>
+        <v>508</v>
       </c>
       <c r="D386" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="387">
-      <c r="A387" s="10" t="s">
+      <c r="A387" s="5" t="s">
         <v>729</v>
       </c>
       <c r="B387" s="6"/>
@@ -7368,7 +7393,7 @@
       </c>
     </row>
     <row r="388">
-      <c r="A388" s="10" t="s">
+      <c r="A388" s="5" t="s">
         <v>731</v>
       </c>
       <c r="B388" s="6"/>
@@ -7380,7 +7405,7 @@
       </c>
     </row>
     <row r="389">
-      <c r="A389" s="5" t="s">
+      <c r="A389" s="10" t="s">
         <v>733</v>
       </c>
       <c r="B389" s="6"/>
@@ -7404,22 +7429,40 @@
       </c>
     </row>
     <row r="391">
-      <c r="A391" s="6"/>
+      <c r="A391" s="10" t="s">
+        <v>737</v>
+      </c>
       <c r="B391" s="6"/>
-      <c r="C391" s="6"/>
-      <c r="D391" s="6"/>
+      <c r="C391" s="7" t="s">
+        <v>738</v>
+      </c>
+      <c r="D391" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="392">
-      <c r="A392" s="6"/>
+      <c r="A392" s="5" t="s">
+        <v>739</v>
+      </c>
       <c r="B392" s="6"/>
-      <c r="C392" s="6"/>
-      <c r="D392" s="6"/>
+      <c r="C392" s="7" t="s">
+        <v>740</v>
+      </c>
+      <c r="D392" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="393">
-      <c r="A393" s="6"/>
+      <c r="A393" s="10" t="s">
+        <v>741</v>
+      </c>
       <c r="B393" s="6"/>
-      <c r="C393" s="6"/>
-      <c r="D393" s="6"/>
+      <c r="C393" s="7" t="s">
+        <v>742</v>
+      </c>
+      <c r="D393" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="6"/>
@@ -12017,9 +12060,27 @@
       <c r="C1159" s="6"/>
       <c r="D1159" s="6"/>
     </row>
+    <row r="1160">
+      <c r="A1160" s="6"/>
+      <c r="B1160" s="6"/>
+      <c r="C1160" s="6"/>
+      <c r="D1160" s="6"/>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="6"/>
+      <c r="B1161" s="6"/>
+      <c r="C1161" s="6"/>
+      <c r="D1161" s="6"/>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="6"/>
+      <c r="B1162" s="6"/>
+      <c r="C1162" s="6"/>
+      <c r="D1162" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D279 D282:D390">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D282 D285:D393">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12027,8 +12088,8 @@
     <hyperlink r:id="rId1" ref="C6"/>
     <hyperlink r:id="rId2" ref="C7"/>
     <hyperlink r:id="rId3" ref="C8"/>
-    <hyperlink r:id="rId4" ref="A84"/>
-    <hyperlink r:id="rId5" ref="A186"/>
+    <hyperlink r:id="rId4" ref="A87"/>
+    <hyperlink r:id="rId5" ref="A189"/>
   </hyperlinks>
   <drawing r:id="rId6"/>
 </worksheet>
@@ -12084,57 +12145,57 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="7" t="s">
-        <v>738</v>
+        <v>744</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="s">
-        <v>739</v>
+      <c r="A3" s="14" t="s">
+        <v>745</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>740</v>
-      </c>
-      <c r="D3" s="12" t="s">
+        <v>746</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="s">
-        <v>741</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>742</v>
-      </c>
-      <c r="D4" s="12" t="s">
+      <c r="A4" s="14" t="s">
+        <v>747</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>748</v>
+      </c>
+      <c r="D4" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="s">
-        <v>743</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>744</v>
-      </c>
-      <c r="D5" s="12" t="s">
+      <c r="A5" s="14" t="s">
+        <v>749</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>750</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="s">
-        <v>745</v>
-      </c>
-      <c r="C6" s="25" t="s">
-        <v>746</v>
-      </c>
-      <c r="D6" s="12" t="s">
+      <c r="A6" s="14" t="s">
+        <v>751</v>
+      </c>
+      <c r="C6" s="27" t="s">
+        <v>752</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Note list + Delete node + Note added success header
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1267" uniqueCount="799">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1274" uniqueCount="803">
   <si>
     <t>Key</t>
   </si>
@@ -914,9 +914,6 @@
     <t>Edit Birthday</t>
   </si>
   <si>
-    <t>profile_info.edit_name.save</t>
-  </si>
-  <si>
     <t>header.live</t>
   </si>
   <si>
@@ -1090,6 +1087,12 @@
   </si>
   <si>
     <t>Delete Alarm</t>
+  </si>
+  <si>
+    <t>alarm.label.default</t>
+  </si>
+  <si>
+    <t>Alarm</t>
   </si>
   <si>
     <t>onboarding.wear.title</t>
@@ -1473,9 +1476,6 @@
     <t>Keep wearing your ring during the entirety of the {days} days calibration period for improved results!</t>
   </si>
   <si>
-    <t>profile.header.title</t>
-  </si>
-  <si>
     <t>alarm.new.edit_vibration.type.discharge</t>
   </si>
   <si>
@@ -1506,12 +1506,6 @@
     <t>Work Time</t>
   </si>
   <si>
-    <t>alarm.new.label.placeholder</t>
-  </si>
-  <si>
-    <t>Enter label here</t>
-  </si>
-  <si>
     <t>profile_advanced_info.work_time.day</t>
   </si>
   <si>
@@ -1647,7 +1641,13 @@
     <t>profile_advanced_info.sleeper_type.light</t>
   </si>
   <si>
+    <t>Morning type</t>
+  </si>
+  <si>
     <t>profile_advanced_info.sleeper_type.night</t>
+  </si>
+  <si>
+    <t>Night type</t>
   </si>
   <si>
     <t>profile_advanced_info.period_tracking_info</t>
@@ -1856,9 +1856,6 @@
     <t>profile_advanced_info.chrono_type.morning</t>
   </si>
   <si>
-    <t>Morning type</t>
-  </si>
-  <si>
     <t>profile_advanced_info.chrono_type.solar</t>
   </si>
   <si>
@@ -1866,9 +1863,6 @@
   </si>
   <si>
     <t>profile_advanced_info.chrono_type.night</t>
-  </si>
-  <si>
-    <t>Night type</t>
   </si>
   <si>
     <t>profile_advanced_info.chrono_type.morning_erratic</t>
@@ -2431,6 +2425,24 @@
   </si>
   <si>
     <t>Edit End Time</t>
+  </si>
+  <si>
+    <t>calendar.delete_note</t>
+  </si>
+  <si>
+    <t>DELETE</t>
+  </si>
+  <si>
+    <t>calendar.note_added_success.one</t>
+  </si>
+  <si>
+    <t>Your new note “&lt;bold&gt;{notes}&lt;/bold&gt;” has been added successfully</t>
+  </si>
+  <si>
+    <t>calendar.note_added_success.many</t>
+  </si>
+  <si>
+    <t>Your new notes “&lt;bold&gt;{notes}&lt;/bold&gt;” have been added successfully</t>
   </si>
   <si>
     <t>months</t>
@@ -2467,7 +2479,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -2503,6 +2515,7 @@
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -2513,7 +2526,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2538,12 +2551,6 @@
         <bgColor rgb="FFFFA500"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FFFF0000"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -2551,7 +2558,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2597,25 +2604,24 @@
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
@@ -4760,24 +4766,24 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="15" t="s">
+      <c r="A159" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="B159" s="16"/>
-      <c r="C159" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="D159" s="15" t="s">
+      <c r="B159" s="6"/>
+      <c r="C159" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="D159" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="7" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D160" s="5" t="s">
         <v>6</v>
@@ -4785,11 +4791,11 @@
     </row>
     <row r="161">
       <c r="A161" s="5" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D161" s="5" t="s">
         <v>6</v>
@@ -4797,11 +4803,11 @@
     </row>
     <row r="162">
       <c r="A162" s="5" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="7" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>6</v>
@@ -4809,11 +4815,11 @@
     </row>
     <row r="163">
       <c r="A163" s="5" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D163" s="5" t="s">
         <v>6</v>
@@ -4821,11 +4827,11 @@
     </row>
     <row r="164">
       <c r="A164" s="5" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D164" s="5" t="s">
         <v>6</v>
@@ -4833,11 +4839,11 @@
     </row>
     <row r="165">
       <c r="A165" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D165" s="5" t="s">
         <v>6</v>
@@ -4845,11 +4851,11 @@
     </row>
     <row r="166">
       <c r="A166" s="5" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D166" s="5" t="s">
         <v>6</v>
@@ -4857,11 +4863,11 @@
     </row>
     <row r="167">
       <c r="A167" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="7" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D167" s="5" t="s">
         <v>6</v>
@@ -4869,11 +4875,11 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="7" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D168" s="5" t="s">
         <v>6</v>
@@ -4881,11 +4887,11 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="7" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D169" s="5" t="s">
         <v>6</v>
@@ -4893,11 +4899,11 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="7" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D170" s="5" t="s">
         <v>6</v>
@@ -4905,11 +4911,11 @@
     </row>
     <row r="171">
       <c r="A171" s="5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="7" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D171" s="5" t="s">
         <v>6</v>
@@ -4917,11 +4923,11 @@
     </row>
     <row r="172">
       <c r="A172" s="5" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="7" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D172" s="5" t="s">
         <v>6</v>
@@ -4929,11 +4935,11 @@
     </row>
     <row r="173">
       <c r="A173" s="5" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="7" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D173" s="5" t="s">
         <v>6</v>
@@ -4941,23 +4947,23 @@
     </row>
     <row r="174">
       <c r="A174" s="5" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B174" s="6"/>
       <c r="C174" s="7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="5" t="s">
-        <v>325</v>
+      <c r="A175" s="10" t="s">
+        <v>326</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="7" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>6</v>
@@ -4965,11 +4971,11 @@
     </row>
     <row r="176">
       <c r="A176" s="10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="7" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>6</v>
@@ -4977,23 +4983,23 @@
     </row>
     <row r="177">
       <c r="A177" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B177" s="6"/>
       <c r="C177" s="7" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="10" t="s">
-        <v>331</v>
+      <c r="A178" s="5" t="s">
+        <v>332</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>332</v>
+        <v>263</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
@@ -5005,7 +5011,7 @@
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>263</v>
+        <v>334</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
@@ -5013,11 +5019,11 @@
     </row>
     <row r="180">
       <c r="A180" s="5" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>335</v>
+        <v>67</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
@@ -5029,7 +5035,7 @@
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>67</v>
+        <v>337</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
@@ -5037,11 +5043,11 @@
     </row>
     <row r="182">
       <c r="A182" s="5" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="7" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>6</v>
@@ -5049,11 +5055,11 @@
     </row>
     <row r="183">
       <c r="A183" s="5" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="7" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>6</v>
@@ -5061,11 +5067,11 @@
     </row>
     <row r="184">
       <c r="A184" s="5" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="7" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D184" s="5" t="s">
         <v>6</v>
@@ -5073,11 +5079,11 @@
     </row>
     <row r="185">
       <c r="A185" s="5" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="7" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D185" s="5" t="s">
         <v>6</v>
@@ -5085,11 +5091,11 @@
     </row>
     <row r="186">
       <c r="A186" s="5" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="7" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D186" s="5" t="s">
         <v>6</v>
@@ -5097,11 +5103,11 @@
     </row>
     <row r="187">
       <c r="A187" s="5" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="7" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>6</v>
@@ -5109,23 +5115,23 @@
     </row>
     <row r="188">
       <c r="A188" s="5" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="7" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D188" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="5" t="s">
-        <v>351</v>
+      <c r="A189" s="15" t="s">
+        <v>352</v>
       </c>
       <c r="B189" s="6"/>
-      <c r="C189" s="7" t="s">
-        <v>352</v>
+      <c r="C189" s="16" t="s">
+        <v>353</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>6</v>
@@ -5133,11 +5139,11 @@
     </row>
     <row r="190">
       <c r="A190" s="5" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="7" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>6</v>
@@ -5145,11 +5151,11 @@
     </row>
     <row r="191">
       <c r="A191" s="17" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="7" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>6</v>
@@ -5157,11 +5163,11 @@
     </row>
     <row r="192">
       <c r="A192" s="5" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="7" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>6</v>
@@ -5169,11 +5175,11 @@
     </row>
     <row r="193">
       <c r="A193" s="5" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="7" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>6</v>
@@ -5181,11 +5187,11 @@
     </row>
     <row r="194">
       <c r="A194" s="5" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B194" s="6"/>
       <c r="C194" s="7" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>6</v>
@@ -5193,11 +5199,11 @@
     </row>
     <row r="195">
       <c r="A195" s="5" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B195" s="6"/>
       <c r="C195" s="7" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D195" s="5" t="s">
         <v>6</v>
@@ -5205,11 +5211,11 @@
     </row>
     <row r="196">
       <c r="A196" s="10" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B196" s="6"/>
       <c r="C196" s="7" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D196" s="5" t="s">
         <v>6</v>
@@ -5217,11 +5223,11 @@
     </row>
     <row r="197">
       <c r="A197" s="5" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B197" s="6"/>
       <c r="C197" s="7" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D197" s="5" t="s">
         <v>6</v>
@@ -5229,11 +5235,11 @@
     </row>
     <row r="198">
       <c r="A198" s="5" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B198" s="6"/>
       <c r="C198" s="7" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D198" s="5" t="s">
         <v>6</v>
@@ -5241,11 +5247,11 @@
     </row>
     <row r="199">
       <c r="A199" s="5" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B199" s="6"/>
       <c r="C199" s="7" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D199" s="5" t="s">
         <v>6</v>
@@ -5253,11 +5259,11 @@
     </row>
     <row r="200">
       <c r="A200" s="5" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B200" s="6"/>
       <c r="C200" s="7" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D200" s="5" t="s">
         <v>6</v>
@@ -5265,11 +5271,11 @@
     </row>
     <row r="201">
       <c r="A201" s="5" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B201" s="6"/>
       <c r="C201" s="7" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D201" s="5" t="s">
         <v>6</v>
@@ -5277,11 +5283,11 @@
     </row>
     <row r="202">
       <c r="A202" s="5" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B202" s="6"/>
       <c r="C202" s="7" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D202" s="5" t="s">
         <v>6</v>
@@ -5289,11 +5295,11 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B203" s="6"/>
       <c r="C203" s="7" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D203" s="5" t="s">
         <v>6</v>
@@ -5301,11 +5307,11 @@
     </row>
     <row r="204">
       <c r="A204" s="5" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B204" s="6"/>
       <c r="C204" s="7" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D204" s="5" t="s">
         <v>6</v>
@@ -5313,11 +5319,11 @@
     </row>
     <row r="205">
       <c r="A205" s="5" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B205" s="6"/>
       <c r="C205" s="7" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D205" s="5" t="s">
         <v>6</v>
@@ -5325,11 +5331,11 @@
     </row>
     <row r="206">
       <c r="A206" s="5" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B206" s="6"/>
       <c r="C206" s="7" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D206" s="5" t="s">
         <v>6</v>
@@ -5337,11 +5343,11 @@
     </row>
     <row r="207">
       <c r="A207" s="5" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B207" s="6"/>
       <c r="C207" s="7" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D207" s="5" t="s">
         <v>6</v>
@@ -5349,11 +5355,11 @@
     </row>
     <row r="208">
       <c r="A208" s="5" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B208" s="6"/>
       <c r="C208" s="7" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D208" s="5" t="s">
         <v>6</v>
@@ -5361,11 +5367,11 @@
     </row>
     <row r="209">
       <c r="A209" s="5" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B209" s="6"/>
       <c r="C209" s="7" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D209" s="5" t="s">
         <v>6</v>
@@ -5373,11 +5379,11 @@
     </row>
     <row r="210">
       <c r="A210" s="5" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B210" s="6"/>
       <c r="C210" s="7" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D210" s="5" t="s">
         <v>6</v>
@@ -5385,7 +5391,7 @@
     </row>
     <row r="211">
       <c r="A211" s="5" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B211" s="6"/>
       <c r="C211" s="7" t="s">
@@ -5397,11 +5403,11 @@
     </row>
     <row r="212">
       <c r="A212" s="5" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B212" s="6"/>
       <c r="C212" s="7" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D212" s="5" t="s">
         <v>6</v>
@@ -5409,11 +5415,11 @@
     </row>
     <row r="213">
       <c r="A213" s="5" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B213" s="6"/>
       <c r="C213" s="7" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D213" s="5" t="s">
         <v>6</v>
@@ -5421,11 +5427,11 @@
     </row>
     <row r="214">
       <c r="A214" s="5" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B214" s="6"/>
       <c r="C214" s="7" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D214" s="5" t="s">
         <v>6</v>
@@ -5433,11 +5439,11 @@
     </row>
     <row r="215">
       <c r="A215" s="12" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B215" s="6"/>
       <c r="C215" s="7" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D215" s="5" t="s">
         <v>6</v>
@@ -5445,11 +5451,11 @@
     </row>
     <row r="216">
       <c r="A216" s="12" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B216" s="6"/>
       <c r="C216" s="7" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D216" s="5" t="s">
         <v>6</v>
@@ -5457,11 +5463,11 @@
     </row>
     <row r="217">
       <c r="A217" s="12" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B217" s="6"/>
       <c r="C217" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D217" s="5" t="s">
         <v>6</v>
@@ -5469,11 +5475,11 @@
     </row>
     <row r="218">
       <c r="A218" s="12" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B218" s="6"/>
       <c r="C218" s="7" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D218" s="5" t="s">
         <v>6</v>
@@ -5481,11 +5487,11 @@
     </row>
     <row r="219">
       <c r="A219" s="12" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B219" s="6"/>
       <c r="C219" s="7" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D219" s="5" t="s">
         <v>6</v>
@@ -5493,11 +5499,11 @@
     </row>
     <row r="220">
       <c r="A220" s="12" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B220" s="6"/>
       <c r="C220" s="7" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D220" s="5" t="s">
         <v>6</v>
@@ -5505,7 +5511,7 @@
     </row>
     <row r="221">
       <c r="A221" s="5" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B221" s="6"/>
       <c r="C221" s="7" t="s">
@@ -5517,11 +5523,11 @@
     </row>
     <row r="222">
       <c r="A222" s="5" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B222" s="6"/>
       <c r="C222" s="7" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D222" s="5" t="s">
         <v>6</v>
@@ -5529,11 +5535,11 @@
     </row>
     <row r="223">
       <c r="A223" s="5" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B223" s="6"/>
       <c r="C223" s="7" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D223" s="5" t="s">
         <v>6</v>
@@ -5541,11 +5547,11 @@
     </row>
     <row r="224">
       <c r="A224" s="5" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B224" s="6"/>
       <c r="C224" s="7" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D224" s="5" t="s">
         <v>6</v>
@@ -5553,11 +5559,11 @@
     </row>
     <row r="225">
       <c r="A225" s="5" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B225" s="6"/>
       <c r="C225" s="7" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D225" s="5" t="s">
         <v>6</v>
@@ -5565,11 +5571,11 @@
     </row>
     <row r="226">
       <c r="A226" s="5" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B226" s="6"/>
       <c r="C226" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D226" s="5" t="s">
         <v>6</v>
@@ -5577,11 +5583,11 @@
     </row>
     <row r="227">
       <c r="A227" s="5" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B227" s="6"/>
       <c r="C227" s="7" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D227" s="5" t="s">
         <v>6</v>
@@ -5589,11 +5595,11 @@
     </row>
     <row r="228">
       <c r="A228" s="5" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B228" s="6"/>
       <c r="C228" s="7" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D228" s="5" t="s">
         <v>6</v>
@@ -5601,11 +5607,11 @@
     </row>
     <row r="229">
       <c r="A229" s="5" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B229" s="6"/>
       <c r="C229" s="7" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D229" s="5" t="s">
         <v>6</v>
@@ -5613,11 +5619,11 @@
     </row>
     <row r="230">
       <c r="A230" s="5" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B230" s="6"/>
       <c r="C230" s="7" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D230" s="5" t="s">
         <v>6</v>
@@ -5625,11 +5631,11 @@
     </row>
     <row r="231">
       <c r="A231" s="5" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B231" s="6"/>
       <c r="C231" s="7" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D231" s="5" t="s">
         <v>6</v>
@@ -5637,11 +5643,11 @@
     </row>
     <row r="232">
       <c r="A232" s="5" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B232" s="6"/>
       <c r="C232" s="7" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D232" s="5" t="s">
         <v>6</v>
@@ -5649,11 +5655,11 @@
     </row>
     <row r="233">
       <c r="A233" s="5" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B233" s="6"/>
       <c r="C233" s="7" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D233" s="5" t="s">
         <v>6</v>
@@ -5661,11 +5667,11 @@
     </row>
     <row r="234">
       <c r="A234" s="18" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B234" s="19"/>
       <c r="C234" s="20" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D234" s="18" t="s">
         <v>6</v>
@@ -5673,11 +5679,11 @@
     </row>
     <row r="235">
       <c r="A235" s="5" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B235" s="6"/>
       <c r="C235" s="7" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D235" s="5" t="s">
         <v>6</v>
@@ -5685,11 +5691,11 @@
     </row>
     <row r="236">
       <c r="A236" s="5" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B236" s="6"/>
       <c r="C236" s="7" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D236" s="5" t="s">
         <v>6</v>
@@ -5697,11 +5703,11 @@
     </row>
     <row r="237">
       <c r="A237" s="5" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B237" s="6"/>
       <c r="C237" s="7" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D237" s="5" t="s">
         <v>6</v>
@@ -5709,11 +5715,11 @@
     </row>
     <row r="238">
       <c r="A238" s="5" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B238" s="6"/>
       <c r="C238" s="7" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D238" s="5" t="s">
         <v>6</v>
@@ -5721,11 +5727,11 @@
     </row>
     <row r="239">
       <c r="A239" s="5" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B239" s="6"/>
       <c r="C239" s="7" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D239" s="5" t="s">
         <v>6</v>
@@ -5733,11 +5739,11 @@
     </row>
     <row r="240">
       <c r="A240" s="5" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B240" s="6"/>
       <c r="C240" s="7" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D240" s="5" t="s">
         <v>6</v>
@@ -5745,11 +5751,11 @@
     </row>
     <row r="241">
       <c r="A241" s="5" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B241" s="6"/>
       <c r="C241" s="7" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D241" s="5" t="s">
         <v>6</v>
@@ -5757,11 +5763,11 @@
     </row>
     <row r="242">
       <c r="A242" s="5" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B242" s="6"/>
       <c r="C242" s="7" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D242" s="5" t="s">
         <v>6</v>
@@ -5769,11 +5775,11 @@
     </row>
     <row r="243">
       <c r="A243" s="5" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B243" s="6"/>
       <c r="C243" s="7" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D243" s="5" t="s">
         <v>6</v>
@@ -5781,11 +5787,11 @@
     </row>
     <row r="244">
       <c r="A244" s="5" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B244" s="6"/>
       <c r="C244" s="7" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D244" s="5" t="s">
         <v>6</v>
@@ -5793,11 +5799,11 @@
     </row>
     <row r="245">
       <c r="A245" s="5" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B245" s="6"/>
       <c r="C245" s="7" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D245" s="5" t="s">
         <v>6</v>
@@ -5805,11 +5811,11 @@
     </row>
     <row r="246">
       <c r="A246" s="5" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B246" s="6"/>
       <c r="C246" s="7" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D246" s="5" t="s">
         <v>6</v>
@@ -5817,7 +5823,7 @@
     </row>
     <row r="247">
       <c r="A247" s="5" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B247" s="6"/>
       <c r="C247" s="7" t="s">
@@ -5829,11 +5835,11 @@
     </row>
     <row r="248">
       <c r="A248" s="5" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B248" s="6"/>
       <c r="C248" s="7" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D248" s="5" t="s">
         <v>6</v>
@@ -5841,7 +5847,7 @@
     </row>
     <row r="249">
       <c r="A249" s="5" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B249" s="6"/>
       <c r="C249" s="7" t="s">
@@ -5853,11 +5859,11 @@
     </row>
     <row r="250">
       <c r="A250" s="5" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B250" s="6"/>
       <c r="C250" s="7" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D250" s="5" t="s">
         <v>6</v>
@@ -5865,11 +5871,11 @@
     </row>
     <row r="251">
       <c r="A251" s="5" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B251" s="6"/>
       <c r="C251" s="7" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D251" s="5" t="s">
         <v>6</v>
@@ -5877,11 +5883,11 @@
     </row>
     <row r="252">
       <c r="A252" s="5" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B252" s="6"/>
       <c r="C252" s="7" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D252" s="5" t="s">
         <v>6</v>
@@ -5889,57 +5895,35 @@
     </row>
     <row r="253">
       <c r="A253" s="5" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B253" s="6"/>
       <c r="C253" s="7" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D253" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="18" t="s">
-        <v>476</v>
-      </c>
-      <c r="B254" s="19"/>
-      <c r="C254" s="20" t="s">
-        <v>263</v>
-      </c>
-      <c r="D254" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="E254" s="21"/>
-      <c r="F254" s="21"/>
-      <c r="G254" s="21"/>
-      <c r="H254" s="21"/>
-      <c r="I254" s="21"/>
-      <c r="J254" s="21"/>
-      <c r="K254" s="21"/>
-      <c r="L254" s="21"/>
-      <c r="M254" s="21"/>
-      <c r="N254" s="21"/>
-      <c r="O254" s="21"/>
-      <c r="P254" s="21"/>
-      <c r="Q254" s="21"/>
-      <c r="R254" s="21"/>
-      <c r="S254" s="21"/>
-      <c r="T254" s="21"/>
-      <c r="U254" s="21"/>
-      <c r="V254" s="21"/>
-      <c r="W254" s="21"/>
-      <c r="X254" s="21"/>
-      <c r="Y254" s="21"/>
-      <c r="Z254" s="21"/>
+      <c r="A254" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B254" s="6"/>
+      <c r="C254" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="D254" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="5" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B255" s="6"/>
       <c r="C255" s="7" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D255" s="5" t="s">
         <v>6</v>
@@ -5947,11 +5931,11 @@
     </row>
     <row r="256">
       <c r="A256" s="5" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B256" s="6"/>
       <c r="C256" s="7" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="D256" s="5" t="s">
         <v>6</v>
@@ -5959,11 +5943,11 @@
     </row>
     <row r="257">
       <c r="A257" s="5" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B257" s="6"/>
       <c r="C257" s="7" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="D257" s="5" t="s">
         <v>6</v>
@@ -5971,11 +5955,11 @@
     </row>
     <row r="258">
       <c r="A258" s="5" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B258" s="6"/>
       <c r="C258" s="7" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="D258" s="5" t="s">
         <v>6</v>
@@ -5983,36 +5967,35 @@
     </row>
     <row r="259">
       <c r="A259" s="5" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B259" s="6"/>
       <c r="C259" s="7" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="D259" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="18" t="s">
-        <v>487</v>
-      </c>
-      <c r="B260" s="19"/>
-      <c r="C260" s="20" t="s">
-        <v>488</v>
-      </c>
-      <c r="D260" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="E260" s="21"/>
+      <c r="A260" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="B260" s="6"/>
+      <c r="C260" s="7" t="s">
+        <v>490</v>
+      </c>
+      <c r="D260" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="5" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B261" s="6"/>
       <c r="C261" s="7" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="D261" s="5" t="s">
         <v>6</v>
@@ -6020,11 +6003,11 @@
     </row>
     <row r="262">
       <c r="A262" s="5" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B262" s="6"/>
       <c r="C262" s="7" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="D262" s="5" t="s">
         <v>6</v>
@@ -6032,11 +6015,11 @@
     </row>
     <row r="263">
       <c r="A263" s="5" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B263" s="6"/>
       <c r="C263" s="7" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="D263" s="5" t="s">
         <v>6</v>
@@ -6044,11 +6027,11 @@
     </row>
     <row r="264">
       <c r="A264" s="5" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B264" s="6"/>
       <c r="C264" s="7" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D264" s="5" t="s">
         <v>6</v>
@@ -6056,11 +6039,11 @@
     </row>
     <row r="265">
       <c r="A265" s="5" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B265" s="6"/>
       <c r="C265" s="7" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="D265" s="5" t="s">
         <v>6</v>
@@ -6068,11 +6051,11 @@
     </row>
     <row r="266">
       <c r="A266" s="5" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B266" s="6"/>
       <c r="C266" s="7" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="D266" s="5" t="s">
         <v>6</v>
@@ -6080,11 +6063,11 @@
     </row>
     <row r="267">
       <c r="A267" s="5" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B267" s="6"/>
       <c r="C267" s="7" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D267" s="5" t="s">
         <v>6</v>
@@ -6092,11 +6075,11 @@
     </row>
     <row r="268">
       <c r="A268" s="5" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B268" s="6"/>
       <c r="C268" s="7" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="D268" s="5" t="s">
         <v>6</v>
@@ -6104,11 +6087,11 @@
     </row>
     <row r="269">
       <c r="A269" s="5" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B269" s="6"/>
       <c r="C269" s="7" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="D269" s="5" t="s">
         <v>6</v>
@@ -6116,11 +6099,11 @@
     </row>
     <row r="270">
       <c r="A270" s="5" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B270" s="6"/>
       <c r="C270" s="7" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D270" s="5" t="s">
         <v>6</v>
@@ -6128,11 +6111,11 @@
     </row>
     <row r="271">
       <c r="A271" s="5" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B271" s="6"/>
       <c r="C271" s="7" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="D271" s="5" t="s">
         <v>6</v>
@@ -6140,11 +6123,11 @@
     </row>
     <row r="272">
       <c r="A272" s="5" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B272" s="6"/>
       <c r="C272" s="7" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D272" s="5" t="s">
         <v>6</v>
@@ -6152,11 +6135,11 @@
     </row>
     <row r="273">
       <c r="A273" s="5" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B273" s="6"/>
       <c r="C273" s="7" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="D273" s="5" t="s">
         <v>6</v>
@@ -6164,11 +6147,11 @@
     </row>
     <row r="274">
       <c r="A274" s="5" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B274" s="6"/>
       <c r="C274" s="7" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D274" s="5" t="s">
         <v>6</v>
@@ -6176,11 +6159,11 @@
     </row>
     <row r="275">
       <c r="A275" s="5" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B275" s="6"/>
       <c r="C275" s="7" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D275" s="5" t="s">
         <v>6</v>
@@ -6188,11 +6171,11 @@
     </row>
     <row r="276">
       <c r="A276" s="5" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B276" s="6"/>
       <c r="C276" s="7" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D276" s="5" t="s">
         <v>6</v>
@@ -6200,11 +6183,11 @@
     </row>
     <row r="277">
       <c r="A277" s="5" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B277" s="6"/>
       <c r="C277" s="7" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="D277" s="5" t="s">
         <v>6</v>
@@ -6212,11 +6195,11 @@
     </row>
     <row r="278">
       <c r="A278" s="5" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B278" s="6"/>
       <c r="C278" s="7" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D278" s="5" t="s">
         <v>6</v>
@@ -6224,11 +6207,11 @@
     </row>
     <row r="279">
       <c r="A279" s="5" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B279" s="6"/>
       <c r="C279" s="7" t="s">
-        <v>526</v>
+        <v>516</v>
       </c>
       <c r="D279" s="5" t="s">
         <v>6</v>
@@ -6236,11 +6219,11 @@
     </row>
     <row r="280">
       <c r="A280" s="5" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B280" s="6"/>
       <c r="C280" s="7" t="s">
-        <v>528</v>
+        <v>518</v>
       </c>
       <c r="D280" s="5" t="s">
         <v>6</v>
@@ -6252,7 +6235,7 @@
       </c>
       <c r="B281" s="6"/>
       <c r="C281" s="7" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D281" s="5" t="s">
         <v>6</v>
@@ -6264,7 +6247,7 @@
       </c>
       <c r="B282" s="6"/>
       <c r="C282" s="7" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D282" s="5" t="s">
         <v>6</v>
@@ -6275,8 +6258,8 @@
         <v>531</v>
       </c>
       <c r="B283" s="6"/>
-      <c r="C283" s="7" t="s">
-        <v>522</v>
+      <c r="C283" s="16" t="s">
+        <v>532</v>
       </c>
       <c r="D283" s="5" t="s">
         <v>6</v>
@@ -6284,11 +6267,11 @@
     </row>
     <row r="284">
       <c r="A284" s="5" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B284" s="6"/>
-      <c r="C284" s="7" t="s">
-        <v>524</v>
+      <c r="C284" s="16" t="s">
+        <v>534</v>
       </c>
       <c r="D284" s="5" t="s">
         <v>6</v>
@@ -6296,27 +6279,35 @@
     </row>
     <row r="285">
       <c r="A285" s="5" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B285" s="6"/>
-      <c r="C285" s="6"/>
-      <c r="D285" s="6"/>
+      <c r="C285" s="7" t="s">
+        <v>536</v>
+      </c>
+      <c r="D285" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="5" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B286" s="6"/>
-      <c r="C286" s="6"/>
-      <c r="D286" s="6"/>
+      <c r="C286" s="7" t="s">
+        <v>538</v>
+      </c>
+      <c r="D286" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="5" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="B287" s="6"/>
       <c r="C287" s="7" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="D287" s="5" t="s">
         <v>6</v>
@@ -6324,11 +6315,11 @@
     </row>
     <row r="288">
       <c r="A288" s="5" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="B288" s="6"/>
       <c r="C288" s="7" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="D288" s="5" t="s">
         <v>6</v>
@@ -6336,11 +6327,11 @@
     </row>
     <row r="289">
       <c r="A289" s="5" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="B289" s="6"/>
       <c r="C289" s="7" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="D289" s="5" t="s">
         <v>6</v>
@@ -6348,11 +6339,11 @@
     </row>
     <row r="290">
       <c r="A290" s="5" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="B290" s="6"/>
       <c r="C290" s="7" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="D290" s="5" t="s">
         <v>6</v>
@@ -6360,11 +6351,11 @@
     </row>
     <row r="291">
       <c r="A291" s="5" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="B291" s="6"/>
       <c r="C291" s="7" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="D291" s="5" t="s">
         <v>6</v>
@@ -6372,11 +6363,11 @@
     </row>
     <row r="292">
       <c r="A292" s="5" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="B292" s="6"/>
       <c r="C292" s="7" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="D292" s="5" t="s">
         <v>6</v>
@@ -6384,11 +6375,11 @@
     </row>
     <row r="293">
       <c r="A293" s="5" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="B293" s="6"/>
       <c r="C293" s="7" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="D293" s="5" t="s">
         <v>6</v>
@@ -6396,11 +6387,11 @@
     </row>
     <row r="294">
       <c r="A294" s="5" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="B294" s="6"/>
       <c r="C294" s="7" t="s">
-        <v>550</v>
+        <v>516</v>
       </c>
       <c r="D294" s="5" t="s">
         <v>6</v>
@@ -6408,11 +6399,11 @@
     </row>
     <row r="295">
       <c r="A295" s="5" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B295" s="6"/>
       <c r="C295" s="7" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="D295" s="5" t="s">
         <v>6</v>
@@ -6420,11 +6411,11 @@
     </row>
     <row r="296">
       <c r="A296" s="5" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B296" s="6"/>
       <c r="C296" s="7" t="s">
-        <v>518</v>
+        <v>557</v>
       </c>
       <c r="D296" s="5" t="s">
         <v>6</v>
@@ -6432,11 +6423,11 @@
     </row>
     <row r="297">
       <c r="A297" s="5" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="B297" s="6"/>
       <c r="C297" s="7" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="D297" s="5" t="s">
         <v>6</v>
@@ -6444,11 +6435,11 @@
     </row>
     <row r="298">
       <c r="A298" s="5" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="B298" s="6"/>
       <c r="C298" s="7" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="D298" s="5" t="s">
         <v>6</v>
@@ -6456,11 +6447,11 @@
     </row>
     <row r="299">
       <c r="A299" s="5" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="B299" s="6"/>
       <c r="C299" s="7" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D299" s="5" t="s">
         <v>6</v>
@@ -6468,11 +6459,11 @@
     </row>
     <row r="300">
       <c r="A300" s="5" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="B300" s="6"/>
       <c r="C300" s="7" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="D300" s="5" t="s">
         <v>6</v>
@@ -6480,11 +6471,11 @@
     </row>
     <row r="301">
       <c r="A301" s="5" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="B301" s="6"/>
       <c r="C301" s="7" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="D301" s="5" t="s">
         <v>6</v>
@@ -6492,11 +6483,11 @@
     </row>
     <row r="302">
       <c r="A302" s="5" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="B302" s="6"/>
       <c r="C302" s="7" t="s">
-        <v>565</v>
+        <v>510</v>
       </c>
       <c r="D302" s="5" t="s">
         <v>6</v>
@@ -6504,11 +6495,11 @@
     </row>
     <row r="303">
       <c r="A303" s="5" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B303" s="6"/>
       <c r="C303" s="7" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="D303" s="5" t="s">
         <v>6</v>
@@ -6516,11 +6507,11 @@
     </row>
     <row r="304">
       <c r="A304" s="5" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="B304" s="6"/>
       <c r="C304" s="7" t="s">
-        <v>512</v>
+        <v>572</v>
       </c>
       <c r="D304" s="5" t="s">
         <v>6</v>
@@ -6528,11 +6519,11 @@
     </row>
     <row r="305">
       <c r="A305" s="5" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="B305" s="6"/>
       <c r="C305" s="7" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="D305" s="5" t="s">
         <v>6</v>
@@ -6540,11 +6531,11 @@
     </row>
     <row r="306">
       <c r="A306" s="5" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="B306" s="6"/>
       <c r="C306" s="7" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="D306" s="5" t="s">
         <v>6</v>
@@ -6552,11 +6543,11 @@
     </row>
     <row r="307">
       <c r="A307" s="5" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B307" s="6"/>
       <c r="C307" s="7" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D307" s="5" t="s">
         <v>6</v>
@@ -6564,11 +6555,11 @@
     </row>
     <row r="308">
       <c r="A308" s="5" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="B308" s="6"/>
       <c r="C308" s="7" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="D308" s="5" t="s">
         <v>6</v>
@@ -6576,11 +6567,11 @@
     </row>
     <row r="309">
       <c r="A309" s="5" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="B309" s="6"/>
       <c r="C309" s="7" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="D309" s="5" t="s">
         <v>6</v>
@@ -6588,11 +6579,11 @@
     </row>
     <row r="310">
       <c r="A310" s="5" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="B310" s="6"/>
       <c r="C310" s="7" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="D310" s="5" t="s">
         <v>6</v>
@@ -6600,11 +6591,11 @@
     </row>
     <row r="311">
       <c r="A311" s="5" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="B311" s="6"/>
       <c r="C311" s="7" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="D311" s="5" t="s">
         <v>6</v>
@@ -6612,11 +6603,11 @@
     </row>
     <row r="312">
       <c r="A312" s="5" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="B312" s="6"/>
       <c r="C312" s="7" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="D312" s="5" t="s">
         <v>6</v>
@@ -6624,11 +6615,11 @@
     </row>
     <row r="313">
       <c r="A313" s="5" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="B313" s="6"/>
       <c r="C313" s="7" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="D313" s="5" t="s">
         <v>6</v>
@@ -6636,11 +6627,11 @@
     </row>
     <row r="314">
       <c r="A314" s="5" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="B314" s="6"/>
       <c r="C314" s="7" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="D314" s="5" t="s">
         <v>6</v>
@@ -6648,11 +6639,11 @@
     </row>
     <row r="315">
       <c r="A315" s="5" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="B315" s="6"/>
       <c r="C315" s="7" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="D315" s="5" t="s">
         <v>6</v>
@@ -6660,11 +6651,11 @@
     </row>
     <row r="316">
       <c r="A316" s="5" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="B316" s="6"/>
       <c r="C316" s="7" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D316" s="5" t="s">
         <v>6</v>
@@ -6672,11 +6663,11 @@
     </row>
     <row r="317">
       <c r="A317" s="5" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="B317" s="6"/>
       <c r="C317" s="7" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="D317" s="5" t="s">
         <v>6</v>
@@ -6684,11 +6675,11 @@
     </row>
     <row r="318">
       <c r="A318" s="5" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="B318" s="6"/>
       <c r="C318" s="7" t="s">
-        <v>590</v>
+        <v>599</v>
       </c>
       <c r="D318" s="5" t="s">
         <v>6</v>
@@ -6696,35 +6687,35 @@
     </row>
     <row r="319">
       <c r="A319" s="5" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="B319" s="6"/>
       <c r="C319" s="7" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="D319" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="320">
-      <c r="A320" s="5" t="s">
-        <v>598</v>
+      <c r="A320" s="21" t="s">
+        <v>602</v>
       </c>
       <c r="B320" s="6"/>
       <c r="C320" s="7" t="s">
-        <v>599</v>
+        <v>532</v>
       </c>
       <c r="D320" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="5" t="s">
-        <v>600</v>
+      <c r="A321" s="22" t="s">
+        <v>603</v>
       </c>
       <c r="B321" s="6"/>
       <c r="C321" s="7" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="D321" s="5" t="s">
         <v>6</v>
@@ -6732,47 +6723,47 @@
     </row>
     <row r="322">
       <c r="A322" s="22" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="B322" s="6"/>
       <c r="C322" s="7" t="s">
-        <v>603</v>
+        <v>534</v>
       </c>
       <c r="D322" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="323">
-      <c r="A323" s="23" t="s">
-        <v>604</v>
+      <c r="A323" s="22" t="s">
+        <v>606</v>
       </c>
       <c r="B323" s="6"/>
       <c r="C323" s="7" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="D323" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="324">
-      <c r="A324" s="23" t="s">
-        <v>606</v>
+      <c r="A324" s="22" t="s">
+        <v>608</v>
       </c>
       <c r="B324" s="6"/>
       <c r="C324" s="7" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="D324" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="325">
-      <c r="A325" s="23" t="s">
-        <v>608</v>
+      <c r="A325" s="22" t="s">
+        <v>610</v>
       </c>
       <c r="B325" s="6"/>
       <c r="C325" s="7" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="D325" s="5" t="s">
         <v>6</v>
@@ -6780,11 +6771,11 @@
     </row>
     <row r="326">
       <c r="A326" s="23" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="B326" s="6"/>
       <c r="C326" s="7" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="D326" s="5" t="s">
         <v>6</v>
@@ -6792,83 +6783,83 @@
     </row>
     <row r="327">
       <c r="A327" s="23" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="B327" s="6"/>
       <c r="C327" s="7" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D327" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="328">
-      <c r="A328" s="24" t="s">
-        <v>614</v>
+      <c r="A328" s="23" t="s">
+        <v>616</v>
       </c>
       <c r="B328" s="6"/>
       <c r="C328" s="7" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="D328" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="329">
-      <c r="A329" s="24" t="s">
-        <v>616</v>
+      <c r="A329" s="23" t="s">
+        <v>618</v>
       </c>
       <c r="B329" s="6"/>
       <c r="C329" s="7" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="D329" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="330">
-      <c r="A330" s="24" t="s">
-        <v>618</v>
+      <c r="A330" s="23" t="s">
+        <v>620</v>
       </c>
       <c r="B330" s="6"/>
       <c r="C330" s="7" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="D330" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="331">
-      <c r="A331" s="24" t="s">
-        <v>620</v>
+      <c r="A331" s="23" t="s">
+        <v>622</v>
       </c>
       <c r="B331" s="6"/>
       <c r="C331" s="7" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="D331" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="332">
-      <c r="A332" s="24" t="s">
-        <v>622</v>
+      <c r="A332" s="5" t="s">
+        <v>624</v>
       </c>
       <c r="B332" s="6"/>
       <c r="C332" s="7" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="D332" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="333">
-      <c r="A333" s="24" t="s">
-        <v>624</v>
+      <c r="A333" s="5" t="s">
+        <v>626</v>
       </c>
       <c r="B333" s="6"/>
       <c r="C333" s="7" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="D333" s="5" t="s">
         <v>6</v>
@@ -6876,11 +6867,11 @@
     </row>
     <row r="334">
       <c r="A334" s="5" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="B334" s="6"/>
       <c r="C334" s="7" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="D334" s="5" t="s">
         <v>6</v>
@@ -6888,11 +6879,11 @@
     </row>
     <row r="335">
       <c r="A335" s="5" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="B335" s="6"/>
       <c r="C335" s="7" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="D335" s="5" t="s">
         <v>6</v>
@@ -6900,11 +6891,11 @@
     </row>
     <row r="336">
       <c r="A336" s="5" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B336" s="6"/>
       <c r="C336" s="7" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="D336" s="5" t="s">
         <v>6</v>
@@ -6912,11 +6903,11 @@
     </row>
     <row r="337">
       <c r="A337" s="5" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="B337" s="6"/>
       <c r="C337" s="7" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="D337" s="5" t="s">
         <v>6</v>
@@ -6924,11 +6915,11 @@
     </row>
     <row r="338">
       <c r="A338" s="5" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="B338" s="6"/>
       <c r="C338" s="7" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="D338" s="5" t="s">
         <v>6</v>
@@ -6936,11 +6927,11 @@
     </row>
     <row r="339">
       <c r="A339" s="5" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="B339" s="6"/>
       <c r="C339" s="7" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="D339" s="5" t="s">
         <v>6</v>
@@ -6948,11 +6939,11 @@
     </row>
     <row r="340">
       <c r="A340" s="5" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="B340" s="6"/>
       <c r="C340" s="7" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="D340" s="5" t="s">
         <v>6</v>
@@ -6960,11 +6951,11 @@
     </row>
     <row r="341">
       <c r="A341" s="5" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B341" s="6"/>
       <c r="C341" s="7" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="D341" s="5" t="s">
         <v>6</v>
@@ -6972,11 +6963,11 @@
     </row>
     <row r="342">
       <c r="A342" s="5" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="B342" s="6"/>
       <c r="C342" s="7" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="D342" s="5" t="s">
         <v>6</v>
@@ -6984,11 +6975,11 @@
     </row>
     <row r="343">
       <c r="A343" s="5" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="B343" s="6"/>
       <c r="C343" s="7" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="D343" s="5" t="s">
         <v>6</v>
@@ -6996,11 +6987,11 @@
     </row>
     <row r="344">
       <c r="A344" s="5" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="B344" s="6"/>
       <c r="C344" s="7" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="D344" s="5" t="s">
         <v>6</v>
@@ -7008,11 +6999,11 @@
     </row>
     <row r="345">
       <c r="A345" s="5" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="B345" s="6"/>
       <c r="C345" s="7" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="D345" s="5" t="s">
         <v>6</v>
@@ -7020,11 +7011,11 @@
     </row>
     <row r="346">
       <c r="A346" s="5" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="B346" s="6"/>
       <c r="C346" s="7" t="s">
-        <v>651</v>
+        <v>461</v>
       </c>
       <c r="D346" s="5" t="s">
         <v>6</v>
@@ -7032,11 +7023,11 @@
     </row>
     <row r="347">
       <c r="A347" s="5" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B347" s="6"/>
       <c r="C347" s="7" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="D347" s="5" t="s">
         <v>6</v>
@@ -7044,11 +7035,11 @@
     </row>
     <row r="348">
       <c r="A348" s="5" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B348" s="6"/>
       <c r="C348" s="7" t="s">
-        <v>460</v>
+        <v>656</v>
       </c>
       <c r="D348" s="5" t="s">
         <v>6</v>
@@ -7056,11 +7047,11 @@
     </row>
     <row r="349">
       <c r="A349" s="5" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B349" s="6"/>
       <c r="C349" s="7" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="D349" s="5" t="s">
         <v>6</v>
@@ -7068,11 +7059,11 @@
     </row>
     <row r="350">
       <c r="A350" s="5" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="B350" s="6"/>
       <c r="C350" s="7" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="D350" s="5" t="s">
         <v>6</v>
@@ -7080,11 +7071,11 @@
     </row>
     <row r="351">
       <c r="A351" s="5" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="B351" s="6"/>
       <c r="C351" s="7" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="D351" s="5" t="s">
         <v>6</v>
@@ -7092,11 +7083,11 @@
     </row>
     <row r="352">
       <c r="A352" s="5" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="B352" s="6"/>
       <c r="C352" s="7" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="D352" s="5" t="s">
         <v>6</v>
@@ -7104,11 +7095,11 @@
     </row>
     <row r="353">
       <c r="A353" s="5" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="B353" s="6"/>
       <c r="C353" s="7" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="D353" s="5" t="s">
         <v>6</v>
@@ -7116,11 +7107,11 @@
     </row>
     <row r="354">
       <c r="A354" s="5" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="B354" s="6"/>
       <c r="C354" s="7" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="D354" s="5" t="s">
         <v>6</v>
@@ -7128,11 +7119,11 @@
     </row>
     <row r="355">
       <c r="A355" s="5" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B355" s="6"/>
       <c r="C355" s="7" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="D355" s="5" t="s">
         <v>6</v>
@@ -7140,11 +7131,11 @@
     </row>
     <row r="356">
       <c r="A356" s="5" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="B356" s="6"/>
       <c r="C356" s="7" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="D356" s="5" t="s">
         <v>6</v>
@@ -7152,11 +7143,11 @@
     </row>
     <row r="357">
       <c r="A357" s="5" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="B357" s="6"/>
       <c r="C357" s="7" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="D357" s="5" t="s">
         <v>6</v>
@@ -7164,11 +7155,11 @@
     </row>
     <row r="358">
       <c r="A358" s="5" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="B358" s="6"/>
       <c r="C358" s="7" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="D358" s="5" t="s">
         <v>6</v>
@@ -7176,11 +7167,11 @@
     </row>
     <row r="359">
       <c r="A359" s="5" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="B359" s="6"/>
       <c r="C359" s="7" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="D359" s="5" t="s">
         <v>6</v>
@@ -7188,11 +7179,11 @@
     </row>
     <row r="360">
       <c r="A360" s="5" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="B360" s="6"/>
       <c r="C360" s="7" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="D360" s="5" t="s">
         <v>6</v>
@@ -7200,11 +7191,11 @@
     </row>
     <row r="361">
       <c r="A361" s="5" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="B361" s="6"/>
       <c r="C361" s="7" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="D361" s="5" t="s">
         <v>6</v>
@@ -7212,11 +7203,11 @@
     </row>
     <row r="362">
       <c r="A362" s="5" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="B362" s="6"/>
       <c r="C362" s="7" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="D362" s="5" t="s">
         <v>6</v>
@@ -7224,11 +7215,11 @@
     </row>
     <row r="363">
       <c r="A363" s="5" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="B363" s="6"/>
       <c r="C363" s="7" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="D363" s="5" t="s">
         <v>6</v>
@@ -7236,11 +7227,11 @@
     </row>
     <row r="364">
       <c r="A364" s="5" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B364" s="6"/>
       <c r="C364" s="7" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="D364" s="5" t="s">
         <v>6</v>
@@ -7248,11 +7239,11 @@
     </row>
     <row r="365">
       <c r="A365" s="5" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="B365" s="6"/>
       <c r="C365" s="7" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="D365" s="5" t="s">
         <v>6</v>
@@ -7260,11 +7251,11 @@
     </row>
     <row r="366">
       <c r="A366" s="5" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B366" s="6"/>
       <c r="C366" s="7" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="D366" s="5" t="s">
         <v>6</v>
@@ -7272,11 +7263,11 @@
     </row>
     <row r="367">
       <c r="A367" s="5" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="B367" s="6"/>
       <c r="C367" s="7" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="D367" s="5" t="s">
         <v>6</v>
@@ -7284,11 +7275,11 @@
     </row>
     <row r="368">
       <c r="A368" s="5" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="B368" s="6"/>
       <c r="C368" s="7" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="D368" s="5" t="s">
         <v>6</v>
@@ -7296,11 +7287,11 @@
     </row>
     <row r="369">
       <c r="A369" s="5" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="B369" s="6"/>
       <c r="C369" s="7" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="D369" s="5" t="s">
         <v>6</v>
@@ -7308,11 +7299,11 @@
     </row>
     <row r="370">
       <c r="A370" s="5" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="B370" s="6"/>
       <c r="C370" s="7" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="D370" s="5" t="s">
         <v>6</v>
@@ -7320,11 +7311,11 @@
     </row>
     <row r="371">
       <c r="A371" s="5" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B371" s="6"/>
       <c r="C371" s="7" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="D371" s="5" t="s">
         <v>6</v>
@@ -7332,11 +7323,11 @@
     </row>
     <row r="372">
       <c r="A372" s="5" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="B372" s="6"/>
       <c r="C372" s="7" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="D372" s="5" t="s">
         <v>6</v>
@@ -7344,11 +7335,11 @@
     </row>
     <row r="373">
       <c r="A373" s="5" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="B373" s="6"/>
       <c r="C373" s="7" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="D373" s="5" t="s">
         <v>6</v>
@@ -7356,11 +7347,11 @@
     </row>
     <row r="374">
       <c r="A374" s="5" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="B374" s="6"/>
       <c r="C374" s="7" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="D374" s="5" t="s">
         <v>6</v>
@@ -7368,11 +7359,11 @@
     </row>
     <row r="375">
       <c r="A375" s="5" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B375" s="6"/>
       <c r="C375" s="7" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="D375" s="5" t="s">
         <v>6</v>
@@ -7380,11 +7371,11 @@
     </row>
     <row r="376">
       <c r="A376" s="5" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="B376" s="6"/>
       <c r="C376" s="7" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="D376" s="5" t="s">
         <v>6</v>
@@ -7392,11 +7383,11 @@
     </row>
     <row r="377">
       <c r="A377" s="5" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="B377" s="6"/>
       <c r="C377" s="7" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="D377" s="5" t="s">
         <v>6</v>
@@ -7404,11 +7395,11 @@
     </row>
     <row r="378">
       <c r="A378" s="5" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B378" s="6"/>
       <c r="C378" s="7" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="D378" s="5" t="s">
         <v>6</v>
@@ -7416,11 +7407,11 @@
     </row>
     <row r="379">
       <c r="A379" s="5" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="B379" s="6"/>
       <c r="C379" s="7" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="D379" s="5" t="s">
         <v>6</v>
@@ -7428,11 +7419,11 @@
     </row>
     <row r="380">
       <c r="A380" s="5" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="B380" s="6"/>
       <c r="C380" s="7" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="D380" s="5" t="s">
         <v>6</v>
@@ -7440,11 +7431,11 @@
     </row>
     <row r="381">
       <c r="A381" s="5" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="B381" s="6"/>
       <c r="C381" s="7" t="s">
-        <v>720</v>
+        <v>633</v>
       </c>
       <c r="D381" s="5" t="s">
         <v>6</v>
@@ -7452,11 +7443,11 @@
     </row>
     <row r="382">
       <c r="A382" s="5" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B382" s="6"/>
       <c r="C382" s="7" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="D382" s="5" t="s">
         <v>6</v>
@@ -7464,11 +7455,11 @@
     </row>
     <row r="383">
       <c r="A383" s="5" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B383" s="6"/>
       <c r="C383" s="7" t="s">
-        <v>635</v>
+        <v>725</v>
       </c>
       <c r="D383" s="5" t="s">
         <v>6</v>
@@ -7476,11 +7467,11 @@
     </row>
     <row r="384">
       <c r="A384" s="5" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B384" s="6"/>
       <c r="C384" s="7" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="D384" s="5" t="s">
         <v>6</v>
@@ -7488,11 +7479,11 @@
     </row>
     <row r="385">
       <c r="A385" s="5" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="B385" s="6"/>
       <c r="C385" s="7" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="D385" s="5" t="s">
         <v>6</v>
@@ -7500,11 +7491,11 @@
     </row>
     <row r="386">
       <c r="A386" s="5" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="B386" s="6"/>
       <c r="C386" s="7" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="D386" s="5" t="s">
         <v>6</v>
@@ -7512,11 +7503,11 @@
     </row>
     <row r="387">
       <c r="A387" s="5" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B387" s="6"/>
       <c r="C387" s="7" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D387" s="5" t="s">
         <v>6</v>
@@ -7524,11 +7515,11 @@
     </row>
     <row r="388">
       <c r="A388" s="5" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="B388" s="6"/>
       <c r="C388" s="7" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="D388" s="5" t="s">
         <v>6</v>
@@ -7536,11 +7527,11 @@
     </row>
     <row r="389">
       <c r="A389" s="5" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="B389" s="6"/>
       <c r="C389" s="7" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="D389" s="5" t="s">
         <v>6</v>
@@ -7548,11 +7539,11 @@
     </row>
     <row r="390">
       <c r="A390" s="5" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="B390" s="6"/>
       <c r="C390" s="7" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="D390" s="5" t="s">
         <v>6</v>
@@ -7560,11 +7551,11 @@
     </row>
     <row r="391">
       <c r="A391" s="5" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="B391" s="6"/>
       <c r="C391" s="7" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="D391" s="5" t="s">
         <v>6</v>
@@ -7572,11 +7563,11 @@
     </row>
     <row r="392">
       <c r="A392" s="5" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="B392" s="6"/>
       <c r="C392" s="7" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="D392" s="5" t="s">
         <v>6</v>
@@ -7584,11 +7575,11 @@
     </row>
     <row r="393">
       <c r="A393" s="5" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="B393" s="6"/>
       <c r="C393" s="7" t="s">
-        <v>743</v>
+        <v>510</v>
       </c>
       <c r="D393" s="5" t="s">
         <v>6</v>
@@ -7596,11 +7587,11 @@
     </row>
     <row r="394">
       <c r="A394" s="5" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B394" s="6"/>
       <c r="C394" s="7" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="D394" s="5" t="s">
         <v>6</v>
@@ -7608,35 +7599,35 @@
     </row>
     <row r="395">
       <c r="A395" s="5" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B395" s="6"/>
       <c r="C395" s="7" t="s">
-        <v>512</v>
+        <v>748</v>
       </c>
       <c r="D395" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="396">
-      <c r="A396" s="5" t="s">
-        <v>747</v>
+      <c r="A396" s="10" t="s">
+        <v>749</v>
       </c>
       <c r="B396" s="6"/>
       <c r="C396" s="7" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="D396" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="397">
-      <c r="A397" s="5" t="s">
-        <v>749</v>
+      <c r="A397" s="10" t="s">
+        <v>751</v>
       </c>
       <c r="B397" s="6"/>
       <c r="C397" s="7" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="D397" s="5" t="s">
         <v>6</v>
@@ -7644,23 +7635,23 @@
     </row>
     <row r="398">
       <c r="A398" s="10" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="B398" s="6"/>
       <c r="C398" s="7" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="D398" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="399">
-      <c r="A399" s="10" t="s">
-        <v>753</v>
+      <c r="A399" s="5" t="s">
+        <v>755</v>
       </c>
       <c r="B399" s="6"/>
       <c r="C399" s="7" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D399" s="5" t="s">
         <v>6</v>
@@ -7668,11 +7659,11 @@
     </row>
     <row r="400">
       <c r="A400" s="10" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="B400" s="6"/>
       <c r="C400" s="7" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="D400" s="5" t="s">
         <v>6</v>
@@ -7680,23 +7671,23 @@
     </row>
     <row r="401">
       <c r="A401" s="5" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="B401" s="6"/>
       <c r="C401" s="7" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="D401" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="402">
-      <c r="A402" s="10" t="s">
-        <v>759</v>
+      <c r="A402" s="5" t="s">
+        <v>761</v>
       </c>
       <c r="B402" s="6"/>
       <c r="C402" s="7" t="s">
-        <v>760</v>
+        <v>164</v>
       </c>
       <c r="D402" s="5" t="s">
         <v>6</v>
@@ -7704,11 +7695,11 @@
     </row>
     <row r="403">
       <c r="A403" s="5" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="B403" s="6"/>
       <c r="C403" s="7" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="D403" s="5" t="s">
         <v>6</v>
@@ -7716,11 +7707,11 @@
     </row>
     <row r="404">
       <c r="A404" s="5" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="B404" s="6"/>
       <c r="C404" s="7" t="s">
-        <v>164</v>
+        <v>765</v>
       </c>
       <c r="D404" s="5" t="s">
         <v>6</v>
@@ -7728,11 +7719,11 @@
     </row>
     <row r="405">
       <c r="A405" s="5" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="B405" s="6"/>
       <c r="C405" s="7" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="D405" s="5" t="s">
         <v>6</v>
@@ -7740,11 +7731,11 @@
     </row>
     <row r="406">
       <c r="A406" s="5" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="B406" s="6"/>
       <c r="C406" s="7" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="D406" s="5" t="s">
         <v>6</v>
@@ -7752,11 +7743,11 @@
     </row>
     <row r="407">
       <c r="A407" s="5" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="B407" s="6"/>
       <c r="C407" s="7" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="D407" s="5" t="s">
         <v>6</v>
@@ -7764,11 +7755,11 @@
     </row>
     <row r="408">
       <c r="A408" s="5" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="B408" s="6"/>
       <c r="C408" s="7" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="D408" s="5" t="s">
         <v>6</v>
@@ -7776,11 +7767,11 @@
     </row>
     <row r="409">
       <c r="A409" s="5" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="B409" s="6"/>
       <c r="C409" s="7" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="D409" s="5" t="s">
         <v>6</v>
@@ -7788,11 +7779,11 @@
     </row>
     <row r="410">
       <c r="A410" s="5" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="B410" s="6"/>
       <c r="C410" s="7" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="D410" s="5" t="s">
         <v>6</v>
@@ -7800,11 +7791,11 @@
     </row>
     <row r="411">
       <c r="A411" s="5" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="B411" s="6"/>
       <c r="C411" s="7" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="D411" s="5" t="s">
         <v>6</v>
@@ -7812,11 +7803,11 @@
     </row>
     <row r="412">
       <c r="A412" s="5" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="B412" s="6"/>
       <c r="C412" s="7" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="D412" s="5" t="s">
         <v>6</v>
@@ -7824,11 +7815,11 @@
     </row>
     <row r="413">
       <c r="A413" s="5" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="B413" s="6"/>
       <c r="C413" s="7" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="D413" s="5" t="s">
         <v>6</v>
@@ -7836,11 +7827,11 @@
     </row>
     <row r="414">
       <c r="A414" s="5" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B414" s="6"/>
       <c r="C414" s="7" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="D414" s="5" t="s">
         <v>6</v>
@@ -7848,11 +7839,11 @@
     </row>
     <row r="415">
       <c r="A415" s="5" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="B415" s="6"/>
       <c r="C415" s="7" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="D415" s="5" t="s">
         <v>6</v>
@@ -7860,33 +7851,39 @@
     </row>
     <row r="416">
       <c r="A416" s="5" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="B416" s="6"/>
       <c r="C416" s="7" t="s">
-        <v>781</v>
+        <v>788</v>
       </c>
       <c r="D416" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="417">
-      <c r="A417" s="5" t="s">
-        <v>787</v>
+      <c r="A417" s="15" t="s">
+        <v>789</v>
       </c>
       <c r="B417" s="6"/>
-      <c r="C417" s="7" t="s">
-        <v>788</v>
+      <c r="C417" s="16" t="s">
+        <v>790</v>
       </c>
       <c r="D417" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="418">
-      <c r="A418" s="6"/>
+      <c r="A418" s="15" t="s">
+        <v>791</v>
+      </c>
       <c r="B418" s="6"/>
-      <c r="C418" s="6"/>
-      <c r="D418" s="6"/>
+      <c r="C418" s="16" t="s">
+        <v>792</v>
+      </c>
+      <c r="D418" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="419">
       <c r="A419" s="6"/>
@@ -12406,21 +12403,9 @@
       <c r="C1171" s="6"/>
       <c r="D1171" s="6"/>
     </row>
-    <row r="1172">
-      <c r="A1172" s="6"/>
-      <c r="B1172" s="6"/>
-      <c r="C1172" s="6"/>
-      <c r="D1172" s="6"/>
-    </row>
-    <row r="1173">
-      <c r="A1173" s="6"/>
-      <c r="B1173" s="6"/>
-      <c r="C1173" s="6"/>
-      <c r="D1173" s="6"/>
-    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D284 D287:D417">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D418">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12485,11 +12470,11 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="7" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>6</v>
@@ -12497,10 +12482,10 @@
     </row>
     <row r="3">
       <c r="A3" s="12" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>6</v>
@@ -12508,10 +12493,10 @@
     </row>
     <row r="4">
       <c r="A4" s="12" t="s">
-        <v>793</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>794</v>
+        <v>797</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>798</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>6</v>
@@ -12519,10 +12504,10 @@
     </row>
     <row r="5">
       <c r="A5" s="12" t="s">
-        <v>795</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>796</v>
+        <v>799</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>800</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>6</v>
@@ -12530,10 +12515,10 @@
     </row>
     <row r="6">
       <c r="A6" s="12" t="s">
-        <v>797</v>
-      </c>
-      <c r="C6" s="25" t="s">
-        <v>798</v>
+        <v>801</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>802</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
Fix tag list is managed according to user logged-in state + Search tag screen has "check" button
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1274" uniqueCount="803">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1277" uniqueCount="805">
   <si>
     <t>Key</t>
   </si>
@@ -509,6 +509,12 @@
   </si>
   <si>
     <t>Edit</t>
+  </si>
+  <si>
+    <t>global.add</t>
+  </si>
+  <si>
+    <t>Add</t>
   </si>
   <si>
     <t>home.sync.syncing</t>
@@ -2479,7 +2485,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -2515,6 +2521,7 @@
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -2557,7 +2564,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2603,16 +2610,19 @@
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -3955,14 +3965,13 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="5" t="s">
+      <c r="A92" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="B92" s="6"/>
-      <c r="C92" s="7" t="s">
+      <c r="C92" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="D92" s="5" t="s">
+      <c r="D92" s="12" t="s">
         <v>6</v>
       </c>
     </row>
@@ -4123,7 +4132,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="10" t="s">
+      <c r="A106" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B106" s="6"/>
@@ -4147,7 +4156,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="5" t="s">
+      <c r="A108" s="10" t="s">
         <v>197</v>
       </c>
       <c r="B108" s="6"/>
@@ -4452,7 +4461,7 @@
       </c>
       <c r="B133" s="6"/>
       <c r="C133" s="7" t="s">
-        <v>46</v>
+        <v>248</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>6</v>
@@ -4460,7 +4469,7 @@
     </row>
     <row r="134">
       <c r="A134" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B134" s="6"/>
       <c r="C134" s="7" t="s">
@@ -4472,11 +4481,11 @@
     </row>
     <row r="135">
       <c r="A135" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B135" s="6"/>
       <c r="C135" s="7" t="s">
-        <v>250</v>
+        <v>46</v>
       </c>
       <c r="D135" s="5" t="s">
         <v>6</v>
@@ -4486,7 +4495,7 @@
       <c r="A136" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="B136" s="5"/>
+      <c r="B136" s="6"/>
       <c r="C136" s="7" t="s">
         <v>252</v>
       </c>
@@ -4498,7 +4507,7 @@
       <c r="A137" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="B137" s="6"/>
+      <c r="B137" s="5"/>
       <c r="C137" s="7" t="s">
         <v>254</v>
       </c>
@@ -4536,7 +4545,7 @@
       </c>
       <c r="B140" s="6"/>
       <c r="C140" s="7" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="D140" s="5" t="s">
         <v>6</v>
@@ -4544,11 +4553,11 @@
     </row>
     <row r="141">
       <c r="A141" s="5" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="7" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="D141" s="5" t="s">
         <v>6</v>
@@ -4584,7 +4593,7 @@
       </c>
       <c r="B144" s="6"/>
       <c r="C144" s="7" t="s">
-        <v>250</v>
+        <v>267</v>
       </c>
       <c r="D144" s="5" t="s">
         <v>6</v>
@@ -4592,11 +4601,11 @@
     </row>
     <row r="145">
       <c r="A145" s="5" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B145" s="6"/>
       <c r="C145" s="7" t="s">
-        <v>268</v>
+        <v>252</v>
       </c>
       <c r="D145" s="5" t="s">
         <v>6</v>
@@ -4675,7 +4684,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="10" t="s">
+      <c r="A152" s="5" t="s">
         <v>281</v>
       </c>
       <c r="B152" s="6"/>
@@ -4692,7 +4701,7 @@
       </c>
       <c r="B153" s="6"/>
       <c r="C153" s="7" t="s">
-        <v>256</v>
+        <v>284</v>
       </c>
       <c r="D153" s="5" t="s">
         <v>6</v>
@@ -4700,18 +4709,18 @@
     </row>
     <row r="154">
       <c r="A154" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B154" s="6"/>
       <c r="C154" s="7" t="s">
-        <v>285</v>
+        <v>258</v>
       </c>
       <c r="D154" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="5" t="s">
+      <c r="A155" s="10" t="s">
         <v>286</v>
       </c>
       <c r="B155" s="6"/>
@@ -4951,7 +4960,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="10" t="s">
+      <c r="A175" s="5" t="s">
         <v>326</v>
       </c>
       <c r="B175" s="6"/>
@@ -4987,12 +4996,12 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="5" t="s">
+      <c r="A178" s="10" t="s">
         <v>332</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="7" t="s">
-        <v>263</v>
+        <v>333</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>6</v>
@@ -5000,11 +5009,11 @@
     </row>
     <row r="179">
       <c r="A179" s="5" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="7" t="s">
-        <v>334</v>
+        <v>265</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>6</v>
@@ -5016,7 +5025,7 @@
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="7" t="s">
-        <v>67</v>
+        <v>336</v>
       </c>
       <c r="D180" s="5" t="s">
         <v>6</v>
@@ -5024,11 +5033,11 @@
     </row>
     <row r="181">
       <c r="A181" s="5" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="7" t="s">
-        <v>337</v>
+        <v>67</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>6</v>
@@ -5143,7 +5152,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="15" t="s">
+      <c r="A191" s="5" t="s">
         <v>356</v>
       </c>
       <c r="B191" s="6"/>
@@ -5155,7 +5164,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="5" t="s">
+      <c r="A192" s="16" t="s">
         <v>358</v>
       </c>
       <c r="B192" s="6"/>
@@ -5203,7 +5212,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="10" t="s">
+      <c r="A196" s="5" t="s">
         <v>366</v>
       </c>
       <c r="B196" s="6"/>
@@ -5215,7 +5224,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="5" t="s">
+      <c r="A197" s="10" t="s">
         <v>368</v>
       </c>
       <c r="B197" s="6"/>
@@ -5388,7 +5397,7 @@
       </c>
       <c r="B211" s="6"/>
       <c r="C211" s="7" t="s">
-        <v>57</v>
+        <v>397</v>
       </c>
       <c r="D211" s="5" t="s">
         <v>6</v>
@@ -5396,11 +5405,11 @@
     </row>
     <row r="212">
       <c r="A212" s="5" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B212" s="6"/>
       <c r="C212" s="7" t="s">
-        <v>398</v>
+        <v>57</v>
       </c>
       <c r="D212" s="5" t="s">
         <v>6</v>
@@ -5431,7 +5440,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="12" t="s">
+      <c r="A215" s="5" t="s">
         <v>403</v>
       </c>
       <c r="B215" s="6"/>
@@ -5503,12 +5512,12 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="5" t="s">
+      <c r="A221" s="12" t="s">
         <v>415</v>
       </c>
       <c r="B221" s="6"/>
       <c r="C221" s="7" t="s">
-        <v>150</v>
+        <v>416</v>
       </c>
       <c r="D221" s="5" t="s">
         <v>6</v>
@@ -5516,11 +5525,11 @@
     </row>
     <row r="222">
       <c r="A222" s="5" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B222" s="6"/>
       <c r="C222" s="7" t="s">
-        <v>417</v>
+        <v>150</v>
       </c>
       <c r="D222" s="5" t="s">
         <v>6</v>
@@ -5659,26 +5668,26 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="16" t="s">
+      <c r="A234" s="5" t="s">
         <v>440</v>
       </c>
-      <c r="B234" s="17"/>
-      <c r="C234" s="18" t="s">
+      <c r="B234" s="6"/>
+      <c r="C234" s="7" t="s">
         <v>441</v>
       </c>
-      <c r="D234" s="16" t="s">
+      <c r="D234" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="5" t="s">
+      <c r="A235" s="17" t="s">
         <v>442</v>
       </c>
-      <c r="B235" s="6"/>
-      <c r="C235" s="7" t="s">
+      <c r="B235" s="18"/>
+      <c r="C235" s="19" t="s">
         <v>443</v>
       </c>
-      <c r="D235" s="5" t="s">
+      <c r="D235" s="17" t="s">
         <v>6</v>
       </c>
     </row>
@@ -5820,7 +5829,7 @@
       </c>
       <c r="B247" s="6"/>
       <c r="C247" s="7" t="s">
-        <v>67</v>
+        <v>467</v>
       </c>
       <c r="D247" s="5" t="s">
         <v>6</v>
@@ -5828,11 +5837,11 @@
     </row>
     <row r="248">
       <c r="A248" s="5" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B248" s="6"/>
       <c r="C248" s="7" t="s">
-        <v>468</v>
+        <v>67</v>
       </c>
       <c r="D248" s="5" t="s">
         <v>6</v>
@@ -5844,7 +5853,7 @@
       </c>
       <c r="B249" s="6"/>
       <c r="C249" s="7" t="s">
-        <v>200</v>
+        <v>470</v>
       </c>
       <c r="D249" s="5" t="s">
         <v>6</v>
@@ -5852,11 +5861,11 @@
     </row>
     <row r="250">
       <c r="A250" s="5" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B250" s="6"/>
       <c r="C250" s="7" t="s">
-        <v>471</v>
+        <v>202</v>
       </c>
       <c r="D250" s="5" t="s">
         <v>6</v>
@@ -5868,7 +5877,7 @@
       </c>
       <c r="B251" s="6"/>
       <c r="C251" s="7" t="s">
-        <v>341</v>
+        <v>473</v>
       </c>
       <c r="D251" s="5" t="s">
         <v>6</v>
@@ -5876,11 +5885,11 @@
     </row>
     <row r="252">
       <c r="A252" s="5" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B252" s="6"/>
       <c r="C252" s="7" t="s">
-        <v>474</v>
+        <v>343</v>
       </c>
       <c r="D252" s="5" t="s">
         <v>6</v>
@@ -6204,7 +6213,7 @@
       </c>
       <c r="B279" s="6"/>
       <c r="C279" s="7" t="s">
-        <v>516</v>
+        <v>528</v>
       </c>
       <c r="D279" s="5" t="s">
         <v>6</v>
@@ -6212,7 +6221,7 @@
     </row>
     <row r="280">
       <c r="A280" s="5" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B280" s="6"/>
       <c r="C280" s="7" t="s">
@@ -6224,7 +6233,7 @@
     </row>
     <row r="281">
       <c r="A281" s="5" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B281" s="6"/>
       <c r="C281" s="7" t="s">
@@ -6236,7 +6245,7 @@
     </row>
     <row r="282">
       <c r="A282" s="5" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B282" s="6"/>
       <c r="C282" s="7" t="s">
@@ -6248,11 +6257,11 @@
     </row>
     <row r="283">
       <c r="A283" s="5" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B283" s="6"/>
       <c r="C283" s="7" t="s">
-        <v>532</v>
+        <v>524</v>
       </c>
       <c r="D283" s="5" t="s">
         <v>6</v>
@@ -6384,7 +6393,7 @@
       </c>
       <c r="B294" s="6"/>
       <c r="C294" s="7" t="s">
-        <v>516</v>
+        <v>554</v>
       </c>
       <c r="D294" s="5" t="s">
         <v>6</v>
@@ -6392,11 +6401,11 @@
     </row>
     <row r="295">
       <c r="A295" s="5" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B295" s="6"/>
       <c r="C295" s="7" t="s">
-        <v>555</v>
+        <v>518</v>
       </c>
       <c r="D295" s="5" t="s">
         <v>6</v>
@@ -6480,7 +6489,7 @@
       </c>
       <c r="B302" s="6"/>
       <c r="C302" s="7" t="s">
-        <v>510</v>
+        <v>569</v>
       </c>
       <c r="D302" s="5" t="s">
         <v>6</v>
@@ -6488,11 +6497,11 @@
     </row>
     <row r="303">
       <c r="A303" s="5" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B303" s="6"/>
       <c r="C303" s="7" t="s">
-        <v>570</v>
+        <v>512</v>
       </c>
       <c r="D303" s="5" t="s">
         <v>6</v>
@@ -6648,7 +6657,7 @@
       </c>
       <c r="B316" s="6"/>
       <c r="C316" s="7" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
       <c r="D316" s="5" t="s">
         <v>6</v>
@@ -6656,11 +6665,11 @@
     </row>
     <row r="317">
       <c r="A317" s="5" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B317" s="6"/>
       <c r="C317" s="7" t="s">
-        <v>597</v>
+        <v>592</v>
       </c>
       <c r="D317" s="5" t="s">
         <v>6</v>
@@ -6691,12 +6700,12 @@
       </c>
     </row>
     <row r="320">
-      <c r="A320" s="19" t="s">
+      <c r="A320" s="5" t="s">
         <v>602</v>
       </c>
       <c r="B320" s="6"/>
       <c r="C320" s="7" t="s">
-        <v>532</v>
+        <v>603</v>
       </c>
       <c r="D320" s="5" t="s">
         <v>6</v>
@@ -6704,42 +6713,42 @@
     </row>
     <row r="321">
       <c r="A321" s="20" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="B321" s="6"/>
       <c r="C321" s="7" t="s">
-        <v>604</v>
+        <v>534</v>
       </c>
       <c r="D321" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="322">
-      <c r="A322" s="20" t="s">
+      <c r="A322" s="21" t="s">
         <v>605</v>
       </c>
       <c r="B322" s="6"/>
       <c r="C322" s="7" t="s">
-        <v>534</v>
+        <v>606</v>
       </c>
       <c r="D322" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="323">
-      <c r="A323" s="20" t="s">
-        <v>606</v>
+      <c r="A323" s="21" t="s">
+        <v>607</v>
       </c>
       <c r="B323" s="6"/>
       <c r="C323" s="7" t="s">
-        <v>607</v>
+        <v>536</v>
       </c>
       <c r="D323" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="324">
-      <c r="A324" s="20" t="s">
+      <c r="A324" s="21" t="s">
         <v>608</v>
       </c>
       <c r="B324" s="6"/>
@@ -6751,7 +6760,7 @@
       </c>
     </row>
     <row r="325">
-      <c r="A325" s="20" t="s">
+      <c r="A325" s="21" t="s">
         <v>610</v>
       </c>
       <c r="B325" s="6"/>
@@ -6775,7 +6784,7 @@
       </c>
     </row>
     <row r="327">
-      <c r="A327" s="21" t="s">
+      <c r="A327" s="22" t="s">
         <v>614</v>
       </c>
       <c r="B327" s="6"/>
@@ -6787,7 +6796,7 @@
       </c>
     </row>
     <row r="328">
-      <c r="A328" s="21" t="s">
+      <c r="A328" s="22" t="s">
         <v>616</v>
       </c>
       <c r="B328" s="6"/>
@@ -6799,7 +6808,7 @@
       </c>
     </row>
     <row r="329">
-      <c r="A329" s="21" t="s">
+      <c r="A329" s="22" t="s">
         <v>618</v>
       </c>
       <c r="B329" s="6"/>
@@ -6811,7 +6820,7 @@
       </c>
     </row>
     <row r="330">
-      <c r="A330" s="21" t="s">
+      <c r="A330" s="22" t="s">
         <v>620</v>
       </c>
       <c r="B330" s="6"/>
@@ -6823,7 +6832,7 @@
       </c>
     </row>
     <row r="331">
-      <c r="A331" s="21" t="s">
+      <c r="A331" s="22" t="s">
         <v>622</v>
       </c>
       <c r="B331" s="6"/>
@@ -6835,7 +6844,7 @@
       </c>
     </row>
     <row r="332">
-      <c r="A332" s="5" t="s">
+      <c r="A332" s="22" t="s">
         <v>624</v>
       </c>
       <c r="B332" s="6"/>
@@ -7008,7 +7017,7 @@
       </c>
       <c r="B346" s="6"/>
       <c r="C346" s="7" t="s">
-        <v>461</v>
+        <v>653</v>
       </c>
       <c r="D346" s="5" t="s">
         <v>6</v>
@@ -7016,11 +7025,11 @@
     </row>
     <row r="347">
       <c r="A347" s="5" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B347" s="6"/>
       <c r="C347" s="7" t="s">
-        <v>654</v>
+        <v>463</v>
       </c>
       <c r="D347" s="5" t="s">
         <v>6</v>
@@ -7428,7 +7437,7 @@
       </c>
       <c r="B381" s="6"/>
       <c r="C381" s="7" t="s">
-        <v>633</v>
+        <v>722</v>
       </c>
       <c r="D381" s="5" t="s">
         <v>6</v>
@@ -7436,11 +7445,11 @@
     </row>
     <row r="382">
       <c r="A382" s="5" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B382" s="6"/>
       <c r="C382" s="7" t="s">
-        <v>723</v>
+        <v>635</v>
       </c>
       <c r="D382" s="5" t="s">
         <v>6</v>
@@ -7572,7 +7581,7 @@
       </c>
       <c r="B393" s="6"/>
       <c r="C393" s="7" t="s">
-        <v>510</v>
+        <v>745</v>
       </c>
       <c r="D393" s="5" t="s">
         <v>6</v>
@@ -7580,11 +7589,11 @@
     </row>
     <row r="394">
       <c r="A394" s="5" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B394" s="6"/>
       <c r="C394" s="7" t="s">
-        <v>746</v>
+        <v>512</v>
       </c>
       <c r="D394" s="5" t="s">
         <v>6</v>
@@ -7603,7 +7612,7 @@
       </c>
     </row>
     <row r="396">
-      <c r="A396" s="10" t="s">
+      <c r="A396" s="5" t="s">
         <v>749</v>
       </c>
       <c r="B396" s="6"/>
@@ -7639,7 +7648,7 @@
       </c>
     </row>
     <row r="399">
-      <c r="A399" s="5" t="s">
+      <c r="A399" s="10" t="s">
         <v>755</v>
       </c>
       <c r="B399" s="6"/>
@@ -7651,7 +7660,7 @@
       </c>
     </row>
     <row r="400">
-      <c r="A400" s="10" t="s">
+      <c r="A400" s="5" t="s">
         <v>757</v>
       </c>
       <c r="B400" s="6"/>
@@ -7663,7 +7672,7 @@
       </c>
     </row>
     <row r="401">
-      <c r="A401" s="5" t="s">
+      <c r="A401" s="10" t="s">
         <v>759</v>
       </c>
       <c r="B401" s="6"/>
@@ -7680,7 +7689,7 @@
       </c>
       <c r="B402" s="6"/>
       <c r="C402" s="7" t="s">
-        <v>164</v>
+        <v>762</v>
       </c>
       <c r="D402" s="5" t="s">
         <v>6</v>
@@ -7688,11 +7697,11 @@
     </row>
     <row r="403">
       <c r="A403" s="5" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B403" s="6"/>
       <c r="C403" s="7" t="s">
-        <v>763</v>
+        <v>164</v>
       </c>
       <c r="D403" s="5" t="s">
         <v>6</v>
@@ -7824,7 +7833,7 @@
       </c>
       <c r="B414" s="6"/>
       <c r="C414" s="7" t="s">
-        <v>779</v>
+        <v>785</v>
       </c>
       <c r="D414" s="5" t="s">
         <v>6</v>
@@ -7832,11 +7841,11 @@
     </row>
     <row r="415">
       <c r="A415" s="5" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="B415" s="6"/>
       <c r="C415" s="7" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="D415" s="5" t="s">
         <v>6</v>
@@ -7879,10 +7888,16 @@
       </c>
     </row>
     <row r="419">
-      <c r="A419" s="6"/>
+      <c r="A419" s="5" t="s">
+        <v>793</v>
+      </c>
       <c r="B419" s="6"/>
-      <c r="C419" s="6"/>
-      <c r="D419" s="6"/>
+      <c r="C419" s="7" t="s">
+        <v>794</v>
+      </c>
+      <c r="D419" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="420">
       <c r="A420" s="6"/>
@@ -12396,9 +12411,15 @@
       <c r="C1171" s="6"/>
       <c r="D1171" s="6"/>
     </row>
+    <row r="1172">
+      <c r="A1172" s="6"/>
+      <c r="B1172" s="6"/>
+      <c r="C1172" s="6"/>
+      <c r="D1172" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D418">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D419">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12407,7 +12428,7 @@
     <hyperlink r:id="rId2" ref="C7"/>
     <hyperlink r:id="rId3" ref="C8"/>
     <hyperlink r:id="rId4" ref="A87"/>
-    <hyperlink r:id="rId5" ref="A191"/>
+    <hyperlink r:id="rId5" ref="A192"/>
   </hyperlinks>
   <drawing r:id="rId6"/>
 </worksheet>
@@ -12463,11 +12484,11 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="7" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>6</v>
@@ -12475,10 +12496,10 @@
     </row>
     <row r="3">
       <c r="A3" s="12" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>6</v>
@@ -12486,10 +12507,10 @@
     </row>
     <row r="4">
       <c r="A4" s="12" t="s">
-        <v>797</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>798</v>
+        <v>799</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>800</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>6</v>
@@ -12497,10 +12518,10 @@
     </row>
     <row r="5">
       <c r="A5" s="12" t="s">
-        <v>799</v>
-      </c>
-      <c r="C5" s="22" t="s">
-        <v>800</v>
+        <v>801</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>802</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>6</v>
@@ -12508,10 +12529,10 @@
     </row>
     <row r="6">
       <c r="A6" s="12" t="s">
-        <v>801</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>802</v>
+        <v>803</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>804</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
circles titles on 2 lines
</commit_message>
<xml_diff>
--- a/wording.xlsx
+++ b/wording.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1277" uniqueCount="805">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="807">
   <si>
     <t>Key</t>
   </si>
@@ -568,25 +568,29 @@
     <t>home.circles.activity.label</t>
   </si>
   <si>
-    <t>Activity analysis</t>
+    <t>Activity
+analysis</t>
   </si>
   <si>
     <t>home.circles.live.label</t>
   </si>
   <si>
-    <t>Live measurement</t>
+    <t>Live
+measurement</t>
   </si>
   <si>
     <t>home.circles.alarm.label</t>
   </si>
   <si>
-    <t>Alarm clock</t>
+    <t>Alarm
+clock</t>
   </si>
   <si>
     <t>home.circles.sleep.label</t>
   </si>
   <si>
-    <t>Sleep analysis</t>
+    <t>Sleep
+analysis</t>
   </si>
   <si>
     <t>header.alarm</t>
@@ -2451,6 +2455,12 @@
     <t>Your new notes “&lt;bold&gt;{notes}&lt;/bold&gt;” have been added successfully</t>
   </si>
   <si>
+    <t>home.banner.common.select</t>
+  </si>
+  <si>
+    <t>Pick one</t>
+  </si>
+  <si>
     <t>months</t>
   </si>
   <si>
@@ -2485,7 +2495,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -2531,8 +2541,13 @@
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <strike/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2557,6 +2572,12 @@
         <bgColor rgb="FFFFA500"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -2564,7 +2585,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2624,6 +2645,12 @@
     </xf>
     <xf borderId="0" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
@@ -3965,10 +3992,10 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="13" t="s">
+      <c r="A92" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="C92" s="15" t="s">
+      <c r="C92" s="7" t="s">
         <v>166</v>
       </c>
       <c r="D92" s="12" t="s">
@@ -4076,7 +4103,7 @@
         <v>183</v>
       </c>
       <c r="B101" s="6"/>
-      <c r="C101" s="7" t="s">
+      <c r="C101" s="15" t="s">
         <v>184</v>
       </c>
       <c r="D101" s="5" t="s">
@@ -4088,7 +4115,7 @@
         <v>185</v>
       </c>
       <c r="B102" s="6"/>
-      <c r="C102" s="7" t="s">
+      <c r="C102" s="15" t="s">
         <v>186</v>
       </c>
       <c r="D102" s="5" t="s">
@@ -4100,7 +4127,7 @@
         <v>187</v>
       </c>
       <c r="B103" s="6"/>
-      <c r="C103" s="7" t="s">
+      <c r="C103" s="15" t="s">
         <v>188</v>
       </c>
       <c r="D103" s="5" t="s">
@@ -4112,7 +4139,7 @@
         <v>189</v>
       </c>
       <c r="B104" s="6"/>
-      <c r="C104" s="7" t="s">
+      <c r="C104" s="15" t="s">
         <v>190</v>
       </c>
       <c r="D104" s="5" t="s">
@@ -5896,26 +5923,26 @@
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="5" t="s">
+      <c r="A253" s="20" t="s">
         <v>475</v>
       </c>
-      <c r="B253" s="6"/>
-      <c r="C253" s="7" t="s">
+      <c r="B253" s="21"/>
+      <c r="C253" s="20" t="s">
         <v>476</v>
       </c>
-      <c r="D253" s="5" t="s">
+      <c r="D253" s="20" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="5" t="s">
+      <c r="A254" s="20" t="s">
         <v>477</v>
       </c>
-      <c r="B254" s="6"/>
-      <c r="C254" s="7" t="s">
+      <c r="B254" s="21"/>
+      <c r="C254" s="20" t="s">
         <v>478</v>
       </c>
-      <c r="D254" s="5" t="s">
+      <c r="D254" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -6712,7 +6739,7 @@
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="20" t="s">
+      <c r="A321" s="22" t="s">
         <v>604</v>
       </c>
       <c r="B321" s="6"/>
@@ -6724,7 +6751,7 @@
       </c>
     </row>
     <row r="322">
-      <c r="A322" s="21" t="s">
+      <c r="A322" s="23" t="s">
         <v>605</v>
       </c>
       <c r="B322" s="6"/>
@@ -6736,7 +6763,7 @@
       </c>
     </row>
     <row r="323">
-      <c r="A323" s="21" t="s">
+      <c r="A323" s="23" t="s">
         <v>607</v>
       </c>
       <c r="B323" s="6"/>
@@ -6748,7 +6775,7 @@
       </c>
     </row>
     <row r="324">
-      <c r="A324" s="21" t="s">
+      <c r="A324" s="23" t="s">
         <v>608</v>
       </c>
       <c r="B324" s="6"/>
@@ -6760,7 +6787,7 @@
       </c>
     </row>
     <row r="325">
-      <c r="A325" s="21" t="s">
+      <c r="A325" s="23" t="s">
         <v>610</v>
       </c>
       <c r="B325" s="6"/>
@@ -6772,7 +6799,7 @@
       </c>
     </row>
     <row r="326">
-      <c r="A326" s="21" t="s">
+      <c r="A326" s="23" t="s">
         <v>612</v>
       </c>
       <c r="B326" s="6"/>
@@ -6784,7 +6811,7 @@
       </c>
     </row>
     <row r="327">
-      <c r="A327" s="22" t="s">
+      <c r="A327" s="24" t="s">
         <v>614</v>
       </c>
       <c r="B327" s="6"/>
@@ -6796,7 +6823,7 @@
       </c>
     </row>
     <row r="328">
-      <c r="A328" s="22" t="s">
+      <c r="A328" s="24" t="s">
         <v>616</v>
       </c>
       <c r="B328" s="6"/>
@@ -6808,7 +6835,7 @@
       </c>
     </row>
     <row r="329">
-      <c r="A329" s="22" t="s">
+      <c r="A329" s="24" t="s">
         <v>618</v>
       </c>
       <c r="B329" s="6"/>
@@ -6820,7 +6847,7 @@
       </c>
     </row>
     <row r="330">
-      <c r="A330" s="22" t="s">
+      <c r="A330" s="24" t="s">
         <v>620</v>
       </c>
       <c r="B330" s="6"/>
@@ -6832,7 +6859,7 @@
       </c>
     </row>
     <row r="331">
-      <c r="A331" s="22" t="s">
+      <c r="A331" s="24" t="s">
         <v>622</v>
       </c>
       <c r="B331" s="6"/>
@@ -6844,7 +6871,7 @@
       </c>
     </row>
     <row r="332">
-      <c r="A332" s="22" t="s">
+      <c r="A332" s="24" t="s">
         <v>624</v>
       </c>
       <c r="B332" s="6"/>
@@ -7420,26 +7447,26 @@
       </c>
     </row>
     <row r="380">
-      <c r="A380" s="5" t="s">
+      <c r="A380" s="20" t="s">
         <v>719</v>
       </c>
-      <c r="B380" s="6"/>
-      <c r="C380" s="7" t="s">
+      <c r="B380" s="21"/>
+      <c r="C380" s="20" t="s">
         <v>720</v>
       </c>
-      <c r="D380" s="5" t="s">
+      <c r="D380" s="20" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="381">
-      <c r="A381" s="5" t="s">
+      <c r="A381" s="20" t="s">
         <v>721</v>
       </c>
-      <c r="B381" s="6"/>
-      <c r="C381" s="7" t="s">
+      <c r="B381" s="21"/>
+      <c r="C381" s="20" t="s">
         <v>722</v>
       </c>
-      <c r="D381" s="5" t="s">
+      <c r="D381" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -7900,10 +7927,16 @@
       </c>
     </row>
     <row r="420">
-      <c r="A420" s="6"/>
+      <c r="A420" s="5" t="s">
+        <v>795</v>
+      </c>
       <c r="B420" s="6"/>
-      <c r="C420" s="6"/>
-      <c r="D420" s="6"/>
+      <c r="C420" s="7" t="s">
+        <v>796</v>
+      </c>
+      <c r="D420" s="5" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="421">
       <c r="A421" s="6"/>
@@ -12419,7 +12452,7 @@
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D419">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D420">
       <formula1>"Validé,A valider"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12484,11 +12517,11 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="7" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>6</v>
@@ -12496,10 +12529,10 @@
     </row>
     <row r="3">
       <c r="A3" s="12" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>798</v>
+        <v>800</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>6</v>
@@ -12507,10 +12540,10 @@
     </row>
     <row r="4">
       <c r="A4" s="12" t="s">
-        <v>799</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>800</v>
+        <v>801</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>802</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>6</v>
@@ -12518,10 +12551,10 @@
     </row>
     <row r="5">
       <c r="A5" s="12" t="s">
-        <v>801</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>802</v>
+        <v>803</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>804</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>6</v>
@@ -12529,10 +12562,10 @@
     </row>
     <row r="6">
       <c r="A6" s="12" t="s">
-        <v>803</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>804</v>
+        <v>805</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>806</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>6</v>

</xml_diff>